<commit_message>
chore: update IPO data
</commit_message>
<xml_diff>
--- a/IPO_analysis.xlsx
+++ b/IPO_analysis.xlsx
@@ -618,7 +618,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>기준일 2026-07-08 · 청구일 직전 사업연도 · 별도/개별 재무제표 · 단위 백만원(별도 표기 시 USD)</t>
+          <t>기준일 2026-07-09 · 청구일 직전 사업연도 · 별도/개별 재무제표 · 단위 백만원(별도 표기 시 USD)</t>
         </is>
       </c>
     </row>
@@ -6576,25 +6576,19 @@
           <t>20,000</t>
         </is>
       </c>
-      <c r="F7" s="18" t="inlineStr">
-        <is>
-          <t>수집예정</t>
-        </is>
-      </c>
-      <c r="G7" s="6" t="inlineStr">
-        <is>
-          <t>10,000</t>
-        </is>
-      </c>
-      <c r="H7" s="18" t="inlineStr">
-        <is>
-          <t>수집예정</t>
-        </is>
-      </c>
-      <c r="I7" s="18" t="inlineStr">
-        <is>
-          <t>수집예정</t>
-        </is>
+      <c r="F7" s="6" t="inlineStr">
+        <is>
+          <t>상대가치법·PER / 비교회사 평균 PER 25.48배 (2027 추정 순이익), 주당평가 14,844원</t>
+        </is>
+      </c>
+      <c r="G7" s="6" t="n">
+        <v>10000</v>
+      </c>
+      <c r="H7" s="6" t="n">
+        <v>1238</v>
+      </c>
+      <c r="I7" s="6" t="n">
+        <v>2233</v>
       </c>
       <c r="J7" s="6" t="inlineStr">
         <is>
@@ -6660,25 +6654,19 @@
           <t>16,000</t>
         </is>
       </c>
-      <c r="F8" s="18" t="inlineStr">
-        <is>
-          <t>수집예정</t>
-        </is>
-      </c>
-      <c r="G8" s="6" t="inlineStr">
-        <is>
-          <t>8,000</t>
-        </is>
-      </c>
-      <c r="H8" s="18" t="inlineStr">
-        <is>
-          <t>수집예정</t>
-        </is>
-      </c>
-      <c r="I8" s="18" t="inlineStr">
-        <is>
-          <t>수집예정</t>
-        </is>
+      <c r="F8" s="6" t="inlineStr">
+        <is>
+          <t>상대가치법·PER / 유사기업 PER 24.57배, 주당평가 11,573원, 할인율 39.5~30.8%</t>
+        </is>
+      </c>
+      <c r="G8" s="6" t="n">
+        <v>8000</v>
+      </c>
+      <c r="H8" s="6" t="n">
+        <v>1396.29</v>
+      </c>
+      <c r="I8" s="6" t="n">
+        <v>2392</v>
       </c>
       <c r="J8" s="6" t="inlineStr">
         <is>
@@ -6754,14 +6742,14 @@
           <t>2,000</t>
         </is>
       </c>
-      <c r="H9" s="19" t="inlineStr">
-        <is>
-          <t>해당없음</t>
-        </is>
-      </c>
-      <c r="I9" s="19" t="inlineStr">
-        <is>
-          <t>해당없음</t>
+      <c r="H9" s="18" t="inlineStr">
+        <is>
+          <t>수집예정</t>
+        </is>
+      </c>
+      <c r="I9" s="18" t="inlineStr">
+        <is>
+          <t>수집예정</t>
         </is>
       </c>
       <c r="J9" s="6" t="inlineStr">
@@ -6828,25 +6816,19 @@
           <t>84,000</t>
         </is>
       </c>
-      <c r="F10" s="18" t="inlineStr">
-        <is>
-          <t>수집예정</t>
-        </is>
-      </c>
-      <c r="G10" s="6" t="inlineStr">
-        <is>
-          <t>12,000</t>
-        </is>
-      </c>
-      <c r="H10" s="18" t="inlineStr">
-        <is>
-          <t>수집예정</t>
-        </is>
-      </c>
-      <c r="I10" s="18" t="inlineStr">
-        <is>
-          <t>수집예정</t>
-        </is>
+      <c r="F10" s="6" t="inlineStr">
+        <is>
+          <t>상대가치법·PER / 비교 3사(현대오토에버·슈어소프트테크·엠디에스테크) 2025 실적 PER, 적용 37.45배, 주당평가 17,585원</t>
+        </is>
+      </c>
+      <c r="G10" s="6" t="n">
+        <v>12000</v>
+      </c>
+      <c r="H10" s="6" t="n">
+        <v>381.3</v>
+      </c>
+      <c r="I10" s="6" t="n">
+        <v>1604</v>
       </c>
       <c r="J10" s="6" t="inlineStr">
         <is>
@@ -6912,25 +6894,19 @@
           <t>20,000</t>
         </is>
       </c>
-      <c r="F11" s="18" t="inlineStr">
-        <is>
-          <t>수집예정</t>
-        </is>
-      </c>
-      <c r="G11" s="6" t="inlineStr">
-        <is>
-          <t>12,500</t>
-        </is>
-      </c>
-      <c r="H11" s="18" t="inlineStr">
-        <is>
-          <t>수집예정</t>
-        </is>
-      </c>
-      <c r="I11" s="18" t="inlineStr">
-        <is>
-          <t>수집예정</t>
-        </is>
+      <c r="F11" s="6" t="inlineStr">
+        <is>
+          <t>상대가치법·PER / 유사기업 PER 26.82배, 주당평가 16,139원, 할인율 22.55~34.94%</t>
+        </is>
+      </c>
+      <c r="G11" s="6" t="n">
+        <v>12500</v>
+      </c>
+      <c r="H11" s="6" t="n">
+        <v>1294.99</v>
+      </c>
+      <c r="I11" s="6" t="n">
+        <v>2252</v>
       </c>
       <c r="J11" s="6" t="inlineStr">
         <is>
@@ -7006,14 +6982,14 @@
           <t>2,000</t>
         </is>
       </c>
-      <c r="H12" s="19" t="inlineStr">
-        <is>
-          <t>해당없음</t>
-        </is>
-      </c>
-      <c r="I12" s="19" t="inlineStr">
-        <is>
-          <t>해당없음</t>
+      <c r="H12" s="18" t="inlineStr">
+        <is>
+          <t>수집예정</t>
+        </is>
+      </c>
+      <c r="I12" s="18" t="inlineStr">
+        <is>
+          <t>수집예정</t>
         </is>
       </c>
       <c r="J12" s="6" t="inlineStr">
@@ -7080,25 +7056,19 @@
           <t>48,862</t>
         </is>
       </c>
-      <c r="F13" s="18" t="inlineStr">
-        <is>
-          <t>수집예정</t>
-        </is>
-      </c>
-      <c r="G13" s="6" t="inlineStr">
-        <is>
-          <t>21,500</t>
-        </is>
-      </c>
-      <c r="H13" s="6" t="inlineStr">
-        <is>
-          <t>847.76</t>
-        </is>
-      </c>
-      <c r="I13" s="6" t="inlineStr">
-        <is>
-          <t>2,329</t>
-        </is>
+      <c r="F13" s="6" t="inlineStr">
+        <is>
+          <t>상대가치법·PER / 비교회사 PER 21.48배 (2025 조정 순이익), 주당평가 24,902원, 할인율 23.70~13.66%</t>
+        </is>
+      </c>
+      <c r="G13" s="6" t="n">
+        <v>21500</v>
+      </c>
+      <c r="H13" s="6" t="n">
+        <v>847.76</v>
+      </c>
+      <c r="I13" s="6" t="n">
+        <v>2329</v>
       </c>
       <c r="J13" s="6" t="inlineStr">
         <is>
@@ -7178,14 +7148,14 @@
           <t>2,000</t>
         </is>
       </c>
-      <c r="H14" s="19" t="inlineStr">
-        <is>
-          <t>해당없음</t>
-        </is>
-      </c>
-      <c r="I14" s="19" t="inlineStr">
-        <is>
-          <t>해당없음</t>
+      <c r="H14" s="18" t="inlineStr">
+        <is>
+          <t>수집예정</t>
+        </is>
+      </c>
+      <c r="I14" s="18" t="inlineStr">
+        <is>
+          <t>수집예정</t>
         </is>
       </c>
       <c r="J14" s="6" t="inlineStr">
@@ -7252,25 +7222,19 @@
           <t>39,525</t>
         </is>
       </c>
-      <c r="F15" s="18" t="inlineStr">
-        <is>
-          <t>수집예정</t>
-        </is>
-      </c>
-      <c r="G15" s="6" t="inlineStr">
-        <is>
-          <t>15,000</t>
-        </is>
-      </c>
-      <c r="H15" s="18" t="inlineStr">
-        <is>
-          <t>수집예정</t>
-        </is>
-      </c>
-      <c r="I15" s="18" t="inlineStr">
-        <is>
-          <t>수집예정</t>
-        </is>
+      <c r="F15" s="6" t="inlineStr">
+        <is>
+          <t>상대가치법·PER / 유사기업 PER 40.5배 (2028 추정 순이익), 주당평가 23,143원, 할인율 35.2~46.0%</t>
+        </is>
+      </c>
+      <c r="G15" s="6" t="n">
+        <v>15000</v>
+      </c>
+      <c r="H15" s="6" t="n">
+        <v>1196.08</v>
+      </c>
+      <c r="I15" s="6" t="n">
+        <v>2427</v>
       </c>
       <c r="J15" s="6" t="inlineStr">
         <is>
@@ -7336,25 +7300,19 @@
           <t>13,000</t>
         </is>
       </c>
-      <c r="F16" s="18" t="inlineStr">
-        <is>
-          <t>수집예정</t>
-        </is>
-      </c>
-      <c r="G16" s="6" t="inlineStr">
-        <is>
-          <t>5,000</t>
-        </is>
-      </c>
-      <c r="H16" s="18" t="inlineStr">
-        <is>
-          <t>수집예정</t>
-        </is>
-      </c>
-      <c r="I16" s="18" t="inlineStr">
-        <is>
-          <t>수집예정</t>
-        </is>
+      <c r="F16" s="6" t="inlineStr">
+        <is>
+          <t>상대가치법·PER / 유사기업 PER 19.05배 (2025 실적 순이익), 주당평가 6,178원, 할인율 33.64~19.07%</t>
+        </is>
+      </c>
+      <c r="G16" s="6" t="n">
+        <v>5000</v>
+      </c>
+      <c r="H16" s="6" t="n">
+        <v>1486.66</v>
+      </c>
+      <c r="I16" s="6" t="n">
+        <v>2372</v>
       </c>
       <c r="J16" s="6" t="inlineStr">
         <is>
@@ -7420,25 +7378,19 @@
           <t>25,020</t>
         </is>
       </c>
-      <c r="F17" s="18" t="inlineStr">
-        <is>
-          <t>수집예정</t>
-        </is>
-      </c>
-      <c r="G17" s="6" t="inlineStr">
-        <is>
-          <t>6,000</t>
-        </is>
-      </c>
-      <c r="H17" s="6" t="inlineStr">
-        <is>
-          <t>1,140.11</t>
-        </is>
-      </c>
-      <c r="I17" s="6" t="inlineStr">
-        <is>
-          <t>2,257</t>
-        </is>
+      <c r="F17" s="6" t="inlineStr">
+        <is>
+          <t>상대가치법·PER / 유사기업 PER 47.45배 (2028 추정 순이익)</t>
+        </is>
+      </c>
+      <c r="G17" s="6" t="n">
+        <v>6000</v>
+      </c>
+      <c r="H17" s="6" t="n">
+        <v>1140.11</v>
+      </c>
+      <c r="I17" s="6" t="n">
+        <v>2257</v>
       </c>
       <c r="J17" s="6" t="inlineStr">
         <is>
@@ -7518,14 +7470,14 @@
           <t>2,000</t>
         </is>
       </c>
-      <c r="H18" s="19" t="inlineStr">
-        <is>
-          <t>해당없음</t>
-        </is>
-      </c>
-      <c r="I18" s="19" t="inlineStr">
-        <is>
-          <t>해당없음</t>
+      <c r="H18" s="18" t="inlineStr">
+        <is>
+          <t>수집예정</t>
+        </is>
+      </c>
+      <c r="I18" s="18" t="inlineStr">
+        <is>
+          <t>수집예정</t>
         </is>
       </c>
       <c r="J18" s="6" t="inlineStr">
@@ -7592,25 +7544,19 @@
           <t>110,700</t>
         </is>
       </c>
-      <c r="F19" s="18" t="inlineStr">
-        <is>
-          <t>수집예정</t>
-        </is>
-      </c>
-      <c r="G19" s="6" t="inlineStr">
-        <is>
-          <t>12,300</t>
-        </is>
-      </c>
-      <c r="H19" s="6" t="inlineStr">
-        <is>
-          <t>55.23</t>
-        </is>
-      </c>
-      <c r="I19" s="6" t="inlineStr">
-        <is>
-          <t>751</t>
-        </is>
+      <c r="F19" s="6" t="inlineStr">
+        <is>
+          <t>상대가치법·EV/EBITDA / 비교기업 평균 24.0배 (2028 추정 EBITDA)</t>
+        </is>
+      </c>
+      <c r="G19" s="6" t="n">
+        <v>12300</v>
+      </c>
+      <c r="H19" s="6" t="n">
+        <v>55.23</v>
+      </c>
+      <c r="I19" s="6" t="n">
+        <v>751</v>
       </c>
       <c r="J19" s="6" t="inlineStr">
         <is>
@@ -7690,14 +7636,14 @@
           <t>2,000</t>
         </is>
       </c>
-      <c r="H20" s="19" t="inlineStr">
-        <is>
-          <t>해당없음</t>
-        </is>
-      </c>
-      <c r="I20" s="19" t="inlineStr">
-        <is>
-          <t>해당없음</t>
+      <c r="H20" s="18" t="inlineStr">
+        <is>
+          <t>수집예정</t>
+        </is>
+      </c>
+      <c r="I20" s="18" t="inlineStr">
+        <is>
+          <t>수집예정</t>
         </is>
       </c>
       <c r="J20" s="6" t="inlineStr">
@@ -7774,14 +7720,14 @@
           <t>2,000</t>
         </is>
       </c>
-      <c r="H21" s="19" t="inlineStr">
-        <is>
-          <t>해당없음</t>
-        </is>
-      </c>
-      <c r="I21" s="19" t="inlineStr">
-        <is>
-          <t>해당없음</t>
+      <c r="H21" s="18" t="inlineStr">
+        <is>
+          <t>수집예정</t>
+        </is>
+      </c>
+      <c r="I21" s="18" t="inlineStr">
+        <is>
+          <t>수집예정</t>
         </is>
       </c>
       <c r="J21" s="6" t="inlineStr">
@@ -7848,25 +7794,19 @@
           <t>19,588</t>
         </is>
       </c>
-      <c r="F22" s="18" t="inlineStr">
-        <is>
-          <t>수집예정</t>
-        </is>
-      </c>
-      <c r="G22" s="6" t="inlineStr">
-        <is>
-          <t>16,600</t>
-        </is>
-      </c>
-      <c r="H22" s="18" t="inlineStr">
-        <is>
-          <t>수집예정</t>
-        </is>
-      </c>
-      <c r="I22" s="18" t="inlineStr">
-        <is>
-          <t>수집예정</t>
-        </is>
+      <c r="F22" s="6" t="inlineStr">
+        <is>
+          <t>상대가치법·PER / 유사기업 PER 24.34배 (2029 추정 순이익), 주당평가 21,257원, 할인율 43.08~21.91%</t>
+        </is>
+      </c>
+      <c r="G22" s="6" t="n">
+        <v>16600</v>
+      </c>
+      <c r="H22" s="6" t="n">
+        <v>1328.82</v>
+      </c>
+      <c r="I22" s="6" t="n">
+        <v>2309</v>
       </c>
       <c r="J22" s="6" t="inlineStr">
         <is>
@@ -7942,14 +7882,14 @@
           <t>2,000</t>
         </is>
       </c>
-      <c r="H23" s="19" t="inlineStr">
-        <is>
-          <t>해당없음</t>
-        </is>
-      </c>
-      <c r="I23" s="19" t="inlineStr">
-        <is>
-          <t>해당없음</t>
+      <c r="H23" s="18" t="inlineStr">
+        <is>
+          <t>수집예정</t>
+        </is>
+      </c>
+      <c r="I23" s="18" t="inlineStr">
+        <is>
+          <t>수집예정</t>
         </is>
       </c>
       <c r="J23" s="6" t="inlineStr">
@@ -8016,25 +7956,19 @@
           <t>15,400</t>
         </is>
       </c>
-      <c r="F24" s="18" t="inlineStr">
-        <is>
-          <t>수집예정</t>
-        </is>
-      </c>
-      <c r="G24" s="6" t="inlineStr">
-        <is>
-          <t>11,000</t>
-        </is>
-      </c>
-      <c r="H24" s="18" t="inlineStr">
-        <is>
-          <t>수집예정</t>
-        </is>
-      </c>
-      <c r="I24" s="18" t="inlineStr">
-        <is>
-          <t>수집예정</t>
-        </is>
+      <c r="F24" s="6" t="inlineStr">
+        <is>
+          <t>상대가치법·PER / 비교회사 PER 31.33배 (2027 추정 순이익), 주당평가 16,177원, 할인율 44.37~32.00%</t>
+        </is>
+      </c>
+      <c r="G24" s="6" t="n">
+        <v>11000</v>
+      </c>
+      <c r="H24" s="6" t="n">
+        <v>1352.63</v>
+      </c>
+      <c r="I24" s="6" t="n">
+        <v>2261</v>
       </c>
       <c r="J24" s="6" t="inlineStr">
         <is>
@@ -8114,14 +8048,14 @@
           <t>2,000</t>
         </is>
       </c>
-      <c r="H25" s="19" t="inlineStr">
-        <is>
-          <t>해당없음</t>
-        </is>
-      </c>
-      <c r="I25" s="19" t="inlineStr">
-        <is>
-          <t>해당없음</t>
+      <c r="H25" s="18" t="inlineStr">
+        <is>
+          <t>수집예정</t>
+        </is>
+      </c>
+      <c r="I25" s="18" t="inlineStr">
+        <is>
+          <t>수집예정</t>
         </is>
       </c>
       <c r="J25" s="6" t="inlineStr">
@@ -8188,25 +8122,19 @@
           <t>29,052</t>
         </is>
       </c>
-      <c r="F26" s="18" t="inlineStr">
-        <is>
-          <t>수집예정</t>
-        </is>
-      </c>
-      <c r="G26" s="6" t="inlineStr">
-        <is>
-          <t>21,600</t>
-        </is>
-      </c>
-      <c r="H26" s="18" t="inlineStr">
-        <is>
-          <t>수집예정</t>
-        </is>
-      </c>
-      <c r="I26" s="18" t="inlineStr">
-        <is>
-          <t>수집예정</t>
-        </is>
+      <c r="F26" s="6" t="inlineStr">
+        <is>
+          <t>상대가치법·PER / 비교기업 PER 20.66배 (2028 추정 순이익), 주당평가 26,899원, 할인율 38.00~19.80%</t>
+        </is>
+      </c>
+      <c r="G26" s="6" t="n">
+        <v>21600</v>
+      </c>
+      <c r="H26" s="6" t="n">
+        <v>1108.93</v>
+      </c>
+      <c r="I26" s="6" t="n">
+        <v>2320</v>
       </c>
       <c r="J26" s="6" t="inlineStr">
         <is>
@@ -8272,25 +8200,19 @@
           <t>20,900</t>
         </is>
       </c>
-      <c r="F27" s="18" t="inlineStr">
-        <is>
-          <t>수집예정</t>
-        </is>
-      </c>
-      <c r="G27" s="6" t="inlineStr">
-        <is>
-          <t>19,000</t>
-        </is>
-      </c>
-      <c r="H27" s="6" t="inlineStr">
-        <is>
-          <t>1,172.59</t>
-        </is>
-      </c>
-      <c r="I27" s="6" t="inlineStr">
-        <is>
-          <t>2,229</t>
-        </is>
+      <c r="F27" s="6" t="inlineStr">
+        <is>
+          <t>상대가치법·PER / 유사기업 PER 29.09배, 주당평가 27,244원, 할인율 37.60~30.26%</t>
+        </is>
+      </c>
+      <c r="G27" s="6" t="n">
+        <v>19000</v>
+      </c>
+      <c r="H27" s="6" t="n">
+        <v>1172.59</v>
+      </c>
+      <c r="I27" s="6" t="n">
+        <v>2229</v>
       </c>
       <c r="J27" s="6" t="inlineStr">
         <is>
@@ -8356,25 +8278,19 @@
           <t>52,000</t>
         </is>
       </c>
-      <c r="F28" s="18" t="inlineStr">
-        <is>
-          <t>수집예정</t>
-        </is>
-      </c>
-      <c r="G28" s="6" t="inlineStr">
-        <is>
-          <t>26,000</t>
-        </is>
-      </c>
-      <c r="H28" s="6" t="inlineStr">
-        <is>
-          <t>839.23</t>
-        </is>
-      </c>
-      <c r="I28" s="6" t="inlineStr">
-        <is>
-          <t>2,333</t>
-        </is>
+      <c r="F28" s="6" t="inlineStr">
+        <is>
+          <t>상대가치법·PER / 비교회사 PER 21.46배 (2028 추정 순이익), 주당평가 41,663원, 할인율 37.59~54.40%</t>
+        </is>
+      </c>
+      <c r="G28" s="6" t="n">
+        <v>26000</v>
+      </c>
+      <c r="H28" s="6" t="n">
+        <v>839.23</v>
+      </c>
+      <c r="I28" s="6" t="n">
+        <v>2333</v>
       </c>
       <c r="J28" s="6" t="inlineStr">
         <is>
@@ -8440,25 +8356,19 @@
           <t>40,000</t>
         </is>
       </c>
-      <c r="F29" s="18" t="inlineStr">
-        <is>
-          <t>수집예정</t>
-        </is>
-      </c>
-      <c r="G29" s="6" t="inlineStr">
-        <is>
-          <t>20,000</t>
-        </is>
-      </c>
-      <c r="H29" s="18" t="inlineStr">
-        <is>
-          <t>수집예정</t>
-        </is>
-      </c>
-      <c r="I29" s="18" t="inlineStr">
-        <is>
-          <t>수집예정</t>
-        </is>
+      <c r="F29" s="6" t="inlineStr">
+        <is>
+          <t>상대가치법·PER / 비교대상회사 PER 23.59배, 할인율 35.30~19.13%</t>
+        </is>
+      </c>
+      <c r="G29" s="6" t="n">
+        <v>20000</v>
+      </c>
+      <c r="H29" s="6" t="n">
+        <v>962.1</v>
+      </c>
+      <c r="I29" s="6" t="n">
+        <v>2327</v>
       </c>
       <c r="J29" s="6" t="inlineStr">
         <is>
@@ -8524,25 +8434,19 @@
           <t>26,450</t>
         </is>
       </c>
-      <c r="F30" s="18" t="inlineStr">
-        <is>
-          <t>수집예정</t>
-        </is>
-      </c>
-      <c r="G30" s="6" t="inlineStr">
-        <is>
-          <t>11,500</t>
-        </is>
-      </c>
-      <c r="H30" s="18" t="inlineStr">
-        <is>
-          <t>수집예정</t>
-        </is>
-      </c>
-      <c r="I30" s="18" t="inlineStr">
-        <is>
-          <t>수집예정</t>
-        </is>
+      <c r="F30" s="6" t="inlineStr">
+        <is>
+          <t>상대가치법·PER / 유사기업 PER 27.60배, 할인율 23.40~32.73%</t>
+        </is>
+      </c>
+      <c r="G30" s="6" t="n">
+        <v>11500</v>
+      </c>
+      <c r="H30" s="6" t="n">
+        <v>1124.21</v>
+      </c>
+      <c r="I30" s="6" t="n">
+        <v>2411</v>
       </c>
       <c r="J30" s="6" t="inlineStr">
         <is>
@@ -8608,25 +8512,19 @@
           <t>15,300</t>
         </is>
       </c>
-      <c r="F31" s="18" t="inlineStr">
-        <is>
-          <t>수집예정</t>
-        </is>
-      </c>
-      <c r="G31" s="6" t="inlineStr">
-        <is>
-          <t>8,500</t>
-        </is>
-      </c>
-      <c r="H31" s="18" t="inlineStr">
-        <is>
-          <t>수집예정</t>
-        </is>
-      </c>
-      <c r="I31" s="18" t="inlineStr">
-        <is>
-          <t>수집예정</t>
-        </is>
+      <c r="F31" s="6" t="inlineStr">
+        <is>
+          <t>상대가치법·EV/EBITDA / 비교대상기업 EV/EBITDA 17.71배</t>
+        </is>
+      </c>
+      <c r="G31" s="6" t="n">
+        <v>8500</v>
+      </c>
+      <c r="H31" s="6" t="n">
+        <v>1334.91</v>
+      </c>
+      <c r="I31" s="6" t="n">
+        <v>2263</v>
       </c>
       <c r="J31" s="6" t="inlineStr">
         <is>
@@ -8692,25 +8590,19 @@
           <t>498,000</t>
         </is>
       </c>
-      <c r="F32" s="18" t="inlineStr">
-        <is>
-          <t>수집예정</t>
-        </is>
-      </c>
-      <c r="G32" s="6" t="inlineStr">
-        <is>
-          <t>8,300</t>
-        </is>
-      </c>
-      <c r="H32" s="18" t="inlineStr">
-        <is>
-          <t>수집예정</t>
-        </is>
-      </c>
-      <c r="I32" s="18" t="inlineStr">
-        <is>
-          <t>수집예정</t>
-        </is>
+      <c r="F32" s="6" t="inlineStr">
+        <is>
+          <t>상대가치법·PBR / 유사기업 PBR 1.80배 (2025 3Q 자본총계 기준)</t>
+        </is>
+      </c>
+      <c r="G32" s="6" t="n">
+        <v>8300</v>
+      </c>
+      <c r="H32" s="6" t="n">
+        <v>198.53</v>
+      </c>
+      <c r="I32" s="6" t="n">
+        <v>2007</v>
       </c>
       <c r="J32" s="6" t="inlineStr">
         <is>
@@ -8864,25 +8756,19 @@
           <t>75,000</t>
         </is>
       </c>
-      <c r="F34" s="18" t="inlineStr">
-        <is>
-          <t>수집예정</t>
-        </is>
-      </c>
-      <c r="G34" s="6" t="inlineStr">
-        <is>
-          <t>10,000</t>
-        </is>
-      </c>
-      <c r="H34" s="18" t="inlineStr">
-        <is>
-          <t>수집예정</t>
-        </is>
-      </c>
-      <c r="I34" s="18" t="inlineStr">
-        <is>
-          <t>수집예정</t>
-        </is>
+      <c r="F34" s="6" t="inlineStr">
+        <is>
+          <t>상대가치법·EV/EBITDA / 유사기업 EV/EBITDA 30.32배, 할인율 36.02~24.73%</t>
+        </is>
+      </c>
+      <c r="G34" s="6" t="n">
+        <v>10000</v>
+      </c>
+      <c r="H34" s="6" t="n">
+        <v>650.14</v>
+      </c>
+      <c r="I34" s="6" t="n">
+        <v>2324</v>
       </c>
       <c r="J34" s="6" t="inlineStr">
         <is>
@@ -9046,14 +8932,14 @@
           <t>2,000</t>
         </is>
       </c>
-      <c r="H36" s="19" t="inlineStr">
-        <is>
-          <t>해당없음</t>
-        </is>
-      </c>
-      <c r="I36" s="19" t="inlineStr">
-        <is>
-          <t>해당없음</t>
+      <c r="H36" s="18" t="inlineStr">
+        <is>
+          <t>수집예정</t>
+        </is>
+      </c>
+      <c r="I36" s="18" t="inlineStr">
+        <is>
+          <t>수집예정</t>
         </is>
       </c>
       <c r="J36" s="6" t="inlineStr">

</xml_diff>

<commit_message>
chore: update IPO data 2026-07-09
</commit_message>
<xml_diff>
--- a/IPO_analysis.xlsx
+++ b/IPO_analysis.xlsx
@@ -6652,10 +6652,8 @@
           <t>2026-06-24~25</t>
         </is>
       </c>
-      <c r="K7" s="18" t="inlineStr">
-        <is>
-          <t>수집예정</t>
-        </is>
+      <c r="K7" s="6" t="n">
+        <v>1510.57</v>
       </c>
       <c r="L7" s="6" t="inlineStr"/>
       <c r="M7" s="6" t="inlineStr">
@@ -6730,10 +6728,8 @@
           <t>2026-06-23~24</t>
         </is>
       </c>
-      <c r="K8" s="18" t="inlineStr">
-        <is>
-          <t>수집예정</t>
-        </is>
+      <c r="K8" s="6" t="n">
+        <v>3304.76</v>
       </c>
       <c r="L8" s="6" t="inlineStr"/>
       <c r="M8" s="6" t="inlineStr">
@@ -6774,40 +6770,36 @@
           <t>해당없음</t>
         </is>
       </c>
-      <c r="C9" s="19" t="inlineStr">
+      <c r="C9" s="6" t="inlineStr">
+        <is>
+          <t>2,000</t>
+        </is>
+      </c>
+      <c r="D9" s="7" t="inlineStr">
+        <is>
+          <t>5,500,000</t>
+        </is>
+      </c>
+      <c r="E9" s="7" t="inlineStr">
+        <is>
+          <t>11,000</t>
+        </is>
+      </c>
+      <c r="F9" s="19" t="inlineStr">
         <is>
           <t>해당없음</t>
         </is>
       </c>
-      <c r="D9" s="7" t="inlineStr">
-        <is>
-          <t>5,500,000</t>
-        </is>
-      </c>
-      <c r="E9" s="7" t="inlineStr">
-        <is>
-          <t>11,000</t>
-        </is>
-      </c>
-      <c r="F9" s="19" t="inlineStr">
-        <is>
-          <t>해당없음</t>
-        </is>
-      </c>
       <c r="G9" s="6" t="inlineStr">
         <is>
           <t>2,000</t>
         </is>
       </c>
-      <c r="H9" s="18" t="inlineStr">
-        <is>
-          <t>수집예정</t>
-        </is>
-      </c>
-      <c r="I9" s="18" t="inlineStr">
-        <is>
-          <t>수집예정</t>
-        </is>
+      <c r="H9" s="6" t="n">
+        <v>1364.09</v>
+      </c>
+      <c r="I9" s="6" t="n">
+        <v>2089</v>
       </c>
       <c r="J9" s="6" t="inlineStr">
         <is>
@@ -7014,40 +7006,36 @@
           <t>해당없음</t>
         </is>
       </c>
-      <c r="C12" s="19" t="inlineStr">
+      <c r="C12" s="6" t="inlineStr">
+        <is>
+          <t>2,000</t>
+        </is>
+      </c>
+      <c r="D12" s="7" t="inlineStr">
+        <is>
+          <t>7,000,000</t>
+        </is>
+      </c>
+      <c r="E12" s="7" t="inlineStr">
+        <is>
+          <t>14,000</t>
+        </is>
+      </c>
+      <c r="F12" s="19" t="inlineStr">
         <is>
           <t>해당없음</t>
         </is>
       </c>
-      <c r="D12" s="7" t="inlineStr">
-        <is>
-          <t>7,000,000</t>
-        </is>
-      </c>
-      <c r="E12" s="7" t="inlineStr">
-        <is>
-          <t>14,000</t>
-        </is>
-      </c>
-      <c r="F12" s="19" t="inlineStr">
-        <is>
-          <t>해당없음</t>
-        </is>
-      </c>
       <c r="G12" s="6" t="inlineStr">
         <is>
           <t>2,000</t>
         </is>
       </c>
-      <c r="H12" s="18" t="inlineStr">
-        <is>
-          <t>수집예정</t>
-        </is>
-      </c>
-      <c r="I12" s="18" t="inlineStr">
-        <is>
-          <t>수집예정</t>
-        </is>
+      <c r="H12" s="6" t="n">
+        <v>1087.58</v>
+      </c>
+      <c r="I12" s="6" t="n">
+        <v>1798</v>
       </c>
       <c r="J12" s="6" t="inlineStr">
         <is>
@@ -7180,40 +7168,36 @@
           <t>해당없음</t>
         </is>
       </c>
-      <c r="C14" s="19" t="inlineStr">
+      <c r="C14" s="6" t="inlineStr">
+        <is>
+          <t>2,000</t>
+        </is>
+      </c>
+      <c r="D14" s="7" t="inlineStr">
+        <is>
+          <t>6,500,000</t>
+        </is>
+      </c>
+      <c r="E14" s="7" t="inlineStr">
+        <is>
+          <t>13,000</t>
+        </is>
+      </c>
+      <c r="F14" s="19" t="inlineStr">
         <is>
           <t>해당없음</t>
         </is>
       </c>
-      <c r="D14" s="7" t="inlineStr">
-        <is>
-          <t>6,500,000</t>
-        </is>
-      </c>
-      <c r="E14" s="7" t="inlineStr">
-        <is>
-          <t>13,000</t>
-        </is>
-      </c>
-      <c r="F14" s="19" t="inlineStr">
-        <is>
-          <t>해당없음</t>
-        </is>
-      </c>
       <c r="G14" s="6" t="inlineStr">
         <is>
           <t>2,000</t>
         </is>
       </c>
-      <c r="H14" s="18" t="inlineStr">
-        <is>
-          <t>수집예정</t>
-        </is>
-      </c>
-      <c r="I14" s="18" t="inlineStr">
-        <is>
-          <t>수집예정</t>
-        </is>
+      <c r="H14" s="6" t="n">
+        <v>1327.13</v>
+      </c>
+      <c r="I14" s="6" t="n">
+        <v>2194</v>
       </c>
       <c r="J14" s="6" t="inlineStr">
         <is>
@@ -7502,40 +7486,36 @@
           <t>해당없음</t>
         </is>
       </c>
-      <c r="C18" s="19" t="inlineStr">
+      <c r="C18" s="6" t="inlineStr">
+        <is>
+          <t>2,000</t>
+        </is>
+      </c>
+      <c r="D18" s="7" t="inlineStr">
+        <is>
+          <t>5,000,000</t>
+        </is>
+      </c>
+      <c r="E18" s="7" t="inlineStr">
+        <is>
+          <t>10,000</t>
+        </is>
+      </c>
+      <c r="F18" s="19" t="inlineStr">
         <is>
           <t>해당없음</t>
         </is>
       </c>
-      <c r="D18" s="7" t="inlineStr">
-        <is>
-          <t>5,000,000</t>
-        </is>
-      </c>
-      <c r="E18" s="7" t="inlineStr">
-        <is>
-          <t>10,000</t>
-        </is>
-      </c>
-      <c r="F18" s="19" t="inlineStr">
-        <is>
-          <t>해당없음</t>
-        </is>
-      </c>
       <c r="G18" s="6" t="inlineStr">
         <is>
           <t>2,000</t>
         </is>
       </c>
-      <c r="H18" s="18" t="inlineStr">
-        <is>
-          <t>수집예정</t>
-        </is>
-      </c>
-      <c r="I18" s="18" t="inlineStr">
-        <is>
-          <t>수집예정</t>
-        </is>
+      <c r="H18" s="6" t="n">
+        <v>1388.6</v>
+      </c>
+      <c r="I18" s="6" t="n">
+        <v>2044</v>
       </c>
       <c r="J18" s="6" t="inlineStr">
         <is>
@@ -7668,40 +7648,36 @@
           <t>해당없음</t>
         </is>
       </c>
-      <c r="C20" s="19" t="inlineStr">
+      <c r="C20" s="6" t="inlineStr">
+        <is>
+          <t>2,000</t>
+        </is>
+      </c>
+      <c r="D20" s="7" t="inlineStr">
+        <is>
+          <t>6,000,000</t>
+        </is>
+      </c>
+      <c r="E20" s="7" t="inlineStr">
+        <is>
+          <t>12,000</t>
+        </is>
+      </c>
+      <c r="F20" s="19" t="inlineStr">
         <is>
           <t>해당없음</t>
         </is>
       </c>
-      <c r="D20" s="7" t="inlineStr">
-        <is>
-          <t>6,000,000</t>
-        </is>
-      </c>
-      <c r="E20" s="7" t="inlineStr">
-        <is>
-          <t>12,000</t>
-        </is>
-      </c>
-      <c r="F20" s="19" t="inlineStr">
-        <is>
-          <t>해당없음</t>
-        </is>
-      </c>
       <c r="G20" s="6" t="inlineStr">
         <is>
           <t>2,000</t>
         </is>
       </c>
-      <c r="H20" s="18" t="inlineStr">
-        <is>
-          <t>수집예정</t>
-        </is>
-      </c>
-      <c r="I20" s="18" t="inlineStr">
-        <is>
-          <t>수집예정</t>
-        </is>
+      <c r="H20" s="6" t="n">
+        <v>1271.12</v>
+      </c>
+      <c r="I20" s="6" t="n">
+        <v>2054</v>
       </c>
       <c r="J20" s="6" t="inlineStr">
         <is>
@@ -7752,40 +7728,36 @@
           <t>해당없음</t>
         </is>
       </c>
-      <c r="C21" s="19" t="inlineStr">
+      <c r="C21" s="6" t="inlineStr">
+        <is>
+          <t>2,000</t>
+        </is>
+      </c>
+      <c r="D21" s="7" t="inlineStr">
+        <is>
+          <t>5,400,000</t>
+        </is>
+      </c>
+      <c r="E21" s="7" t="inlineStr">
+        <is>
+          <t>10,800</t>
+        </is>
+      </c>
+      <c r="F21" s="19" t="inlineStr">
         <is>
           <t>해당없음</t>
         </is>
       </c>
-      <c r="D21" s="7" t="inlineStr">
-        <is>
-          <t>5,400,000</t>
-        </is>
-      </c>
-      <c r="E21" s="7" t="inlineStr">
-        <is>
-          <t>10,800</t>
-        </is>
-      </c>
-      <c r="F21" s="19" t="inlineStr">
-        <is>
-          <t>해당없음</t>
-        </is>
-      </c>
       <c r="G21" s="6" t="inlineStr">
         <is>
           <t>2,000</t>
         </is>
       </c>
-      <c r="H21" s="18" t="inlineStr">
-        <is>
-          <t>수집예정</t>
-        </is>
-      </c>
-      <c r="I21" s="18" t="inlineStr">
-        <is>
-          <t>수집예정</t>
-        </is>
+      <c r="H21" s="6" t="n">
+        <v>1196.99</v>
+      </c>
+      <c r="I21" s="6" t="n">
+        <v>1855</v>
       </c>
       <c r="J21" s="6" t="inlineStr">
         <is>
@@ -7914,40 +7886,36 @@
           <t>해당없음</t>
         </is>
       </c>
-      <c r="C23" s="19" t="inlineStr">
+      <c r="C23" s="6" t="inlineStr">
+        <is>
+          <t>2,000</t>
+        </is>
+      </c>
+      <c r="D23" s="7" t="inlineStr">
+        <is>
+          <t>5,000,000</t>
+        </is>
+      </c>
+      <c r="E23" s="7" t="inlineStr">
+        <is>
+          <t>10,000</t>
+        </is>
+      </c>
+      <c r="F23" s="19" t="inlineStr">
         <is>
           <t>해당없음</t>
         </is>
       </c>
-      <c r="D23" s="7" t="inlineStr">
-        <is>
-          <t>5,000,000</t>
-        </is>
-      </c>
-      <c r="E23" s="7" t="inlineStr">
-        <is>
-          <t>10,000</t>
-        </is>
-      </c>
-      <c r="F23" s="19" t="inlineStr">
-        <is>
-          <t>해당없음</t>
-        </is>
-      </c>
       <c r="G23" s="6" t="inlineStr">
         <is>
           <t>2,000</t>
         </is>
       </c>
-      <c r="H23" s="18" t="inlineStr">
-        <is>
-          <t>수집예정</t>
-        </is>
-      </c>
-      <c r="I23" s="18" t="inlineStr">
-        <is>
-          <t>수집예정</t>
-        </is>
+      <c r="H23" s="6" t="n">
+        <v>1343.8</v>
+      </c>
+      <c r="I23" s="6" t="n">
+        <v>2022</v>
       </c>
       <c r="J23" s="6" t="inlineStr">
         <is>
@@ -8080,40 +8048,36 @@
           <t>해당없음</t>
         </is>
       </c>
-      <c r="C25" s="19" t="inlineStr">
+      <c r="C25" s="6" t="inlineStr">
+        <is>
+          <t>2,000</t>
+        </is>
+      </c>
+      <c r="D25" s="7" t="inlineStr">
+        <is>
+          <t>6,350,000</t>
+        </is>
+      </c>
+      <c r="E25" s="7" t="inlineStr">
+        <is>
+          <t>12,700</t>
+        </is>
+      </c>
+      <c r="F25" s="19" t="inlineStr">
         <is>
           <t>해당없음</t>
         </is>
       </c>
-      <c r="D25" s="7" t="inlineStr">
-        <is>
-          <t>6,350,000</t>
-        </is>
-      </c>
-      <c r="E25" s="7" t="inlineStr">
-        <is>
-          <t>12,700</t>
-        </is>
-      </c>
-      <c r="F25" s="19" t="inlineStr">
-        <is>
-          <t>해당없음</t>
-        </is>
-      </c>
       <c r="G25" s="6" t="inlineStr">
         <is>
           <t>2,000</t>
         </is>
       </c>
-      <c r="H25" s="18" t="inlineStr">
-        <is>
-          <t>수집예정</t>
-        </is>
-      </c>
-      <c r="I25" s="18" t="inlineStr">
-        <is>
-          <t>수집예정</t>
-        </is>
+      <c r="H25" s="6" t="n">
+        <v>1228.71</v>
+      </c>
+      <c r="I25" s="6" t="n">
+        <v>2058</v>
       </c>
       <c r="J25" s="6" t="inlineStr">
         <is>
@@ -8964,40 +8928,36 @@
           <t>해당없음</t>
         </is>
       </c>
-      <c r="C36" s="19" t="inlineStr">
+      <c r="C36" s="6" t="inlineStr">
+        <is>
+          <t>2,000</t>
+        </is>
+      </c>
+      <c r="D36" s="7" t="inlineStr">
+        <is>
+          <t>6,000,000</t>
+        </is>
+      </c>
+      <c r="E36" s="7" t="inlineStr">
+        <is>
+          <t>12,000</t>
+        </is>
+      </c>
+      <c r="F36" s="19" t="inlineStr">
         <is>
           <t>해당없음</t>
         </is>
       </c>
-      <c r="D36" s="7" t="inlineStr">
-        <is>
-          <t>6,000,000</t>
-        </is>
-      </c>
-      <c r="E36" s="7" t="inlineStr">
-        <is>
-          <t>12,000</t>
-        </is>
-      </c>
-      <c r="F36" s="19" t="inlineStr">
-        <is>
-          <t>해당없음</t>
-        </is>
-      </c>
       <c r="G36" s="6" t="inlineStr">
         <is>
           <t>2,000</t>
         </is>
       </c>
-      <c r="H36" s="18" t="inlineStr">
-        <is>
-          <t>수집예정</t>
-        </is>
-      </c>
-      <c r="I36" s="18" t="inlineStr">
-        <is>
-          <t>수집예정</t>
-        </is>
+      <c r="H36" s="6" t="n">
+        <v>1159.11</v>
+      </c>
+      <c r="I36" s="6" t="n">
+        <v>1892</v>
       </c>
       <c r="J36" s="6" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
chore: update IPO data 2026-07-10
</commit_message>
<xml_diff>
--- a/IPO_analysis.xlsx
+++ b/IPO_analysis.xlsx
@@ -618,7 +618,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>기준일 2026-07-09 · 청구일 직전 사업연도 · 별도/개별 재무제표 · 단위 백만원(별도 표기 시 USD)</t>
+          <t>기준일 2026-07-10 · 청구일 직전 사업연도 · 별도/개별 재무제표 · 단위 백만원(별도 표기 시 USD)</t>
         </is>
       </c>
     </row>
@@ -9138,7 +9138,7 @@
       </c>
       <c r="G40" s="6" t="inlineStr">
         <is>
-          <t>18,500</t>
+          <t>21,500</t>
         </is>
       </c>
       <c r="H40" s="6" t="inlineStr"/>
@@ -9177,7 +9177,7 @@
       </c>
       <c r="R40" s="6" t="inlineStr">
         <is>
-          <t>정정</t>
+          <t>발행조건확정</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore: update IPO data 2026-07-11
</commit_message>
<xml_diff>
--- a/IPO_analysis.xlsx
+++ b/IPO_analysis.xlsx
@@ -618,7 +618,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>기준일 2026-07-10 · 청구일 직전 사업연도 · 별도/개별 재무제표 · 단위 백만원(별도 표기 시 USD)</t>
+          <t>기준일 2026-07-11 · 청구일 직전 사업연도 · 별도/개별 재무제표 · 단위 백만원(별도 표기 시 USD)</t>
         </is>
       </c>
     </row>
@@ -4284,7 +4284,7 @@
       </c>
       <c r="K70" s="6" t="inlineStr">
         <is>
-          <t>상장완료</t>
+          <t>상장승인(상장예정)</t>
         </is>
       </c>
     </row>
@@ -5034,7 +5034,7 @@
       </c>
       <c r="K84" s="6" t="inlineStr">
         <is>
-          <t>상장완료</t>
+          <t>상장승인(상장예정)</t>
         </is>
       </c>
     </row>
@@ -5132,7 +5132,7 @@
       </c>
       <c r="K86" s="6" t="inlineStr">
         <is>
-          <t>상장완료</t>
+          <t>상장승인(상장예정)</t>
         </is>
       </c>
     </row>
@@ -9185,7 +9185,7 @@
       </c>
       <c r="E40" s="7" t="inlineStr">
         <is>
-          <t>47,452,500,000</t>
+          <t>55,147,500,000</t>
         </is>
       </c>
       <c r="F40" s="6" t="inlineStr">
@@ -9333,11 +9333,7 @@
           <t>47.97배 (PER)</t>
         </is>
       </c>
-      <c r="G42" s="6" t="inlineStr">
-        <is>
-          <t>9,000</t>
-        </is>
-      </c>
+      <c r="G42" s="6" t="inlineStr"/>
       <c r="H42" s="6" t="inlineStr"/>
       <c r="I42" s="6" t="inlineStr"/>
       <c r="J42" s="6" t="inlineStr">
@@ -9388,12 +9384,12 @@
       </c>
       <c r="D43" s="7" t="inlineStr">
         <is>
-          <t>2,000,000</t>
+          <t>100</t>
         </is>
       </c>
       <c r="E43" s="7" t="inlineStr">
         <is>
-          <t>40,000,000,000</t>
+          <t>500</t>
         </is>
       </c>
       <c r="F43" s="6" t="inlineStr">
@@ -9456,12 +9452,12 @@
       </c>
       <c r="D44" s="7" t="inlineStr">
         <is>
-          <t>2,200,000</t>
+          <t>109,200</t>
         </is>
       </c>
       <c r="E44" s="7" t="inlineStr">
         <is>
-          <t>11,000,000,000</t>
+          <t>5,248,620</t>
         </is>
       </c>
       <c r="F44" s="6" t="inlineStr">
@@ -9520,12 +9516,12 @@
       </c>
       <c r="D45" s="7" t="inlineStr">
         <is>
-          <t>910,000</t>
+          <t>1,216,410</t>
         </is>
       </c>
       <c r="E45" s="7" t="inlineStr">
         <is>
-          <t>27,300,000,000</t>
+          <t>776,880</t>
         </is>
       </c>
       <c r="F45" s="6" t="inlineStr">
@@ -9712,12 +9708,12 @@
       </c>
       <c r="D48" s="7" t="inlineStr">
         <is>
-          <t>2,000,000</t>
+          <t>23,252</t>
         </is>
       </c>
       <c r="E48" s="7" t="inlineStr">
         <is>
-          <t>26,000,000,000</t>
+          <t>253,238</t>
         </is>
       </c>
       <c r="F48" s="6" t="inlineStr">
@@ -10340,7 +10336,7 @@
       </c>
       <c r="C17" s="6" t="inlineStr">
         <is>
-          <t>47,452,739,540</t>
+          <t>55,147,739,540</t>
         </is>
       </c>
     </row>
@@ -10362,105 +10358,105 @@
     <row r="19">
       <c r="A19" s="6" t="inlineStr">
         <is>
-          <t>유진</t>
+          <t>DB</t>
         </is>
       </c>
       <c r="B19" s="6" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C19" s="6" t="inlineStr">
         <is>
-          <t>40,000,025,020</t>
+          <t>23,000,000,000</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="6" t="inlineStr">
         <is>
-          <t>한국</t>
+          <t>IBK</t>
         </is>
       </c>
       <c r="B20" s="6" t="n">
-        <v>8</v>
+        <v>2</v>
       </c>
       <c r="C20" s="6" t="inlineStr">
         <is>
-          <t>37,000,154,600</t>
+          <t>21,600,000,000</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="6" t="inlineStr">
         <is>
-          <t>삼성</t>
+          <t>한국</t>
         </is>
       </c>
       <c r="B21" s="6" t="n">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="C21" s="6" t="inlineStr">
         <is>
-          <t>27,300,092,000</t>
+          <t>5,656,458</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="6" t="inlineStr">
         <is>
-          <t>DB</t>
+          <t>삼성</t>
         </is>
       </c>
       <c r="B22" s="6" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="C22" s="6" t="inlineStr">
         <is>
-          <t>23,000,000,000</t>
+          <t>868,880</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="6" t="inlineStr">
         <is>
-          <t>IBK</t>
+          <t>NH</t>
         </is>
       </c>
       <c r="B23" s="6" t="n">
-        <v>2</v>
+        <v>7</v>
       </c>
       <c r="C23" s="6" t="inlineStr">
         <is>
-          <t>21,600,000,000</t>
+          <t>618,288</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="6" t="inlineStr">
         <is>
-          <t>NH</t>
+          <t>신한</t>
         </is>
       </c>
       <c r="B24" s="6" t="n">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="C24" s="6" t="inlineStr">
         <is>
-          <t>618,288</t>
+          <t>49,052</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="6" t="inlineStr">
         <is>
-          <t>신한</t>
+          <t>유진</t>
         </is>
       </c>
       <c r="B25" s="6" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="C25" s="6" t="inlineStr">
         <is>
-          <t>49,052</t>
+          <t>25,520</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore: update IPO data 2026-07-14
</commit_message>
<xml_diff>
--- a/IPO_analysis.xlsx
+++ b/IPO_analysis.xlsx
@@ -618,7 +618,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>기준일 2026-07-13 · 청구일 직전 사업연도 · 별도/개별 재무제표 · 단위 백만원(별도 표기 시 USD)</t>
+          <t>기준일 2026-07-14 · 청구일 직전 사업연도 · 별도/개별 재무제표 · 단위 백만원(별도 표기 시 USD)</t>
         </is>
       </c>
     </row>
@@ -9411,32 +9411,32 @@
     <row r="42" ht="30" customHeight="1">
       <c r="A42" s="6" t="inlineStr">
         <is>
-          <t>케이앤에스아이앤씨</t>
+          <t>딜리셔스</t>
         </is>
       </c>
       <c r="B42" s="6" t="inlineStr">
         <is>
-          <t>07-27~07-31</t>
+          <t>07-23~07-29</t>
         </is>
       </c>
       <c r="C42" s="6" t="inlineStr">
         <is>
-          <t>9,000~11,000</t>
+          <t>5,000~7,000</t>
         </is>
       </c>
       <c r="D42" s="7" t="inlineStr">
         <is>
-          <t>2,400,000</t>
+          <t>2,200,000</t>
         </is>
       </c>
       <c r="E42" s="7" t="inlineStr">
         <is>
-          <t>21,600,000,000</t>
+          <t>11,000,000,000</t>
         </is>
       </c>
       <c r="F42" s="6" t="inlineStr">
         <is>
-          <t>47.97배 (PER)</t>
+          <t>23.93배 (PER)</t>
         </is>
       </c>
       <c r="G42" s="6" t="inlineStr"/>
@@ -9444,7 +9444,7 @@
       <c r="I42" s="6" t="inlineStr"/>
       <c r="J42" s="6" t="inlineStr">
         <is>
-          <t>08-04~08-05</t>
+          <t>08-03~08-04</t>
         </is>
       </c>
       <c r="K42" s="6" t="inlineStr"/>
@@ -9452,18 +9452,18 @@
       <c r="M42" s="6" t="inlineStr"/>
       <c r="N42" s="6" t="inlineStr">
         <is>
-          <t>아이비케이투자증권</t>
+          <t>한국투자증권</t>
         </is>
       </c>
       <c r="O42" s="6" t="inlineStr"/>
       <c r="P42" s="7" t="inlineStr">
         <is>
-          <t>1,500,000,000</t>
+          <t>566,500,000</t>
         </is>
       </c>
       <c r="Q42" s="6" t="inlineStr">
         <is>
-          <t>3.5%</t>
+          <t>5.0%</t>
         </is>
       </c>
       <c r="R42" s="6" t="inlineStr">
@@ -9475,7 +9475,7 @@
     <row r="43" ht="30" customHeight="1">
       <c r="A43" s="6" t="inlineStr">
         <is>
-          <t>빅웨이브로보틱스</t>
+          <t>케이앤에스아이앤씨</t>
         </is>
       </c>
       <c r="B43" s="6" t="inlineStr">
@@ -9485,22 +9485,22 @@
       </c>
       <c r="C43" s="6" t="inlineStr">
         <is>
-          <t>20,000~24,000</t>
+          <t>9,000~11,000</t>
         </is>
       </c>
       <c r="D43" s="7" t="inlineStr">
         <is>
-          <t>2,000,000</t>
+          <t>2,400,000</t>
         </is>
       </c>
       <c r="E43" s="7" t="inlineStr">
         <is>
-          <t>40,000,000,000</t>
+          <t>21,600,000,000</t>
         </is>
       </c>
       <c r="F43" s="6" t="inlineStr">
         <is>
-          <t>16.19 (PSR)</t>
+          <t>47.97배 (PER)</t>
         </is>
       </c>
       <c r="G43" s="6" t="inlineStr"/>
@@ -9508,7 +9508,7 @@
       <c r="I43" s="6" t="inlineStr"/>
       <c r="J43" s="6" t="inlineStr">
         <is>
-          <t>08-05~08-06</t>
+          <t>08-04~08-05</t>
         </is>
       </c>
       <c r="K43" s="6" t="inlineStr"/>
@@ -9516,22 +9516,18 @@
       <c r="M43" s="6" t="inlineStr"/>
       <c r="N43" s="6" t="inlineStr">
         <is>
-          <t>유진투자증권</t>
-        </is>
-      </c>
-      <c r="O43" s="6" t="inlineStr">
-        <is>
-          <t>미래</t>
-        </is>
-      </c>
+          <t>아이비케이투자증권</t>
+        </is>
+      </c>
+      <c r="O43" s="6" t="inlineStr"/>
       <c r="P43" s="7" t="inlineStr">
         <is>
-          <t>627,300,000</t>
+          <t>1,500,000,000</t>
         </is>
       </c>
       <c r="Q43" s="6" t="inlineStr">
         <is>
-          <t>3.0%</t>
+          <t>3.5%</t>
         </is>
       </c>
       <c r="R43" s="6" t="inlineStr">
@@ -9543,32 +9539,32 @@
     <row r="44" ht="30" customHeight="1">
       <c r="A44" s="6" t="inlineStr">
         <is>
-          <t>딜리셔스</t>
+          <t>빅웨이브로보틱스</t>
         </is>
       </c>
       <c r="B44" s="6" t="inlineStr">
         <is>
-          <t>07-23~07-29</t>
+          <t>07-27~07-31</t>
         </is>
       </c>
       <c r="C44" s="6" t="inlineStr">
         <is>
-          <t>5,000~7,000</t>
+          <t>20,000~24,000</t>
         </is>
       </c>
       <c r="D44" s="7" t="inlineStr">
         <is>
-          <t>2,200,000</t>
+          <t>2,000,000</t>
         </is>
       </c>
       <c r="E44" s="7" t="inlineStr">
         <is>
-          <t>11,000,000,000</t>
+          <t>40,000,000,000</t>
         </is>
       </c>
       <c r="F44" s="6" t="inlineStr">
         <is>
-          <t>23.93배 (PER)</t>
+          <t>16.19 (PSR)</t>
         </is>
       </c>
       <c r="G44" s="6" t="inlineStr"/>
@@ -9576,7 +9572,7 @@
       <c r="I44" s="6" t="inlineStr"/>
       <c r="J44" s="6" t="inlineStr">
         <is>
-          <t>08-03~08-04</t>
+          <t>08-05~08-06</t>
         </is>
       </c>
       <c r="K44" s="6" t="inlineStr"/>
@@ -9584,55 +9580,59 @@
       <c r="M44" s="6" t="inlineStr"/>
       <c r="N44" s="6" t="inlineStr">
         <is>
-          <t>한국투자증권</t>
-        </is>
-      </c>
-      <c r="O44" s="6" t="inlineStr"/>
+          <t>유진투자증권</t>
+        </is>
+      </c>
+      <c r="O44" s="6" t="inlineStr">
+        <is>
+          <t>미래</t>
+        </is>
+      </c>
       <c r="P44" s="7" t="inlineStr">
         <is>
-          <t>566,500,000</t>
+          <t>627,300,000</t>
         </is>
       </c>
       <c r="Q44" s="6" t="inlineStr">
         <is>
-          <t>5.0%</t>
+          <t>3.0%</t>
         </is>
       </c>
       <c r="R44" s="6" t="inlineStr">
         <is>
-          <t>최초</t>
+          <t>정정</t>
         </is>
       </c>
     </row>
     <row r="45" ht="30" customHeight="1">
       <c r="A45" s="6" t="inlineStr">
         <is>
-          <t>니어스랩</t>
+          <t>기도산업</t>
         </is>
       </c>
       <c r="B45" s="6" t="inlineStr">
         <is>
-          <t>07-27~07-31</t>
+          <t>07-31~08-06</t>
         </is>
       </c>
       <c r="C45" s="6" t="inlineStr">
         <is>
-          <t>30,000~41,200</t>
+          <t>24,800~28,400</t>
         </is>
       </c>
       <c r="D45" s="7" t="inlineStr">
         <is>
-          <t>910,000</t>
+          <t>1,700,000</t>
         </is>
       </c>
       <c r="E45" s="7" t="inlineStr">
         <is>
-          <t>27,300,000,000</t>
+          <t>42,160,000,000</t>
         </is>
       </c>
       <c r="F45" s="6" t="inlineStr">
         <is>
-          <t>47.56배 (PER)</t>
+          <t>10.01배 (PER)</t>
         </is>
       </c>
       <c r="G45" s="6" t="inlineStr"/>
@@ -9640,7 +9640,7 @@
       <c r="I45" s="6" t="inlineStr"/>
       <c r="J45" s="6" t="inlineStr">
         <is>
-          <t>08-05~08-06</t>
+          <t>08-11~08-12</t>
         </is>
       </c>
       <c r="K45" s="6" t="inlineStr"/>
@@ -9648,55 +9648,55 @@
       <c r="M45" s="6" t="inlineStr"/>
       <c r="N45" s="6" t="inlineStr">
         <is>
-          <t>삼성증권</t>
+          <t>미래에셋증권</t>
         </is>
       </c>
       <c r="O45" s="6" t="inlineStr"/>
       <c r="P45" s="7" t="inlineStr">
         <is>
-          <t>1,265,355,000</t>
+          <t>716,720,000</t>
         </is>
       </c>
       <c r="Q45" s="6" t="inlineStr">
         <is>
-          <t>4.50%</t>
+          <t>1.0%</t>
         </is>
       </c>
       <c r="R45" s="6" t="inlineStr">
         <is>
-          <t>최초</t>
+          <t>정정</t>
         </is>
       </c>
     </row>
     <row r="46" ht="30" customHeight="1">
       <c r="A46" s="6" t="inlineStr">
         <is>
-          <t>해치텍</t>
+          <t>니어스랩</t>
         </is>
       </c>
       <c r="B46" s="6" t="inlineStr">
         <is>
-          <t>07-29~08-04</t>
+          <t>08-03~08-07</t>
         </is>
       </c>
       <c r="C46" s="6" t="inlineStr">
         <is>
-          <t>23,000~28,000</t>
+          <t>30,000~41,200</t>
         </is>
       </c>
       <c r="D46" s="7" t="inlineStr">
         <is>
-          <t>1,000,000</t>
+          <t>910,000</t>
         </is>
       </c>
       <c r="E46" s="7" t="inlineStr">
         <is>
-          <t>23,000,000,000</t>
+          <t>27,300,000,000</t>
         </is>
       </c>
       <c r="F46" s="6" t="inlineStr">
         <is>
-          <t>36.99배 (PER)</t>
+          <t>47.56배 (PER)</t>
         </is>
       </c>
       <c r="G46" s="6" t="inlineStr"/>
@@ -9704,7 +9704,7 @@
       <c r="I46" s="6" t="inlineStr"/>
       <c r="J46" s="6" t="inlineStr">
         <is>
-          <t>08-06~08-07</t>
+          <t>08-12~08-13</t>
         </is>
       </c>
       <c r="K46" s="6" t="inlineStr"/>
@@ -9712,55 +9712,55 @@
       <c r="M46" s="6" t="inlineStr"/>
       <c r="N46" s="6" t="inlineStr">
         <is>
-          <t>DB증권</t>
+          <t>삼성증권</t>
         </is>
       </c>
       <c r="O46" s="6" t="inlineStr"/>
       <c r="P46" s="7" t="inlineStr">
         <is>
-          <t>1,302,950,000</t>
+          <t>1,265,355,000</t>
         </is>
       </c>
       <c r="Q46" s="6" t="inlineStr">
         <is>
-          <t>5.5%</t>
+          <t>4.50%</t>
         </is>
       </c>
       <c r="R46" s="6" t="inlineStr">
         <is>
-          <t>최초</t>
+          <t>정정</t>
         </is>
       </c>
     </row>
     <row r="47" ht="30" customHeight="1">
       <c r="A47" s="6" t="inlineStr">
         <is>
-          <t>기도산업</t>
+          <t>해치텍</t>
         </is>
       </c>
       <c r="B47" s="6" t="inlineStr">
         <is>
-          <t>07-31~08-06</t>
+          <t>07-29~08-04</t>
         </is>
       </c>
       <c r="C47" s="6" t="inlineStr">
         <is>
-          <t>24,800~28,400</t>
+          <t>23,000~28,000</t>
         </is>
       </c>
       <c r="D47" s="7" t="inlineStr">
         <is>
-          <t>1,7000,000</t>
+          <t>1,000,000</t>
         </is>
       </c>
       <c r="E47" s="7" t="inlineStr">
         <is>
-          <t>42,160,000,000</t>
+          <t>23,000,000,000</t>
         </is>
       </c>
       <c r="F47" s="6" t="inlineStr">
         <is>
-          <t>10.01배 (PER)</t>
+          <t>36.99배 (PER)</t>
         </is>
       </c>
       <c r="G47" s="6" t="inlineStr"/>
@@ -9768,7 +9768,7 @@
       <c r="I47" s="6" t="inlineStr"/>
       <c r="J47" s="6" t="inlineStr">
         <is>
-          <t>08-11~08-12</t>
+          <t>08-06~08-07</t>
         </is>
       </c>
       <c r="K47" s="6" t="inlineStr"/>
@@ -9776,18 +9776,18 @@
       <c r="M47" s="6" t="inlineStr"/>
       <c r="N47" s="6" t="inlineStr">
         <is>
-          <t>미래에셋증권</t>
+          <t>DB증권</t>
         </is>
       </c>
       <c r="O47" s="6" t="inlineStr"/>
       <c r="P47" s="7" t="inlineStr">
         <is>
-          <t>716,720,000</t>
+          <t>1,302,950,000</t>
         </is>
       </c>
       <c r="Q47" s="6" t="inlineStr">
         <is>
-          <t>1.0%</t>
+          <t>5.5%</t>
         </is>
       </c>
       <c r="R47" s="6" t="inlineStr">

</xml_diff>

<commit_message>
chore: update IPO data 2026-07-16
</commit_message>
<xml_diff>
--- a/IPO_analysis.xlsx
+++ b/IPO_analysis.xlsx
@@ -9340,7 +9340,7 @@
       </c>
       <c r="R40" s="6" t="inlineStr">
         <is>
-          <t>발행조건확정</t>
+          <t>청약완료·상장대기</t>
         </is>
       </c>
     </row>
@@ -9740,7 +9740,7 @@
       </c>
       <c r="B47" s="6" t="inlineStr">
         <is>
-          <t>07-29~08-04</t>
+          <t>08-03~08-07</t>
         </is>
       </c>
       <c r="C47" s="6" t="inlineStr">
@@ -9768,7 +9768,7 @@
       <c r="I47" s="6" t="inlineStr"/>
       <c r="J47" s="6" t="inlineStr">
         <is>
-          <t>08-06~08-07</t>
+          <t>08-12~08-13</t>
         </is>
       </c>
       <c r="K47" s="6" t="inlineStr"/>
@@ -9792,7 +9792,7 @@
       </c>
       <c r="R47" s="6" t="inlineStr">
         <is>
-          <t>최초</t>
+          <t>정정</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore: update IPO data 2026-07-20
</commit_message>
<xml_diff>
--- a/IPO_analysis.xlsx
+++ b/IPO_analysis.xlsx
@@ -592,7 +592,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K113"/>
+  <dimension ref="A1:K112"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -618,14 +618,14 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>기준일 2026-07-19 · 청구일 직전 사업연도 · 별도/개별 재무제표 · 단위 백만원(별도 표기 시 USD)</t>
+          <t>기준일 2026-07-20 · 청구일 직전 사업연도 · 별도/개별 재무제표 · 단위 백만원(별도 표기 시 USD)</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
-          <t>■ 심사 신청(진행중)  (51건)</t>
+          <t>■ 심사 신청(진행중)  (50건)</t>
         </is>
       </c>
       <c r="B4" s="4" t="n"/>
@@ -3081,12 +3081,12 @@
     <row r="48">
       <c r="A48" s="6" t="inlineStr">
         <is>
-          <t>2026-04-13</t>
+          <t>2026-04-10</t>
         </is>
       </c>
       <c r="B48" s="6" t="inlineStr">
         <is>
-          <t>글로벌테크놀로지</t>
+          <t>엠비디</t>
         </is>
       </c>
       <c r="C48" s="6" t="inlineStr">
@@ -3106,27 +3106,27 @@
       </c>
       <c r="F48" s="7" t="inlineStr">
         <is>
-          <t>29,689</t>
+          <t>1,524</t>
         </is>
       </c>
       <c r="G48" s="7" t="inlineStr">
         <is>
-          <t>-25,889</t>
+          <t>-2,125</t>
         </is>
       </c>
       <c r="H48" s="7" t="inlineStr">
         <is>
-          <t>6,402</t>
+          <t>2,753</t>
         </is>
       </c>
       <c r="I48" s="6" t="inlineStr">
         <is>
-          <t>반도체 제조업</t>
+          <t>물질 검사, 측정 및 분석기구 제조업</t>
         </is>
       </c>
       <c r="J48" s="6" t="inlineStr">
         <is>
-          <t>한국</t>
+          <t>하나</t>
         </is>
       </c>
       <c r="K48" s="6" t="inlineStr">
@@ -3138,12 +3138,12 @@
     <row r="49">
       <c r="A49" s="6" t="inlineStr">
         <is>
-          <t>2026-04-10</t>
+          <t>2026-04-08</t>
         </is>
       </c>
       <c r="B49" s="6" t="inlineStr">
         <is>
-          <t>엠비디</t>
+          <t>옵토닉스</t>
         </is>
       </c>
       <c r="C49" s="6" t="inlineStr">
@@ -3163,27 +3163,27 @@
       </c>
       <c r="F49" s="7" t="inlineStr">
         <is>
-          <t>1,524</t>
+          <t>25,368</t>
         </is>
       </c>
       <c r="G49" s="7" t="inlineStr">
         <is>
-          <t>-2,125</t>
+          <t>1,901</t>
         </is>
       </c>
       <c r="H49" s="7" t="inlineStr">
         <is>
-          <t>2,753</t>
+          <t>730</t>
         </is>
       </c>
       <c r="I49" s="6" t="inlineStr">
         <is>
-          <t>물질 검사, 측정 및 분석기구 제조업</t>
+          <t>광학렌즈 및 광학요소 제조업</t>
         </is>
       </c>
       <c r="J49" s="6" t="inlineStr">
         <is>
-          <t>하나</t>
+          <t>한국</t>
         </is>
       </c>
       <c r="K49" s="6" t="inlineStr">
@@ -3195,12 +3195,12 @@
     <row r="50">
       <c r="A50" s="6" t="inlineStr">
         <is>
-          <t>2026-04-08</t>
+          <t>2026-04-07</t>
         </is>
       </c>
       <c r="B50" s="6" t="inlineStr">
         <is>
-          <t>옵토닉스</t>
+          <t>크리에이츠</t>
         </is>
       </c>
       <c r="C50" s="6" t="inlineStr">
@@ -3220,27 +3220,27 @@
       </c>
       <c r="F50" s="7" t="inlineStr">
         <is>
-          <t>25,368</t>
+          <t>76,395</t>
         </is>
       </c>
       <c r="G50" s="7" t="inlineStr">
         <is>
-          <t>1,901</t>
+          <t>23,749</t>
         </is>
       </c>
       <c r="H50" s="7" t="inlineStr">
         <is>
-          <t>730</t>
+          <t>2,335</t>
         </is>
       </c>
       <c r="I50" s="6" t="inlineStr">
         <is>
-          <t>광학렌즈 및 광학요소 제조업</t>
+          <t>그외 기타 제품 제조업</t>
         </is>
       </c>
       <c r="J50" s="6" t="inlineStr">
         <is>
-          <t>한국</t>
+          <t>삼성</t>
         </is>
       </c>
       <c r="K50" s="6" t="inlineStr">
@@ -3252,12 +3252,12 @@
     <row r="51">
       <c r="A51" s="6" t="inlineStr">
         <is>
-          <t>2026-04-07</t>
+          <t>2026-03-24</t>
         </is>
       </c>
       <c r="B51" s="6" t="inlineStr">
         <is>
-          <t>크리에이츠</t>
+          <t>인텔리빅스</t>
         </is>
       </c>
       <c r="C51" s="6" t="inlineStr">
@@ -3277,27 +3277,27 @@
       </c>
       <c r="F51" s="7" t="inlineStr">
         <is>
-          <t>76,395</t>
+          <t>46,644</t>
         </is>
       </c>
       <c r="G51" s="7" t="inlineStr">
         <is>
-          <t>23,749</t>
+          <t>5,357</t>
         </is>
       </c>
       <c r="H51" s="7" t="inlineStr">
         <is>
-          <t>2,335</t>
+          <t>1,048</t>
         </is>
       </c>
       <c r="I51" s="6" t="inlineStr">
         <is>
-          <t>그외 기타 제품 제조업</t>
+          <t>소프트웨어 개발 및 공급업</t>
         </is>
       </c>
       <c r="J51" s="6" t="inlineStr">
         <is>
-          <t>삼성</t>
+          <t>미래</t>
         </is>
       </c>
       <c r="K51" s="6" t="inlineStr">
@@ -3309,12 +3309,12 @@
     <row r="52">
       <c r="A52" s="6" t="inlineStr">
         <is>
-          <t>2026-03-24</t>
+          <t>2026-02-27</t>
         </is>
       </c>
       <c r="B52" s="6" t="inlineStr">
         <is>
-          <t>인텔리빅스</t>
+          <t>피지티</t>
         </is>
       </c>
       <c r="C52" s="6" t="inlineStr">
@@ -3334,27 +3334,27 @@
       </c>
       <c r="F52" s="7" t="inlineStr">
         <is>
-          <t>46,644</t>
+          <t>40,141</t>
         </is>
       </c>
       <c r="G52" s="7" t="inlineStr">
         <is>
-          <t>5,357</t>
+          <t>-69,722</t>
         </is>
       </c>
       <c r="H52" s="7" t="inlineStr">
         <is>
-          <t>1,048</t>
+          <t>6,029</t>
         </is>
       </c>
       <c r="I52" s="6" t="inlineStr">
         <is>
-          <t>소프트웨어 개발 및 공급업</t>
+          <t>기타 화학제품 제조업</t>
         </is>
       </c>
       <c r="J52" s="6" t="inlineStr">
         <is>
-          <t>미래</t>
+          <t>한국</t>
         </is>
       </c>
       <c r="K52" s="6" t="inlineStr">
@@ -3366,12 +3366,12 @@
     <row r="53">
       <c r="A53" s="6" t="inlineStr">
         <is>
-          <t>2026-02-27</t>
+          <t>2025-11-11</t>
         </is>
       </c>
       <c r="B53" s="6" t="inlineStr">
         <is>
-          <t>피지티</t>
+          <t>덕산넵코어스</t>
         </is>
       </c>
       <c r="C53" s="6" t="inlineStr">
@@ -3386,32 +3386,32 @@
       </c>
       <c r="E53" s="6" t="inlineStr">
         <is>
-          <t>FY25</t>
+          <t>FY24</t>
         </is>
       </c>
       <c r="F53" s="7" t="inlineStr">
         <is>
-          <t>40,141</t>
+          <t>48,504</t>
         </is>
       </c>
       <c r="G53" s="7" t="inlineStr">
         <is>
-          <t>-69,722</t>
+          <t>3,668</t>
         </is>
       </c>
       <c r="H53" s="7" t="inlineStr">
         <is>
-          <t>6,029</t>
+          <t>8,448</t>
         </is>
       </c>
       <c r="I53" s="6" t="inlineStr">
         <is>
-          <t>기타 화학제품 제조업</t>
+          <t>항공기,우주선 및 부품 제조업</t>
         </is>
       </c>
       <c r="J53" s="6" t="inlineStr">
         <is>
-          <t>한국</t>
+          <t>대신</t>
         </is>
       </c>
       <c r="K53" s="6" t="inlineStr">
@@ -3423,12 +3423,12 @@
     <row r="54">
       <c r="A54" s="6" t="inlineStr">
         <is>
-          <t>2025-11-11</t>
+          <t>2025-09-18</t>
         </is>
       </c>
       <c r="B54" s="6" t="inlineStr">
         <is>
-          <t>덕산넵코어스</t>
+          <t>디티에스</t>
         </is>
       </c>
       <c r="C54" s="6" t="inlineStr">
@@ -3448,22 +3448,22 @@
       </c>
       <c r="F54" s="7" t="inlineStr">
         <is>
-          <t>48,504</t>
+          <t>142,718</t>
         </is>
       </c>
       <c r="G54" s="7" t="inlineStr">
         <is>
-          <t>3,668</t>
+          <t>18,765</t>
         </is>
       </c>
       <c r="H54" s="7" t="inlineStr">
         <is>
-          <t>8,448</t>
+          <t>63,153</t>
         </is>
       </c>
       <c r="I54" s="6" t="inlineStr">
         <is>
-          <t>항공기,우주선 및 부품 제조업</t>
+          <t>특수 목적용 기계 제조업</t>
         </is>
       </c>
       <c r="J54" s="6" t="inlineStr">
@@ -3480,12 +3480,12 @@
     <row r="55">
       <c r="A55" s="6" t="inlineStr">
         <is>
-          <t>2025-09-18</t>
+          <t>2025-09-11</t>
         </is>
       </c>
       <c r="B55" s="6" t="inlineStr">
         <is>
-          <t>디티에스</t>
+          <t>씨엠디엘</t>
         </is>
       </c>
       <c r="C55" s="6" t="inlineStr">
@@ -3495,173 +3495,173 @@
       </c>
       <c r="D55" s="6" t="inlineStr">
         <is>
+          <t>스팩 소멸합병</t>
+        </is>
+      </c>
+      <c r="E55" s="6" t="inlineStr">
+        <is>
+          <t>FY24</t>
+        </is>
+      </c>
+      <c r="F55" s="7" t="inlineStr">
+        <is>
+          <t>39,991</t>
+        </is>
+      </c>
+      <c r="G55" s="7" t="inlineStr">
+        <is>
+          <t>3,541</t>
+        </is>
+      </c>
+      <c r="H55" s="7" t="inlineStr">
+        <is>
+          <t>503</t>
+        </is>
+      </c>
+      <c r="I55" s="6" t="inlineStr">
+        <is>
+          <t>기타 기초 유기 화학물질 제조업</t>
+        </is>
+      </c>
+      <c r="J55" s="6" t="inlineStr">
+        <is>
+          <t>교보</t>
+        </is>
+      </c>
+      <c r="K55" s="6" t="inlineStr">
+        <is>
+          <t>예심 진행중</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="3" t="inlineStr">
+        <is>
+          <t>■ 심사 승인  (36건)</t>
+        </is>
+      </c>
+      <c r="B57" s="4" t="n"/>
+      <c r="C57" s="4" t="n"/>
+      <c r="D57" s="4" t="n"/>
+      <c r="E57" s="4" t="n"/>
+      <c r="F57" s="4" t="n"/>
+      <c r="G57" s="4" t="n"/>
+      <c r="H57" s="4" t="n"/>
+      <c r="I57" s="4" t="n"/>
+      <c r="J57" s="4" t="n"/>
+      <c r="K57" s="4" t="n"/>
+    </row>
+    <row r="58">
+      <c r="A58" s="5" t="inlineStr">
+        <is>
+          <t>일자</t>
+        </is>
+      </c>
+      <c r="B58" s="5" t="inlineStr">
+        <is>
+          <t>회사명</t>
+        </is>
+      </c>
+      <c r="C58" s="5" t="inlineStr">
+        <is>
+          <t>시장</t>
+        </is>
+      </c>
+      <c r="D58" s="5" t="inlineStr">
+        <is>
+          <t>상장유형</t>
+        </is>
+      </c>
+      <c r="E58" s="5" t="inlineStr">
+        <is>
+          <t>기준연도</t>
+        </is>
+      </c>
+      <c r="F58" s="5" t="inlineStr">
+        <is>
+          <t>매출액</t>
+        </is>
+      </c>
+      <c r="G58" s="5" t="inlineStr">
+        <is>
+          <t>순이익</t>
+        </is>
+      </c>
+      <c r="H58" s="5" t="inlineStr">
+        <is>
+          <t>자기자본</t>
+        </is>
+      </c>
+      <c r="I58" s="5" t="inlineStr">
+        <is>
+          <t>업종</t>
+        </is>
+      </c>
+      <c r="J58" s="5" t="inlineStr">
+        <is>
+          <t>대표주관사</t>
+        </is>
+      </c>
+      <c r="K58" s="5" t="inlineStr">
+        <is>
+          <t>현황</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="6" t="inlineStr">
+        <is>
+          <t>2026-07-10</t>
+        </is>
+      </c>
+      <c r="B59" s="6" t="inlineStr">
+        <is>
+          <t>네오사피엔스</t>
+        </is>
+      </c>
+      <c r="C59" s="6" t="inlineStr">
+        <is>
+          <t>코스닥</t>
+        </is>
+      </c>
+      <c r="D59" s="6" t="inlineStr">
+        <is>
           <t>신규상장</t>
         </is>
       </c>
-      <c r="E55" s="6" t="inlineStr">
-        <is>
-          <t>FY24</t>
-        </is>
-      </c>
-      <c r="F55" s="7" t="inlineStr">
-        <is>
-          <t>142,718</t>
-        </is>
-      </c>
-      <c r="G55" s="7" t="inlineStr">
-        <is>
-          <t>18,765</t>
-        </is>
-      </c>
-      <c r="H55" s="7" t="inlineStr">
-        <is>
-          <t>63,153</t>
-        </is>
-      </c>
-      <c r="I55" s="6" t="inlineStr">
-        <is>
-          <t>특수 목적용 기계 제조업</t>
-        </is>
-      </c>
-      <c r="J55" s="6" t="inlineStr">
+      <c r="E59" s="6" t="inlineStr">
+        <is>
+          <t>FY25</t>
+        </is>
+      </c>
+      <c r="F59" s="7" t="inlineStr">
+        <is>
+          <t>10,649</t>
+        </is>
+      </c>
+      <c r="G59" s="7" t="inlineStr">
+        <is>
+          <t>-6,994</t>
+        </is>
+      </c>
+      <c r="H59" s="7" t="inlineStr">
+        <is>
+          <t>-39,962</t>
+        </is>
+      </c>
+      <c r="I59" s="6" t="inlineStr">
+        <is>
+          <t>소프트웨어 개발 및 공급업</t>
+        </is>
+      </c>
+      <c r="J59" s="6" t="inlineStr">
         <is>
           <t>대신</t>
         </is>
       </c>
-      <c r="K55" s="6" t="inlineStr">
-        <is>
-          <t>예심 진행중</t>
-        </is>
-      </c>
-    </row>
-    <row r="56">
-      <c r="A56" s="6" t="inlineStr">
-        <is>
-          <t>2025-09-11</t>
-        </is>
-      </c>
-      <c r="B56" s="6" t="inlineStr">
-        <is>
-          <t>씨엠디엘</t>
-        </is>
-      </c>
-      <c r="C56" s="6" t="inlineStr">
-        <is>
-          <t>코스닥</t>
-        </is>
-      </c>
-      <c r="D56" s="6" t="inlineStr">
-        <is>
-          <t>스팩 소멸합병</t>
-        </is>
-      </c>
-      <c r="E56" s="6" t="inlineStr">
-        <is>
-          <t>FY24</t>
-        </is>
-      </c>
-      <c r="F56" s="7" t="inlineStr">
-        <is>
-          <t>39,991</t>
-        </is>
-      </c>
-      <c r="G56" s="7" t="inlineStr">
-        <is>
-          <t>3,541</t>
-        </is>
-      </c>
-      <c r="H56" s="7" t="inlineStr">
-        <is>
-          <t>503</t>
-        </is>
-      </c>
-      <c r="I56" s="6" t="inlineStr">
-        <is>
-          <t>기타 기초 유기 화학물질 제조업</t>
-        </is>
-      </c>
-      <c r="J56" s="6" t="inlineStr">
-        <is>
-          <t>교보</t>
-        </is>
-      </c>
-      <c r="K56" s="6" t="inlineStr">
-        <is>
-          <t>예심 진행중</t>
-        </is>
-      </c>
-    </row>
-    <row r="58">
-      <c r="A58" s="3" t="inlineStr">
-        <is>
-          <t>■ 심사 승인  (36건)</t>
-        </is>
-      </c>
-      <c r="B58" s="4" t="n"/>
-      <c r="C58" s="4" t="n"/>
-      <c r="D58" s="4" t="n"/>
-      <c r="E58" s="4" t="n"/>
-      <c r="F58" s="4" t="n"/>
-      <c r="G58" s="4" t="n"/>
-      <c r="H58" s="4" t="n"/>
-      <c r="I58" s="4" t="n"/>
-      <c r="J58" s="4" t="n"/>
-      <c r="K58" s="4" t="n"/>
-    </row>
-    <row r="59">
-      <c r="A59" s="5" t="inlineStr">
-        <is>
-          <t>일자</t>
-        </is>
-      </c>
-      <c r="B59" s="5" t="inlineStr">
-        <is>
-          <t>회사명</t>
-        </is>
-      </c>
-      <c r="C59" s="5" t="inlineStr">
-        <is>
-          <t>시장</t>
-        </is>
-      </c>
-      <c r="D59" s="5" t="inlineStr">
-        <is>
-          <t>상장유형</t>
-        </is>
-      </c>
-      <c r="E59" s="5" t="inlineStr">
-        <is>
-          <t>기준연도</t>
-        </is>
-      </c>
-      <c r="F59" s="5" t="inlineStr">
-        <is>
-          <t>매출액</t>
-        </is>
-      </c>
-      <c r="G59" s="5" t="inlineStr">
-        <is>
-          <t>순이익</t>
-        </is>
-      </c>
-      <c r="H59" s="5" t="inlineStr">
-        <is>
-          <t>자기자본</t>
-        </is>
-      </c>
-      <c r="I59" s="5" t="inlineStr">
-        <is>
-          <t>업종</t>
-        </is>
-      </c>
-      <c r="J59" s="5" t="inlineStr">
-        <is>
-          <t>대표주관사</t>
-        </is>
-      </c>
-      <c r="K59" s="5" t="inlineStr">
-        <is>
-          <t>현황</t>
+      <c r="K59" s="6" t="inlineStr">
+        <is>
+          <t>상장전</t>
         </is>
       </c>
     </row>
@@ -3673,7 +3673,7 @@
       </c>
       <c r="B60" s="6" t="inlineStr">
         <is>
-          <t>네오사피엔스</t>
+          <t>엠에스바이오</t>
         </is>
       </c>
       <c r="C60" s="6" t="inlineStr">
@@ -3693,27 +3693,27 @@
       </c>
       <c r="F60" s="7" t="inlineStr">
         <is>
-          <t>10,649</t>
+          <t>23,787</t>
         </is>
       </c>
       <c r="G60" s="7" t="inlineStr">
         <is>
-          <t>-6,994</t>
+          <t>7,288</t>
         </is>
       </c>
       <c r="H60" s="7" t="inlineStr">
         <is>
-          <t>-39,962</t>
+          <t>1,942</t>
         </is>
       </c>
       <c r="I60" s="6" t="inlineStr">
         <is>
-          <t>소프트웨어 개발 및 공급업</t>
+          <t>의료용 기기 제조업</t>
         </is>
       </c>
       <c r="J60" s="6" t="inlineStr">
         <is>
-          <t>대신</t>
+          <t>KB</t>
         </is>
       </c>
       <c r="K60" s="6" t="inlineStr">
@@ -3725,12 +3725,12 @@
     <row r="61">
       <c r="A61" s="6" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
+          <t>2026-06-25</t>
         </is>
       </c>
       <c r="B61" s="6" t="inlineStr">
         <is>
-          <t>엠에스바이오</t>
+          <t>기도산업</t>
         </is>
       </c>
       <c r="C61" s="6" t="inlineStr">
@@ -3750,27 +3750,27 @@
       </c>
       <c r="F61" s="7" t="inlineStr">
         <is>
-          <t>23,787</t>
+          <t>346,551</t>
         </is>
       </c>
       <c r="G61" s="7" t="inlineStr">
         <is>
-          <t>7,288</t>
+          <t>35,334</t>
         </is>
       </c>
       <c r="H61" s="7" t="inlineStr">
         <is>
-          <t>1,942</t>
+          <t>145,991</t>
         </is>
       </c>
       <c r="I61" s="6" t="inlineStr">
         <is>
-          <t>의료용 기기 제조업</t>
+          <t>봉제의복 제조업</t>
         </is>
       </c>
       <c r="J61" s="6" t="inlineStr">
         <is>
-          <t>KB</t>
+          <t>미래</t>
         </is>
       </c>
       <c r="K61" s="6" t="inlineStr">
@@ -3787,7 +3787,7 @@
       </c>
       <c r="B62" s="6" t="inlineStr">
         <is>
-          <t>기도산업</t>
+          <t>브릴스</t>
         </is>
       </c>
       <c r="C62" s="6" t="inlineStr">
@@ -3807,27 +3807,27 @@
       </c>
       <c r="F62" s="7" t="inlineStr">
         <is>
-          <t>346,551</t>
+          <t>23,759</t>
         </is>
       </c>
       <c r="G62" s="7" t="inlineStr">
         <is>
-          <t>35,334</t>
+          <t>1,744</t>
         </is>
       </c>
       <c r="H62" s="7" t="inlineStr">
         <is>
-          <t>145,991</t>
+          <t>4,785</t>
         </is>
       </c>
       <c r="I62" s="6" t="inlineStr">
         <is>
-          <t>봉제의복 제조업</t>
+          <t>특수 목적용 기계 제조업</t>
         </is>
       </c>
       <c r="J62" s="6" t="inlineStr">
         <is>
-          <t>미래</t>
+          <t>IBK</t>
         </is>
       </c>
       <c r="K62" s="6" t="inlineStr">
@@ -3844,7 +3844,7 @@
       </c>
       <c r="B63" s="6" t="inlineStr">
         <is>
-          <t>브릴스</t>
+          <t>와이즈플래닛컴퍼니</t>
         </is>
       </c>
       <c r="C63" s="6" t="inlineStr">
@@ -3864,27 +3864,27 @@
       </c>
       <c r="F63" s="7" t="inlineStr">
         <is>
-          <t>23,759</t>
+          <t>44,578</t>
         </is>
       </c>
       <c r="G63" s="7" t="inlineStr">
         <is>
-          <t>1,744</t>
+          <t>7,748</t>
         </is>
       </c>
       <c r="H63" s="7" t="inlineStr">
         <is>
-          <t>4,785</t>
+          <t>959</t>
         </is>
       </c>
       <c r="I63" s="6" t="inlineStr">
         <is>
-          <t>특수 목적용 기계 제조업</t>
+          <t>광고물 문안, 도안, 설계 등 작성업</t>
         </is>
       </c>
       <c r="J63" s="6" t="inlineStr">
         <is>
-          <t>IBK</t>
+          <t>대신</t>
         </is>
       </c>
       <c r="K63" s="6" t="inlineStr">
@@ -3896,12 +3896,12 @@
     <row r="64">
       <c r="A64" s="6" t="inlineStr">
         <is>
-          <t>2026-06-25</t>
+          <t>2026-06-24</t>
         </is>
       </c>
       <c r="B64" s="6" t="inlineStr">
         <is>
-          <t>와이즈플래닛컴퍼니</t>
+          <t>니어스랩</t>
         </is>
       </c>
       <c r="C64" s="6" t="inlineStr">
@@ -3921,27 +3921,27 @@
       </c>
       <c r="F64" s="7" t="inlineStr">
         <is>
-          <t>44,578</t>
+          <t>6,361</t>
         </is>
       </c>
       <c r="G64" s="7" t="inlineStr">
         <is>
-          <t>7,748</t>
+          <t>-7,287</t>
         </is>
       </c>
       <c r="H64" s="7" t="inlineStr">
         <is>
-          <t>959</t>
+          <t>127</t>
         </is>
       </c>
       <c r="I64" s="6" t="inlineStr">
         <is>
-          <t>광고물 문안, 도안, 설계 등 작성업</t>
+          <t>소프트웨어 개발 및 공급업</t>
         </is>
       </c>
       <c r="J64" s="6" t="inlineStr">
         <is>
-          <t>대신</t>
+          <t>삼성</t>
         </is>
       </c>
       <c r="K64" s="6" t="inlineStr">
@@ -3958,7 +3958,7 @@
       </c>
       <c r="B65" s="6" t="inlineStr">
         <is>
-          <t>니어스랩</t>
+          <t>해치텍</t>
         </is>
       </c>
       <c r="C65" s="6" t="inlineStr">
@@ -3978,27 +3978,27 @@
       </c>
       <c r="F65" s="7" t="inlineStr">
         <is>
-          <t>6,361</t>
+          <t>14,079</t>
         </is>
       </c>
       <c r="G65" s="7" t="inlineStr">
         <is>
-          <t>-7,287</t>
+          <t>-8,009</t>
         </is>
       </c>
       <c r="H65" s="7" t="inlineStr">
         <is>
-          <t>127</t>
+          <t>2,229</t>
         </is>
       </c>
       <c r="I65" s="6" t="inlineStr">
         <is>
-          <t>소프트웨어 개발 및 공급업</t>
+          <t>반도체 제조업</t>
         </is>
       </c>
       <c r="J65" s="6" t="inlineStr">
         <is>
-          <t>삼성</t>
+          <t>DB</t>
         </is>
       </c>
       <c r="K65" s="6" t="inlineStr">
@@ -4015,7 +4015,7 @@
       </c>
       <c r="B66" s="6" t="inlineStr">
         <is>
-          <t>해치텍</t>
+          <t>스카이랩스</t>
         </is>
       </c>
       <c r="C66" s="6" t="inlineStr">
@@ -4035,27 +4035,27 @@
       </c>
       <c r="F66" s="7" t="inlineStr">
         <is>
-          <t>14,079</t>
+          <t>7,936</t>
         </is>
       </c>
       <c r="G66" s="7" t="inlineStr">
         <is>
-          <t>-8,009</t>
+          <t>-62,995</t>
         </is>
       </c>
       <c r="H66" s="7" t="inlineStr">
         <is>
-          <t>2,229</t>
+          <t>8,341</t>
         </is>
       </c>
       <c r="I66" s="6" t="inlineStr">
         <is>
-          <t>반도체 제조업</t>
+          <t>의료용 기기 제조업</t>
         </is>
       </c>
       <c r="J66" s="6" t="inlineStr">
         <is>
-          <t>DB</t>
+          <t>한국</t>
         </is>
       </c>
       <c r="K66" s="6" t="inlineStr">
@@ -4067,12 +4067,12 @@
     <row r="67">
       <c r="A67" s="6" t="inlineStr">
         <is>
-          <t>2026-06-24</t>
+          <t>2026-06-15</t>
         </is>
       </c>
       <c r="B67" s="6" t="inlineStr">
         <is>
-          <t>스카이랩스</t>
+          <t>에이치엘지노믹스</t>
         </is>
       </c>
       <c r="C67" s="6" t="inlineStr">
@@ -4092,27 +4092,27 @@
       </c>
       <c r="F67" s="7" t="inlineStr">
         <is>
-          <t>7,936</t>
+          <t>28,877</t>
         </is>
       </c>
       <c r="G67" s="7" t="inlineStr">
         <is>
-          <t>-62,995</t>
+          <t>8,452</t>
         </is>
       </c>
       <c r="H67" s="7" t="inlineStr">
         <is>
-          <t>8,341</t>
+          <t>83,552</t>
         </is>
       </c>
       <c r="I67" s="6" t="inlineStr">
         <is>
-          <t>의료용 기기 제조업</t>
+          <t>기초 의약물질 제조업</t>
         </is>
       </c>
       <c r="J67" s="6" t="inlineStr">
         <is>
-          <t>한국</t>
+          <t>KB, IBK</t>
         </is>
       </c>
       <c r="K67" s="6" t="inlineStr">
@@ -4129,7 +4129,7 @@
       </c>
       <c r="B68" s="6" t="inlineStr">
         <is>
-          <t>에이치엘지노믹스</t>
+          <t>딜리셔스</t>
         </is>
       </c>
       <c r="C68" s="6" t="inlineStr">
@@ -4149,27 +4149,27 @@
       </c>
       <c r="F68" s="7" t="inlineStr">
         <is>
-          <t>28,877</t>
+          <t>25,149</t>
         </is>
       </c>
       <c r="G68" s="7" t="inlineStr">
         <is>
-          <t>8,452</t>
+          <t>-20,419</t>
         </is>
       </c>
       <c r="H68" s="7" t="inlineStr">
         <is>
-          <t>83,552</t>
+          <t>-114,384</t>
         </is>
       </c>
       <c r="I68" s="6" t="inlineStr">
         <is>
-          <t>기초 의약물질 제조업</t>
+          <t>무점포 소매업</t>
         </is>
       </c>
       <c r="J68" s="6" t="inlineStr">
         <is>
-          <t>KB, IBK</t>
+          <t>한국</t>
         </is>
       </c>
       <c r="K68" s="6" t="inlineStr">
@@ -4181,12 +4181,12 @@
     <row r="69">
       <c r="A69" s="6" t="inlineStr">
         <is>
-          <t>2026-06-15</t>
+          <t>2026-05-21</t>
         </is>
       </c>
       <c r="B69" s="6" t="inlineStr">
         <is>
-          <t>딜리셔스</t>
+          <t>인제니아테라퓨틱스</t>
         </is>
       </c>
       <c r="C69" s="6" t="inlineStr">
@@ -4206,27 +4206,27 @@
       </c>
       <c r="F69" s="7" t="inlineStr">
         <is>
-          <t>25,149</t>
+          <t>2,588,400</t>
         </is>
       </c>
       <c r="G69" s="7" t="inlineStr">
         <is>
-          <t>-20,419</t>
+          <t>15,755,864</t>
         </is>
       </c>
       <c r="H69" s="7" t="inlineStr">
         <is>
-          <t>-114,384</t>
+          <t>30,841,690</t>
         </is>
       </c>
       <c r="I69" s="6" t="inlineStr">
         <is>
-          <t>무점포 소매업</t>
+          <t>자연과학 및 공학 연구개발업</t>
         </is>
       </c>
       <c r="J69" s="6" t="inlineStr">
         <is>
-          <t>한국</t>
+          <t>삼성</t>
         </is>
       </c>
       <c r="K69" s="6" t="inlineStr">
@@ -4238,12 +4238,12 @@
     <row r="70">
       <c r="A70" s="6" t="inlineStr">
         <is>
-          <t>2026-05-21</t>
+          <t>2026-05-20</t>
         </is>
       </c>
       <c r="B70" s="6" t="inlineStr">
         <is>
-          <t>인제니아테라퓨틱스</t>
+          <t>한국제16호스팩</t>
         </is>
       </c>
       <c r="C70" s="6" t="inlineStr">
@@ -4261,46 +4261,30 @@
           <t>FY25</t>
         </is>
       </c>
-      <c r="F70" s="7" t="inlineStr">
-        <is>
-          <t>2,588,400</t>
-        </is>
-      </c>
-      <c r="G70" s="7" t="inlineStr">
-        <is>
-          <t>15,755,864</t>
-        </is>
-      </c>
-      <c r="H70" s="7" t="inlineStr">
-        <is>
-          <t>30,841,690</t>
-        </is>
-      </c>
-      <c r="I70" s="6" t="inlineStr">
-        <is>
-          <t>자연과학 및 공학 연구개발업</t>
-        </is>
-      </c>
+      <c r="F70" s="7" t="inlineStr"/>
+      <c r="G70" s="7" t="inlineStr"/>
+      <c r="H70" s="7" t="inlineStr"/>
+      <c r="I70" s="6" t="inlineStr"/>
       <c r="J70" s="6" t="inlineStr">
         <is>
-          <t>삼성</t>
+          <t>한국</t>
         </is>
       </c>
       <c r="K70" s="6" t="inlineStr">
         <is>
-          <t>상장전</t>
+          <t>상장완료 (2026-06-30)</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" s="6" t="inlineStr">
         <is>
-          <t>2026-05-20</t>
+          <t>2026-05-07</t>
         </is>
       </c>
       <c r="B71" s="6" t="inlineStr">
         <is>
-          <t>한국제16호스팩</t>
+          <t>레메디</t>
         </is>
       </c>
       <c r="C71" s="6" t="inlineStr">
@@ -4318,18 +4302,34 @@
           <t>FY25</t>
         </is>
       </c>
-      <c r="F71" s="7" t="inlineStr"/>
-      <c r="G71" s="7" t="inlineStr"/>
-      <c r="H71" s="7" t="inlineStr"/>
-      <c r="I71" s="6" t="inlineStr"/>
+      <c r="F71" s="7" t="inlineStr">
+        <is>
+          <t>13,441</t>
+        </is>
+      </c>
+      <c r="G71" s="7" t="inlineStr">
+        <is>
+          <t>741</t>
+        </is>
+      </c>
+      <c r="H71" s="7" t="inlineStr">
+        <is>
+          <t>5,870</t>
+        </is>
+      </c>
+      <c r="I71" s="6" t="inlineStr">
+        <is>
+          <t>의료용 기기 제조업</t>
+        </is>
+      </c>
       <c r="J71" s="6" t="inlineStr">
         <is>
-          <t>한국</t>
+          <t>KB</t>
         </is>
       </c>
       <c r="K71" s="6" t="inlineStr">
         <is>
-          <t>상장완료 (2026-06-30)</t>
+          <t>상장완료 (2026-07-13)</t>
         </is>
       </c>
     </row>
@@ -4341,7 +4341,7 @@
       </c>
       <c r="B72" s="6" t="inlineStr">
         <is>
-          <t>레메디</t>
+          <t>케이앤에스아이앤씨</t>
         </is>
       </c>
       <c r="C72" s="6" t="inlineStr">
@@ -4361,44 +4361,44 @@
       </c>
       <c r="F72" s="7" t="inlineStr">
         <is>
-          <t>13,441</t>
+          <t>13,482</t>
         </is>
       </c>
       <c r="G72" s="7" t="inlineStr">
         <is>
-          <t>741</t>
+          <t>-2,213</t>
         </is>
       </c>
       <c r="H72" s="7" t="inlineStr">
         <is>
-          <t>5,870</t>
+          <t>4,273</t>
         </is>
       </c>
       <c r="I72" s="6" t="inlineStr">
         <is>
-          <t>의료용 기기 제조업</t>
+          <t>통신 및 방송 장비 제조업</t>
         </is>
       </c>
       <c r="J72" s="6" t="inlineStr">
         <is>
-          <t>KB</t>
+          <t>IBK</t>
         </is>
       </c>
       <c r="K72" s="6" t="inlineStr">
         <is>
-          <t>상장완료 (2026-07-13)</t>
+          <t>상장전</t>
         </is>
       </c>
     </row>
     <row r="73">
       <c r="A73" s="6" t="inlineStr">
         <is>
-          <t>2026-05-07</t>
+          <t>2026-04-27</t>
         </is>
       </c>
       <c r="B73" s="6" t="inlineStr">
         <is>
-          <t>케이앤에스아이앤씨</t>
+          <t>메리츠제2호스팩</t>
         </is>
       </c>
       <c r="C73" s="6" t="inlineStr">
@@ -4416,46 +4416,30 @@
           <t>FY25</t>
         </is>
       </c>
-      <c r="F73" s="7" t="inlineStr">
-        <is>
-          <t>13,482</t>
-        </is>
-      </c>
-      <c r="G73" s="7" t="inlineStr">
-        <is>
-          <t>-2,213</t>
-        </is>
-      </c>
-      <c r="H73" s="7" t="inlineStr">
-        <is>
-          <t>4,273</t>
-        </is>
-      </c>
-      <c r="I73" s="6" t="inlineStr">
-        <is>
-          <t>통신 및 방송 장비 제조업</t>
-        </is>
-      </c>
+      <c r="F73" s="7" t="inlineStr"/>
+      <c r="G73" s="7" t="inlineStr"/>
+      <c r="H73" s="7" t="inlineStr"/>
+      <c r="I73" s="6" t="inlineStr"/>
       <c r="J73" s="6" t="inlineStr">
         <is>
-          <t>IBK</t>
+          <t>메리츠</t>
         </is>
       </c>
       <c r="K73" s="6" t="inlineStr">
         <is>
-          <t>상장전</t>
+          <t>상장완료 (2026-06-19)</t>
         </is>
       </c>
     </row>
     <row r="74">
       <c r="A74" s="6" t="inlineStr">
         <is>
-          <t>2026-04-27</t>
+          <t>2026-04-23</t>
         </is>
       </c>
       <c r="B74" s="6" t="inlineStr">
         <is>
-          <t>메리츠제2호스팩</t>
+          <t>빅웨이브로보틱스</t>
         </is>
       </c>
       <c r="C74" s="6" t="inlineStr">
@@ -4470,33 +4454,49 @@
       </c>
       <c r="E74" s="6" t="inlineStr">
         <is>
-          <t>FY25</t>
-        </is>
-      </c>
-      <c r="F74" s="7" t="inlineStr"/>
-      <c r="G74" s="7" t="inlineStr"/>
-      <c r="H74" s="7" t="inlineStr"/>
-      <c r="I74" s="6" t="inlineStr"/>
+          <t>FY24</t>
+        </is>
+      </c>
+      <c r="F74" s="7" t="inlineStr">
+        <is>
+          <t>13,851</t>
+        </is>
+      </c>
+      <c r="G74" s="7" t="inlineStr">
+        <is>
+          <t>-5,856</t>
+        </is>
+      </c>
+      <c r="H74" s="7" t="inlineStr">
+        <is>
+          <t>9,470</t>
+        </is>
+      </c>
+      <c r="I74" s="6" t="inlineStr">
+        <is>
+          <t>소프트웨어 개발 및 공급업</t>
+        </is>
+      </c>
       <c r="J74" s="6" t="inlineStr">
         <is>
-          <t>메리츠</t>
+          <t>유진, 미래</t>
         </is>
       </c>
       <c r="K74" s="6" t="inlineStr">
         <is>
-          <t>상장완료 (2026-06-19)</t>
+          <t>상장전</t>
         </is>
       </c>
     </row>
     <row r="75">
       <c r="A75" s="6" t="inlineStr">
         <is>
-          <t>2026-04-23</t>
+          <t>2026-04-09</t>
         </is>
       </c>
       <c r="B75" s="6" t="inlineStr">
         <is>
-          <t>빅웨이브로보틱스</t>
+          <t>매드업</t>
         </is>
       </c>
       <c r="C75" s="6" t="inlineStr">
@@ -4516,44 +4516,44 @@
       </c>
       <c r="F75" s="7" t="inlineStr">
         <is>
-          <t>13,851</t>
+          <t>34,989</t>
         </is>
       </c>
       <c r="G75" s="7" t="inlineStr">
         <is>
-          <t>-5,856</t>
+          <t>-2,747</t>
         </is>
       </c>
       <c r="H75" s="7" t="inlineStr">
         <is>
-          <t>9,470</t>
+          <t>-15,766</t>
         </is>
       </c>
       <c r="I75" s="6" t="inlineStr">
         <is>
-          <t>소프트웨어 개발 및 공급업</t>
+          <t>광고</t>
         </is>
       </c>
       <c r="J75" s="6" t="inlineStr">
         <is>
-          <t>유진, 미래</t>
+          <t>미래</t>
         </is>
       </c>
       <c r="K75" s="6" t="inlineStr">
         <is>
-          <t>상장전</t>
+          <t>상장완료 (2026-07-01)</t>
         </is>
       </c>
     </row>
     <row r="76">
       <c r="A76" s="6" t="inlineStr">
         <is>
-          <t>2026-04-09</t>
+          <t>2026-04-02</t>
         </is>
       </c>
       <c r="B76" s="6" t="inlineStr">
         <is>
-          <t>매드업</t>
+          <t>져스텍</t>
         </is>
       </c>
       <c r="C76" s="6" t="inlineStr">
@@ -4573,32 +4573,32 @@
       </c>
       <c r="F76" s="7" t="inlineStr">
         <is>
-          <t>34,989</t>
+          <t>19,851</t>
         </is>
       </c>
       <c r="G76" s="7" t="inlineStr">
         <is>
-          <t>-2,747</t>
+          <t>444</t>
         </is>
       </c>
       <c r="H76" s="7" t="inlineStr">
         <is>
-          <t>-15,766</t>
+          <t>10,953</t>
         </is>
       </c>
       <c r="I76" s="6" t="inlineStr">
         <is>
-          <t>광고</t>
+          <t>기계</t>
         </is>
       </c>
       <c r="J76" s="6" t="inlineStr">
         <is>
-          <t>미래</t>
+          <t>삼성</t>
         </is>
       </c>
       <c r="K76" s="6" t="inlineStr">
         <is>
-          <t>상장완료 (2026-07-01)</t>
+          <t>상장완료 (2026-06-29)</t>
         </is>
       </c>
     </row>
@@ -4610,7 +4610,7 @@
       </c>
       <c r="B77" s="6" t="inlineStr">
         <is>
-          <t>져스텍</t>
+          <t>스트라드비젼</t>
         </is>
       </c>
       <c r="C77" s="6" t="inlineStr">
@@ -4630,44 +4630,44 @@
       </c>
       <c r="F77" s="7" t="inlineStr">
         <is>
-          <t>19,851</t>
+          <t>11,539</t>
         </is>
       </c>
       <c r="G77" s="7" t="inlineStr">
         <is>
-          <t>444</t>
+          <t>-65,529</t>
         </is>
       </c>
       <c r="H77" s="7" t="inlineStr">
         <is>
-          <t>10,953</t>
+          <t>-245,151</t>
         </is>
       </c>
       <c r="I77" s="6" t="inlineStr">
         <is>
-          <t>기계</t>
+          <t>소프트웨어</t>
         </is>
       </c>
       <c r="J77" s="6" t="inlineStr">
         <is>
-          <t>삼성</t>
+          <t>KB</t>
         </is>
       </c>
       <c r="K77" s="6" t="inlineStr">
         <is>
-          <t>상장완료 (2026-06-29)</t>
+          <t>상장완료 (2026-06-30)</t>
         </is>
       </c>
     </row>
     <row r="78">
       <c r="A78" s="6" t="inlineStr">
         <is>
-          <t>2026-04-02</t>
+          <t>2026-03-30</t>
         </is>
       </c>
       <c r="B78" s="6" t="inlineStr">
         <is>
-          <t>스트라드비젼</t>
+          <t>대신밸런스제20호스팩</t>
         </is>
       </c>
       <c r="C78" s="6" t="inlineStr">
@@ -4682,49 +4682,33 @@
       </c>
       <c r="E78" s="6" t="inlineStr">
         <is>
-          <t>FY24</t>
-        </is>
-      </c>
-      <c r="F78" s="7" t="inlineStr">
-        <is>
-          <t>11,539</t>
-        </is>
-      </c>
-      <c r="G78" s="7" t="inlineStr">
-        <is>
-          <t>-65,529</t>
-        </is>
-      </c>
-      <c r="H78" s="7" t="inlineStr">
-        <is>
-          <t>-245,151</t>
-        </is>
-      </c>
-      <c r="I78" s="6" t="inlineStr">
-        <is>
-          <t>소프트웨어</t>
-        </is>
-      </c>
+          <t>FY25</t>
+        </is>
+      </c>
+      <c r="F78" s="7" t="inlineStr"/>
+      <c r="G78" s="7" t="inlineStr"/>
+      <c r="H78" s="7" t="inlineStr"/>
+      <c r="I78" s="6" t="inlineStr"/>
       <c r="J78" s="6" t="inlineStr">
         <is>
-          <t>KB</t>
+          <t>대신</t>
         </is>
       </c>
       <c r="K78" s="6" t="inlineStr">
         <is>
-          <t>상장완료 (2026-06-30)</t>
+          <t>상장완료 (2026-06-05)</t>
         </is>
       </c>
     </row>
     <row r="79">
       <c r="A79" s="6" t="inlineStr">
         <is>
-          <t>2026-03-30</t>
+          <t>2026-03-26</t>
         </is>
       </c>
       <c r="B79" s="6" t="inlineStr">
         <is>
-          <t>대신밸런스제20호스팩</t>
+          <t>피스피스스튜디오</t>
         </is>
       </c>
       <c r="C79" s="6" t="inlineStr">
@@ -4739,21 +4723,37 @@
       </c>
       <c r="E79" s="6" t="inlineStr">
         <is>
-          <t>FY25</t>
-        </is>
-      </c>
-      <c r="F79" s="7" t="inlineStr"/>
-      <c r="G79" s="7" t="inlineStr"/>
-      <c r="H79" s="7" t="inlineStr"/>
-      <c r="I79" s="6" t="inlineStr"/>
+          <t>FY24</t>
+        </is>
+      </c>
+      <c r="F79" s="7" t="inlineStr">
+        <is>
+          <t>113,777</t>
+        </is>
+      </c>
+      <c r="G79" s="7" t="inlineStr">
+        <is>
+          <t>17,603</t>
+        </is>
+      </c>
+      <c r="H79" s="7" t="inlineStr">
+        <is>
+          <t>55,861</t>
+        </is>
+      </c>
+      <c r="I79" s="6" t="inlineStr">
+        <is>
+          <t>섬유,의류,신발,호화품</t>
+        </is>
+      </c>
       <c r="J79" s="6" t="inlineStr">
         <is>
-          <t>대신</t>
+          <t>NH, 미래</t>
         </is>
       </c>
       <c r="K79" s="6" t="inlineStr">
         <is>
-          <t>상장완료 (2026-06-05)</t>
+          <t>상장완료 (2026-06-08)</t>
         </is>
       </c>
     </row>
@@ -4765,7 +4765,7 @@
       </c>
       <c r="B80" s="6" t="inlineStr">
         <is>
-          <t>피스피스스튜디오</t>
+          <t>폴레드</t>
         </is>
       </c>
       <c r="C80" s="6" t="inlineStr">
@@ -4785,32 +4785,32 @@
       </c>
       <c r="F80" s="7" t="inlineStr">
         <is>
-          <t>113,777</t>
+          <t>52,808</t>
         </is>
       </c>
       <c r="G80" s="7" t="inlineStr">
         <is>
-          <t>17,603</t>
+          <t>543</t>
         </is>
       </c>
       <c r="H80" s="7" t="inlineStr">
         <is>
-          <t>55,861</t>
+          <t>25,416</t>
         </is>
       </c>
       <c r="I80" s="6" t="inlineStr">
         <is>
-          <t>섬유,의류,신발,호화품</t>
+          <t>가정용기기와용품</t>
         </is>
       </c>
       <c r="J80" s="6" t="inlineStr">
         <is>
-          <t>NH, 미래</t>
+          <t>NH</t>
         </is>
       </c>
       <c r="K80" s="6" t="inlineStr">
         <is>
-          <t>상장완료 (2026-06-08)</t>
+          <t>상장완료 (2026-05-14)</t>
         </is>
       </c>
     </row>
@@ -4822,7 +4822,7 @@
       </c>
       <c r="B81" s="6" t="inlineStr">
         <is>
-          <t>폴레드</t>
+          <t>레몬헬스케어</t>
         </is>
       </c>
       <c r="C81" s="6" t="inlineStr">
@@ -4842,44 +4842,44 @@
       </c>
       <c r="F81" s="7" t="inlineStr">
         <is>
-          <t>52,808</t>
+          <t>14,877</t>
         </is>
       </c>
       <c r="G81" s="7" t="inlineStr">
         <is>
-          <t>543</t>
+          <t>-2,898</t>
         </is>
       </c>
       <c r="H81" s="7" t="inlineStr">
         <is>
-          <t>25,416</t>
+          <t>-31,162</t>
         </is>
       </c>
       <c r="I81" s="6" t="inlineStr">
         <is>
-          <t>가정용기기와용품</t>
+          <t>건강관리업체및서비스</t>
         </is>
       </c>
       <c r="J81" s="6" t="inlineStr">
         <is>
-          <t>NH</t>
+          <t>KB</t>
         </is>
       </c>
       <c r="K81" s="6" t="inlineStr">
         <is>
-          <t>상장완료 (2026-05-14)</t>
+          <t>상장완료 (2026-07-06)</t>
         </is>
       </c>
     </row>
     <row r="82">
       <c r="A82" s="6" t="inlineStr">
         <is>
-          <t>2026-03-26</t>
+          <t>2026-02-27</t>
         </is>
       </c>
       <c r="B82" s="6" t="inlineStr">
         <is>
-          <t>레몬헬스케어</t>
+          <t>마키나락스</t>
         </is>
       </c>
       <c r="C82" s="6" t="inlineStr">
@@ -4899,32 +4899,32 @@
       </c>
       <c r="F82" s="7" t="inlineStr">
         <is>
-          <t>14,877</t>
+          <t>8,294</t>
         </is>
       </c>
       <c r="G82" s="7" t="inlineStr">
         <is>
-          <t>-2,898</t>
+          <t>-6,073</t>
         </is>
       </c>
       <c r="H82" s="7" t="inlineStr">
         <is>
-          <t>-31,162</t>
+          <t>2,680</t>
         </is>
       </c>
       <c r="I82" s="6" t="inlineStr">
         <is>
-          <t>건강관리업체및서비스</t>
+          <t>소프트웨어</t>
         </is>
       </c>
       <c r="J82" s="6" t="inlineStr">
         <is>
-          <t>KB</t>
+          <t>미래</t>
         </is>
       </c>
       <c r="K82" s="6" t="inlineStr">
         <is>
-          <t>상장완료 (2026-07-06)</t>
+          <t>상장완료 (2026-05-20)</t>
         </is>
       </c>
     </row>
@@ -4936,7 +4936,7 @@
       </c>
       <c r="B83" s="6" t="inlineStr">
         <is>
-          <t>마키나락스</t>
+          <t>채비</t>
         </is>
       </c>
       <c r="C83" s="6" t="inlineStr">
@@ -4956,44 +4956,44 @@
       </c>
       <c r="F83" s="7" t="inlineStr">
         <is>
-          <t>8,294</t>
+          <t>85,082</t>
         </is>
       </c>
       <c r="G83" s="7" t="inlineStr">
         <is>
-          <t>-6,073</t>
+          <t>-54,495</t>
         </is>
       </c>
       <c r="H83" s="7" t="inlineStr">
         <is>
-          <t>2,680</t>
+          <t>96,866</t>
         </is>
       </c>
       <c r="I83" s="6" t="inlineStr">
         <is>
-          <t>소프트웨어</t>
+          <t>전기제품</t>
         </is>
       </c>
       <c r="J83" s="6" t="inlineStr">
         <is>
-          <t>미래</t>
+          <t>KB, 삼성, 대신, 하나</t>
         </is>
       </c>
       <c r="K83" s="6" t="inlineStr">
         <is>
-          <t>상장완료 (2026-05-20)</t>
+          <t>상장완료 (2026-04-29)</t>
         </is>
       </c>
     </row>
     <row r="84">
       <c r="A84" s="6" t="inlineStr">
         <is>
-          <t>2026-02-27</t>
+          <t>2026-02-10</t>
         </is>
       </c>
       <c r="B84" s="6" t="inlineStr">
         <is>
-          <t>채비</t>
+          <t>키움히어로제2호스팩</t>
         </is>
       </c>
       <c r="C84" s="6" t="inlineStr">
@@ -5011,46 +5011,30 @@
           <t>FY24</t>
         </is>
       </c>
-      <c r="F84" s="7" t="inlineStr">
-        <is>
-          <t>85,082</t>
-        </is>
-      </c>
-      <c r="G84" s="7" t="inlineStr">
-        <is>
-          <t>-54,495</t>
-        </is>
-      </c>
-      <c r="H84" s="7" t="inlineStr">
-        <is>
-          <t>96,866</t>
-        </is>
-      </c>
-      <c r="I84" s="6" t="inlineStr">
-        <is>
-          <t>전기제품</t>
-        </is>
-      </c>
+      <c r="F84" s="7" t="inlineStr"/>
+      <c r="G84" s="7" t="inlineStr"/>
+      <c r="H84" s="7" t="inlineStr"/>
+      <c r="I84" s="6" t="inlineStr"/>
       <c r="J84" s="6" t="inlineStr">
         <is>
-          <t>KB, 삼성, 대신, 하나</t>
+          <t>키움</t>
         </is>
       </c>
       <c r="K84" s="6" t="inlineStr">
         <is>
-          <t>상장완료 (2026-04-29)</t>
+          <t>상장완료 (2026-04-23)</t>
         </is>
       </c>
     </row>
     <row r="85">
       <c r="A85" s="6" t="inlineStr">
         <is>
-          <t>2026-02-10</t>
+          <t>2026-02-05</t>
         </is>
       </c>
       <c r="B85" s="6" t="inlineStr">
         <is>
-          <t>키움히어로제2호스팩</t>
+          <t>세미티에스</t>
         </is>
       </c>
       <c r="C85" s="6" t="inlineStr">
@@ -5060,7 +5044,7 @@
       </c>
       <c r="D85" s="6" t="inlineStr">
         <is>
-          <t>신규상장</t>
+          <t>스팩 소멸합병</t>
         </is>
       </c>
       <c r="E85" s="6" t="inlineStr">
@@ -5068,30 +5052,46 @@
           <t>FY24</t>
         </is>
       </c>
-      <c r="F85" s="7" t="inlineStr"/>
-      <c r="G85" s="7" t="inlineStr"/>
-      <c r="H85" s="7" t="inlineStr"/>
-      <c r="I85" s="6" t="inlineStr"/>
+      <c r="F85" s="7" t="inlineStr">
+        <is>
+          <t>20,808</t>
+        </is>
+      </c>
+      <c r="G85" s="7" t="inlineStr">
+        <is>
+          <t>7,337</t>
+        </is>
+      </c>
+      <c r="H85" s="7" t="inlineStr">
+        <is>
+          <t>26,616</t>
+        </is>
+      </c>
+      <c r="I85" s="6" t="inlineStr">
+        <is>
+          <t>반도체와반도체장비</t>
+        </is>
+      </c>
       <c r="J85" s="6" t="inlineStr">
         <is>
-          <t>키움</t>
+          <t>NH</t>
         </is>
       </c>
       <c r="K85" s="6" t="inlineStr">
         <is>
-          <t>상장완료 (2026-04-23)</t>
+          <t>상장완료 (2026-02-05)</t>
         </is>
       </c>
     </row>
     <row r="86">
       <c r="A86" s="6" t="inlineStr">
         <is>
-          <t>2026-02-05</t>
+          <t>2026-02-02</t>
         </is>
       </c>
       <c r="B86" s="6" t="inlineStr">
         <is>
-          <t>세미티에스</t>
+          <t>교보20호스팩</t>
         </is>
       </c>
       <c r="C86" s="6" t="inlineStr">
@@ -5101,7 +5101,7 @@
       </c>
       <c r="D86" s="6" t="inlineStr">
         <is>
-          <t>스팩 소멸합병</t>
+          <t>신규상장</t>
         </is>
       </c>
       <c r="E86" s="6" t="inlineStr">
@@ -5109,46 +5109,30 @@
           <t>FY24</t>
         </is>
       </c>
-      <c r="F86" s="7" t="inlineStr">
-        <is>
-          <t>20,808</t>
-        </is>
-      </c>
-      <c r="G86" s="7" t="inlineStr">
-        <is>
-          <t>7,337</t>
-        </is>
-      </c>
-      <c r="H86" s="7" t="inlineStr">
-        <is>
-          <t>26,616</t>
-        </is>
-      </c>
-      <c r="I86" s="6" t="inlineStr">
-        <is>
-          <t>반도체와반도체장비</t>
-        </is>
-      </c>
+      <c r="F86" s="7" t="inlineStr"/>
+      <c r="G86" s="7" t="inlineStr"/>
+      <c r="H86" s="7" t="inlineStr"/>
+      <c r="I86" s="6" t="inlineStr"/>
       <c r="J86" s="6" t="inlineStr">
         <is>
-          <t>NH</t>
+          <t>교보</t>
         </is>
       </c>
       <c r="K86" s="6" t="inlineStr">
         <is>
-          <t>상장완료 (2026-02-05)</t>
+          <t>상장완료 (2026-04-02)</t>
         </is>
       </c>
     </row>
     <row r="87">
       <c r="A87" s="6" t="inlineStr">
         <is>
-          <t>2026-02-02</t>
+          <t>2026-01-29</t>
         </is>
       </c>
       <c r="B87" s="6" t="inlineStr">
         <is>
-          <t>교보20호스팩</t>
+          <t>케이피항공산업</t>
         </is>
       </c>
       <c r="C87" s="6" t="inlineStr">
@@ -5158,7 +5142,7 @@
       </c>
       <c r="D87" s="6" t="inlineStr">
         <is>
-          <t>신규상장</t>
+          <t>스팩 소멸합병</t>
         </is>
       </c>
       <c r="E87" s="6" t="inlineStr">
@@ -5166,18 +5150,34 @@
           <t>FY24</t>
         </is>
       </c>
-      <c r="F87" s="7" t="inlineStr"/>
-      <c r="G87" s="7" t="inlineStr"/>
-      <c r="H87" s="7" t="inlineStr"/>
-      <c r="I87" s="6" t="inlineStr"/>
+      <c r="F87" s="7" t="inlineStr">
+        <is>
+          <t>49,651</t>
+        </is>
+      </c>
+      <c r="G87" s="7" t="inlineStr">
+        <is>
+          <t>3,018</t>
+        </is>
+      </c>
+      <c r="H87" s="7" t="inlineStr">
+        <is>
+          <t>15,901</t>
+        </is>
+      </c>
+      <c r="I87" s="6" t="inlineStr">
+        <is>
+          <t>우주항공과국방</t>
+        </is>
+      </c>
       <c r="J87" s="6" t="inlineStr">
         <is>
-          <t>교보</t>
+          <t>NH</t>
         </is>
       </c>
       <c r="K87" s="6" t="inlineStr">
         <is>
-          <t>상장완료 (2026-04-02)</t>
+          <t>상장완료 (2026-01-29)</t>
         </is>
       </c>
     </row>
@@ -5189,7 +5189,7 @@
       </c>
       <c r="B88" s="6" t="inlineStr">
         <is>
-          <t>케이피항공산업</t>
+          <t>한패스</t>
         </is>
       </c>
       <c r="C88" s="6" t="inlineStr">
@@ -5199,7 +5199,7 @@
       </c>
       <c r="D88" s="6" t="inlineStr">
         <is>
-          <t>스팩 소멸합병</t>
+          <t>신규상장</t>
         </is>
       </c>
       <c r="E88" s="6" t="inlineStr">
@@ -5209,44 +5209,44 @@
       </c>
       <c r="F88" s="7" t="inlineStr">
         <is>
-          <t>49,651</t>
+          <t>55,297</t>
         </is>
       </c>
       <c r="G88" s="7" t="inlineStr">
         <is>
-          <t>3,018</t>
+          <t>4,403</t>
         </is>
       </c>
       <c r="H88" s="7" t="inlineStr">
         <is>
-          <t>15,901</t>
+          <t>-28,065</t>
         </is>
       </c>
       <c r="I88" s="6" t="inlineStr">
         <is>
-          <t>우주항공과국방</t>
+          <t>IT서비스</t>
         </is>
       </c>
       <c r="J88" s="6" t="inlineStr">
         <is>
-          <t>NH</t>
+          <t>한국, 대신</t>
         </is>
       </c>
       <c r="K88" s="6" t="inlineStr">
         <is>
-          <t>상장완료 (2026-01-29)</t>
+          <t>상장완료 (2026-03-25)</t>
         </is>
       </c>
     </row>
     <row r="89">
       <c r="A89" s="6" t="inlineStr">
         <is>
-          <t>2026-01-29</t>
+          <t>2026-01-22</t>
         </is>
       </c>
       <c r="B89" s="6" t="inlineStr">
         <is>
-          <t>한패스</t>
+          <t>신한제18호스팩</t>
         </is>
       </c>
       <c r="C89" s="6" t="inlineStr">
@@ -5264,46 +5264,30 @@
           <t>FY24</t>
         </is>
       </c>
-      <c r="F89" s="7" t="inlineStr">
-        <is>
-          <t>55,297</t>
-        </is>
-      </c>
-      <c r="G89" s="7" t="inlineStr">
-        <is>
-          <t>4,403</t>
-        </is>
-      </c>
-      <c r="H89" s="7" t="inlineStr">
-        <is>
-          <t>-28,065</t>
-        </is>
-      </c>
-      <c r="I89" s="6" t="inlineStr">
-        <is>
-          <t>IT서비스</t>
-        </is>
-      </c>
+      <c r="F89" s="7" t="inlineStr"/>
+      <c r="G89" s="7" t="inlineStr"/>
+      <c r="H89" s="7" t="inlineStr"/>
+      <c r="I89" s="6" t="inlineStr"/>
       <c r="J89" s="6" t="inlineStr">
         <is>
-          <t>한국, 대신</t>
+          <t>신한</t>
         </is>
       </c>
       <c r="K89" s="6" t="inlineStr">
         <is>
-          <t>상장완료 (2026-03-25)</t>
+          <t>상장완료 (2026-04-30)</t>
         </is>
       </c>
     </row>
     <row r="90">
       <c r="A90" s="6" t="inlineStr">
         <is>
-          <t>2026-01-22</t>
+          <t>2026-01-20</t>
         </is>
       </c>
       <c r="B90" s="6" t="inlineStr">
         <is>
-          <t>신한제18호스팩</t>
+          <t>엔에이치스팩33호</t>
         </is>
       </c>
       <c r="C90" s="6" t="inlineStr">
@@ -5327,24 +5311,24 @@
       <c r="I90" s="6" t="inlineStr"/>
       <c r="J90" s="6" t="inlineStr">
         <is>
-          <t>신한</t>
+          <t>NH</t>
         </is>
       </c>
       <c r="K90" s="6" t="inlineStr">
         <is>
-          <t>상장완료 (2026-04-30)</t>
+          <t>상장완료 (2026-03-27)</t>
         </is>
       </c>
     </row>
     <row r="91">
       <c r="A91" s="6" t="inlineStr">
         <is>
-          <t>2026-01-20</t>
+          <t>2026-01-19</t>
         </is>
       </c>
       <c r="B91" s="6" t="inlineStr">
         <is>
-          <t>엔에이치스팩33호</t>
+          <t>신한제17호스팩</t>
         </is>
       </c>
       <c r="C91" s="6" t="inlineStr">
@@ -5368,24 +5352,24 @@
       <c r="I91" s="6" t="inlineStr"/>
       <c r="J91" s="6" t="inlineStr">
         <is>
-          <t>NH</t>
+          <t>신한</t>
         </is>
       </c>
       <c r="K91" s="6" t="inlineStr">
         <is>
-          <t>상장완료 (2026-03-27)</t>
+          <t>상장완료 (2026-04-01)</t>
         </is>
       </c>
     </row>
     <row r="92">
       <c r="A92" s="6" t="inlineStr">
         <is>
-          <t>2026-01-19</t>
+          <t>2026-01-16</t>
         </is>
       </c>
       <c r="B92" s="6" t="inlineStr">
         <is>
-          <t>신한제17호스팩</t>
+          <t>아이엠바이오로직스</t>
         </is>
       </c>
       <c r="C92" s="6" t="inlineStr">
@@ -5403,18 +5387,34 @@
           <t>FY24</t>
         </is>
       </c>
-      <c r="F92" s="7" t="inlineStr"/>
-      <c r="G92" s="7" t="inlineStr"/>
-      <c r="H92" s="7" t="inlineStr"/>
-      <c r="I92" s="6" t="inlineStr"/>
+      <c r="F92" s="7" t="inlineStr">
+        <is>
+          <t>27,594</t>
+        </is>
+      </c>
+      <c r="G92" s="7" t="inlineStr">
+        <is>
+          <t>-11,884</t>
+        </is>
+      </c>
+      <c r="H92" s="7" t="inlineStr">
+        <is>
+          <t>-77,202</t>
+        </is>
+      </c>
+      <c r="I92" s="6" t="inlineStr">
+        <is>
+          <t>제약</t>
+        </is>
+      </c>
       <c r="J92" s="6" t="inlineStr">
         <is>
-          <t>신한</t>
+          <t>한국, 신한</t>
         </is>
       </c>
       <c r="K92" s="6" t="inlineStr">
         <is>
-          <t>상장완료 (2026-04-01)</t>
+          <t>상장완료 (2026-03-20)</t>
         </is>
       </c>
     </row>
@@ -5426,7 +5426,7 @@
       </c>
       <c r="B93" s="6" t="inlineStr">
         <is>
-          <t>아이엠바이오로직스</t>
+          <t>에스팀</t>
         </is>
       </c>
       <c r="C93" s="6" t="inlineStr">
@@ -5446,232 +5446,232 @@
       </c>
       <c r="F93" s="7" t="inlineStr">
         <is>
-          <t>27,594</t>
+          <t>35,574</t>
         </is>
       </c>
       <c r="G93" s="7" t="inlineStr">
         <is>
-          <t>-11,884</t>
+          <t>1,372</t>
         </is>
       </c>
       <c r="H93" s="7" t="inlineStr">
         <is>
-          <t>-77,202</t>
+          <t>12,331</t>
         </is>
       </c>
       <c r="I93" s="6" t="inlineStr">
         <is>
-          <t>제약</t>
+          <t>광고</t>
         </is>
       </c>
       <c r="J93" s="6" t="inlineStr">
         <is>
-          <t>한국, 신한</t>
+          <t>한국</t>
         </is>
       </c>
       <c r="K93" s="6" t="inlineStr">
         <is>
-          <t>상장완료 (2026-03-20)</t>
+          <t>상장완료 (2026-03-06)</t>
         </is>
       </c>
     </row>
     <row r="94">
       <c r="A94" s="6" t="inlineStr">
         <is>
-          <t>2026-01-16</t>
+          <t>2026-01-12</t>
         </is>
       </c>
       <c r="B94" s="6" t="inlineStr">
         <is>
-          <t>에스팀</t>
+          <t>케이뱅크</t>
         </is>
       </c>
       <c r="C94" s="6" t="inlineStr">
         <is>
+          <t>유가</t>
+        </is>
+      </c>
+      <c r="D94" s="6" t="inlineStr">
+        <is>
+          <t>신규상장</t>
+        </is>
+      </c>
+      <c r="E94" s="6" t="inlineStr">
+        <is>
+          <t>FY24</t>
+        </is>
+      </c>
+      <c r="F94" s="7" t="inlineStr">
+        <is>
+          <t>1,228,501</t>
+        </is>
+      </c>
+      <c r="G94" s="7" t="inlineStr">
+        <is>
+          <t>128,053</t>
+        </is>
+      </c>
+      <c r="H94" s="7" t="inlineStr">
+        <is>
+          <t>1,995,845</t>
+        </is>
+      </c>
+      <c r="I94" s="6" t="inlineStr">
+        <is>
+          <t>은행</t>
+        </is>
+      </c>
+      <c r="J94" s="6" t="inlineStr">
+        <is>
+          <t>NH, 삼성</t>
+        </is>
+      </c>
+      <c r="K94" s="6" t="inlineStr">
+        <is>
+          <t>상장완료 (2026-03-05)</t>
+        </is>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" s="3" t="inlineStr">
+        <is>
+          <t>■ 철회·미승인  (15건)</t>
+        </is>
+      </c>
+      <c r="B96" s="4" t="n"/>
+      <c r="C96" s="4" t="n"/>
+      <c r="D96" s="4" t="n"/>
+      <c r="E96" s="4" t="n"/>
+      <c r="F96" s="4" t="n"/>
+      <c r="G96" s="4" t="n"/>
+      <c r="H96" s="4" t="n"/>
+      <c r="I96" s="4" t="n"/>
+      <c r="J96" s="4" t="n"/>
+      <c r="K96" s="4" t="n"/>
+    </row>
+    <row r="97">
+      <c r="A97" s="5" t="inlineStr">
+        <is>
+          <t>일자</t>
+        </is>
+      </c>
+      <c r="B97" s="5" t="inlineStr">
+        <is>
+          <t>회사명</t>
+        </is>
+      </c>
+      <c r="C97" s="5" t="inlineStr">
+        <is>
+          <t>시장</t>
+        </is>
+      </c>
+      <c r="D97" s="5" t="inlineStr">
+        <is>
+          <t>상장유형</t>
+        </is>
+      </c>
+      <c r="E97" s="5" t="inlineStr">
+        <is>
+          <t>기준연도</t>
+        </is>
+      </c>
+      <c r="F97" s="5" t="inlineStr">
+        <is>
+          <t>매출액</t>
+        </is>
+      </c>
+      <c r="G97" s="5" t="inlineStr">
+        <is>
+          <t>순이익</t>
+        </is>
+      </c>
+      <c r="H97" s="5" t="inlineStr">
+        <is>
+          <t>자기자본</t>
+        </is>
+      </c>
+      <c r="I97" s="5" t="inlineStr">
+        <is>
+          <t>업종</t>
+        </is>
+      </c>
+      <c r="J97" s="5" t="inlineStr">
+        <is>
+          <t>대표주관사</t>
+        </is>
+      </c>
+      <c r="K97" s="5" t="inlineStr">
+        <is>
+          <t>현황</t>
+        </is>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" s="6" t="inlineStr">
+        <is>
+          <t>2026-06-16</t>
+        </is>
+      </c>
+      <c r="B98" s="6" t="inlineStr">
+        <is>
+          <t>넥스트젠바이오</t>
+        </is>
+      </c>
+      <c r="C98" s="6" t="inlineStr">
+        <is>
           <t>코스닥</t>
         </is>
       </c>
-      <c r="D94" s="6" t="inlineStr">
+      <c r="D98" s="6" t="inlineStr">
         <is>
           <t>신규상장</t>
         </is>
       </c>
-      <c r="E94" s="6" t="inlineStr">
+      <c r="E98" s="6" t="inlineStr">
         <is>
           <t>FY24</t>
         </is>
       </c>
-      <c r="F94" s="7" t="inlineStr">
-        <is>
-          <t>35,574</t>
-        </is>
-      </c>
-      <c r="G94" s="7" t="inlineStr">
-        <is>
-          <t>1,372</t>
-        </is>
-      </c>
-      <c r="H94" s="7" t="inlineStr">
-        <is>
-          <t>12,331</t>
-        </is>
-      </c>
-      <c r="I94" s="6" t="inlineStr">
-        <is>
-          <t>광고</t>
-        </is>
-      </c>
-      <c r="J94" s="6" t="inlineStr">
+      <c r="F98" s="7" t="inlineStr">
+        <is>
+          <t>100</t>
+        </is>
+      </c>
+      <c r="G98" s="7" t="inlineStr">
+        <is>
+          <t>69</t>
+        </is>
+      </c>
+      <c r="H98" s="7" t="inlineStr">
+        <is>
+          <t>4,792</t>
+        </is>
+      </c>
+      <c r="I98" s="6" t="inlineStr">
+        <is>
+          <t>자연과학 및 공학 연구개발업</t>
+        </is>
+      </c>
+      <c r="J98" s="6" t="inlineStr">
         <is>
           <t>한국</t>
         </is>
       </c>
-      <c r="K94" s="6" t="inlineStr">
-        <is>
-          <t>상장완료 (2026-03-06)</t>
-        </is>
-      </c>
-    </row>
-    <row r="95">
-      <c r="A95" s="6" t="inlineStr">
-        <is>
-          <t>2026-01-12</t>
-        </is>
-      </c>
-      <c r="B95" s="6" t="inlineStr">
-        <is>
-          <t>케이뱅크</t>
-        </is>
-      </c>
-      <c r="C95" s="6" t="inlineStr">
-        <is>
-          <t>유가</t>
-        </is>
-      </c>
-      <c r="D95" s="6" t="inlineStr">
-        <is>
-          <t>신규상장</t>
-        </is>
-      </c>
-      <c r="E95" s="6" t="inlineStr">
-        <is>
-          <t>FY24</t>
-        </is>
-      </c>
-      <c r="F95" s="7" t="inlineStr">
-        <is>
-          <t>1,228,501</t>
-        </is>
-      </c>
-      <c r="G95" s="7" t="inlineStr">
-        <is>
-          <t>128,053</t>
-        </is>
-      </c>
-      <c r="H95" s="7" t="inlineStr">
-        <is>
-          <t>1,995,845</t>
-        </is>
-      </c>
-      <c r="I95" s="6" t="inlineStr">
-        <is>
-          <t>은행</t>
-        </is>
-      </c>
-      <c r="J95" s="6" t="inlineStr">
-        <is>
-          <t>NH, 삼성</t>
-        </is>
-      </c>
-      <c r="K95" s="6" t="inlineStr">
-        <is>
-          <t>상장완료 (2026-03-05)</t>
-        </is>
-      </c>
-    </row>
-    <row r="97">
-      <c r="A97" s="3" t="inlineStr">
-        <is>
-          <t>■ 철회·미승인  (15건)</t>
-        </is>
-      </c>
-      <c r="B97" s="4" t="n"/>
-      <c r="C97" s="4" t="n"/>
-      <c r="D97" s="4" t="n"/>
-      <c r="E97" s="4" t="n"/>
-      <c r="F97" s="4" t="n"/>
-      <c r="G97" s="4" t="n"/>
-      <c r="H97" s="4" t="n"/>
-      <c r="I97" s="4" t="n"/>
-      <c r="J97" s="4" t="n"/>
-      <c r="K97" s="4" t="n"/>
-    </row>
-    <row r="98">
-      <c r="A98" s="5" t="inlineStr">
-        <is>
-          <t>일자</t>
-        </is>
-      </c>
-      <c r="B98" s="5" t="inlineStr">
-        <is>
-          <t>회사명</t>
-        </is>
-      </c>
-      <c r="C98" s="5" t="inlineStr">
-        <is>
-          <t>시장</t>
-        </is>
-      </c>
-      <c r="D98" s="5" t="inlineStr">
-        <is>
-          <t>상장유형</t>
-        </is>
-      </c>
-      <c r="E98" s="5" t="inlineStr">
-        <is>
-          <t>기준연도</t>
-        </is>
-      </c>
-      <c r="F98" s="5" t="inlineStr">
-        <is>
-          <t>매출액</t>
-        </is>
-      </c>
-      <c r="G98" s="5" t="inlineStr">
-        <is>
-          <t>순이익</t>
-        </is>
-      </c>
-      <c r="H98" s="5" t="inlineStr">
-        <is>
-          <t>자기자본</t>
-        </is>
-      </c>
-      <c r="I98" s="5" t="inlineStr">
-        <is>
-          <t>업종</t>
-        </is>
-      </c>
-      <c r="J98" s="5" t="inlineStr">
-        <is>
-          <t>대표주관사</t>
-        </is>
-      </c>
-      <c r="K98" s="5" t="inlineStr">
-        <is>
-          <t>현황</t>
+      <c r="K98" s="6" t="inlineStr">
+        <is>
+          <t>심사 철회</t>
         </is>
       </c>
     </row>
     <row r="99">
       <c r="A99" s="6" t="inlineStr">
         <is>
-          <t>2026-06-16</t>
+          <t>2026-06-15</t>
         </is>
       </c>
       <c r="B99" s="6" t="inlineStr">
         <is>
-          <t>넥스트젠바이오</t>
+          <t>파워큐브세미</t>
         </is>
       </c>
       <c r="C99" s="6" t="inlineStr">
@@ -5686,32 +5686,32 @@
       </c>
       <c r="E99" s="6" t="inlineStr">
         <is>
-          <t>FY24</t>
+          <t>FY25</t>
         </is>
       </c>
       <c r="F99" s="7" t="inlineStr">
         <is>
-          <t>100</t>
+          <t>10,341</t>
         </is>
       </c>
       <c r="G99" s="7" t="inlineStr">
         <is>
-          <t>69</t>
+          <t>-10,837</t>
         </is>
       </c>
       <c r="H99" s="7" t="inlineStr">
         <is>
-          <t>4,792</t>
+          <t>841</t>
         </is>
       </c>
       <c r="I99" s="6" t="inlineStr">
         <is>
-          <t>자연과학 및 공학 연구개발업</t>
+          <t>반도체 제조업</t>
         </is>
       </c>
       <c r="J99" s="6" t="inlineStr">
         <is>
-          <t>한국</t>
+          <t>하나, BNK</t>
         </is>
       </c>
       <c r="K99" s="6" t="inlineStr">
@@ -5723,12 +5723,12 @@
     <row r="100">
       <c r="A100" s="6" t="inlineStr">
         <is>
-          <t>2026-06-15</t>
+          <t>2026-05-29</t>
         </is>
       </c>
       <c r="B100" s="6" t="inlineStr">
         <is>
-          <t>파워큐브세미</t>
+          <t>제이피이노베이션</t>
         </is>
       </c>
       <c r="C100" s="6" t="inlineStr">
@@ -5748,27 +5748,27 @@
       </c>
       <c r="F100" s="7" t="inlineStr">
         <is>
-          <t>10,341</t>
+          <t>56,324</t>
         </is>
       </c>
       <c r="G100" s="7" t="inlineStr">
         <is>
-          <t>-10,837</t>
+          <t>5,588</t>
         </is>
       </c>
       <c r="H100" s="7" t="inlineStr">
         <is>
-          <t>841</t>
+          <t>3,684</t>
         </is>
       </c>
       <c r="I100" s="6" t="inlineStr">
         <is>
-          <t>반도체 제조업</t>
+          <t>특수 목적용 기계 제조업</t>
         </is>
       </c>
       <c r="J100" s="6" t="inlineStr">
         <is>
-          <t>하나, BNK</t>
+          <t>삼성</t>
         </is>
       </c>
       <c r="K100" s="6" t="inlineStr">
@@ -5780,12 +5780,12 @@
     <row r="101">
       <c r="A101" s="6" t="inlineStr">
         <is>
-          <t>2026-05-29</t>
+          <t>2026-05-26</t>
         </is>
       </c>
       <c r="B101" s="6" t="inlineStr">
         <is>
-          <t>제이피이노베이션</t>
+          <t>케이솔루션</t>
         </is>
       </c>
       <c r="C101" s="6" t="inlineStr">
@@ -5795,7 +5795,7 @@
       </c>
       <c r="D101" s="6" t="inlineStr">
         <is>
-          <t>신규상장</t>
+          <t>스팩 존속합병</t>
         </is>
       </c>
       <c r="E101" s="6" t="inlineStr">
@@ -5805,27 +5805,27 @@
       </c>
       <c r="F101" s="7" t="inlineStr">
         <is>
-          <t>56,324</t>
+          <t>34,565</t>
         </is>
       </c>
       <c r="G101" s="7" t="inlineStr">
         <is>
-          <t>5,588</t>
+          <t>1,158</t>
         </is>
       </c>
       <c r="H101" s="7" t="inlineStr">
         <is>
-          <t>3,684</t>
+          <t>653</t>
         </is>
       </c>
       <c r="I101" s="6" t="inlineStr">
         <is>
-          <t>특수 목적용 기계 제조업</t>
+          <t>차체 및 특장차 제조업</t>
         </is>
       </c>
       <c r="J101" s="6" t="inlineStr">
         <is>
-          <t>삼성</t>
+          <t>DB</t>
         </is>
       </c>
       <c r="K101" s="6" t="inlineStr">
@@ -5837,12 +5837,12 @@
     <row r="102">
       <c r="A102" s="6" t="inlineStr">
         <is>
-          <t>2026-05-26</t>
+          <t>2026-04-30</t>
         </is>
       </c>
       <c r="B102" s="6" t="inlineStr">
         <is>
-          <t>케이솔루션</t>
+          <t>디토닉</t>
         </is>
       </c>
       <c r="C102" s="6" t="inlineStr">
@@ -5852,37 +5852,37 @@
       </c>
       <c r="D102" s="6" t="inlineStr">
         <is>
-          <t>스팩 존속합병</t>
+          <t>신규상장</t>
         </is>
       </c>
       <c r="E102" s="6" t="inlineStr">
         <is>
-          <t>FY25</t>
+          <t>FY24</t>
         </is>
       </c>
       <c r="F102" s="7" t="inlineStr">
         <is>
-          <t>34,565</t>
+          <t>31,293</t>
         </is>
       </c>
       <c r="G102" s="7" t="inlineStr">
         <is>
-          <t>1,158</t>
+          <t>-1,633</t>
         </is>
       </c>
       <c r="H102" s="7" t="inlineStr">
         <is>
-          <t>653</t>
+          <t>-21,926</t>
         </is>
       </c>
       <c r="I102" s="6" t="inlineStr">
         <is>
-          <t>차체 및 특장차 제조업</t>
+          <t>소프트웨어 개발 및 공급업</t>
         </is>
       </c>
       <c r="J102" s="6" t="inlineStr">
         <is>
-          <t>DB</t>
+          <t>NH</t>
         </is>
       </c>
       <c r="K102" s="6" t="inlineStr">
@@ -5894,12 +5894,12 @@
     <row r="103">
       <c r="A103" s="6" t="inlineStr">
         <is>
-          <t>2026-04-30</t>
+          <t>2026-04-22</t>
         </is>
       </c>
       <c r="B103" s="6" t="inlineStr">
         <is>
-          <t>디토닉</t>
+          <t>에스케이팩</t>
         </is>
       </c>
       <c r="C103" s="6" t="inlineStr">
@@ -5909,7 +5909,7 @@
       </c>
       <c r="D103" s="6" t="inlineStr">
         <is>
-          <t>신규상장</t>
+          <t>스팩 소멸합병</t>
         </is>
       </c>
       <c r="E103" s="6" t="inlineStr">
@@ -5919,27 +5919,27 @@
       </c>
       <c r="F103" s="7" t="inlineStr">
         <is>
-          <t>31,293</t>
+          <t>27,310</t>
         </is>
       </c>
       <c r="G103" s="7" t="inlineStr">
         <is>
-          <t>-1,633</t>
+          <t>2,257</t>
         </is>
       </c>
       <c r="H103" s="7" t="inlineStr">
         <is>
-          <t>-21,926</t>
+          <t>3,207</t>
         </is>
       </c>
       <c r="I103" s="6" t="inlineStr">
         <is>
-          <t>소프트웨어 개발 및 공급업</t>
+          <t>용기 세척, 포장 및 충전기 제조업</t>
         </is>
       </c>
       <c r="J103" s="6" t="inlineStr">
         <is>
-          <t>NH</t>
+          <t>교보</t>
         </is>
       </c>
       <c r="K103" s="6" t="inlineStr">
@@ -5951,12 +5951,12 @@
     <row r="104">
       <c r="A104" s="6" t="inlineStr">
         <is>
-          <t>2026-04-22</t>
+          <t>2026-04-20</t>
         </is>
       </c>
       <c r="B104" s="6" t="inlineStr">
         <is>
-          <t>에스케이팩</t>
+          <t>메타넷엑스</t>
         </is>
       </c>
       <c r="C104" s="6" t="inlineStr">
@@ -5966,7 +5966,7 @@
       </c>
       <c r="D104" s="6" t="inlineStr">
         <is>
-          <t>스팩 소멸합병</t>
+          <t>신규상장</t>
         </is>
       </c>
       <c r="E104" s="6" t="inlineStr">
@@ -5976,27 +5976,27 @@
       </c>
       <c r="F104" s="7" t="inlineStr">
         <is>
-          <t>27,310</t>
+          <t>244,130</t>
         </is>
       </c>
       <c r="G104" s="7" t="inlineStr">
         <is>
-          <t>2,257</t>
+          <t>13,455</t>
         </is>
       </c>
       <c r="H104" s="7" t="inlineStr">
         <is>
-          <t>3,207</t>
+          <t>9,995</t>
         </is>
       </c>
       <c r="I104" s="6" t="inlineStr">
         <is>
-          <t>용기 세척, 포장 및 충전기 제조업</t>
+          <t>컴퓨터 프로그래밍, 시스템 통합 및 관리업</t>
         </is>
       </c>
       <c r="J104" s="6" t="inlineStr">
         <is>
-          <t>교보</t>
+          <t>NH</t>
         </is>
       </c>
       <c r="K104" s="6" t="inlineStr">
@@ -6008,12 +6008,12 @@
     <row r="105">
       <c r="A105" s="6" t="inlineStr">
         <is>
-          <t>2026-04-20</t>
+          <t>2026-03-17</t>
         </is>
       </c>
       <c r="B105" s="6" t="inlineStr">
         <is>
-          <t>메타넷엑스</t>
+          <t>무아스</t>
         </is>
       </c>
       <c r="C105" s="6" t="inlineStr">
@@ -6023,7 +6023,7 @@
       </c>
       <c r="D105" s="6" t="inlineStr">
         <is>
-          <t>신규상장</t>
+          <t>스팩 소멸합병</t>
         </is>
       </c>
       <c r="E105" s="6" t="inlineStr">
@@ -6033,27 +6033,27 @@
       </c>
       <c r="F105" s="7" t="inlineStr">
         <is>
-          <t>244,130</t>
+          <t>41,813</t>
         </is>
       </c>
       <c r="G105" s="7" t="inlineStr">
         <is>
-          <t>13,455</t>
+          <t>3,903</t>
         </is>
       </c>
       <c r="H105" s="7" t="inlineStr">
         <is>
-          <t>9,995</t>
+          <t>532</t>
         </is>
       </c>
       <c r="I105" s="6" t="inlineStr">
         <is>
-          <t>컴퓨터 프로그래밍, 시스템 통합 및 관리업</t>
+          <t>가정용 전기기기 제조업</t>
         </is>
       </c>
       <c r="J105" s="6" t="inlineStr">
         <is>
-          <t>NH</t>
+          <t>신한</t>
         </is>
       </c>
       <c r="K105" s="6" t="inlineStr">
@@ -6070,7 +6070,7 @@
       </c>
       <c r="B106" s="6" t="inlineStr">
         <is>
-          <t>무아스</t>
+          <t>유빅스테라퓨틱스</t>
         </is>
       </c>
       <c r="C106" s="6" t="inlineStr">
@@ -6080,7 +6080,7 @@
       </c>
       <c r="D106" s="6" t="inlineStr">
         <is>
-          <t>스팩 소멸합병</t>
+          <t>신규상장</t>
         </is>
       </c>
       <c r="E106" s="6" t="inlineStr">
@@ -6090,27 +6090,27 @@
       </c>
       <c r="F106" s="7" t="inlineStr">
         <is>
-          <t>41,813</t>
+          <t>1,071</t>
         </is>
       </c>
       <c r="G106" s="7" t="inlineStr">
         <is>
-          <t>3,903</t>
+          <t>-15,145</t>
         </is>
       </c>
       <c r="H106" s="7" t="inlineStr">
         <is>
-          <t>532</t>
+          <t>5,489</t>
         </is>
       </c>
       <c r="I106" s="6" t="inlineStr">
         <is>
-          <t>가정용 전기기기 제조업</t>
+          <t>자연과학 및 공학 연구개발업</t>
         </is>
       </c>
       <c r="J106" s="6" t="inlineStr">
         <is>
-          <t>신한</t>
+          <t>대신</t>
         </is>
       </c>
       <c r="K106" s="6" t="inlineStr">
@@ -6122,12 +6122,12 @@
     <row r="107">
       <c r="A107" s="6" t="inlineStr">
         <is>
-          <t>2026-03-17</t>
+          <t>2026-03-16</t>
         </is>
       </c>
       <c r="B107" s="6" t="inlineStr">
         <is>
-          <t>유빅스테라퓨틱스</t>
+          <t>코드잇</t>
         </is>
       </c>
       <c r="C107" s="6" t="inlineStr">
@@ -6147,27 +6147,27 @@
       </c>
       <c r="F107" s="7" t="inlineStr">
         <is>
-          <t>1,071</t>
+          <t>30,747</t>
         </is>
       </c>
       <c r="G107" s="7" t="inlineStr">
         <is>
-          <t>-15,145</t>
+          <t>6,652</t>
         </is>
       </c>
       <c r="H107" s="7" t="inlineStr">
         <is>
-          <t>5,489</t>
+          <t>2,403</t>
         </is>
       </c>
       <c r="I107" s="6" t="inlineStr">
         <is>
-          <t>자연과학 및 공학 연구개발업</t>
+          <t>교육지원 서비스업</t>
         </is>
       </c>
       <c r="J107" s="6" t="inlineStr">
         <is>
-          <t>대신</t>
+          <t>미래</t>
         </is>
       </c>
       <c r="K107" s="6" t="inlineStr">
@@ -6179,12 +6179,12 @@
     <row r="108">
       <c r="A108" s="6" t="inlineStr">
         <is>
-          <t>2026-03-16</t>
+          <t>2026-02-05</t>
         </is>
       </c>
       <c r="B108" s="6" t="inlineStr">
         <is>
-          <t>코드잇</t>
+          <t>한컴인스페이스</t>
         </is>
       </c>
       <c r="C108" s="6" t="inlineStr">
@@ -6204,44 +6204,44 @@
       </c>
       <c r="F108" s="7" t="inlineStr">
         <is>
-          <t>30,747</t>
+          <t>23,492</t>
         </is>
       </c>
       <c r="G108" s="7" t="inlineStr">
         <is>
-          <t>6,652</t>
+          <t>-3,104</t>
         </is>
       </c>
       <c r="H108" s="7" t="inlineStr">
         <is>
-          <t>2,403</t>
+          <t>5,815</t>
         </is>
       </c>
       <c r="I108" s="6" t="inlineStr">
         <is>
-          <t>교육지원 서비스업</t>
+          <t>소프트웨어 개발 및 공급업</t>
         </is>
       </c>
       <c r="J108" s="6" t="inlineStr">
         <is>
-          <t>미래</t>
+          <t>대신</t>
         </is>
       </c>
       <c r="K108" s="6" t="inlineStr">
         <is>
-          <t>심사 철회</t>
+          <t>심사 미승인</t>
         </is>
       </c>
     </row>
     <row r="109">
       <c r="A109" s="6" t="inlineStr">
         <is>
-          <t>2026-02-05</t>
+          <t>2026-01-28</t>
         </is>
       </c>
       <c r="B109" s="6" t="inlineStr">
         <is>
-          <t>한컴인스페이스</t>
+          <t>크몽</t>
         </is>
       </c>
       <c r="C109" s="6" t="inlineStr">
@@ -6261,44 +6261,44 @@
       </c>
       <c r="F109" s="7" t="inlineStr">
         <is>
-          <t>23,492</t>
+          <t>48,572</t>
         </is>
       </c>
       <c r="G109" s="7" t="inlineStr">
         <is>
-          <t>-3,104</t>
+          <t>3,988</t>
         </is>
       </c>
       <c r="H109" s="7" t="inlineStr">
         <is>
-          <t>5,815</t>
+          <t>4,930</t>
         </is>
       </c>
       <c r="I109" s="6" t="inlineStr">
         <is>
-          <t>소프트웨어 개발 및 공급업</t>
+          <t>기타 정보 서비스업</t>
         </is>
       </c>
       <c r="J109" s="6" t="inlineStr">
         <is>
-          <t>대신</t>
+          <t>삼성</t>
         </is>
       </c>
       <c r="K109" s="6" t="inlineStr">
         <is>
-          <t>심사 미승인</t>
+          <t>심사 철회</t>
         </is>
       </c>
     </row>
     <row r="110">
       <c r="A110" s="6" t="inlineStr">
         <is>
-          <t>2026-01-28</t>
+          <t>2026-01-27</t>
         </is>
       </c>
       <c r="B110" s="6" t="inlineStr">
         <is>
-          <t>크몽</t>
+          <t>한화플러스제6호스팩</t>
         </is>
       </c>
       <c r="C110" s="6" t="inlineStr">
@@ -6318,27 +6318,27 @@
       </c>
       <c r="F110" s="7" t="inlineStr">
         <is>
-          <t>48,572</t>
+          <t>-</t>
         </is>
       </c>
       <c r="G110" s="7" t="inlineStr">
         <is>
-          <t>3,988</t>
+          <t>-</t>
         </is>
       </c>
       <c r="H110" s="7" t="inlineStr">
         <is>
-          <t>4,930</t>
+          <t>41</t>
         </is>
       </c>
       <c r="I110" s="6" t="inlineStr">
         <is>
-          <t>기타 정보 서비스업</t>
+          <t>기타 금융업</t>
         </is>
       </c>
       <c r="J110" s="6" t="inlineStr">
         <is>
-          <t>삼성</t>
+          <t>한화</t>
         </is>
       </c>
       <c r="K110" s="6" t="inlineStr">
@@ -6350,17 +6350,17 @@
     <row r="111">
       <c r="A111" s="6" t="inlineStr">
         <is>
-          <t>2026-01-27</t>
+          <t>2026-01-26</t>
         </is>
       </c>
       <c r="B111" s="6" t="inlineStr">
         <is>
-          <t>한화플러스제6호스팩</t>
+          <t>에식스솔루션즈</t>
         </is>
       </c>
       <c r="C111" s="6" t="inlineStr">
         <is>
-          <t>코스닥</t>
+          <t>유가</t>
         </is>
       </c>
       <c r="D111" s="6" t="inlineStr">
@@ -6375,27 +6375,27 @@
       </c>
       <c r="F111" s="7" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>2,461</t>
         </is>
       </c>
       <c r="G111" s="7" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>46</t>
         </is>
       </c>
       <c r="H111" s="7" t="inlineStr">
         <is>
-          <t>41</t>
+          <t>200</t>
         </is>
       </c>
       <c r="I111" s="6" t="inlineStr">
         <is>
-          <t>기타 금융업</t>
+          <t>절연선 및 케이블 제조업</t>
         </is>
       </c>
       <c r="J111" s="6" t="inlineStr">
         <is>
-          <t>한화</t>
+          <t>한국, 미래</t>
         </is>
       </c>
       <c r="K111" s="6" t="inlineStr">
@@ -6407,17 +6407,17 @@
     <row r="112">
       <c r="A112" s="6" t="inlineStr">
         <is>
-          <t>2026-01-26</t>
+          <t>2026-01-23</t>
         </is>
       </c>
       <c r="B112" s="6" t="inlineStr">
         <is>
-          <t>에식스솔루션즈</t>
+          <t>에코크레이션</t>
         </is>
       </c>
       <c r="C112" s="6" t="inlineStr">
         <is>
-          <t>유가</t>
+          <t>코스닥</t>
         </is>
       </c>
       <c r="D112" s="6" t="inlineStr">
@@ -6432,87 +6432,30 @@
       </c>
       <c r="F112" s="7" t="inlineStr">
         <is>
-          <t>2,461</t>
+          <t>18,544</t>
         </is>
       </c>
       <c r="G112" s="7" t="inlineStr">
         <is>
-          <t>46</t>
+          <t>-15,634</t>
         </is>
       </c>
       <c r="H112" s="7" t="inlineStr">
         <is>
-          <t>200</t>
+          <t>4,550</t>
         </is>
       </c>
       <c r="I112" s="6" t="inlineStr">
         <is>
-          <t>절연선 및 케이블 제조업</t>
+          <t>일반 목적용 기계 제조업</t>
         </is>
       </c>
       <c r="J112" s="6" t="inlineStr">
         <is>
-          <t>한국, 미래</t>
+          <t>키움</t>
         </is>
       </c>
       <c r="K112" s="6" t="inlineStr">
-        <is>
-          <t>심사 철회</t>
-        </is>
-      </c>
-    </row>
-    <row r="113">
-      <c r="A113" s="6" t="inlineStr">
-        <is>
-          <t>2026-01-23</t>
-        </is>
-      </c>
-      <c r="B113" s="6" t="inlineStr">
-        <is>
-          <t>에코크레이션</t>
-        </is>
-      </c>
-      <c r="C113" s="6" t="inlineStr">
-        <is>
-          <t>코스닥</t>
-        </is>
-      </c>
-      <c r="D113" s="6" t="inlineStr">
-        <is>
-          <t>신규상장</t>
-        </is>
-      </c>
-      <c r="E113" s="6" t="inlineStr">
-        <is>
-          <t>FY24</t>
-        </is>
-      </c>
-      <c r="F113" s="7" t="inlineStr">
-        <is>
-          <t>18,544</t>
-        </is>
-      </c>
-      <c r="G113" s="7" t="inlineStr">
-        <is>
-          <t>-15,634</t>
-        </is>
-      </c>
-      <c r="H113" s="7" t="inlineStr">
-        <is>
-          <t>4,550</t>
-        </is>
-      </c>
-      <c r="I113" s="6" t="inlineStr">
-        <is>
-          <t>일반 목적용 기계 제조업</t>
-        </is>
-      </c>
-      <c r="J113" s="6" t="inlineStr">
-        <is>
-          <t>키움</t>
-        </is>
-      </c>
-      <c r="K113" s="6" t="inlineStr">
         <is>
           <t>심사 철회</t>
         </is>
@@ -10296,7 +10239,7 @@
         <v>14</v>
       </c>
       <c r="C9" s="6" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="D9" s="6" t="n">
         <v>3</v>

</xml_diff>

<commit_message>
chore: update IPO data 2026-07-22
</commit_message>
<xml_diff>
--- a/IPO_analysis.xlsx
+++ b/IPO_analysis.xlsx
@@ -618,14 +618,14 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>기준일 2026-07-21 · 청구일 직전 사업연도 · 별도/개별 재무제표 · 단위 백만원(별도 표기 시 USD)</t>
+          <t>기준일 2026-07-22 · 청구일 직전 사업연도 · 별도/개별 재무제표 · 단위 백만원(별도 표기 시 USD)</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
-          <t>■ 심사 신청(진행중)  (51건)</t>
+          <t>■ 심사 신청(진행중)  (49건)</t>
         </is>
       </c>
       <c r="B4" s="4" t="n"/>
@@ -2117,7 +2117,7 @@
       </c>
       <c r="B31" s="6" t="inlineStr">
         <is>
-          <t>엔에이치스팩34호</t>
+          <t>유캐스트</t>
         </is>
       </c>
       <c r="C31" s="6" t="inlineStr">
@@ -2137,27 +2137,27 @@
       </c>
       <c r="F31" s="7" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>5,934</t>
         </is>
       </c>
       <c r="G31" s="7" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>-3,557</t>
         </is>
       </c>
       <c r="H31" s="7" t="inlineStr">
         <is>
-          <t>55</t>
+          <t>1,881</t>
         </is>
       </c>
       <c r="I31" s="6" t="inlineStr">
         <is>
-          <t>금융 지원 서비스업</t>
+          <t>통신 및 방송 장비 제조업</t>
         </is>
       </c>
       <c r="J31" s="6" t="inlineStr">
         <is>
-          <t>NH</t>
+          <t>유진</t>
         </is>
       </c>
       <c r="K31" s="6" t="inlineStr">
@@ -2174,7 +2174,7 @@
       </c>
       <c r="B32" s="6" t="inlineStr">
         <is>
-          <t>유캐스트</t>
+          <t>인터엑스</t>
         </is>
       </c>
       <c r="C32" s="6" t="inlineStr">
@@ -2194,27 +2194,27 @@
       </c>
       <c r="F32" s="7" t="inlineStr">
         <is>
-          <t>5,934</t>
+          <t>8,645</t>
         </is>
       </c>
       <c r="G32" s="7" t="inlineStr">
         <is>
-          <t>-3,557</t>
+          <t>-20,272</t>
         </is>
       </c>
       <c r="H32" s="7" t="inlineStr">
         <is>
-          <t>1,881</t>
+          <t>4,530</t>
         </is>
       </c>
       <c r="I32" s="6" t="inlineStr">
         <is>
-          <t>통신 및 방송 장비 제조업</t>
+          <t>소프트웨어 개발 및 공급업</t>
         </is>
       </c>
       <c r="J32" s="6" t="inlineStr">
         <is>
-          <t>유진</t>
+          <t>한국</t>
         </is>
       </c>
       <c r="K32" s="6" t="inlineStr">
@@ -2231,7 +2231,7 @@
       </c>
       <c r="B33" s="6" t="inlineStr">
         <is>
-          <t>인터엑스</t>
+          <t>케이엠에프</t>
         </is>
       </c>
       <c r="C33" s="6" t="inlineStr">
@@ -2251,27 +2251,27 @@
       </c>
       <c r="F33" s="7" t="inlineStr">
         <is>
-          <t>8,645</t>
+          <t>25,751</t>
         </is>
       </c>
       <c r="G33" s="7" t="inlineStr">
         <is>
-          <t>-20,272</t>
+          <t>11,463</t>
         </is>
       </c>
       <c r="H33" s="7" t="inlineStr">
         <is>
-          <t>4,530</t>
+          <t>642</t>
         </is>
       </c>
       <c r="I33" s="6" t="inlineStr">
         <is>
-          <t>소프트웨어 개발 및 공급업</t>
+          <t>기타 식품 제조업</t>
         </is>
       </c>
       <c r="J33" s="6" t="inlineStr">
         <is>
-          <t>한국</t>
+          <t>IBK</t>
         </is>
       </c>
       <c r="K33" s="6" t="inlineStr">
@@ -2288,7 +2288,7 @@
       </c>
       <c r="B34" s="6" t="inlineStr">
         <is>
-          <t>케이엠에프</t>
+          <t>하나에어로다이내믹스</t>
         </is>
       </c>
       <c r="C34" s="6" t="inlineStr">
@@ -2308,22 +2308,22 @@
       </c>
       <c r="F34" s="7" t="inlineStr">
         <is>
-          <t>25,751</t>
+          <t>33,286</t>
         </is>
       </c>
       <c r="G34" s="7" t="inlineStr">
         <is>
-          <t>11,463</t>
+          <t>2,420</t>
         </is>
       </c>
       <c r="H34" s="7" t="inlineStr">
         <is>
-          <t>642</t>
+          <t>890</t>
         </is>
       </c>
       <c r="I34" s="6" t="inlineStr">
         <is>
-          <t>기타 식품 제조업</t>
+          <t>항공기,우주선 및 부품 제조업</t>
         </is>
       </c>
       <c r="J34" s="6" t="inlineStr">
@@ -2340,12 +2340,12 @@
     <row r="35">
       <c r="A35" s="6" t="inlineStr">
         <is>
-          <t>2026-05-29</t>
+          <t>2026-05-28</t>
         </is>
       </c>
       <c r="B35" s="6" t="inlineStr">
         <is>
-          <t>하나에어로다이내믹스</t>
+          <t>다비오</t>
         </is>
       </c>
       <c r="C35" s="6" t="inlineStr">
@@ -2365,27 +2365,27 @@
       </c>
       <c r="F35" s="7" t="inlineStr">
         <is>
-          <t>33,286</t>
+          <t>9,251</t>
         </is>
       </c>
       <c r="G35" s="7" t="inlineStr">
         <is>
-          <t>2,420</t>
+          <t>-3,473</t>
         </is>
       </c>
       <c r="H35" s="7" t="inlineStr">
         <is>
-          <t>890</t>
+          <t>300</t>
         </is>
       </c>
       <c r="I35" s="6" t="inlineStr">
         <is>
-          <t>항공기,우주선 및 부품 제조업</t>
+          <t>소프트웨어 개발 및 공급업</t>
         </is>
       </c>
       <c r="J35" s="6" t="inlineStr">
         <is>
-          <t>IBK</t>
+          <t>대신</t>
         </is>
       </c>
       <c r="K35" s="6" t="inlineStr">
@@ -2402,7 +2402,7 @@
       </c>
       <c r="B36" s="6" t="inlineStr">
         <is>
-          <t>다비오</t>
+          <t>삼홍아크튜리온</t>
         </is>
       </c>
       <c r="C36" s="6" t="inlineStr">
@@ -2422,27 +2422,27 @@
       </c>
       <c r="F36" s="7" t="inlineStr">
         <is>
-          <t>9,251</t>
+          <t>26,162</t>
         </is>
       </c>
       <c r="G36" s="7" t="inlineStr">
         <is>
-          <t>-3,473</t>
+          <t>-10,314</t>
         </is>
       </c>
       <c r="H36" s="7" t="inlineStr">
         <is>
-          <t>300</t>
+          <t>6,369</t>
         </is>
       </c>
       <c r="I36" s="6" t="inlineStr">
         <is>
-          <t>소프트웨어 개발 및 공급업</t>
+          <t>구조용 금속제품, 탱크 및 증기발생기 제조업</t>
         </is>
       </c>
       <c r="J36" s="6" t="inlineStr">
         <is>
-          <t>대신</t>
+          <t>삼성, 미래</t>
         </is>
       </c>
       <c r="K36" s="6" t="inlineStr">
@@ -2454,12 +2454,12 @@
     <row r="37">
       <c r="A37" s="6" t="inlineStr">
         <is>
-          <t>2026-05-28</t>
+          <t>2026-05-22</t>
         </is>
       </c>
       <c r="B37" s="6" t="inlineStr">
         <is>
-          <t>삼홍아크튜리온</t>
+          <t>에이엘로봇</t>
         </is>
       </c>
       <c r="C37" s="6" t="inlineStr">
@@ -2479,27 +2479,27 @@
       </c>
       <c r="F37" s="7" t="inlineStr">
         <is>
-          <t>26,162</t>
+          <t>14,985</t>
         </is>
       </c>
       <c r="G37" s="7" t="inlineStr">
         <is>
-          <t>-10,314</t>
+          <t>-21,891</t>
         </is>
       </c>
       <c r="H37" s="7" t="inlineStr">
         <is>
-          <t>6,369</t>
+          <t>129</t>
         </is>
       </c>
       <c r="I37" s="6" t="inlineStr">
         <is>
-          <t>구조용 금속제품, 탱크 및 증기발생기 제조업</t>
+          <t>산업용 로봇 제조업</t>
         </is>
       </c>
       <c r="J37" s="6" t="inlineStr">
         <is>
-          <t>삼성, 미래</t>
+          <t>대신</t>
         </is>
       </c>
       <c r="K37" s="6" t="inlineStr">
@@ -2511,12 +2511,12 @@
     <row r="38">
       <c r="A38" s="6" t="inlineStr">
         <is>
-          <t>2026-05-22</t>
+          <t>2026-05-21</t>
         </is>
       </c>
       <c r="B38" s="6" t="inlineStr">
         <is>
-          <t>에이엘로봇</t>
+          <t>넥스트에어로스페이스</t>
         </is>
       </c>
       <c r="C38" s="6" t="inlineStr">
@@ -2536,27 +2536,27 @@
       </c>
       <c r="F38" s="7" t="inlineStr">
         <is>
-          <t>14,985</t>
+          <t>12,084</t>
         </is>
       </c>
       <c r="G38" s="7" t="inlineStr">
         <is>
-          <t>-21,891</t>
+          <t>-17,270</t>
         </is>
       </c>
       <c r="H38" s="7" t="inlineStr">
         <is>
-          <t>129</t>
+          <t>6,158</t>
         </is>
       </c>
       <c r="I38" s="6" t="inlineStr">
         <is>
-          <t>산업용 로봇 제조업</t>
+          <t>유인 항공기, 항공우주선 및 보조장치 제조업</t>
         </is>
       </c>
       <c r="J38" s="6" t="inlineStr">
         <is>
-          <t>대신</t>
+          <t>삼성</t>
         </is>
       </c>
       <c r="K38" s="6" t="inlineStr">
@@ -2573,7 +2573,7 @@
       </c>
       <c r="B39" s="6" t="inlineStr">
         <is>
-          <t>넥스트에어로스페이스</t>
+          <t>래블업</t>
         </is>
       </c>
       <c r="C39" s="6" t="inlineStr">
@@ -2593,27 +2593,27 @@
       </c>
       <c r="F39" s="7" t="inlineStr">
         <is>
-          <t>12,084</t>
+          <t>6,712</t>
         </is>
       </c>
       <c r="G39" s="7" t="inlineStr">
         <is>
-          <t>-17,270</t>
+          <t>-1,526</t>
         </is>
       </c>
       <c r="H39" s="7" t="inlineStr">
         <is>
-          <t>6,158</t>
+          <t>373</t>
         </is>
       </c>
       <c r="I39" s="6" t="inlineStr">
         <is>
-          <t>유인 항공기, 항공우주선 및 보조장치 제조업</t>
+          <t>데이터베이스 및 온라인정보 제공업</t>
         </is>
       </c>
       <c r="J39" s="6" t="inlineStr">
         <is>
-          <t>삼성</t>
+          <t>NH</t>
         </is>
       </c>
       <c r="K39" s="6" t="inlineStr">
@@ -2630,7 +2630,7 @@
       </c>
       <c r="B40" s="6" t="inlineStr">
         <is>
-          <t>래블업</t>
+          <t>비앤비코리아</t>
         </is>
       </c>
       <c r="C40" s="6" t="inlineStr">
@@ -2650,27 +2650,27 @@
       </c>
       <c r="F40" s="7" t="inlineStr">
         <is>
-          <t>6,712</t>
+          <t>141,169</t>
         </is>
       </c>
       <c r="G40" s="7" t="inlineStr">
         <is>
-          <t>-1,526</t>
+          <t>21,406</t>
         </is>
       </c>
       <c r="H40" s="7" t="inlineStr">
         <is>
-          <t>373</t>
+          <t>43,932</t>
         </is>
       </c>
       <c r="I40" s="6" t="inlineStr">
         <is>
-          <t>데이터베이스 및 온라인정보 제공업</t>
+          <t>기타 화학제품 제조업</t>
         </is>
       </c>
       <c r="J40" s="6" t="inlineStr">
         <is>
-          <t>NH</t>
+          <t>미래</t>
         </is>
       </c>
       <c r="K40" s="6" t="inlineStr">
@@ -2687,7 +2687,7 @@
       </c>
       <c r="B41" s="6" t="inlineStr">
         <is>
-          <t>비앤비코리아</t>
+          <t>에이엔에이치스트럭쳐</t>
         </is>
       </c>
       <c r="C41" s="6" t="inlineStr">
@@ -2707,27 +2707,27 @@
       </c>
       <c r="F41" s="7" t="inlineStr">
         <is>
-          <t>141,169</t>
+          <t>19,784</t>
         </is>
       </c>
       <c r="G41" s="7" t="inlineStr">
         <is>
-          <t>21,406</t>
+          <t>-4,296</t>
         </is>
       </c>
       <c r="H41" s="7" t="inlineStr">
         <is>
-          <t>43,932</t>
+          <t>24,561</t>
         </is>
       </c>
       <c r="I41" s="6" t="inlineStr">
         <is>
-          <t>기타 화학제품 제조업</t>
+          <t>건축기술, 엔지니어링 및 관련 기술 서비스업</t>
         </is>
       </c>
       <c r="J41" s="6" t="inlineStr">
         <is>
-          <t>미래</t>
+          <t>NH</t>
         </is>
       </c>
       <c r="K41" s="6" t="inlineStr">
@@ -2739,12 +2739,12 @@
     <row r="42">
       <c r="A42" s="6" t="inlineStr">
         <is>
-          <t>2026-05-21</t>
+          <t>2026-05-19</t>
         </is>
       </c>
       <c r="B42" s="6" t="inlineStr">
         <is>
-          <t>에이엔에이치스트럭쳐</t>
+          <t>엘리스그룹</t>
         </is>
       </c>
       <c r="C42" s="6" t="inlineStr">
@@ -2764,27 +2764,27 @@
       </c>
       <c r="F42" s="7" t="inlineStr">
         <is>
-          <t>19,784</t>
+          <t>39,513</t>
         </is>
       </c>
       <c r="G42" s="7" t="inlineStr">
         <is>
-          <t>-4,296</t>
+          <t>15,666</t>
         </is>
       </c>
       <c r="H42" s="7" t="inlineStr">
         <is>
-          <t>24,561</t>
+          <t>85,400</t>
         </is>
       </c>
       <c r="I42" s="6" t="inlineStr">
         <is>
-          <t>건축기술, 엔지니어링 및 관련 기술 서비스업</t>
+          <t>소프트웨어 개발 및 공급업</t>
         </is>
       </c>
       <c r="J42" s="6" t="inlineStr">
         <is>
-          <t>NH</t>
+          <t>미래, 삼성</t>
         </is>
       </c>
       <c r="K42" s="6" t="inlineStr">
@@ -2796,12 +2796,12 @@
     <row r="43">
       <c r="A43" s="6" t="inlineStr">
         <is>
-          <t>2026-05-19</t>
+          <t>2026-05-12</t>
         </is>
       </c>
       <c r="B43" s="6" t="inlineStr">
         <is>
-          <t>엘리스그룹</t>
+          <t>오토핸즈</t>
         </is>
       </c>
       <c r="C43" s="6" t="inlineStr">
@@ -2811,7 +2811,7 @@
       </c>
       <c r="D43" s="6" t="inlineStr">
         <is>
-          <t>신규상장</t>
+          <t>스팩 소멸합병</t>
         </is>
       </c>
       <c r="E43" s="6" t="inlineStr">
@@ -2821,27 +2821,27 @@
       </c>
       <c r="F43" s="7" t="inlineStr">
         <is>
-          <t>39,513</t>
+          <t>238,564</t>
         </is>
       </c>
       <c r="G43" s="7" t="inlineStr">
         <is>
-          <t>15,666</t>
+          <t>6,047</t>
         </is>
       </c>
       <c r="H43" s="7" t="inlineStr">
         <is>
-          <t>85,400</t>
+          <t>6,129</t>
         </is>
       </c>
       <c r="I43" s="6" t="inlineStr">
         <is>
-          <t>소프트웨어 개발 및 공급업</t>
+          <t>자동차 판매업</t>
         </is>
       </c>
       <c r="J43" s="6" t="inlineStr">
         <is>
-          <t>미래, 삼성</t>
+          <t>미래</t>
         </is>
       </c>
       <c r="K43" s="6" t="inlineStr">
@@ -2853,12 +2853,12 @@
     <row r="44">
       <c r="A44" s="6" t="inlineStr">
         <is>
-          <t>2026-05-12</t>
+          <t>2026-05-06</t>
         </is>
       </c>
       <c r="B44" s="6" t="inlineStr">
         <is>
-          <t>오토핸즈</t>
+          <t>아이벡스메디칼시스템즈</t>
         </is>
       </c>
       <c r="C44" s="6" t="inlineStr">
@@ -2868,7 +2868,7 @@
       </c>
       <c r="D44" s="6" t="inlineStr">
         <is>
-          <t>스팩 소멸합병</t>
+          <t>신규상장</t>
         </is>
       </c>
       <c r="E44" s="6" t="inlineStr">
@@ -2878,27 +2878,27 @@
       </c>
       <c r="F44" s="7" t="inlineStr">
         <is>
-          <t>238,564</t>
+          <t>15,282</t>
         </is>
       </c>
       <c r="G44" s="7" t="inlineStr">
         <is>
-          <t>6,047</t>
+          <t>-7,227</t>
         </is>
       </c>
       <c r="H44" s="7" t="inlineStr">
         <is>
-          <t>6,129</t>
+          <t>744</t>
         </is>
       </c>
       <c r="I44" s="6" t="inlineStr">
         <is>
-          <t>자동차 판매업</t>
+          <t>의료용 기기 제조업</t>
         </is>
       </c>
       <c r="J44" s="6" t="inlineStr">
         <is>
-          <t>미래</t>
+          <t>NH</t>
         </is>
       </c>
       <c r="K44" s="6" t="inlineStr">
@@ -2910,12 +2910,12 @@
     <row r="45">
       <c r="A45" s="6" t="inlineStr">
         <is>
-          <t>2026-05-06</t>
+          <t>2026-04-30</t>
         </is>
       </c>
       <c r="B45" s="6" t="inlineStr">
         <is>
-          <t>아이벡스메디칼시스템즈</t>
+          <t>멜콘</t>
         </is>
       </c>
       <c r="C45" s="6" t="inlineStr">
@@ -2935,27 +2935,27 @@
       </c>
       <c r="F45" s="7" t="inlineStr">
         <is>
-          <t>15,282</t>
+          <t>39,319</t>
         </is>
       </c>
       <c r="G45" s="7" t="inlineStr">
         <is>
-          <t>-7,227</t>
+          <t>4,739</t>
         </is>
       </c>
       <c r="H45" s="7" t="inlineStr">
         <is>
-          <t>744</t>
+          <t>1,250</t>
         </is>
       </c>
       <c r="I45" s="6" t="inlineStr">
         <is>
-          <t>의료용 기기 제조업</t>
+          <t>특수 목적용 기계 제조업</t>
         </is>
       </c>
       <c r="J45" s="6" t="inlineStr">
         <is>
-          <t>NH</t>
+          <t>대신</t>
         </is>
       </c>
       <c r="K45" s="6" t="inlineStr">
@@ -2972,7 +2972,7 @@
       </c>
       <c r="B46" s="6" t="inlineStr">
         <is>
-          <t>멜콘</t>
+          <t>모비어스</t>
         </is>
       </c>
       <c r="C46" s="6" t="inlineStr">
@@ -2992,27 +2992,27 @@
       </c>
       <c r="F46" s="7" t="inlineStr">
         <is>
-          <t>39,319</t>
+          <t>31,989</t>
         </is>
       </c>
       <c r="G46" s="7" t="inlineStr">
         <is>
-          <t>4,739</t>
+          <t>-45,307</t>
         </is>
       </c>
       <c r="H46" s="7" t="inlineStr">
         <is>
-          <t>1,250</t>
+          <t>-96,707</t>
         </is>
       </c>
       <c r="I46" s="6" t="inlineStr">
         <is>
-          <t>특수 목적용 기계 제조업</t>
+          <t>컴퓨터 프로그래밍, 시스템 통합 및 관리업</t>
         </is>
       </c>
       <c r="J46" s="6" t="inlineStr">
         <is>
-          <t>대신</t>
+          <t>미래</t>
         </is>
       </c>
       <c r="K46" s="6" t="inlineStr">
@@ -3029,7 +3029,7 @@
       </c>
       <c r="B47" s="6" t="inlineStr">
         <is>
-          <t>모비어스</t>
+          <t>바로팜</t>
         </is>
       </c>
       <c r="C47" s="6" t="inlineStr">
@@ -3049,22 +3049,22 @@
       </c>
       <c r="F47" s="7" t="inlineStr">
         <is>
-          <t>31,989</t>
+          <t>96,724</t>
         </is>
       </c>
       <c r="G47" s="7" t="inlineStr">
         <is>
-          <t>-45,307</t>
+          <t>-9,679</t>
         </is>
       </c>
       <c r="H47" s="7" t="inlineStr">
         <is>
-          <t>-96,707</t>
+          <t>30,673</t>
         </is>
       </c>
       <c r="I47" s="6" t="inlineStr">
         <is>
-          <t>컴퓨터 프로그래밍, 시스템 통합 및 관리업</t>
+          <t>상품 중개업</t>
         </is>
       </c>
       <c r="J47" s="6" t="inlineStr">
@@ -3086,7 +3086,7 @@
       </c>
       <c r="B48" s="6" t="inlineStr">
         <is>
-          <t>바로팜</t>
+          <t>텔레픽스</t>
         </is>
       </c>
       <c r="C48" s="6" t="inlineStr">
@@ -3106,22 +3106,22 @@
       </c>
       <c r="F48" s="7" t="inlineStr">
         <is>
-          <t>96,724</t>
+          <t>4,896</t>
         </is>
       </c>
       <c r="G48" s="7" t="inlineStr">
         <is>
-          <t>-9,679</t>
+          <t>-16,214</t>
         </is>
       </c>
       <c r="H48" s="7" t="inlineStr">
         <is>
-          <t>30,673</t>
+          <t>9,146</t>
         </is>
       </c>
       <c r="I48" s="6" t="inlineStr">
         <is>
-          <t>상품 중개업</t>
+          <t>소프트웨어 개발 및 공급업</t>
         </is>
       </c>
       <c r="J48" s="6" t="inlineStr">
@@ -3138,12 +3138,12 @@
     <row r="49">
       <c r="A49" s="6" t="inlineStr">
         <is>
-          <t>2026-04-30</t>
+          <t>2026-04-10</t>
         </is>
       </c>
       <c r="B49" s="6" t="inlineStr">
         <is>
-          <t>텔레픽스</t>
+          <t>엠비디</t>
         </is>
       </c>
       <c r="C49" s="6" t="inlineStr">
@@ -3163,27 +3163,27 @@
       </c>
       <c r="F49" s="7" t="inlineStr">
         <is>
-          <t>4,896</t>
+          <t>1,524</t>
         </is>
       </c>
       <c r="G49" s="7" t="inlineStr">
         <is>
-          <t>-16,214</t>
+          <t>-2,125</t>
         </is>
       </c>
       <c r="H49" s="7" t="inlineStr">
         <is>
-          <t>9,146</t>
+          <t>2,753</t>
         </is>
       </c>
       <c r="I49" s="6" t="inlineStr">
         <is>
-          <t>소프트웨어 개발 및 공급업</t>
+          <t>물질 검사, 측정 및 분석기구 제조업</t>
         </is>
       </c>
       <c r="J49" s="6" t="inlineStr">
         <is>
-          <t>미래</t>
+          <t>하나</t>
         </is>
       </c>
       <c r="K49" s="6" t="inlineStr">
@@ -3195,12 +3195,12 @@
     <row r="50">
       <c r="A50" s="6" t="inlineStr">
         <is>
-          <t>2026-04-10</t>
+          <t>2026-04-08</t>
         </is>
       </c>
       <c r="B50" s="6" t="inlineStr">
         <is>
-          <t>엠비디</t>
+          <t>옵토닉스</t>
         </is>
       </c>
       <c r="C50" s="6" t="inlineStr">
@@ -3220,27 +3220,27 @@
       </c>
       <c r="F50" s="7" t="inlineStr">
         <is>
-          <t>1,524</t>
+          <t>25,368</t>
         </is>
       </c>
       <c r="G50" s="7" t="inlineStr">
         <is>
-          <t>-2,125</t>
+          <t>1,901</t>
         </is>
       </c>
       <c r="H50" s="7" t="inlineStr">
         <is>
-          <t>2,753</t>
+          <t>730</t>
         </is>
       </c>
       <c r="I50" s="6" t="inlineStr">
         <is>
-          <t>물질 검사, 측정 및 분석기구 제조업</t>
+          <t>광학렌즈 및 광학요소 제조업</t>
         </is>
       </c>
       <c r="J50" s="6" t="inlineStr">
         <is>
-          <t>하나</t>
+          <t>한국</t>
         </is>
       </c>
       <c r="K50" s="6" t="inlineStr">
@@ -3252,12 +3252,12 @@
     <row r="51">
       <c r="A51" s="6" t="inlineStr">
         <is>
-          <t>2026-04-08</t>
+          <t>2026-04-07</t>
         </is>
       </c>
       <c r="B51" s="6" t="inlineStr">
         <is>
-          <t>옵토닉스</t>
+          <t>크리에이츠</t>
         </is>
       </c>
       <c r="C51" s="6" t="inlineStr">
@@ -3277,27 +3277,27 @@
       </c>
       <c r="F51" s="7" t="inlineStr">
         <is>
-          <t>25,368</t>
+          <t>76,395</t>
         </is>
       </c>
       <c r="G51" s="7" t="inlineStr">
         <is>
-          <t>1,901</t>
+          <t>23,749</t>
         </is>
       </c>
       <c r="H51" s="7" t="inlineStr">
         <is>
-          <t>730</t>
+          <t>2,335</t>
         </is>
       </c>
       <c r="I51" s="6" t="inlineStr">
         <is>
-          <t>광학렌즈 및 광학요소 제조업</t>
+          <t>그외 기타 제품 제조업</t>
         </is>
       </c>
       <c r="J51" s="6" t="inlineStr">
         <is>
-          <t>한국</t>
+          <t>삼성</t>
         </is>
       </c>
       <c r="K51" s="6" t="inlineStr">
@@ -3309,12 +3309,12 @@
     <row r="52">
       <c r="A52" s="6" t="inlineStr">
         <is>
-          <t>2026-04-07</t>
+          <t>2026-03-24</t>
         </is>
       </c>
       <c r="B52" s="6" t="inlineStr">
         <is>
-          <t>크리에이츠</t>
+          <t>인텔리빅스</t>
         </is>
       </c>
       <c r="C52" s="6" t="inlineStr">
@@ -3334,27 +3334,27 @@
       </c>
       <c r="F52" s="7" t="inlineStr">
         <is>
-          <t>76,395</t>
+          <t>46,644</t>
         </is>
       </c>
       <c r="G52" s="7" t="inlineStr">
         <is>
-          <t>23,749</t>
+          <t>5,357</t>
         </is>
       </c>
       <c r="H52" s="7" t="inlineStr">
         <is>
-          <t>2,335</t>
+          <t>1,048</t>
         </is>
       </c>
       <c r="I52" s="6" t="inlineStr">
         <is>
-          <t>그외 기타 제품 제조업</t>
+          <t>소프트웨어 개발 및 공급업</t>
         </is>
       </c>
       <c r="J52" s="6" t="inlineStr">
         <is>
-          <t>삼성</t>
+          <t>미래</t>
         </is>
       </c>
       <c r="K52" s="6" t="inlineStr">
@@ -3366,12 +3366,12 @@
     <row r="53">
       <c r="A53" s="6" t="inlineStr">
         <is>
-          <t>2026-03-24</t>
+          <t>2026-02-27</t>
         </is>
       </c>
       <c r="B53" s="6" t="inlineStr">
         <is>
-          <t>인텔리빅스</t>
+          <t>피지티</t>
         </is>
       </c>
       <c r="C53" s="6" t="inlineStr">
@@ -3391,27 +3391,27 @@
       </c>
       <c r="F53" s="7" t="inlineStr">
         <is>
-          <t>46,644</t>
+          <t>40,141</t>
         </is>
       </c>
       <c r="G53" s="7" t="inlineStr">
         <is>
-          <t>5,357</t>
+          <t>-69,722</t>
         </is>
       </c>
       <c r="H53" s="7" t="inlineStr">
         <is>
-          <t>1,048</t>
+          <t>6,029</t>
         </is>
       </c>
       <c r="I53" s="6" t="inlineStr">
         <is>
-          <t>소프트웨어 개발 및 공급업</t>
+          <t>기타 화학제품 제조업</t>
         </is>
       </c>
       <c r="J53" s="6" t="inlineStr">
         <is>
-          <t>미래</t>
+          <t>한국</t>
         </is>
       </c>
       <c r="K53" s="6" t="inlineStr">
@@ -3423,12 +3423,12 @@
     <row r="54">
       <c r="A54" s="6" t="inlineStr">
         <is>
-          <t>2026-02-27</t>
+          <t>2025-09-11</t>
         </is>
       </c>
       <c r="B54" s="6" t="inlineStr">
         <is>
-          <t>피지티</t>
+          <t>씨엠디엘</t>
         </is>
       </c>
       <c r="C54" s="6" t="inlineStr">
@@ -3438,230 +3438,230 @@
       </c>
       <c r="D54" s="6" t="inlineStr">
         <is>
+          <t>스팩 소멸합병</t>
+        </is>
+      </c>
+      <c r="E54" s="6" t="inlineStr">
+        <is>
+          <t>FY24</t>
+        </is>
+      </c>
+      <c r="F54" s="7" t="inlineStr">
+        <is>
+          <t>39,991</t>
+        </is>
+      </c>
+      <c r="G54" s="7" t="inlineStr">
+        <is>
+          <t>3,541</t>
+        </is>
+      </c>
+      <c r="H54" s="7" t="inlineStr">
+        <is>
+          <t>503</t>
+        </is>
+      </c>
+      <c r="I54" s="6" t="inlineStr">
+        <is>
+          <t>기타 기초 유기 화학물질 제조업</t>
+        </is>
+      </c>
+      <c r="J54" s="6" t="inlineStr">
+        <is>
+          <t>교보</t>
+        </is>
+      </c>
+      <c r="K54" s="6" t="inlineStr">
+        <is>
+          <t>예심 진행중</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="3" t="inlineStr">
+        <is>
+          <t>■ 심사 승인  (39건)</t>
+        </is>
+      </c>
+      <c r="B56" s="4" t="n"/>
+      <c r="C56" s="4" t="n"/>
+      <c r="D56" s="4" t="n"/>
+      <c r="E56" s="4" t="n"/>
+      <c r="F56" s="4" t="n"/>
+      <c r="G56" s="4" t="n"/>
+      <c r="H56" s="4" t="n"/>
+      <c r="I56" s="4" t="n"/>
+      <c r="J56" s="4" t="n"/>
+      <c r="K56" s="4" t="n"/>
+    </row>
+    <row r="57">
+      <c r="A57" s="5" t="inlineStr">
+        <is>
+          <t>일자</t>
+        </is>
+      </c>
+      <c r="B57" s="5" t="inlineStr">
+        <is>
+          <t>회사명</t>
+        </is>
+      </c>
+      <c r="C57" s="5" t="inlineStr">
+        <is>
+          <t>시장</t>
+        </is>
+      </c>
+      <c r="D57" s="5" t="inlineStr">
+        <is>
+          <t>상장유형</t>
+        </is>
+      </c>
+      <c r="E57" s="5" t="inlineStr">
+        <is>
+          <t>기준연도</t>
+        </is>
+      </c>
+      <c r="F57" s="5" t="inlineStr">
+        <is>
+          <t>매출액</t>
+        </is>
+      </c>
+      <c r="G57" s="5" t="inlineStr">
+        <is>
+          <t>순이익</t>
+        </is>
+      </c>
+      <c r="H57" s="5" t="inlineStr">
+        <is>
+          <t>자기자본</t>
+        </is>
+      </c>
+      <c r="I57" s="5" t="inlineStr">
+        <is>
+          <t>업종</t>
+        </is>
+      </c>
+      <c r="J57" s="5" t="inlineStr">
+        <is>
+          <t>대표주관사</t>
+        </is>
+      </c>
+      <c r="K57" s="5" t="inlineStr">
+        <is>
+          <t>현황</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="6" t="inlineStr">
+        <is>
+          <t>2026-07-22</t>
+        </is>
+      </c>
+      <c r="B58" s="6" t="inlineStr">
+        <is>
+          <t>엔에이치스팩34호</t>
+        </is>
+      </c>
+      <c r="C58" s="6" t="inlineStr">
+        <is>
+          <t>코스닥</t>
+        </is>
+      </c>
+      <c r="D58" s="6" t="inlineStr">
+        <is>
           <t>신규상장</t>
         </is>
       </c>
-      <c r="E54" s="6" t="inlineStr">
+      <c r="E58" s="6" t="inlineStr">
         <is>
           <t>FY25</t>
         </is>
       </c>
-      <c r="F54" s="7" t="inlineStr">
-        <is>
-          <t>40,141</t>
-        </is>
-      </c>
-      <c r="G54" s="7" t="inlineStr">
-        <is>
-          <t>-69,722</t>
-        </is>
-      </c>
-      <c r="H54" s="7" t="inlineStr">
-        <is>
-          <t>6,029</t>
-        </is>
-      </c>
-      <c r="I54" s="6" t="inlineStr">
-        <is>
-          <t>기타 화학제품 제조업</t>
-        </is>
-      </c>
-      <c r="J54" s="6" t="inlineStr">
-        <is>
-          <t>한국</t>
-        </is>
-      </c>
-      <c r="K54" s="6" t="inlineStr">
-        <is>
-          <t>예심 진행중</t>
-        </is>
-      </c>
-    </row>
-    <row r="55">
-      <c r="A55" s="6" t="inlineStr">
-        <is>
-          <t>2025-09-18</t>
-        </is>
-      </c>
-      <c r="B55" s="6" t="inlineStr">
-        <is>
-          <t>디티에스</t>
-        </is>
-      </c>
-      <c r="C55" s="6" t="inlineStr">
+      <c r="F58" s="7" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G58" s="7" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H58" s="7" t="inlineStr">
+        <is>
+          <t>55</t>
+        </is>
+      </c>
+      <c r="I58" s="6" t="inlineStr">
+        <is>
+          <t>금융 지원 서비스업</t>
+        </is>
+      </c>
+      <c r="J58" s="6" t="inlineStr">
+        <is>
+          <t>NH</t>
+        </is>
+      </c>
+      <c r="K58" s="6" t="inlineStr">
+        <is>
+          <t>상장전</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="6" t="inlineStr">
+        <is>
+          <t>2026-07-20</t>
+        </is>
+      </c>
+      <c r="B59" s="6" t="inlineStr">
+        <is>
+          <t>덕산넵코어스</t>
+        </is>
+      </c>
+      <c r="C59" s="6" t="inlineStr">
         <is>
           <t>코스닥</t>
         </is>
       </c>
-      <c r="D55" s="6" t="inlineStr">
+      <c r="D59" s="6" t="inlineStr">
         <is>
           <t>신규상장</t>
         </is>
       </c>
-      <c r="E55" s="6" t="inlineStr">
+      <c r="E59" s="6" t="inlineStr">
         <is>
           <t>FY24</t>
         </is>
       </c>
-      <c r="F55" s="7" t="inlineStr">
-        <is>
-          <t>142,718</t>
-        </is>
-      </c>
-      <c r="G55" s="7" t="inlineStr">
-        <is>
-          <t>18,765</t>
-        </is>
-      </c>
-      <c r="H55" s="7" t="inlineStr">
-        <is>
-          <t>63,153</t>
-        </is>
-      </c>
-      <c r="I55" s="6" t="inlineStr">
-        <is>
-          <t>특수 목적용 기계 제조업</t>
-        </is>
-      </c>
-      <c r="J55" s="6" t="inlineStr">
+      <c r="F59" s="7" t="inlineStr">
+        <is>
+          <t>48,504</t>
+        </is>
+      </c>
+      <c r="G59" s="7" t="inlineStr">
+        <is>
+          <t>3,668</t>
+        </is>
+      </c>
+      <c r="H59" s="7" t="inlineStr">
+        <is>
+          <t>8,448</t>
+        </is>
+      </c>
+      <c r="I59" s="6" t="inlineStr">
+        <is>
+          <t>항공기,우주선 및 부품 제조업</t>
+        </is>
+      </c>
+      <c r="J59" s="6" t="inlineStr">
         <is>
           <t>대신</t>
         </is>
       </c>
-      <c r="K55" s="6" t="inlineStr">
-        <is>
-          <t>예심 진행중</t>
-        </is>
-      </c>
-    </row>
-    <row r="56">
-      <c r="A56" s="6" t="inlineStr">
-        <is>
-          <t>2025-09-11</t>
-        </is>
-      </c>
-      <c r="B56" s="6" t="inlineStr">
-        <is>
-          <t>씨엠디엘</t>
-        </is>
-      </c>
-      <c r="C56" s="6" t="inlineStr">
-        <is>
-          <t>코스닥</t>
-        </is>
-      </c>
-      <c r="D56" s="6" t="inlineStr">
-        <is>
-          <t>스팩 소멸합병</t>
-        </is>
-      </c>
-      <c r="E56" s="6" t="inlineStr">
-        <is>
-          <t>FY24</t>
-        </is>
-      </c>
-      <c r="F56" s="7" t="inlineStr">
-        <is>
-          <t>39,991</t>
-        </is>
-      </c>
-      <c r="G56" s="7" t="inlineStr">
-        <is>
-          <t>3,541</t>
-        </is>
-      </c>
-      <c r="H56" s="7" t="inlineStr">
-        <is>
-          <t>503</t>
-        </is>
-      </c>
-      <c r="I56" s="6" t="inlineStr">
-        <is>
-          <t>기타 기초 유기 화학물질 제조업</t>
-        </is>
-      </c>
-      <c r="J56" s="6" t="inlineStr">
-        <is>
-          <t>교보</t>
-        </is>
-      </c>
-      <c r="K56" s="6" t="inlineStr">
-        <is>
-          <t>예심 진행중</t>
-        </is>
-      </c>
-    </row>
-    <row r="58">
-      <c r="A58" s="3" t="inlineStr">
-        <is>
-          <t>■ 심사 승인  (37건)</t>
-        </is>
-      </c>
-      <c r="B58" s="4" t="n"/>
-      <c r="C58" s="4" t="n"/>
-      <c r="D58" s="4" t="n"/>
-      <c r="E58" s="4" t="n"/>
-      <c r="F58" s="4" t="n"/>
-      <c r="G58" s="4" t="n"/>
-      <c r="H58" s="4" t="n"/>
-      <c r="I58" s="4" t="n"/>
-      <c r="J58" s="4" t="n"/>
-      <c r="K58" s="4" t="n"/>
-    </row>
-    <row r="59">
-      <c r="A59" s="5" t="inlineStr">
-        <is>
-          <t>일자</t>
-        </is>
-      </c>
-      <c r="B59" s="5" t="inlineStr">
-        <is>
-          <t>회사명</t>
-        </is>
-      </c>
-      <c r="C59" s="5" t="inlineStr">
-        <is>
-          <t>시장</t>
-        </is>
-      </c>
-      <c r="D59" s="5" t="inlineStr">
-        <is>
-          <t>상장유형</t>
-        </is>
-      </c>
-      <c r="E59" s="5" t="inlineStr">
-        <is>
-          <t>기준연도</t>
-        </is>
-      </c>
-      <c r="F59" s="5" t="inlineStr">
-        <is>
-          <t>매출액</t>
-        </is>
-      </c>
-      <c r="G59" s="5" t="inlineStr">
-        <is>
-          <t>순이익</t>
-        </is>
-      </c>
-      <c r="H59" s="5" t="inlineStr">
-        <is>
-          <t>자기자본</t>
-        </is>
-      </c>
-      <c r="I59" s="5" t="inlineStr">
-        <is>
-          <t>업종</t>
-        </is>
-      </c>
-      <c r="J59" s="5" t="inlineStr">
-        <is>
-          <t>대표주관사</t>
-        </is>
-      </c>
-      <c r="K59" s="5" t="inlineStr">
-        <is>
-          <t>현황</t>
+      <c r="K59" s="6" t="inlineStr">
+        <is>
+          <t>상장전</t>
         </is>
       </c>
     </row>
@@ -3673,7 +3673,7 @@
       </c>
       <c r="B60" s="6" t="inlineStr">
         <is>
-          <t>덕산넵코어스</t>
+          <t>디티에스</t>
         </is>
       </c>
       <c r="C60" s="6" t="inlineStr">
@@ -3693,22 +3693,22 @@
       </c>
       <c r="F60" s="7" t="inlineStr">
         <is>
-          <t>48,504</t>
+          <t>142,718</t>
         </is>
       </c>
       <c r="G60" s="7" t="inlineStr">
         <is>
-          <t>3,668</t>
+          <t>18,765</t>
         </is>
       </c>
       <c r="H60" s="7" t="inlineStr">
         <is>
-          <t>8,448</t>
+          <t>63,153</t>
         </is>
       </c>
       <c r="I60" s="6" t="inlineStr">
         <is>
-          <t>항공기,우주선 및 부품 제조업</t>
+          <t>특수 목적용 기계 제조업</t>
         </is>
       </c>
       <c r="J60" s="6" t="inlineStr">
@@ -4231,7 +4231,7 @@
       </c>
       <c r="K69" s="6" t="inlineStr">
         <is>
-          <t>상장전</t>
+          <t>상장승인(상장예정)</t>
         </is>
       </c>
     </row>
@@ -6586,7 +6586,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R57"/>
+  <dimension ref="A1:R59"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="1"/>
@@ -9300,7 +9300,7 @@
     <row r="39" ht="22" customHeight="1">
       <c r="A39" s="3" t="inlineStr">
         <is>
-          <t>■ 공모 진행 (예심 승인법인)  (14건)</t>
+          <t>■ 공모 진행 (예심 승인법인)  (16건)</t>
         </is>
       </c>
       <c r="B39" s="4" t="n"/>
@@ -9984,7 +9984,7 @@
     <row r="50" ht="30" customHeight="1">
       <c r="A50" s="6" t="inlineStr">
         <is>
-          <t>와이즈플래닛컴퍼니</t>
+          <t>엔에이치스팩34호</t>
         </is>
       </c>
       <c r="B50" s="18" t="inlineStr">
@@ -10023,9 +10023,9 @@
       <c r="K50" s="6" t="inlineStr"/>
       <c r="L50" s="6" t="inlineStr"/>
       <c r="M50" s="6" t="inlineStr"/>
-      <c r="N50" s="6" t="inlineStr">
-        <is>
-          <t>대신</t>
+      <c r="N50" s="18" t="inlineStr">
+        <is>
+          <t>수집예정</t>
         </is>
       </c>
       <c r="O50" s="6" t="inlineStr"/>
@@ -10041,14 +10041,14 @@
       </c>
       <c r="R50" s="6" t="inlineStr">
         <is>
-          <t>신고서 대기</t>
+          <t>corp_code 미확보(수동확인)</t>
         </is>
       </c>
     </row>
     <row r="51" ht="30" customHeight="1">
       <c r="A51" s="6" t="inlineStr">
         <is>
-          <t>네오사피엔스</t>
+          <t>와이즈플래닛컴퍼니</t>
         </is>
       </c>
       <c r="B51" s="18" t="inlineStr">
@@ -10087,9 +10087,9 @@
       <c r="K51" s="6" t="inlineStr"/>
       <c r="L51" s="6" t="inlineStr"/>
       <c r="M51" s="6" t="inlineStr"/>
-      <c r="N51" s="18" t="inlineStr">
-        <is>
-          <t>수집예정</t>
+      <c r="N51" s="6" t="inlineStr">
+        <is>
+          <t>대신</t>
         </is>
       </c>
       <c r="O51" s="6" t="inlineStr"/>
@@ -10112,7 +10112,7 @@
     <row r="52" ht="30" customHeight="1">
       <c r="A52" s="6" t="inlineStr">
         <is>
-          <t>엠에스바이오</t>
+          <t>네오사피엔스</t>
         </is>
       </c>
       <c r="B52" s="18" t="inlineStr">
@@ -10176,7 +10176,7 @@
     <row r="53" ht="30" customHeight="1">
       <c r="A53" s="6" t="inlineStr">
         <is>
-          <t>덕산넵코어스</t>
+          <t>엠에스바이오</t>
         </is>
       </c>
       <c r="B53" s="18" t="inlineStr">
@@ -10237,22 +10237,150 @@
         </is>
       </c>
     </row>
-    <row r="55">
-      <c r="A55" s="20" t="inlineStr">
-        <is>
-          <t>※ 상장 완료 = KIND 신규상장 페이지 기준(스팩합병 포함) · 스팩 공모상장은 밴드·밸류에이션 등 해당없음(공모가 2,000원 고정).</t>
-        </is>
-      </c>
-    </row>
-    <row r="56">
-      <c r="A56" s="20" t="inlineStr">
-        <is>
-          <t>※ 기재정정 신고서 내 정정 전·후 병존 → 자동수집은 "정정 후" 값만 취함.</t>
+    <row r="54" ht="30" customHeight="1">
+      <c r="A54" s="6" t="inlineStr">
+        <is>
+          <t>덕산넵코어스</t>
+        </is>
+      </c>
+      <c r="B54" s="18" t="inlineStr">
+        <is>
+          <t>수집예정</t>
+        </is>
+      </c>
+      <c r="C54" s="18" t="inlineStr">
+        <is>
+          <t>수집예정</t>
+        </is>
+      </c>
+      <c r="D54" s="18" t="inlineStr">
+        <is>
+          <t>수집예정</t>
+        </is>
+      </c>
+      <c r="E54" s="18" t="inlineStr">
+        <is>
+          <t>수집예정</t>
+        </is>
+      </c>
+      <c r="F54" s="18" t="inlineStr">
+        <is>
+          <t>수집예정</t>
+        </is>
+      </c>
+      <c r="G54" s="6" t="inlineStr"/>
+      <c r="H54" s="6" t="inlineStr"/>
+      <c r="I54" s="6" t="inlineStr"/>
+      <c r="J54" s="18" t="inlineStr">
+        <is>
+          <t>수집예정</t>
+        </is>
+      </c>
+      <c r="K54" s="6" t="inlineStr"/>
+      <c r="L54" s="6" t="inlineStr"/>
+      <c r="M54" s="6" t="inlineStr"/>
+      <c r="N54" s="18" t="inlineStr">
+        <is>
+          <t>수집예정</t>
+        </is>
+      </c>
+      <c r="O54" s="6" t="inlineStr"/>
+      <c r="P54" s="18" t="inlineStr">
+        <is>
+          <t>수집예정</t>
+        </is>
+      </c>
+      <c r="Q54" s="18" t="inlineStr">
+        <is>
+          <t>수집예정</t>
+        </is>
+      </c>
+      <c r="R54" s="6" t="inlineStr">
+        <is>
+          <t>신고서 대기</t>
+        </is>
+      </c>
+    </row>
+    <row r="55" ht="30" customHeight="1">
+      <c r="A55" s="6" t="inlineStr">
+        <is>
+          <t>디티에스</t>
+        </is>
+      </c>
+      <c r="B55" s="18" t="inlineStr">
+        <is>
+          <t>수집예정</t>
+        </is>
+      </c>
+      <c r="C55" s="18" t="inlineStr">
+        <is>
+          <t>수집예정</t>
+        </is>
+      </c>
+      <c r="D55" s="18" t="inlineStr">
+        <is>
+          <t>수집예정</t>
+        </is>
+      </c>
+      <c r="E55" s="18" t="inlineStr">
+        <is>
+          <t>수집예정</t>
+        </is>
+      </c>
+      <c r="F55" s="18" t="inlineStr">
+        <is>
+          <t>수집예정</t>
+        </is>
+      </c>
+      <c r="G55" s="6" t="inlineStr"/>
+      <c r="H55" s="6" t="inlineStr"/>
+      <c r="I55" s="6" t="inlineStr"/>
+      <c r="J55" s="18" t="inlineStr">
+        <is>
+          <t>수집예정</t>
+        </is>
+      </c>
+      <c r="K55" s="6" t="inlineStr"/>
+      <c r="L55" s="6" t="inlineStr"/>
+      <c r="M55" s="6" t="inlineStr"/>
+      <c r="N55" s="18" t="inlineStr">
+        <is>
+          <t>수집예정</t>
+        </is>
+      </c>
+      <c r="O55" s="6" t="inlineStr"/>
+      <c r="P55" s="18" t="inlineStr">
+        <is>
+          <t>수집예정</t>
+        </is>
+      </c>
+      <c r="Q55" s="18" t="inlineStr">
+        <is>
+          <t>수집예정</t>
+        </is>
+      </c>
+      <c r="R55" s="6" t="inlineStr">
+        <is>
+          <t>신고서 대기</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" s="20" t="inlineStr">
+        <is>
+          <t>※ 상장 완료 = KIND 신규상장 페이지 기준(스팩합병 포함) · 스팩 공모상장은 밴드·밸류에이션 등 해당없음(공모가 2,000원 고정).</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="20" t="inlineStr">
+        <is>
+          <t>※ 기재정정 신고서 내 정정 전·후 병존 → 자동수집은 "정정 후" 값만 취함.</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="20" t="inlineStr">
         <is>
           <t>※ 청약경쟁률=일반투자자 청약수량÷최종배정수량 · "MM-DD~"는 종료일 자동수집 예정.</t>
         </is>
@@ -10486,7 +10614,7 @@
         <v>8</v>
       </c>
       <c r="C12" s="6" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="D12" s="6" t="n">
         <v>0</v>

</xml_diff>

<commit_message>
chore: update IPO data 2026-07-23
</commit_message>
<xml_diff>
--- a/IPO_analysis.xlsx
+++ b/IPO_analysis.xlsx
@@ -10101,56 +10101,56 @@
           <t>네오사피엔스</t>
         </is>
       </c>
-      <c r="B50" s="18" t="inlineStr">
-        <is>
-          <t>수집예정</t>
-        </is>
-      </c>
-      <c r="C50" s="18" t="inlineStr">
-        <is>
-          <t>수집예정</t>
-        </is>
-      </c>
-      <c r="D50" s="18" t="inlineStr">
-        <is>
-          <t>수집예정</t>
-        </is>
-      </c>
-      <c r="E50" s="18" t="inlineStr">
-        <is>
-          <t>수집예정</t>
-        </is>
-      </c>
-      <c r="F50" s="18" t="inlineStr">
-        <is>
-          <t>수집예정</t>
+      <c r="B50" s="6" t="inlineStr">
+        <is>
+          <t>08-31~09-04</t>
+        </is>
+      </c>
+      <c r="C50" s="6" t="inlineStr">
+        <is>
+          <t>13,800~15,800</t>
+        </is>
+      </c>
+      <c r="D50" s="7" t="inlineStr">
+        <is>
+          <t>2,000,000</t>
+        </is>
+      </c>
+      <c r="E50" s="7" t="inlineStr">
+        <is>
+          <t>27,600,000,000</t>
+        </is>
+      </c>
+      <c r="F50" s="6" t="inlineStr">
+        <is>
+          <t>26.76배 (PER)</t>
         </is>
       </c>
       <c r="G50" s="6" t="inlineStr"/>
       <c r="H50" s="6" t="inlineStr"/>
       <c r="I50" s="6" t="inlineStr"/>
-      <c r="J50" s="18" t="inlineStr">
-        <is>
-          <t>수집예정</t>
+      <c r="J50" s="6" t="inlineStr">
+        <is>
+          <t>09-08~09-09</t>
         </is>
       </c>
       <c r="K50" s="6" t="inlineStr"/>
       <c r="L50" s="6" t="inlineStr"/>
       <c r="M50" s="6" t="inlineStr"/>
-      <c r="N50" s="18" t="inlineStr">
-        <is>
-          <t>수집예정</t>
+      <c r="N50" s="6" t="inlineStr">
+        <is>
+          <t>대신증권</t>
         </is>
       </c>
       <c r="O50" s="6" t="inlineStr"/>
-      <c r="P50" s="18" t="inlineStr">
-        <is>
-          <t>수집예정</t>
-        </is>
-      </c>
-      <c r="Q50" s="18" t="inlineStr">
-        <is>
-          <t>수집예정</t>
+      <c r="P50" s="7" t="inlineStr">
+        <is>
+          <t>1,080,264,000</t>
+        </is>
+      </c>
+      <c r="Q50" s="6" t="inlineStr">
+        <is>
+          <t>3.8%</t>
         </is>
       </c>
       <c r="R50" s="6" t="inlineStr">
@@ -10575,7 +10575,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F33"/>
+  <dimension ref="A1:F34"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -10936,127 +10936,127 @@
     <row r="22">
       <c r="A22" s="6" t="inlineStr">
         <is>
-          <t>삼성증권</t>
+          <t>대신증권</t>
         </is>
       </c>
       <c r="B22" s="6" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C22" s="6" t="inlineStr">
         <is>
-          <t>27,300,060,000</t>
+          <t>27,600,000,000</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="6" t="inlineStr">
         <is>
-          <t>DB증권</t>
+          <t>삼성증권</t>
         </is>
       </c>
       <c r="B23" s="6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C23" s="6" t="inlineStr">
         <is>
-          <t>23,000,000,000</t>
+          <t>27,300,060,000</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="6" t="inlineStr">
         <is>
-          <t>NH</t>
+          <t>DB증권</t>
         </is>
       </c>
       <c r="B24" s="6" t="n">
-        <v>7</v>
+        <v>1</v>
       </c>
       <c r="C24" s="6" t="inlineStr">
         <is>
-          <t>618,288</t>
+          <t>23,000,000,000</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="6" t="inlineStr">
         <is>
-          <t>한국</t>
+          <t>NH</t>
         </is>
       </c>
       <c r="B25" s="6" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="C25" s="6" t="inlineStr">
         <is>
-          <t>154,600</t>
+          <t>618,288</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="6" t="inlineStr">
         <is>
-          <t>미래</t>
+          <t>한국</t>
         </is>
       </c>
       <c r="B26" s="6" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="C26" s="6" t="inlineStr">
         <is>
-          <t>130,837</t>
+          <t>154,600</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="6" t="inlineStr">
         <is>
-          <t>신한</t>
+          <t>미래</t>
         </is>
       </c>
       <c r="B27" s="6" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="C27" s="6" t="inlineStr">
         <is>
-          <t>49,052</t>
+          <t>130,837</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="6" t="inlineStr">
         <is>
-          <t>삼성</t>
+          <t>신한</t>
         </is>
       </c>
       <c r="B28" s="6" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C28" s="6" t="inlineStr">
         <is>
-          <t>32,000</t>
+          <t>49,052</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="6" t="inlineStr">
         <is>
-          <t>유진</t>
+          <t>삼성</t>
         </is>
       </c>
       <c r="B29" s="6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C29" s="6" t="inlineStr">
         <is>
-          <t>25,020</t>
+          <t>32,000</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="6" t="inlineStr">
         <is>
-          <t>메리츠</t>
+          <t>유진</t>
         </is>
       </c>
       <c r="B30" s="6" t="n">
@@ -11064,50 +11064,65 @@
       </c>
       <c r="C30" s="6" t="inlineStr">
         <is>
-          <t>14,000</t>
+          <t>25,020</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="6" t="inlineStr">
         <is>
-          <t>대신</t>
+          <t>메리츠</t>
         </is>
       </c>
       <c r="B31" s="6" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C31" s="6" t="inlineStr">
         <is>
-          <t>13,000</t>
+          <t>14,000</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="6" t="inlineStr">
         <is>
-          <t>키움</t>
+          <t>대신</t>
         </is>
       </c>
       <c r="B32" s="6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C32" s="6" t="inlineStr">
         <is>
-          <t>12,000</t>
+          <t>13,000</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="6" t="inlineStr">
         <is>
-          <t>교보</t>
+          <t>키움</t>
         </is>
       </c>
       <c r="B33" s="6" t="n">
         <v>1</v>
       </c>
       <c r="C33" s="6" t="inlineStr">
+        <is>
+          <t>12,000</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="6" t="inlineStr">
+        <is>
+          <t>교보</t>
+        </is>
+      </c>
+      <c r="B34" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="C34" s="6" t="inlineStr">
         <is>
           <t>10,800</t>
         </is>

</xml_diff>

<commit_message>
chore: update IPO data 2026-07-27
</commit_message>
<xml_diff>
--- a/IPO_analysis.xlsx
+++ b/IPO_analysis.xlsx
@@ -6859,7 +6859,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R61"/>
+  <dimension ref="A1:R60"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="1"/>
@@ -7075,7 +7075,7 @@
     <row r="6" ht="22" customHeight="1">
       <c r="A6" s="3" t="inlineStr">
         <is>
-          <t>■ 상장 완료 (2026)  (33건)</t>
+          <t>■ 상장 완료 (2026)  (32건)</t>
         </is>
       </c>
       <c r="B6" s="4" t="n"/>
@@ -7099,48 +7099,44 @@
     <row r="7" ht="30" customHeight="1">
       <c r="A7" s="6" t="inlineStr">
         <is>
-          <t>네오뷰</t>
-        </is>
-      </c>
-      <c r="B7" s="18" t="inlineStr">
-        <is>
-          <t>수집예정</t>
-        </is>
-      </c>
-      <c r="C7" s="18" t="inlineStr">
-        <is>
-          <t>수집예정</t>
-        </is>
-      </c>
-      <c r="D7" s="18" t="inlineStr">
-        <is>
-          <t>수집예정</t>
-        </is>
-      </c>
-      <c r="E7" s="18" t="inlineStr">
-        <is>
-          <t>수집예정</t>
-        </is>
-      </c>
-      <c r="F7" s="18" t="inlineStr">
-        <is>
-          <t>수집예정</t>
-        </is>
-      </c>
-      <c r="G7" s="18" t="inlineStr">
-        <is>
-          <t>수집예정</t>
-        </is>
-      </c>
-      <c r="H7" s="18" t="inlineStr">
-        <is>
-          <t>수집예정</t>
-        </is>
-      </c>
-      <c r="I7" s="18" t="inlineStr">
-        <is>
-          <t>수집예정</t>
-        </is>
+          <t>에이치엘지노믹스</t>
+        </is>
+      </c>
+      <c r="B7" s="6" t="inlineStr">
+        <is>
+          <t>07-02~07-08</t>
+        </is>
+      </c>
+      <c r="C7" s="6" t="inlineStr">
+        <is>
+          <t>18,500~21,500</t>
+        </is>
+      </c>
+      <c r="D7" s="7" t="inlineStr">
+        <is>
+          <t>2,565,000</t>
+        </is>
+      </c>
+      <c r="E7" s="7" t="inlineStr">
+        <is>
+          <t>55,147,500,000</t>
+        </is>
+      </c>
+      <c r="F7" s="6" t="inlineStr">
+        <is>
+          <t>12.85배 (EV/EBITDA)</t>
+        </is>
+      </c>
+      <c r="G7" s="6" t="inlineStr">
+        <is>
+          <t>21,500</t>
+        </is>
+      </c>
+      <c r="H7" s="6" t="n">
+        <v>714.52</v>
+      </c>
+      <c r="I7" s="6" t="n">
+        <v>2148</v>
       </c>
       <c r="J7" s="18" t="inlineStr">
         <is>
@@ -7155,23 +7151,27 @@
       <c r="L7" s="6" t="inlineStr"/>
       <c r="M7" s="6" t="inlineStr">
         <is>
-          <t>2026-07-27</t>
-        </is>
-      </c>
-      <c r="N7" s="18" t="inlineStr">
-        <is>
-          <t>수집예정</t>
-        </is>
-      </c>
-      <c r="O7" s="6" t="inlineStr"/>
-      <c r="P7" s="18" t="inlineStr">
-        <is>
-          <t>수집예정</t>
-        </is>
-      </c>
-      <c r="Q7" s="18" t="inlineStr">
-        <is>
-          <t>수집예정</t>
+          <t>2026-07-24</t>
+        </is>
+      </c>
+      <c r="N7" s="6" t="inlineStr">
+        <is>
+          <t>KB</t>
+        </is>
+      </c>
+      <c r="O7" s="6" t="inlineStr">
+        <is>
+          <t>아이비케이투자증권, IBK투자증권, IBK투자증권, IBK투자증권, IBK투자증권, IBK투자증권㈜, 보통주, IBK투자증권㈜</t>
+        </is>
+      </c>
+      <c r="P7" s="7" t="inlineStr">
+        <is>
+          <t>1,211</t>
+        </is>
+      </c>
+      <c r="Q7" s="6" t="inlineStr">
+        <is>
+          <t>2.5%</t>
         </is>
       </c>
       <c r="R7" s="6" t="inlineStr">
@@ -7183,59 +7183,63 @@
     <row r="8" ht="30" customHeight="1">
       <c r="A8" s="6" t="inlineStr">
         <is>
-          <t>에이치엘지노믹스</t>
-        </is>
-      </c>
-      <c r="B8" s="6" t="inlineStr">
-        <is>
-          <t>07-02~07-08</t>
+          <t>레메디</t>
+        </is>
+      </c>
+      <c r="B8" s="18" t="inlineStr">
+        <is>
+          <t>수집예정</t>
         </is>
       </c>
       <c r="C8" s="6" t="inlineStr">
         <is>
-          <t>18,500~21,500</t>
+          <t>17,800~20,700</t>
         </is>
       </c>
       <c r="D8" s="7" t="inlineStr">
         <is>
-          <t>2,565,000</t>
+          <t>1,200,000</t>
         </is>
       </c>
       <c r="E8" s="7" t="inlineStr">
         <is>
-          <t>55,147,500,000</t>
+          <t>24,840,000,000</t>
         </is>
       </c>
       <c r="F8" s="6" t="inlineStr">
         <is>
-          <t>12.85배 (EV/EBITDA)</t>
+          <t>21.95배 (PER)</t>
         </is>
       </c>
       <c r="G8" s="6" t="inlineStr">
         <is>
-          <t>21,500</t>
-        </is>
-      </c>
-      <c r="H8" s="6" t="n">
-        <v>714.52</v>
-      </c>
-      <c r="I8" s="6" t="n">
-        <v>2148</v>
+          <t>20,700</t>
+        </is>
+      </c>
+      <c r="H8" s="6" t="inlineStr">
+        <is>
+          <t>1,146.41</t>
+        </is>
+      </c>
+      <c r="I8" s="6" t="inlineStr">
+        <is>
+          <t>2,246</t>
+        </is>
       </c>
       <c r="J8" s="18" t="inlineStr">
         <is>
           <t>수집예정</t>
         </is>
       </c>
-      <c r="K8" s="18" t="inlineStr">
-        <is>
-          <t>수집예정</t>
+      <c r="K8" s="6" t="inlineStr">
+        <is>
+          <t>1,706.71</t>
         </is>
       </c>
       <c r="L8" s="6" t="inlineStr"/>
       <c r="M8" s="6" t="inlineStr">
         <is>
-          <t>2026-07-24</t>
+          <t>2026-07-13</t>
         </is>
       </c>
       <c r="N8" s="6" t="inlineStr">
@@ -7243,19 +7247,15 @@
           <t>KB</t>
         </is>
       </c>
-      <c r="O8" s="6" t="inlineStr">
-        <is>
-          <t>아이비케이투자증권, IBK투자증권, IBK투자증권, IBK투자증권, IBK투자증권, IBK투자증권㈜, 보통주, IBK투자증권㈜</t>
-        </is>
-      </c>
+      <c r="O8" s="6" t="inlineStr"/>
       <c r="P8" s="7" t="inlineStr">
         <is>
-          <t>1,211</t>
+          <t>1,279</t>
         </is>
       </c>
       <c r="Q8" s="6" t="inlineStr">
         <is>
-          <t>2.5%</t>
+          <t>5.0%</t>
         </is>
       </c>
       <c r="R8" s="6" t="inlineStr">
@@ -7267,7 +7267,7 @@
     <row r="9" ht="30" customHeight="1">
       <c r="A9" s="6" t="inlineStr">
         <is>
-          <t>레메디</t>
+          <t>레몬헬스케어</t>
         </is>
       </c>
       <c r="B9" s="18" t="inlineStr">
@@ -7277,53 +7277,45 @@
       </c>
       <c r="C9" s="6" t="inlineStr">
         <is>
-          <t>17,800~20,700</t>
+          <t>7,500~10,000</t>
         </is>
       </c>
       <c r="D9" s="7" t="inlineStr">
         <is>
-          <t>1,200,000</t>
+          <t>2,000,000</t>
         </is>
       </c>
       <c r="E9" s="7" t="inlineStr">
         <is>
-          <t>24,840,000,000</t>
+          <t>20,000</t>
         </is>
       </c>
       <c r="F9" s="6" t="inlineStr">
         <is>
-          <t>21.95배 (PER)</t>
-        </is>
-      </c>
-      <c r="G9" s="6" t="inlineStr">
-        <is>
-          <t>20,700</t>
-        </is>
-      </c>
-      <c r="H9" s="6" t="inlineStr">
-        <is>
-          <t>1,146.41</t>
-        </is>
-      </c>
-      <c r="I9" s="6" t="inlineStr">
-        <is>
-          <t>2,246</t>
-        </is>
-      </c>
-      <c r="J9" s="18" t="inlineStr">
-        <is>
-          <t>수집예정</t>
-        </is>
-      </c>
-      <c r="K9" s="6" t="inlineStr">
-        <is>
-          <t>1,706.71</t>
-        </is>
+          <t>25.48배 (PER)</t>
+        </is>
+      </c>
+      <c r="G9" s="6" t="n">
+        <v>10000</v>
+      </c>
+      <c r="H9" s="6" t="n">
+        <v>1238</v>
+      </c>
+      <c r="I9" s="6" t="n">
+        <v>2233</v>
+      </c>
+      <c r="J9" s="6" t="inlineStr">
+        <is>
+          <t>2026-06-24~25</t>
+        </is>
+      </c>
+      <c r="K9" s="6" t="n">
+        <v>1510.57</v>
       </c>
       <c r="L9" s="6" t="inlineStr"/>
       <c r="M9" s="6" t="inlineStr">
         <is>
-          <t>2026-07-13</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="N9" s="6" t="inlineStr">
@@ -7334,12 +7326,12 @@
       <c r="O9" s="6" t="inlineStr"/>
       <c r="P9" s="7" t="inlineStr">
         <is>
-          <t>1,279</t>
+          <t>824</t>
         </is>
       </c>
       <c r="Q9" s="6" t="inlineStr">
         <is>
-          <t>5.0%</t>
+          <t>4.0%</t>
         </is>
       </c>
       <c r="R9" s="6" t="inlineStr">
@@ -7351,7 +7343,7 @@
     <row r="10" ht="30" customHeight="1">
       <c r="A10" s="6" t="inlineStr">
         <is>
-          <t>레몬헬스케어</t>
+          <t>매드업</t>
         </is>
       </c>
       <c r="B10" s="18" t="inlineStr">
@@ -7361,7 +7353,7 @@
       </c>
       <c r="C10" s="6" t="inlineStr">
         <is>
-          <t>7,500~10,000</t>
+          <t>7,000~8,000</t>
         </is>
       </c>
       <c r="D10" s="7" t="inlineStr">
@@ -7371,51 +7363,51 @@
       </c>
       <c r="E10" s="7" t="inlineStr">
         <is>
-          <t>20,000</t>
+          <t>16,000</t>
         </is>
       </c>
       <c r="F10" s="6" t="inlineStr">
         <is>
-          <t>25.48배 (PER)</t>
+          <t>24.57배 (PER)</t>
         </is>
       </c>
       <c r="G10" s="6" t="n">
-        <v>10000</v>
+        <v>8000</v>
       </c>
       <c r="H10" s="6" t="n">
-        <v>1238</v>
+        <v>1396.29</v>
       </c>
       <c r="I10" s="6" t="n">
-        <v>2233</v>
+        <v>2392</v>
       </c>
       <c r="J10" s="6" t="inlineStr">
         <is>
-          <t>2026-06-24~25</t>
+          <t>2026-06-23~24</t>
         </is>
       </c>
       <c r="K10" s="6" t="n">
-        <v>1510.57</v>
+        <v>3304.76</v>
       </c>
       <c r="L10" s="6" t="inlineStr"/>
       <c r="M10" s="6" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-07-01</t>
         </is>
       </c>
       <c r="N10" s="6" t="inlineStr">
         <is>
-          <t>KB</t>
+          <t>미래</t>
         </is>
       </c>
       <c r="O10" s="6" t="inlineStr"/>
       <c r="P10" s="7" t="inlineStr">
         <is>
-          <t>824</t>
+          <t>742</t>
         </is>
       </c>
       <c r="Q10" s="6" t="inlineStr">
         <is>
-          <t>4.0%</t>
+          <t>4.5%</t>
         </is>
       </c>
       <c r="R10" s="6" t="inlineStr">
@@ -7427,71 +7419,75 @@
     <row r="11" ht="30" customHeight="1">
       <c r="A11" s="6" t="inlineStr">
         <is>
-          <t>매드업</t>
-        </is>
-      </c>
-      <c r="B11" s="18" t="inlineStr">
-        <is>
-          <t>수집예정</t>
+          <t>한국제16호스팩</t>
+        </is>
+      </c>
+      <c r="B11" s="19" t="inlineStr">
+        <is>
+          <t>해당없음</t>
         </is>
       </c>
       <c r="C11" s="6" t="inlineStr">
         <is>
-          <t>7,000~8,000</t>
+          <t>2,000</t>
         </is>
       </c>
       <c r="D11" s="7" t="inlineStr">
         <is>
-          <t>2,000,000</t>
+          <t>5,500,000</t>
         </is>
       </c>
       <c r="E11" s="7" t="inlineStr">
         <is>
-          <t>16,000</t>
-        </is>
-      </c>
-      <c r="F11" s="6" t="inlineStr">
-        <is>
-          <t>24.57배 (PER)</t>
-        </is>
-      </c>
-      <c r="G11" s="6" t="n">
-        <v>8000</v>
+          <t>11,000</t>
+        </is>
+      </c>
+      <c r="F11" s="19" t="inlineStr">
+        <is>
+          <t>해당없음</t>
+        </is>
+      </c>
+      <c r="G11" s="6" t="inlineStr">
+        <is>
+          <t>2,000</t>
+        </is>
       </c>
       <c r="H11" s="6" t="n">
-        <v>1396.29</v>
+        <v>1364.09</v>
       </c>
       <c r="I11" s="6" t="n">
-        <v>2392</v>
+        <v>2089</v>
       </c>
       <c r="J11" s="6" t="inlineStr">
         <is>
-          <t>2026-06-23~24</t>
-        </is>
-      </c>
-      <c r="K11" s="6" t="n">
-        <v>3304.76</v>
+          <t>2026-06-22~06-23</t>
+        </is>
+      </c>
+      <c r="K11" s="6" t="inlineStr">
+        <is>
+          <t>1,274.77</t>
+        </is>
       </c>
       <c r="L11" s="6" t="inlineStr"/>
       <c r="M11" s="6" t="inlineStr">
         <is>
-          <t>2026-07-01</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="N11" s="6" t="inlineStr">
         <is>
-          <t>미래</t>
+          <t>한국</t>
         </is>
       </c>
       <c r="O11" s="6" t="inlineStr"/>
       <c r="P11" s="7" t="inlineStr">
         <is>
-          <t>742</t>
+          <t>330</t>
         </is>
       </c>
       <c r="Q11" s="6" t="inlineStr">
         <is>
-          <t>4.5%</t>
+          <t>3.00%</t>
         </is>
       </c>
       <c r="R11" s="6" t="inlineStr">
@@ -7503,53 +7499,51 @@
     <row r="12" ht="30" customHeight="1">
       <c r="A12" s="6" t="inlineStr">
         <is>
-          <t>한국제16호스팩</t>
-        </is>
-      </c>
-      <c r="B12" s="19" t="inlineStr">
-        <is>
-          <t>해당없음</t>
+          <t>스트라드비젼</t>
+        </is>
+      </c>
+      <c r="B12" s="18" t="inlineStr">
+        <is>
+          <t>수집예정</t>
         </is>
       </c>
       <c r="C12" s="6" t="inlineStr">
         <is>
-          <t>2,000</t>
+          <t>12,000~14,000</t>
         </is>
       </c>
       <c r="D12" s="7" t="inlineStr">
         <is>
-          <t>5,500,000</t>
+          <t>7,000,000</t>
         </is>
       </c>
       <c r="E12" s="7" t="inlineStr">
         <is>
-          <t>11,000</t>
-        </is>
-      </c>
-      <c r="F12" s="19" t="inlineStr">
-        <is>
-          <t>해당없음</t>
-        </is>
-      </c>
-      <c r="G12" s="6" t="inlineStr">
-        <is>
-          <t>2,000</t>
-        </is>
+          <t>84,000</t>
+        </is>
+      </c>
+      <c r="F12" s="6" t="inlineStr">
+        <is>
+          <t>37.45배 (PER)</t>
+        </is>
+      </c>
+      <c r="G12" s="6" t="n">
+        <v>12000</v>
       </c>
       <c r="H12" s="6" t="n">
-        <v>1364.09</v>
+        <v>381.3</v>
       </c>
       <c r="I12" s="6" t="n">
-        <v>2089</v>
+        <v>1604</v>
       </c>
       <c r="J12" s="6" t="inlineStr">
         <is>
-          <t>2026-06-22~06-23</t>
+          <t>2026-06-18~06-19</t>
         </is>
       </c>
       <c r="K12" s="6" t="inlineStr">
         <is>
-          <t>1,274.77</t>
+          <t>45.81</t>
         </is>
       </c>
       <c r="L12" s="6" t="inlineStr"/>
@@ -7560,13 +7554,13 @@
       </c>
       <c r="N12" s="6" t="inlineStr">
         <is>
-          <t>한국</t>
+          <t>KB</t>
         </is>
       </c>
       <c r="O12" s="6" t="inlineStr"/>
       <c r="P12" s="7" t="inlineStr">
         <is>
-          <t>330</t>
+          <t>2,575</t>
         </is>
       </c>
       <c r="Q12" s="6" t="inlineStr">
@@ -7583,7 +7577,7 @@
     <row r="13" ht="30" customHeight="1">
       <c r="A13" s="6" t="inlineStr">
         <is>
-          <t>스트라드비젼</t>
+          <t>져스텍</t>
         </is>
       </c>
       <c r="B13" s="18" t="inlineStr">
@@ -7593,32 +7587,32 @@
       </c>
       <c r="C13" s="6" t="inlineStr">
         <is>
-          <t>12,000~14,000</t>
+          <t>10,500~12,500</t>
         </is>
       </c>
       <c r="D13" s="7" t="inlineStr">
         <is>
-          <t>7,000,000</t>
+          <t>1,600,000</t>
         </is>
       </c>
       <c r="E13" s="7" t="inlineStr">
         <is>
-          <t>84,000</t>
+          <t>20,000</t>
         </is>
       </c>
       <c r="F13" s="6" t="inlineStr">
         <is>
-          <t>37.45배 (PER)</t>
+          <t>26.82배 (PER)</t>
         </is>
       </c>
       <c r="G13" s="6" t="n">
-        <v>12000</v>
+        <v>12500</v>
       </c>
       <c r="H13" s="6" t="n">
-        <v>381.3</v>
+        <v>1294.99</v>
       </c>
       <c r="I13" s="6" t="n">
-        <v>1604</v>
+        <v>2252</v>
       </c>
       <c r="J13" s="6" t="inlineStr">
         <is>
@@ -7627,29 +7621,29 @@
       </c>
       <c r="K13" s="6" t="inlineStr">
         <is>
-          <t>45.81</t>
+          <t>2,783.89</t>
         </is>
       </c>
       <c r="L13" s="6" t="inlineStr"/>
       <c r="M13" s="6" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-06-29</t>
         </is>
       </c>
       <c r="N13" s="6" t="inlineStr">
         <is>
-          <t>KB</t>
+          <t>삼성</t>
         </is>
       </c>
       <c r="O13" s="6" t="inlineStr"/>
       <c r="P13" s="7" t="inlineStr">
         <is>
-          <t>2,575</t>
+          <t>1,164</t>
         </is>
       </c>
       <c r="Q13" s="6" t="inlineStr">
         <is>
-          <t>3.00%</t>
+          <t>5.65%</t>
         </is>
       </c>
       <c r="R13" s="6" t="inlineStr">
@@ -7661,73 +7655,75 @@
     <row r="14" ht="30" customHeight="1">
       <c r="A14" s="6" t="inlineStr">
         <is>
-          <t>져스텍</t>
-        </is>
-      </c>
-      <c r="B14" s="18" t="inlineStr">
-        <is>
-          <t>수집예정</t>
+          <t>메리츠제2호스팩</t>
+        </is>
+      </c>
+      <c r="B14" s="19" t="inlineStr">
+        <is>
+          <t>해당없음</t>
         </is>
       </c>
       <c r="C14" s="6" t="inlineStr">
         <is>
-          <t>10,500~12,500</t>
+          <t>2,000</t>
         </is>
       </c>
       <c r="D14" s="7" t="inlineStr">
         <is>
-          <t>1,600,000</t>
+          <t>7,000,000</t>
         </is>
       </c>
       <c r="E14" s="7" t="inlineStr">
         <is>
-          <t>20,000</t>
-        </is>
-      </c>
-      <c r="F14" s="6" t="inlineStr">
-        <is>
-          <t>26.82배 (PER)</t>
-        </is>
-      </c>
-      <c r="G14" s="6" t="n">
-        <v>12500</v>
+          <t>14,000</t>
+        </is>
+      </c>
+      <c r="F14" s="19" t="inlineStr">
+        <is>
+          <t>해당없음</t>
+        </is>
+      </c>
+      <c r="G14" s="6" t="inlineStr">
+        <is>
+          <t>2,000</t>
+        </is>
       </c>
       <c r="H14" s="6" t="n">
-        <v>1294.99</v>
+        <v>1087.58</v>
       </c>
       <c r="I14" s="6" t="n">
-        <v>2252</v>
+        <v>1798</v>
       </c>
       <c r="J14" s="6" t="inlineStr">
         <is>
-          <t>2026-06-18~06-19</t>
+          <t>2026-06-09~06-10</t>
         </is>
       </c>
       <c r="K14" s="6" t="inlineStr">
         <is>
-          <t>2,783.89</t>
+          <t>1,338.66</t>
         </is>
       </c>
       <c r="L14" s="6" t="inlineStr"/>
       <c r="M14" s="6" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-06-19</t>
         </is>
       </c>
       <c r="N14" s="6" t="inlineStr">
         <is>
-          <t>삼성</t>
+          <t>메리츠</t>
         </is>
       </c>
       <c r="O14" s="6" t="inlineStr"/>
       <c r="P14" s="7" t="inlineStr">
         <is>
-          <t>1,164</t>
+          <t>245</t>
         </is>
       </c>
       <c r="Q14" s="6" t="inlineStr">
         <is>
-          <t>5.65%</t>
+          <t>1.75%</t>
         </is>
       </c>
       <c r="R14" s="6" t="inlineStr">
@@ -7739,75 +7735,77 @@
     <row r="15" ht="30" customHeight="1">
       <c r="A15" s="6" t="inlineStr">
         <is>
-          <t>메리츠제2호스팩</t>
-        </is>
-      </c>
-      <c r="B15" s="19" t="inlineStr">
-        <is>
-          <t>해당없음</t>
+          <t>피스피스스튜디오</t>
+        </is>
+      </c>
+      <c r="B15" s="18" t="inlineStr">
+        <is>
+          <t>수집예정</t>
         </is>
       </c>
       <c r="C15" s="6" t="inlineStr">
         <is>
-          <t>2,000</t>
+          <t>19,000~21,500</t>
         </is>
       </c>
       <c r="D15" s="7" t="inlineStr">
         <is>
-          <t>7,000,000</t>
+          <t>2,272,637</t>
         </is>
       </c>
       <c r="E15" s="7" t="inlineStr">
         <is>
-          <t>14,000</t>
-        </is>
-      </c>
-      <c r="F15" s="19" t="inlineStr">
-        <is>
-          <t>해당없음</t>
-        </is>
-      </c>
-      <c r="G15" s="6" t="inlineStr">
-        <is>
-          <t>2,000</t>
-        </is>
+          <t>48,862</t>
+        </is>
+      </c>
+      <c r="F15" s="6" t="inlineStr">
+        <is>
+          <t>21.48배 (PER)</t>
+        </is>
+      </c>
+      <c r="G15" s="6" t="n">
+        <v>21500</v>
       </c>
       <c r="H15" s="6" t="n">
-        <v>1087.58</v>
+        <v>847.76</v>
       </c>
       <c r="I15" s="6" t="n">
-        <v>1798</v>
+        <v>2329</v>
       </c>
       <c r="J15" s="6" t="inlineStr">
         <is>
-          <t>2026-06-09~06-10</t>
+          <t>2026-05-26~05-27</t>
         </is>
       </c>
       <c r="K15" s="6" t="inlineStr">
         <is>
-          <t>1,338.66</t>
+          <t>1,191.15</t>
         </is>
       </c>
       <c r="L15" s="6" t="inlineStr"/>
       <c r="M15" s="6" t="inlineStr">
         <is>
-          <t>2026-06-19</t>
+          <t>2026-06-08</t>
         </is>
       </c>
       <c r="N15" s="6" t="inlineStr">
         <is>
-          <t>메리츠</t>
-        </is>
-      </c>
-      <c r="O15" s="6" t="inlineStr"/>
+          <t>미래</t>
+        </is>
+      </c>
+      <c r="O15" s="6" t="inlineStr">
+        <is>
+          <t>NH</t>
+        </is>
+      </c>
       <c r="P15" s="7" t="inlineStr">
         <is>
-          <t>245</t>
+          <t>1,994</t>
         </is>
       </c>
       <c r="Q15" s="6" t="inlineStr">
         <is>
-          <t>1.75%</t>
+          <t>4.00%</t>
         </is>
       </c>
       <c r="R15" s="6" t="inlineStr">
@@ -7819,77 +7817,75 @@
     <row r="16" ht="30" customHeight="1">
       <c r="A16" s="6" t="inlineStr">
         <is>
-          <t>피스피스스튜디오</t>
-        </is>
-      </c>
-      <c r="B16" s="18" t="inlineStr">
-        <is>
-          <t>수집예정</t>
+          <t>대신밸런스제20호스팩</t>
+        </is>
+      </c>
+      <c r="B16" s="19" t="inlineStr">
+        <is>
+          <t>해당없음</t>
         </is>
       </c>
       <c r="C16" s="6" t="inlineStr">
         <is>
-          <t>19,000~21,500</t>
+          <t>2,000</t>
         </is>
       </c>
       <c r="D16" s="7" t="inlineStr">
         <is>
-          <t>2,272,637</t>
+          <t>6,500,000</t>
         </is>
       </c>
       <c r="E16" s="7" t="inlineStr">
         <is>
-          <t>48,862</t>
-        </is>
-      </c>
-      <c r="F16" s="6" t="inlineStr">
-        <is>
-          <t>21.48배 (PER)</t>
-        </is>
-      </c>
-      <c r="G16" s="6" t="n">
-        <v>21500</v>
+          <t>13,000</t>
+        </is>
+      </c>
+      <c r="F16" s="19" t="inlineStr">
+        <is>
+          <t>해당없음</t>
+        </is>
+      </c>
+      <c r="G16" s="6" t="inlineStr">
+        <is>
+          <t>2,000</t>
+        </is>
       </c>
       <c r="H16" s="6" t="n">
-        <v>847.76</v>
+        <v>1327.13</v>
       </c>
       <c r="I16" s="6" t="n">
-        <v>2329</v>
+        <v>2194</v>
       </c>
       <c r="J16" s="6" t="inlineStr">
         <is>
-          <t>2026-05-26~05-27</t>
+          <t>2026-05-22~05-25</t>
         </is>
       </c>
       <c r="K16" s="6" t="inlineStr">
         <is>
-          <t>1,191.15</t>
+          <t>1,486.88</t>
         </is>
       </c>
       <c r="L16" s="6" t="inlineStr"/>
       <c r="M16" s="6" t="inlineStr">
         <is>
-          <t>2026-06-08</t>
+          <t>2026-06-05</t>
         </is>
       </c>
       <c r="N16" s="6" t="inlineStr">
         <is>
-          <t>미래</t>
-        </is>
-      </c>
-      <c r="O16" s="6" t="inlineStr">
-        <is>
-          <t>NH</t>
-        </is>
-      </c>
+          <t>대신</t>
+        </is>
+      </c>
+      <c r="O16" s="6" t="inlineStr"/>
       <c r="P16" s="7" t="inlineStr">
         <is>
-          <t>1,994</t>
+          <t>390</t>
         </is>
       </c>
       <c r="Q16" s="6" t="inlineStr">
         <is>
-          <t>4.00%</t>
+          <t>3.00%</t>
         </is>
       </c>
       <c r="R16" s="6" t="inlineStr">
@@ -7901,75 +7897,73 @@
     <row r="17" ht="30" customHeight="1">
       <c r="A17" s="6" t="inlineStr">
         <is>
-          <t>대신밸런스제20호스팩</t>
-        </is>
-      </c>
-      <c r="B17" s="19" t="inlineStr">
-        <is>
-          <t>해당없음</t>
+          <t>마키나락스</t>
+        </is>
+      </c>
+      <c r="B17" s="18" t="inlineStr">
+        <is>
+          <t>수집예정</t>
         </is>
       </c>
       <c r="C17" s="6" t="inlineStr">
         <is>
-          <t>2,000</t>
+          <t>12,500~15,000</t>
         </is>
       </c>
       <c r="D17" s="7" t="inlineStr">
         <is>
-          <t>6,500,000</t>
+          <t>2,635,000</t>
         </is>
       </c>
       <c r="E17" s="7" t="inlineStr">
         <is>
-          <t>13,000</t>
-        </is>
-      </c>
-      <c r="F17" s="19" t="inlineStr">
-        <is>
-          <t>해당없음</t>
-        </is>
-      </c>
-      <c r="G17" s="6" t="inlineStr">
-        <is>
-          <t>2,000</t>
-        </is>
+          <t>39,525</t>
+        </is>
+      </c>
+      <c r="F17" s="6" t="inlineStr">
+        <is>
+          <t>40.5배 (PER)</t>
+        </is>
+      </c>
+      <c r="G17" s="6" t="n">
+        <v>15000</v>
       </c>
       <c r="H17" s="6" t="n">
-        <v>1327.13</v>
+        <v>1196.08</v>
       </c>
       <c r="I17" s="6" t="n">
-        <v>2194</v>
+        <v>2427</v>
       </c>
       <c r="J17" s="6" t="inlineStr">
         <is>
-          <t>2026-05-22~05-25</t>
+          <t>2026-05-11~05-12</t>
         </is>
       </c>
       <c r="K17" s="6" t="inlineStr">
         <is>
-          <t>1,486.88</t>
+          <t>2,807.79</t>
         </is>
       </c>
       <c r="L17" s="6" t="inlineStr"/>
       <c r="M17" s="6" t="inlineStr">
         <is>
-          <t>2026-06-05</t>
+          <t>2026-05-20</t>
         </is>
       </c>
       <c r="N17" s="6" t="inlineStr">
         <is>
-          <t>대신</t>
+          <t>미래</t>
         </is>
       </c>
       <c r="O17" s="6" t="inlineStr"/>
       <c r="P17" s="7" t="inlineStr">
         <is>
-          <t>390</t>
+          <t>2,026</t>
         </is>
       </c>
       <c r="Q17" s="6" t="inlineStr">
         <is>
-          <t>3.00%</t>
+          <t>5.00%</t>
         </is>
       </c>
       <c r="R17" s="6" t="inlineStr">
@@ -7981,7 +7975,7 @@
     <row r="18" ht="30" customHeight="1">
       <c r="A18" s="6" t="inlineStr">
         <is>
-          <t>마키나락스</t>
+          <t>폴레드</t>
         </is>
       </c>
       <c r="B18" s="18" t="inlineStr">
@@ -7991,63 +7985,63 @@
       </c>
       <c r="C18" s="6" t="inlineStr">
         <is>
-          <t>12,500~15,000</t>
+          <t>4,100~5,000</t>
         </is>
       </c>
       <c r="D18" s="7" t="inlineStr">
         <is>
-          <t>2,635,000</t>
+          <t>2,600,000</t>
         </is>
       </c>
       <c r="E18" s="7" t="inlineStr">
         <is>
-          <t>39,525</t>
+          <t>13,000</t>
         </is>
       </c>
       <c r="F18" s="6" t="inlineStr">
         <is>
-          <t>40.5배 (PER)</t>
+          <t>19.05배 (PER)</t>
         </is>
       </c>
       <c r="G18" s="6" t="n">
-        <v>15000</v>
+        <v>5000</v>
       </c>
       <c r="H18" s="6" t="n">
-        <v>1196.08</v>
+        <v>1486.66</v>
       </c>
       <c r="I18" s="6" t="n">
-        <v>2427</v>
+        <v>2372</v>
       </c>
       <c r="J18" s="6" t="inlineStr">
         <is>
-          <t>2026-05-11~05-12</t>
+          <t>2026-05-04~05-05</t>
         </is>
       </c>
       <c r="K18" s="6" t="inlineStr">
         <is>
-          <t>2,807.79</t>
+          <t>3,169.86</t>
         </is>
       </c>
       <c r="L18" s="6" t="inlineStr"/>
       <c r="M18" s="6" t="inlineStr">
         <is>
-          <t>2026-05-20</t>
+          <t>2026-05-14</t>
         </is>
       </c>
       <c r="N18" s="6" t="inlineStr">
         <is>
-          <t>미래</t>
+          <t>NH</t>
         </is>
       </c>
       <c r="O18" s="6" t="inlineStr"/>
       <c r="P18" s="7" t="inlineStr">
         <is>
-          <t>2,026</t>
+          <t>540</t>
         </is>
       </c>
       <c r="Q18" s="6" t="inlineStr">
         <is>
-          <t>5.00%</t>
+          <t>4.03%</t>
         </is>
       </c>
       <c r="R18" s="6" t="inlineStr">
@@ -8059,7 +8053,7 @@
     <row r="19" ht="30" customHeight="1">
       <c r="A19" s="6" t="inlineStr">
         <is>
-          <t>폴레드</t>
+          <t>코스모로보틱스</t>
         </is>
       </c>
       <c r="B19" s="18" t="inlineStr">
@@ -8069,63 +8063,67 @@
       </c>
       <c r="C19" s="6" t="inlineStr">
         <is>
-          <t>4,100~5,000</t>
+          <t>5,300~6,000</t>
         </is>
       </c>
       <c r="D19" s="7" t="inlineStr">
         <is>
-          <t>2,600,000</t>
+          <t>4,170,000</t>
         </is>
       </c>
       <c r="E19" s="7" t="inlineStr">
         <is>
-          <t>13,000</t>
+          <t>25,020</t>
         </is>
       </c>
       <c r="F19" s="6" t="inlineStr">
         <is>
-          <t>19.05배 (PER)</t>
+          <t>47.45배 (PER)</t>
         </is>
       </c>
       <c r="G19" s="6" t="n">
-        <v>5000</v>
+        <v>6000</v>
       </c>
       <c r="H19" s="6" t="n">
-        <v>1486.66</v>
+        <v>1140.11</v>
       </c>
       <c r="I19" s="6" t="n">
-        <v>2372</v>
+        <v>2257</v>
       </c>
       <c r="J19" s="6" t="inlineStr">
         <is>
-          <t>2026-05-04~05-05</t>
+          <t>2026-04-27~04-28</t>
         </is>
       </c>
       <c r="K19" s="6" t="inlineStr">
         <is>
-          <t>3,169.86</t>
+          <t>2,013.80</t>
         </is>
       </c>
       <c r="L19" s="6" t="inlineStr"/>
       <c r="M19" s="6" t="inlineStr">
         <is>
-          <t>2026-05-14</t>
+          <t>2026-05-11</t>
         </is>
       </c>
       <c r="N19" s="6" t="inlineStr">
         <is>
+          <t>유진</t>
+        </is>
+      </c>
+      <c r="O19" s="6" t="inlineStr">
+        <is>
           <t>NH</t>
         </is>
       </c>
-      <c r="O19" s="6" t="inlineStr"/>
       <c r="P19" s="7" t="inlineStr">
         <is>
-          <t>540</t>
+          <t>1,289</t>
         </is>
       </c>
       <c r="Q19" s="6" t="inlineStr">
         <is>
-          <t>4.03%</t>
+          <t>3.78%</t>
         </is>
       </c>
       <c r="R19" s="6" t="inlineStr">
@@ -8137,77 +8135,75 @@
     <row r="20" ht="30" customHeight="1">
       <c r="A20" s="6" t="inlineStr">
         <is>
-          <t>코스모로보틱스</t>
-        </is>
-      </c>
-      <c r="B20" s="18" t="inlineStr">
-        <is>
-          <t>수집예정</t>
+          <t>신한스팩18호</t>
+        </is>
+      </c>
+      <c r="B20" s="19" t="inlineStr">
+        <is>
+          <t>해당없음</t>
         </is>
       </c>
       <c r="C20" s="6" t="inlineStr">
         <is>
-          <t>5,300~6,000</t>
+          <t>2,000</t>
         </is>
       </c>
       <c r="D20" s="7" t="inlineStr">
         <is>
-          <t>4,170,000</t>
+          <t>5,000,000</t>
         </is>
       </c>
       <c r="E20" s="7" t="inlineStr">
         <is>
-          <t>25,020</t>
-        </is>
-      </c>
-      <c r="F20" s="6" t="inlineStr">
-        <is>
-          <t>47.45배 (PER)</t>
-        </is>
-      </c>
-      <c r="G20" s="6" t="n">
-        <v>6000</v>
+          <t>10,000</t>
+        </is>
+      </c>
+      <c r="F20" s="19" t="inlineStr">
+        <is>
+          <t>해당없음</t>
+        </is>
+      </c>
+      <c r="G20" s="6" t="inlineStr">
+        <is>
+          <t>2,000</t>
+        </is>
       </c>
       <c r="H20" s="6" t="n">
-        <v>1140.11</v>
+        <v>1388.6</v>
       </c>
       <c r="I20" s="6" t="n">
-        <v>2257</v>
+        <v>2044</v>
       </c>
       <c r="J20" s="6" t="inlineStr">
         <is>
-          <t>2026-04-27~04-28</t>
+          <t>2026-04-20~04-21</t>
         </is>
       </c>
       <c r="K20" s="6" t="inlineStr">
         <is>
-          <t>2,013.80</t>
+          <t>1,601.36</t>
         </is>
       </c>
       <c r="L20" s="6" t="inlineStr"/>
       <c r="M20" s="6" t="inlineStr">
         <is>
-          <t>2026-05-11</t>
+          <t>2026-04-30</t>
         </is>
       </c>
       <c r="N20" s="6" t="inlineStr">
         <is>
-          <t>유진</t>
-        </is>
-      </c>
-      <c r="O20" s="6" t="inlineStr">
-        <is>
-          <t>NH</t>
-        </is>
-      </c>
+          <t>신한</t>
+        </is>
+      </c>
+      <c r="O20" s="6" t="inlineStr"/>
       <c r="P20" s="7" t="inlineStr">
         <is>
-          <t>1,289</t>
+          <t>350</t>
         </is>
       </c>
       <c r="Q20" s="6" t="inlineStr">
         <is>
-          <t>3.78%</t>
+          <t>3.50%</t>
         </is>
       </c>
       <c r="R20" s="6" t="inlineStr">
@@ -8219,44 +8215,42 @@
     <row r="21" ht="30" customHeight="1">
       <c r="A21" s="6" t="inlineStr">
         <is>
-          <t>신한스팩18호</t>
-        </is>
-      </c>
-      <c r="B21" s="19" t="inlineStr">
-        <is>
-          <t>해당없음</t>
+          <t>채비</t>
+        </is>
+      </c>
+      <c r="B21" s="18" t="inlineStr">
+        <is>
+          <t>수집예정</t>
         </is>
       </c>
       <c r="C21" s="6" t="inlineStr">
         <is>
-          <t>2,000</t>
+          <t>12,300~15,300</t>
         </is>
       </c>
       <c r="D21" s="7" t="inlineStr">
         <is>
-          <t>5,000,000</t>
+          <t>9,000,000</t>
         </is>
       </c>
       <c r="E21" s="7" t="inlineStr">
         <is>
-          <t>10,000</t>
-        </is>
-      </c>
-      <c r="F21" s="19" t="inlineStr">
-        <is>
-          <t>해당없음</t>
-        </is>
-      </c>
-      <c r="G21" s="6" t="inlineStr">
-        <is>
-          <t>2,000</t>
-        </is>
+          <t>110,700</t>
+        </is>
+      </c>
+      <c r="F21" s="6" t="inlineStr">
+        <is>
+          <t>24.0배 (EV/EBITDA)</t>
+        </is>
+      </c>
+      <c r="G21" s="6" t="n">
+        <v>12300</v>
       </c>
       <c r="H21" s="6" t="n">
-        <v>1388.6</v>
+        <v>55.23</v>
       </c>
       <c r="I21" s="6" t="n">
-        <v>2044</v>
+        <v>751</v>
       </c>
       <c r="J21" s="6" t="inlineStr">
         <is>
@@ -8265,29 +8259,33 @@
       </c>
       <c r="K21" s="6" t="inlineStr">
         <is>
-          <t>1,601.36</t>
+          <t>302.11</t>
         </is>
       </c>
       <c r="L21" s="6" t="inlineStr"/>
       <c r="M21" s="6" t="inlineStr">
         <is>
-          <t>2026-04-30</t>
+          <t>2026-04-29</t>
         </is>
       </c>
       <c r="N21" s="6" t="inlineStr">
         <is>
-          <t>신한</t>
-        </is>
-      </c>
-      <c r="O21" s="6" t="inlineStr"/>
+          <t>KB</t>
+        </is>
+      </c>
+      <c r="O21" s="6" t="inlineStr">
+        <is>
+          <t>삼성</t>
+        </is>
+      </c>
       <c r="P21" s="7" t="inlineStr">
         <is>
-          <t>350</t>
+          <t>3,384</t>
         </is>
       </c>
       <c r="Q21" s="6" t="inlineStr">
         <is>
-          <t>3.50%</t>
+          <t>3.00%</t>
         </is>
       </c>
       <c r="R21" s="6" t="inlineStr">
@@ -8299,77 +8297,75 @@
     <row r="22" ht="30" customHeight="1">
       <c r="A22" s="6" t="inlineStr">
         <is>
-          <t>채비</t>
-        </is>
-      </c>
-      <c r="B22" s="18" t="inlineStr">
-        <is>
-          <t>수집예정</t>
+          <t>키움히어로스펙2호</t>
+        </is>
+      </c>
+      <c r="B22" s="19" t="inlineStr">
+        <is>
+          <t>해당없음</t>
         </is>
       </c>
       <c r="C22" s="6" t="inlineStr">
         <is>
-          <t>12,300~15,300</t>
+          <t>2,000</t>
         </is>
       </c>
       <c r="D22" s="7" t="inlineStr">
         <is>
-          <t>9,000,000</t>
+          <t>6,000,000</t>
         </is>
       </c>
       <c r="E22" s="7" t="inlineStr">
         <is>
-          <t>110,700</t>
-        </is>
-      </c>
-      <c r="F22" s="6" t="inlineStr">
-        <is>
-          <t>24.0배 (EV/EBITDA)</t>
-        </is>
-      </c>
-      <c r="G22" s="6" t="n">
-        <v>12300</v>
+          <t>12,000</t>
+        </is>
+      </c>
+      <c r="F22" s="19" t="inlineStr">
+        <is>
+          <t>해당없음</t>
+        </is>
+      </c>
+      <c r="G22" s="6" t="inlineStr">
+        <is>
+          <t>2,000</t>
+        </is>
       </c>
       <c r="H22" s="6" t="n">
-        <v>55.23</v>
+        <v>1271.12</v>
       </c>
       <c r="I22" s="6" t="n">
-        <v>751</v>
+        <v>2054</v>
       </c>
       <c r="J22" s="6" t="inlineStr">
         <is>
-          <t>2026-04-20~04-21</t>
+          <t>2026-04-14~04-15</t>
         </is>
       </c>
       <c r="K22" s="6" t="inlineStr">
         <is>
-          <t>302.11</t>
+          <t>1,727.59</t>
         </is>
       </c>
       <c r="L22" s="6" t="inlineStr"/>
       <c r="M22" s="6" t="inlineStr">
         <is>
-          <t>2026-04-29</t>
+          <t>2026-04-23</t>
         </is>
       </c>
       <c r="N22" s="6" t="inlineStr">
         <is>
-          <t>KB</t>
-        </is>
-      </c>
-      <c r="O22" s="6" t="inlineStr">
-        <is>
-          <t>삼성</t>
-        </is>
-      </c>
+          <t>키움</t>
+        </is>
+      </c>
+      <c r="O22" s="6" t="inlineStr"/>
       <c r="P22" s="7" t="inlineStr">
         <is>
-          <t>3,384</t>
+          <t>300</t>
         </is>
       </c>
       <c r="Q22" s="6" t="inlineStr">
         <is>
-          <t>3.00%</t>
+          <t>2.50%</t>
         </is>
       </c>
       <c r="R22" s="6" t="inlineStr">
@@ -8381,7 +8377,7 @@
     <row r="23" ht="30" customHeight="1">
       <c r="A23" s="6" t="inlineStr">
         <is>
-          <t>키움히어로스펙2호</t>
+          <t>교보스팩20호</t>
         </is>
       </c>
       <c r="B23" s="19" t="inlineStr">
@@ -8396,12 +8392,12 @@
       </c>
       <c r="D23" s="7" t="inlineStr">
         <is>
-          <t>6,000,000</t>
+          <t>5,400,000</t>
         </is>
       </c>
       <c r="E23" s="7" t="inlineStr">
         <is>
-          <t>12,000</t>
+          <t>10,800</t>
         </is>
       </c>
       <c r="F23" s="19" t="inlineStr">
@@ -8415,30 +8411,30 @@
         </is>
       </c>
       <c r="H23" s="6" t="n">
-        <v>1271.12</v>
+        <v>1196.99</v>
       </c>
       <c r="I23" s="6" t="n">
-        <v>2054</v>
+        <v>1855</v>
       </c>
       <c r="J23" s="6" t="inlineStr">
         <is>
-          <t>2026-04-14~04-15</t>
+          <t>2026-03-23~03-24</t>
         </is>
       </c>
       <c r="K23" s="6" t="inlineStr">
         <is>
-          <t>1,727.59</t>
+          <t>747.00</t>
         </is>
       </c>
       <c r="L23" s="6" t="inlineStr"/>
       <c r="M23" s="6" t="inlineStr">
         <is>
-          <t>2026-04-23</t>
+          <t>2026-04-02</t>
         </is>
       </c>
       <c r="N23" s="6" t="inlineStr">
         <is>
-          <t>키움</t>
+          <t>교보</t>
         </is>
       </c>
       <c r="O23" s="6" t="inlineStr"/>
@@ -8449,7 +8445,7 @@
       </c>
       <c r="Q23" s="6" t="inlineStr">
         <is>
-          <t>2.50%</t>
+          <t>2.78%</t>
         </is>
       </c>
       <c r="R23" s="6" t="inlineStr">
@@ -8461,44 +8457,42 @@
     <row r="24" ht="30" customHeight="1">
       <c r="A24" s="6" t="inlineStr">
         <is>
-          <t>교보스팩20호</t>
-        </is>
-      </c>
-      <c r="B24" s="19" t="inlineStr">
-        <is>
-          <t>해당없음</t>
+          <t>인벤테라</t>
+        </is>
+      </c>
+      <c r="B24" s="18" t="inlineStr">
+        <is>
+          <t>수집예정</t>
         </is>
       </c>
       <c r="C24" s="6" t="inlineStr">
         <is>
-          <t>2,000</t>
+          <t>12,100~16,600</t>
         </is>
       </c>
       <c r="D24" s="7" t="inlineStr">
         <is>
-          <t>5,400,000</t>
+          <t>1,180,000</t>
         </is>
       </c>
       <c r="E24" s="7" t="inlineStr">
         <is>
-          <t>10,800</t>
-        </is>
-      </c>
-      <c r="F24" s="19" t="inlineStr">
-        <is>
-          <t>해당없음</t>
-        </is>
-      </c>
-      <c r="G24" s="6" t="inlineStr">
-        <is>
-          <t>2,000</t>
-        </is>
+          <t>19,588</t>
+        </is>
+      </c>
+      <c r="F24" s="6" t="inlineStr">
+        <is>
+          <t>24.34배 (PER)</t>
+        </is>
+      </c>
+      <c r="G24" s="6" t="n">
+        <v>16600</v>
       </c>
       <c r="H24" s="6" t="n">
-        <v>1196.99</v>
+        <v>1328.82</v>
       </c>
       <c r="I24" s="6" t="n">
-        <v>1855</v>
+        <v>2309</v>
       </c>
       <c r="J24" s="6" t="inlineStr">
         <is>
@@ -8507,7 +8501,7 @@
       </c>
       <c r="K24" s="6" t="inlineStr">
         <is>
-          <t>747.00</t>
+          <t>1,913.00</t>
         </is>
       </c>
       <c r="L24" s="6" t="inlineStr"/>
@@ -8518,18 +8512,18 @@
       </c>
       <c r="N24" s="6" t="inlineStr">
         <is>
-          <t>교보</t>
+          <t>NH</t>
         </is>
       </c>
       <c r="O24" s="6" t="inlineStr"/>
       <c r="P24" s="7" t="inlineStr">
         <is>
-          <t>300</t>
+          <t>1,211</t>
         </is>
       </c>
       <c r="Q24" s="6" t="inlineStr">
         <is>
-          <t>2.78%</t>
+          <t>6.00%</t>
         </is>
       </c>
       <c r="R24" s="6" t="inlineStr">
@@ -8541,73 +8535,75 @@
     <row r="25" ht="30" customHeight="1">
       <c r="A25" s="6" t="inlineStr">
         <is>
-          <t>인벤테라</t>
-        </is>
-      </c>
-      <c r="B25" s="18" t="inlineStr">
-        <is>
-          <t>수집예정</t>
+          <t>신한스팩17호</t>
+        </is>
+      </c>
+      <c r="B25" s="19" t="inlineStr">
+        <is>
+          <t>해당없음</t>
         </is>
       </c>
       <c r="C25" s="6" t="inlineStr">
         <is>
-          <t>12,100~16,600</t>
+          <t>2,000</t>
         </is>
       </c>
       <c r="D25" s="7" t="inlineStr">
         <is>
-          <t>1,180,000</t>
+          <t>5,000,000</t>
         </is>
       </c>
       <c r="E25" s="7" t="inlineStr">
         <is>
-          <t>19,588</t>
-        </is>
-      </c>
-      <c r="F25" s="6" t="inlineStr">
-        <is>
-          <t>24.34배 (PER)</t>
-        </is>
-      </c>
-      <c r="G25" s="6" t="n">
-        <v>16600</v>
+          <t>10,000</t>
+        </is>
+      </c>
+      <c r="F25" s="19" t="inlineStr">
+        <is>
+          <t>해당없음</t>
+        </is>
+      </c>
+      <c r="G25" s="6" t="inlineStr">
+        <is>
+          <t>2,000</t>
+        </is>
       </c>
       <c r="H25" s="6" t="n">
-        <v>1328.82</v>
+        <v>1343.8</v>
       </c>
       <c r="I25" s="6" t="n">
-        <v>2309</v>
+        <v>2022</v>
       </c>
       <c r="J25" s="6" t="inlineStr">
         <is>
-          <t>2026-03-23~03-24</t>
+          <t>2026-03-19~03-20</t>
         </is>
       </c>
       <c r="K25" s="6" t="inlineStr">
         <is>
-          <t>1,913.00</t>
+          <t>1,403.74</t>
         </is>
       </c>
       <c r="L25" s="6" t="inlineStr"/>
       <c r="M25" s="6" t="inlineStr">
         <is>
-          <t>2026-04-02</t>
+          <t>2026-04-01</t>
         </is>
       </c>
       <c r="N25" s="6" t="inlineStr">
         <is>
-          <t>NH</t>
+          <t>신한</t>
         </is>
       </c>
       <c r="O25" s="6" t="inlineStr"/>
       <c r="P25" s="7" t="inlineStr">
         <is>
-          <t>1,211</t>
+          <t>350</t>
         </is>
       </c>
       <c r="Q25" s="6" t="inlineStr">
         <is>
-          <t>6.00%</t>
+          <t>3.50%</t>
         </is>
       </c>
       <c r="R25" s="6" t="inlineStr">
@@ -8619,44 +8615,42 @@
     <row r="26" ht="30" customHeight="1">
       <c r="A26" s="6" t="inlineStr">
         <is>
-          <t>신한스팩17호</t>
-        </is>
-      </c>
-      <c r="B26" s="19" t="inlineStr">
-        <is>
-          <t>해당없음</t>
+          <t>리센스메디컬</t>
+        </is>
+      </c>
+      <c r="B26" s="18" t="inlineStr">
+        <is>
+          <t>수집예정</t>
         </is>
       </c>
       <c r="C26" s="6" t="inlineStr">
         <is>
-          <t>2,000</t>
+          <t>9,000~11,000</t>
         </is>
       </c>
       <c r="D26" s="7" t="inlineStr">
         <is>
-          <t>5,000,000</t>
+          <t>1,400,000</t>
         </is>
       </c>
       <c r="E26" s="7" t="inlineStr">
         <is>
-          <t>10,000</t>
-        </is>
-      </c>
-      <c r="F26" s="19" t="inlineStr">
-        <is>
-          <t>해당없음</t>
-        </is>
-      </c>
-      <c r="G26" s="6" t="inlineStr">
-        <is>
-          <t>2,000</t>
-        </is>
+          <t>15,400</t>
+        </is>
+      </c>
+      <c r="F26" s="6" t="inlineStr">
+        <is>
+          <t>31.33배 (PER)</t>
+        </is>
+      </c>
+      <c r="G26" s="6" t="n">
+        <v>11000</v>
       </c>
       <c r="H26" s="6" t="n">
-        <v>1343.8</v>
+        <v>1352.63</v>
       </c>
       <c r="I26" s="6" t="n">
-        <v>2022</v>
+        <v>2261</v>
       </c>
       <c r="J26" s="6" t="inlineStr">
         <is>
@@ -8665,29 +8659,33 @@
       </c>
       <c r="K26" s="6" t="inlineStr">
         <is>
-          <t>1,403.74</t>
+          <t>2,097.68</t>
         </is>
       </c>
       <c r="L26" s="6" t="inlineStr"/>
       <c r="M26" s="6" t="inlineStr">
         <is>
-          <t>2026-04-01</t>
+          <t>2026-03-31</t>
         </is>
       </c>
       <c r="N26" s="6" t="inlineStr">
         <is>
-          <t>신한</t>
-        </is>
-      </c>
-      <c r="O26" s="6" t="inlineStr"/>
+          <t>한국</t>
+        </is>
+      </c>
+      <c r="O26" s="6" t="inlineStr">
+        <is>
+          <t>KB</t>
+        </is>
+      </c>
       <c r="P26" s="7" t="inlineStr">
         <is>
-          <t>350</t>
+          <t>916</t>
         </is>
       </c>
       <c r="Q26" s="6" t="inlineStr">
         <is>
-          <t>3.50%</t>
+          <t>5.77%</t>
         </is>
       </c>
       <c r="R26" s="6" t="inlineStr">
@@ -8699,77 +8697,75 @@
     <row r="27" ht="30" customHeight="1">
       <c r="A27" s="6" t="inlineStr">
         <is>
-          <t>리센스메디컬</t>
-        </is>
-      </c>
-      <c r="B27" s="18" t="inlineStr">
-        <is>
-          <t>수집예정</t>
+          <t>NH스팩33호</t>
+        </is>
+      </c>
+      <c r="B27" s="19" t="inlineStr">
+        <is>
+          <t>해당없음</t>
         </is>
       </c>
       <c r="C27" s="6" t="inlineStr">
         <is>
-          <t>9,000~11,000</t>
+          <t>2,000</t>
         </is>
       </c>
       <c r="D27" s="7" t="inlineStr">
         <is>
-          <t>1,400,000</t>
+          <t>6,350,000</t>
         </is>
       </c>
       <c r="E27" s="7" t="inlineStr">
         <is>
-          <t>15,400</t>
-        </is>
-      </c>
-      <c r="F27" s="6" t="inlineStr">
-        <is>
-          <t>31.33배 (PER)</t>
-        </is>
-      </c>
-      <c r="G27" s="6" t="n">
-        <v>11000</v>
+          <t>12,700</t>
+        </is>
+      </c>
+      <c r="F27" s="19" t="inlineStr">
+        <is>
+          <t>해당없음</t>
+        </is>
+      </c>
+      <c r="G27" s="6" t="inlineStr">
+        <is>
+          <t>2,000</t>
+        </is>
       </c>
       <c r="H27" s="6" t="n">
-        <v>1352.63</v>
+        <v>1228.71</v>
       </c>
       <c r="I27" s="6" t="n">
-        <v>2261</v>
+        <v>2058</v>
       </c>
       <c r="J27" s="6" t="inlineStr">
         <is>
-          <t>2026-03-19~03-20</t>
+          <t>2026-03-17~03-18</t>
         </is>
       </c>
       <c r="K27" s="6" t="inlineStr">
         <is>
-          <t>2,097.68</t>
+          <t>569.27</t>
         </is>
       </c>
       <c r="L27" s="6" t="inlineStr"/>
       <c r="M27" s="6" t="inlineStr">
         <is>
-          <t>2026-03-31</t>
+          <t>2026-03-27</t>
         </is>
       </c>
       <c r="N27" s="6" t="inlineStr">
         <is>
-          <t>한국</t>
-        </is>
-      </c>
-      <c r="O27" s="6" t="inlineStr">
-        <is>
-          <t>KB</t>
-        </is>
-      </c>
+          <t>NH</t>
+        </is>
+      </c>
+      <c r="O27" s="6" t="inlineStr"/>
       <c r="P27" s="7" t="inlineStr">
         <is>
-          <t>916</t>
+          <t>381</t>
         </is>
       </c>
       <c r="Q27" s="6" t="inlineStr">
         <is>
-          <t>5.77%</t>
+          <t>3.00%</t>
         </is>
       </c>
       <c r="R27" s="6" t="inlineStr">
@@ -8781,75 +8777,73 @@
     <row r="28" ht="30" customHeight="1">
       <c r="A28" s="6" t="inlineStr">
         <is>
-          <t>NH스팩33호</t>
-        </is>
-      </c>
-      <c r="B28" s="19" t="inlineStr">
-        <is>
-          <t>해당없음</t>
+          <t>메쥬</t>
+        </is>
+      </c>
+      <c r="B28" s="18" t="inlineStr">
+        <is>
+          <t>수집예정</t>
         </is>
       </c>
       <c r="C28" s="6" t="inlineStr">
         <is>
-          <t>2,000</t>
+          <t>16,700~21,600</t>
         </is>
       </c>
       <c r="D28" s="7" t="inlineStr">
         <is>
-          <t>6,350,000</t>
+          <t>1,345,000</t>
         </is>
       </c>
       <c r="E28" s="7" t="inlineStr">
         <is>
-          <t>12,700</t>
-        </is>
-      </c>
-      <c r="F28" s="19" t="inlineStr">
-        <is>
-          <t>해당없음</t>
-        </is>
-      </c>
-      <c r="G28" s="6" t="inlineStr">
-        <is>
-          <t>2,000</t>
-        </is>
+          <t>29,052</t>
+        </is>
+      </c>
+      <c r="F28" s="6" t="inlineStr">
+        <is>
+          <t>20.66배 (PER)</t>
+        </is>
+      </c>
+      <c r="G28" s="6" t="n">
+        <v>21600</v>
       </c>
       <c r="H28" s="6" t="n">
-        <v>1228.71</v>
+        <v>1108.93</v>
       </c>
       <c r="I28" s="6" t="n">
-        <v>2058</v>
+        <v>2320</v>
       </c>
       <c r="J28" s="6" t="inlineStr">
         <is>
-          <t>2026-03-17~03-18</t>
+          <t>2026-03-16~03-17</t>
         </is>
       </c>
       <c r="K28" s="6" t="inlineStr">
         <is>
-          <t>569.27</t>
+          <t>2,428.25</t>
         </is>
       </c>
       <c r="L28" s="6" t="inlineStr"/>
       <c r="M28" s="6" t="inlineStr">
         <is>
-          <t>2026-03-27</t>
+          <t>2026-03-26</t>
         </is>
       </c>
       <c r="N28" s="6" t="inlineStr">
         <is>
-          <t>NH</t>
+          <t>신한</t>
         </is>
       </c>
       <c r="O28" s="6" t="inlineStr"/>
       <c r="P28" s="7" t="inlineStr">
         <is>
-          <t>381</t>
+          <t>1,496</t>
         </is>
       </c>
       <c r="Q28" s="6" t="inlineStr">
         <is>
-          <t>3.00%</t>
+          <t>5.00%</t>
         </is>
       </c>
       <c r="R28" s="6" t="inlineStr">
@@ -8861,7 +8855,7 @@
     <row r="29" ht="30" customHeight="1">
       <c r="A29" s="6" t="inlineStr">
         <is>
-          <t>메쥬</t>
+          <t>한패스</t>
         </is>
       </c>
       <c r="B29" s="18" t="inlineStr">
@@ -8871,32 +8865,32 @@
       </c>
       <c r="C29" s="6" t="inlineStr">
         <is>
-          <t>16,700~21,600</t>
+          <t>17,000~19,000</t>
         </is>
       </c>
       <c r="D29" s="7" t="inlineStr">
         <is>
-          <t>1,345,000</t>
+          <t>1,100,000</t>
         </is>
       </c>
       <c r="E29" s="7" t="inlineStr">
         <is>
-          <t>29,052</t>
+          <t>20,900</t>
         </is>
       </c>
       <c r="F29" s="6" t="inlineStr">
         <is>
-          <t>20.66배 (PER)</t>
+          <t>29.09배 (PER)</t>
         </is>
       </c>
       <c r="G29" s="6" t="n">
-        <v>21600</v>
+        <v>19000</v>
       </c>
       <c r="H29" s="6" t="n">
-        <v>1108.93</v>
+        <v>1172.59</v>
       </c>
       <c r="I29" s="6" t="n">
-        <v>2320</v>
+        <v>2229</v>
       </c>
       <c r="J29" s="6" t="inlineStr">
         <is>
@@ -8905,29 +8899,29 @@
       </c>
       <c r="K29" s="6" t="inlineStr">
         <is>
-          <t>2,428.25</t>
+          <t>1,673.04</t>
         </is>
       </c>
       <c r="L29" s="6" t="inlineStr"/>
       <c r="M29" s="6" t="inlineStr">
         <is>
-          <t>2026-03-26</t>
+          <t>2026-03-25</t>
         </is>
       </c>
       <c r="N29" s="6" t="inlineStr">
         <is>
-          <t>신한</t>
+          <t>한국</t>
         </is>
       </c>
       <c r="O29" s="6" t="inlineStr"/>
       <c r="P29" s="7" t="inlineStr">
         <is>
-          <t>1,496</t>
+          <t>753</t>
         </is>
       </c>
       <c r="Q29" s="6" t="inlineStr">
         <is>
-          <t>5.00%</t>
+          <t>3.50%</t>
         </is>
       </c>
       <c r="R29" s="6" t="inlineStr">
@@ -8939,7 +8933,7 @@
     <row r="30" ht="30" customHeight="1">
       <c r="A30" s="6" t="inlineStr">
         <is>
-          <t>한패스</t>
+          <t>아이엠바이오로직스</t>
         </is>
       </c>
       <c r="B30" s="18" t="inlineStr">
@@ -8949,47 +8943,47 @@
       </c>
       <c r="C30" s="6" t="inlineStr">
         <is>
-          <t>17,000~19,000</t>
+          <t>19,000~26,000</t>
         </is>
       </c>
       <c r="D30" s="7" t="inlineStr">
         <is>
-          <t>1,100,000</t>
+          <t>2,000,000</t>
         </is>
       </c>
       <c r="E30" s="7" t="inlineStr">
         <is>
-          <t>20,900</t>
+          <t>52,000</t>
         </is>
       </c>
       <c r="F30" s="6" t="inlineStr">
         <is>
-          <t>29.09배 (PER)</t>
+          <t>21.46배 (PER)</t>
         </is>
       </c>
       <c r="G30" s="6" t="n">
-        <v>19000</v>
+        <v>26000</v>
       </c>
       <c r="H30" s="6" t="n">
-        <v>1172.59</v>
+        <v>839.23</v>
       </c>
       <c r="I30" s="6" t="n">
-        <v>2229</v>
+        <v>2333</v>
       </c>
       <c r="J30" s="6" t="inlineStr">
         <is>
-          <t>2026-03-16~03-17</t>
+          <t>2026-03-11~03-12</t>
         </is>
       </c>
       <c r="K30" s="6" t="inlineStr">
         <is>
-          <t>1,673.04</t>
+          <t>1,806.00</t>
         </is>
       </c>
       <c r="L30" s="6" t="inlineStr"/>
       <c r="M30" s="6" t="inlineStr">
         <is>
-          <t>2026-03-25</t>
+          <t>2026-03-20</t>
         </is>
       </c>
       <c r="N30" s="6" t="inlineStr">
@@ -9000,12 +8994,12 @@
       <c r="O30" s="6" t="inlineStr"/>
       <c r="P30" s="7" t="inlineStr">
         <is>
-          <t>753</t>
+          <t>2,650</t>
         </is>
       </c>
       <c r="Q30" s="6" t="inlineStr">
         <is>
-          <t>3.50%</t>
+          <t>5.00%</t>
         </is>
       </c>
       <c r="R30" s="6" t="inlineStr">
@@ -9017,7 +9011,7 @@
     <row r="31" ht="30" customHeight="1">
       <c r="A31" s="6" t="inlineStr">
         <is>
-          <t>아이엠바이오로직스</t>
+          <t>카나프테라퓨틱스</t>
         </is>
       </c>
       <c r="B31" s="18" t="inlineStr">
@@ -9027,7 +9021,7 @@
       </c>
       <c r="C31" s="6" t="inlineStr">
         <is>
-          <t>19,000~26,000</t>
+          <t>16,000~20,000</t>
         </is>
       </c>
       <c r="D31" s="7" t="inlineStr">
@@ -9037,37 +9031,37 @@
       </c>
       <c r="E31" s="7" t="inlineStr">
         <is>
-          <t>52,000</t>
+          <t>40,000</t>
         </is>
       </c>
       <c r="F31" s="6" t="inlineStr">
         <is>
-          <t>21.46배 (PER)</t>
+          <t>23.59배 (PER)</t>
         </is>
       </c>
       <c r="G31" s="6" t="n">
-        <v>26000</v>
+        <v>20000</v>
       </c>
       <c r="H31" s="6" t="n">
-        <v>839.23</v>
+        <v>962.1</v>
       </c>
       <c r="I31" s="6" t="n">
-        <v>2333</v>
+        <v>2327</v>
       </c>
       <c r="J31" s="6" t="inlineStr">
         <is>
-          <t>2026-03-11~03-12</t>
+          <t>2026-03-05~03-06</t>
         </is>
       </c>
       <c r="K31" s="6" t="inlineStr">
         <is>
-          <t>1,806.00</t>
+          <t>1,899.29</t>
         </is>
       </c>
       <c r="L31" s="6" t="inlineStr"/>
       <c r="M31" s="6" t="inlineStr">
         <is>
-          <t>2026-03-20</t>
+          <t>2026-03-16</t>
         </is>
       </c>
       <c r="N31" s="6" t="inlineStr">
@@ -9078,7 +9072,7 @@
       <c r="O31" s="6" t="inlineStr"/>
       <c r="P31" s="7" t="inlineStr">
         <is>
-          <t>2,650</t>
+          <t>2,050</t>
         </is>
       </c>
       <c r="Q31" s="6" t="inlineStr">
@@ -9095,7 +9089,7 @@
     <row r="32" ht="30" customHeight="1">
       <c r="A32" s="6" t="inlineStr">
         <is>
-          <t>카나프테라퓨틱스</t>
+          <t>액스비스</t>
         </is>
       </c>
       <c r="B32" s="18" t="inlineStr">
@@ -9105,63 +9099,63 @@
       </c>
       <c r="C32" s="6" t="inlineStr">
         <is>
-          <t>16,000~20,000</t>
+          <t>10,100~11,500</t>
         </is>
       </c>
       <c r="D32" s="7" t="inlineStr">
         <is>
-          <t>2,000,000</t>
+          <t>2,300,000</t>
         </is>
       </c>
       <c r="E32" s="7" t="inlineStr">
         <is>
-          <t>40,000</t>
+          <t>26,450</t>
         </is>
       </c>
       <c r="F32" s="6" t="inlineStr">
         <is>
-          <t>23.59배 (PER)</t>
+          <t>27.60배 (PER)</t>
         </is>
       </c>
       <c r="G32" s="6" t="n">
-        <v>20000</v>
+        <v>11500</v>
       </c>
       <c r="H32" s="6" t="n">
-        <v>962.1</v>
+        <v>1124.21</v>
       </c>
       <c r="I32" s="6" t="n">
-        <v>2327</v>
+        <v>2411</v>
       </c>
       <c r="J32" s="6" t="inlineStr">
         <is>
-          <t>2026-03-05~03-06</t>
+          <t>2026-02-23~02-24</t>
         </is>
       </c>
       <c r="K32" s="6" t="inlineStr">
         <is>
-          <t>1,899.29</t>
+          <t>1,960.87</t>
         </is>
       </c>
       <c r="L32" s="6" t="inlineStr"/>
       <c r="M32" s="6" t="inlineStr">
         <is>
-          <t>2026-03-16</t>
+          <t>2026-03-09</t>
         </is>
       </c>
       <c r="N32" s="6" t="inlineStr">
         <is>
-          <t>한국</t>
+          <t>미래</t>
         </is>
       </c>
       <c r="O32" s="6" t="inlineStr"/>
       <c r="P32" s="7" t="inlineStr">
         <is>
-          <t>2,050</t>
+          <t>1,090</t>
         </is>
       </c>
       <c r="Q32" s="6" t="inlineStr">
         <is>
-          <t>5.00%</t>
+          <t>4.00%</t>
         </is>
       </c>
       <c r="R32" s="6" t="inlineStr">
@@ -9173,7 +9167,7 @@
     <row r="33" ht="30" customHeight="1">
       <c r="A33" s="6" t="inlineStr">
         <is>
-          <t>액스비스</t>
+          <t>에스팀</t>
         </is>
       </c>
       <c r="B33" s="18" t="inlineStr">
@@ -9183,32 +9177,32 @@
       </c>
       <c r="C33" s="6" t="inlineStr">
         <is>
-          <t>10,100~11,500</t>
+          <t>7,000~8,500</t>
         </is>
       </c>
       <c r="D33" s="7" t="inlineStr">
         <is>
-          <t>2,300,000</t>
+          <t>1,800,000</t>
         </is>
       </c>
       <c r="E33" s="7" t="inlineStr">
         <is>
-          <t>26,450</t>
+          <t>15,300</t>
         </is>
       </c>
       <c r="F33" s="6" t="inlineStr">
         <is>
-          <t>27.60배 (PER)</t>
+          <t>17.71배 (EV/EBITDA)</t>
         </is>
       </c>
       <c r="G33" s="6" t="n">
-        <v>11500</v>
+        <v>8500</v>
       </c>
       <c r="H33" s="6" t="n">
-        <v>1124.21</v>
+        <v>1334.91</v>
       </c>
       <c r="I33" s="6" t="n">
-        <v>2411</v>
+        <v>2263</v>
       </c>
       <c r="J33" s="6" t="inlineStr">
         <is>
@@ -9217,29 +9211,29 @@
       </c>
       <c r="K33" s="6" t="inlineStr">
         <is>
-          <t>1,960.87</t>
+          <t>1,334.91</t>
         </is>
       </c>
       <c r="L33" s="6" t="inlineStr"/>
       <c r="M33" s="6" t="inlineStr">
         <is>
-          <t>2026-03-09</t>
+          <t>2026-03-06</t>
         </is>
       </c>
       <c r="N33" s="6" t="inlineStr">
         <is>
-          <t>미래</t>
+          <t>한국</t>
         </is>
       </c>
       <c r="O33" s="6" t="inlineStr"/>
       <c r="P33" s="7" t="inlineStr">
         <is>
-          <t>1,090</t>
+          <t>788</t>
         </is>
       </c>
       <c r="Q33" s="6" t="inlineStr">
         <is>
-          <t>4.00%</t>
+          <t>5.00%</t>
         </is>
       </c>
       <c r="R33" s="6" t="inlineStr">
@@ -9251,7 +9245,7 @@
     <row r="34" ht="30" customHeight="1">
       <c r="A34" s="6" t="inlineStr">
         <is>
-          <t>에스팀</t>
+          <t>케이뱅크 (유가)</t>
         </is>
       </c>
       <c r="B34" s="18" t="inlineStr">
@@ -9261,63 +9255,67 @@
       </c>
       <c r="C34" s="6" t="inlineStr">
         <is>
-          <t>7,000~8,500</t>
+          <t>8,300~9,500</t>
         </is>
       </c>
       <c r="D34" s="7" t="inlineStr">
         <is>
-          <t>1,800,000</t>
+          <t>60,000,000</t>
         </is>
       </c>
       <c r="E34" s="7" t="inlineStr">
         <is>
-          <t>15,300</t>
+          <t>498,000</t>
         </is>
       </c>
       <c r="F34" s="6" t="inlineStr">
         <is>
-          <t>17.71배 (EV/EBITDA)</t>
+          <t>1.80배 (PBR)</t>
         </is>
       </c>
       <c r="G34" s="6" t="n">
-        <v>8500</v>
+        <v>8300</v>
       </c>
       <c r="H34" s="6" t="n">
-        <v>1334.91</v>
+        <v>198.53</v>
       </c>
       <c r="I34" s="6" t="n">
-        <v>2263</v>
+        <v>2007</v>
       </c>
       <c r="J34" s="6" t="inlineStr">
         <is>
-          <t>2026-02-23~02-24</t>
+          <t>2026-02-20~23</t>
         </is>
       </c>
       <c r="K34" s="6" t="inlineStr">
         <is>
-          <t>1,334.91</t>
+          <t>134.59</t>
         </is>
       </c>
       <c r="L34" s="6" t="inlineStr"/>
       <c r="M34" s="6" t="inlineStr">
         <is>
-          <t>2026-03-06</t>
+          <t>2026-03-05</t>
         </is>
       </c>
       <c r="N34" s="6" t="inlineStr">
         <is>
-          <t>한국</t>
-        </is>
-      </c>
-      <c r="O34" s="6" t="inlineStr"/>
+          <t>NH</t>
+        </is>
+      </c>
+      <c r="O34" s="6" t="inlineStr">
+        <is>
+          <t>삼성</t>
+        </is>
+      </c>
       <c r="P34" s="7" t="inlineStr">
         <is>
-          <t>788</t>
+          <t>5,976</t>
         </is>
       </c>
       <c r="Q34" s="6" t="inlineStr">
         <is>
-          <t>5.00%</t>
+          <t>1.2%</t>
         </is>
       </c>
       <c r="R34" s="6" t="inlineStr">
@@ -9329,57 +9327,63 @@
     <row r="35" ht="30" customHeight="1">
       <c r="A35" s="6" t="inlineStr">
         <is>
-          <t>케이뱅크 (유가)</t>
-        </is>
-      </c>
-      <c r="B35" s="18" t="inlineStr">
-        <is>
-          <t>수집예정</t>
-        </is>
-      </c>
-      <c r="C35" s="6" t="inlineStr">
-        <is>
-          <t>8,300~9,500</t>
-        </is>
-      </c>
-      <c r="D35" s="7" t="inlineStr">
-        <is>
-          <t>60,000,000</t>
-        </is>
-      </c>
-      <c r="E35" s="7" t="inlineStr">
-        <is>
-          <t>498,000</t>
-        </is>
-      </c>
-      <c r="F35" s="6" t="inlineStr">
-        <is>
-          <t>1.80배 (PBR)</t>
-        </is>
-      </c>
-      <c r="G35" s="6" t="n">
-        <v>8300</v>
-      </c>
-      <c r="H35" s="6" t="n">
-        <v>198.53</v>
-      </c>
-      <c r="I35" s="6" t="n">
-        <v>2007</v>
-      </c>
-      <c r="J35" s="6" t="inlineStr">
-        <is>
-          <t>2026-02-20~23</t>
-        </is>
-      </c>
-      <c r="K35" s="6" t="inlineStr">
-        <is>
-          <t>134.59</t>
+          <t>세미티에스</t>
+        </is>
+      </c>
+      <c r="B35" s="19" t="inlineStr">
+        <is>
+          <t>해당없음</t>
+        </is>
+      </c>
+      <c r="C35" s="19" t="inlineStr">
+        <is>
+          <t>해당없음</t>
+        </is>
+      </c>
+      <c r="D35" s="19" t="inlineStr">
+        <is>
+          <t>해당없음</t>
+        </is>
+      </c>
+      <c r="E35" s="19" t="inlineStr">
+        <is>
+          <t>해당없음</t>
+        </is>
+      </c>
+      <c r="F35" s="19" t="inlineStr">
+        <is>
+          <t>해당없음</t>
+        </is>
+      </c>
+      <c r="G35" s="19" t="inlineStr">
+        <is>
+          <t>해당없음</t>
+        </is>
+      </c>
+      <c r="H35" s="19" t="inlineStr">
+        <is>
+          <t>해당없음</t>
+        </is>
+      </c>
+      <c r="I35" s="19" t="inlineStr">
+        <is>
+          <t>해당없음</t>
+        </is>
+      </c>
+      <c r="J35" s="19" t="inlineStr">
+        <is>
+          <t>해당없음</t>
+        </is>
+      </c>
+      <c r="K35" s="19" t="inlineStr">
+        <is>
+          <t>해당없음</t>
         </is>
       </c>
       <c r="L35" s="6" t="inlineStr"/>
       <c r="M35" s="6" t="inlineStr">
         <is>
-          <t>2026-03-05</t>
+          <t>2026-02-05</t>
         </is>
       </c>
       <c r="N35" s="6" t="inlineStr">
@@ -9387,87 +9391,77 @@
           <t>NH</t>
         </is>
       </c>
-      <c r="O35" s="6" t="inlineStr">
-        <is>
-          <t>삼성</t>
-        </is>
-      </c>
-      <c r="P35" s="7" t="inlineStr">
-        <is>
-          <t>5,976</t>
-        </is>
-      </c>
-      <c r="Q35" s="6" t="inlineStr">
-        <is>
-          <t>1.2%</t>
+      <c r="O35" s="6" t="inlineStr"/>
+      <c r="P35" s="19" t="inlineStr">
+        <is>
+          <t>해당없음</t>
+        </is>
+      </c>
+      <c r="Q35" s="19" t="inlineStr">
+        <is>
+          <t>해당없음</t>
         </is>
       </c>
       <c r="R35" s="6" t="inlineStr">
         <is>
-          <t>상장완료</t>
+          <t>상장완료(스팩합병)</t>
         </is>
       </c>
     </row>
     <row r="36" ht="30" customHeight="1">
       <c r="A36" s="6" t="inlineStr">
         <is>
-          <t>세미티에스</t>
-        </is>
-      </c>
-      <c r="B36" s="19" t="inlineStr">
-        <is>
-          <t>해당없음</t>
-        </is>
-      </c>
-      <c r="C36" s="19" t="inlineStr">
-        <is>
-          <t>해당없음</t>
-        </is>
-      </c>
-      <c r="D36" s="19" t="inlineStr">
-        <is>
-          <t>해당없음</t>
-        </is>
-      </c>
-      <c r="E36" s="19" t="inlineStr">
-        <is>
-          <t>해당없음</t>
-        </is>
-      </c>
-      <c r="F36" s="19" t="inlineStr">
-        <is>
-          <t>해당없음</t>
-        </is>
-      </c>
-      <c r="G36" s="19" t="inlineStr">
-        <is>
-          <t>해당없음</t>
-        </is>
-      </c>
-      <c r="H36" s="19" t="inlineStr">
-        <is>
-          <t>해당없음</t>
-        </is>
-      </c>
-      <c r="I36" s="19" t="inlineStr">
-        <is>
-          <t>해당없음</t>
-        </is>
-      </c>
-      <c r="J36" s="19" t="inlineStr">
-        <is>
-          <t>해당없음</t>
-        </is>
-      </c>
-      <c r="K36" s="19" t="inlineStr">
-        <is>
-          <t>해당없음</t>
+          <t>덕양에너젠</t>
+        </is>
+      </c>
+      <c r="B36" s="18" t="inlineStr">
+        <is>
+          <t>수집예정</t>
+        </is>
+      </c>
+      <c r="C36" s="6" t="inlineStr">
+        <is>
+          <t>8,500~10,000</t>
+        </is>
+      </c>
+      <c r="D36" s="7" t="inlineStr">
+        <is>
+          <t>7,500,000</t>
+        </is>
+      </c>
+      <c r="E36" s="7" t="inlineStr">
+        <is>
+          <t>75,000</t>
+        </is>
+      </c>
+      <c r="F36" s="6" t="inlineStr">
+        <is>
+          <t>30.32배 (EV/EBITDA)</t>
+        </is>
+      </c>
+      <c r="G36" s="6" t="n">
+        <v>10000</v>
+      </c>
+      <c r="H36" s="6" t="n">
+        <v>650.14</v>
+      </c>
+      <c r="I36" s="6" t="n">
+        <v>2324</v>
+      </c>
+      <c r="J36" s="6" t="inlineStr">
+        <is>
+          <t>2026-01-20~01-21</t>
+        </is>
+      </c>
+      <c r="K36" s="6" t="inlineStr">
+        <is>
+          <t>1,354.00</t>
         </is>
       </c>
       <c r="L36" s="6" t="inlineStr"/>
       <c r="M36" s="6" t="inlineStr">
         <is>
-          <t>2026-02-05</t>
+          <t>2026-01-30</t>
         </is>
       </c>
       <c r="N36" s="6" t="inlineStr">
@@ -9475,77 +9469,87 @@
           <t>NH</t>
         </is>
       </c>
-      <c r="O36" s="6" t="inlineStr"/>
-      <c r="P36" s="19" t="inlineStr">
-        <is>
-          <t>해당없음</t>
-        </is>
-      </c>
-      <c r="Q36" s="19" t="inlineStr">
-        <is>
-          <t>해당없음</t>
+      <c r="O36" s="6" t="inlineStr">
+        <is>
+          <t>미래</t>
+        </is>
+      </c>
+      <c r="P36" s="7" t="inlineStr">
+        <is>
+          <t>2,000</t>
+        </is>
+      </c>
+      <c r="Q36" s="6" t="inlineStr">
+        <is>
+          <t>2.92%</t>
         </is>
       </c>
       <c r="R36" s="6" t="inlineStr">
         <is>
-          <t>상장완료(스팩합병)</t>
+          <t>상장완료</t>
         </is>
       </c>
     </row>
     <row r="37" ht="30" customHeight="1">
       <c r="A37" s="6" t="inlineStr">
         <is>
-          <t>덕양에너젠</t>
-        </is>
-      </c>
-      <c r="B37" s="18" t="inlineStr">
-        <is>
-          <t>수집예정</t>
-        </is>
-      </c>
-      <c r="C37" s="6" t="inlineStr">
-        <is>
-          <t>8,500~10,000</t>
-        </is>
-      </c>
-      <c r="D37" s="7" t="inlineStr">
-        <is>
-          <t>7,500,000</t>
-        </is>
-      </c>
-      <c r="E37" s="7" t="inlineStr">
-        <is>
-          <t>75,000</t>
-        </is>
-      </c>
-      <c r="F37" s="6" t="inlineStr">
-        <is>
-          <t>30.32배 (EV/EBITDA)</t>
-        </is>
-      </c>
-      <c r="G37" s="6" t="n">
-        <v>10000</v>
-      </c>
-      <c r="H37" s="6" t="n">
-        <v>650.14</v>
-      </c>
-      <c r="I37" s="6" t="n">
-        <v>2324</v>
-      </c>
-      <c r="J37" s="6" t="inlineStr">
-        <is>
-          <t>2026-01-20~01-21</t>
-        </is>
-      </c>
-      <c r="K37" s="6" t="inlineStr">
-        <is>
-          <t>1,354.00</t>
+          <t>케이피항공산업</t>
+        </is>
+      </c>
+      <c r="B37" s="19" t="inlineStr">
+        <is>
+          <t>해당없음</t>
+        </is>
+      </c>
+      <c r="C37" s="19" t="inlineStr">
+        <is>
+          <t>해당없음</t>
+        </is>
+      </c>
+      <c r="D37" s="19" t="inlineStr">
+        <is>
+          <t>해당없음</t>
+        </is>
+      </c>
+      <c r="E37" s="19" t="inlineStr">
+        <is>
+          <t>해당없음</t>
+        </is>
+      </c>
+      <c r="F37" s="19" t="inlineStr">
+        <is>
+          <t>해당없음</t>
+        </is>
+      </c>
+      <c r="G37" s="19" t="inlineStr">
+        <is>
+          <t>해당없음</t>
+        </is>
+      </c>
+      <c r="H37" s="19" t="inlineStr">
+        <is>
+          <t>해당없음</t>
+        </is>
+      </c>
+      <c r="I37" s="19" t="inlineStr">
+        <is>
+          <t>해당없음</t>
+        </is>
+      </c>
+      <c r="J37" s="19" t="inlineStr">
+        <is>
+          <t>해당없음</t>
+        </is>
+      </c>
+      <c r="K37" s="19" t="inlineStr">
+        <is>
+          <t>해당없음</t>
         </is>
       </c>
       <c r="L37" s="6" t="inlineStr"/>
       <c r="M37" s="6" t="inlineStr">
         <is>
-          <t>2026-01-30</t>
+          <t>2026-01-29</t>
         </is>
       </c>
       <c r="N37" s="6" t="inlineStr">
@@ -9553,31 +9557,27 @@
           <t>NH</t>
         </is>
       </c>
-      <c r="O37" s="6" t="inlineStr">
-        <is>
-          <t>미래</t>
-        </is>
-      </c>
-      <c r="P37" s="7" t="inlineStr">
-        <is>
-          <t>2,000</t>
-        </is>
-      </c>
-      <c r="Q37" s="6" t="inlineStr">
-        <is>
-          <t>2.92%</t>
+      <c r="O37" s="6" t="inlineStr"/>
+      <c r="P37" s="19" t="inlineStr">
+        <is>
+          <t>해당없음</t>
+        </is>
+      </c>
+      <c r="Q37" s="19" t="inlineStr">
+        <is>
+          <t>해당없음</t>
         </is>
       </c>
       <c r="R37" s="6" t="inlineStr">
         <is>
-          <t>상장완료</t>
+          <t>상장완료(스팩합병)</t>
         </is>
       </c>
     </row>
     <row r="38" ht="30" customHeight="1">
       <c r="A38" s="6" t="inlineStr">
         <is>
-          <t>케이피항공산업</t>
+          <t>삼성스팩13호</t>
         </is>
       </c>
       <c r="B38" s="19" t="inlineStr">
@@ -9585,212 +9585,192 @@
           <t>해당없음</t>
         </is>
       </c>
-      <c r="C38" s="19" t="inlineStr">
+      <c r="C38" s="6" t="inlineStr">
+        <is>
+          <t>2,000</t>
+        </is>
+      </c>
+      <c r="D38" s="7" t="inlineStr">
+        <is>
+          <t>6,000,000</t>
+        </is>
+      </c>
+      <c r="E38" s="7" t="inlineStr">
+        <is>
+          <t>12,000</t>
+        </is>
+      </c>
+      <c r="F38" s="19" t="inlineStr">
         <is>
           <t>해당없음</t>
         </is>
       </c>
-      <c r="D38" s="19" t="inlineStr">
-        <is>
-          <t>해당없음</t>
-        </is>
-      </c>
-      <c r="E38" s="19" t="inlineStr">
-        <is>
-          <t>해당없음</t>
-        </is>
-      </c>
-      <c r="F38" s="19" t="inlineStr">
-        <is>
-          <t>해당없음</t>
-        </is>
-      </c>
-      <c r="G38" s="19" t="inlineStr">
-        <is>
-          <t>해당없음</t>
-        </is>
-      </c>
-      <c r="H38" s="19" t="inlineStr">
-        <is>
-          <t>해당없음</t>
-        </is>
-      </c>
-      <c r="I38" s="19" t="inlineStr">
-        <is>
-          <t>해당없음</t>
-        </is>
-      </c>
-      <c r="J38" s="19" t="inlineStr">
-        <is>
-          <t>해당없음</t>
-        </is>
-      </c>
-      <c r="K38" s="19" t="inlineStr">
-        <is>
-          <t>해당없음</t>
+      <c r="G38" s="6" t="inlineStr">
+        <is>
+          <t>2,000</t>
+        </is>
+      </c>
+      <c r="H38" s="6" t="n">
+        <v>1159.11</v>
+      </c>
+      <c r="I38" s="6" t="n">
+        <v>1892</v>
+      </c>
+      <c r="J38" s="6" t="inlineStr">
+        <is>
+          <t>2026-01-12~01-13</t>
+        </is>
+      </c>
+      <c r="K38" s="6" t="inlineStr">
+        <is>
+          <t>1,870.40</t>
         </is>
       </c>
       <c r="L38" s="6" t="inlineStr"/>
       <c r="M38" s="6" t="inlineStr">
         <is>
-          <t>2026-01-29</t>
+          <t>2026-01-21</t>
         </is>
       </c>
       <c r="N38" s="6" t="inlineStr">
         <is>
-          <t>NH</t>
+          <t>삼성</t>
         </is>
       </c>
       <c r="O38" s="6" t="inlineStr"/>
-      <c r="P38" s="19" t="inlineStr">
-        <is>
-          <t>해당없음</t>
-        </is>
-      </c>
-      <c r="Q38" s="19" t="inlineStr">
-        <is>
-          <t>해당없음</t>
+      <c r="P38" s="7" t="inlineStr">
+        <is>
+          <t>360</t>
+        </is>
+      </c>
+      <c r="Q38" s="6" t="inlineStr">
+        <is>
+          <t>3.00%</t>
         </is>
       </c>
       <c r="R38" s="6" t="inlineStr">
         <is>
-          <t>상장완료(스팩합병)</t>
-        </is>
-      </c>
-    </row>
-    <row r="39" ht="30" customHeight="1">
-      <c r="A39" s="6" t="inlineStr">
-        <is>
-          <t>삼성스팩13호</t>
-        </is>
-      </c>
-      <c r="B39" s="19" t="inlineStr">
-        <is>
-          <t>해당없음</t>
-        </is>
-      </c>
-      <c r="C39" s="6" t="inlineStr">
-        <is>
-          <t>2,000</t>
-        </is>
-      </c>
-      <c r="D39" s="7" t="inlineStr">
-        <is>
-          <t>6,000,000</t>
-        </is>
-      </c>
-      <c r="E39" s="7" t="inlineStr">
-        <is>
-          <t>12,000</t>
-        </is>
-      </c>
-      <c r="F39" s="19" t="inlineStr">
-        <is>
-          <t>해당없음</t>
-        </is>
-      </c>
-      <c r="G39" s="6" t="inlineStr">
-        <is>
-          <t>2,000</t>
-        </is>
-      </c>
-      <c r="H39" s="6" t="n">
-        <v>1159.11</v>
-      </c>
-      <c r="I39" s="6" t="n">
-        <v>1892</v>
-      </c>
-      <c r="J39" s="6" t="inlineStr">
-        <is>
-          <t>2026-01-12~01-13</t>
-        </is>
-      </c>
-      <c r="K39" s="6" t="inlineStr">
-        <is>
-          <t>1,870.40</t>
-        </is>
-      </c>
-      <c r="L39" s="6" t="inlineStr"/>
-      <c r="M39" s="6" t="inlineStr">
-        <is>
-          <t>2026-01-21</t>
-        </is>
-      </c>
-      <c r="N39" s="6" t="inlineStr">
-        <is>
-          <t>삼성</t>
-        </is>
-      </c>
-      <c r="O39" s="6" t="inlineStr"/>
-      <c r="P39" s="7" t="inlineStr">
-        <is>
-          <t>360</t>
-        </is>
-      </c>
-      <c r="Q39" s="6" t="inlineStr">
-        <is>
-          <t>3.00%</t>
-        </is>
-      </c>
-      <c r="R39" s="6" t="inlineStr">
-        <is>
           <t>상장완료</t>
         </is>
       </c>
     </row>
-    <row r="41" ht="22" customHeight="1">
-      <c r="A41" s="3" t="inlineStr">
+    <row r="40" ht="22" customHeight="1">
+      <c r="A40" s="3" t="inlineStr">
         <is>
           <t>■ 공모 진행 (예심 승인법인)  (16건)</t>
         </is>
       </c>
-      <c r="B41" s="4" t="n"/>
-      <c r="C41" s="4" t="n"/>
-      <c r="D41" s="4" t="n"/>
-      <c r="E41" s="4" t="n"/>
-      <c r="F41" s="4" t="n"/>
-      <c r="G41" s="4" t="n"/>
-      <c r="H41" s="4" t="n"/>
-      <c r="I41" s="4" t="n"/>
-      <c r="J41" s="4" t="n"/>
-      <c r="K41" s="4" t="n"/>
-      <c r="L41" s="4" t="n"/>
-      <c r="M41" s="4" t="n"/>
-      <c r="N41" s="4" t="n"/>
-      <c r="O41" s="4" t="n"/>
-      <c r="P41" s="4" t="n"/>
-      <c r="Q41" s="4" t="n"/>
-      <c r="R41" s="4" t="n"/>
+      <c r="B40" s="4" t="n"/>
+      <c r="C40" s="4" t="n"/>
+      <c r="D40" s="4" t="n"/>
+      <c r="E40" s="4" t="n"/>
+      <c r="F40" s="4" t="n"/>
+      <c r="G40" s="4" t="n"/>
+      <c r="H40" s="4" t="n"/>
+      <c r="I40" s="4" t="n"/>
+      <c r="J40" s="4" t="n"/>
+      <c r="K40" s="4" t="n"/>
+      <c r="L40" s="4" t="n"/>
+      <c r="M40" s="4" t="n"/>
+      <c r="N40" s="4" t="n"/>
+      <c r="O40" s="4" t="n"/>
+      <c r="P40" s="4" t="n"/>
+      <c r="Q40" s="4" t="n"/>
+      <c r="R40" s="4" t="n"/>
+    </row>
+    <row r="41" ht="30" customHeight="1">
+      <c r="A41" s="6" t="inlineStr">
+        <is>
+          <t>인제니아테라퓨틱스</t>
+        </is>
+      </c>
+      <c r="B41" s="6" t="inlineStr">
+        <is>
+          <t>07-20~07-24</t>
+        </is>
+      </c>
+      <c r="C41" s="6" t="inlineStr">
+        <is>
+          <t>12,000~14,500</t>
+        </is>
+      </c>
+      <c r="D41" s="7" t="inlineStr">
+        <is>
+          <t>5,000,000</t>
+        </is>
+      </c>
+      <c r="E41" s="7" t="inlineStr">
+        <is>
+          <t>60,000 (하단)</t>
+        </is>
+      </c>
+      <c r="F41" s="6" t="inlineStr">
+        <is>
+          <t>22.89배 (PER)</t>
+        </is>
+      </c>
+      <c r="G41" s="6" t="inlineStr"/>
+      <c r="H41" s="6" t="inlineStr"/>
+      <c r="I41" s="6" t="inlineStr"/>
+      <c r="J41" s="6" t="inlineStr">
+        <is>
+          <t>07-30~07-31</t>
+        </is>
+      </c>
+      <c r="K41" s="6" t="inlineStr"/>
+      <c r="L41" s="6" t="inlineStr"/>
+      <c r="M41" s="6" t="inlineStr"/>
+      <c r="N41" s="6" t="inlineStr">
+        <is>
+          <t>삼성증권</t>
+        </is>
+      </c>
+      <c r="O41" s="6" t="inlineStr"/>
+      <c r="P41" s="7" t="inlineStr">
+        <is>
+          <t>4,095,000,000</t>
+        </is>
+      </c>
+      <c r="Q41" s="6" t="inlineStr">
+        <is>
+          <t>6.5%</t>
+        </is>
+      </c>
+      <c r="R41" s="6" t="inlineStr">
+        <is>
+          <t>정정</t>
+        </is>
+      </c>
     </row>
     <row r="42" ht="30" customHeight="1">
       <c r="A42" s="6" t="inlineStr">
         <is>
-          <t>인제니아테라퓨틱스</t>
+          <t>딜리셔스</t>
         </is>
       </c>
       <c r="B42" s="6" t="inlineStr">
         <is>
-          <t>07-20~07-24</t>
+          <t>07-23~07-29</t>
         </is>
       </c>
       <c r="C42" s="6" t="inlineStr">
         <is>
-          <t>12,000~14,500</t>
+          <t>5,000~7,000</t>
         </is>
       </c>
       <c r="D42" s="7" t="inlineStr">
         <is>
-          <t>5,000,000</t>
+          <t>2,200,000</t>
         </is>
       </c>
       <c r="E42" s="7" t="inlineStr">
         <is>
-          <t>60,000 (하단)</t>
+          <t>11,000,000,000</t>
         </is>
       </c>
       <c r="F42" s="6" t="inlineStr">
         <is>
-          <t>22.89배 (PER)</t>
+          <t>23.93배 (PER)</t>
         </is>
       </c>
       <c r="G42" s="6" t="inlineStr"/>
@@ -9798,7 +9778,7 @@
       <c r="I42" s="6" t="inlineStr"/>
       <c r="J42" s="6" t="inlineStr">
         <is>
-          <t>07-30~07-31</t>
+          <t>08-03~08-04</t>
         </is>
       </c>
       <c r="K42" s="6" t="inlineStr"/>
@@ -9806,18 +9786,18 @@
       <c r="M42" s="6" t="inlineStr"/>
       <c r="N42" s="6" t="inlineStr">
         <is>
-          <t>삼성증권</t>
+          <t>한국투자증권</t>
         </is>
       </c>
       <c r="O42" s="6" t="inlineStr"/>
       <c r="P42" s="7" t="inlineStr">
         <is>
-          <t>4,095,000,000</t>
+          <t>566,500,000</t>
         </is>
       </c>
       <c r="Q42" s="6" t="inlineStr">
         <is>
-          <t>6.5%</t>
+          <t>5.0%</t>
         </is>
       </c>
       <c r="R42" s="6" t="inlineStr">
@@ -9829,32 +9809,32 @@
     <row r="43" ht="30" customHeight="1">
       <c r="A43" s="6" t="inlineStr">
         <is>
-          <t>딜리셔스</t>
+          <t>케이앤에스아이앤씨</t>
         </is>
       </c>
       <c r="B43" s="6" t="inlineStr">
         <is>
-          <t>07-23~07-29</t>
+          <t>07-27~07-31</t>
         </is>
       </c>
       <c r="C43" s="6" t="inlineStr">
         <is>
-          <t>5,000~7,000</t>
+          <t>9,000~11,000</t>
         </is>
       </c>
       <c r="D43" s="7" t="inlineStr">
         <is>
-          <t>2,200,000</t>
+          <t>2,400,000</t>
         </is>
       </c>
       <c r="E43" s="7" t="inlineStr">
         <is>
-          <t>11,000,000,000</t>
+          <t>21,600,000,000</t>
         </is>
       </c>
       <c r="F43" s="6" t="inlineStr">
         <is>
-          <t>23.93배 (PER)</t>
+          <t>47.97배 (PER)</t>
         </is>
       </c>
       <c r="G43" s="6" t="inlineStr"/>
@@ -9862,7 +9842,7 @@
       <c r="I43" s="6" t="inlineStr"/>
       <c r="J43" s="6" t="inlineStr">
         <is>
-          <t>08-03~08-04</t>
+          <t>08-04~08-05</t>
         </is>
       </c>
       <c r="K43" s="6" t="inlineStr"/>
@@ -9870,18 +9850,18 @@
       <c r="M43" s="6" t="inlineStr"/>
       <c r="N43" s="6" t="inlineStr">
         <is>
-          <t>한국투자증권</t>
+          <t>아이비케이투자증권</t>
         </is>
       </c>
       <c r="O43" s="6" t="inlineStr"/>
       <c r="P43" s="7" t="inlineStr">
         <is>
-          <t>566,500,000</t>
+          <t>1,500,000,000</t>
         </is>
       </c>
       <c r="Q43" s="6" t="inlineStr">
         <is>
-          <t>5.0%</t>
+          <t>3.5%</t>
         </is>
       </c>
       <c r="R43" s="6" t="inlineStr">
@@ -9893,32 +9873,32 @@
     <row r="44" ht="30" customHeight="1">
       <c r="A44" s="6" t="inlineStr">
         <is>
-          <t>케이앤에스아이앤씨</t>
+          <t>기도산업</t>
         </is>
       </c>
       <c r="B44" s="6" t="inlineStr">
         <is>
-          <t>07-27~07-31</t>
+          <t>07-31~08-06</t>
         </is>
       </c>
       <c r="C44" s="6" t="inlineStr">
         <is>
-          <t>9,000~11,000</t>
+          <t>24,800~28,400</t>
         </is>
       </c>
       <c r="D44" s="7" t="inlineStr">
         <is>
-          <t>2,400,000</t>
+          <t>1,700,000</t>
         </is>
       </c>
       <c r="E44" s="7" t="inlineStr">
         <is>
-          <t>21,600,000,000</t>
+          <t>42,160,000,000</t>
         </is>
       </c>
       <c r="F44" s="6" t="inlineStr">
         <is>
-          <t>47.97배 (PER)</t>
+          <t>10.01배 (PER)</t>
         </is>
       </c>
       <c r="G44" s="6" t="inlineStr"/>
@@ -9926,7 +9906,7 @@
       <c r="I44" s="6" t="inlineStr"/>
       <c r="J44" s="6" t="inlineStr">
         <is>
-          <t>08-04~08-05</t>
+          <t>08-11~08-12</t>
         </is>
       </c>
       <c r="K44" s="6" t="inlineStr"/>
@@ -9934,18 +9914,18 @@
       <c r="M44" s="6" t="inlineStr"/>
       <c r="N44" s="6" t="inlineStr">
         <is>
-          <t>아이비케이투자증권</t>
+          <t>미래에셋증권</t>
         </is>
       </c>
       <c r="O44" s="6" t="inlineStr"/>
       <c r="P44" s="7" t="inlineStr">
         <is>
-          <t>1,500,000,000</t>
+          <t>716,720,000</t>
         </is>
       </c>
       <c r="Q44" s="6" t="inlineStr">
         <is>
-          <t>3.5%</t>
+          <t>1.0%</t>
         </is>
       </c>
       <c r="R44" s="6" t="inlineStr">
@@ -9957,32 +9937,32 @@
     <row r="45" ht="30" customHeight="1">
       <c r="A45" s="6" t="inlineStr">
         <is>
-          <t>기도산업</t>
+          <t>니어스랩</t>
         </is>
       </c>
       <c r="B45" s="6" t="inlineStr">
         <is>
-          <t>07-31~08-06</t>
+          <t>08-03~08-07</t>
         </is>
       </c>
       <c r="C45" s="6" t="inlineStr">
         <is>
-          <t>24,800~28,400</t>
+          <t>30,000~41,200</t>
         </is>
       </c>
       <c r="D45" s="7" t="inlineStr">
         <is>
-          <t>1,700,000</t>
+          <t>910,000</t>
         </is>
       </c>
       <c r="E45" s="7" t="inlineStr">
         <is>
-          <t>42,160,000,000</t>
+          <t>27,300,000,000</t>
         </is>
       </c>
       <c r="F45" s="6" t="inlineStr">
         <is>
-          <t>10.01배 (PER)</t>
+          <t>44.41배 (PER)</t>
         </is>
       </c>
       <c r="G45" s="6" t="inlineStr"/>
@@ -9990,7 +9970,7 @@
       <c r="I45" s="6" t="inlineStr"/>
       <c r="J45" s="6" t="inlineStr">
         <is>
-          <t>08-11~08-12</t>
+          <t>08-12~08-13</t>
         </is>
       </c>
       <c r="K45" s="6" t="inlineStr"/>
@@ -9998,18 +9978,18 @@
       <c r="M45" s="6" t="inlineStr"/>
       <c r="N45" s="6" t="inlineStr">
         <is>
-          <t>미래에셋증권</t>
+          <t>삼성증권</t>
         </is>
       </c>
       <c r="O45" s="6" t="inlineStr"/>
       <c r="P45" s="7" t="inlineStr">
         <is>
-          <t>716,720,000</t>
+          <t>1,265,355,000</t>
         </is>
       </c>
       <c r="Q45" s="6" t="inlineStr">
         <is>
-          <t>1.0%</t>
+          <t>4.50%</t>
         </is>
       </c>
       <c r="R45" s="6" t="inlineStr">
@@ -10021,7 +10001,7 @@
     <row r="46" ht="30" customHeight="1">
       <c r="A46" s="6" t="inlineStr">
         <is>
-          <t>니어스랩</t>
+          <t>해치텍</t>
         </is>
       </c>
       <c r="B46" s="6" t="inlineStr">
@@ -10031,22 +10011,22 @@
       </c>
       <c r="C46" s="6" t="inlineStr">
         <is>
-          <t>30,000~41,200</t>
+          <t>23,000~28,000</t>
         </is>
       </c>
       <c r="D46" s="7" t="inlineStr">
         <is>
-          <t>910,000</t>
+          <t>1,000,000</t>
         </is>
       </c>
       <c r="E46" s="7" t="inlineStr">
         <is>
-          <t>27,300,000,000</t>
+          <t>23,000,000,000</t>
         </is>
       </c>
       <c r="F46" s="6" t="inlineStr">
         <is>
-          <t>44.41배 (PER)</t>
+          <t>36.99배 (PER)</t>
         </is>
       </c>
       <c r="G46" s="6" t="inlineStr"/>
@@ -10062,18 +10042,18 @@
       <c r="M46" s="6" t="inlineStr"/>
       <c r="N46" s="6" t="inlineStr">
         <is>
-          <t>삼성증권</t>
+          <t>DB증권</t>
         </is>
       </c>
       <c r="O46" s="6" t="inlineStr"/>
       <c r="P46" s="7" t="inlineStr">
         <is>
-          <t>1,265,355,000</t>
+          <t>1,302,950,000</t>
         </is>
       </c>
       <c r="Q46" s="6" t="inlineStr">
         <is>
-          <t>4.50%</t>
+          <t>5.5%</t>
         </is>
       </c>
       <c r="R46" s="6" t="inlineStr">
@@ -10085,32 +10065,32 @@
     <row r="47" ht="30" customHeight="1">
       <c r="A47" s="6" t="inlineStr">
         <is>
-          <t>해치텍</t>
+          <t>빅웨이브로보틱스</t>
         </is>
       </c>
       <c r="B47" s="6" t="inlineStr">
         <is>
-          <t>08-03~08-07</t>
+          <t>08-04~08-10</t>
         </is>
       </c>
       <c r="C47" s="6" t="inlineStr">
         <is>
-          <t>23,000~28,000</t>
+          <t>20,000~24,000</t>
         </is>
       </c>
       <c r="D47" s="7" t="inlineStr">
         <is>
-          <t>1,000,000</t>
+          <t>2,000,000</t>
         </is>
       </c>
       <c r="E47" s="7" t="inlineStr">
         <is>
-          <t>23,000,000,000</t>
+          <t>40,000,000,000</t>
         </is>
       </c>
       <c r="F47" s="6" t="inlineStr">
         <is>
-          <t>36.99배 (PER)</t>
+          <t>15.41 (PSR)</t>
         </is>
       </c>
       <c r="G47" s="6" t="inlineStr"/>
@@ -10118,7 +10098,7 @@
       <c r="I47" s="6" t="inlineStr"/>
       <c r="J47" s="6" t="inlineStr">
         <is>
-          <t>08-12~08-13</t>
+          <t>08-13~08-14</t>
         </is>
       </c>
       <c r="K47" s="6" t="inlineStr"/>
@@ -10126,18 +10106,22 @@
       <c r="M47" s="6" t="inlineStr"/>
       <c r="N47" s="6" t="inlineStr">
         <is>
-          <t>DB증권</t>
-        </is>
-      </c>
-      <c r="O47" s="6" t="inlineStr"/>
+          <t>유진투자증권</t>
+        </is>
+      </c>
+      <c r="O47" s="6" t="inlineStr">
+        <is>
+          <t>미래</t>
+        </is>
+      </c>
       <c r="P47" s="7" t="inlineStr">
         <is>
-          <t>1,302,950,000</t>
+          <t>627,300,000</t>
         </is>
       </c>
       <c r="Q47" s="6" t="inlineStr">
         <is>
-          <t>5.5%</t>
+          <t>3.0%</t>
         </is>
       </c>
       <c r="R47" s="6" t="inlineStr">
@@ -10149,17 +10133,17 @@
     <row r="48" ht="30" customHeight="1">
       <c r="A48" s="6" t="inlineStr">
         <is>
-          <t>빅웨이브로보틱스</t>
+          <t>스카이랩스</t>
         </is>
       </c>
       <c r="B48" s="6" t="inlineStr">
         <is>
-          <t>08-04~08-10</t>
+          <t>08-03~08-07</t>
         </is>
       </c>
       <c r="C48" s="6" t="inlineStr">
         <is>
-          <t>20,000~24,000</t>
+          <t>13,000~16,000</t>
         </is>
       </c>
       <c r="D48" s="7" t="inlineStr">
@@ -10169,12 +10153,12 @@
       </c>
       <c r="E48" s="7" t="inlineStr">
         <is>
-          <t>40,000,000,000</t>
+          <t>26,000,000,000</t>
         </is>
       </c>
       <c r="F48" s="6" t="inlineStr">
         <is>
-          <t>15.41 (PSR)</t>
+          <t>29.52배 (PER)</t>
         </is>
       </c>
       <c r="G48" s="6" t="inlineStr"/>
@@ -10190,59 +10174,55 @@
       <c r="M48" s="6" t="inlineStr"/>
       <c r="N48" s="6" t="inlineStr">
         <is>
-          <t>유진투자증권</t>
-        </is>
-      </c>
-      <c r="O48" s="6" t="inlineStr">
-        <is>
-          <t>미래</t>
-        </is>
-      </c>
+          <t>한국투자증권</t>
+        </is>
+      </c>
+      <c r="O48" s="6" t="inlineStr"/>
       <c r="P48" s="7" t="inlineStr">
         <is>
-          <t>627,300,000</t>
-        </is>
-      </c>
-      <c r="Q48" s="6" t="inlineStr">
-        <is>
-          <t>3.0%</t>
+          <t>1,071,200,000</t>
+        </is>
+      </c>
+      <c r="Q48" s="18" t="inlineStr">
+        <is>
+          <t>수집예정</t>
         </is>
       </c>
       <c r="R48" s="6" t="inlineStr">
         <is>
-          <t>정정</t>
+          <t>최초</t>
         </is>
       </c>
     </row>
     <row r="49" ht="30" customHeight="1">
       <c r="A49" s="6" t="inlineStr">
         <is>
-          <t>스카이랩스</t>
+          <t>브릴스</t>
         </is>
       </c>
       <c r="B49" s="6" t="inlineStr">
         <is>
-          <t>08-03~08-07</t>
+          <t>08-14~08-21</t>
         </is>
       </c>
       <c r="C49" s="6" t="inlineStr">
         <is>
-          <t>13,000~16,000</t>
+          <t>16,500~19,500</t>
         </is>
       </c>
       <c r="D49" s="7" t="inlineStr">
         <is>
-          <t>2,000,000</t>
+          <t>1,200,000</t>
         </is>
       </c>
       <c r="E49" s="7" t="inlineStr">
         <is>
-          <t>26,000,000,000</t>
+          <t>19,800,000,000</t>
         </is>
       </c>
       <c r="F49" s="6" t="inlineStr">
         <is>
-          <t>29.52배 (PER)</t>
+          <t>13.44 (PSR)</t>
         </is>
       </c>
       <c r="G49" s="6" t="inlineStr"/>
@@ -10250,7 +10230,7 @@
       <c r="I49" s="6" t="inlineStr"/>
       <c r="J49" s="6" t="inlineStr">
         <is>
-          <t>08-13~08-14</t>
+          <t>08-25~08-26</t>
         </is>
       </c>
       <c r="K49" s="6" t="inlineStr"/>
@@ -10258,18 +10238,18 @@
       <c r="M49" s="6" t="inlineStr"/>
       <c r="N49" s="6" t="inlineStr">
         <is>
-          <t>한국투자증권</t>
+          <t>아이비케이투자증권</t>
         </is>
       </c>
       <c r="O49" s="6" t="inlineStr"/>
       <c r="P49" s="7" t="inlineStr">
         <is>
-          <t>1,071,200,000</t>
-        </is>
-      </c>
-      <c r="Q49" s="18" t="inlineStr">
-        <is>
-          <t>수집예정</t>
+          <t>713,790,000</t>
+        </is>
+      </c>
+      <c r="Q49" s="6" t="inlineStr">
+        <is>
+          <t>3.5%</t>
         </is>
       </c>
       <c r="R49" s="6" t="inlineStr">
@@ -10281,32 +10261,32 @@
     <row r="50" ht="30" customHeight="1">
       <c r="A50" s="6" t="inlineStr">
         <is>
-          <t>브릴스</t>
+          <t>네오사피엔스</t>
         </is>
       </c>
       <c r="B50" s="6" t="inlineStr">
         <is>
-          <t>08-14~08-21</t>
+          <t>08-31~09-04</t>
         </is>
       </c>
       <c r="C50" s="6" t="inlineStr">
         <is>
-          <t>16,500~19,500</t>
+          <t>13,800~15,800</t>
         </is>
       </c>
       <c r="D50" s="7" t="inlineStr">
         <is>
-          <t>1,200,000</t>
+          <t>2,000,000</t>
         </is>
       </c>
       <c r="E50" s="7" t="inlineStr">
         <is>
-          <t>19,800,000,000</t>
+          <t>27,600,000,000</t>
         </is>
       </c>
       <c r="F50" s="6" t="inlineStr">
         <is>
-          <t>13.44 (PSR)</t>
+          <t>26.76배 (PER)</t>
         </is>
       </c>
       <c r="G50" s="6" t="inlineStr"/>
@@ -10314,7 +10294,7 @@
       <c r="I50" s="6" t="inlineStr"/>
       <c r="J50" s="6" t="inlineStr">
         <is>
-          <t>08-25~08-26</t>
+          <t>09-08~09-09</t>
         </is>
       </c>
       <c r="K50" s="6" t="inlineStr"/>
@@ -10322,18 +10302,18 @@
       <c r="M50" s="6" t="inlineStr"/>
       <c r="N50" s="6" t="inlineStr">
         <is>
-          <t>아이비케이투자증권</t>
+          <t>대신증권</t>
         </is>
       </c>
       <c r="O50" s="6" t="inlineStr"/>
       <c r="P50" s="7" t="inlineStr">
         <is>
-          <t>713,790,000</t>
+          <t>1,080,264,000</t>
         </is>
       </c>
       <c r="Q50" s="6" t="inlineStr">
         <is>
-          <t>3.5%</t>
+          <t>3.8%</t>
         </is>
       </c>
       <c r="R50" s="6" t="inlineStr">
@@ -10345,32 +10325,32 @@
     <row r="51" ht="30" customHeight="1">
       <c r="A51" s="6" t="inlineStr">
         <is>
-          <t>네오사피엔스</t>
+          <t>덕산넵코어스</t>
         </is>
       </c>
       <c r="B51" s="6" t="inlineStr">
         <is>
-          <t>08-31~09-04</t>
+          <t>09-08~09-14</t>
         </is>
       </c>
       <c r="C51" s="6" t="inlineStr">
         <is>
-          <t>13,800~15,800</t>
+          <t>12,400~14,600</t>
         </is>
       </c>
       <c r="D51" s="7" t="inlineStr">
         <is>
-          <t>2,000,000</t>
+          <t>3,000,000</t>
         </is>
       </c>
       <c r="E51" s="7" t="inlineStr">
         <is>
-          <t>27,600,000,000</t>
+          <t>37,200,000,000</t>
         </is>
       </c>
       <c r="F51" s="6" t="inlineStr">
         <is>
-          <t>26.76배 (PER)</t>
+          <t>34.08배 (PER)</t>
         </is>
       </c>
       <c r="G51" s="6" t="inlineStr"/>
@@ -10378,7 +10358,7 @@
       <c r="I51" s="6" t="inlineStr"/>
       <c r="J51" s="6" t="inlineStr">
         <is>
-          <t>09-08~09-09</t>
+          <t>09-16~09-17</t>
         </is>
       </c>
       <c r="K51" s="6" t="inlineStr"/>
@@ -10392,12 +10372,12 @@
       <c r="O51" s="6" t="inlineStr"/>
       <c r="P51" s="7" t="inlineStr">
         <is>
-          <t>1,080,264,000</t>
+          <t>1,413,399,926</t>
         </is>
       </c>
       <c r="Q51" s="6" t="inlineStr">
         <is>
-          <t>3.8%</t>
+          <t>3.7%</t>
         </is>
       </c>
       <c r="R51" s="6" t="inlineStr">
@@ -10409,71 +10389,71 @@
     <row r="52" ht="30" customHeight="1">
       <c r="A52" s="6" t="inlineStr">
         <is>
-          <t>덕산넵코어스</t>
-        </is>
-      </c>
-      <c r="B52" s="6" t="inlineStr">
-        <is>
-          <t>09-08~09-14</t>
-        </is>
-      </c>
-      <c r="C52" s="6" t="inlineStr">
-        <is>
-          <t>12,400~14,600</t>
-        </is>
-      </c>
-      <c r="D52" s="7" t="inlineStr">
-        <is>
-          <t>3,000,000</t>
-        </is>
-      </c>
-      <c r="E52" s="7" t="inlineStr">
-        <is>
-          <t>37,200,000,000</t>
-        </is>
-      </c>
-      <c r="F52" s="6" t="inlineStr">
-        <is>
-          <t>34.08배 (PER)</t>
+          <t>엔에이치스팩34호</t>
+        </is>
+      </c>
+      <c r="B52" s="18" t="inlineStr">
+        <is>
+          <t>수집예정</t>
+        </is>
+      </c>
+      <c r="C52" s="18" t="inlineStr">
+        <is>
+          <t>수집예정</t>
+        </is>
+      </c>
+      <c r="D52" s="18" t="inlineStr">
+        <is>
+          <t>수집예정</t>
+        </is>
+      </c>
+      <c r="E52" s="18" t="inlineStr">
+        <is>
+          <t>수집예정</t>
+        </is>
+      </c>
+      <c r="F52" s="18" t="inlineStr">
+        <is>
+          <t>수집예정</t>
         </is>
       </c>
       <c r="G52" s="6" t="inlineStr"/>
       <c r="H52" s="6" t="inlineStr"/>
       <c r="I52" s="6" t="inlineStr"/>
-      <c r="J52" s="6" t="inlineStr">
-        <is>
-          <t>09-16~09-17</t>
+      <c r="J52" s="18" t="inlineStr">
+        <is>
+          <t>수집예정</t>
         </is>
       </c>
       <c r="K52" s="6" t="inlineStr"/>
       <c r="L52" s="6" t="inlineStr"/>
       <c r="M52" s="6" t="inlineStr"/>
-      <c r="N52" s="6" t="inlineStr">
-        <is>
-          <t>대신증권</t>
+      <c r="N52" s="18" t="inlineStr">
+        <is>
+          <t>수집예정</t>
         </is>
       </c>
       <c r="O52" s="6" t="inlineStr"/>
-      <c r="P52" s="7" t="inlineStr">
-        <is>
-          <t>1,413,399,926</t>
-        </is>
-      </c>
-      <c r="Q52" s="6" t="inlineStr">
-        <is>
-          <t>3.7%</t>
+      <c r="P52" s="18" t="inlineStr">
+        <is>
+          <t>수집예정</t>
+        </is>
+      </c>
+      <c r="Q52" s="18" t="inlineStr">
+        <is>
+          <t>수집예정</t>
         </is>
       </c>
       <c r="R52" s="6" t="inlineStr">
         <is>
-          <t>최초</t>
+          <t>corp_code 미확보(수동확인)</t>
         </is>
       </c>
     </row>
     <row r="53" ht="30" customHeight="1">
       <c r="A53" s="6" t="inlineStr">
         <is>
-          <t>엔에이치스팩34호</t>
+          <t>와이즈플래닛컴퍼니</t>
         </is>
       </c>
       <c r="B53" s="18" t="inlineStr">
@@ -10512,9 +10492,9 @@
       <c r="K53" s="6" t="inlineStr"/>
       <c r="L53" s="6" t="inlineStr"/>
       <c r="M53" s="6" t="inlineStr"/>
-      <c r="N53" s="18" t="inlineStr">
-        <is>
-          <t>수집예정</t>
+      <c r="N53" s="6" t="inlineStr">
+        <is>
+          <t>대신</t>
         </is>
       </c>
       <c r="O53" s="6" t="inlineStr"/>
@@ -10530,14 +10510,14 @@
       </c>
       <c r="R53" s="6" t="inlineStr">
         <is>
-          <t>corp_code 미확보(수동확인)</t>
+          <t>신고서 대기</t>
         </is>
       </c>
     </row>
     <row r="54" ht="30" customHeight="1">
       <c r="A54" s="6" t="inlineStr">
         <is>
-          <t>와이즈플래닛컴퍼니</t>
+          <t>엠에스바이오</t>
         </is>
       </c>
       <c r="B54" s="18" t="inlineStr">
@@ -10576,9 +10556,9 @@
       <c r="K54" s="6" t="inlineStr"/>
       <c r="L54" s="6" t="inlineStr"/>
       <c r="M54" s="6" t="inlineStr"/>
-      <c r="N54" s="6" t="inlineStr">
-        <is>
-          <t>대신</t>
+      <c r="N54" s="18" t="inlineStr">
+        <is>
+          <t>수집예정</t>
         </is>
       </c>
       <c r="O54" s="6" t="inlineStr"/>
@@ -10601,7 +10581,7 @@
     <row r="55" ht="30" customHeight="1">
       <c r="A55" s="6" t="inlineStr">
         <is>
-          <t>엠에스바이오</t>
+          <t>디티에스</t>
         </is>
       </c>
       <c r="B55" s="18" t="inlineStr">
@@ -10665,7 +10645,7 @@
     <row r="56" ht="30" customHeight="1">
       <c r="A56" s="6" t="inlineStr">
         <is>
-          <t>디티에스</t>
+          <t>글로벌테크놀로지</t>
         </is>
       </c>
       <c r="B56" s="18" t="inlineStr">
@@ -10726,86 +10706,22 @@
         </is>
       </c>
     </row>
-    <row r="57" ht="30" customHeight="1">
-      <c r="A57" s="6" t="inlineStr">
-        <is>
-          <t>글로벌테크놀로지</t>
-        </is>
-      </c>
-      <c r="B57" s="18" t="inlineStr">
-        <is>
-          <t>수집예정</t>
-        </is>
-      </c>
-      <c r="C57" s="18" t="inlineStr">
-        <is>
-          <t>수집예정</t>
-        </is>
-      </c>
-      <c r="D57" s="18" t="inlineStr">
-        <is>
-          <t>수집예정</t>
-        </is>
-      </c>
-      <c r="E57" s="18" t="inlineStr">
-        <is>
-          <t>수집예정</t>
-        </is>
-      </c>
-      <c r="F57" s="18" t="inlineStr">
-        <is>
-          <t>수집예정</t>
-        </is>
-      </c>
-      <c r="G57" s="6" t="inlineStr"/>
-      <c r="H57" s="6" t="inlineStr"/>
-      <c r="I57" s="6" t="inlineStr"/>
-      <c r="J57" s="18" t="inlineStr">
-        <is>
-          <t>수집예정</t>
-        </is>
-      </c>
-      <c r="K57" s="6" t="inlineStr"/>
-      <c r="L57" s="6" t="inlineStr"/>
-      <c r="M57" s="6" t="inlineStr"/>
-      <c r="N57" s="18" t="inlineStr">
-        <is>
-          <t>수집예정</t>
-        </is>
-      </c>
-      <c r="O57" s="6" t="inlineStr"/>
-      <c r="P57" s="18" t="inlineStr">
-        <is>
-          <t>수집예정</t>
-        </is>
-      </c>
-      <c r="Q57" s="18" t="inlineStr">
-        <is>
-          <t>수집예정</t>
-        </is>
-      </c>
-      <c r="R57" s="6" t="inlineStr">
-        <is>
-          <t>신고서 대기</t>
+    <row r="58">
+      <c r="A58" s="20" t="inlineStr">
+        <is>
+          <t>※ 상장 완료 = KIND 신규상장 페이지 기준(스팩합병 포함) · 스팩 공모상장은 밴드·밸류에이션 등 해당없음(공모가 2,000원 고정).</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" s="20" t="inlineStr">
         <is>
-          <t>※ 상장 완료 = KIND 신규상장 페이지 기준(스팩합병 포함) · 스팩 공모상장은 밴드·밸류에이션 등 해당없음(공모가 2,000원 고정).</t>
+          <t>※ 기재정정 신고서 내 정정 전·후 병존 → 자동수집은 "정정 후" 값만 취함.</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" s="20" t="inlineStr">
-        <is>
-          <t>※ 기재정정 신고서 내 정정 전·후 병존 → 자동수집은 "정정 후" 값만 취함.</t>
-        </is>
-      </c>
-    </row>
-    <row r="61">
-      <c r="A61" s="20" t="inlineStr">
         <is>
           <t>※ 청약경쟁률=일반투자자 청약수량÷최종배정수량 · "MM-DD~"는 종료일 자동수집 예정.</t>
         </is>
@@ -11045,7 +10961,7 @@
         <v>1</v>
       </c>
       <c r="E12" s="6" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F12" s="21">
         <f>IF((C12+D12)=0,"-",C12/(C12+D12))</f>

</xml_diff>

<commit_message>
chore: update IPO data 2026-07-28
</commit_message>
<xml_diff>
--- a/IPO_analysis.xlsx
+++ b/IPO_analysis.xlsx
@@ -9710,8 +9710,12 @@
         </is>
       </c>
       <c r="G41" s="6" t="inlineStr"/>
-      <c r="H41" s="6" t="inlineStr"/>
-      <c r="I41" s="6" t="inlineStr"/>
+      <c r="H41" s="6" t="n">
+        <v>50.4</v>
+      </c>
+      <c r="I41" s="6" t="n">
+        <v>307</v>
+      </c>
       <c r="J41" s="6" t="inlineStr">
         <is>
           <t>07-30~07-31</t>
@@ -9738,7 +9742,7 @@
       </c>
       <c r="R41" s="6" t="inlineStr">
         <is>
-          <t>정정</t>
+          <t>발행조건확정</t>
         </is>
       </c>
     </row>
@@ -10325,32 +10329,32 @@
     <row r="51" ht="30" customHeight="1">
       <c r="A51" s="6" t="inlineStr">
         <is>
-          <t>덕산넵코어스</t>
+          <t>글로벌테크놀로지</t>
         </is>
       </c>
       <c r="B51" s="6" t="inlineStr">
         <is>
-          <t>09-08~09-14</t>
+          <t>09-07~09-11</t>
         </is>
       </c>
       <c r="C51" s="6" t="inlineStr">
         <is>
-          <t>12,400~14,600</t>
+          <t>13,000~15,000</t>
         </is>
       </c>
       <c r="D51" s="7" t="inlineStr">
         <is>
-          <t>3,000,000</t>
+          <t>4,000,000</t>
         </is>
       </c>
       <c r="E51" s="7" t="inlineStr">
         <is>
-          <t>37,200,000,000</t>
+          <t>52,000,000,000</t>
         </is>
       </c>
       <c r="F51" s="6" t="inlineStr">
         <is>
-          <t>34.08배 (PER)</t>
+          <t>20.77배 (PER)</t>
         </is>
       </c>
       <c r="G51" s="6" t="inlineStr"/>
@@ -10366,18 +10370,18 @@
       <c r="M51" s="6" t="inlineStr"/>
       <c r="N51" s="6" t="inlineStr">
         <is>
-          <t>대신증권</t>
+          <t>한국투자증권</t>
         </is>
       </c>
       <c r="O51" s="6" t="inlineStr"/>
       <c r="P51" s="7" t="inlineStr">
         <is>
-          <t>1,413,399,926</t>
-        </is>
-      </c>
-      <c r="Q51" s="6" t="inlineStr">
-        <is>
-          <t>3.7%</t>
+          <t>2,119,999,960</t>
+        </is>
+      </c>
+      <c r="Q51" s="18" t="inlineStr">
+        <is>
+          <t>수집예정</t>
         </is>
       </c>
       <c r="R51" s="6" t="inlineStr">
@@ -10389,71 +10393,71 @@
     <row r="52" ht="30" customHeight="1">
       <c r="A52" s="6" t="inlineStr">
         <is>
-          <t>엔에이치스팩34호</t>
-        </is>
-      </c>
-      <c r="B52" s="18" t="inlineStr">
-        <is>
-          <t>수집예정</t>
-        </is>
-      </c>
-      <c r="C52" s="18" t="inlineStr">
-        <is>
-          <t>수집예정</t>
-        </is>
-      </c>
-      <c r="D52" s="18" t="inlineStr">
-        <is>
-          <t>수집예정</t>
-        </is>
-      </c>
-      <c r="E52" s="18" t="inlineStr">
-        <is>
-          <t>수집예정</t>
-        </is>
-      </c>
-      <c r="F52" s="18" t="inlineStr">
-        <is>
-          <t>수집예정</t>
+          <t>덕산넵코어스</t>
+        </is>
+      </c>
+      <c r="B52" s="6" t="inlineStr">
+        <is>
+          <t>09-08~09-14</t>
+        </is>
+      </c>
+      <c r="C52" s="6" t="inlineStr">
+        <is>
+          <t>12,400~14,600</t>
+        </is>
+      </c>
+      <c r="D52" s="7" t="inlineStr">
+        <is>
+          <t>3,000,000</t>
+        </is>
+      </c>
+      <c r="E52" s="7" t="inlineStr">
+        <is>
+          <t>37,200,000,000</t>
+        </is>
+      </c>
+      <c r="F52" s="6" t="inlineStr">
+        <is>
+          <t>34.08배 (PER)</t>
         </is>
       </c>
       <c r="G52" s="6" t="inlineStr"/>
       <c r="H52" s="6" t="inlineStr"/>
       <c r="I52" s="6" t="inlineStr"/>
-      <c r="J52" s="18" t="inlineStr">
-        <is>
-          <t>수집예정</t>
+      <c r="J52" s="6" t="inlineStr">
+        <is>
+          <t>09-16~09-17</t>
         </is>
       </c>
       <c r="K52" s="6" t="inlineStr"/>
       <c r="L52" s="6" t="inlineStr"/>
       <c r="M52" s="6" t="inlineStr"/>
-      <c r="N52" s="18" t="inlineStr">
-        <is>
-          <t>수집예정</t>
+      <c r="N52" s="6" t="inlineStr">
+        <is>
+          <t>대신증권</t>
         </is>
       </c>
       <c r="O52" s="6" t="inlineStr"/>
-      <c r="P52" s="18" t="inlineStr">
-        <is>
-          <t>수집예정</t>
-        </is>
-      </c>
-      <c r="Q52" s="18" t="inlineStr">
-        <is>
-          <t>수집예정</t>
+      <c r="P52" s="7" t="inlineStr">
+        <is>
+          <t>1,413,399,926</t>
+        </is>
+      </c>
+      <c r="Q52" s="6" t="inlineStr">
+        <is>
+          <t>3.7%</t>
         </is>
       </c>
       <c r="R52" s="6" t="inlineStr">
         <is>
-          <t>corp_code 미확보(수동확인)</t>
+          <t>최초</t>
         </is>
       </c>
     </row>
     <row r="53" ht="30" customHeight="1">
       <c r="A53" s="6" t="inlineStr">
         <is>
-          <t>와이즈플래닛컴퍼니</t>
+          <t>엔에이치스팩34호</t>
         </is>
       </c>
       <c r="B53" s="18" t="inlineStr">
@@ -10492,9 +10496,9 @@
       <c r="K53" s="6" t="inlineStr"/>
       <c r="L53" s="6" t="inlineStr"/>
       <c r="M53" s="6" t="inlineStr"/>
-      <c r="N53" s="6" t="inlineStr">
-        <is>
-          <t>대신</t>
+      <c r="N53" s="18" t="inlineStr">
+        <is>
+          <t>수집예정</t>
         </is>
       </c>
       <c r="O53" s="6" t="inlineStr"/>
@@ -10510,14 +10514,14 @@
       </c>
       <c r="R53" s="6" t="inlineStr">
         <is>
-          <t>신고서 대기</t>
+          <t>corp_code 미확보(수동확인)</t>
         </is>
       </c>
     </row>
     <row r="54" ht="30" customHeight="1">
       <c r="A54" s="6" t="inlineStr">
         <is>
-          <t>엠에스바이오</t>
+          <t>와이즈플래닛컴퍼니</t>
         </is>
       </c>
       <c r="B54" s="18" t="inlineStr">
@@ -10556,9 +10560,9 @@
       <c r="K54" s="6" t="inlineStr"/>
       <c r="L54" s="6" t="inlineStr"/>
       <c r="M54" s="6" t="inlineStr"/>
-      <c r="N54" s="18" t="inlineStr">
-        <is>
-          <t>수집예정</t>
+      <c r="N54" s="6" t="inlineStr">
+        <is>
+          <t>대신</t>
         </is>
       </c>
       <c r="O54" s="6" t="inlineStr"/>
@@ -10581,7 +10585,7 @@
     <row r="55" ht="30" customHeight="1">
       <c r="A55" s="6" t="inlineStr">
         <is>
-          <t>디티에스</t>
+          <t>엠에스바이오</t>
         </is>
       </c>
       <c r="B55" s="18" t="inlineStr">
@@ -10645,7 +10649,7 @@
     <row r="56" ht="30" customHeight="1">
       <c r="A56" s="6" t="inlineStr">
         <is>
-          <t>글로벌테크놀로지</t>
+          <t>디티에스</t>
         </is>
       </c>
       <c r="B56" s="18" t="inlineStr">
@@ -11039,75 +11043,75 @@
     <row r="18">
       <c r="A18" s="6" t="inlineStr">
         <is>
-          <t>대신증권</t>
+          <t>한국투자증권</t>
         </is>
       </c>
       <c r="B18" s="6" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C18" s="6" t="inlineStr">
         <is>
-          <t>64,800,000,000</t>
+          <t>89,000,000,000</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="6" t="inlineStr">
         <is>
-          <t>미래에셋증권</t>
+          <t>대신증권</t>
         </is>
       </c>
       <c r="B19" s="6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C19" s="6" t="inlineStr">
         <is>
-          <t>42,160,000,000</t>
+          <t>64,800,000,000</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="6" t="inlineStr">
         <is>
-          <t>아이비케이투자증권</t>
+          <t>미래에셋증권</t>
         </is>
       </c>
       <c r="B20" s="6" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C20" s="6" t="inlineStr">
         <is>
-          <t>41,400,000,000</t>
+          <t>42,160,000,000</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="6" t="inlineStr">
         <is>
-          <t>유진투자증권</t>
+          <t>아이비케이투자증권</t>
         </is>
       </c>
       <c r="B21" s="6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C21" s="6" t="inlineStr">
         <is>
-          <t>40,000,000,000</t>
+          <t>41,400,000,000</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="6" t="inlineStr">
         <is>
-          <t>한국투자증권</t>
+          <t>유진투자증권</t>
         </is>
       </c>
       <c r="B22" s="6" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C22" s="6" t="inlineStr">
         <is>
-          <t>37,000,000,000</t>
+          <t>40,000,000,000</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore: update IPO data 2026-07-29
</commit_message>
<xml_diff>
--- a/IPO_analysis.xlsx
+++ b/IPO_analysis.xlsx
@@ -618,14 +618,14 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>기준일 2026-07-28 · 청구일 직전 사업연도 · 별도/개별 재무제표 · 단위 백만원(별도 표기 시 USD)</t>
+          <t>기준일 2026-07-29 · 청구일 직전 사업연도 · 별도/개별 재무제표 · 단위 백만원(별도 표기 시 USD)</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
-          <t>■ 심사 신청(진행중)  (52건)</t>
+          <t>■ 심사 신청(진행중)  (48건)</t>
         </is>
       </c>
       <c r="B4" s="4" t="n"/>
@@ -1986,12 +1986,12 @@
     <row r="29">
       <c r="A29" s="6" t="inlineStr">
         <is>
-          <t>2026-06-12</t>
+          <t>2026-06-11</t>
         </is>
       </c>
       <c r="B29" s="6" t="inlineStr">
         <is>
-          <t>에스케이증권제14호기업인수목적</t>
+          <t>씨엔티테크</t>
         </is>
       </c>
       <c r="C29" s="6" t="inlineStr">
@@ -2011,27 +2011,27 @@
       </c>
       <c r="F29" s="7" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>27,015</t>
         </is>
       </c>
       <c r="G29" s="7" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>3,987</t>
         </is>
       </c>
       <c r="H29" s="7" t="inlineStr">
         <is>
-          <t>17</t>
+          <t>2,613</t>
         </is>
       </c>
       <c r="I29" s="6" t="inlineStr">
         <is>
-          <t>기타 금융업</t>
+          <t>소프트웨어 개발 및 공급업</t>
         </is>
       </c>
       <c r="J29" s="6" t="inlineStr">
         <is>
-          <t>SK</t>
+          <t>한화, 하나</t>
         </is>
       </c>
       <c r="K29" s="6" t="inlineStr">
@@ -2043,12 +2043,12 @@
     <row r="30">
       <c r="A30" s="6" t="inlineStr">
         <is>
-          <t>2026-06-12</t>
+          <t>2026-06-11</t>
         </is>
       </c>
       <c r="B30" s="6" t="inlineStr">
         <is>
-          <t>케이비제34호스팩</t>
+          <t>제이앤티지</t>
         </is>
       </c>
       <c r="C30" s="6" t="inlineStr">
@@ -2068,27 +2068,27 @@
       </c>
       <c r="F30" s="7" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>72,378</t>
         </is>
       </c>
       <c r="G30" s="7" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>9,904</t>
         </is>
       </c>
       <c r="H30" s="7" t="inlineStr">
         <is>
-          <t>21</t>
+          <t>6,743</t>
         </is>
       </c>
       <c r="I30" s="6" t="inlineStr">
         <is>
-          <t>기타 금융업</t>
+          <t>전자부품 제조업</t>
         </is>
       </c>
       <c r="J30" s="6" t="inlineStr">
         <is>
-          <t>KB</t>
+          <t>대신, NH</t>
         </is>
       </c>
       <c r="K30" s="6" t="inlineStr">
@@ -2100,12 +2100,12 @@
     <row r="31">
       <c r="A31" s="6" t="inlineStr">
         <is>
-          <t>2026-06-12</t>
+          <t>2026-05-29</t>
         </is>
       </c>
       <c r="B31" s="6" t="inlineStr">
         <is>
-          <t>한국제17호스팩</t>
+          <t>유캐스트</t>
         </is>
       </c>
       <c r="C31" s="6" t="inlineStr">
@@ -2125,27 +2125,27 @@
       </c>
       <c r="F31" s="7" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>5,934</t>
         </is>
       </c>
       <c r="G31" s="7" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>-3,557</t>
         </is>
       </c>
       <c r="H31" s="7" t="inlineStr">
         <is>
-          <t>170</t>
+          <t>1,881</t>
         </is>
       </c>
       <c r="I31" s="6" t="inlineStr">
         <is>
-          <t>기타 금융업</t>
+          <t>통신 및 방송 장비 제조업</t>
         </is>
       </c>
       <c r="J31" s="6" t="inlineStr">
         <is>
-          <t>한국</t>
+          <t>유진</t>
         </is>
       </c>
       <c r="K31" s="6" t="inlineStr">
@@ -2157,12 +2157,12 @@
     <row r="32">
       <c r="A32" s="6" t="inlineStr">
         <is>
-          <t>2026-06-12</t>
+          <t>2026-05-29</t>
         </is>
       </c>
       <c r="B32" s="6" t="inlineStr">
         <is>
-          <t>한화플러스제6호스팩</t>
+          <t>인터엑스</t>
         </is>
       </c>
       <c r="C32" s="6" t="inlineStr">
@@ -2182,27 +2182,27 @@
       </c>
       <c r="F32" s="7" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>8,645</t>
         </is>
       </c>
       <c r="G32" s="7" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>-20,272</t>
         </is>
       </c>
       <c r="H32" s="7" t="inlineStr">
         <is>
-          <t>41</t>
+          <t>4,530</t>
         </is>
       </c>
       <c r="I32" s="6" t="inlineStr">
         <is>
-          <t>기타 금융업</t>
+          <t>소프트웨어 개발 및 공급업</t>
         </is>
       </c>
       <c r="J32" s="6" t="inlineStr">
         <is>
-          <t>한화</t>
+          <t>한국</t>
         </is>
       </c>
       <c r="K32" s="6" t="inlineStr">
@@ -2214,12 +2214,12 @@
     <row r="33">
       <c r="A33" s="6" t="inlineStr">
         <is>
-          <t>2026-06-11</t>
+          <t>2026-05-29</t>
         </is>
       </c>
       <c r="B33" s="6" t="inlineStr">
         <is>
-          <t>씨엔티테크</t>
+          <t>케이엠에프</t>
         </is>
       </c>
       <c r="C33" s="6" t="inlineStr">
@@ -2239,27 +2239,27 @@
       </c>
       <c r="F33" s="7" t="inlineStr">
         <is>
-          <t>27,015</t>
+          <t>25,751</t>
         </is>
       </c>
       <c r="G33" s="7" t="inlineStr">
         <is>
-          <t>3,987</t>
+          <t>11,463</t>
         </is>
       </c>
       <c r="H33" s="7" t="inlineStr">
         <is>
-          <t>2,613</t>
+          <t>642</t>
         </is>
       </c>
       <c r="I33" s="6" t="inlineStr">
         <is>
-          <t>소프트웨어 개발 및 공급업</t>
+          <t>기타 식품 제조업</t>
         </is>
       </c>
       <c r="J33" s="6" t="inlineStr">
         <is>
-          <t>한화, 하나</t>
+          <t>IBK</t>
         </is>
       </c>
       <c r="K33" s="6" t="inlineStr">
@@ -2271,12 +2271,12 @@
     <row r="34">
       <c r="A34" s="6" t="inlineStr">
         <is>
-          <t>2026-06-11</t>
+          <t>2026-05-29</t>
         </is>
       </c>
       <c r="B34" s="6" t="inlineStr">
         <is>
-          <t>제이앤티지</t>
+          <t>하나에어로다이내믹스</t>
         </is>
       </c>
       <c r="C34" s="6" t="inlineStr">
@@ -2296,27 +2296,27 @@
       </c>
       <c r="F34" s="7" t="inlineStr">
         <is>
-          <t>72,378</t>
+          <t>33,286</t>
         </is>
       </c>
       <c r="G34" s="7" t="inlineStr">
         <is>
-          <t>9,904</t>
+          <t>2,420</t>
         </is>
       </c>
       <c r="H34" s="7" t="inlineStr">
         <is>
-          <t>6,743</t>
+          <t>890</t>
         </is>
       </c>
       <c r="I34" s="6" t="inlineStr">
         <is>
-          <t>전자부품 제조업</t>
+          <t>항공기,우주선 및 부품 제조업</t>
         </is>
       </c>
       <c r="J34" s="6" t="inlineStr">
         <is>
-          <t>대신, NH</t>
+          <t>IBK</t>
         </is>
       </c>
       <c r="K34" s="6" t="inlineStr">
@@ -2328,12 +2328,12 @@
     <row r="35">
       <c r="A35" s="6" t="inlineStr">
         <is>
-          <t>2026-05-29</t>
+          <t>2026-05-28</t>
         </is>
       </c>
       <c r="B35" s="6" t="inlineStr">
         <is>
-          <t>유캐스트</t>
+          <t>다비오</t>
         </is>
       </c>
       <c r="C35" s="6" t="inlineStr">
@@ -2353,27 +2353,27 @@
       </c>
       <c r="F35" s="7" t="inlineStr">
         <is>
-          <t>5,934</t>
+          <t>9,251</t>
         </is>
       </c>
       <c r="G35" s="7" t="inlineStr">
         <is>
-          <t>-3,557</t>
+          <t>-3,473</t>
         </is>
       </c>
       <c r="H35" s="7" t="inlineStr">
         <is>
-          <t>1,881</t>
+          <t>300</t>
         </is>
       </c>
       <c r="I35" s="6" t="inlineStr">
         <is>
-          <t>통신 및 방송 장비 제조업</t>
+          <t>소프트웨어 개발 및 공급업</t>
         </is>
       </c>
       <c r="J35" s="6" t="inlineStr">
         <is>
-          <t>유진</t>
+          <t>대신</t>
         </is>
       </c>
       <c r="K35" s="6" t="inlineStr">
@@ -2385,12 +2385,12 @@
     <row r="36">
       <c r="A36" s="6" t="inlineStr">
         <is>
-          <t>2026-05-29</t>
+          <t>2026-05-28</t>
         </is>
       </c>
       <c r="B36" s="6" t="inlineStr">
         <is>
-          <t>인터엑스</t>
+          <t>삼홍아크튜리온</t>
         </is>
       </c>
       <c r="C36" s="6" t="inlineStr">
@@ -2410,27 +2410,27 @@
       </c>
       <c r="F36" s="7" t="inlineStr">
         <is>
-          <t>8,645</t>
+          <t>26,162</t>
         </is>
       </c>
       <c r="G36" s="7" t="inlineStr">
         <is>
-          <t>-20,272</t>
+          <t>-10,314</t>
         </is>
       </c>
       <c r="H36" s="7" t="inlineStr">
         <is>
-          <t>4,530</t>
+          <t>6,369</t>
         </is>
       </c>
       <c r="I36" s="6" t="inlineStr">
         <is>
-          <t>소프트웨어 개발 및 공급업</t>
+          <t>구조용 금속제품, 탱크 및 증기발생기 제조업</t>
         </is>
       </c>
       <c r="J36" s="6" t="inlineStr">
         <is>
-          <t>한국</t>
+          <t>삼성, 미래</t>
         </is>
       </c>
       <c r="K36" s="6" t="inlineStr">
@@ -2442,12 +2442,12 @@
     <row r="37">
       <c r="A37" s="6" t="inlineStr">
         <is>
-          <t>2026-05-29</t>
+          <t>2026-05-22</t>
         </is>
       </c>
       <c r="B37" s="6" t="inlineStr">
         <is>
-          <t>케이엠에프</t>
+          <t>에이엘로봇</t>
         </is>
       </c>
       <c r="C37" s="6" t="inlineStr">
@@ -2467,27 +2467,27 @@
       </c>
       <c r="F37" s="7" t="inlineStr">
         <is>
-          <t>25,751</t>
+          <t>14,985</t>
         </is>
       </c>
       <c r="G37" s="7" t="inlineStr">
         <is>
-          <t>11,463</t>
+          <t>-21,891</t>
         </is>
       </c>
       <c r="H37" s="7" t="inlineStr">
         <is>
-          <t>642</t>
+          <t>129</t>
         </is>
       </c>
       <c r="I37" s="6" t="inlineStr">
         <is>
-          <t>기타 식품 제조업</t>
+          <t>산업용 로봇 제조업</t>
         </is>
       </c>
       <c r="J37" s="6" t="inlineStr">
         <is>
-          <t>IBK</t>
+          <t>대신</t>
         </is>
       </c>
       <c r="K37" s="6" t="inlineStr">
@@ -2499,12 +2499,12 @@
     <row r="38">
       <c r="A38" s="6" t="inlineStr">
         <is>
-          <t>2026-05-29</t>
+          <t>2026-05-21</t>
         </is>
       </c>
       <c r="B38" s="6" t="inlineStr">
         <is>
-          <t>하나에어로다이내믹스</t>
+          <t>넥스트에어로스페이스</t>
         </is>
       </c>
       <c r="C38" s="6" t="inlineStr">
@@ -2524,27 +2524,27 @@
       </c>
       <c r="F38" s="7" t="inlineStr">
         <is>
-          <t>33,286</t>
+          <t>12,084</t>
         </is>
       </c>
       <c r="G38" s="7" t="inlineStr">
         <is>
-          <t>2,420</t>
+          <t>-17,270</t>
         </is>
       </c>
       <c r="H38" s="7" t="inlineStr">
         <is>
-          <t>890</t>
+          <t>6,158</t>
         </is>
       </c>
       <c r="I38" s="6" t="inlineStr">
         <is>
-          <t>항공기,우주선 및 부품 제조업</t>
+          <t>유인 항공기, 항공우주선 및 보조장치 제조업</t>
         </is>
       </c>
       <c r="J38" s="6" t="inlineStr">
         <is>
-          <t>IBK</t>
+          <t>삼성</t>
         </is>
       </c>
       <c r="K38" s="6" t="inlineStr">
@@ -2556,12 +2556,12 @@
     <row r="39">
       <c r="A39" s="6" t="inlineStr">
         <is>
-          <t>2026-05-28</t>
+          <t>2026-05-21</t>
         </is>
       </c>
       <c r="B39" s="6" t="inlineStr">
         <is>
-          <t>다비오</t>
+          <t>래블업</t>
         </is>
       </c>
       <c r="C39" s="6" t="inlineStr">
@@ -2581,27 +2581,27 @@
       </c>
       <c r="F39" s="7" t="inlineStr">
         <is>
-          <t>9,251</t>
+          <t>6,712</t>
         </is>
       </c>
       <c r="G39" s="7" t="inlineStr">
         <is>
-          <t>-3,473</t>
+          <t>-1,526</t>
         </is>
       </c>
       <c r="H39" s="7" t="inlineStr">
         <is>
-          <t>300</t>
+          <t>373</t>
         </is>
       </c>
       <c r="I39" s="6" t="inlineStr">
         <is>
-          <t>소프트웨어 개발 및 공급업</t>
+          <t>데이터베이스 및 온라인정보 제공업</t>
         </is>
       </c>
       <c r="J39" s="6" t="inlineStr">
         <is>
-          <t>대신</t>
+          <t>NH</t>
         </is>
       </c>
       <c r="K39" s="6" t="inlineStr">
@@ -2613,12 +2613,12 @@
     <row r="40">
       <c r="A40" s="6" t="inlineStr">
         <is>
-          <t>2026-05-28</t>
+          <t>2026-05-21</t>
         </is>
       </c>
       <c r="B40" s="6" t="inlineStr">
         <is>
-          <t>삼홍아크튜리온</t>
+          <t>비앤비코리아</t>
         </is>
       </c>
       <c r="C40" s="6" t="inlineStr">
@@ -2638,27 +2638,27 @@
       </c>
       <c r="F40" s="7" t="inlineStr">
         <is>
-          <t>26,162</t>
+          <t>141,169</t>
         </is>
       </c>
       <c r="G40" s="7" t="inlineStr">
         <is>
-          <t>-10,314</t>
+          <t>21,406</t>
         </is>
       </c>
       <c r="H40" s="7" t="inlineStr">
         <is>
-          <t>6,369</t>
+          <t>43,932</t>
         </is>
       </c>
       <c r="I40" s="6" t="inlineStr">
         <is>
-          <t>구조용 금속제품, 탱크 및 증기발생기 제조업</t>
+          <t>기타 화학제품 제조업</t>
         </is>
       </c>
       <c r="J40" s="6" t="inlineStr">
         <is>
-          <t>삼성, 미래</t>
+          <t>미래</t>
         </is>
       </c>
       <c r="K40" s="6" t="inlineStr">
@@ -2670,12 +2670,12 @@
     <row r="41">
       <c r="A41" s="6" t="inlineStr">
         <is>
-          <t>2026-05-22</t>
+          <t>2026-05-21</t>
         </is>
       </c>
       <c r="B41" s="6" t="inlineStr">
         <is>
-          <t>에이엘로봇</t>
+          <t>에이엔에이치스트럭쳐</t>
         </is>
       </c>
       <c r="C41" s="6" t="inlineStr">
@@ -2695,27 +2695,27 @@
       </c>
       <c r="F41" s="7" t="inlineStr">
         <is>
-          <t>14,985</t>
+          <t>19,784</t>
         </is>
       </c>
       <c r="G41" s="7" t="inlineStr">
         <is>
-          <t>-21,891</t>
+          <t>-4,296</t>
         </is>
       </c>
       <c r="H41" s="7" t="inlineStr">
         <is>
-          <t>129</t>
+          <t>24,561</t>
         </is>
       </c>
       <c r="I41" s="6" t="inlineStr">
         <is>
-          <t>산업용 로봇 제조업</t>
+          <t>건축기술, 엔지니어링 및 관련 기술 서비스업</t>
         </is>
       </c>
       <c r="J41" s="6" t="inlineStr">
         <is>
-          <t>대신</t>
+          <t>NH</t>
         </is>
       </c>
       <c r="K41" s="6" t="inlineStr">
@@ -2727,12 +2727,12 @@
     <row r="42">
       <c r="A42" s="6" t="inlineStr">
         <is>
-          <t>2026-05-21</t>
+          <t>2026-05-19</t>
         </is>
       </c>
       <c r="B42" s="6" t="inlineStr">
         <is>
-          <t>넥스트에어로스페이스</t>
+          <t>엘리스그룹</t>
         </is>
       </c>
       <c r="C42" s="6" t="inlineStr">
@@ -2752,27 +2752,27 @@
       </c>
       <c r="F42" s="7" t="inlineStr">
         <is>
-          <t>12,084</t>
+          <t>39,513</t>
         </is>
       </c>
       <c r="G42" s="7" t="inlineStr">
         <is>
-          <t>-17,270</t>
+          <t>15,666</t>
         </is>
       </c>
       <c r="H42" s="7" t="inlineStr">
         <is>
-          <t>6,158</t>
+          <t>85,400</t>
         </is>
       </c>
       <c r="I42" s="6" t="inlineStr">
         <is>
-          <t>유인 항공기, 항공우주선 및 보조장치 제조업</t>
+          <t>소프트웨어 개발 및 공급업</t>
         </is>
       </c>
       <c r="J42" s="6" t="inlineStr">
         <is>
-          <t>삼성</t>
+          <t>미래, 삼성</t>
         </is>
       </c>
       <c r="K42" s="6" t="inlineStr">
@@ -2784,12 +2784,12 @@
     <row r="43">
       <c r="A43" s="6" t="inlineStr">
         <is>
-          <t>2026-05-21</t>
+          <t>2026-05-12</t>
         </is>
       </c>
       <c r="B43" s="6" t="inlineStr">
         <is>
-          <t>래블업</t>
+          <t>오토핸즈</t>
         </is>
       </c>
       <c r="C43" s="6" t="inlineStr">
@@ -2799,7 +2799,7 @@
       </c>
       <c r="D43" s="6" t="inlineStr">
         <is>
-          <t>신규상장</t>
+          <t>스팩 소멸합병</t>
         </is>
       </c>
       <c r="E43" s="6" t="inlineStr">
@@ -2809,27 +2809,27 @@
       </c>
       <c r="F43" s="7" t="inlineStr">
         <is>
-          <t>6,712</t>
+          <t>238,564</t>
         </is>
       </c>
       <c r="G43" s="7" t="inlineStr">
         <is>
-          <t>-1,526</t>
+          <t>6,047</t>
         </is>
       </c>
       <c r="H43" s="7" t="inlineStr">
         <is>
-          <t>373</t>
+          <t>6,129</t>
         </is>
       </c>
       <c r="I43" s="6" t="inlineStr">
         <is>
-          <t>데이터베이스 및 온라인정보 제공업</t>
+          <t>자동차 판매업</t>
         </is>
       </c>
       <c r="J43" s="6" t="inlineStr">
         <is>
-          <t>NH</t>
+          <t>미래</t>
         </is>
       </c>
       <c r="K43" s="6" t="inlineStr">
@@ -2841,12 +2841,12 @@
     <row r="44">
       <c r="A44" s="6" t="inlineStr">
         <is>
-          <t>2026-05-21</t>
+          <t>2026-05-06</t>
         </is>
       </c>
       <c r="B44" s="6" t="inlineStr">
         <is>
-          <t>비앤비코리아</t>
+          <t>아이벡스메디칼시스템즈</t>
         </is>
       </c>
       <c r="C44" s="6" t="inlineStr">
@@ -2866,27 +2866,27 @@
       </c>
       <c r="F44" s="7" t="inlineStr">
         <is>
-          <t>141,169</t>
+          <t>15,282</t>
         </is>
       </c>
       <c r="G44" s="7" t="inlineStr">
         <is>
-          <t>21,406</t>
+          <t>-7,227</t>
         </is>
       </c>
       <c r="H44" s="7" t="inlineStr">
         <is>
-          <t>43,932</t>
+          <t>744</t>
         </is>
       </c>
       <c r="I44" s="6" t="inlineStr">
         <is>
-          <t>기타 화학제품 제조업</t>
+          <t>의료용 기기 제조업</t>
         </is>
       </c>
       <c r="J44" s="6" t="inlineStr">
         <is>
-          <t>미래</t>
+          <t>NH</t>
         </is>
       </c>
       <c r="K44" s="6" t="inlineStr">
@@ -2898,12 +2898,12 @@
     <row r="45">
       <c r="A45" s="6" t="inlineStr">
         <is>
-          <t>2026-05-21</t>
+          <t>2026-04-30</t>
         </is>
       </c>
       <c r="B45" s="6" t="inlineStr">
         <is>
-          <t>에이엔에이치스트럭쳐</t>
+          <t>멜콘</t>
         </is>
       </c>
       <c r="C45" s="6" t="inlineStr">
@@ -2923,27 +2923,27 @@
       </c>
       <c r="F45" s="7" t="inlineStr">
         <is>
-          <t>19,784</t>
+          <t>39,319</t>
         </is>
       </c>
       <c r="G45" s="7" t="inlineStr">
         <is>
-          <t>-4,296</t>
+          <t>4,739</t>
         </is>
       </c>
       <c r="H45" s="7" t="inlineStr">
         <is>
-          <t>24,561</t>
+          <t>1,250</t>
         </is>
       </c>
       <c r="I45" s="6" t="inlineStr">
         <is>
-          <t>건축기술, 엔지니어링 및 관련 기술 서비스업</t>
+          <t>특수 목적용 기계 제조업</t>
         </is>
       </c>
       <c r="J45" s="6" t="inlineStr">
         <is>
-          <t>NH</t>
+          <t>대신</t>
         </is>
       </c>
       <c r="K45" s="6" t="inlineStr">
@@ -2955,12 +2955,12 @@
     <row r="46">
       <c r="A46" s="6" t="inlineStr">
         <is>
-          <t>2026-05-19</t>
+          <t>2026-04-30</t>
         </is>
       </c>
       <c r="B46" s="6" t="inlineStr">
         <is>
-          <t>엘리스그룹</t>
+          <t>바로팜</t>
         </is>
       </c>
       <c r="C46" s="6" t="inlineStr">
@@ -2980,27 +2980,27 @@
       </c>
       <c r="F46" s="7" t="inlineStr">
         <is>
-          <t>39,513</t>
+          <t>96,724</t>
         </is>
       </c>
       <c r="G46" s="7" t="inlineStr">
         <is>
-          <t>15,666</t>
+          <t>-9,679</t>
         </is>
       </c>
       <c r="H46" s="7" t="inlineStr">
         <is>
-          <t>85,400</t>
+          <t>30,673</t>
         </is>
       </c>
       <c r="I46" s="6" t="inlineStr">
         <is>
-          <t>소프트웨어 개발 및 공급업</t>
+          <t>상품 중개업</t>
         </is>
       </c>
       <c r="J46" s="6" t="inlineStr">
         <is>
-          <t>미래, 삼성</t>
+          <t>미래</t>
         </is>
       </c>
       <c r="K46" s="6" t="inlineStr">
@@ -3012,12 +3012,12 @@
     <row r="47">
       <c r="A47" s="6" t="inlineStr">
         <is>
-          <t>2026-05-12</t>
+          <t>2026-04-30</t>
         </is>
       </c>
       <c r="B47" s="6" t="inlineStr">
         <is>
-          <t>오토핸즈</t>
+          <t>텔레픽스</t>
         </is>
       </c>
       <c r="C47" s="6" t="inlineStr">
@@ -3027,7 +3027,7 @@
       </c>
       <c r="D47" s="6" t="inlineStr">
         <is>
-          <t>스팩 소멸합병</t>
+          <t>신규상장</t>
         </is>
       </c>
       <c r="E47" s="6" t="inlineStr">
@@ -3037,22 +3037,22 @@
       </c>
       <c r="F47" s="7" t="inlineStr">
         <is>
-          <t>238,564</t>
+          <t>4,896</t>
         </is>
       </c>
       <c r="G47" s="7" t="inlineStr">
         <is>
-          <t>6,047</t>
+          <t>-16,214</t>
         </is>
       </c>
       <c r="H47" s="7" t="inlineStr">
         <is>
-          <t>6,129</t>
+          <t>9,146</t>
         </is>
       </c>
       <c r="I47" s="6" t="inlineStr">
         <is>
-          <t>자동차 판매업</t>
+          <t>소프트웨어 개발 및 공급업</t>
         </is>
       </c>
       <c r="J47" s="6" t="inlineStr">
@@ -3069,12 +3069,12 @@
     <row r="48">
       <c r="A48" s="6" t="inlineStr">
         <is>
-          <t>2026-05-06</t>
+          <t>2026-04-10</t>
         </is>
       </c>
       <c r="B48" s="6" t="inlineStr">
         <is>
-          <t>아이벡스메디칼시스템즈</t>
+          <t>엠비디</t>
         </is>
       </c>
       <c r="C48" s="6" t="inlineStr">
@@ -3094,27 +3094,27 @@
       </c>
       <c r="F48" s="7" t="inlineStr">
         <is>
-          <t>15,282</t>
+          <t>1,524</t>
         </is>
       </c>
       <c r="G48" s="7" t="inlineStr">
         <is>
-          <t>-7,227</t>
+          <t>-2,125</t>
         </is>
       </c>
       <c r="H48" s="7" t="inlineStr">
         <is>
-          <t>744</t>
+          <t>2,753</t>
         </is>
       </c>
       <c r="I48" s="6" t="inlineStr">
         <is>
-          <t>의료용 기기 제조업</t>
+          <t>물질 검사, 측정 및 분석기구 제조업</t>
         </is>
       </c>
       <c r="J48" s="6" t="inlineStr">
         <is>
-          <t>NH</t>
+          <t>하나</t>
         </is>
       </c>
       <c r="K48" s="6" t="inlineStr">
@@ -3126,12 +3126,12 @@
     <row r="49">
       <c r="A49" s="6" t="inlineStr">
         <is>
-          <t>2026-04-30</t>
+          <t>2026-04-08</t>
         </is>
       </c>
       <c r="B49" s="6" t="inlineStr">
         <is>
-          <t>멜콘</t>
+          <t>옵토닉스</t>
         </is>
       </c>
       <c r="C49" s="6" t="inlineStr">
@@ -3151,27 +3151,27 @@
       </c>
       <c r="F49" s="7" t="inlineStr">
         <is>
-          <t>39,319</t>
+          <t>25,368</t>
         </is>
       </c>
       <c r="G49" s="7" t="inlineStr">
         <is>
-          <t>4,739</t>
+          <t>1,901</t>
         </is>
       </c>
       <c r="H49" s="7" t="inlineStr">
         <is>
-          <t>1,250</t>
+          <t>730</t>
         </is>
       </c>
       <c r="I49" s="6" t="inlineStr">
         <is>
-          <t>특수 목적용 기계 제조업</t>
+          <t>광학렌즈 및 광학요소 제조업</t>
         </is>
       </c>
       <c r="J49" s="6" t="inlineStr">
         <is>
-          <t>대신</t>
+          <t>한국</t>
         </is>
       </c>
       <c r="K49" s="6" t="inlineStr">
@@ -3183,12 +3183,12 @@
     <row r="50">
       <c r="A50" s="6" t="inlineStr">
         <is>
-          <t>2026-04-30</t>
+          <t>2026-04-07</t>
         </is>
       </c>
       <c r="B50" s="6" t="inlineStr">
         <is>
-          <t>바로팜</t>
+          <t>크리에이츠</t>
         </is>
       </c>
       <c r="C50" s="6" t="inlineStr">
@@ -3208,27 +3208,27 @@
       </c>
       <c r="F50" s="7" t="inlineStr">
         <is>
-          <t>96,724</t>
+          <t>76,395</t>
         </is>
       </c>
       <c r="G50" s="7" t="inlineStr">
         <is>
-          <t>-9,679</t>
+          <t>23,749</t>
         </is>
       </c>
       <c r="H50" s="7" t="inlineStr">
         <is>
-          <t>30,673</t>
+          <t>2,335</t>
         </is>
       </c>
       <c r="I50" s="6" t="inlineStr">
         <is>
-          <t>상품 중개업</t>
+          <t>그외 기타 제품 제조업</t>
         </is>
       </c>
       <c r="J50" s="6" t="inlineStr">
         <is>
-          <t>미래</t>
+          <t>삼성</t>
         </is>
       </c>
       <c r="K50" s="6" t="inlineStr">
@@ -3240,12 +3240,12 @@
     <row r="51">
       <c r="A51" s="6" t="inlineStr">
         <is>
-          <t>2026-04-30</t>
+          <t>2026-03-24</t>
         </is>
       </c>
       <c r="B51" s="6" t="inlineStr">
         <is>
-          <t>텔레픽스</t>
+          <t>인텔리빅스</t>
         </is>
       </c>
       <c r="C51" s="6" t="inlineStr">
@@ -3265,17 +3265,17 @@
       </c>
       <c r="F51" s="7" t="inlineStr">
         <is>
-          <t>4,896</t>
+          <t>46,644</t>
         </is>
       </c>
       <c r="G51" s="7" t="inlineStr">
         <is>
-          <t>-16,214</t>
+          <t>5,357</t>
         </is>
       </c>
       <c r="H51" s="7" t="inlineStr">
         <is>
-          <t>9,146</t>
+          <t>1,048</t>
         </is>
       </c>
       <c r="I51" s="6" t="inlineStr">
@@ -3297,12 +3297,12 @@
     <row r="52">
       <c r="A52" s="6" t="inlineStr">
         <is>
-          <t>2026-04-10</t>
+          <t>2026-02-27</t>
         </is>
       </c>
       <c r="B52" s="6" t="inlineStr">
         <is>
-          <t>엠비디</t>
+          <t>피지티</t>
         </is>
       </c>
       <c r="C52" s="6" t="inlineStr">
@@ -3322,27 +3322,27 @@
       </c>
       <c r="F52" s="7" t="inlineStr">
         <is>
-          <t>1,524</t>
+          <t>40,141</t>
         </is>
       </c>
       <c r="G52" s="7" t="inlineStr">
         <is>
-          <t>-2,125</t>
+          <t>-69,722</t>
         </is>
       </c>
       <c r="H52" s="7" t="inlineStr">
         <is>
-          <t>2,753</t>
+          <t>6,029</t>
         </is>
       </c>
       <c r="I52" s="6" t="inlineStr">
         <is>
-          <t>물질 검사, 측정 및 분석기구 제조업</t>
+          <t>기타 화학제품 제조업</t>
         </is>
       </c>
       <c r="J52" s="6" t="inlineStr">
         <is>
-          <t>하나</t>
+          <t>한국</t>
         </is>
       </c>
       <c r="K52" s="6" t="inlineStr">
@@ -3354,12 +3354,12 @@
     <row r="53">
       <c r="A53" s="6" t="inlineStr">
         <is>
-          <t>2026-04-08</t>
+          <t>2025-09-11</t>
         </is>
       </c>
       <c r="B53" s="6" t="inlineStr">
         <is>
-          <t>옵토닉스</t>
+          <t>씨엠디엘</t>
         </is>
       </c>
       <c r="C53" s="6" t="inlineStr">
@@ -3369,37 +3369,37 @@
       </c>
       <c r="D53" s="6" t="inlineStr">
         <is>
-          <t>신규상장</t>
+          <t>스팩 소멸합병</t>
         </is>
       </c>
       <c r="E53" s="6" t="inlineStr">
         <is>
-          <t>FY25</t>
+          <t>FY24</t>
         </is>
       </c>
       <c r="F53" s="7" t="inlineStr">
         <is>
-          <t>25,368</t>
+          <t>39,991</t>
         </is>
       </c>
       <c r="G53" s="7" t="inlineStr">
         <is>
-          <t>1,901</t>
+          <t>3,541</t>
         </is>
       </c>
       <c r="H53" s="7" t="inlineStr">
         <is>
-          <t>730</t>
+          <t>503</t>
         </is>
       </c>
       <c r="I53" s="6" t="inlineStr">
         <is>
-          <t>광학렌즈 및 광학요소 제조업</t>
+          <t>기타 기초 유기 화학물질 제조업</t>
         </is>
       </c>
       <c r="J53" s="6" t="inlineStr">
         <is>
-          <t>한국</t>
+          <t>교보</t>
         </is>
       </c>
       <c r="K53" s="6" t="inlineStr">
@@ -3408,186 +3408,89 @@
         </is>
       </c>
     </row>
-    <row r="54">
-      <c r="A54" s="6" t="inlineStr">
-        <is>
-          <t>2026-04-07</t>
-        </is>
-      </c>
-      <c r="B54" s="6" t="inlineStr">
-        <is>
-          <t>크리에이츠</t>
-        </is>
-      </c>
-      <c r="C54" s="6" t="inlineStr">
-        <is>
-          <t>코스닥</t>
-        </is>
-      </c>
-      <c r="D54" s="6" t="inlineStr">
-        <is>
-          <t>신규상장</t>
-        </is>
-      </c>
-      <c r="E54" s="6" t="inlineStr">
-        <is>
-          <t>FY25</t>
-        </is>
-      </c>
-      <c r="F54" s="7" t="inlineStr">
-        <is>
-          <t>76,395</t>
-        </is>
-      </c>
-      <c r="G54" s="7" t="inlineStr">
-        <is>
-          <t>23,749</t>
-        </is>
-      </c>
-      <c r="H54" s="7" t="inlineStr">
-        <is>
-          <t>2,335</t>
-        </is>
-      </c>
-      <c r="I54" s="6" t="inlineStr">
-        <is>
-          <t>그외 기타 제품 제조업</t>
-        </is>
-      </c>
-      <c r="J54" s="6" t="inlineStr">
-        <is>
-          <t>삼성</t>
-        </is>
-      </c>
-      <c r="K54" s="6" t="inlineStr">
-        <is>
-          <t>예심 진행중</t>
-        </is>
-      </c>
-    </row>
     <row r="55">
-      <c r="A55" s="6" t="inlineStr">
-        <is>
-          <t>2026-03-24</t>
-        </is>
-      </c>
-      <c r="B55" s="6" t="inlineStr">
-        <is>
-          <t>인텔리빅스</t>
-        </is>
-      </c>
-      <c r="C55" s="6" t="inlineStr">
-        <is>
-          <t>코스닥</t>
-        </is>
-      </c>
-      <c r="D55" s="6" t="inlineStr">
-        <is>
-          <t>신규상장</t>
-        </is>
-      </c>
-      <c r="E55" s="6" t="inlineStr">
-        <is>
-          <t>FY25</t>
-        </is>
-      </c>
-      <c r="F55" s="7" t="inlineStr">
-        <is>
-          <t>46,644</t>
-        </is>
-      </c>
-      <c r="G55" s="7" t="inlineStr">
-        <is>
-          <t>5,357</t>
-        </is>
-      </c>
-      <c r="H55" s="7" t="inlineStr">
-        <is>
-          <t>1,048</t>
-        </is>
-      </c>
-      <c r="I55" s="6" t="inlineStr">
-        <is>
-          <t>소프트웨어 개발 및 공급업</t>
-        </is>
-      </c>
-      <c r="J55" s="6" t="inlineStr">
-        <is>
-          <t>미래</t>
-        </is>
-      </c>
-      <c r="K55" s="6" t="inlineStr">
-        <is>
-          <t>예심 진행중</t>
-        </is>
-      </c>
+      <c r="A55" s="3" t="inlineStr">
+        <is>
+          <t>■ 심사 승인  (44건)</t>
+        </is>
+      </c>
+      <c r="B55" s="4" t="n"/>
+      <c r="C55" s="4" t="n"/>
+      <c r="D55" s="4" t="n"/>
+      <c r="E55" s="4" t="n"/>
+      <c r="F55" s="4" t="n"/>
+      <c r="G55" s="4" t="n"/>
+      <c r="H55" s="4" t="n"/>
+      <c r="I55" s="4" t="n"/>
+      <c r="J55" s="4" t="n"/>
+      <c r="K55" s="4" t="n"/>
     </row>
     <row r="56">
-      <c r="A56" s="6" t="inlineStr">
-        <is>
-          <t>2026-02-27</t>
-        </is>
-      </c>
-      <c r="B56" s="6" t="inlineStr">
-        <is>
-          <t>피지티</t>
-        </is>
-      </c>
-      <c r="C56" s="6" t="inlineStr">
-        <is>
-          <t>코스닥</t>
-        </is>
-      </c>
-      <c r="D56" s="6" t="inlineStr">
-        <is>
-          <t>신규상장</t>
-        </is>
-      </c>
-      <c r="E56" s="6" t="inlineStr">
-        <is>
-          <t>FY25</t>
-        </is>
-      </c>
-      <c r="F56" s="7" t="inlineStr">
-        <is>
-          <t>40,141</t>
-        </is>
-      </c>
-      <c r="G56" s="7" t="inlineStr">
-        <is>
-          <t>-69,722</t>
-        </is>
-      </c>
-      <c r="H56" s="7" t="inlineStr">
-        <is>
-          <t>6,029</t>
-        </is>
-      </c>
-      <c r="I56" s="6" t="inlineStr">
-        <is>
-          <t>기타 화학제품 제조업</t>
-        </is>
-      </c>
-      <c r="J56" s="6" t="inlineStr">
-        <is>
-          <t>한국</t>
-        </is>
-      </c>
-      <c r="K56" s="6" t="inlineStr">
-        <is>
-          <t>예심 진행중</t>
+      <c r="A56" s="5" t="inlineStr">
+        <is>
+          <t>일자</t>
+        </is>
+      </c>
+      <c r="B56" s="5" t="inlineStr">
+        <is>
+          <t>회사명</t>
+        </is>
+      </c>
+      <c r="C56" s="5" t="inlineStr">
+        <is>
+          <t>시장</t>
+        </is>
+      </c>
+      <c r="D56" s="5" t="inlineStr">
+        <is>
+          <t>상장유형</t>
+        </is>
+      </c>
+      <c r="E56" s="5" t="inlineStr">
+        <is>
+          <t>기준연도</t>
+        </is>
+      </c>
+      <c r="F56" s="5" t="inlineStr">
+        <is>
+          <t>매출액</t>
+        </is>
+      </c>
+      <c r="G56" s="5" t="inlineStr">
+        <is>
+          <t>순이익</t>
+        </is>
+      </c>
+      <c r="H56" s="5" t="inlineStr">
+        <is>
+          <t>자기자본</t>
+        </is>
+      </c>
+      <c r="I56" s="5" t="inlineStr">
+        <is>
+          <t>업종</t>
+        </is>
+      </c>
+      <c r="J56" s="5" t="inlineStr">
+        <is>
+          <t>대표주관사</t>
+        </is>
+      </c>
+      <c r="K56" s="5" t="inlineStr">
+        <is>
+          <t>현황</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" s="6" t="inlineStr">
         <is>
-          <t>2025-09-11</t>
+          <t>2026-07-29</t>
         </is>
       </c>
       <c r="B57" s="6" t="inlineStr">
         <is>
-          <t>씨엠디엘</t>
+          <t>에스케이증권제14호기업인수목적</t>
         </is>
       </c>
       <c r="C57" s="6" t="inlineStr">
@@ -3597,116 +3500,213 @@
       </c>
       <c r="D57" s="6" t="inlineStr">
         <is>
-          <t>스팩 소멸합병</t>
+          <t>신규상장</t>
         </is>
       </c>
       <c r="E57" s="6" t="inlineStr">
         <is>
-          <t>FY24</t>
+          <t>FY25</t>
         </is>
       </c>
       <c r="F57" s="7" t="inlineStr">
         <is>
-          <t>39,991</t>
+          <t>-</t>
         </is>
       </c>
       <c r="G57" s="7" t="inlineStr">
         <is>
-          <t>3,541</t>
+          <t>-</t>
         </is>
       </c>
       <c r="H57" s="7" t="inlineStr">
         <is>
-          <t>503</t>
+          <t>17</t>
         </is>
       </c>
       <c r="I57" s="6" t="inlineStr">
         <is>
-          <t>기타 기초 유기 화학물질 제조업</t>
+          <t>기타 금융업</t>
         </is>
       </c>
       <c r="J57" s="6" t="inlineStr">
         <is>
-          <t>교보</t>
+          <t>SK</t>
         </is>
       </c>
       <c r="K57" s="6" t="inlineStr">
         <is>
-          <t>예심 진행중</t>
+          <t>상장전</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="6" t="inlineStr">
+        <is>
+          <t>2026-07-29</t>
+        </is>
+      </c>
+      <c r="B58" s="6" t="inlineStr">
+        <is>
+          <t>케이비제34호스팩</t>
+        </is>
+      </c>
+      <c r="C58" s="6" t="inlineStr">
+        <is>
+          <t>코스닥</t>
+        </is>
+      </c>
+      <c r="D58" s="6" t="inlineStr">
+        <is>
+          <t>신규상장</t>
+        </is>
+      </c>
+      <c r="E58" s="6" t="inlineStr">
+        <is>
+          <t>FY25</t>
+        </is>
+      </c>
+      <c r="F58" s="7" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G58" s="7" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H58" s="7" t="inlineStr">
+        <is>
+          <t>21</t>
+        </is>
+      </c>
+      <c r="I58" s="6" t="inlineStr">
+        <is>
+          <t>기타 금융업</t>
+        </is>
+      </c>
+      <c r="J58" s="6" t="inlineStr">
+        <is>
+          <t>KB</t>
+        </is>
+      </c>
+      <c r="K58" s="6" t="inlineStr">
+        <is>
+          <t>상장전</t>
         </is>
       </c>
     </row>
     <row r="59">
-      <c r="A59" s="3" t="inlineStr">
-        <is>
-          <t>■ 심사 승인  (40건)</t>
-        </is>
-      </c>
-      <c r="B59" s="4" t="n"/>
-      <c r="C59" s="4" t="n"/>
-      <c r="D59" s="4" t="n"/>
-      <c r="E59" s="4" t="n"/>
-      <c r="F59" s="4" t="n"/>
-      <c r="G59" s="4" t="n"/>
-      <c r="H59" s="4" t="n"/>
-      <c r="I59" s="4" t="n"/>
-      <c r="J59" s="4" t="n"/>
-      <c r="K59" s="4" t="n"/>
+      <c r="A59" s="6" t="inlineStr">
+        <is>
+          <t>2026-07-29</t>
+        </is>
+      </c>
+      <c r="B59" s="6" t="inlineStr">
+        <is>
+          <t>한국제17호스팩</t>
+        </is>
+      </c>
+      <c r="C59" s="6" t="inlineStr">
+        <is>
+          <t>코스닥</t>
+        </is>
+      </c>
+      <c r="D59" s="6" t="inlineStr">
+        <is>
+          <t>신규상장</t>
+        </is>
+      </c>
+      <c r="E59" s="6" t="inlineStr">
+        <is>
+          <t>FY25</t>
+        </is>
+      </c>
+      <c r="F59" s="7" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G59" s="7" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H59" s="7" t="inlineStr">
+        <is>
+          <t>170</t>
+        </is>
+      </c>
+      <c r="I59" s="6" t="inlineStr">
+        <is>
+          <t>기타 금융업</t>
+        </is>
+      </c>
+      <c r="J59" s="6" t="inlineStr">
+        <is>
+          <t>한국</t>
+        </is>
+      </c>
+      <c r="K59" s="6" t="inlineStr">
+        <is>
+          <t>상장전</t>
+        </is>
+      </c>
     </row>
     <row r="60">
-      <c r="A60" s="5" t="inlineStr">
-        <is>
-          <t>일자</t>
-        </is>
-      </c>
-      <c r="B60" s="5" t="inlineStr">
-        <is>
-          <t>회사명</t>
-        </is>
-      </c>
-      <c r="C60" s="5" t="inlineStr">
-        <is>
-          <t>시장</t>
-        </is>
-      </c>
-      <c r="D60" s="5" t="inlineStr">
-        <is>
-          <t>상장유형</t>
-        </is>
-      </c>
-      <c r="E60" s="5" t="inlineStr">
-        <is>
-          <t>기준연도</t>
-        </is>
-      </c>
-      <c r="F60" s="5" t="inlineStr">
-        <is>
-          <t>매출액</t>
-        </is>
-      </c>
-      <c r="G60" s="5" t="inlineStr">
-        <is>
-          <t>순이익</t>
-        </is>
-      </c>
-      <c r="H60" s="5" t="inlineStr">
-        <is>
-          <t>자기자본</t>
-        </is>
-      </c>
-      <c r="I60" s="5" t="inlineStr">
-        <is>
-          <t>업종</t>
-        </is>
-      </c>
-      <c r="J60" s="5" t="inlineStr">
-        <is>
-          <t>대표주관사</t>
-        </is>
-      </c>
-      <c r="K60" s="5" t="inlineStr">
-        <is>
-          <t>현황</t>
+      <c r="A60" s="6" t="inlineStr">
+        <is>
+          <t>2026-07-29</t>
+        </is>
+      </c>
+      <c r="B60" s="6" t="inlineStr">
+        <is>
+          <t>한화플러스제6호스팩</t>
+        </is>
+      </c>
+      <c r="C60" s="6" t="inlineStr">
+        <is>
+          <t>코스닥</t>
+        </is>
+      </c>
+      <c r="D60" s="6" t="inlineStr">
+        <is>
+          <t>신규상장</t>
+        </is>
+      </c>
+      <c r="E60" s="6" t="inlineStr">
+        <is>
+          <t>FY25</t>
+        </is>
+      </c>
+      <c r="F60" s="7" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G60" s="7" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H60" s="7" t="inlineStr">
+        <is>
+          <t>41</t>
+        </is>
+      </c>
+      <c r="I60" s="6" t="inlineStr">
+        <is>
+          <t>기타 금융업</t>
+        </is>
+      </c>
+      <c r="J60" s="6" t="inlineStr">
+        <is>
+          <t>한화</t>
+        </is>
+      </c>
+      <c r="K60" s="6" t="inlineStr">
+        <is>
+          <t>상장전</t>
         </is>
       </c>
     </row>
@@ -6859,7 +6859,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R60"/>
+  <dimension ref="A1:R64"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="1"/>
@@ -9657,7 +9657,7 @@
     <row r="40" ht="22" customHeight="1">
       <c r="A40" s="3" t="inlineStr">
         <is>
-          <t>■ 공모 진행 (예심 승인법인)  (16건)</t>
+          <t>■ 공모 진행 (예심 승인법인)  (20건)</t>
         </is>
       </c>
       <c r="B40" s="4" t="n"/>
@@ -10142,7 +10142,7 @@
       </c>
       <c r="B48" s="6" t="inlineStr">
         <is>
-          <t>08-03~08-07</t>
+          <t>08-14~08-21</t>
         </is>
       </c>
       <c r="C48" s="6" t="inlineStr">
@@ -10170,7 +10170,7 @@
       <c r="I48" s="6" t="inlineStr"/>
       <c r="J48" s="6" t="inlineStr">
         <is>
-          <t>08-13~08-14</t>
+          <t>08-26~08-27</t>
         </is>
       </c>
       <c r="K48" s="6" t="inlineStr"/>
@@ -10194,7 +10194,7 @@
       </c>
       <c r="R48" s="6" t="inlineStr">
         <is>
-          <t>최초</t>
+          <t>정정</t>
         </is>
       </c>
     </row>
@@ -10329,32 +10329,32 @@
     <row r="51" ht="30" customHeight="1">
       <c r="A51" s="6" t="inlineStr">
         <is>
-          <t>글로벌테크놀로지</t>
+          <t>와이즈플래닛컴퍼니</t>
         </is>
       </c>
       <c r="B51" s="6" t="inlineStr">
         <is>
-          <t>09-07~09-11</t>
+          <t>09-04~09-10</t>
         </is>
       </c>
       <c r="C51" s="6" t="inlineStr">
         <is>
-          <t>13,000~15,000</t>
+          <t>10,000~12,000</t>
         </is>
       </c>
       <c r="D51" s="7" t="inlineStr">
         <is>
-          <t>4,000,000</t>
+          <t>1,600,000</t>
         </is>
       </c>
       <c r="E51" s="7" t="inlineStr">
         <is>
-          <t>52,000,000,000</t>
+          <t>16,000,000,000</t>
         </is>
       </c>
       <c r="F51" s="6" t="inlineStr">
         <is>
-          <t>20.77배 (PER)</t>
+          <t>21.59배 (PER)</t>
         </is>
       </c>
       <c r="G51" s="6" t="inlineStr"/>
@@ -10362,7 +10362,7 @@
       <c r="I51" s="6" t="inlineStr"/>
       <c r="J51" s="6" t="inlineStr">
         <is>
-          <t>09-16~09-17</t>
+          <t>09-14~09-15</t>
         </is>
       </c>
       <c r="K51" s="6" t="inlineStr"/>
@@ -10370,18 +10370,18 @@
       <c r="M51" s="6" t="inlineStr"/>
       <c r="N51" s="6" t="inlineStr">
         <is>
-          <t>한국투자증권</t>
+          <t>대신증권</t>
         </is>
       </c>
       <c r="O51" s="6" t="inlineStr"/>
       <c r="P51" s="7" t="inlineStr">
         <is>
-          <t>2,119,999,960</t>
-        </is>
-      </c>
-      <c r="Q51" s="18" t="inlineStr">
-        <is>
-          <t>수집예정</t>
+          <t>494,400,000</t>
+        </is>
+      </c>
+      <c r="Q51" s="6" t="inlineStr">
+        <is>
+          <t>3.0%</t>
         </is>
       </c>
       <c r="R51" s="6" t="inlineStr">
@@ -10393,32 +10393,32 @@
     <row r="52" ht="30" customHeight="1">
       <c r="A52" s="6" t="inlineStr">
         <is>
-          <t>덕산넵코어스</t>
+          <t>글로벌테크놀로지</t>
         </is>
       </c>
       <c r="B52" s="6" t="inlineStr">
         <is>
-          <t>09-08~09-14</t>
+          <t>09-07~09-11</t>
         </is>
       </c>
       <c r="C52" s="6" t="inlineStr">
         <is>
-          <t>12,400~14,600</t>
+          <t>13,000~15,000</t>
         </is>
       </c>
       <c r="D52" s="7" t="inlineStr">
         <is>
-          <t>3,000,000</t>
+          <t>4,000,000</t>
         </is>
       </c>
       <c r="E52" s="7" t="inlineStr">
         <is>
-          <t>37,200,000,000</t>
+          <t>52,000,000,000</t>
         </is>
       </c>
       <c r="F52" s="6" t="inlineStr">
         <is>
-          <t>34.08배 (PER)</t>
+          <t>20.77배 (PER)</t>
         </is>
       </c>
       <c r="G52" s="6" t="inlineStr"/>
@@ -10434,18 +10434,18 @@
       <c r="M52" s="6" t="inlineStr"/>
       <c r="N52" s="6" t="inlineStr">
         <is>
-          <t>대신증권</t>
+          <t>한국투자증권</t>
         </is>
       </c>
       <c r="O52" s="6" t="inlineStr"/>
       <c r="P52" s="7" t="inlineStr">
         <is>
-          <t>1,413,399,926</t>
-        </is>
-      </c>
-      <c r="Q52" s="6" t="inlineStr">
-        <is>
-          <t>3.7%</t>
+          <t>2,119,999,960</t>
+        </is>
+      </c>
+      <c r="Q52" s="18" t="inlineStr">
+        <is>
+          <t>수집예정</t>
         </is>
       </c>
       <c r="R52" s="6" t="inlineStr">
@@ -10457,71 +10457,71 @@
     <row r="53" ht="30" customHeight="1">
       <c r="A53" s="6" t="inlineStr">
         <is>
-          <t>엔에이치스팩34호</t>
-        </is>
-      </c>
-      <c r="B53" s="18" t="inlineStr">
-        <is>
-          <t>수집예정</t>
-        </is>
-      </c>
-      <c r="C53" s="18" t="inlineStr">
-        <is>
-          <t>수집예정</t>
-        </is>
-      </c>
-      <c r="D53" s="18" t="inlineStr">
-        <is>
-          <t>수집예정</t>
-        </is>
-      </c>
-      <c r="E53" s="18" t="inlineStr">
-        <is>
-          <t>수집예정</t>
-        </is>
-      </c>
-      <c r="F53" s="18" t="inlineStr">
-        <is>
-          <t>수집예정</t>
+          <t>덕산넵코어스</t>
+        </is>
+      </c>
+      <c r="B53" s="6" t="inlineStr">
+        <is>
+          <t>09-08~09-14</t>
+        </is>
+      </c>
+      <c r="C53" s="6" t="inlineStr">
+        <is>
+          <t>12,400~14,600</t>
+        </is>
+      </c>
+      <c r="D53" s="7" t="inlineStr">
+        <is>
+          <t>3,000,000</t>
+        </is>
+      </c>
+      <c r="E53" s="7" t="inlineStr">
+        <is>
+          <t>37,200,000,000</t>
+        </is>
+      </c>
+      <c r="F53" s="6" t="inlineStr">
+        <is>
+          <t>34.08배 (PER)</t>
         </is>
       </c>
       <c r="G53" s="6" t="inlineStr"/>
       <c r="H53" s="6" t="inlineStr"/>
       <c r="I53" s="6" t="inlineStr"/>
-      <c r="J53" s="18" t="inlineStr">
-        <is>
-          <t>수집예정</t>
+      <c r="J53" s="6" t="inlineStr">
+        <is>
+          <t>09-16~09-17</t>
         </is>
       </c>
       <c r="K53" s="6" t="inlineStr"/>
       <c r="L53" s="6" t="inlineStr"/>
       <c r="M53" s="6" t="inlineStr"/>
-      <c r="N53" s="18" t="inlineStr">
-        <is>
-          <t>수집예정</t>
+      <c r="N53" s="6" t="inlineStr">
+        <is>
+          <t>대신증권</t>
         </is>
       </c>
       <c r="O53" s="6" t="inlineStr"/>
-      <c r="P53" s="18" t="inlineStr">
-        <is>
-          <t>수집예정</t>
-        </is>
-      </c>
-      <c r="Q53" s="18" t="inlineStr">
-        <is>
-          <t>수집예정</t>
+      <c r="P53" s="7" t="inlineStr">
+        <is>
+          <t>1,413,399,926</t>
+        </is>
+      </c>
+      <c r="Q53" s="6" t="inlineStr">
+        <is>
+          <t>3.7%</t>
         </is>
       </c>
       <c r="R53" s="6" t="inlineStr">
         <is>
-          <t>corp_code 미확보(수동확인)</t>
+          <t>최초</t>
         </is>
       </c>
     </row>
     <row r="54" ht="30" customHeight="1">
       <c r="A54" s="6" t="inlineStr">
         <is>
-          <t>와이즈플래닛컴퍼니</t>
+          <t>엔에이치스팩34호</t>
         </is>
       </c>
       <c r="B54" s="18" t="inlineStr">
@@ -10560,9 +10560,9 @@
       <c r="K54" s="6" t="inlineStr"/>
       <c r="L54" s="6" t="inlineStr"/>
       <c r="M54" s="6" t="inlineStr"/>
-      <c r="N54" s="6" t="inlineStr">
-        <is>
-          <t>대신</t>
+      <c r="N54" s="18" t="inlineStr">
+        <is>
+          <t>수집예정</t>
         </is>
       </c>
       <c r="O54" s="6" t="inlineStr"/>
@@ -10578,14 +10578,14 @@
       </c>
       <c r="R54" s="6" t="inlineStr">
         <is>
-          <t>신고서 대기</t>
+          <t>corp_code 미확보(수동확인)</t>
         </is>
       </c>
     </row>
     <row r="55" ht="30" customHeight="1">
       <c r="A55" s="6" t="inlineStr">
         <is>
-          <t>엠에스바이오</t>
+          <t>케이비제34호스팩</t>
         </is>
       </c>
       <c r="B55" s="18" t="inlineStr">
@@ -10642,14 +10642,14 @@
       </c>
       <c r="R55" s="6" t="inlineStr">
         <is>
-          <t>신고서 대기</t>
+          <t>corp_code 미확보(수동확인)</t>
         </is>
       </c>
     </row>
     <row r="56" ht="30" customHeight="1">
       <c r="A56" s="6" t="inlineStr">
         <is>
-          <t>디티에스</t>
+          <t>한국제17호스팩</t>
         </is>
       </c>
       <c r="B56" s="18" t="inlineStr">
@@ -10706,26 +10706,282 @@
       </c>
       <c r="R56" s="6" t="inlineStr">
         <is>
+          <t>corp_code 미확보(수동확인)</t>
+        </is>
+      </c>
+    </row>
+    <row r="57" ht="30" customHeight="1">
+      <c r="A57" s="6" t="inlineStr">
+        <is>
+          <t>한화플러스제6호스팩</t>
+        </is>
+      </c>
+      <c r="B57" s="18" t="inlineStr">
+        <is>
+          <t>수집예정</t>
+        </is>
+      </c>
+      <c r="C57" s="18" t="inlineStr">
+        <is>
+          <t>수집예정</t>
+        </is>
+      </c>
+      <c r="D57" s="18" t="inlineStr">
+        <is>
+          <t>수집예정</t>
+        </is>
+      </c>
+      <c r="E57" s="18" t="inlineStr">
+        <is>
+          <t>수집예정</t>
+        </is>
+      </c>
+      <c r="F57" s="18" t="inlineStr">
+        <is>
+          <t>수집예정</t>
+        </is>
+      </c>
+      <c r="G57" s="6" t="inlineStr"/>
+      <c r="H57" s="6" t="inlineStr"/>
+      <c r="I57" s="6" t="inlineStr"/>
+      <c r="J57" s="18" t="inlineStr">
+        <is>
+          <t>수집예정</t>
+        </is>
+      </c>
+      <c r="K57" s="6" t="inlineStr"/>
+      <c r="L57" s="6" t="inlineStr"/>
+      <c r="M57" s="6" t="inlineStr"/>
+      <c r="N57" s="18" t="inlineStr">
+        <is>
+          <t>수집예정</t>
+        </is>
+      </c>
+      <c r="O57" s="6" t="inlineStr"/>
+      <c r="P57" s="18" t="inlineStr">
+        <is>
+          <t>수집예정</t>
+        </is>
+      </c>
+      <c r="Q57" s="18" t="inlineStr">
+        <is>
+          <t>수집예정</t>
+        </is>
+      </c>
+      <c r="R57" s="6" t="inlineStr">
+        <is>
+          <t>corp_code 미확보(수동확인)</t>
+        </is>
+      </c>
+    </row>
+    <row r="58" ht="30" customHeight="1">
+      <c r="A58" s="6" t="inlineStr">
+        <is>
+          <t>엠에스바이오</t>
+        </is>
+      </c>
+      <c r="B58" s="18" t="inlineStr">
+        <is>
+          <t>수집예정</t>
+        </is>
+      </c>
+      <c r="C58" s="18" t="inlineStr">
+        <is>
+          <t>수집예정</t>
+        </is>
+      </c>
+      <c r="D58" s="18" t="inlineStr">
+        <is>
+          <t>수집예정</t>
+        </is>
+      </c>
+      <c r="E58" s="18" t="inlineStr">
+        <is>
+          <t>수집예정</t>
+        </is>
+      </c>
+      <c r="F58" s="18" t="inlineStr">
+        <is>
+          <t>수집예정</t>
+        </is>
+      </c>
+      <c r="G58" s="6" t="inlineStr"/>
+      <c r="H58" s="6" t="inlineStr"/>
+      <c r="I58" s="6" t="inlineStr"/>
+      <c r="J58" s="18" t="inlineStr">
+        <is>
+          <t>수집예정</t>
+        </is>
+      </c>
+      <c r="K58" s="6" t="inlineStr"/>
+      <c r="L58" s="6" t="inlineStr"/>
+      <c r="M58" s="6" t="inlineStr"/>
+      <c r="N58" s="18" t="inlineStr">
+        <is>
+          <t>수집예정</t>
+        </is>
+      </c>
+      <c r="O58" s="6" t="inlineStr"/>
+      <c r="P58" s="18" t="inlineStr">
+        <is>
+          <t>수집예정</t>
+        </is>
+      </c>
+      <c r="Q58" s="18" t="inlineStr">
+        <is>
+          <t>수집예정</t>
+        </is>
+      </c>
+      <c r="R58" s="6" t="inlineStr">
+        <is>
           <t>신고서 대기</t>
         </is>
       </c>
     </row>
-    <row r="58">
-      <c r="A58" s="20" t="inlineStr">
+    <row r="59" ht="30" customHeight="1">
+      <c r="A59" s="6" t="inlineStr">
+        <is>
+          <t>디티에스</t>
+        </is>
+      </c>
+      <c r="B59" s="18" t="inlineStr">
+        <is>
+          <t>수집예정</t>
+        </is>
+      </c>
+      <c r="C59" s="18" t="inlineStr">
+        <is>
+          <t>수집예정</t>
+        </is>
+      </c>
+      <c r="D59" s="18" t="inlineStr">
+        <is>
+          <t>수집예정</t>
+        </is>
+      </c>
+      <c r="E59" s="18" t="inlineStr">
+        <is>
+          <t>수집예정</t>
+        </is>
+      </c>
+      <c r="F59" s="18" t="inlineStr">
+        <is>
+          <t>수집예정</t>
+        </is>
+      </c>
+      <c r="G59" s="6" t="inlineStr"/>
+      <c r="H59" s="6" t="inlineStr"/>
+      <c r="I59" s="6" t="inlineStr"/>
+      <c r="J59" s="18" t="inlineStr">
+        <is>
+          <t>수집예정</t>
+        </is>
+      </c>
+      <c r="K59" s="6" t="inlineStr"/>
+      <c r="L59" s="6" t="inlineStr"/>
+      <c r="M59" s="6" t="inlineStr"/>
+      <c r="N59" s="18" t="inlineStr">
+        <is>
+          <t>수집예정</t>
+        </is>
+      </c>
+      <c r="O59" s="6" t="inlineStr"/>
+      <c r="P59" s="18" t="inlineStr">
+        <is>
+          <t>수집예정</t>
+        </is>
+      </c>
+      <c r="Q59" s="18" t="inlineStr">
+        <is>
+          <t>수집예정</t>
+        </is>
+      </c>
+      <c r="R59" s="6" t="inlineStr">
+        <is>
+          <t>신고서 대기</t>
+        </is>
+      </c>
+    </row>
+    <row r="60" ht="30" customHeight="1">
+      <c r="A60" s="6" t="inlineStr">
+        <is>
+          <t>에스케이증권제14호기업인수목적</t>
+        </is>
+      </c>
+      <c r="B60" s="18" t="inlineStr">
+        <is>
+          <t>수집예정</t>
+        </is>
+      </c>
+      <c r="C60" s="18" t="inlineStr">
+        <is>
+          <t>수집예정</t>
+        </is>
+      </c>
+      <c r="D60" s="18" t="inlineStr">
+        <is>
+          <t>수집예정</t>
+        </is>
+      </c>
+      <c r="E60" s="18" t="inlineStr">
+        <is>
+          <t>수집예정</t>
+        </is>
+      </c>
+      <c r="F60" s="18" t="inlineStr">
+        <is>
+          <t>수집예정</t>
+        </is>
+      </c>
+      <c r="G60" s="6" t="inlineStr"/>
+      <c r="H60" s="6" t="inlineStr"/>
+      <c r="I60" s="6" t="inlineStr"/>
+      <c r="J60" s="18" t="inlineStr">
+        <is>
+          <t>수집예정</t>
+        </is>
+      </c>
+      <c r="K60" s="6" t="inlineStr"/>
+      <c r="L60" s="6" t="inlineStr"/>
+      <c r="M60" s="6" t="inlineStr"/>
+      <c r="N60" s="18" t="inlineStr">
+        <is>
+          <t>수집예정</t>
+        </is>
+      </c>
+      <c r="O60" s="6" t="inlineStr"/>
+      <c r="P60" s="18" t="inlineStr">
+        <is>
+          <t>수집예정</t>
+        </is>
+      </c>
+      <c r="Q60" s="18" t="inlineStr">
+        <is>
+          <t>수집예정</t>
+        </is>
+      </c>
+      <c r="R60" s="6" t="inlineStr">
+        <is>
+          <t>신고서 대기</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" s="20" t="inlineStr">
         <is>
           <t>※ 상장 완료 = KIND 신규상장 페이지 기준(스팩합병 포함) · 스팩 공모상장은 밴드·밸류에이션 등 해당없음(공모가 2,000원 고정).</t>
         </is>
       </c>
     </row>
-    <row r="59">
-      <c r="A59" s="20" t="inlineStr">
+    <row r="63">
+      <c r="A63" s="20" t="inlineStr">
         <is>
           <t>※ 기재정정 신고서 내 정정 전·후 병존 → 자동수집은 "정정 후" 값만 취함.</t>
         </is>
       </c>
     </row>
-    <row r="60">
-      <c r="A60" s="20" t="inlineStr">
+    <row r="64">
+      <c r="A64" s="20" t="inlineStr">
         <is>
           <t>※ 청약경쟁률=일반투자자 청약수량÷최종배정수량 · "MM-DD~"는 종료일 자동수집 예정.</t>
         </is>
@@ -10959,7 +11215,7 @@
         <v>12</v>
       </c>
       <c r="C12" s="6" t="n">
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="D12" s="6" t="n">
         <v>1</v>
@@ -11062,11 +11318,11 @@
         </is>
       </c>
       <c r="B19" s="6" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C19" s="6" t="inlineStr">
         <is>
-          <t>64,800,000,000</t>
+          <t>80,800,000,000</t>
         </is>
       </c>
     </row>
@@ -11257,7 +11513,7 @@
         </is>
       </c>
       <c r="B32" s="6" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C32" s="6" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
chore: update IPO data 2026-07-30
</commit_message>
<xml_diff>
--- a/IPO_analysis.xlsx
+++ b/IPO_analysis.xlsx
@@ -618,14 +618,14 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>기준일 2026-07-29 · 청구일 직전 사업연도 · 별도/개별 재무제표 · 단위 백만원(별도 표기 시 USD)</t>
+          <t>기준일 2026-07-30 · 청구일 직전 사업연도 · 별도/개별 재무제표 · 단위 백만원(별도 표기 시 USD)</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
-          <t>■ 심사 신청(진행중)  (48건)</t>
+          <t>■ 심사 신청(진행중)  (47건)</t>
         </is>
       </c>
       <c r="B4" s="4" t="n"/>
@@ -699,12 +699,12 @@
     <row r="6">
       <c r="A6" s="6" t="inlineStr">
         <is>
-          <t>2026-07-27</t>
+          <t>2026-07-30</t>
         </is>
       </c>
       <c r="B6" s="6" t="inlineStr">
         <is>
-          <t>솔리스</t>
+          <t>데스틴파워</t>
         </is>
       </c>
       <c r="C6" s="6" t="inlineStr">
@@ -714,7 +714,7 @@
       </c>
       <c r="D6" s="6" t="inlineStr">
         <is>
-          <t>스팩 소멸합병</t>
+          <t>신규상장</t>
         </is>
       </c>
       <c r="E6" s="6" t="inlineStr">
@@ -722,17 +722,29 @@
           <t>FY25</t>
         </is>
       </c>
-      <c r="F6" s="7" t="inlineStr"/>
-      <c r="G6" s="7" t="inlineStr"/>
-      <c r="H6" s="7" t="inlineStr"/>
+      <c r="F6" s="7" t="inlineStr">
+        <is>
+          <t>29,851</t>
+        </is>
+      </c>
+      <c r="G6" s="7" t="inlineStr">
+        <is>
+          <t>5,852</t>
+        </is>
+      </c>
+      <c r="H6" s="7" t="inlineStr">
+        <is>
+          <t>-30,114</t>
+        </is>
+      </c>
       <c r="I6" s="6" t="inlineStr">
         <is>
-          <t>금융 지원 서비스업</t>
+          <t>전동기, 발전기 및 전기 변환 · 공급 · 제어 장치 제조업</t>
         </is>
       </c>
       <c r="J6" s="6" t="inlineStr">
         <is>
-          <t>한화</t>
+          <t>한국</t>
         </is>
       </c>
       <c r="K6" s="6" t="inlineStr">
@@ -744,12 +756,12 @@
     <row r="7">
       <c r="A7" s="6" t="inlineStr">
         <is>
-          <t>2026-07-27</t>
+          <t>2026-07-30</t>
         </is>
       </c>
       <c r="B7" s="6" t="inlineStr">
         <is>
-          <t>이노보테라퓨틱스</t>
+          <t>유림테크</t>
         </is>
       </c>
       <c r="C7" s="6" t="inlineStr">
@@ -769,27 +781,27 @@
       </c>
       <c r="F7" s="7" t="inlineStr">
         <is>
-          <t>209</t>
+          <t>102,586</t>
         </is>
       </c>
       <c r="G7" s="7" t="inlineStr">
         <is>
-          <t>-5,429</t>
+          <t>-18,278</t>
         </is>
       </c>
       <c r="H7" s="7" t="inlineStr">
         <is>
-          <t>-53,200</t>
+          <t>-4,832</t>
         </is>
       </c>
       <c r="I7" s="6" t="inlineStr">
         <is>
-          <t>의약품 제조업</t>
+          <t>자동차 신품 부품 제조업</t>
         </is>
       </c>
       <c r="J7" s="6" t="inlineStr">
         <is>
-          <t>한국</t>
+          <t>대신</t>
         </is>
       </c>
       <c r="K7" s="6" t="inlineStr">
@@ -801,22 +813,22 @@
     <row r="8">
       <c r="A8" s="6" t="inlineStr">
         <is>
-          <t>2026-07-24</t>
+          <t>2026-07-27</t>
         </is>
       </c>
       <c r="B8" s="6" t="inlineStr">
         <is>
-          <t>에스에프씨</t>
+          <t>솔리스</t>
         </is>
       </c>
       <c r="C8" s="6" t="inlineStr">
         <is>
-          <t>유가</t>
+          <t>코스닥</t>
         </is>
       </c>
       <c r="D8" s="6" t="inlineStr">
         <is>
-          <t>신규상장</t>
+          <t>스팩 소멸합병</t>
         </is>
       </c>
       <c r="E8" s="6" t="inlineStr">
@@ -824,29 +836,17 @@
           <t>FY25</t>
         </is>
       </c>
-      <c r="F8" s="7" t="inlineStr">
-        <is>
-          <t>160,792</t>
-        </is>
-      </c>
-      <c r="G8" s="7" t="inlineStr">
-        <is>
-          <t>25,509</t>
-        </is>
-      </c>
-      <c r="H8" s="7" t="inlineStr">
-        <is>
-          <t>243,562</t>
-        </is>
-      </c>
+      <c r="F8" s="7" t="inlineStr"/>
+      <c r="G8" s="7" t="inlineStr"/>
+      <c r="H8" s="7" t="inlineStr"/>
       <c r="I8" s="6" t="inlineStr">
         <is>
-          <t>기타 화학제품 제조업</t>
+          <t>금융 지원 서비스업</t>
         </is>
       </c>
       <c r="J8" s="6" t="inlineStr">
         <is>
-          <t>미래, 한국</t>
+          <t>한화</t>
         </is>
       </c>
       <c r="K8" s="6" t="inlineStr">
@@ -858,12 +858,12 @@
     <row r="9">
       <c r="A9" s="6" t="inlineStr">
         <is>
-          <t>2026-07-23</t>
+          <t>2026-07-27</t>
         </is>
       </c>
       <c r="B9" s="6" t="inlineStr">
         <is>
-          <t>제논</t>
+          <t>이노보테라퓨틱스</t>
         </is>
       </c>
       <c r="C9" s="6" t="inlineStr">
@@ -883,27 +883,27 @@
       </c>
       <c r="F9" s="7" t="inlineStr">
         <is>
-          <t>11,744</t>
+          <t>209</t>
         </is>
       </c>
       <c r="G9" s="7" t="inlineStr">
         <is>
-          <t>1,139</t>
+          <t>-5,429</t>
         </is>
       </c>
       <c r="H9" s="7" t="inlineStr">
         <is>
-          <t>-1,220</t>
+          <t>-53,200</t>
         </is>
       </c>
       <c r="I9" s="6" t="inlineStr">
         <is>
-          <t>소프트웨어 개발 및 공급업</t>
+          <t>의약품 제조업</t>
         </is>
       </c>
       <c r="J9" s="6" t="inlineStr">
         <is>
-          <t>삼성</t>
+          <t>한국</t>
         </is>
       </c>
       <c r="K9" s="6" t="inlineStr">
@@ -915,17 +915,17 @@
     <row r="10">
       <c r="A10" s="6" t="inlineStr">
         <is>
-          <t>2026-07-21</t>
+          <t>2026-07-24</t>
         </is>
       </c>
       <c r="B10" s="6" t="inlineStr">
         <is>
-          <t>넥스아이</t>
+          <t>에스에프씨</t>
         </is>
       </c>
       <c r="C10" s="6" t="inlineStr">
         <is>
-          <t>코스닥</t>
+          <t>유가</t>
         </is>
       </c>
       <c r="D10" s="6" t="inlineStr">
@@ -940,27 +940,27 @@
       </c>
       <c r="F10" s="7" t="inlineStr">
         <is>
-          <t>5,110</t>
+          <t>160,792</t>
         </is>
       </c>
       <c r="G10" s="7" t="inlineStr">
         <is>
-          <t>-52,331</t>
+          <t>25,509</t>
         </is>
       </c>
       <c r="H10" s="7" t="inlineStr">
         <is>
-          <t>-82,348</t>
+          <t>243,562</t>
         </is>
       </c>
       <c r="I10" s="6" t="inlineStr">
         <is>
-          <t>의약품 제조업</t>
+          <t>기타 화학제품 제조업</t>
         </is>
       </c>
       <c r="J10" s="6" t="inlineStr">
         <is>
-          <t>한국</t>
+          <t>미래, 한국</t>
         </is>
       </c>
       <c r="K10" s="6" t="inlineStr">
@@ -972,12 +972,12 @@
     <row r="11">
       <c r="A11" s="6" t="inlineStr">
         <is>
-          <t>2026-07-21</t>
+          <t>2026-07-23</t>
         </is>
       </c>
       <c r="B11" s="6" t="inlineStr">
         <is>
-          <t>아델</t>
+          <t>제논</t>
         </is>
       </c>
       <c r="C11" s="6" t="inlineStr">
@@ -997,27 +997,27 @@
       </c>
       <c r="F11" s="7" t="inlineStr">
         <is>
-          <t>62,057</t>
+          <t>11,744</t>
         </is>
       </c>
       <c r="G11" s="7" t="inlineStr">
         <is>
-          <t>-64,210</t>
+          <t>1,139</t>
         </is>
       </c>
       <c r="H11" s="7" t="inlineStr">
         <is>
-          <t>-80,776</t>
+          <t>-1,220</t>
         </is>
       </c>
       <c r="I11" s="6" t="inlineStr">
         <is>
-          <t>그외 기타 전문, 과학 및 기술 서비스업</t>
+          <t>소프트웨어 개발 및 공급업</t>
         </is>
       </c>
       <c r="J11" s="6" t="inlineStr">
         <is>
-          <t>삼성, 미래</t>
+          <t>삼성</t>
         </is>
       </c>
       <c r="K11" s="6" t="inlineStr">
@@ -1029,12 +1029,12 @@
     <row r="12">
       <c r="A12" s="6" t="inlineStr">
         <is>
-          <t>2026-07-13</t>
+          <t>2026-07-21</t>
         </is>
       </c>
       <c r="B12" s="6" t="inlineStr">
         <is>
-          <t>아이엠스팩1호</t>
+          <t>넥스아이</t>
         </is>
       </c>
       <c r="C12" s="6" t="inlineStr">
@@ -1052,17 +1052,29 @@
           <t>FY25</t>
         </is>
       </c>
-      <c r="F12" s="7" t="inlineStr"/>
-      <c r="G12" s="7" t="inlineStr"/>
-      <c r="H12" s="7" t="inlineStr"/>
+      <c r="F12" s="7" t="inlineStr">
+        <is>
+          <t>5,110</t>
+        </is>
+      </c>
+      <c r="G12" s="7" t="inlineStr">
+        <is>
+          <t>-52,331</t>
+        </is>
+      </c>
+      <c r="H12" s="7" t="inlineStr">
+        <is>
+          <t>-82,348</t>
+        </is>
+      </c>
       <c r="I12" s="6" t="inlineStr">
         <is>
-          <t>금융 지원 서비스업</t>
+          <t>의약품 제조업</t>
         </is>
       </c>
       <c r="J12" s="6" t="inlineStr">
         <is>
-          <t>iM증권</t>
+          <t>한국</t>
         </is>
       </c>
       <c r="K12" s="6" t="inlineStr">
@@ -1074,12 +1086,12 @@
     <row r="13">
       <c r="A13" s="6" t="inlineStr">
         <is>
-          <t>2026-07-13</t>
+          <t>2026-07-21</t>
         </is>
       </c>
       <c r="B13" s="6" t="inlineStr">
         <is>
-          <t>에버온</t>
+          <t>아델</t>
         </is>
       </c>
       <c r="C13" s="6" t="inlineStr">
@@ -1099,27 +1111,27 @@
       </c>
       <c r="F13" s="7" t="inlineStr">
         <is>
-          <t>65,225</t>
+          <t>62,057</t>
         </is>
       </c>
       <c r="G13" s="7" t="inlineStr">
         <is>
-          <t>-3,606</t>
+          <t>-64,210</t>
         </is>
       </c>
       <c r="H13" s="7" t="inlineStr">
         <is>
-          <t>54,955</t>
+          <t>-80,776</t>
         </is>
       </c>
       <c r="I13" s="6" t="inlineStr">
         <is>
-          <t>전기업</t>
+          <t>그외 기타 전문, 과학 및 기술 서비스업</t>
         </is>
       </c>
       <c r="J13" s="6" t="inlineStr">
         <is>
-          <t>미래</t>
+          <t>삼성, 미래</t>
         </is>
       </c>
       <c r="K13" s="6" t="inlineStr">
@@ -1131,12 +1143,12 @@
     <row r="14">
       <c r="A14" s="6" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
+          <t>2026-07-13</t>
         </is>
       </c>
       <c r="B14" s="6" t="inlineStr">
         <is>
-          <t>엔키화이트햇</t>
+          <t>아이엠스팩1호</t>
         </is>
       </c>
       <c r="C14" s="6" t="inlineStr">
@@ -1154,29 +1166,17 @@
           <t>FY25</t>
         </is>
       </c>
-      <c r="F14" s="7" t="inlineStr">
-        <is>
-          <t>14,176</t>
-        </is>
-      </c>
-      <c r="G14" s="7" t="inlineStr">
-        <is>
-          <t>-3,211</t>
-        </is>
-      </c>
-      <c r="H14" s="7" t="inlineStr">
-        <is>
-          <t>8,338</t>
-        </is>
-      </c>
+      <c r="F14" s="7" t="inlineStr"/>
+      <c r="G14" s="7" t="inlineStr"/>
+      <c r="H14" s="7" t="inlineStr"/>
       <c r="I14" s="6" t="inlineStr">
         <is>
-          <t>소프트웨어 개발 및 공급업</t>
+          <t>금융 지원 서비스업</t>
         </is>
       </c>
       <c r="J14" s="6" t="inlineStr">
         <is>
-          <t>신영</t>
+          <t>iM증권</t>
         </is>
       </c>
       <c r="K14" s="6" t="inlineStr">
@@ -1188,12 +1188,12 @@
     <row r="15">
       <c r="A15" s="6" t="inlineStr">
         <is>
-          <t>2026-07-09</t>
+          <t>2026-07-13</t>
         </is>
       </c>
       <c r="B15" s="6" t="inlineStr">
         <is>
-          <t>씨아이에스케미칼</t>
+          <t>에버온</t>
         </is>
       </c>
       <c r="C15" s="6" t="inlineStr">
@@ -1213,27 +1213,27 @@
       </c>
       <c r="F15" s="7" t="inlineStr">
         <is>
-          <t>15,985</t>
+          <t>65,225</t>
         </is>
       </c>
       <c r="G15" s="7" t="inlineStr">
         <is>
-          <t>-11,440</t>
+          <t>-3,606</t>
         </is>
       </c>
       <c r="H15" s="7" t="inlineStr">
         <is>
-          <t>23,706</t>
+          <t>54,955</t>
         </is>
       </c>
       <c r="I15" s="6" t="inlineStr">
         <is>
-          <t>기초 화학물질 제조업</t>
+          <t>전기업</t>
         </is>
       </c>
       <c r="J15" s="6" t="inlineStr">
         <is>
-          <t>KB</t>
+          <t>미래</t>
         </is>
       </c>
       <c r="K15" s="6" t="inlineStr">
@@ -1245,12 +1245,12 @@
     <row r="16">
       <c r="A16" s="6" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-07-10</t>
         </is>
       </c>
       <c r="B16" s="6" t="inlineStr">
         <is>
-          <t>진코스텍</t>
+          <t>엔키화이트햇</t>
         </is>
       </c>
       <c r="C16" s="6" t="inlineStr">
@@ -1260,7 +1260,7 @@
       </c>
       <c r="D16" s="6" t="inlineStr">
         <is>
-          <t>이전상장</t>
+          <t>신규상장</t>
         </is>
       </c>
       <c r="E16" s="6" t="inlineStr">
@@ -1270,27 +1270,27 @@
       </c>
       <c r="F16" s="7" t="inlineStr">
         <is>
-          <t>48,646</t>
+          <t>14,176</t>
         </is>
       </c>
       <c r="G16" s="7" t="inlineStr">
         <is>
-          <t>6,017</t>
+          <t>-3,211</t>
         </is>
       </c>
       <c r="H16" s="7" t="inlineStr">
         <is>
-          <t>18,795</t>
+          <t>8,338</t>
         </is>
       </c>
       <c r="I16" s="6" t="inlineStr">
         <is>
-          <t>기타 화학제품 제조업</t>
+          <t>소프트웨어 개발 및 공급업</t>
         </is>
       </c>
       <c r="J16" s="6" t="inlineStr">
         <is>
-          <t>하나</t>
+          <t>신영</t>
         </is>
       </c>
       <c r="K16" s="6" t="inlineStr">
@@ -1302,12 +1302,12 @@
     <row r="17">
       <c r="A17" s="6" t="inlineStr">
         <is>
-          <t>2026-07-03</t>
+          <t>2026-07-09</t>
         </is>
       </c>
       <c r="B17" s="6" t="inlineStr">
         <is>
-          <t>엠디에스코리아</t>
+          <t>씨아이에스케미칼</t>
         </is>
       </c>
       <c r="C17" s="6" t="inlineStr">
@@ -1327,27 +1327,27 @@
       </c>
       <c r="F17" s="7" t="inlineStr">
         <is>
-          <t>97,972</t>
+          <t>15,985</t>
         </is>
       </c>
       <c r="G17" s="7" t="inlineStr">
         <is>
-          <t>6,512</t>
+          <t>-11,440</t>
         </is>
       </c>
       <c r="H17" s="7" t="inlineStr">
         <is>
-          <t>53,818</t>
+          <t>23,706</t>
         </is>
       </c>
       <c r="I17" s="6" t="inlineStr">
         <is>
-          <t>기타 식품 제조업</t>
+          <t>기초 화학물질 제조업</t>
         </is>
       </c>
       <c r="J17" s="6" t="inlineStr">
         <is>
-          <t>미래</t>
+          <t>KB</t>
         </is>
       </c>
       <c r="K17" s="6" t="inlineStr">
@@ -1359,12 +1359,12 @@
     <row r="18">
       <c r="A18" s="6" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="B18" s="6" t="inlineStr">
         <is>
-          <t>동승</t>
+          <t>진코스텍</t>
         </is>
       </c>
       <c r="C18" s="6" t="inlineStr">
@@ -1374,7 +1374,7 @@
       </c>
       <c r="D18" s="6" t="inlineStr">
         <is>
-          <t>신규상장</t>
+          <t>이전상장</t>
         </is>
       </c>
       <c r="E18" s="6" t="inlineStr">
@@ -1384,27 +1384,27 @@
       </c>
       <c r="F18" s="7" t="inlineStr">
         <is>
-          <t>78,625</t>
+          <t>48,646</t>
         </is>
       </c>
       <c r="G18" s="7" t="inlineStr">
         <is>
-          <t>14,525</t>
+          <t>6,017</t>
         </is>
       </c>
       <c r="H18" s="7" t="inlineStr">
         <is>
-          <t>5,438</t>
+          <t>18,795</t>
         </is>
       </c>
       <c r="I18" s="6" t="inlineStr">
         <is>
-          <t>부동산 임대 및 공급업</t>
+          <t>기타 화학제품 제조업</t>
         </is>
       </c>
       <c r="J18" s="6" t="inlineStr">
         <is>
-          <t>NH</t>
+          <t>하나</t>
         </is>
       </c>
       <c r="K18" s="6" t="inlineStr">
@@ -1416,12 +1416,12 @@
     <row r="19">
       <c r="A19" s="6" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-07-03</t>
         </is>
       </c>
       <c r="B19" s="6" t="inlineStr">
         <is>
-          <t>셀트릭스</t>
+          <t>엠디에스코리아</t>
         </is>
       </c>
       <c r="C19" s="6" t="inlineStr">
@@ -1431,7 +1431,7 @@
       </c>
       <c r="D19" s="6" t="inlineStr">
         <is>
-          <t>스팩 소멸합병</t>
+          <t>신규상장</t>
         </is>
       </c>
       <c r="E19" s="6" t="inlineStr">
@@ -1441,27 +1441,27 @@
       </c>
       <c r="F19" s="7" t="inlineStr">
         <is>
-          <t>16,976</t>
+          <t>97,972</t>
         </is>
       </c>
       <c r="G19" s="7" t="inlineStr">
         <is>
-          <t>4,545</t>
+          <t>6,512</t>
         </is>
       </c>
       <c r="H19" s="7" t="inlineStr">
         <is>
-          <t>2,213</t>
+          <t>53,818</t>
         </is>
       </c>
       <c r="I19" s="6" t="inlineStr">
         <is>
-          <t>의료용품 및 기타 의약 관련제품 제조업</t>
+          <t>기타 식품 제조업</t>
         </is>
       </c>
       <c r="J19" s="6" t="inlineStr">
         <is>
-          <t>IBK</t>
+          <t>미래</t>
         </is>
       </c>
       <c r="K19" s="6" t="inlineStr">
@@ -1478,7 +1478,7 @@
       </c>
       <c r="B20" s="6" t="inlineStr">
         <is>
-          <t>에프엠더블유</t>
+          <t>동승</t>
         </is>
       </c>
       <c r="C20" s="6" t="inlineStr">
@@ -1488,7 +1488,7 @@
       </c>
       <c r="D20" s="6" t="inlineStr">
         <is>
-          <t>스팩 소멸합병</t>
+          <t>신규상장</t>
         </is>
       </c>
       <c r="E20" s="6" t="inlineStr">
@@ -1498,27 +1498,27 @@
       </c>
       <c r="F20" s="7" t="inlineStr">
         <is>
-          <t>30,282</t>
+          <t>78,625</t>
         </is>
       </c>
       <c r="G20" s="7" t="inlineStr">
         <is>
-          <t>4,762</t>
+          <t>14,525</t>
         </is>
       </c>
       <c r="H20" s="7" t="inlineStr">
         <is>
-          <t>32</t>
+          <t>5,438</t>
         </is>
       </c>
       <c r="I20" s="6" t="inlineStr">
         <is>
-          <t>기타 식품 제조업</t>
+          <t>부동산 임대 및 공급업</t>
         </is>
       </c>
       <c r="J20" s="6" t="inlineStr">
         <is>
-          <t>유진</t>
+          <t>NH</t>
         </is>
       </c>
       <c r="K20" s="6" t="inlineStr">
@@ -1530,22 +1530,22 @@
     <row r="21">
       <c r="A21" s="6" t="inlineStr">
         <is>
-          <t>2026-06-26</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="B21" s="6" t="inlineStr">
         <is>
-          <t>소노인터내셔널</t>
+          <t>셀트릭스</t>
         </is>
       </c>
       <c r="C21" s="6" t="inlineStr">
         <is>
-          <t>유가</t>
+          <t>코스닥</t>
         </is>
       </c>
       <c r="D21" s="6" t="inlineStr">
         <is>
-          <t>신규상장</t>
+          <t>스팩 소멸합병</t>
         </is>
       </c>
       <c r="E21" s="6" t="inlineStr">
@@ -1555,27 +1555,27 @@
       </c>
       <c r="F21" s="7" t="inlineStr">
         <is>
-          <t>2,093,051</t>
+          <t>16,976</t>
         </is>
       </c>
       <c r="G21" s="7" t="inlineStr">
         <is>
-          <t>-148,064</t>
+          <t>4,545</t>
         </is>
       </c>
       <c r="H21" s="7" t="inlineStr">
         <is>
-          <t>852,372</t>
+          <t>2,213</t>
         </is>
       </c>
       <c r="I21" s="6" t="inlineStr">
         <is>
-          <t>일반 및 생활 숙박시설 운영업</t>
+          <t>의료용품 및 기타 의약 관련제품 제조업</t>
         </is>
       </c>
       <c r="J21" s="6" t="inlineStr">
         <is>
-          <t>대신, 미래</t>
+          <t>IBK</t>
         </is>
       </c>
       <c r="K21" s="6" t="inlineStr">
@@ -1587,12 +1587,12 @@
     <row r="22">
       <c r="A22" s="6" t="inlineStr">
         <is>
-          <t>2026-06-25</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="B22" s="6" t="inlineStr">
         <is>
-          <t>싸이몬</t>
+          <t>에프엠더블유</t>
         </is>
       </c>
       <c r="C22" s="6" t="inlineStr">
@@ -1602,7 +1602,7 @@
       </c>
       <c r="D22" s="6" t="inlineStr">
         <is>
-          <t>신규상장</t>
+          <t>스팩 소멸합병</t>
         </is>
       </c>
       <c r="E22" s="6" t="inlineStr">
@@ -1612,27 +1612,27 @@
       </c>
       <c r="F22" s="7" t="inlineStr">
         <is>
-          <t>48,695</t>
+          <t>30,282</t>
         </is>
       </c>
       <c r="G22" s="7" t="inlineStr">
         <is>
-          <t>15,714</t>
+          <t>4,762</t>
         </is>
       </c>
       <c r="H22" s="7" t="inlineStr">
         <is>
-          <t>61,761</t>
+          <t>32</t>
         </is>
       </c>
       <c r="I22" s="6" t="inlineStr">
         <is>
-          <t>측정, 시험, 항해, 제어 및 기타 정밀기기 제조업</t>
+          <t>기타 식품 제조업</t>
         </is>
       </c>
       <c r="J22" s="6" t="inlineStr">
         <is>
-          <t>미래</t>
+          <t>유진</t>
         </is>
       </c>
       <c r="K22" s="6" t="inlineStr">
@@ -1644,17 +1644,17 @@
     <row r="23">
       <c r="A23" s="6" t="inlineStr">
         <is>
-          <t>2026-06-23</t>
+          <t>2026-06-26</t>
         </is>
       </c>
       <c r="B23" s="6" t="inlineStr">
         <is>
-          <t>바이다</t>
+          <t>소노인터내셔널</t>
         </is>
       </c>
       <c r="C23" s="6" t="inlineStr">
         <is>
-          <t>코스닥</t>
+          <t>유가</t>
         </is>
       </c>
       <c r="D23" s="6" t="inlineStr">
@@ -1669,27 +1669,27 @@
       </c>
       <c r="F23" s="7" t="inlineStr">
         <is>
-          <t>14,432</t>
+          <t>2,093,051</t>
         </is>
       </c>
       <c r="G23" s="7" t="inlineStr">
         <is>
-          <t>-3,951</t>
+          <t>-148,064</t>
         </is>
       </c>
       <c r="H23" s="7" t="inlineStr">
         <is>
-          <t>15,108</t>
+          <t>852,372</t>
         </is>
       </c>
       <c r="I23" s="6" t="inlineStr">
         <is>
-          <t>전자부품 제조업</t>
+          <t>일반 및 생활 숙박시설 운영업</t>
         </is>
       </c>
       <c r="J23" s="6" t="inlineStr">
         <is>
-          <t>NH</t>
+          <t>대신, 미래</t>
         </is>
       </c>
       <c r="K23" s="6" t="inlineStr">
@@ -1701,12 +1701,12 @@
     <row r="24">
       <c r="A24" s="6" t="inlineStr">
         <is>
-          <t>2026-06-19</t>
+          <t>2026-06-25</t>
         </is>
       </c>
       <c r="B24" s="6" t="inlineStr">
         <is>
-          <t>럭스코</t>
+          <t>싸이몬</t>
         </is>
       </c>
       <c r="C24" s="6" t="inlineStr">
@@ -1716,7 +1716,7 @@
       </c>
       <c r="D24" s="6" t="inlineStr">
         <is>
-          <t>스팩 소멸합병</t>
+          <t>신규상장</t>
         </is>
       </c>
       <c r="E24" s="6" t="inlineStr">
@@ -1726,27 +1726,27 @@
       </c>
       <c r="F24" s="7" t="inlineStr">
         <is>
-          <t>67,976</t>
+          <t>48,695</t>
         </is>
       </c>
       <c r="G24" s="7" t="inlineStr">
         <is>
-          <t>6,893</t>
+          <t>15,714</t>
         </is>
       </c>
       <c r="H24" s="7" t="inlineStr">
         <is>
-          <t>1,000</t>
+          <t>61,761</t>
         </is>
       </c>
       <c r="I24" s="6" t="inlineStr">
         <is>
-          <t>전동기, 발전기 및 전기 변환 · 공급 · 제어 장치 제조업</t>
+          <t>측정, 시험, 항해, 제어 및 기타 정밀기기 제조업</t>
         </is>
       </c>
       <c r="J24" s="6" t="inlineStr">
         <is>
-          <t>IBK</t>
+          <t>미래</t>
         </is>
       </c>
       <c r="K24" s="6" t="inlineStr">
@@ -1758,12 +1758,12 @@
     <row r="25">
       <c r="A25" s="6" t="inlineStr">
         <is>
-          <t>2026-06-19</t>
+          <t>2026-06-23</t>
         </is>
       </c>
       <c r="B25" s="6" t="inlineStr">
         <is>
-          <t>아이알큐더스</t>
+          <t>바이다</t>
         </is>
       </c>
       <c r="C25" s="6" t="inlineStr">
@@ -1783,27 +1783,27 @@
       </c>
       <c r="F25" s="7" t="inlineStr">
         <is>
-          <t>10,231</t>
+          <t>14,432</t>
         </is>
       </c>
       <c r="G25" s="7" t="inlineStr">
         <is>
-          <t>-986</t>
+          <t>-3,951</t>
         </is>
       </c>
       <c r="H25" s="7" t="inlineStr">
         <is>
-          <t>1,800</t>
+          <t>15,108</t>
         </is>
       </c>
       <c r="I25" s="6" t="inlineStr">
         <is>
-          <t>소프트웨어 개발 및 공급업</t>
+          <t>전자부품 제조업</t>
         </is>
       </c>
       <c r="J25" s="6" t="inlineStr">
         <is>
-          <t>DB</t>
+          <t>NH</t>
         </is>
       </c>
       <c r="K25" s="6" t="inlineStr">
@@ -1820,7 +1820,7 @@
       </c>
       <c r="B26" s="6" t="inlineStr">
         <is>
-          <t>이에스티</t>
+          <t>럭스코</t>
         </is>
       </c>
       <c r="C26" s="6" t="inlineStr">
@@ -1830,7 +1830,7 @@
       </c>
       <c r="D26" s="6" t="inlineStr">
         <is>
-          <t>신규상장</t>
+          <t>스팩 소멸합병</t>
         </is>
       </c>
       <c r="E26" s="6" t="inlineStr">
@@ -1840,27 +1840,27 @@
       </c>
       <c r="F26" s="7" t="inlineStr">
         <is>
-          <t>33,190</t>
+          <t>67,976</t>
         </is>
       </c>
       <c r="G26" s="7" t="inlineStr">
         <is>
-          <t>2,966</t>
+          <t>6,893</t>
         </is>
       </c>
       <c r="H26" s="7" t="inlineStr">
         <is>
-          <t>4,325</t>
+          <t>1,000</t>
         </is>
       </c>
       <c r="I26" s="6" t="inlineStr">
         <is>
-          <t>특수 목적용 기계 제조업</t>
+          <t>전동기, 발전기 및 전기 변환 · 공급 · 제어 장치 제조업</t>
         </is>
       </c>
       <c r="J26" s="6" t="inlineStr">
         <is>
-          <t>대신</t>
+          <t>IBK</t>
         </is>
       </c>
       <c r="K26" s="6" t="inlineStr">
@@ -1872,12 +1872,12 @@
     <row r="27">
       <c r="A27" s="6" t="inlineStr">
         <is>
-          <t>2026-06-18</t>
+          <t>2026-06-19</t>
         </is>
       </c>
       <c r="B27" s="6" t="inlineStr">
         <is>
-          <t>영광</t>
+          <t>아이알큐더스</t>
         </is>
       </c>
       <c r="C27" s="6" t="inlineStr">
@@ -1897,27 +1897,27 @@
       </c>
       <c r="F27" s="7" t="inlineStr">
         <is>
-          <t>113,133</t>
+          <t>10,231</t>
         </is>
       </c>
       <c r="G27" s="7" t="inlineStr">
         <is>
-          <t>10,328</t>
+          <t>-986</t>
         </is>
       </c>
       <c r="H27" s="7" t="inlineStr">
         <is>
-          <t>3,052</t>
+          <t>1,800</t>
         </is>
       </c>
       <c r="I27" s="6" t="inlineStr">
         <is>
-          <t>구조용 금속제품, 탱크 및 증기발생기 제조업</t>
+          <t>소프트웨어 개발 및 공급업</t>
         </is>
       </c>
       <c r="J27" s="6" t="inlineStr">
         <is>
-          <t>한국</t>
+          <t>DB</t>
         </is>
       </c>
       <c r="K27" s="6" t="inlineStr">
@@ -1929,12 +1929,12 @@
     <row r="28">
       <c r="A28" s="6" t="inlineStr">
         <is>
-          <t>2026-06-17</t>
+          <t>2026-06-19</t>
         </is>
       </c>
       <c r="B28" s="6" t="inlineStr">
         <is>
-          <t>티앤이코리아</t>
+          <t>이에스티</t>
         </is>
       </c>
       <c r="C28" s="6" t="inlineStr">
@@ -1954,27 +1954,27 @@
       </c>
       <c r="F28" s="7" t="inlineStr">
         <is>
-          <t>22,339</t>
+          <t>33,190</t>
         </is>
       </c>
       <c r="G28" s="7" t="inlineStr">
         <is>
-          <t>-7,091</t>
+          <t>2,966</t>
         </is>
       </c>
       <c r="H28" s="7" t="inlineStr">
         <is>
-          <t>481</t>
+          <t>4,325</t>
         </is>
       </c>
       <c r="I28" s="6" t="inlineStr">
         <is>
-          <t>일반 목적용 기계 제조업</t>
+          <t>특수 목적용 기계 제조업</t>
         </is>
       </c>
       <c r="J28" s="6" t="inlineStr">
         <is>
-          <t>신한</t>
+          <t>대신</t>
         </is>
       </c>
       <c r="K28" s="6" t="inlineStr">
@@ -1986,12 +1986,12 @@
     <row r="29">
       <c r="A29" s="6" t="inlineStr">
         <is>
-          <t>2026-06-11</t>
+          <t>2026-06-18</t>
         </is>
       </c>
       <c r="B29" s="6" t="inlineStr">
         <is>
-          <t>씨엔티테크</t>
+          <t>영광</t>
         </is>
       </c>
       <c r="C29" s="6" t="inlineStr">
@@ -2011,27 +2011,27 @@
       </c>
       <c r="F29" s="7" t="inlineStr">
         <is>
-          <t>27,015</t>
+          <t>113,133</t>
         </is>
       </c>
       <c r="G29" s="7" t="inlineStr">
         <is>
-          <t>3,987</t>
+          <t>10,328</t>
         </is>
       </c>
       <c r="H29" s="7" t="inlineStr">
         <is>
-          <t>2,613</t>
+          <t>3,052</t>
         </is>
       </c>
       <c r="I29" s="6" t="inlineStr">
         <is>
-          <t>소프트웨어 개발 및 공급업</t>
+          <t>구조용 금속제품, 탱크 및 증기발생기 제조업</t>
         </is>
       </c>
       <c r="J29" s="6" t="inlineStr">
         <is>
-          <t>한화, 하나</t>
+          <t>한국</t>
         </is>
       </c>
       <c r="K29" s="6" t="inlineStr">
@@ -2043,12 +2043,12 @@
     <row r="30">
       <c r="A30" s="6" t="inlineStr">
         <is>
-          <t>2026-06-11</t>
+          <t>2026-06-17</t>
         </is>
       </c>
       <c r="B30" s="6" t="inlineStr">
         <is>
-          <t>제이앤티지</t>
+          <t>티앤이코리아</t>
         </is>
       </c>
       <c r="C30" s="6" t="inlineStr">
@@ -2068,27 +2068,27 @@
       </c>
       <c r="F30" s="7" t="inlineStr">
         <is>
-          <t>72,378</t>
+          <t>22,339</t>
         </is>
       </c>
       <c r="G30" s="7" t="inlineStr">
         <is>
-          <t>9,904</t>
+          <t>-7,091</t>
         </is>
       </c>
       <c r="H30" s="7" t="inlineStr">
         <is>
-          <t>6,743</t>
+          <t>481</t>
         </is>
       </c>
       <c r="I30" s="6" t="inlineStr">
         <is>
-          <t>전자부품 제조업</t>
+          <t>일반 목적용 기계 제조업</t>
         </is>
       </c>
       <c r="J30" s="6" t="inlineStr">
         <is>
-          <t>대신, NH</t>
+          <t>신한</t>
         </is>
       </c>
       <c r="K30" s="6" t="inlineStr">
@@ -2100,12 +2100,12 @@
     <row r="31">
       <c r="A31" s="6" t="inlineStr">
         <is>
-          <t>2026-05-29</t>
+          <t>2026-06-11</t>
         </is>
       </c>
       <c r="B31" s="6" t="inlineStr">
         <is>
-          <t>유캐스트</t>
+          <t>씨엔티테크</t>
         </is>
       </c>
       <c r="C31" s="6" t="inlineStr">
@@ -2125,27 +2125,27 @@
       </c>
       <c r="F31" s="7" t="inlineStr">
         <is>
-          <t>5,934</t>
+          <t>27,015</t>
         </is>
       </c>
       <c r="G31" s="7" t="inlineStr">
         <is>
-          <t>-3,557</t>
+          <t>3,987</t>
         </is>
       </c>
       <c r="H31" s="7" t="inlineStr">
         <is>
-          <t>1,881</t>
+          <t>2,613</t>
         </is>
       </c>
       <c r="I31" s="6" t="inlineStr">
         <is>
-          <t>통신 및 방송 장비 제조업</t>
+          <t>소프트웨어 개발 및 공급업</t>
         </is>
       </c>
       <c r="J31" s="6" t="inlineStr">
         <is>
-          <t>유진</t>
+          <t>한화, 하나</t>
         </is>
       </c>
       <c r="K31" s="6" t="inlineStr">
@@ -2157,12 +2157,12 @@
     <row r="32">
       <c r="A32" s="6" t="inlineStr">
         <is>
-          <t>2026-05-29</t>
+          <t>2026-06-11</t>
         </is>
       </c>
       <c r="B32" s="6" t="inlineStr">
         <is>
-          <t>인터엑스</t>
+          <t>제이앤티지</t>
         </is>
       </c>
       <c r="C32" s="6" t="inlineStr">
@@ -2182,27 +2182,27 @@
       </c>
       <c r="F32" s="7" t="inlineStr">
         <is>
-          <t>8,645</t>
+          <t>72,378</t>
         </is>
       </c>
       <c r="G32" s="7" t="inlineStr">
         <is>
-          <t>-20,272</t>
+          <t>9,904</t>
         </is>
       </c>
       <c r="H32" s="7" t="inlineStr">
         <is>
-          <t>4,530</t>
+          <t>6,743</t>
         </is>
       </c>
       <c r="I32" s="6" t="inlineStr">
         <is>
-          <t>소프트웨어 개발 및 공급업</t>
+          <t>전자부품 제조업</t>
         </is>
       </c>
       <c r="J32" s="6" t="inlineStr">
         <is>
-          <t>한국</t>
+          <t>대신, NH</t>
         </is>
       </c>
       <c r="K32" s="6" t="inlineStr">
@@ -2219,7 +2219,7 @@
       </c>
       <c r="B33" s="6" t="inlineStr">
         <is>
-          <t>케이엠에프</t>
+          <t>유캐스트</t>
         </is>
       </c>
       <c r="C33" s="6" t="inlineStr">
@@ -2239,27 +2239,27 @@
       </c>
       <c r="F33" s="7" t="inlineStr">
         <is>
-          <t>25,751</t>
+          <t>5,934</t>
         </is>
       </c>
       <c r="G33" s="7" t="inlineStr">
         <is>
-          <t>11,463</t>
+          <t>-3,557</t>
         </is>
       </c>
       <c r="H33" s="7" t="inlineStr">
         <is>
-          <t>642</t>
+          <t>1,881</t>
         </is>
       </c>
       <c r="I33" s="6" t="inlineStr">
         <is>
-          <t>기타 식품 제조업</t>
+          <t>통신 및 방송 장비 제조업</t>
         </is>
       </c>
       <c r="J33" s="6" t="inlineStr">
         <is>
-          <t>IBK</t>
+          <t>유진</t>
         </is>
       </c>
       <c r="K33" s="6" t="inlineStr">
@@ -2276,7 +2276,7 @@
       </c>
       <c r="B34" s="6" t="inlineStr">
         <is>
-          <t>하나에어로다이내믹스</t>
+          <t>인터엑스</t>
         </is>
       </c>
       <c r="C34" s="6" t="inlineStr">
@@ -2296,27 +2296,27 @@
       </c>
       <c r="F34" s="7" t="inlineStr">
         <is>
-          <t>33,286</t>
+          <t>8,645</t>
         </is>
       </c>
       <c r="G34" s="7" t="inlineStr">
         <is>
-          <t>2,420</t>
+          <t>-20,272</t>
         </is>
       </c>
       <c r="H34" s="7" t="inlineStr">
         <is>
-          <t>890</t>
+          <t>4,530</t>
         </is>
       </c>
       <c r="I34" s="6" t="inlineStr">
         <is>
-          <t>항공기,우주선 및 부품 제조업</t>
+          <t>소프트웨어 개발 및 공급업</t>
         </is>
       </c>
       <c r="J34" s="6" t="inlineStr">
         <is>
-          <t>IBK</t>
+          <t>한국</t>
         </is>
       </c>
       <c r="K34" s="6" t="inlineStr">
@@ -2328,12 +2328,12 @@
     <row r="35">
       <c r="A35" s="6" t="inlineStr">
         <is>
-          <t>2026-05-28</t>
+          <t>2026-05-29</t>
         </is>
       </c>
       <c r="B35" s="6" t="inlineStr">
         <is>
-          <t>다비오</t>
+          <t>케이엠에프</t>
         </is>
       </c>
       <c r="C35" s="6" t="inlineStr">
@@ -2353,27 +2353,27 @@
       </c>
       <c r="F35" s="7" t="inlineStr">
         <is>
-          <t>9,251</t>
+          <t>25,751</t>
         </is>
       </c>
       <c r="G35" s="7" t="inlineStr">
         <is>
-          <t>-3,473</t>
+          <t>11,463</t>
         </is>
       </c>
       <c r="H35" s="7" t="inlineStr">
         <is>
-          <t>300</t>
+          <t>642</t>
         </is>
       </c>
       <c r="I35" s="6" t="inlineStr">
         <is>
-          <t>소프트웨어 개발 및 공급업</t>
+          <t>기타 식품 제조업</t>
         </is>
       </c>
       <c r="J35" s="6" t="inlineStr">
         <is>
-          <t>대신</t>
+          <t>IBK</t>
         </is>
       </c>
       <c r="K35" s="6" t="inlineStr">
@@ -2385,12 +2385,12 @@
     <row r="36">
       <c r="A36" s="6" t="inlineStr">
         <is>
-          <t>2026-05-28</t>
+          <t>2026-05-29</t>
         </is>
       </c>
       <c r="B36" s="6" t="inlineStr">
         <is>
-          <t>삼홍아크튜리온</t>
+          <t>하나에어로다이내믹스</t>
         </is>
       </c>
       <c r="C36" s="6" t="inlineStr">
@@ -2410,27 +2410,27 @@
       </c>
       <c r="F36" s="7" t="inlineStr">
         <is>
-          <t>26,162</t>
+          <t>33,286</t>
         </is>
       </c>
       <c r="G36" s="7" t="inlineStr">
         <is>
-          <t>-10,314</t>
+          <t>2,420</t>
         </is>
       </c>
       <c r="H36" s="7" t="inlineStr">
         <is>
-          <t>6,369</t>
+          <t>890</t>
         </is>
       </c>
       <c r="I36" s="6" t="inlineStr">
         <is>
-          <t>구조용 금속제품, 탱크 및 증기발생기 제조업</t>
+          <t>항공기,우주선 및 부품 제조업</t>
         </is>
       </c>
       <c r="J36" s="6" t="inlineStr">
         <is>
-          <t>삼성, 미래</t>
+          <t>IBK</t>
         </is>
       </c>
       <c r="K36" s="6" t="inlineStr">
@@ -2442,12 +2442,12 @@
     <row r="37">
       <c r="A37" s="6" t="inlineStr">
         <is>
-          <t>2026-05-22</t>
+          <t>2026-05-28</t>
         </is>
       </c>
       <c r="B37" s="6" t="inlineStr">
         <is>
-          <t>에이엘로봇</t>
+          <t>다비오</t>
         </is>
       </c>
       <c r="C37" s="6" t="inlineStr">
@@ -2467,22 +2467,22 @@
       </c>
       <c r="F37" s="7" t="inlineStr">
         <is>
-          <t>14,985</t>
+          <t>9,251</t>
         </is>
       </c>
       <c r="G37" s="7" t="inlineStr">
         <is>
-          <t>-21,891</t>
+          <t>-3,473</t>
         </is>
       </c>
       <c r="H37" s="7" t="inlineStr">
         <is>
-          <t>129</t>
+          <t>300</t>
         </is>
       </c>
       <c r="I37" s="6" t="inlineStr">
         <is>
-          <t>산업용 로봇 제조업</t>
+          <t>소프트웨어 개발 및 공급업</t>
         </is>
       </c>
       <c r="J37" s="6" t="inlineStr">
@@ -2499,12 +2499,12 @@
     <row r="38">
       <c r="A38" s="6" t="inlineStr">
         <is>
-          <t>2026-05-21</t>
+          <t>2026-05-28</t>
         </is>
       </c>
       <c r="B38" s="6" t="inlineStr">
         <is>
-          <t>넥스트에어로스페이스</t>
+          <t>삼홍아크튜리온</t>
         </is>
       </c>
       <c r="C38" s="6" t="inlineStr">
@@ -2524,27 +2524,27 @@
       </c>
       <c r="F38" s="7" t="inlineStr">
         <is>
-          <t>12,084</t>
+          <t>26,162</t>
         </is>
       </c>
       <c r="G38" s="7" t="inlineStr">
         <is>
-          <t>-17,270</t>
+          <t>-10,314</t>
         </is>
       </c>
       <c r="H38" s="7" t="inlineStr">
         <is>
-          <t>6,158</t>
+          <t>6,369</t>
         </is>
       </c>
       <c r="I38" s="6" t="inlineStr">
         <is>
-          <t>유인 항공기, 항공우주선 및 보조장치 제조업</t>
+          <t>구조용 금속제품, 탱크 및 증기발생기 제조업</t>
         </is>
       </c>
       <c r="J38" s="6" t="inlineStr">
         <is>
-          <t>삼성</t>
+          <t>삼성, 미래</t>
         </is>
       </c>
       <c r="K38" s="6" t="inlineStr">
@@ -2556,12 +2556,12 @@
     <row r="39">
       <c r="A39" s="6" t="inlineStr">
         <is>
-          <t>2026-05-21</t>
+          <t>2026-05-22</t>
         </is>
       </c>
       <c r="B39" s="6" t="inlineStr">
         <is>
-          <t>래블업</t>
+          <t>에이엘로봇</t>
         </is>
       </c>
       <c r="C39" s="6" t="inlineStr">
@@ -2581,27 +2581,27 @@
       </c>
       <c r="F39" s="7" t="inlineStr">
         <is>
-          <t>6,712</t>
+          <t>14,985</t>
         </is>
       </c>
       <c r="G39" s="7" t="inlineStr">
         <is>
-          <t>-1,526</t>
+          <t>-21,891</t>
         </is>
       </c>
       <c r="H39" s="7" t="inlineStr">
         <is>
-          <t>373</t>
+          <t>129</t>
         </is>
       </c>
       <c r="I39" s="6" t="inlineStr">
         <is>
-          <t>데이터베이스 및 온라인정보 제공업</t>
+          <t>산업용 로봇 제조업</t>
         </is>
       </c>
       <c r="J39" s="6" t="inlineStr">
         <is>
-          <t>NH</t>
+          <t>대신</t>
         </is>
       </c>
       <c r="K39" s="6" t="inlineStr">
@@ -2618,7 +2618,7 @@
       </c>
       <c r="B40" s="6" t="inlineStr">
         <is>
-          <t>비앤비코리아</t>
+          <t>넥스트에어로스페이스</t>
         </is>
       </c>
       <c r="C40" s="6" t="inlineStr">
@@ -2638,27 +2638,27 @@
       </c>
       <c r="F40" s="7" t="inlineStr">
         <is>
-          <t>141,169</t>
+          <t>12,084</t>
         </is>
       </c>
       <c r="G40" s="7" t="inlineStr">
         <is>
-          <t>21,406</t>
+          <t>-17,270</t>
         </is>
       </c>
       <c r="H40" s="7" t="inlineStr">
         <is>
-          <t>43,932</t>
+          <t>6,158</t>
         </is>
       </c>
       <c r="I40" s="6" t="inlineStr">
         <is>
-          <t>기타 화학제품 제조업</t>
+          <t>유인 항공기, 항공우주선 및 보조장치 제조업</t>
         </is>
       </c>
       <c r="J40" s="6" t="inlineStr">
         <is>
-          <t>미래</t>
+          <t>삼성</t>
         </is>
       </c>
       <c r="K40" s="6" t="inlineStr">
@@ -2675,7 +2675,7 @@
       </c>
       <c r="B41" s="6" t="inlineStr">
         <is>
-          <t>에이엔에이치스트럭쳐</t>
+          <t>비앤비코리아</t>
         </is>
       </c>
       <c r="C41" s="6" t="inlineStr">
@@ -2695,27 +2695,27 @@
       </c>
       <c r="F41" s="7" t="inlineStr">
         <is>
-          <t>19,784</t>
+          <t>141,169</t>
         </is>
       </c>
       <c r="G41" s="7" t="inlineStr">
         <is>
-          <t>-4,296</t>
+          <t>21,406</t>
         </is>
       </c>
       <c r="H41" s="7" t="inlineStr">
         <is>
-          <t>24,561</t>
+          <t>43,932</t>
         </is>
       </c>
       <c r="I41" s="6" t="inlineStr">
         <is>
-          <t>건축기술, 엔지니어링 및 관련 기술 서비스업</t>
+          <t>기타 화학제품 제조업</t>
         </is>
       </c>
       <c r="J41" s="6" t="inlineStr">
         <is>
-          <t>NH</t>
+          <t>미래</t>
         </is>
       </c>
       <c r="K41" s="6" t="inlineStr">
@@ -2727,12 +2727,12 @@
     <row r="42">
       <c r="A42" s="6" t="inlineStr">
         <is>
-          <t>2026-05-19</t>
+          <t>2026-05-21</t>
         </is>
       </c>
       <c r="B42" s="6" t="inlineStr">
         <is>
-          <t>엘리스그룹</t>
+          <t>에이엔에이치스트럭쳐</t>
         </is>
       </c>
       <c r="C42" s="6" t="inlineStr">
@@ -2752,27 +2752,27 @@
       </c>
       <c r="F42" s="7" t="inlineStr">
         <is>
-          <t>39,513</t>
+          <t>19,784</t>
         </is>
       </c>
       <c r="G42" s="7" t="inlineStr">
         <is>
-          <t>15,666</t>
+          <t>-4,296</t>
         </is>
       </c>
       <c r="H42" s="7" t="inlineStr">
         <is>
-          <t>85,400</t>
+          <t>24,561</t>
         </is>
       </c>
       <c r="I42" s="6" t="inlineStr">
         <is>
-          <t>소프트웨어 개발 및 공급업</t>
+          <t>건축기술, 엔지니어링 및 관련 기술 서비스업</t>
         </is>
       </c>
       <c r="J42" s="6" t="inlineStr">
         <is>
-          <t>미래, 삼성</t>
+          <t>NH</t>
         </is>
       </c>
       <c r="K42" s="6" t="inlineStr">
@@ -2784,12 +2784,12 @@
     <row r="43">
       <c r="A43" s="6" t="inlineStr">
         <is>
-          <t>2026-05-12</t>
+          <t>2026-05-19</t>
         </is>
       </c>
       <c r="B43" s="6" t="inlineStr">
         <is>
-          <t>오토핸즈</t>
+          <t>엘리스그룹</t>
         </is>
       </c>
       <c r="C43" s="6" t="inlineStr">
@@ -2799,7 +2799,7 @@
       </c>
       <c r="D43" s="6" t="inlineStr">
         <is>
-          <t>스팩 소멸합병</t>
+          <t>신규상장</t>
         </is>
       </c>
       <c r="E43" s="6" t="inlineStr">
@@ -2809,27 +2809,27 @@
       </c>
       <c r="F43" s="7" t="inlineStr">
         <is>
-          <t>238,564</t>
+          <t>39,513</t>
         </is>
       </c>
       <c r="G43" s="7" t="inlineStr">
         <is>
-          <t>6,047</t>
+          <t>15,666</t>
         </is>
       </c>
       <c r="H43" s="7" t="inlineStr">
         <is>
-          <t>6,129</t>
+          <t>85,400</t>
         </is>
       </c>
       <c r="I43" s="6" t="inlineStr">
         <is>
-          <t>자동차 판매업</t>
+          <t>소프트웨어 개발 및 공급업</t>
         </is>
       </c>
       <c r="J43" s="6" t="inlineStr">
         <is>
-          <t>미래</t>
+          <t>미래, 삼성</t>
         </is>
       </c>
       <c r="K43" s="6" t="inlineStr">
@@ -2841,12 +2841,12 @@
     <row r="44">
       <c r="A44" s="6" t="inlineStr">
         <is>
-          <t>2026-05-06</t>
+          <t>2026-05-12</t>
         </is>
       </c>
       <c r="B44" s="6" t="inlineStr">
         <is>
-          <t>아이벡스메디칼시스템즈</t>
+          <t>오토핸즈</t>
         </is>
       </c>
       <c r="C44" s="6" t="inlineStr">
@@ -2856,7 +2856,7 @@
       </c>
       <c r="D44" s="6" t="inlineStr">
         <is>
-          <t>신규상장</t>
+          <t>스팩 소멸합병</t>
         </is>
       </c>
       <c r="E44" s="6" t="inlineStr">
@@ -2866,27 +2866,27 @@
       </c>
       <c r="F44" s="7" t="inlineStr">
         <is>
-          <t>15,282</t>
+          <t>238,564</t>
         </is>
       </c>
       <c r="G44" s="7" t="inlineStr">
         <is>
-          <t>-7,227</t>
+          <t>6,047</t>
         </is>
       </c>
       <c r="H44" s="7" t="inlineStr">
         <is>
-          <t>744</t>
+          <t>6,129</t>
         </is>
       </c>
       <c r="I44" s="6" t="inlineStr">
         <is>
-          <t>의료용 기기 제조업</t>
+          <t>자동차 판매업</t>
         </is>
       </c>
       <c r="J44" s="6" t="inlineStr">
         <is>
-          <t>NH</t>
+          <t>미래</t>
         </is>
       </c>
       <c r="K44" s="6" t="inlineStr">
@@ -2898,12 +2898,12 @@
     <row r="45">
       <c r="A45" s="6" t="inlineStr">
         <is>
-          <t>2026-04-30</t>
+          <t>2026-05-06</t>
         </is>
       </c>
       <c r="B45" s="6" t="inlineStr">
         <is>
-          <t>멜콘</t>
+          <t>아이벡스메디칼시스템즈</t>
         </is>
       </c>
       <c r="C45" s="6" t="inlineStr">
@@ -2923,27 +2923,27 @@
       </c>
       <c r="F45" s="7" t="inlineStr">
         <is>
-          <t>39,319</t>
+          <t>15,282</t>
         </is>
       </c>
       <c r="G45" s="7" t="inlineStr">
         <is>
-          <t>4,739</t>
+          <t>-7,227</t>
         </is>
       </c>
       <c r="H45" s="7" t="inlineStr">
         <is>
-          <t>1,250</t>
+          <t>744</t>
         </is>
       </c>
       <c r="I45" s="6" t="inlineStr">
         <is>
-          <t>특수 목적용 기계 제조업</t>
+          <t>의료용 기기 제조업</t>
         </is>
       </c>
       <c r="J45" s="6" t="inlineStr">
         <is>
-          <t>대신</t>
+          <t>NH</t>
         </is>
       </c>
       <c r="K45" s="6" t="inlineStr">
@@ -3069,12 +3069,12 @@
     <row r="48">
       <c r="A48" s="6" t="inlineStr">
         <is>
-          <t>2026-04-10</t>
+          <t>2026-04-08</t>
         </is>
       </c>
       <c r="B48" s="6" t="inlineStr">
         <is>
-          <t>엠비디</t>
+          <t>옵토닉스</t>
         </is>
       </c>
       <c r="C48" s="6" t="inlineStr">
@@ -3094,27 +3094,27 @@
       </c>
       <c r="F48" s="7" t="inlineStr">
         <is>
-          <t>1,524</t>
+          <t>25,368</t>
         </is>
       </c>
       <c r="G48" s="7" t="inlineStr">
         <is>
-          <t>-2,125</t>
+          <t>1,901</t>
         </is>
       </c>
       <c r="H48" s="7" t="inlineStr">
         <is>
-          <t>2,753</t>
+          <t>730</t>
         </is>
       </c>
       <c r="I48" s="6" t="inlineStr">
         <is>
-          <t>물질 검사, 측정 및 분석기구 제조업</t>
+          <t>광학렌즈 및 광학요소 제조업</t>
         </is>
       </c>
       <c r="J48" s="6" t="inlineStr">
         <is>
-          <t>하나</t>
+          <t>한국</t>
         </is>
       </c>
       <c r="K48" s="6" t="inlineStr">
@@ -3126,12 +3126,12 @@
     <row r="49">
       <c r="A49" s="6" t="inlineStr">
         <is>
-          <t>2026-04-08</t>
+          <t>2026-04-07</t>
         </is>
       </c>
       <c r="B49" s="6" t="inlineStr">
         <is>
-          <t>옵토닉스</t>
+          <t>크리에이츠</t>
         </is>
       </c>
       <c r="C49" s="6" t="inlineStr">
@@ -3151,27 +3151,27 @@
       </c>
       <c r="F49" s="7" t="inlineStr">
         <is>
-          <t>25,368</t>
+          <t>76,395</t>
         </is>
       </c>
       <c r="G49" s="7" t="inlineStr">
         <is>
-          <t>1,901</t>
+          <t>23,749</t>
         </is>
       </c>
       <c r="H49" s="7" t="inlineStr">
         <is>
-          <t>730</t>
+          <t>2,335</t>
         </is>
       </c>
       <c r="I49" s="6" t="inlineStr">
         <is>
-          <t>광학렌즈 및 광학요소 제조업</t>
+          <t>그외 기타 제품 제조업</t>
         </is>
       </c>
       <c r="J49" s="6" t="inlineStr">
         <is>
-          <t>한국</t>
+          <t>삼성</t>
         </is>
       </c>
       <c r="K49" s="6" t="inlineStr">
@@ -3183,12 +3183,12 @@
     <row r="50">
       <c r="A50" s="6" t="inlineStr">
         <is>
-          <t>2026-04-07</t>
+          <t>2026-03-24</t>
         </is>
       </c>
       <c r="B50" s="6" t="inlineStr">
         <is>
-          <t>크리에이츠</t>
+          <t>인텔리빅스</t>
         </is>
       </c>
       <c r="C50" s="6" t="inlineStr">
@@ -3208,27 +3208,27 @@
       </c>
       <c r="F50" s="7" t="inlineStr">
         <is>
-          <t>76,395</t>
+          <t>46,644</t>
         </is>
       </c>
       <c r="G50" s="7" t="inlineStr">
         <is>
-          <t>23,749</t>
+          <t>5,357</t>
         </is>
       </c>
       <c r="H50" s="7" t="inlineStr">
         <is>
-          <t>2,335</t>
+          <t>1,048</t>
         </is>
       </c>
       <c r="I50" s="6" t="inlineStr">
         <is>
-          <t>그외 기타 제품 제조업</t>
+          <t>소프트웨어 개발 및 공급업</t>
         </is>
       </c>
       <c r="J50" s="6" t="inlineStr">
         <is>
-          <t>삼성</t>
+          <t>미래</t>
         </is>
       </c>
       <c r="K50" s="6" t="inlineStr">
@@ -3240,12 +3240,12 @@
     <row r="51">
       <c r="A51" s="6" t="inlineStr">
         <is>
-          <t>2026-03-24</t>
+          <t>2026-02-27</t>
         </is>
       </c>
       <c r="B51" s="6" t="inlineStr">
         <is>
-          <t>인텔리빅스</t>
+          <t>피지티</t>
         </is>
       </c>
       <c r="C51" s="6" t="inlineStr">
@@ -3265,27 +3265,27 @@
       </c>
       <c r="F51" s="7" t="inlineStr">
         <is>
-          <t>46,644</t>
+          <t>40,141</t>
         </is>
       </c>
       <c r="G51" s="7" t="inlineStr">
         <is>
-          <t>5,357</t>
+          <t>-69,722</t>
         </is>
       </c>
       <c r="H51" s="7" t="inlineStr">
         <is>
-          <t>1,048</t>
+          <t>6,029</t>
         </is>
       </c>
       <c r="I51" s="6" t="inlineStr">
         <is>
-          <t>소프트웨어 개발 및 공급업</t>
+          <t>기타 화학제품 제조업</t>
         </is>
       </c>
       <c r="J51" s="6" t="inlineStr">
         <is>
-          <t>미래</t>
+          <t>한국</t>
         </is>
       </c>
       <c r="K51" s="6" t="inlineStr">
@@ -3297,12 +3297,12 @@
     <row r="52">
       <c r="A52" s="6" t="inlineStr">
         <is>
-          <t>2026-02-27</t>
+          <t>2025-09-11</t>
         </is>
       </c>
       <c r="B52" s="6" t="inlineStr">
         <is>
-          <t>피지티</t>
+          <t>씨엠디엘</t>
         </is>
       </c>
       <c r="C52" s="6" t="inlineStr">
@@ -3312,173 +3312,173 @@
       </c>
       <c r="D52" s="6" t="inlineStr">
         <is>
+          <t>스팩 소멸합병</t>
+        </is>
+      </c>
+      <c r="E52" s="6" t="inlineStr">
+        <is>
+          <t>FY24</t>
+        </is>
+      </c>
+      <c r="F52" s="7" t="inlineStr">
+        <is>
+          <t>39,991</t>
+        </is>
+      </c>
+      <c r="G52" s="7" t="inlineStr">
+        <is>
+          <t>3,541</t>
+        </is>
+      </c>
+      <c r="H52" s="7" t="inlineStr">
+        <is>
+          <t>503</t>
+        </is>
+      </c>
+      <c r="I52" s="6" t="inlineStr">
+        <is>
+          <t>기타 기초 유기 화학물질 제조업</t>
+        </is>
+      </c>
+      <c r="J52" s="6" t="inlineStr">
+        <is>
+          <t>교보</t>
+        </is>
+      </c>
+      <c r="K52" s="6" t="inlineStr">
+        <is>
+          <t>예심 진행중</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="3" t="inlineStr">
+        <is>
+          <t>■ 심사 승인  (45건)</t>
+        </is>
+      </c>
+      <c r="B54" s="4" t="n"/>
+      <c r="C54" s="4" t="n"/>
+      <c r="D54" s="4" t="n"/>
+      <c r="E54" s="4" t="n"/>
+      <c r="F54" s="4" t="n"/>
+      <c r="G54" s="4" t="n"/>
+      <c r="H54" s="4" t="n"/>
+      <c r="I54" s="4" t="n"/>
+      <c r="J54" s="4" t="n"/>
+      <c r="K54" s="4" t="n"/>
+    </row>
+    <row r="55">
+      <c r="A55" s="5" t="inlineStr">
+        <is>
+          <t>일자</t>
+        </is>
+      </c>
+      <c r="B55" s="5" t="inlineStr">
+        <is>
+          <t>회사명</t>
+        </is>
+      </c>
+      <c r="C55" s="5" t="inlineStr">
+        <is>
+          <t>시장</t>
+        </is>
+      </c>
+      <c r="D55" s="5" t="inlineStr">
+        <is>
+          <t>상장유형</t>
+        </is>
+      </c>
+      <c r="E55" s="5" t="inlineStr">
+        <is>
+          <t>기준연도</t>
+        </is>
+      </c>
+      <c r="F55" s="5" t="inlineStr">
+        <is>
+          <t>매출액</t>
+        </is>
+      </c>
+      <c r="G55" s="5" t="inlineStr">
+        <is>
+          <t>순이익</t>
+        </is>
+      </c>
+      <c r="H55" s="5" t="inlineStr">
+        <is>
+          <t>자기자본</t>
+        </is>
+      </c>
+      <c r="I55" s="5" t="inlineStr">
+        <is>
+          <t>업종</t>
+        </is>
+      </c>
+      <c r="J55" s="5" t="inlineStr">
+        <is>
+          <t>대표주관사</t>
+        </is>
+      </c>
+      <c r="K55" s="5" t="inlineStr">
+        <is>
+          <t>현황</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="6" t="inlineStr">
+        <is>
+          <t>2026-07-30</t>
+        </is>
+      </c>
+      <c r="B56" s="6" t="inlineStr">
+        <is>
+          <t>래블업</t>
+        </is>
+      </c>
+      <c r="C56" s="6" t="inlineStr">
+        <is>
+          <t>코스닥</t>
+        </is>
+      </c>
+      <c r="D56" s="6" t="inlineStr">
+        <is>
           <t>신규상장</t>
         </is>
       </c>
-      <c r="E52" s="6" t="inlineStr">
+      <c r="E56" s="6" t="inlineStr">
         <is>
           <t>FY25</t>
         </is>
       </c>
-      <c r="F52" s="7" t="inlineStr">
-        <is>
-          <t>40,141</t>
-        </is>
-      </c>
-      <c r="G52" s="7" t="inlineStr">
-        <is>
-          <t>-69,722</t>
-        </is>
-      </c>
-      <c r="H52" s="7" t="inlineStr">
-        <is>
-          <t>6,029</t>
-        </is>
-      </c>
-      <c r="I52" s="6" t="inlineStr">
-        <is>
-          <t>기타 화학제품 제조업</t>
-        </is>
-      </c>
-      <c r="J52" s="6" t="inlineStr">
-        <is>
-          <t>한국</t>
-        </is>
-      </c>
-      <c r="K52" s="6" t="inlineStr">
-        <is>
-          <t>예심 진행중</t>
-        </is>
-      </c>
-    </row>
-    <row r="53">
-      <c r="A53" s="6" t="inlineStr">
-        <is>
-          <t>2025-09-11</t>
-        </is>
-      </c>
-      <c r="B53" s="6" t="inlineStr">
-        <is>
-          <t>씨엠디엘</t>
-        </is>
-      </c>
-      <c r="C53" s="6" t="inlineStr">
-        <is>
-          <t>코스닥</t>
-        </is>
-      </c>
-      <c r="D53" s="6" t="inlineStr">
-        <is>
-          <t>스팩 소멸합병</t>
-        </is>
-      </c>
-      <c r="E53" s="6" t="inlineStr">
-        <is>
-          <t>FY24</t>
-        </is>
-      </c>
-      <c r="F53" s="7" t="inlineStr">
-        <is>
-          <t>39,991</t>
-        </is>
-      </c>
-      <c r="G53" s="7" t="inlineStr">
-        <is>
-          <t>3,541</t>
-        </is>
-      </c>
-      <c r="H53" s="7" t="inlineStr">
-        <is>
-          <t>503</t>
-        </is>
-      </c>
-      <c r="I53" s="6" t="inlineStr">
-        <is>
-          <t>기타 기초 유기 화학물질 제조업</t>
-        </is>
-      </c>
-      <c r="J53" s="6" t="inlineStr">
-        <is>
-          <t>교보</t>
-        </is>
-      </c>
-      <c r="K53" s="6" t="inlineStr">
-        <is>
-          <t>예심 진행중</t>
-        </is>
-      </c>
-    </row>
-    <row r="55">
-      <c r="A55" s="3" t="inlineStr">
-        <is>
-          <t>■ 심사 승인  (44건)</t>
-        </is>
-      </c>
-      <c r="B55" s="4" t="n"/>
-      <c r="C55" s="4" t="n"/>
-      <c r="D55" s="4" t="n"/>
-      <c r="E55" s="4" t="n"/>
-      <c r="F55" s="4" t="n"/>
-      <c r="G55" s="4" t="n"/>
-      <c r="H55" s="4" t="n"/>
-      <c r="I55" s="4" t="n"/>
-      <c r="J55" s="4" t="n"/>
-      <c r="K55" s="4" t="n"/>
-    </row>
-    <row r="56">
-      <c r="A56" s="5" t="inlineStr">
-        <is>
-          <t>일자</t>
-        </is>
-      </c>
-      <c r="B56" s="5" t="inlineStr">
-        <is>
-          <t>회사명</t>
-        </is>
-      </c>
-      <c r="C56" s="5" t="inlineStr">
-        <is>
-          <t>시장</t>
-        </is>
-      </c>
-      <c r="D56" s="5" t="inlineStr">
-        <is>
-          <t>상장유형</t>
-        </is>
-      </c>
-      <c r="E56" s="5" t="inlineStr">
-        <is>
-          <t>기준연도</t>
-        </is>
-      </c>
-      <c r="F56" s="5" t="inlineStr">
-        <is>
-          <t>매출액</t>
-        </is>
-      </c>
-      <c r="G56" s="5" t="inlineStr">
-        <is>
-          <t>순이익</t>
-        </is>
-      </c>
-      <c r="H56" s="5" t="inlineStr">
-        <is>
-          <t>자기자본</t>
-        </is>
-      </c>
-      <c r="I56" s="5" t="inlineStr">
-        <is>
-          <t>업종</t>
-        </is>
-      </c>
-      <c r="J56" s="5" t="inlineStr">
-        <is>
-          <t>대표주관사</t>
-        </is>
-      </c>
-      <c r="K56" s="5" t="inlineStr">
-        <is>
-          <t>현황</t>
+      <c r="F56" s="7" t="inlineStr">
+        <is>
+          <t>6,712</t>
+        </is>
+      </c>
+      <c r="G56" s="7" t="inlineStr">
+        <is>
+          <t>-1,526</t>
+        </is>
+      </c>
+      <c r="H56" s="7" t="inlineStr">
+        <is>
+          <t>373</t>
+        </is>
+      </c>
+      <c r="I56" s="6" t="inlineStr">
+        <is>
+          <t>데이터베이스 및 온라인정보 제공업</t>
+        </is>
+      </c>
+      <c r="J56" s="6" t="inlineStr">
+        <is>
+          <t>NH</t>
+        </is>
+      </c>
+      <c r="K56" s="6" t="inlineStr">
+        <is>
+          <t>상장전</t>
         </is>
       </c>
     </row>
@@ -6859,7 +6859,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R64"/>
+  <dimension ref="A1:R65"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="1"/>
@@ -9657,7 +9657,7 @@
     <row r="40" ht="22" customHeight="1">
       <c r="A40" s="3" t="inlineStr">
         <is>
-          <t>■ 공모 진행 (예심 승인법인)  (20건)</t>
+          <t>■ 공모 진행 (예심 승인법인)  (21건)</t>
         </is>
       </c>
       <c r="B40" s="4" t="n"/>
@@ -10966,22 +10966,86 @@
         </is>
       </c>
     </row>
-    <row r="62">
-      <c r="A62" s="20" t="inlineStr">
-        <is>
-          <t>※ 상장 완료 = KIND 신규상장 페이지 기준(스팩합병 포함) · 스팩 공모상장은 밴드·밸류에이션 등 해당없음(공모가 2,000원 고정).</t>
+    <row r="61" ht="30" customHeight="1">
+      <c r="A61" s="6" t="inlineStr">
+        <is>
+          <t>래블업</t>
+        </is>
+      </c>
+      <c r="B61" s="18" t="inlineStr">
+        <is>
+          <t>수집예정</t>
+        </is>
+      </c>
+      <c r="C61" s="18" t="inlineStr">
+        <is>
+          <t>수집예정</t>
+        </is>
+      </c>
+      <c r="D61" s="18" t="inlineStr">
+        <is>
+          <t>수집예정</t>
+        </is>
+      </c>
+      <c r="E61" s="18" t="inlineStr">
+        <is>
+          <t>수집예정</t>
+        </is>
+      </c>
+      <c r="F61" s="18" t="inlineStr">
+        <is>
+          <t>수집예정</t>
+        </is>
+      </c>
+      <c r="G61" s="6" t="inlineStr"/>
+      <c r="H61" s="6" t="inlineStr"/>
+      <c r="I61" s="6" t="inlineStr"/>
+      <c r="J61" s="18" t="inlineStr">
+        <is>
+          <t>수집예정</t>
+        </is>
+      </c>
+      <c r="K61" s="6" t="inlineStr"/>
+      <c r="L61" s="6" t="inlineStr"/>
+      <c r="M61" s="6" t="inlineStr"/>
+      <c r="N61" s="18" t="inlineStr">
+        <is>
+          <t>수집예정</t>
+        </is>
+      </c>
+      <c r="O61" s="6" t="inlineStr"/>
+      <c r="P61" s="18" t="inlineStr">
+        <is>
+          <t>수집예정</t>
+        </is>
+      </c>
+      <c r="Q61" s="18" t="inlineStr">
+        <is>
+          <t>수집예정</t>
+        </is>
+      </c>
+      <c r="R61" s="6" t="inlineStr">
+        <is>
+          <t>신고서 대기</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" s="20" t="inlineStr">
         <is>
-          <t>※ 기재정정 신고서 내 정정 전·후 병존 → 자동수집은 "정정 후" 값만 취함.</t>
+          <t>※ 상장 완료 = KIND 신규상장 페이지 기준(스팩합병 포함) · 스팩 공모상장은 밴드·밸류에이션 등 해당없음(공모가 2,000원 고정).</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" s="20" t="inlineStr">
+        <is>
+          <t>※ 기재정정 신고서 내 정정 전·후 병존 → 자동수집은 "정정 후" 값만 취함.</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" s="20" t="inlineStr">
         <is>
           <t>※ 청약경쟁률=일반투자자 청약수량÷최종배정수량 · "MM-DD~"는 종료일 자동수집 예정.</t>
         </is>
@@ -11146,7 +11210,7 @@
         <v>14</v>
       </c>
       <c r="C9" s="6" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="D9" s="6" t="n">
         <v>3</v>
@@ -11212,10 +11276,10 @@
         </is>
       </c>
       <c r="B12" s="6" t="n">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="C12" s="6" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="D12" s="6" t="n">
         <v>1</v>

</xml_diff>

<commit_message>
chore: update IPO data 2026-08-03
</commit_message>
<xml_diff>
--- a/IPO_analysis.xlsx
+++ b/IPO_analysis.xlsx
@@ -592,7 +592,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K122"/>
+  <dimension ref="A1:K123"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -618,7 +618,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>기준일 2026-08-02 · 청구일 직전 사업연도 · 별도/개별 재무제표 · 단위 백만원(별도 표기 시 USD)</t>
+          <t>기준일 2026-08-03 · 청구일 직전 사업연도 · 별도/개별 재무제표 · 단위 백만원(별도 표기 시 USD)</t>
         </is>
       </c>
     </row>
@@ -3468,7 +3468,7 @@
     <row r="56">
       <c r="A56" s="3" t="inlineStr">
         <is>
-          <t>■ 심사 승인  (45건)</t>
+          <t>■ 심사 승인  (46건)</t>
         </is>
       </c>
       <c r="B56" s="4" t="n"/>
@@ -3599,12 +3599,12 @@
     <row r="59">
       <c r="A59" s="6" t="inlineStr">
         <is>
-          <t>2026-07-29</t>
+          <t>2026-07-30</t>
         </is>
       </c>
       <c r="B59" s="6" t="inlineStr">
         <is>
-          <t>에스케이증권제14호기업인수목적</t>
+          <t>엠비디</t>
         </is>
       </c>
       <c r="C59" s="6" t="inlineStr">
@@ -3624,27 +3624,27 @@
       </c>
       <c r="F59" s="7" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>1,524</t>
         </is>
       </c>
       <c r="G59" s="7" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>-2,125</t>
         </is>
       </c>
       <c r="H59" s="7" t="inlineStr">
         <is>
-          <t>17</t>
+          <t>2,753</t>
         </is>
       </c>
       <c r="I59" s="6" t="inlineStr">
         <is>
-          <t>기타 금융업</t>
+          <t>물질 검사, 측정 및 분석기구 제조업</t>
         </is>
       </c>
       <c r="J59" s="6" t="inlineStr">
         <is>
-          <t>SK</t>
+          <t>하나</t>
         </is>
       </c>
       <c r="K59" s="6" t="inlineStr">
@@ -3661,7 +3661,7 @@
       </c>
       <c r="B60" s="6" t="inlineStr">
         <is>
-          <t>케이비제34호스팩</t>
+          <t>에스케이증권제14호기업인수목적</t>
         </is>
       </c>
       <c r="C60" s="6" t="inlineStr">
@@ -3691,7 +3691,7 @@
       </c>
       <c r="H60" s="7" t="inlineStr">
         <is>
-          <t>21</t>
+          <t>17</t>
         </is>
       </c>
       <c r="I60" s="6" t="inlineStr">
@@ -3701,7 +3701,7 @@
       </c>
       <c r="J60" s="6" t="inlineStr">
         <is>
-          <t>KB</t>
+          <t>SK</t>
         </is>
       </c>
       <c r="K60" s="6" t="inlineStr">
@@ -3718,7 +3718,7 @@
       </c>
       <c r="B61" s="6" t="inlineStr">
         <is>
-          <t>한국제17호스팩</t>
+          <t>케이비제34호스팩</t>
         </is>
       </c>
       <c r="C61" s="6" t="inlineStr">
@@ -3748,7 +3748,7 @@
       </c>
       <c r="H61" s="7" t="inlineStr">
         <is>
-          <t>170</t>
+          <t>21</t>
         </is>
       </c>
       <c r="I61" s="6" t="inlineStr">
@@ -3758,7 +3758,7 @@
       </c>
       <c r="J61" s="6" t="inlineStr">
         <is>
-          <t>한국</t>
+          <t>KB</t>
         </is>
       </c>
       <c r="K61" s="6" t="inlineStr">
@@ -3775,7 +3775,7 @@
       </c>
       <c r="B62" s="6" t="inlineStr">
         <is>
-          <t>한화플러스제6호스팩</t>
+          <t>한국제17호스팩</t>
         </is>
       </c>
       <c r="C62" s="6" t="inlineStr">
@@ -3805,7 +3805,7 @@
       </c>
       <c r="H62" s="7" t="inlineStr">
         <is>
-          <t>41</t>
+          <t>170</t>
         </is>
       </c>
       <c r="I62" s="6" t="inlineStr">
@@ -3815,7 +3815,7 @@
       </c>
       <c r="J62" s="6" t="inlineStr">
         <is>
-          <t>한화</t>
+          <t>한국</t>
         </is>
       </c>
       <c r="K62" s="6" t="inlineStr">
@@ -3827,12 +3827,12 @@
     <row r="63">
       <c r="A63" s="6" t="inlineStr">
         <is>
-          <t>2026-07-22</t>
+          <t>2026-07-29</t>
         </is>
       </c>
       <c r="B63" s="6" t="inlineStr">
         <is>
-          <t>엔에이치스팩34호</t>
+          <t>한화플러스제6호스팩</t>
         </is>
       </c>
       <c r="C63" s="6" t="inlineStr">
@@ -3862,17 +3862,17 @@
       </c>
       <c r="H63" s="7" t="inlineStr">
         <is>
-          <t>55</t>
+          <t>41</t>
         </is>
       </c>
       <c r="I63" s="6" t="inlineStr">
         <is>
-          <t>금융 지원 서비스업</t>
+          <t>기타 금융업</t>
         </is>
       </c>
       <c r="J63" s="6" t="inlineStr">
         <is>
-          <t>NH</t>
+          <t>한화</t>
         </is>
       </c>
       <c r="K63" s="6" t="inlineStr">
@@ -3884,12 +3884,12 @@
     <row r="64">
       <c r="A64" s="6" t="inlineStr">
         <is>
-          <t>2026-07-20</t>
+          <t>2026-07-22</t>
         </is>
       </c>
       <c r="B64" s="6" t="inlineStr">
         <is>
-          <t>글로벌테크놀로지</t>
+          <t>엔에이치스팩34호</t>
         </is>
       </c>
       <c r="C64" s="6" t="inlineStr">
@@ -3909,27 +3909,27 @@
       </c>
       <c r="F64" s="7" t="inlineStr">
         <is>
-          <t>29,689</t>
+          <t>-</t>
         </is>
       </c>
       <c r="G64" s="7" t="inlineStr">
         <is>
-          <t>-25,889</t>
+          <t>-</t>
         </is>
       </c>
       <c r="H64" s="7" t="inlineStr">
         <is>
-          <t>6,402</t>
+          <t>55</t>
         </is>
       </c>
       <c r="I64" s="6" t="inlineStr">
         <is>
-          <t>반도체 제조업</t>
+          <t>금융 지원 서비스업</t>
         </is>
       </c>
       <c r="J64" s="6" t="inlineStr">
         <is>
-          <t>한국</t>
+          <t>NH</t>
         </is>
       </c>
       <c r="K64" s="6" t="inlineStr">
@@ -3946,7 +3946,7 @@
       </c>
       <c r="B65" s="6" t="inlineStr">
         <is>
-          <t>덕산넵코어스</t>
+          <t>글로벌테크놀로지</t>
         </is>
       </c>
       <c r="C65" s="6" t="inlineStr">
@@ -3961,32 +3961,32 @@
       </c>
       <c r="E65" s="6" t="inlineStr">
         <is>
-          <t>FY24</t>
+          <t>FY25</t>
         </is>
       </c>
       <c r="F65" s="7" t="inlineStr">
         <is>
-          <t>48,504</t>
+          <t>29,689</t>
         </is>
       </c>
       <c r="G65" s="7" t="inlineStr">
         <is>
-          <t>3,668</t>
+          <t>-25,889</t>
         </is>
       </c>
       <c r="H65" s="7" t="inlineStr">
         <is>
-          <t>8,448</t>
+          <t>6,402</t>
         </is>
       </c>
       <c r="I65" s="6" t="inlineStr">
         <is>
-          <t>항공기,우주선 및 부품 제조업</t>
+          <t>반도체 제조업</t>
         </is>
       </c>
       <c r="J65" s="6" t="inlineStr">
         <is>
-          <t>대신</t>
+          <t>한국</t>
         </is>
       </c>
       <c r="K65" s="6" t="inlineStr">
@@ -4003,7 +4003,7 @@
       </c>
       <c r="B66" s="6" t="inlineStr">
         <is>
-          <t>디티에스</t>
+          <t>덕산넵코어스</t>
         </is>
       </c>
       <c r="C66" s="6" t="inlineStr">
@@ -4023,22 +4023,22 @@
       </c>
       <c r="F66" s="7" t="inlineStr">
         <is>
-          <t>142,718</t>
+          <t>48,504</t>
         </is>
       </c>
       <c r="G66" s="7" t="inlineStr">
         <is>
-          <t>18,765</t>
+          <t>3,668</t>
         </is>
       </c>
       <c r="H66" s="7" t="inlineStr">
         <is>
-          <t>63,153</t>
+          <t>8,448</t>
         </is>
       </c>
       <c r="I66" s="6" t="inlineStr">
         <is>
-          <t>특수 목적용 기계 제조업</t>
+          <t>항공기,우주선 및 부품 제조업</t>
         </is>
       </c>
       <c r="J66" s="6" t="inlineStr">
@@ -4055,12 +4055,12 @@
     <row r="67">
       <c r="A67" s="6" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
+          <t>2026-07-20</t>
         </is>
       </c>
       <c r="B67" s="6" t="inlineStr">
         <is>
-          <t>네오사피엔스</t>
+          <t>디티에스</t>
         </is>
       </c>
       <c r="C67" s="6" t="inlineStr">
@@ -4075,27 +4075,27 @@
       </c>
       <c r="E67" s="6" t="inlineStr">
         <is>
-          <t>FY25</t>
+          <t>FY24</t>
         </is>
       </c>
       <c r="F67" s="7" t="inlineStr">
         <is>
-          <t>10,649</t>
+          <t>142,718</t>
         </is>
       </c>
       <c r="G67" s="7" t="inlineStr">
         <is>
-          <t>-6,994</t>
+          <t>18,765</t>
         </is>
       </c>
       <c r="H67" s="7" t="inlineStr">
         <is>
-          <t>-39,962</t>
+          <t>63,153</t>
         </is>
       </c>
       <c r="I67" s="6" t="inlineStr">
         <is>
-          <t>소프트웨어 개발 및 공급업</t>
+          <t>특수 목적용 기계 제조업</t>
         </is>
       </c>
       <c r="J67" s="6" t="inlineStr">
@@ -4117,7 +4117,7 @@
       </c>
       <c r="B68" s="6" t="inlineStr">
         <is>
-          <t>엠에스바이오</t>
+          <t>네오사피엔스</t>
         </is>
       </c>
       <c r="C68" s="6" t="inlineStr">
@@ -4137,27 +4137,27 @@
       </c>
       <c r="F68" s="7" t="inlineStr">
         <is>
-          <t>23,787</t>
+          <t>10,649</t>
         </is>
       </c>
       <c r="G68" s="7" t="inlineStr">
         <is>
-          <t>7,288</t>
+          <t>-6,994</t>
         </is>
       </c>
       <c r="H68" s="7" t="inlineStr">
         <is>
-          <t>1,942</t>
+          <t>-39,962</t>
         </is>
       </c>
       <c r="I68" s="6" t="inlineStr">
         <is>
-          <t>의료용 기기 제조업</t>
+          <t>소프트웨어 개발 및 공급업</t>
         </is>
       </c>
       <c r="J68" s="6" t="inlineStr">
         <is>
-          <t>KB</t>
+          <t>대신</t>
         </is>
       </c>
       <c r="K68" s="6" t="inlineStr">
@@ -4169,12 +4169,12 @@
     <row r="69">
       <c r="A69" s="6" t="inlineStr">
         <is>
-          <t>2026-06-25</t>
+          <t>2026-07-10</t>
         </is>
       </c>
       <c r="B69" s="6" t="inlineStr">
         <is>
-          <t>기도산업</t>
+          <t>엠에스바이오</t>
         </is>
       </c>
       <c r="C69" s="6" t="inlineStr">
@@ -4194,27 +4194,27 @@
       </c>
       <c r="F69" s="7" t="inlineStr">
         <is>
-          <t>346,551</t>
+          <t>23,787</t>
         </is>
       </c>
       <c r="G69" s="7" t="inlineStr">
         <is>
-          <t>35,334</t>
+          <t>7,288</t>
         </is>
       </c>
       <c r="H69" s="7" t="inlineStr">
         <is>
-          <t>145,991</t>
+          <t>1,942</t>
         </is>
       </c>
       <c r="I69" s="6" t="inlineStr">
         <is>
-          <t>봉제의복 제조업</t>
+          <t>의료용 기기 제조업</t>
         </is>
       </c>
       <c r="J69" s="6" t="inlineStr">
         <is>
-          <t>미래</t>
+          <t>KB</t>
         </is>
       </c>
       <c r="K69" s="6" t="inlineStr">
@@ -4231,7 +4231,7 @@
       </c>
       <c r="B70" s="6" t="inlineStr">
         <is>
-          <t>브릴스</t>
+          <t>기도산업</t>
         </is>
       </c>
       <c r="C70" s="6" t="inlineStr">
@@ -4251,27 +4251,27 @@
       </c>
       <c r="F70" s="7" t="inlineStr">
         <is>
-          <t>23,759</t>
+          <t>346,551</t>
         </is>
       </c>
       <c r="G70" s="7" t="inlineStr">
         <is>
-          <t>1,744</t>
+          <t>35,334</t>
         </is>
       </c>
       <c r="H70" s="7" t="inlineStr">
         <is>
-          <t>4,785</t>
+          <t>145,991</t>
         </is>
       </c>
       <c r="I70" s="6" t="inlineStr">
         <is>
-          <t>특수 목적용 기계 제조업</t>
+          <t>봉제의복 제조업</t>
         </is>
       </c>
       <c r="J70" s="6" t="inlineStr">
         <is>
-          <t>IBK</t>
+          <t>미래</t>
         </is>
       </c>
       <c r="K70" s="6" t="inlineStr">
@@ -4288,7 +4288,7 @@
       </c>
       <c r="B71" s="6" t="inlineStr">
         <is>
-          <t>와이즈플래닛컴퍼니</t>
+          <t>브릴스</t>
         </is>
       </c>
       <c r="C71" s="6" t="inlineStr">
@@ -4308,27 +4308,27 @@
       </c>
       <c r="F71" s="7" t="inlineStr">
         <is>
-          <t>44,578</t>
+          <t>23,759</t>
         </is>
       </c>
       <c r="G71" s="7" t="inlineStr">
         <is>
-          <t>7,748</t>
+          <t>1,744</t>
         </is>
       </c>
       <c r="H71" s="7" t="inlineStr">
         <is>
-          <t>959</t>
+          <t>4,785</t>
         </is>
       </c>
       <c r="I71" s="6" t="inlineStr">
         <is>
-          <t>광고물 문안, 도안, 설계 등 작성업</t>
+          <t>특수 목적용 기계 제조업</t>
         </is>
       </c>
       <c r="J71" s="6" t="inlineStr">
         <is>
-          <t>대신</t>
+          <t>IBK</t>
         </is>
       </c>
       <c r="K71" s="6" t="inlineStr">
@@ -4340,12 +4340,12 @@
     <row r="72">
       <c r="A72" s="6" t="inlineStr">
         <is>
-          <t>2026-06-24</t>
+          <t>2026-06-25</t>
         </is>
       </c>
       <c r="B72" s="6" t="inlineStr">
         <is>
-          <t>니어스랩</t>
+          <t>와이즈플래닛컴퍼니</t>
         </is>
       </c>
       <c r="C72" s="6" t="inlineStr">
@@ -4365,27 +4365,27 @@
       </c>
       <c r="F72" s="7" t="inlineStr">
         <is>
-          <t>6,361</t>
+          <t>44,578</t>
         </is>
       </c>
       <c r="G72" s="7" t="inlineStr">
         <is>
-          <t>-7,287</t>
+          <t>7,748</t>
         </is>
       </c>
       <c r="H72" s="7" t="inlineStr">
         <is>
-          <t>127</t>
+          <t>959</t>
         </is>
       </c>
       <c r="I72" s="6" t="inlineStr">
         <is>
-          <t>소프트웨어 개발 및 공급업</t>
+          <t>광고물 문안, 도안, 설계 등 작성업</t>
         </is>
       </c>
       <c r="J72" s="6" t="inlineStr">
         <is>
-          <t>삼성</t>
+          <t>대신</t>
         </is>
       </c>
       <c r="K72" s="6" t="inlineStr">
@@ -4402,7 +4402,7 @@
       </c>
       <c r="B73" s="6" t="inlineStr">
         <is>
-          <t>해치텍</t>
+          <t>니어스랩</t>
         </is>
       </c>
       <c r="C73" s="6" t="inlineStr">
@@ -4422,27 +4422,27 @@
       </c>
       <c r="F73" s="7" t="inlineStr">
         <is>
-          <t>14,079</t>
+          <t>6,361</t>
         </is>
       </c>
       <c r="G73" s="7" t="inlineStr">
         <is>
-          <t>-8,009</t>
+          <t>-7,287</t>
         </is>
       </c>
       <c r="H73" s="7" t="inlineStr">
         <is>
-          <t>2,229</t>
+          <t>127</t>
         </is>
       </c>
       <c r="I73" s="6" t="inlineStr">
         <is>
-          <t>반도체 제조업</t>
+          <t>소프트웨어 개발 및 공급업</t>
         </is>
       </c>
       <c r="J73" s="6" t="inlineStr">
         <is>
-          <t>DB</t>
+          <t>삼성</t>
         </is>
       </c>
       <c r="K73" s="6" t="inlineStr">
@@ -4459,7 +4459,7 @@
       </c>
       <c r="B74" s="6" t="inlineStr">
         <is>
-          <t>스카이랩스</t>
+          <t>해치텍</t>
         </is>
       </c>
       <c r="C74" s="6" t="inlineStr">
@@ -4479,27 +4479,27 @@
       </c>
       <c r="F74" s="7" t="inlineStr">
         <is>
-          <t>7,936</t>
+          <t>14,079</t>
         </is>
       </c>
       <c r="G74" s="7" t="inlineStr">
         <is>
-          <t>-62,995</t>
+          <t>-8,009</t>
         </is>
       </c>
       <c r="H74" s="7" t="inlineStr">
         <is>
-          <t>8,341</t>
+          <t>2,229</t>
         </is>
       </c>
       <c r="I74" s="6" t="inlineStr">
         <is>
-          <t>의료용 기기 제조업</t>
+          <t>반도체 제조업</t>
         </is>
       </c>
       <c r="J74" s="6" t="inlineStr">
         <is>
-          <t>한국</t>
+          <t>DB</t>
         </is>
       </c>
       <c r="K74" s="6" t="inlineStr">
@@ -4511,12 +4511,12 @@
     <row r="75">
       <c r="A75" s="6" t="inlineStr">
         <is>
-          <t>2026-06-15</t>
+          <t>2026-06-24</t>
         </is>
       </c>
       <c r="B75" s="6" t="inlineStr">
         <is>
-          <t>에이치엘지노믹스</t>
+          <t>스카이랩스</t>
         </is>
       </c>
       <c r="C75" s="6" t="inlineStr">
@@ -4536,32 +4536,32 @@
       </c>
       <c r="F75" s="7" t="inlineStr">
         <is>
-          <t>28,877</t>
+          <t>7,936</t>
         </is>
       </c>
       <c r="G75" s="7" t="inlineStr">
         <is>
-          <t>8,452</t>
+          <t>-62,995</t>
         </is>
       </c>
       <c r="H75" s="7" t="inlineStr">
         <is>
-          <t>83,552</t>
+          <t>8,341</t>
         </is>
       </c>
       <c r="I75" s="6" t="inlineStr">
         <is>
-          <t>기초 의약물질 제조업</t>
+          <t>의료용 기기 제조업</t>
         </is>
       </c>
       <c r="J75" s="6" t="inlineStr">
         <is>
-          <t>KB, IBK</t>
+          <t>한국</t>
         </is>
       </c>
       <c r="K75" s="6" t="inlineStr">
         <is>
-          <t>상장완료 (2026-07-24)</t>
+          <t>상장전</t>
         </is>
       </c>
     </row>
@@ -4573,7 +4573,7 @@
       </c>
       <c r="B76" s="6" t="inlineStr">
         <is>
-          <t>딜리셔스</t>
+          <t>에이치엘지노믹스</t>
         </is>
       </c>
       <c r="C76" s="6" t="inlineStr">
@@ -4593,44 +4593,44 @@
       </c>
       <c r="F76" s="7" t="inlineStr">
         <is>
-          <t>25,149</t>
+          <t>28,877</t>
         </is>
       </c>
       <c r="G76" s="7" t="inlineStr">
         <is>
-          <t>-20,419</t>
+          <t>8,452</t>
         </is>
       </c>
       <c r="H76" s="7" t="inlineStr">
         <is>
-          <t>-114,384</t>
+          <t>83,552</t>
         </is>
       </c>
       <c r="I76" s="6" t="inlineStr">
         <is>
-          <t>무점포 소매업</t>
+          <t>기초 의약물질 제조업</t>
         </is>
       </c>
       <c r="J76" s="6" t="inlineStr">
         <is>
-          <t>한국</t>
+          <t>KB, IBK</t>
         </is>
       </c>
       <c r="K76" s="6" t="inlineStr">
         <is>
-          <t>상장전</t>
+          <t>상장완료 (2026-07-24)</t>
         </is>
       </c>
     </row>
     <row r="77">
       <c r="A77" s="6" t="inlineStr">
         <is>
-          <t>2026-05-21</t>
+          <t>2026-06-15</t>
         </is>
       </c>
       <c r="B77" s="6" t="inlineStr">
         <is>
-          <t>인제니아테라퓨틱스</t>
+          <t>딜리셔스</t>
         </is>
       </c>
       <c r="C77" s="6" t="inlineStr">
@@ -4650,27 +4650,27 @@
       </c>
       <c r="F77" s="7" t="inlineStr">
         <is>
-          <t>2,588,400</t>
+          <t>25,149</t>
         </is>
       </c>
       <c r="G77" s="7" t="inlineStr">
         <is>
-          <t>15,755,864</t>
+          <t>-20,419</t>
         </is>
       </c>
       <c r="H77" s="7" t="inlineStr">
         <is>
-          <t>30,841,690</t>
+          <t>-114,384</t>
         </is>
       </c>
       <c r="I77" s="6" t="inlineStr">
         <is>
-          <t>자연과학 및 공학 연구개발업</t>
+          <t>무점포 소매업</t>
         </is>
       </c>
       <c r="J77" s="6" t="inlineStr">
         <is>
-          <t>삼성</t>
+          <t>한국</t>
         </is>
       </c>
       <c r="K77" s="6" t="inlineStr">
@@ -4682,12 +4682,12 @@
     <row r="78">
       <c r="A78" s="6" t="inlineStr">
         <is>
-          <t>2026-05-20</t>
+          <t>2026-05-21</t>
         </is>
       </c>
       <c r="B78" s="6" t="inlineStr">
         <is>
-          <t>한국제16호스팩</t>
+          <t>인제니아테라퓨틱스</t>
         </is>
       </c>
       <c r="C78" s="6" t="inlineStr">
@@ -4705,30 +4705,46 @@
           <t>FY25</t>
         </is>
       </c>
-      <c r="F78" s="7" t="inlineStr"/>
-      <c r="G78" s="7" t="inlineStr"/>
-      <c r="H78" s="7" t="inlineStr"/>
-      <c r="I78" s="6" t="inlineStr"/>
+      <c r="F78" s="7" t="inlineStr">
+        <is>
+          <t>2,588,400</t>
+        </is>
+      </c>
+      <c r="G78" s="7" t="inlineStr">
+        <is>
+          <t>15,755,864</t>
+        </is>
+      </c>
+      <c r="H78" s="7" t="inlineStr">
+        <is>
+          <t>30,841,690</t>
+        </is>
+      </c>
+      <c r="I78" s="6" t="inlineStr">
+        <is>
+          <t>자연과학 및 공학 연구개발업</t>
+        </is>
+      </c>
       <c r="J78" s="6" t="inlineStr">
         <is>
-          <t>한국</t>
+          <t>삼성</t>
         </is>
       </c>
       <c r="K78" s="6" t="inlineStr">
         <is>
-          <t>상장완료 (2026-06-30)</t>
+          <t>상장전</t>
         </is>
       </c>
     </row>
     <row r="79">
       <c r="A79" s="6" t="inlineStr">
         <is>
-          <t>2026-05-07</t>
+          <t>2026-05-20</t>
         </is>
       </c>
       <c r="B79" s="6" t="inlineStr">
         <is>
-          <t>레메디</t>
+          <t>한국제16호스팩</t>
         </is>
       </c>
       <c r="C79" s="6" t="inlineStr">
@@ -4746,34 +4762,18 @@
           <t>FY25</t>
         </is>
       </c>
-      <c r="F79" s="7" t="inlineStr">
-        <is>
-          <t>13,441</t>
-        </is>
-      </c>
-      <c r="G79" s="7" t="inlineStr">
-        <is>
-          <t>741</t>
-        </is>
-      </c>
-      <c r="H79" s="7" t="inlineStr">
-        <is>
-          <t>5,870</t>
-        </is>
-      </c>
-      <c r="I79" s="6" t="inlineStr">
-        <is>
-          <t>의료용 기기 제조업</t>
-        </is>
-      </c>
+      <c r="F79" s="7" t="inlineStr"/>
+      <c r="G79" s="7" t="inlineStr"/>
+      <c r="H79" s="7" t="inlineStr"/>
+      <c r="I79" s="6" t="inlineStr"/>
       <c r="J79" s="6" t="inlineStr">
         <is>
-          <t>KB</t>
+          <t>한국</t>
         </is>
       </c>
       <c r="K79" s="6" t="inlineStr">
         <is>
-          <t>상장완료 (2026-07-13)</t>
+          <t>상장완료 (2026-06-30)</t>
         </is>
       </c>
     </row>
@@ -4785,7 +4785,7 @@
       </c>
       <c r="B80" s="6" t="inlineStr">
         <is>
-          <t>케이앤에스아이앤씨</t>
+          <t>레메디</t>
         </is>
       </c>
       <c r="C80" s="6" t="inlineStr">
@@ -4805,44 +4805,44 @@
       </c>
       <c r="F80" s="7" t="inlineStr">
         <is>
-          <t>13,482</t>
+          <t>13,441</t>
         </is>
       </c>
       <c r="G80" s="7" t="inlineStr">
         <is>
-          <t>-2,213</t>
+          <t>741</t>
         </is>
       </c>
       <c r="H80" s="7" t="inlineStr">
         <is>
-          <t>4,273</t>
+          <t>5,870</t>
         </is>
       </c>
       <c r="I80" s="6" t="inlineStr">
         <is>
-          <t>통신 및 방송 장비 제조업</t>
+          <t>의료용 기기 제조업</t>
         </is>
       </c>
       <c r="J80" s="6" t="inlineStr">
         <is>
-          <t>IBK</t>
+          <t>KB</t>
         </is>
       </c>
       <c r="K80" s="6" t="inlineStr">
         <is>
-          <t>상장전</t>
+          <t>상장완료 (2026-07-13)</t>
         </is>
       </c>
     </row>
     <row r="81">
       <c r="A81" s="6" t="inlineStr">
         <is>
-          <t>2026-04-27</t>
+          <t>2026-05-07</t>
         </is>
       </c>
       <c r="B81" s="6" t="inlineStr">
         <is>
-          <t>메리츠제2호스팩</t>
+          <t>케이앤에스아이앤씨</t>
         </is>
       </c>
       <c r="C81" s="6" t="inlineStr">
@@ -4860,30 +4860,46 @@
           <t>FY25</t>
         </is>
       </c>
-      <c r="F81" s="7" t="inlineStr"/>
-      <c r="G81" s="7" t="inlineStr"/>
-      <c r="H81" s="7" t="inlineStr"/>
-      <c r="I81" s="6" t="inlineStr"/>
+      <c r="F81" s="7" t="inlineStr">
+        <is>
+          <t>13,482</t>
+        </is>
+      </c>
+      <c r="G81" s="7" t="inlineStr">
+        <is>
+          <t>-2,213</t>
+        </is>
+      </c>
+      <c r="H81" s="7" t="inlineStr">
+        <is>
+          <t>4,273</t>
+        </is>
+      </c>
+      <c r="I81" s="6" t="inlineStr">
+        <is>
+          <t>통신 및 방송 장비 제조업</t>
+        </is>
+      </c>
       <c r="J81" s="6" t="inlineStr">
         <is>
-          <t>메리츠</t>
+          <t>IBK</t>
         </is>
       </c>
       <c r="K81" s="6" t="inlineStr">
         <is>
-          <t>상장완료 (2026-06-19)</t>
+          <t>상장전</t>
         </is>
       </c>
     </row>
     <row r="82">
       <c r="A82" s="6" t="inlineStr">
         <is>
-          <t>2026-04-23</t>
+          <t>2026-04-27</t>
         </is>
       </c>
       <c r="B82" s="6" t="inlineStr">
         <is>
-          <t>빅웨이브로보틱스</t>
+          <t>메리츠제2호스팩</t>
         </is>
       </c>
       <c r="C82" s="6" t="inlineStr">
@@ -4898,49 +4914,33 @@
       </c>
       <c r="E82" s="6" t="inlineStr">
         <is>
-          <t>FY24</t>
-        </is>
-      </c>
-      <c r="F82" s="7" t="inlineStr">
-        <is>
-          <t>13,851</t>
-        </is>
-      </c>
-      <c r="G82" s="7" t="inlineStr">
-        <is>
-          <t>-5,856</t>
-        </is>
-      </c>
-      <c r="H82" s="7" t="inlineStr">
-        <is>
-          <t>9,470</t>
-        </is>
-      </c>
-      <c r="I82" s="6" t="inlineStr">
-        <is>
-          <t>소프트웨어 개발 및 공급업</t>
-        </is>
-      </c>
+          <t>FY25</t>
+        </is>
+      </c>
+      <c r="F82" s="7" t="inlineStr"/>
+      <c r="G82" s="7" t="inlineStr"/>
+      <c r="H82" s="7" t="inlineStr"/>
+      <c r="I82" s="6" t="inlineStr"/>
       <c r="J82" s="6" t="inlineStr">
         <is>
-          <t>유진, 미래</t>
+          <t>메리츠</t>
         </is>
       </c>
       <c r="K82" s="6" t="inlineStr">
         <is>
-          <t>상장전</t>
+          <t>상장완료 (2026-06-19)</t>
         </is>
       </c>
     </row>
     <row r="83">
       <c r="A83" s="6" t="inlineStr">
         <is>
-          <t>2026-04-09</t>
+          <t>2026-04-23</t>
         </is>
       </c>
       <c r="B83" s="6" t="inlineStr">
         <is>
-          <t>매드업</t>
+          <t>빅웨이브로보틱스</t>
         </is>
       </c>
       <c r="C83" s="6" t="inlineStr">
@@ -4960,44 +4960,44 @@
       </c>
       <c r="F83" s="7" t="inlineStr">
         <is>
-          <t>34,989</t>
+          <t>13,851</t>
         </is>
       </c>
       <c r="G83" s="7" t="inlineStr">
         <is>
-          <t>-2,747</t>
+          <t>-5,856</t>
         </is>
       </c>
       <c r="H83" s="7" t="inlineStr">
         <is>
-          <t>-15,766</t>
+          <t>9,470</t>
         </is>
       </c>
       <c r="I83" s="6" t="inlineStr">
         <is>
-          <t>광고</t>
+          <t>소프트웨어 개발 및 공급업</t>
         </is>
       </c>
       <c r="J83" s="6" t="inlineStr">
         <is>
-          <t>미래</t>
+          <t>유진, 미래</t>
         </is>
       </c>
       <c r="K83" s="6" t="inlineStr">
         <is>
-          <t>상장완료 (2026-07-01)</t>
+          <t>상장전</t>
         </is>
       </c>
     </row>
     <row r="84">
       <c r="A84" s="6" t="inlineStr">
         <is>
-          <t>2026-04-02</t>
+          <t>2026-04-09</t>
         </is>
       </c>
       <c r="B84" s="6" t="inlineStr">
         <is>
-          <t>져스텍</t>
+          <t>매드업</t>
         </is>
       </c>
       <c r="C84" s="6" t="inlineStr">
@@ -5017,32 +5017,32 @@
       </c>
       <c r="F84" s="7" t="inlineStr">
         <is>
-          <t>19,851</t>
+          <t>34,989</t>
         </is>
       </c>
       <c r="G84" s="7" t="inlineStr">
         <is>
-          <t>444</t>
+          <t>-2,747</t>
         </is>
       </c>
       <c r="H84" s="7" t="inlineStr">
         <is>
-          <t>10,953</t>
+          <t>-15,766</t>
         </is>
       </c>
       <c r="I84" s="6" t="inlineStr">
         <is>
-          <t>기계</t>
+          <t>광고</t>
         </is>
       </c>
       <c r="J84" s="6" t="inlineStr">
         <is>
-          <t>삼성</t>
+          <t>미래</t>
         </is>
       </c>
       <c r="K84" s="6" t="inlineStr">
         <is>
-          <t>상장완료 (2026-06-29)</t>
+          <t>상장완료 (2026-07-01)</t>
         </is>
       </c>
     </row>
@@ -5054,7 +5054,7 @@
       </c>
       <c r="B85" s="6" t="inlineStr">
         <is>
-          <t>스트라드비젼</t>
+          <t>져스텍</t>
         </is>
       </c>
       <c r="C85" s="6" t="inlineStr">
@@ -5074,44 +5074,44 @@
       </c>
       <c r="F85" s="7" t="inlineStr">
         <is>
-          <t>11,539</t>
+          <t>19,851</t>
         </is>
       </c>
       <c r="G85" s="7" t="inlineStr">
         <is>
-          <t>-65,529</t>
+          <t>444</t>
         </is>
       </c>
       <c r="H85" s="7" t="inlineStr">
         <is>
-          <t>-245,151</t>
+          <t>10,953</t>
         </is>
       </c>
       <c r="I85" s="6" t="inlineStr">
         <is>
-          <t>소프트웨어</t>
+          <t>기계</t>
         </is>
       </c>
       <c r="J85" s="6" t="inlineStr">
         <is>
-          <t>KB</t>
+          <t>삼성</t>
         </is>
       </c>
       <c r="K85" s="6" t="inlineStr">
         <is>
-          <t>상장완료 (2026-06-30)</t>
+          <t>상장완료 (2026-06-29)</t>
         </is>
       </c>
     </row>
     <row r="86">
       <c r="A86" s="6" t="inlineStr">
         <is>
-          <t>2026-03-30</t>
+          <t>2026-04-02</t>
         </is>
       </c>
       <c r="B86" s="6" t="inlineStr">
         <is>
-          <t>대신밸런스제20호스팩</t>
+          <t>스트라드비젼</t>
         </is>
       </c>
       <c r="C86" s="6" t="inlineStr">
@@ -5126,33 +5126,49 @@
       </c>
       <c r="E86" s="6" t="inlineStr">
         <is>
-          <t>FY25</t>
-        </is>
-      </c>
-      <c r="F86" s="7" t="inlineStr"/>
-      <c r="G86" s="7" t="inlineStr"/>
-      <c r="H86" s="7" t="inlineStr"/>
-      <c r="I86" s="6" t="inlineStr"/>
+          <t>FY24</t>
+        </is>
+      </c>
+      <c r="F86" s="7" t="inlineStr">
+        <is>
+          <t>11,539</t>
+        </is>
+      </c>
+      <c r="G86" s="7" t="inlineStr">
+        <is>
+          <t>-65,529</t>
+        </is>
+      </c>
+      <c r="H86" s="7" t="inlineStr">
+        <is>
+          <t>-245,151</t>
+        </is>
+      </c>
+      <c r="I86" s="6" t="inlineStr">
+        <is>
+          <t>소프트웨어</t>
+        </is>
+      </c>
       <c r="J86" s="6" t="inlineStr">
         <is>
-          <t>대신</t>
+          <t>KB</t>
         </is>
       </c>
       <c r="K86" s="6" t="inlineStr">
         <is>
-          <t>상장완료 (2026-06-05)</t>
+          <t>상장완료 (2026-06-30)</t>
         </is>
       </c>
     </row>
     <row r="87">
       <c r="A87" s="6" t="inlineStr">
         <is>
-          <t>2026-03-26</t>
+          <t>2026-03-30</t>
         </is>
       </c>
       <c r="B87" s="6" t="inlineStr">
         <is>
-          <t>피스피스스튜디오</t>
+          <t>대신밸런스제20호스팩</t>
         </is>
       </c>
       <c r="C87" s="6" t="inlineStr">
@@ -5167,37 +5183,21 @@
       </c>
       <c r="E87" s="6" t="inlineStr">
         <is>
-          <t>FY24</t>
-        </is>
-      </c>
-      <c r="F87" s="7" t="inlineStr">
-        <is>
-          <t>113,777</t>
-        </is>
-      </c>
-      <c r="G87" s="7" t="inlineStr">
-        <is>
-          <t>17,603</t>
-        </is>
-      </c>
-      <c r="H87" s="7" t="inlineStr">
-        <is>
-          <t>55,861</t>
-        </is>
-      </c>
-      <c r="I87" s="6" t="inlineStr">
-        <is>
-          <t>섬유,의류,신발,호화품</t>
-        </is>
-      </c>
+          <t>FY25</t>
+        </is>
+      </c>
+      <c r="F87" s="7" t="inlineStr"/>
+      <c r="G87" s="7" t="inlineStr"/>
+      <c r="H87" s="7" t="inlineStr"/>
+      <c r="I87" s="6" t="inlineStr"/>
       <c r="J87" s="6" t="inlineStr">
         <is>
-          <t>NH, 미래</t>
+          <t>대신</t>
         </is>
       </c>
       <c r="K87" s="6" t="inlineStr">
         <is>
-          <t>상장완료 (2026-06-08)</t>
+          <t>상장완료 (2026-06-05)</t>
         </is>
       </c>
     </row>
@@ -5209,7 +5209,7 @@
       </c>
       <c r="B88" s="6" t="inlineStr">
         <is>
-          <t>폴레드</t>
+          <t>피스피스스튜디오</t>
         </is>
       </c>
       <c r="C88" s="6" t="inlineStr">
@@ -5229,32 +5229,32 @@
       </c>
       <c r="F88" s="7" t="inlineStr">
         <is>
-          <t>52,808</t>
+          <t>113,777</t>
         </is>
       </c>
       <c r="G88" s="7" t="inlineStr">
         <is>
-          <t>543</t>
+          <t>17,603</t>
         </is>
       </c>
       <c r="H88" s="7" t="inlineStr">
         <is>
-          <t>25,416</t>
+          <t>55,861</t>
         </is>
       </c>
       <c r="I88" s="6" t="inlineStr">
         <is>
-          <t>가정용기기와용품</t>
+          <t>섬유,의류,신발,호화품</t>
         </is>
       </c>
       <c r="J88" s="6" t="inlineStr">
         <is>
-          <t>NH</t>
+          <t>NH, 미래</t>
         </is>
       </c>
       <c r="K88" s="6" t="inlineStr">
         <is>
-          <t>상장완료 (2026-05-14)</t>
+          <t>상장완료 (2026-06-08)</t>
         </is>
       </c>
     </row>
@@ -5266,7 +5266,7 @@
       </c>
       <c r="B89" s="6" t="inlineStr">
         <is>
-          <t>레몬헬스케어</t>
+          <t>폴레드</t>
         </is>
       </c>
       <c r="C89" s="6" t="inlineStr">
@@ -5286,44 +5286,44 @@
       </c>
       <c r="F89" s="7" t="inlineStr">
         <is>
-          <t>14,877</t>
+          <t>52,808</t>
         </is>
       </c>
       <c r="G89" s="7" t="inlineStr">
         <is>
-          <t>-2,898</t>
+          <t>543</t>
         </is>
       </c>
       <c r="H89" s="7" t="inlineStr">
         <is>
-          <t>-31,162</t>
+          <t>25,416</t>
         </is>
       </c>
       <c r="I89" s="6" t="inlineStr">
         <is>
-          <t>건강관리업체및서비스</t>
+          <t>가정용기기와용품</t>
         </is>
       </c>
       <c r="J89" s="6" t="inlineStr">
         <is>
-          <t>KB</t>
+          <t>NH</t>
         </is>
       </c>
       <c r="K89" s="6" t="inlineStr">
         <is>
-          <t>상장완료 (2026-07-06)</t>
+          <t>상장완료 (2026-05-14)</t>
         </is>
       </c>
     </row>
     <row r="90">
       <c r="A90" s="6" t="inlineStr">
         <is>
-          <t>2026-02-27</t>
+          <t>2026-03-26</t>
         </is>
       </c>
       <c r="B90" s="6" t="inlineStr">
         <is>
-          <t>마키나락스</t>
+          <t>레몬헬스케어</t>
         </is>
       </c>
       <c r="C90" s="6" t="inlineStr">
@@ -5343,32 +5343,32 @@
       </c>
       <c r="F90" s="7" t="inlineStr">
         <is>
-          <t>8,294</t>
+          <t>14,877</t>
         </is>
       </c>
       <c r="G90" s="7" t="inlineStr">
         <is>
-          <t>-6,073</t>
+          <t>-2,898</t>
         </is>
       </c>
       <c r="H90" s="7" t="inlineStr">
         <is>
-          <t>2,680</t>
+          <t>-31,162</t>
         </is>
       </c>
       <c r="I90" s="6" t="inlineStr">
         <is>
-          <t>소프트웨어</t>
+          <t>건강관리업체및서비스</t>
         </is>
       </c>
       <c r="J90" s="6" t="inlineStr">
         <is>
-          <t>미래</t>
+          <t>KB</t>
         </is>
       </c>
       <c r="K90" s="6" t="inlineStr">
         <is>
-          <t>상장완료 (2026-05-20)</t>
+          <t>상장완료 (2026-07-06)</t>
         </is>
       </c>
     </row>
@@ -5380,7 +5380,7 @@
       </c>
       <c r="B91" s="6" t="inlineStr">
         <is>
-          <t>채비</t>
+          <t>마키나락스</t>
         </is>
       </c>
       <c r="C91" s="6" t="inlineStr">
@@ -5400,44 +5400,44 @@
       </c>
       <c r="F91" s="7" t="inlineStr">
         <is>
-          <t>85,082</t>
+          <t>8,294</t>
         </is>
       </c>
       <c r="G91" s="7" t="inlineStr">
         <is>
-          <t>-54,495</t>
+          <t>-6,073</t>
         </is>
       </c>
       <c r="H91" s="7" t="inlineStr">
         <is>
-          <t>96,866</t>
+          <t>2,680</t>
         </is>
       </c>
       <c r="I91" s="6" t="inlineStr">
         <is>
-          <t>전기제품</t>
+          <t>소프트웨어</t>
         </is>
       </c>
       <c r="J91" s="6" t="inlineStr">
         <is>
-          <t>KB, 삼성, 대신, 하나</t>
+          <t>미래</t>
         </is>
       </c>
       <c r="K91" s="6" t="inlineStr">
         <is>
-          <t>상장완료 (2026-04-29)</t>
+          <t>상장완료 (2026-05-20)</t>
         </is>
       </c>
     </row>
     <row r="92">
       <c r="A92" s="6" t="inlineStr">
         <is>
-          <t>2026-02-10</t>
+          <t>2026-02-27</t>
         </is>
       </c>
       <c r="B92" s="6" t="inlineStr">
         <is>
-          <t>키움히어로제2호스팩</t>
+          <t>채비</t>
         </is>
       </c>
       <c r="C92" s="6" t="inlineStr">
@@ -5455,30 +5455,46 @@
           <t>FY24</t>
         </is>
       </c>
-      <c r="F92" s="7" t="inlineStr"/>
-      <c r="G92" s="7" t="inlineStr"/>
-      <c r="H92" s="7" t="inlineStr"/>
-      <c r="I92" s="6" t="inlineStr"/>
+      <c r="F92" s="7" t="inlineStr">
+        <is>
+          <t>85,082</t>
+        </is>
+      </c>
+      <c r="G92" s="7" t="inlineStr">
+        <is>
+          <t>-54,495</t>
+        </is>
+      </c>
+      <c r="H92" s="7" t="inlineStr">
+        <is>
+          <t>96,866</t>
+        </is>
+      </c>
+      <c r="I92" s="6" t="inlineStr">
+        <is>
+          <t>전기제품</t>
+        </is>
+      </c>
       <c r="J92" s="6" t="inlineStr">
         <is>
-          <t>키움</t>
+          <t>KB, 삼성, 대신, 하나</t>
         </is>
       </c>
       <c r="K92" s="6" t="inlineStr">
         <is>
-          <t>상장완료 (2026-04-23)</t>
+          <t>상장완료 (2026-04-29)</t>
         </is>
       </c>
     </row>
     <row r="93">
       <c r="A93" s="6" t="inlineStr">
         <is>
-          <t>2026-02-05</t>
+          <t>2026-02-10</t>
         </is>
       </c>
       <c r="B93" s="6" t="inlineStr">
         <is>
-          <t>세미티에스</t>
+          <t>키움히어로제2호스팩</t>
         </is>
       </c>
       <c r="C93" s="6" t="inlineStr">
@@ -5488,7 +5504,7 @@
       </c>
       <c r="D93" s="6" t="inlineStr">
         <is>
-          <t>스팩 소멸합병</t>
+          <t>신규상장</t>
         </is>
       </c>
       <c r="E93" s="6" t="inlineStr">
@@ -5496,46 +5512,30 @@
           <t>FY24</t>
         </is>
       </c>
-      <c r="F93" s="7" t="inlineStr">
-        <is>
-          <t>20,808</t>
-        </is>
-      </c>
-      <c r="G93" s="7" t="inlineStr">
-        <is>
-          <t>7,337</t>
-        </is>
-      </c>
-      <c r="H93" s="7" t="inlineStr">
-        <is>
-          <t>26,616</t>
-        </is>
-      </c>
-      <c r="I93" s="6" t="inlineStr">
-        <is>
-          <t>반도체와반도체장비</t>
-        </is>
-      </c>
+      <c r="F93" s="7" t="inlineStr"/>
+      <c r="G93" s="7" t="inlineStr"/>
+      <c r="H93" s="7" t="inlineStr"/>
+      <c r="I93" s="6" t="inlineStr"/>
       <c r="J93" s="6" t="inlineStr">
         <is>
-          <t>NH</t>
+          <t>키움</t>
         </is>
       </c>
       <c r="K93" s="6" t="inlineStr">
         <is>
-          <t>상장완료 (2026-02-05)</t>
+          <t>상장완료 (2026-04-23)</t>
         </is>
       </c>
     </row>
     <row r="94">
       <c r="A94" s="6" t="inlineStr">
         <is>
-          <t>2026-02-02</t>
+          <t>2026-02-05</t>
         </is>
       </c>
       <c r="B94" s="6" t="inlineStr">
         <is>
-          <t>교보20호스팩</t>
+          <t>세미티에스</t>
         </is>
       </c>
       <c r="C94" s="6" t="inlineStr">
@@ -5545,7 +5545,7 @@
       </c>
       <c r="D94" s="6" t="inlineStr">
         <is>
-          <t>신규상장</t>
+          <t>스팩 소멸합병</t>
         </is>
       </c>
       <c r="E94" s="6" t="inlineStr">
@@ -5553,30 +5553,46 @@
           <t>FY24</t>
         </is>
       </c>
-      <c r="F94" s="7" t="inlineStr"/>
-      <c r="G94" s="7" t="inlineStr"/>
-      <c r="H94" s="7" t="inlineStr"/>
-      <c r="I94" s="6" t="inlineStr"/>
+      <c r="F94" s="7" t="inlineStr">
+        <is>
+          <t>20,808</t>
+        </is>
+      </c>
+      <c r="G94" s="7" t="inlineStr">
+        <is>
+          <t>7,337</t>
+        </is>
+      </c>
+      <c r="H94" s="7" t="inlineStr">
+        <is>
+          <t>26,616</t>
+        </is>
+      </c>
+      <c r="I94" s="6" t="inlineStr">
+        <is>
+          <t>반도체와반도체장비</t>
+        </is>
+      </c>
       <c r="J94" s="6" t="inlineStr">
         <is>
-          <t>교보</t>
+          <t>NH</t>
         </is>
       </c>
       <c r="K94" s="6" t="inlineStr">
         <is>
-          <t>상장완료 (2026-04-02)</t>
+          <t>상장완료 (2026-02-05)</t>
         </is>
       </c>
     </row>
     <row r="95">
       <c r="A95" s="6" t="inlineStr">
         <is>
-          <t>2026-01-29</t>
+          <t>2026-02-02</t>
         </is>
       </c>
       <c r="B95" s="6" t="inlineStr">
         <is>
-          <t>케이피항공산업</t>
+          <t>교보20호스팩</t>
         </is>
       </c>
       <c r="C95" s="6" t="inlineStr">
@@ -5586,7 +5602,7 @@
       </c>
       <c r="D95" s="6" t="inlineStr">
         <is>
-          <t>스팩 소멸합병</t>
+          <t>신규상장</t>
         </is>
       </c>
       <c r="E95" s="6" t="inlineStr">
@@ -5594,34 +5610,18 @@
           <t>FY24</t>
         </is>
       </c>
-      <c r="F95" s="7" t="inlineStr">
-        <is>
-          <t>49,651</t>
-        </is>
-      </c>
-      <c r="G95" s="7" t="inlineStr">
-        <is>
-          <t>3,018</t>
-        </is>
-      </c>
-      <c r="H95" s="7" t="inlineStr">
-        <is>
-          <t>15,901</t>
-        </is>
-      </c>
-      <c r="I95" s="6" t="inlineStr">
-        <is>
-          <t>우주항공과국방</t>
-        </is>
-      </c>
+      <c r="F95" s="7" t="inlineStr"/>
+      <c r="G95" s="7" t="inlineStr"/>
+      <c r="H95" s="7" t="inlineStr"/>
+      <c r="I95" s="6" t="inlineStr"/>
       <c r="J95" s="6" t="inlineStr">
         <is>
-          <t>NH</t>
+          <t>교보</t>
         </is>
       </c>
       <c r="K95" s="6" t="inlineStr">
         <is>
-          <t>상장완료 (2026-01-29)</t>
+          <t>상장완료 (2026-04-02)</t>
         </is>
       </c>
     </row>
@@ -5633,7 +5633,7 @@
       </c>
       <c r="B96" s="6" t="inlineStr">
         <is>
-          <t>한패스</t>
+          <t>케이피항공산업</t>
         </is>
       </c>
       <c r="C96" s="6" t="inlineStr">
@@ -5643,7 +5643,7 @@
       </c>
       <c r="D96" s="6" t="inlineStr">
         <is>
-          <t>신규상장</t>
+          <t>스팩 소멸합병</t>
         </is>
       </c>
       <c r="E96" s="6" t="inlineStr">
@@ -5653,44 +5653,44 @@
       </c>
       <c r="F96" s="7" t="inlineStr">
         <is>
-          <t>55,297</t>
+          <t>49,651</t>
         </is>
       </c>
       <c r="G96" s="7" t="inlineStr">
         <is>
-          <t>4,403</t>
+          <t>3,018</t>
         </is>
       </c>
       <c r="H96" s="7" t="inlineStr">
         <is>
-          <t>-28,065</t>
+          <t>15,901</t>
         </is>
       </c>
       <c r="I96" s="6" t="inlineStr">
         <is>
-          <t>IT서비스</t>
+          <t>우주항공과국방</t>
         </is>
       </c>
       <c r="J96" s="6" t="inlineStr">
         <is>
-          <t>한국, 대신</t>
+          <t>NH</t>
         </is>
       </c>
       <c r="K96" s="6" t="inlineStr">
         <is>
-          <t>상장완료 (2026-03-25)</t>
+          <t>상장완료 (2026-01-29)</t>
         </is>
       </c>
     </row>
     <row r="97">
       <c r="A97" s="6" t="inlineStr">
         <is>
-          <t>2026-01-22</t>
+          <t>2026-01-29</t>
         </is>
       </c>
       <c r="B97" s="6" t="inlineStr">
         <is>
-          <t>신한제18호스팩</t>
+          <t>한패스</t>
         </is>
       </c>
       <c r="C97" s="6" t="inlineStr">
@@ -5708,30 +5708,46 @@
           <t>FY24</t>
         </is>
       </c>
-      <c r="F97" s="7" t="inlineStr"/>
-      <c r="G97" s="7" t="inlineStr"/>
-      <c r="H97" s="7" t="inlineStr"/>
-      <c r="I97" s="6" t="inlineStr"/>
+      <c r="F97" s="7" t="inlineStr">
+        <is>
+          <t>55,297</t>
+        </is>
+      </c>
+      <c r="G97" s="7" t="inlineStr">
+        <is>
+          <t>4,403</t>
+        </is>
+      </c>
+      <c r="H97" s="7" t="inlineStr">
+        <is>
+          <t>-28,065</t>
+        </is>
+      </c>
+      <c r="I97" s="6" t="inlineStr">
+        <is>
+          <t>IT서비스</t>
+        </is>
+      </c>
       <c r="J97" s="6" t="inlineStr">
         <is>
-          <t>신한</t>
+          <t>한국, 대신</t>
         </is>
       </c>
       <c r="K97" s="6" t="inlineStr">
         <is>
-          <t>상장완료 (2026-04-30)</t>
+          <t>상장완료 (2026-03-25)</t>
         </is>
       </c>
     </row>
     <row r="98">
       <c r="A98" s="6" t="inlineStr">
         <is>
-          <t>2026-01-20</t>
+          <t>2026-01-22</t>
         </is>
       </c>
       <c r="B98" s="6" t="inlineStr">
         <is>
-          <t>엔에이치스팩33호</t>
+          <t>신한제18호스팩</t>
         </is>
       </c>
       <c r="C98" s="6" t="inlineStr">
@@ -5755,24 +5771,24 @@
       <c r="I98" s="6" t="inlineStr"/>
       <c r="J98" s="6" t="inlineStr">
         <is>
-          <t>NH</t>
+          <t>신한</t>
         </is>
       </c>
       <c r="K98" s="6" t="inlineStr">
         <is>
-          <t>상장완료 (2026-03-27)</t>
+          <t>상장완료 (2026-04-30)</t>
         </is>
       </c>
     </row>
     <row r="99">
       <c r="A99" s="6" t="inlineStr">
         <is>
-          <t>2026-01-19</t>
+          <t>2026-01-20</t>
         </is>
       </c>
       <c r="B99" s="6" t="inlineStr">
         <is>
-          <t>신한제17호스팩</t>
+          <t>엔에이치스팩33호</t>
         </is>
       </c>
       <c r="C99" s="6" t="inlineStr">
@@ -5796,24 +5812,24 @@
       <c r="I99" s="6" t="inlineStr"/>
       <c r="J99" s="6" t="inlineStr">
         <is>
-          <t>신한</t>
+          <t>NH</t>
         </is>
       </c>
       <c r="K99" s="6" t="inlineStr">
         <is>
-          <t>상장완료 (2026-04-01)</t>
+          <t>상장완료 (2026-03-27)</t>
         </is>
       </c>
     </row>
     <row r="100">
       <c r="A100" s="6" t="inlineStr">
         <is>
-          <t>2026-01-16</t>
+          <t>2026-01-19</t>
         </is>
       </c>
       <c r="B100" s="6" t="inlineStr">
         <is>
-          <t>아이엠바이오로직스</t>
+          <t>신한제17호스팩</t>
         </is>
       </c>
       <c r="C100" s="6" t="inlineStr">
@@ -5831,34 +5847,18 @@
           <t>FY24</t>
         </is>
       </c>
-      <c r="F100" s="7" t="inlineStr">
-        <is>
-          <t>27,594</t>
-        </is>
-      </c>
-      <c r="G100" s="7" t="inlineStr">
-        <is>
-          <t>-11,884</t>
-        </is>
-      </c>
-      <c r="H100" s="7" t="inlineStr">
-        <is>
-          <t>-77,202</t>
-        </is>
-      </c>
-      <c r="I100" s="6" t="inlineStr">
-        <is>
-          <t>제약</t>
-        </is>
-      </c>
+      <c r="F100" s="7" t="inlineStr"/>
+      <c r="G100" s="7" t="inlineStr"/>
+      <c r="H100" s="7" t="inlineStr"/>
+      <c r="I100" s="6" t="inlineStr"/>
       <c r="J100" s="6" t="inlineStr">
         <is>
-          <t>한국, 신한</t>
+          <t>신한</t>
         </is>
       </c>
       <c r="K100" s="6" t="inlineStr">
         <is>
-          <t>상장완료 (2026-03-20)</t>
+          <t>상장완료 (2026-04-01)</t>
         </is>
       </c>
     </row>
@@ -5870,7 +5870,7 @@
       </c>
       <c r="B101" s="6" t="inlineStr">
         <is>
-          <t>에스팀</t>
+          <t>아이엠바이오로직스</t>
         </is>
       </c>
       <c r="C101" s="6" t="inlineStr">
@@ -5890,232 +5890,232 @@
       </c>
       <c r="F101" s="7" t="inlineStr">
         <is>
-          <t>35,574</t>
+          <t>27,594</t>
         </is>
       </c>
       <c r="G101" s="7" t="inlineStr">
         <is>
-          <t>1,372</t>
+          <t>-11,884</t>
         </is>
       </c>
       <c r="H101" s="7" t="inlineStr">
         <is>
-          <t>12,331</t>
+          <t>-77,202</t>
         </is>
       </c>
       <c r="I101" s="6" t="inlineStr">
         <is>
-          <t>광고</t>
+          <t>제약</t>
         </is>
       </c>
       <c r="J101" s="6" t="inlineStr">
         <is>
-          <t>한국</t>
+          <t>한국, 신한</t>
         </is>
       </c>
       <c r="K101" s="6" t="inlineStr">
         <is>
-          <t>상장완료 (2026-03-06)</t>
+          <t>상장완료 (2026-03-20)</t>
         </is>
       </c>
     </row>
     <row r="102">
       <c r="A102" s="6" t="inlineStr">
         <is>
+          <t>2026-01-16</t>
+        </is>
+      </c>
+      <c r="B102" s="6" t="inlineStr">
+        <is>
+          <t>에스팀</t>
+        </is>
+      </c>
+      <c r="C102" s="6" t="inlineStr">
+        <is>
+          <t>코스닥</t>
+        </is>
+      </c>
+      <c r="D102" s="6" t="inlineStr">
+        <is>
+          <t>신규상장</t>
+        </is>
+      </c>
+      <c r="E102" s="6" t="inlineStr">
+        <is>
+          <t>FY24</t>
+        </is>
+      </c>
+      <c r="F102" s="7" t="inlineStr">
+        <is>
+          <t>35,574</t>
+        </is>
+      </c>
+      <c r="G102" s="7" t="inlineStr">
+        <is>
+          <t>1,372</t>
+        </is>
+      </c>
+      <c r="H102" s="7" t="inlineStr">
+        <is>
+          <t>12,331</t>
+        </is>
+      </c>
+      <c r="I102" s="6" t="inlineStr">
+        <is>
+          <t>광고</t>
+        </is>
+      </c>
+      <c r="J102" s="6" t="inlineStr">
+        <is>
+          <t>한국</t>
+        </is>
+      </c>
+      <c r="K102" s="6" t="inlineStr">
+        <is>
+          <t>상장완료 (2026-03-06)</t>
+        </is>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" s="6" t="inlineStr">
+        <is>
           <t>2026-01-12</t>
         </is>
       </c>
-      <c r="B102" s="6" t="inlineStr">
+      <c r="B103" s="6" t="inlineStr">
         <is>
           <t>케이뱅크</t>
         </is>
       </c>
-      <c r="C102" s="6" t="inlineStr">
+      <c r="C103" s="6" t="inlineStr">
         <is>
           <t>유가</t>
         </is>
       </c>
-      <c r="D102" s="6" t="inlineStr">
+      <c r="D103" s="6" t="inlineStr">
         <is>
           <t>신규상장</t>
         </is>
       </c>
-      <c r="E102" s="6" t="inlineStr">
+      <c r="E103" s="6" t="inlineStr">
         <is>
           <t>FY24</t>
         </is>
       </c>
-      <c r="F102" s="7" t="inlineStr">
+      <c r="F103" s="7" t="inlineStr">
         <is>
           <t>1,228,501</t>
         </is>
       </c>
-      <c r="G102" s="7" t="inlineStr">
+      <c r="G103" s="7" t="inlineStr">
         <is>
           <t>128,053</t>
         </is>
       </c>
-      <c r="H102" s="7" t="inlineStr">
+      <c r="H103" s="7" t="inlineStr">
         <is>
           <t>1,995,845</t>
         </is>
       </c>
-      <c r="I102" s="6" t="inlineStr">
+      <c r="I103" s="6" t="inlineStr">
         <is>
           <t>은행</t>
         </is>
       </c>
-      <c r="J102" s="6" t="inlineStr">
+      <c r="J103" s="6" t="inlineStr">
         <is>
           <t>NH, 삼성</t>
         </is>
       </c>
-      <c r="K102" s="6" t="inlineStr">
+      <c r="K103" s="6" t="inlineStr">
         <is>
           <t>상장완료 (2026-03-05)</t>
         </is>
       </c>
     </row>
-    <row r="104">
-      <c r="A104" s="3" t="inlineStr">
+    <row r="105">
+      <c r="A105" s="3" t="inlineStr">
         <is>
           <t>■ 철회·미승인  (17건)</t>
         </is>
       </c>
-      <c r="B104" s="4" t="n"/>
-      <c r="C104" s="4" t="n"/>
-      <c r="D104" s="4" t="n"/>
-      <c r="E104" s="4" t="n"/>
-      <c r="F104" s="4" t="n"/>
-      <c r="G104" s="4" t="n"/>
-      <c r="H104" s="4" t="n"/>
-      <c r="I104" s="4" t="n"/>
-      <c r="J104" s="4" t="n"/>
-      <c r="K104" s="4" t="n"/>
-    </row>
-    <row r="105">
-      <c r="A105" s="5" t="inlineStr">
+      <c r="B105" s="4" t="n"/>
+      <c r="C105" s="4" t="n"/>
+      <c r="D105" s="4" t="n"/>
+      <c r="E105" s="4" t="n"/>
+      <c r="F105" s="4" t="n"/>
+      <c r="G105" s="4" t="n"/>
+      <c r="H105" s="4" t="n"/>
+      <c r="I105" s="4" t="n"/>
+      <c r="J105" s="4" t="n"/>
+      <c r="K105" s="4" t="n"/>
+    </row>
+    <row r="106">
+      <c r="A106" s="5" t="inlineStr">
         <is>
           <t>일자</t>
         </is>
       </c>
-      <c r="B105" s="5" t="inlineStr">
+      <c r="B106" s="5" t="inlineStr">
         <is>
           <t>회사명</t>
         </is>
       </c>
-      <c r="C105" s="5" t="inlineStr">
+      <c r="C106" s="5" t="inlineStr">
         <is>
           <t>시장</t>
         </is>
       </c>
-      <c r="D105" s="5" t="inlineStr">
+      <c r="D106" s="5" t="inlineStr">
         <is>
           <t>상장유형</t>
         </is>
       </c>
-      <c r="E105" s="5" t="inlineStr">
+      <c r="E106" s="5" t="inlineStr">
         <is>
           <t>기준연도</t>
         </is>
       </c>
-      <c r="F105" s="5" t="inlineStr">
+      <c r="F106" s="5" t="inlineStr">
         <is>
           <t>매출액</t>
         </is>
       </c>
-      <c r="G105" s="5" t="inlineStr">
+      <c r="G106" s="5" t="inlineStr">
         <is>
           <t>순이익</t>
         </is>
       </c>
-      <c r="H105" s="5" t="inlineStr">
+      <c r="H106" s="5" t="inlineStr">
         <is>
           <t>자기자본</t>
         </is>
       </c>
-      <c r="I105" s="5" t="inlineStr">
+      <c r="I106" s="5" t="inlineStr">
         <is>
           <t>업종</t>
         </is>
       </c>
-      <c r="J105" s="5" t="inlineStr">
+      <c r="J106" s="5" t="inlineStr">
         <is>
           <t>대표주관사</t>
         </is>
       </c>
-      <c r="K105" s="5" t="inlineStr">
+      <c r="K106" s="5" t="inlineStr">
         <is>
           <t>현황</t>
-        </is>
-      </c>
-    </row>
-    <row r="106">
-      <c r="A106" s="6" t="inlineStr">
-        <is>
-          <t>2026-07-31</t>
-        </is>
-      </c>
-      <c r="B106" s="6" t="inlineStr">
-        <is>
-          <t>씨엠디엘</t>
-        </is>
-      </c>
-      <c r="C106" s="6" t="inlineStr">
-        <is>
-          <t>코스닥</t>
-        </is>
-      </c>
-      <c r="D106" s="6" t="inlineStr">
-        <is>
-          <t>스팩 소멸합병</t>
-        </is>
-      </c>
-      <c r="E106" s="6" t="inlineStr">
-        <is>
-          <t>FY24</t>
-        </is>
-      </c>
-      <c r="F106" s="7" t="inlineStr">
-        <is>
-          <t>39,991</t>
-        </is>
-      </c>
-      <c r="G106" s="7" t="inlineStr">
-        <is>
-          <t>3,541</t>
-        </is>
-      </c>
-      <c r="H106" s="7" t="inlineStr">
-        <is>
-          <t>503</t>
-        </is>
-      </c>
-      <c r="I106" s="6" t="inlineStr">
-        <is>
-          <t>기타 기초 유기 화학물질 제조업</t>
-        </is>
-      </c>
-      <c r="J106" s="6" t="inlineStr">
-        <is>
-          <t>교보</t>
-        </is>
-      </c>
-      <c r="K106" s="6" t="inlineStr">
-        <is>
-          <t>심사 철회</t>
         </is>
       </c>
     </row>
     <row r="107">
       <c r="A107" s="6" t="inlineStr">
         <is>
-          <t>2026-07-23</t>
+          <t>2026-07-31</t>
         </is>
       </c>
       <c r="B107" s="6" t="inlineStr">
         <is>
-          <t>모비어스</t>
+          <t>씨엠디엘</t>
         </is>
       </c>
       <c r="C107" s="6" t="inlineStr">
@@ -6125,37 +6125,37 @@
       </c>
       <c r="D107" s="6" t="inlineStr">
         <is>
-          <t>신규상장</t>
+          <t>스팩 소멸합병</t>
         </is>
       </c>
       <c r="E107" s="6" t="inlineStr">
         <is>
-          <t>FY25</t>
+          <t>FY24</t>
         </is>
       </c>
       <c r="F107" s="7" t="inlineStr">
         <is>
-          <t>31,989</t>
+          <t>39,991</t>
         </is>
       </c>
       <c r="G107" s="7" t="inlineStr">
         <is>
-          <t>-45,307</t>
+          <t>3,541</t>
         </is>
       </c>
       <c r="H107" s="7" t="inlineStr">
         <is>
-          <t>-96,707</t>
+          <t>503</t>
         </is>
       </c>
       <c r="I107" s="6" t="inlineStr">
         <is>
-          <t>컴퓨터 프로그래밍, 시스템 통합 및 관리업</t>
+          <t>기타 기초 유기 화학물질 제조업</t>
         </is>
       </c>
       <c r="J107" s="6" t="inlineStr">
         <is>
-          <t>미래</t>
+          <t>교보</t>
         </is>
       </c>
       <c r="K107" s="6" t="inlineStr">
@@ -6167,12 +6167,12 @@
     <row r="108">
       <c r="A108" s="6" t="inlineStr">
         <is>
-          <t>2026-06-16</t>
+          <t>2026-07-23</t>
         </is>
       </c>
       <c r="B108" s="6" t="inlineStr">
         <is>
-          <t>넥스트젠바이오</t>
+          <t>모비어스</t>
         </is>
       </c>
       <c r="C108" s="6" t="inlineStr">
@@ -6187,32 +6187,32 @@
       </c>
       <c r="E108" s="6" t="inlineStr">
         <is>
-          <t>FY24</t>
+          <t>FY25</t>
         </is>
       </c>
       <c r="F108" s="7" t="inlineStr">
         <is>
-          <t>100</t>
+          <t>31,989</t>
         </is>
       </c>
       <c r="G108" s="7" t="inlineStr">
         <is>
-          <t>69</t>
+          <t>-45,307</t>
         </is>
       </c>
       <c r="H108" s="7" t="inlineStr">
         <is>
-          <t>4,792</t>
+          <t>-96,707</t>
         </is>
       </c>
       <c r="I108" s="6" t="inlineStr">
         <is>
-          <t>자연과학 및 공학 연구개발업</t>
+          <t>컴퓨터 프로그래밍, 시스템 통합 및 관리업</t>
         </is>
       </c>
       <c r="J108" s="6" t="inlineStr">
         <is>
-          <t>한국</t>
+          <t>미래</t>
         </is>
       </c>
       <c r="K108" s="6" t="inlineStr">
@@ -6224,12 +6224,12 @@
     <row r="109">
       <c r="A109" s="6" t="inlineStr">
         <is>
-          <t>2026-06-15</t>
+          <t>2026-06-16</t>
         </is>
       </c>
       <c r="B109" s="6" t="inlineStr">
         <is>
-          <t>파워큐브세미</t>
+          <t>넥스트젠바이오</t>
         </is>
       </c>
       <c r="C109" s="6" t="inlineStr">
@@ -6244,32 +6244,32 @@
       </c>
       <c r="E109" s="6" t="inlineStr">
         <is>
-          <t>FY25</t>
+          <t>FY24</t>
         </is>
       </c>
       <c r="F109" s="7" t="inlineStr">
         <is>
-          <t>10,341</t>
+          <t>100</t>
         </is>
       </c>
       <c r="G109" s="7" t="inlineStr">
         <is>
-          <t>-10,837</t>
+          <t>69</t>
         </is>
       </c>
       <c r="H109" s="7" t="inlineStr">
         <is>
-          <t>841</t>
+          <t>4,792</t>
         </is>
       </c>
       <c r="I109" s="6" t="inlineStr">
         <is>
-          <t>반도체 제조업</t>
+          <t>자연과학 및 공학 연구개발업</t>
         </is>
       </c>
       <c r="J109" s="6" t="inlineStr">
         <is>
-          <t>하나, BNK</t>
+          <t>한국</t>
         </is>
       </c>
       <c r="K109" s="6" t="inlineStr">
@@ -6281,12 +6281,12 @@
     <row r="110">
       <c r="A110" s="6" t="inlineStr">
         <is>
-          <t>2026-05-29</t>
+          <t>2026-06-15</t>
         </is>
       </c>
       <c r="B110" s="6" t="inlineStr">
         <is>
-          <t>제이피이노베이션</t>
+          <t>파워큐브세미</t>
         </is>
       </c>
       <c r="C110" s="6" t="inlineStr">
@@ -6306,27 +6306,27 @@
       </c>
       <c r="F110" s="7" t="inlineStr">
         <is>
-          <t>56,324</t>
+          <t>10,341</t>
         </is>
       </c>
       <c r="G110" s="7" t="inlineStr">
         <is>
-          <t>5,588</t>
+          <t>-10,837</t>
         </is>
       </c>
       <c r="H110" s="7" t="inlineStr">
         <is>
-          <t>3,684</t>
+          <t>841</t>
         </is>
       </c>
       <c r="I110" s="6" t="inlineStr">
         <is>
-          <t>특수 목적용 기계 제조업</t>
+          <t>반도체 제조업</t>
         </is>
       </c>
       <c r="J110" s="6" t="inlineStr">
         <is>
-          <t>삼성</t>
+          <t>하나, BNK</t>
         </is>
       </c>
       <c r="K110" s="6" t="inlineStr">
@@ -6338,12 +6338,12 @@
     <row r="111">
       <c r="A111" s="6" t="inlineStr">
         <is>
-          <t>2026-05-26</t>
+          <t>2026-05-29</t>
         </is>
       </c>
       <c r="B111" s="6" t="inlineStr">
         <is>
-          <t>케이솔루션</t>
+          <t>제이피이노베이션</t>
         </is>
       </c>
       <c r="C111" s="6" t="inlineStr">
@@ -6353,7 +6353,7 @@
       </c>
       <c r="D111" s="6" t="inlineStr">
         <is>
-          <t>스팩 존속합병</t>
+          <t>신규상장</t>
         </is>
       </c>
       <c r="E111" s="6" t="inlineStr">
@@ -6363,27 +6363,27 @@
       </c>
       <c r="F111" s="7" t="inlineStr">
         <is>
-          <t>34,565</t>
+          <t>56,324</t>
         </is>
       </c>
       <c r="G111" s="7" t="inlineStr">
         <is>
-          <t>1,158</t>
+          <t>5,588</t>
         </is>
       </c>
       <c r="H111" s="7" t="inlineStr">
         <is>
-          <t>653</t>
+          <t>3,684</t>
         </is>
       </c>
       <c r="I111" s="6" t="inlineStr">
         <is>
-          <t>차체 및 특장차 제조업</t>
+          <t>특수 목적용 기계 제조업</t>
         </is>
       </c>
       <c r="J111" s="6" t="inlineStr">
         <is>
-          <t>DB</t>
+          <t>삼성</t>
         </is>
       </c>
       <c r="K111" s="6" t="inlineStr">
@@ -6395,12 +6395,12 @@
     <row r="112">
       <c r="A112" s="6" t="inlineStr">
         <is>
-          <t>2026-04-30</t>
+          <t>2026-05-26</t>
         </is>
       </c>
       <c r="B112" s="6" t="inlineStr">
         <is>
-          <t>디토닉</t>
+          <t>케이솔루션</t>
         </is>
       </c>
       <c r="C112" s="6" t="inlineStr">
@@ -6410,37 +6410,37 @@
       </c>
       <c r="D112" s="6" t="inlineStr">
         <is>
-          <t>신규상장</t>
+          <t>스팩 존속합병</t>
         </is>
       </c>
       <c r="E112" s="6" t="inlineStr">
         <is>
-          <t>FY24</t>
+          <t>FY25</t>
         </is>
       </c>
       <c r="F112" s="7" t="inlineStr">
         <is>
-          <t>31,293</t>
+          <t>34,565</t>
         </is>
       </c>
       <c r="G112" s="7" t="inlineStr">
         <is>
-          <t>-1,633</t>
+          <t>1,158</t>
         </is>
       </c>
       <c r="H112" s="7" t="inlineStr">
         <is>
-          <t>-21,926</t>
+          <t>653</t>
         </is>
       </c>
       <c r="I112" s="6" t="inlineStr">
         <is>
-          <t>소프트웨어 개발 및 공급업</t>
+          <t>차체 및 특장차 제조업</t>
         </is>
       </c>
       <c r="J112" s="6" t="inlineStr">
         <is>
-          <t>NH</t>
+          <t>DB</t>
         </is>
       </c>
       <c r="K112" s="6" t="inlineStr">
@@ -6452,12 +6452,12 @@
     <row r="113">
       <c r="A113" s="6" t="inlineStr">
         <is>
-          <t>2026-04-22</t>
+          <t>2026-04-30</t>
         </is>
       </c>
       <c r="B113" s="6" t="inlineStr">
         <is>
-          <t>에스케이팩</t>
+          <t>디토닉</t>
         </is>
       </c>
       <c r="C113" s="6" t="inlineStr">
@@ -6467,7 +6467,7 @@
       </c>
       <c r="D113" s="6" t="inlineStr">
         <is>
-          <t>스팩 소멸합병</t>
+          <t>신규상장</t>
         </is>
       </c>
       <c r="E113" s="6" t="inlineStr">
@@ -6477,27 +6477,27 @@
       </c>
       <c r="F113" s="7" t="inlineStr">
         <is>
-          <t>27,310</t>
+          <t>31,293</t>
         </is>
       </c>
       <c r="G113" s="7" t="inlineStr">
         <is>
-          <t>2,257</t>
+          <t>-1,633</t>
         </is>
       </c>
       <c r="H113" s="7" t="inlineStr">
         <is>
-          <t>3,207</t>
+          <t>-21,926</t>
         </is>
       </c>
       <c r="I113" s="6" t="inlineStr">
         <is>
-          <t>용기 세척, 포장 및 충전기 제조업</t>
+          <t>소프트웨어 개발 및 공급업</t>
         </is>
       </c>
       <c r="J113" s="6" t="inlineStr">
         <is>
-          <t>교보</t>
+          <t>NH</t>
         </is>
       </c>
       <c r="K113" s="6" t="inlineStr">
@@ -6509,12 +6509,12 @@
     <row r="114">
       <c r="A114" s="6" t="inlineStr">
         <is>
-          <t>2026-04-20</t>
+          <t>2026-04-22</t>
         </is>
       </c>
       <c r="B114" s="6" t="inlineStr">
         <is>
-          <t>메타넷엑스</t>
+          <t>에스케이팩</t>
         </is>
       </c>
       <c r="C114" s="6" t="inlineStr">
@@ -6524,7 +6524,7 @@
       </c>
       <c r="D114" s="6" t="inlineStr">
         <is>
-          <t>신규상장</t>
+          <t>스팩 소멸합병</t>
         </is>
       </c>
       <c r="E114" s="6" t="inlineStr">
@@ -6534,27 +6534,27 @@
       </c>
       <c r="F114" s="7" t="inlineStr">
         <is>
-          <t>244,130</t>
+          <t>27,310</t>
         </is>
       </c>
       <c r="G114" s="7" t="inlineStr">
         <is>
-          <t>13,455</t>
+          <t>2,257</t>
         </is>
       </c>
       <c r="H114" s="7" t="inlineStr">
         <is>
-          <t>9,995</t>
+          <t>3,207</t>
         </is>
       </c>
       <c r="I114" s="6" t="inlineStr">
         <is>
-          <t>컴퓨터 프로그래밍, 시스템 통합 및 관리업</t>
+          <t>용기 세척, 포장 및 충전기 제조업</t>
         </is>
       </c>
       <c r="J114" s="6" t="inlineStr">
         <is>
-          <t>NH</t>
+          <t>교보</t>
         </is>
       </c>
       <c r="K114" s="6" t="inlineStr">
@@ -6566,12 +6566,12 @@
     <row r="115">
       <c r="A115" s="6" t="inlineStr">
         <is>
-          <t>2026-03-17</t>
+          <t>2026-04-20</t>
         </is>
       </c>
       <c r="B115" s="6" t="inlineStr">
         <is>
-          <t>무아스</t>
+          <t>메타넷엑스</t>
         </is>
       </c>
       <c r="C115" s="6" t="inlineStr">
@@ -6581,7 +6581,7 @@
       </c>
       <c r="D115" s="6" t="inlineStr">
         <is>
-          <t>스팩 소멸합병</t>
+          <t>신규상장</t>
         </is>
       </c>
       <c r="E115" s="6" t="inlineStr">
@@ -6591,27 +6591,27 @@
       </c>
       <c r="F115" s="7" t="inlineStr">
         <is>
-          <t>41,813</t>
+          <t>244,130</t>
         </is>
       </c>
       <c r="G115" s="7" t="inlineStr">
         <is>
-          <t>3,903</t>
+          <t>13,455</t>
         </is>
       </c>
       <c r="H115" s="7" t="inlineStr">
         <is>
-          <t>532</t>
+          <t>9,995</t>
         </is>
       </c>
       <c r="I115" s="6" t="inlineStr">
         <is>
-          <t>가정용 전기기기 제조업</t>
+          <t>컴퓨터 프로그래밍, 시스템 통합 및 관리업</t>
         </is>
       </c>
       <c r="J115" s="6" t="inlineStr">
         <is>
-          <t>신한</t>
+          <t>NH</t>
         </is>
       </c>
       <c r="K115" s="6" t="inlineStr">
@@ -6628,7 +6628,7 @@
       </c>
       <c r="B116" s="6" t="inlineStr">
         <is>
-          <t>유빅스테라퓨틱스</t>
+          <t>무아스</t>
         </is>
       </c>
       <c r="C116" s="6" t="inlineStr">
@@ -6638,7 +6638,7 @@
       </c>
       <c r="D116" s="6" t="inlineStr">
         <is>
-          <t>신규상장</t>
+          <t>스팩 소멸합병</t>
         </is>
       </c>
       <c r="E116" s="6" t="inlineStr">
@@ -6648,27 +6648,27 @@
       </c>
       <c r="F116" s="7" t="inlineStr">
         <is>
-          <t>1,071</t>
+          <t>41,813</t>
         </is>
       </c>
       <c r="G116" s="7" t="inlineStr">
         <is>
-          <t>-15,145</t>
+          <t>3,903</t>
         </is>
       </c>
       <c r="H116" s="7" t="inlineStr">
         <is>
-          <t>5,489</t>
+          <t>532</t>
         </is>
       </c>
       <c r="I116" s="6" t="inlineStr">
         <is>
-          <t>자연과학 및 공학 연구개발업</t>
+          <t>가정용 전기기기 제조업</t>
         </is>
       </c>
       <c r="J116" s="6" t="inlineStr">
         <is>
-          <t>대신</t>
+          <t>신한</t>
         </is>
       </c>
       <c r="K116" s="6" t="inlineStr">
@@ -6680,12 +6680,12 @@
     <row r="117">
       <c r="A117" s="6" t="inlineStr">
         <is>
-          <t>2026-03-16</t>
+          <t>2026-03-17</t>
         </is>
       </c>
       <c r="B117" s="6" t="inlineStr">
         <is>
-          <t>코드잇</t>
+          <t>유빅스테라퓨틱스</t>
         </is>
       </c>
       <c r="C117" s="6" t="inlineStr">
@@ -6705,27 +6705,27 @@
       </c>
       <c r="F117" s="7" t="inlineStr">
         <is>
-          <t>30,747</t>
+          <t>1,071</t>
         </is>
       </c>
       <c r="G117" s="7" t="inlineStr">
         <is>
-          <t>6,652</t>
+          <t>-15,145</t>
         </is>
       </c>
       <c r="H117" s="7" t="inlineStr">
         <is>
-          <t>2,403</t>
+          <t>5,489</t>
         </is>
       </c>
       <c r="I117" s="6" t="inlineStr">
         <is>
-          <t>교육지원 서비스업</t>
+          <t>자연과학 및 공학 연구개발업</t>
         </is>
       </c>
       <c r="J117" s="6" t="inlineStr">
         <is>
-          <t>미래</t>
+          <t>대신</t>
         </is>
       </c>
       <c r="K117" s="6" t="inlineStr">
@@ -6737,12 +6737,12 @@
     <row r="118">
       <c r="A118" s="6" t="inlineStr">
         <is>
-          <t>2026-02-05</t>
+          <t>2026-03-16</t>
         </is>
       </c>
       <c r="B118" s="6" t="inlineStr">
         <is>
-          <t>한컴인스페이스</t>
+          <t>코드잇</t>
         </is>
       </c>
       <c r="C118" s="6" t="inlineStr">
@@ -6762,44 +6762,44 @@
       </c>
       <c r="F118" s="7" t="inlineStr">
         <is>
-          <t>23,492</t>
+          <t>30,747</t>
         </is>
       </c>
       <c r="G118" s="7" t="inlineStr">
         <is>
-          <t>-3,104</t>
+          <t>6,652</t>
         </is>
       </c>
       <c r="H118" s="7" t="inlineStr">
         <is>
-          <t>5,815</t>
+          <t>2,403</t>
         </is>
       </c>
       <c r="I118" s="6" t="inlineStr">
         <is>
-          <t>소프트웨어 개발 및 공급업</t>
+          <t>교육지원 서비스업</t>
         </is>
       </c>
       <c r="J118" s="6" t="inlineStr">
         <is>
-          <t>대신</t>
+          <t>미래</t>
         </is>
       </c>
       <c r="K118" s="6" t="inlineStr">
         <is>
-          <t>심사 미승인</t>
+          <t>심사 철회</t>
         </is>
       </c>
     </row>
     <row r="119">
       <c r="A119" s="6" t="inlineStr">
         <is>
-          <t>2026-01-28</t>
+          <t>2026-02-05</t>
         </is>
       </c>
       <c r="B119" s="6" t="inlineStr">
         <is>
-          <t>크몽</t>
+          <t>한컴인스페이스</t>
         </is>
       </c>
       <c r="C119" s="6" t="inlineStr">
@@ -6819,44 +6819,44 @@
       </c>
       <c r="F119" s="7" t="inlineStr">
         <is>
-          <t>48,572</t>
+          <t>23,492</t>
         </is>
       </c>
       <c r="G119" s="7" t="inlineStr">
         <is>
-          <t>3,988</t>
+          <t>-3,104</t>
         </is>
       </c>
       <c r="H119" s="7" t="inlineStr">
         <is>
-          <t>4,930</t>
+          <t>5,815</t>
         </is>
       </c>
       <c r="I119" s="6" t="inlineStr">
         <is>
-          <t>기타 정보 서비스업</t>
+          <t>소프트웨어 개발 및 공급업</t>
         </is>
       </c>
       <c r="J119" s="6" t="inlineStr">
         <is>
-          <t>삼성</t>
+          <t>대신</t>
         </is>
       </c>
       <c r="K119" s="6" t="inlineStr">
         <is>
-          <t>심사 철회</t>
+          <t>심사 미승인</t>
         </is>
       </c>
     </row>
     <row r="120">
       <c r="A120" s="6" t="inlineStr">
         <is>
-          <t>2026-01-27</t>
+          <t>2026-01-28</t>
         </is>
       </c>
       <c r="B120" s="6" t="inlineStr">
         <is>
-          <t>한화플러스제6호스팩</t>
+          <t>크몽</t>
         </is>
       </c>
       <c r="C120" s="6" t="inlineStr">
@@ -6876,27 +6876,27 @@
       </c>
       <c r="F120" s="7" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>48,572</t>
         </is>
       </c>
       <c r="G120" s="7" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>3,988</t>
         </is>
       </c>
       <c r="H120" s="7" t="inlineStr">
         <is>
-          <t>41</t>
+          <t>4,930</t>
         </is>
       </c>
       <c r="I120" s="6" t="inlineStr">
         <is>
-          <t>기타 금융업</t>
+          <t>기타 정보 서비스업</t>
         </is>
       </c>
       <c r="J120" s="6" t="inlineStr">
         <is>
-          <t>한화</t>
+          <t>삼성</t>
         </is>
       </c>
       <c r="K120" s="6" t="inlineStr">
@@ -6908,17 +6908,17 @@
     <row r="121">
       <c r="A121" s="6" t="inlineStr">
         <is>
-          <t>2026-01-26</t>
+          <t>2026-01-27</t>
         </is>
       </c>
       <c r="B121" s="6" t="inlineStr">
         <is>
-          <t>에식스솔루션즈</t>
+          <t>한화플러스제6호스팩</t>
         </is>
       </c>
       <c r="C121" s="6" t="inlineStr">
         <is>
-          <t>유가</t>
+          <t>코스닥</t>
         </is>
       </c>
       <c r="D121" s="6" t="inlineStr">
@@ -6933,27 +6933,27 @@
       </c>
       <c r="F121" s="7" t="inlineStr">
         <is>
-          <t>2,461</t>
+          <t>-</t>
         </is>
       </c>
       <c r="G121" s="7" t="inlineStr">
         <is>
-          <t>46</t>
+          <t>-</t>
         </is>
       </c>
       <c r="H121" s="7" t="inlineStr">
         <is>
-          <t>200</t>
+          <t>41</t>
         </is>
       </c>
       <c r="I121" s="6" t="inlineStr">
         <is>
-          <t>절연선 및 케이블 제조업</t>
+          <t>기타 금융업</t>
         </is>
       </c>
       <c r="J121" s="6" t="inlineStr">
         <is>
-          <t>한국, 미래</t>
+          <t>한화</t>
         </is>
       </c>
       <c r="K121" s="6" t="inlineStr">
@@ -6965,55 +6965,112 @@
     <row r="122">
       <c r="A122" s="6" t="inlineStr">
         <is>
+          <t>2026-01-26</t>
+        </is>
+      </c>
+      <c r="B122" s="6" t="inlineStr">
+        <is>
+          <t>에식스솔루션즈</t>
+        </is>
+      </c>
+      <c r="C122" s="6" t="inlineStr">
+        <is>
+          <t>유가</t>
+        </is>
+      </c>
+      <c r="D122" s="6" t="inlineStr">
+        <is>
+          <t>신규상장</t>
+        </is>
+      </c>
+      <c r="E122" s="6" t="inlineStr">
+        <is>
+          <t>FY24</t>
+        </is>
+      </c>
+      <c r="F122" s="7" t="inlineStr">
+        <is>
+          <t>2,461</t>
+        </is>
+      </c>
+      <c r="G122" s="7" t="inlineStr">
+        <is>
+          <t>46</t>
+        </is>
+      </c>
+      <c r="H122" s="7" t="inlineStr">
+        <is>
+          <t>200</t>
+        </is>
+      </c>
+      <c r="I122" s="6" t="inlineStr">
+        <is>
+          <t>절연선 및 케이블 제조업</t>
+        </is>
+      </c>
+      <c r="J122" s="6" t="inlineStr">
+        <is>
+          <t>한국, 미래</t>
+        </is>
+      </c>
+      <c r="K122" s="6" t="inlineStr">
+        <is>
+          <t>심사 철회</t>
+        </is>
+      </c>
+    </row>
+    <row r="123">
+      <c r="A123" s="6" t="inlineStr">
+        <is>
           <t>2026-01-23</t>
         </is>
       </c>
-      <c r="B122" s="6" t="inlineStr">
+      <c r="B123" s="6" t="inlineStr">
         <is>
           <t>에코크레이션</t>
         </is>
       </c>
-      <c r="C122" s="6" t="inlineStr">
+      <c r="C123" s="6" t="inlineStr">
         <is>
           <t>코스닥</t>
         </is>
       </c>
-      <c r="D122" s="6" t="inlineStr">
+      <c r="D123" s="6" t="inlineStr">
         <is>
           <t>신규상장</t>
         </is>
       </c>
-      <c r="E122" s="6" t="inlineStr">
+      <c r="E123" s="6" t="inlineStr">
         <is>
           <t>FY24</t>
         </is>
       </c>
-      <c r="F122" s="7" t="inlineStr">
+      <c r="F123" s="7" t="inlineStr">
         <is>
           <t>18,544</t>
         </is>
       </c>
-      <c r="G122" s="7" t="inlineStr">
+      <c r="G123" s="7" t="inlineStr">
         <is>
           <t>-15,634</t>
         </is>
       </c>
-      <c r="H122" s="7" t="inlineStr">
+      <c r="H123" s="7" t="inlineStr">
         <is>
           <t>4,550</t>
         </is>
       </c>
-      <c r="I122" s="6" t="inlineStr">
+      <c r="I123" s="6" t="inlineStr">
         <is>
           <t>일반 목적용 기계 제조업</t>
         </is>
       </c>
-      <c r="J122" s="6" t="inlineStr">
+      <c r="J123" s="6" t="inlineStr">
         <is>
           <t>키움</t>
         </is>
       </c>
-      <c r="K122" s="6" t="inlineStr">
+      <c r="K123" s="6" t="inlineStr">
         <is>
           <t>심사 철회</t>
         </is>
@@ -7030,7 +7087,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R65"/>
+  <dimension ref="A1:R66"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="1"/>
@@ -9828,7 +9885,7 @@
     <row r="40" ht="22" customHeight="1">
       <c r="A40" s="3" t="inlineStr">
         <is>
-          <t>■ 공모 진행 (예심 승인법인)  (21건)</t>
+          <t>■ 공모 진행 (예심 승인법인)  (22건)</t>
         </is>
       </c>
       <c r="B40" s="4" t="n"/>
@@ -10012,17 +10069,25 @@
       </c>
       <c r="E43" s="7" t="inlineStr">
         <is>
-          <t>21,600,000,000</t>
+          <t>26,400,000,000</t>
         </is>
       </c>
       <c r="F43" s="6" t="inlineStr">
         <is>
-          <t>47.97배 (PER)</t>
-        </is>
-      </c>
-      <c r="G43" s="6" t="inlineStr"/>
-      <c r="H43" s="6" t="inlineStr"/>
-      <c r="I43" s="6" t="inlineStr"/>
+          <t>42.08배 (PER)</t>
+        </is>
+      </c>
+      <c r="G43" s="6" t="inlineStr">
+        <is>
+          <t>11,000</t>
+        </is>
+      </c>
+      <c r="H43" s="6" t="n">
+        <v>938.24</v>
+      </c>
+      <c r="I43" s="6" t="n">
+        <v>2024</v>
+      </c>
       <c r="J43" s="6" t="inlineStr">
         <is>
           <t>08-04~08-05</t>
@@ -10049,7 +10114,7 @@
       </c>
       <c r="R43" s="6" t="inlineStr">
         <is>
-          <t>정정</t>
+          <t>발행조건확정</t>
         </is>
       </c>
     </row>
@@ -10248,17 +10313,17 @@
     <row r="47" ht="30" customHeight="1">
       <c r="A47" s="6" t="inlineStr">
         <is>
-          <t>빅웨이브로보틱스</t>
+          <t>스카이랩스</t>
         </is>
       </c>
       <c r="B47" s="6" t="inlineStr">
         <is>
-          <t>08-04~08-10</t>
+          <t>08-14~08-21</t>
         </is>
       </c>
       <c r="C47" s="6" t="inlineStr">
         <is>
-          <t>20,000~24,000</t>
+          <t>13,000~16,000</t>
         </is>
       </c>
       <c r="D47" s="7" t="inlineStr">
@@ -10268,12 +10333,12 @@
       </c>
       <c r="E47" s="7" t="inlineStr">
         <is>
-          <t>40,000,000,000</t>
+          <t>26,000,000,000</t>
         </is>
       </c>
       <c r="F47" s="6" t="inlineStr">
         <is>
-          <t>15.41 (PSR)</t>
+          <t>29.52배 (PER)</t>
         </is>
       </c>
       <c r="G47" s="6" t="inlineStr"/>
@@ -10281,7 +10346,7 @@
       <c r="I47" s="6" t="inlineStr"/>
       <c r="J47" s="6" t="inlineStr">
         <is>
-          <t>08-13~08-14</t>
+          <t>08-26~08-27</t>
         </is>
       </c>
       <c r="K47" s="6" t="inlineStr"/>
@@ -10289,22 +10354,18 @@
       <c r="M47" s="6" t="inlineStr"/>
       <c r="N47" s="6" t="inlineStr">
         <is>
-          <t>유진투자증권</t>
-        </is>
-      </c>
-      <c r="O47" s="6" t="inlineStr">
-        <is>
-          <t>미래</t>
-        </is>
-      </c>
+          <t>한국투자증권</t>
+        </is>
+      </c>
+      <c r="O47" s="6" t="inlineStr"/>
       <c r="P47" s="7" t="inlineStr">
         <is>
-          <t>627,300,000</t>
-        </is>
-      </c>
-      <c r="Q47" s="6" t="inlineStr">
-        <is>
-          <t>3.0%</t>
+          <t>1,071,200,000</t>
+        </is>
+      </c>
+      <c r="Q47" s="18" t="inlineStr">
+        <is>
+          <t>수집예정</t>
         </is>
       </c>
       <c r="R47" s="6" t="inlineStr">
@@ -10316,17 +10377,17 @@
     <row r="48" ht="30" customHeight="1">
       <c r="A48" s="6" t="inlineStr">
         <is>
-          <t>스카이랩스</t>
+          <t>빅웨이브로보틱스</t>
         </is>
       </c>
       <c r="B48" s="6" t="inlineStr">
         <is>
-          <t>08-14~08-21</t>
+          <t>09-07~09-11</t>
         </is>
       </c>
       <c r="C48" s="6" t="inlineStr">
         <is>
-          <t>13,000~16,000</t>
+          <t>20,000~24,000</t>
         </is>
       </c>
       <c r="D48" s="7" t="inlineStr">
@@ -10336,12 +10397,12 @@
       </c>
       <c r="E48" s="7" t="inlineStr">
         <is>
-          <t>26,000,000,000</t>
+          <t>40,000,000,000</t>
         </is>
       </c>
       <c r="F48" s="6" t="inlineStr">
         <is>
-          <t>29.52배 (PER)</t>
+          <t>15.41 (PSR)</t>
         </is>
       </c>
       <c r="G48" s="6" t="inlineStr"/>
@@ -10349,7 +10410,7 @@
       <c r="I48" s="6" t="inlineStr"/>
       <c r="J48" s="6" t="inlineStr">
         <is>
-          <t>08-26~08-27</t>
+          <t>09-16~09-17</t>
         </is>
       </c>
       <c r="K48" s="6" t="inlineStr"/>
@@ -10357,18 +10418,22 @@
       <c r="M48" s="6" t="inlineStr"/>
       <c r="N48" s="6" t="inlineStr">
         <is>
-          <t>한국투자증권</t>
-        </is>
-      </c>
-      <c r="O48" s="6" t="inlineStr"/>
+          <t>유진투자증권</t>
+        </is>
+      </c>
+      <c r="O48" s="6" t="inlineStr">
+        <is>
+          <t>미래</t>
+        </is>
+      </c>
       <c r="P48" s="7" t="inlineStr">
         <is>
-          <t>1,071,200,000</t>
-        </is>
-      </c>
-      <c r="Q48" s="18" t="inlineStr">
-        <is>
-          <t>수집예정</t>
+          <t>627,300,000</t>
+        </is>
+      </c>
+      <c r="Q48" s="6" t="inlineStr">
+        <is>
+          <t>3.0%</t>
         </is>
       </c>
       <c r="R48" s="6" t="inlineStr">
@@ -11209,22 +11274,86 @@
         </is>
       </c>
     </row>
-    <row r="63">
-      <c r="A63" s="20" t="inlineStr">
-        <is>
-          <t>※ 상장 완료 = KIND 신규상장 페이지 기준(스팩합병 포함) · 스팩 공모상장은 밴드·밸류에이션 등 해당없음(공모가 2,000원 고정).</t>
+    <row r="62" ht="30" customHeight="1">
+      <c r="A62" s="6" t="inlineStr">
+        <is>
+          <t>엠비디</t>
+        </is>
+      </c>
+      <c r="B62" s="18" t="inlineStr">
+        <is>
+          <t>수집예정</t>
+        </is>
+      </c>
+      <c r="C62" s="18" t="inlineStr">
+        <is>
+          <t>수집예정</t>
+        </is>
+      </c>
+      <c r="D62" s="18" t="inlineStr">
+        <is>
+          <t>수집예정</t>
+        </is>
+      </c>
+      <c r="E62" s="18" t="inlineStr">
+        <is>
+          <t>수집예정</t>
+        </is>
+      </c>
+      <c r="F62" s="18" t="inlineStr">
+        <is>
+          <t>수집예정</t>
+        </is>
+      </c>
+      <c r="G62" s="6" t="inlineStr"/>
+      <c r="H62" s="6" t="inlineStr"/>
+      <c r="I62" s="6" t="inlineStr"/>
+      <c r="J62" s="18" t="inlineStr">
+        <is>
+          <t>수집예정</t>
+        </is>
+      </c>
+      <c r="K62" s="6" t="inlineStr"/>
+      <c r="L62" s="6" t="inlineStr"/>
+      <c r="M62" s="6" t="inlineStr"/>
+      <c r="N62" s="18" t="inlineStr">
+        <is>
+          <t>수집예정</t>
+        </is>
+      </c>
+      <c r="O62" s="6" t="inlineStr"/>
+      <c r="P62" s="18" t="inlineStr">
+        <is>
+          <t>수집예정</t>
+        </is>
+      </c>
+      <c r="Q62" s="18" t="inlineStr">
+        <is>
+          <t>수집예정</t>
+        </is>
+      </c>
+      <c r="R62" s="6" t="inlineStr">
+        <is>
+          <t>신고서 대기</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" s="20" t="inlineStr">
         <is>
-          <t>※ 기재정정 신고서 내 정정 전·후 병존 → 자동수집은 "정정 후" 값만 취함.</t>
+          <t>※ 상장 완료 = KIND 신규상장 페이지 기준(스팩합병 포함) · 스팩 공모상장은 밴드·밸류에이션 등 해당없음(공모가 2,000원 고정).</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" s="20" t="inlineStr">
+        <is>
+          <t>※ 기재정정 신고서 내 정정 전·후 병존 → 자동수집은 "정정 후" 값만 취함.</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" s="20" t="inlineStr">
         <is>
           <t>※ 청약경쟁률=일반투자자 청약수량÷최종배정수량 · "MM-DD~"는 종료일 자동수집 예정.</t>
         </is>
@@ -11389,7 +11518,7 @@
         <v>14</v>
       </c>
       <c r="C9" s="6" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="D9" s="6" t="n">
         <v>3</v>
@@ -11458,7 +11587,7 @@
         <v>17</v>
       </c>
       <c r="C12" s="6" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="D12" s="6" t="n">
         <v>2</v>
@@ -11572,30 +11701,30 @@
     <row r="20">
       <c r="A20" s="6" t="inlineStr">
         <is>
-          <t>미래에셋증권</t>
+          <t>아이비케이투자증권</t>
         </is>
       </c>
       <c r="B20" s="6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C20" s="6" t="inlineStr">
         <is>
-          <t>42,160,000,000</t>
+          <t>46,200,000,000</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="6" t="inlineStr">
         <is>
-          <t>아이비케이투자증권</t>
+          <t>미래에셋증권</t>
         </is>
       </c>
       <c r="B21" s="6" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C21" s="6" t="inlineStr">
         <is>
-          <t>41,400,000,000</t>
+          <t>42,160,000,000</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore: update IPO data 2026-08-06
</commit_message>
<xml_diff>
--- a/IPO_analysis.xlsx
+++ b/IPO_analysis.xlsx
@@ -10213,7 +10213,7 @@
       </c>
       <c r="R42" s="6" t="inlineStr">
         <is>
-          <t>발행조건확정</t>
+          <t>청약완료·상장대기</t>
         </is>
       </c>
     </row>
@@ -11192,7 +11192,7 @@
     <row r="58" ht="30" customHeight="1">
       <c r="A58" s="6" t="inlineStr">
         <is>
-          <t>멜콘</t>
+          <t>엠에스바이오</t>
         </is>
       </c>
       <c r="B58" s="18" t="inlineStr">
@@ -11249,14 +11249,14 @@
       </c>
       <c r="R58" s="6" t="inlineStr">
         <is>
-          <t>corp_code 미확보(수동확인)</t>
+          <t>신고서 대기</t>
         </is>
       </c>
     </row>
     <row r="59" ht="30" customHeight="1">
       <c r="A59" s="6" t="inlineStr">
         <is>
-          <t>엠에스바이오</t>
+          <t>디티에스</t>
         </is>
       </c>
       <c r="B59" s="18" t="inlineStr">
@@ -11320,7 +11320,7 @@
     <row r="60" ht="30" customHeight="1">
       <c r="A60" s="6" t="inlineStr">
         <is>
-          <t>디티에스</t>
+          <t>에스케이증권제14호기업인수목적</t>
         </is>
       </c>
       <c r="B60" s="18" t="inlineStr">
@@ -11384,7 +11384,7 @@
     <row r="61" ht="30" customHeight="1">
       <c r="A61" s="6" t="inlineStr">
         <is>
-          <t>에스케이증권제14호기업인수목적</t>
+          <t>래블업</t>
         </is>
       </c>
       <c r="B61" s="18" t="inlineStr">
@@ -11448,7 +11448,7 @@
     <row r="62" ht="30" customHeight="1">
       <c r="A62" s="6" t="inlineStr">
         <is>
-          <t>래블업</t>
+          <t>엠비디</t>
         </is>
       </c>
       <c r="B62" s="18" t="inlineStr">
@@ -11512,7 +11512,7 @@
     <row r="63" ht="30" customHeight="1">
       <c r="A63" s="6" t="inlineStr">
         <is>
-          <t>엠비디</t>
+          <t>멜콘</t>
         </is>
       </c>
       <c r="B63" s="18" t="inlineStr">

</xml_diff>

<commit_message>
chore: update IPO data 2026-08-07
</commit_message>
<xml_diff>
--- a/IPO_analysis.xlsx
+++ b/IPO_analysis.xlsx
@@ -618,7 +618,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>기준일 2026-08-06 · 청구일 직전 사업연도 · 별도/개별 재무제표 · 단위 백만원(별도 표기 시 USD)</t>
+          <t>기준일 2026-08-07 · 청구일 직전 사업연도 · 별도/개별 재무제표 · 단위 백만원(별도 표기 시 USD)</t>
         </is>
       </c>
     </row>
@@ -10285,7 +10285,7 @@
       </c>
       <c r="R43" s="6" t="inlineStr">
         <is>
-          <t>발행조건확정</t>
+          <t>청약완료·상장대기</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore: update IPO data 2026-08-11
</commit_message>
<xml_diff>
--- a/IPO_analysis.xlsx
+++ b/IPO_analysis.xlsx
@@ -618,7 +618,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>기준일 2026-08-10 · 청구일 직전 사업연도 · 별도/개별 재무제표 · 단위 백만원(별도 표기 시 USD)</t>
+          <t>기준일 2026-08-11 · 청구일 직전 사업연도 · 별도/개별 재무제표 · 단위 백만원(별도 표기 시 USD)</t>
         </is>
       </c>
     </row>
@@ -5103,7 +5103,7 @@
       </c>
       <c r="K85" s="6" t="inlineStr">
         <is>
-          <t>상장전</t>
+          <t>상장승인(상장예정)</t>
         </is>
       </c>
     </row>
@@ -10409,7 +10409,7 @@
     <row r="45" ht="30" customHeight="1">
       <c r="A45" s="6" t="inlineStr">
         <is>
-          <t>해치텍</t>
+          <t>니어스랩</t>
         </is>
       </c>
       <c r="B45" s="6" t="inlineStr">
@@ -10419,34 +10419,30 @@
       </c>
       <c r="C45" s="6" t="inlineStr">
         <is>
-          <t>23,000~28,000</t>
+          <t>30,000~41,200</t>
         </is>
       </c>
       <c r="D45" s="7" t="inlineStr">
         <is>
-          <t>1,000,000</t>
+          <t>910,000</t>
         </is>
       </c>
       <c r="E45" s="7" t="inlineStr">
         <is>
-          <t>23,000,000,000</t>
+          <t>37,492,000,000</t>
         </is>
       </c>
       <c r="F45" s="6" t="inlineStr">
         <is>
-          <t>36.99배 (PER)</t>
-        </is>
-      </c>
-      <c r="G45" s="6" t="inlineStr">
-        <is>
-          <t>23,000</t>
-        </is>
-      </c>
+          <t>44.41배 (PER)</t>
+        </is>
+      </c>
+      <c r="G45" s="6" t="inlineStr"/>
       <c r="H45" s="6" t="n">
-        <v>101.91</v>
+        <v>743.49</v>
       </c>
       <c r="I45" s="6" t="n">
-        <v>321</v>
+        <v>1795</v>
       </c>
       <c r="J45" s="6" t="inlineStr">
         <is>
@@ -10458,18 +10454,18 @@
       <c r="M45" s="6" t="inlineStr"/>
       <c r="N45" s="6" t="inlineStr">
         <is>
-          <t>DB증권</t>
+          <t>삼성증권</t>
         </is>
       </c>
       <c r="O45" s="6" t="inlineStr"/>
       <c r="P45" s="7" t="inlineStr">
         <is>
-          <t>1,302,950,000</t>
+          <t>1,265,355,000</t>
         </is>
       </c>
       <c r="Q45" s="6" t="inlineStr">
         <is>
-          <t>5.5%</t>
+          <t>4.50%</t>
         </is>
       </c>
       <c r="R45" s="6" t="inlineStr">
@@ -10481,7 +10477,7 @@
     <row r="46" ht="30" customHeight="1">
       <c r="A46" s="6" t="inlineStr">
         <is>
-          <t>니어스랩</t>
+          <t>해치텍</t>
         </is>
       </c>
       <c r="B46" s="6" t="inlineStr">
@@ -10491,27 +10487,35 @@
       </c>
       <c r="C46" s="6" t="inlineStr">
         <is>
-          <t>30,000~41,200</t>
+          <t>23,000~28,000</t>
         </is>
       </c>
       <c r="D46" s="7" t="inlineStr">
         <is>
-          <t>910,000</t>
+          <t>1,000,000</t>
         </is>
       </c>
       <c r="E46" s="7" t="inlineStr">
         <is>
-          <t>27,300,000,000</t>
+          <t>23,000,000,000</t>
         </is>
       </c>
       <c r="F46" s="6" t="inlineStr">
         <is>
-          <t>44.41배 (PER)</t>
-        </is>
-      </c>
-      <c r="G46" s="6" t="inlineStr"/>
-      <c r="H46" s="6" t="inlineStr"/>
-      <c r="I46" s="6" t="inlineStr"/>
+          <t>36.99배 (PER)</t>
+        </is>
+      </c>
+      <c r="G46" s="6" t="inlineStr">
+        <is>
+          <t>23,000</t>
+        </is>
+      </c>
+      <c r="H46" s="6" t="n">
+        <v>101.91</v>
+      </c>
+      <c r="I46" s="6" t="n">
+        <v>321</v>
+      </c>
       <c r="J46" s="6" t="inlineStr">
         <is>
           <t>08-12~08-13</t>
@@ -10522,23 +10526,23 @@
       <c r="M46" s="6" t="inlineStr"/>
       <c r="N46" s="6" t="inlineStr">
         <is>
-          <t>삼성증권</t>
+          <t>DB증권</t>
         </is>
       </c>
       <c r="O46" s="6" t="inlineStr"/>
       <c r="P46" s="7" t="inlineStr">
         <is>
-          <t>1,265,355,000</t>
+          <t>1,302,950,000</t>
         </is>
       </c>
       <c r="Q46" s="6" t="inlineStr">
         <is>
-          <t>4.50%</t>
+          <t>5.5%</t>
         </is>
       </c>
       <c r="R46" s="6" t="inlineStr">
         <is>
-          <t>정정</t>
+          <t>발행조건확정</t>
         </is>
       </c>
     </row>
@@ -12073,7 +12077,7 @@
       </c>
       <c r="C24" s="6" t="inlineStr">
         <is>
-          <t>27,300,060,000</t>
+          <t>37,492,060,000</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore: update IPO data 2026-08-13
</commit_message>
<xml_diff>
--- a/IPO_analysis.xlsx
+++ b/IPO_analysis.xlsx
@@ -618,7 +618,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>기준일 2026-08-12 · 청구일 직전 사업연도 · 별도/개별 재무제표 · 단위 백만원(별도 표기 시 USD)</t>
+          <t>기준일 2026-08-13 · 청구일 직전 사업연도 · 별도/개별 재무제표 · 단위 백만원(별도 표기 시 USD)</t>
         </is>
       </c>
     </row>
@@ -4993,7 +4993,7 @@
       </c>
       <c r="K83" s="6" t="inlineStr">
         <is>
-          <t>상장전</t>
+          <t>상장승인(상장예정)</t>
         </is>
       </c>
     </row>
@@ -5148,7 +5148,7 @@
       </c>
       <c r="K86" s="6" t="inlineStr">
         <is>
-          <t>상장승인(상장예정)</t>
+          <t>상장완료 (2026-08-13)</t>
         </is>
       </c>
     </row>
@@ -7564,7 +7564,7 @@
     <row r="6" ht="22" customHeight="1">
       <c r="A6" s="3" t="inlineStr">
         <is>
-          <t>■ 상장 완료 (2026)  (33건)</t>
+          <t>■ 상장 완료 (2026)  (34건)</t>
         </is>
       </c>
       <c r="B6" s="4" t="n"/>
@@ -7588,44 +7588,44 @@
     <row r="7" ht="30" customHeight="1">
       <c r="A7" s="6" t="inlineStr">
         <is>
-          <t>딜리셔스</t>
+          <t>케이앤에스아이앤씨</t>
         </is>
       </c>
       <c r="B7" s="6" t="inlineStr">
         <is>
-          <t>07-23~07-29</t>
+          <t>07-27~07-31</t>
         </is>
       </c>
       <c r="C7" s="6" t="inlineStr">
         <is>
-          <t>5,000~7,000</t>
+          <t>9,000~11,000</t>
         </is>
       </c>
       <c r="D7" s="7" t="inlineStr">
         <is>
-          <t>2,200,000</t>
+          <t>2,400,000</t>
         </is>
       </c>
       <c r="E7" s="7" t="inlineStr">
         <is>
-          <t>15,400,000,000</t>
+          <t>26,400,000,000</t>
         </is>
       </c>
       <c r="F7" s="6" t="inlineStr">
         <is>
-          <t>23.93배 (PER)</t>
+          <t>42.08배 (PER)</t>
         </is>
       </c>
       <c r="G7" s="6" t="inlineStr">
         <is>
-          <t>7,000</t>
+          <t>11,000</t>
         </is>
       </c>
       <c r="H7" s="6" t="n">
-        <v>184.06</v>
+        <v>938.24</v>
       </c>
       <c r="I7" s="6" t="n">
-        <v>441</v>
+        <v>2024</v>
       </c>
       <c r="J7" s="18" t="inlineStr">
         <is>
@@ -7640,23 +7640,23 @@
       <c r="L7" s="6" t="inlineStr"/>
       <c r="M7" s="6" t="inlineStr">
         <is>
-          <t>2026-08-12</t>
+          <t>2026-08-13</t>
         </is>
       </c>
       <c r="N7" s="6" t="inlineStr">
         <is>
-          <t>한국투자증권</t>
+          <t>아이비케이투자증권</t>
         </is>
       </c>
       <c r="O7" s="6" t="inlineStr"/>
       <c r="P7" s="7" t="inlineStr">
         <is>
-          <t>566,500,000</t>
+          <t>1,500,000,000</t>
         </is>
       </c>
       <c r="Q7" s="6" t="inlineStr">
         <is>
-          <t>5.0%</t>
+          <t>3.5%</t>
         </is>
       </c>
       <c r="R7" s="6" t="inlineStr">
@@ -7668,44 +7668,44 @@
     <row r="8" ht="30" customHeight="1">
       <c r="A8" s="6" t="inlineStr">
         <is>
-          <t>에이치엘지노믹스</t>
+          <t>딜리셔스</t>
         </is>
       </c>
       <c r="B8" s="6" t="inlineStr">
         <is>
-          <t>07-02~07-08</t>
+          <t>07-23~07-29</t>
         </is>
       </c>
       <c r="C8" s="6" t="inlineStr">
         <is>
-          <t>18,500~21,500</t>
+          <t>5,000~7,000</t>
         </is>
       </c>
       <c r="D8" s="7" t="inlineStr">
         <is>
-          <t>2,565,000</t>
+          <t>2,200,000</t>
         </is>
       </c>
       <c r="E8" s="7" t="inlineStr">
         <is>
-          <t>55,147,500,000</t>
+          <t>15,400,000,000</t>
         </is>
       </c>
       <c r="F8" s="6" t="inlineStr">
         <is>
-          <t>12.85배 (EV/EBITDA)</t>
+          <t>23.93배 (PER)</t>
         </is>
       </c>
       <c r="G8" s="6" t="inlineStr">
         <is>
-          <t>21,500</t>
+          <t>7,000</t>
         </is>
       </c>
       <c r="H8" s="6" t="n">
-        <v>714.52</v>
+        <v>184.06</v>
       </c>
       <c r="I8" s="6" t="n">
-        <v>2148</v>
+        <v>441</v>
       </c>
       <c r="J8" s="18" t="inlineStr">
         <is>
@@ -7720,27 +7720,23 @@
       <c r="L8" s="6" t="inlineStr"/>
       <c r="M8" s="6" t="inlineStr">
         <is>
-          <t>2026-07-24</t>
+          <t>2026-08-12</t>
         </is>
       </c>
       <c r="N8" s="6" t="inlineStr">
         <is>
-          <t>KB</t>
-        </is>
-      </c>
-      <c r="O8" s="6" t="inlineStr">
-        <is>
-          <t>아이비케이투자증권, IBK투자증권, IBK투자증권, IBK투자증권, IBK투자증권, IBK투자증권㈜, 보통주, IBK투자증권㈜</t>
-        </is>
-      </c>
+          <t>한국투자증권</t>
+        </is>
+      </c>
+      <c r="O8" s="6" t="inlineStr"/>
       <c r="P8" s="7" t="inlineStr">
         <is>
-          <t>1,211</t>
+          <t>566,500,000</t>
         </is>
       </c>
       <c r="Q8" s="6" t="inlineStr">
         <is>
-          <t>2.5%</t>
+          <t>5.0%</t>
         </is>
       </c>
       <c r="R8" s="6" t="inlineStr">
@@ -7752,63 +7748,59 @@
     <row r="9" ht="30" customHeight="1">
       <c r="A9" s="6" t="inlineStr">
         <is>
-          <t>레메디</t>
-        </is>
-      </c>
-      <c r="B9" s="18" t="inlineStr">
-        <is>
-          <t>수집예정</t>
+          <t>에이치엘지노믹스</t>
+        </is>
+      </c>
+      <c r="B9" s="6" t="inlineStr">
+        <is>
+          <t>07-02~07-08</t>
         </is>
       </c>
       <c r="C9" s="6" t="inlineStr">
         <is>
-          <t>17,800~20,700</t>
+          <t>18,500~21,500</t>
         </is>
       </c>
       <c r="D9" s="7" t="inlineStr">
         <is>
-          <t>1,200,000</t>
+          <t>2,565,000</t>
         </is>
       </c>
       <c r="E9" s="7" t="inlineStr">
         <is>
-          <t>24,840,000,000</t>
+          <t>55,147,500,000</t>
         </is>
       </c>
       <c r="F9" s="6" t="inlineStr">
         <is>
-          <t>21.95배 (PER)</t>
+          <t>12.85배 (EV/EBITDA)</t>
         </is>
       </c>
       <c r="G9" s="6" t="inlineStr">
         <is>
-          <t>20,700</t>
-        </is>
-      </c>
-      <c r="H9" s="6" t="inlineStr">
-        <is>
-          <t>1,146.41</t>
-        </is>
-      </c>
-      <c r="I9" s="6" t="inlineStr">
-        <is>
-          <t>2,246</t>
-        </is>
+          <t>21,500</t>
+        </is>
+      </c>
+      <c r="H9" s="6" t="n">
+        <v>714.52</v>
+      </c>
+      <c r="I9" s="6" t="n">
+        <v>2148</v>
       </c>
       <c r="J9" s="18" t="inlineStr">
         <is>
           <t>수집예정</t>
         </is>
       </c>
-      <c r="K9" s="6" t="inlineStr">
-        <is>
-          <t>1,706.71</t>
+      <c r="K9" s="18" t="inlineStr">
+        <is>
+          <t>수집예정</t>
         </is>
       </c>
       <c r="L9" s="6" t="inlineStr"/>
       <c r="M9" s="6" t="inlineStr">
         <is>
-          <t>2026-07-13</t>
+          <t>2026-07-24</t>
         </is>
       </c>
       <c r="N9" s="6" t="inlineStr">
@@ -7816,15 +7808,19 @@
           <t>KB</t>
         </is>
       </c>
-      <c r="O9" s="6" t="inlineStr"/>
+      <c r="O9" s="6" t="inlineStr">
+        <is>
+          <t>아이비케이투자증권, IBK투자증권, IBK투자증권, IBK투자증권, IBK투자증권, IBK투자증권㈜, 보통주, IBK투자증권㈜</t>
+        </is>
+      </c>
       <c r="P9" s="7" t="inlineStr">
         <is>
-          <t>1,279</t>
+          <t>1,211</t>
         </is>
       </c>
       <c r="Q9" s="6" t="inlineStr">
         <is>
-          <t>5.0%</t>
+          <t>2.5%</t>
         </is>
       </c>
       <c r="R9" s="6" t="inlineStr">
@@ -7836,7 +7832,7 @@
     <row r="10" ht="30" customHeight="1">
       <c r="A10" s="6" t="inlineStr">
         <is>
-          <t>레몬헬스케어</t>
+          <t>레메디</t>
         </is>
       </c>
       <c r="B10" s="18" t="inlineStr">
@@ -7846,45 +7842,53 @@
       </c>
       <c r="C10" s="6" t="inlineStr">
         <is>
-          <t>7,500~10,000</t>
+          <t>17,800~20,700</t>
         </is>
       </c>
       <c r="D10" s="7" t="inlineStr">
         <is>
-          <t>2,000,000</t>
+          <t>1,200,000</t>
         </is>
       </c>
       <c r="E10" s="7" t="inlineStr">
         <is>
-          <t>20,000</t>
+          <t>24,840,000,000</t>
         </is>
       </c>
       <c r="F10" s="6" t="inlineStr">
         <is>
-          <t>25.48배 (PER)</t>
-        </is>
-      </c>
-      <c r="G10" s="6" t="n">
-        <v>10000</v>
-      </c>
-      <c r="H10" s="6" t="n">
-        <v>1238</v>
-      </c>
-      <c r="I10" s="6" t="n">
-        <v>2233</v>
-      </c>
-      <c r="J10" s="6" t="inlineStr">
-        <is>
-          <t>2026-06-24~25</t>
-        </is>
-      </c>
-      <c r="K10" s="6" t="n">
-        <v>1510.57</v>
+          <t>21.95배 (PER)</t>
+        </is>
+      </c>
+      <c r="G10" s="6" t="inlineStr">
+        <is>
+          <t>20,700</t>
+        </is>
+      </c>
+      <c r="H10" s="6" t="inlineStr">
+        <is>
+          <t>1,146.41</t>
+        </is>
+      </c>
+      <c r="I10" s="6" t="inlineStr">
+        <is>
+          <t>2,246</t>
+        </is>
+      </c>
+      <c r="J10" s="18" t="inlineStr">
+        <is>
+          <t>수집예정</t>
+        </is>
+      </c>
+      <c r="K10" s="6" t="inlineStr">
+        <is>
+          <t>1,706.71</t>
+        </is>
       </c>
       <c r="L10" s="6" t="inlineStr"/>
       <c r="M10" s="6" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-07-13</t>
         </is>
       </c>
       <c r="N10" s="6" t="inlineStr">
@@ -7895,12 +7899,12 @@
       <c r="O10" s="6" t="inlineStr"/>
       <c r="P10" s="7" t="inlineStr">
         <is>
-          <t>824</t>
+          <t>1,279</t>
         </is>
       </c>
       <c r="Q10" s="6" t="inlineStr">
         <is>
-          <t>4.0%</t>
+          <t>5.0%</t>
         </is>
       </c>
       <c r="R10" s="6" t="inlineStr">
@@ -7912,7 +7916,7 @@
     <row r="11" ht="30" customHeight="1">
       <c r="A11" s="6" t="inlineStr">
         <is>
-          <t>매드업</t>
+          <t>레몬헬스케어</t>
         </is>
       </c>
       <c r="B11" s="18" t="inlineStr">
@@ -7922,7 +7926,7 @@
       </c>
       <c r="C11" s="6" t="inlineStr">
         <is>
-          <t>7,000~8,000</t>
+          <t>7,500~10,000</t>
         </is>
       </c>
       <c r="D11" s="7" t="inlineStr">
@@ -7932,51 +7936,51 @@
       </c>
       <c r="E11" s="7" t="inlineStr">
         <is>
-          <t>16,000</t>
+          <t>20,000</t>
         </is>
       </c>
       <c r="F11" s="6" t="inlineStr">
         <is>
-          <t>24.57배 (PER)</t>
+          <t>25.48배 (PER)</t>
         </is>
       </c>
       <c r="G11" s="6" t="n">
-        <v>8000</v>
+        <v>10000</v>
       </c>
       <c r="H11" s="6" t="n">
-        <v>1396.29</v>
+        <v>1238</v>
       </c>
       <c r="I11" s="6" t="n">
-        <v>2392</v>
+        <v>2233</v>
       </c>
       <c r="J11" s="6" t="inlineStr">
         <is>
-          <t>2026-06-23~24</t>
+          <t>2026-06-24~25</t>
         </is>
       </c>
       <c r="K11" s="6" t="n">
-        <v>3304.76</v>
+        <v>1510.57</v>
       </c>
       <c r="L11" s="6" t="inlineStr"/>
       <c r="M11" s="6" t="inlineStr">
         <is>
-          <t>2026-07-01</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="N11" s="6" t="inlineStr">
         <is>
-          <t>미래</t>
+          <t>KB</t>
         </is>
       </c>
       <c r="O11" s="6" t="inlineStr"/>
       <c r="P11" s="7" t="inlineStr">
         <is>
-          <t>742</t>
+          <t>824</t>
         </is>
       </c>
       <c r="Q11" s="6" t="inlineStr">
         <is>
-          <t>4.5%</t>
+          <t>4.0%</t>
         </is>
       </c>
       <c r="R11" s="6" t="inlineStr">
@@ -7988,75 +7992,71 @@
     <row r="12" ht="30" customHeight="1">
       <c r="A12" s="6" t="inlineStr">
         <is>
-          <t>한국제16호스팩</t>
-        </is>
-      </c>
-      <c r="B12" s="19" t="inlineStr">
-        <is>
-          <t>해당없음</t>
+          <t>매드업</t>
+        </is>
+      </c>
+      <c r="B12" s="18" t="inlineStr">
+        <is>
+          <t>수집예정</t>
         </is>
       </c>
       <c r="C12" s="6" t="inlineStr">
         <is>
-          <t>2,000</t>
+          <t>7,000~8,000</t>
         </is>
       </c>
       <c r="D12" s="7" t="inlineStr">
         <is>
-          <t>5,500,000</t>
+          <t>2,000,000</t>
         </is>
       </c>
       <c r="E12" s="7" t="inlineStr">
         <is>
-          <t>11,000</t>
-        </is>
-      </c>
-      <c r="F12" s="19" t="inlineStr">
-        <is>
-          <t>해당없음</t>
-        </is>
-      </c>
-      <c r="G12" s="6" t="inlineStr">
-        <is>
-          <t>2,000</t>
-        </is>
+          <t>16,000</t>
+        </is>
+      </c>
+      <c r="F12" s="6" t="inlineStr">
+        <is>
+          <t>24.57배 (PER)</t>
+        </is>
+      </c>
+      <c r="G12" s="6" t="n">
+        <v>8000</v>
       </c>
       <c r="H12" s="6" t="n">
-        <v>1364.09</v>
+        <v>1396.29</v>
       </c>
       <c r="I12" s="6" t="n">
-        <v>2089</v>
+        <v>2392</v>
       </c>
       <c r="J12" s="6" t="inlineStr">
         <is>
-          <t>2026-06-22~06-23</t>
-        </is>
-      </c>
-      <c r="K12" s="6" t="inlineStr">
-        <is>
-          <t>1,274.77</t>
-        </is>
+          <t>2026-06-23~24</t>
+        </is>
+      </c>
+      <c r="K12" s="6" t="n">
+        <v>3304.76</v>
       </c>
       <c r="L12" s="6" t="inlineStr"/>
       <c r="M12" s="6" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-07-01</t>
         </is>
       </c>
       <c r="N12" s="6" t="inlineStr">
         <is>
-          <t>한국</t>
+          <t>미래</t>
         </is>
       </c>
       <c r="O12" s="6" t="inlineStr"/>
       <c r="P12" s="7" t="inlineStr">
         <is>
-          <t>330</t>
+          <t>742</t>
         </is>
       </c>
       <c r="Q12" s="6" t="inlineStr">
         <is>
-          <t>3.00%</t>
+          <t>4.5%</t>
         </is>
       </c>
       <c r="R12" s="6" t="inlineStr">
@@ -8068,51 +8068,53 @@
     <row r="13" ht="30" customHeight="1">
       <c r="A13" s="6" t="inlineStr">
         <is>
-          <t>스트라드비젼</t>
-        </is>
-      </c>
-      <c r="B13" s="18" t="inlineStr">
-        <is>
-          <t>수집예정</t>
+          <t>한국제16호스팩</t>
+        </is>
+      </c>
+      <c r="B13" s="19" t="inlineStr">
+        <is>
+          <t>해당없음</t>
         </is>
       </c>
       <c r="C13" s="6" t="inlineStr">
         <is>
-          <t>12,000~14,000</t>
+          <t>2,000</t>
         </is>
       </c>
       <c r="D13" s="7" t="inlineStr">
         <is>
-          <t>7,000,000</t>
+          <t>5,500,000</t>
         </is>
       </c>
       <c r="E13" s="7" t="inlineStr">
         <is>
-          <t>84,000</t>
-        </is>
-      </c>
-      <c r="F13" s="6" t="inlineStr">
-        <is>
-          <t>37.45배 (PER)</t>
-        </is>
-      </c>
-      <c r="G13" s="6" t="n">
-        <v>12000</v>
+          <t>11,000</t>
+        </is>
+      </c>
+      <c r="F13" s="19" t="inlineStr">
+        <is>
+          <t>해당없음</t>
+        </is>
+      </c>
+      <c r="G13" s="6" t="inlineStr">
+        <is>
+          <t>2,000</t>
+        </is>
       </c>
       <c r="H13" s="6" t="n">
-        <v>381.3</v>
+        <v>1364.09</v>
       </c>
       <c r="I13" s="6" t="n">
-        <v>1604</v>
+        <v>2089</v>
       </c>
       <c r="J13" s="6" t="inlineStr">
         <is>
-          <t>2026-06-18~06-19</t>
+          <t>2026-06-22~06-23</t>
         </is>
       </c>
       <c r="K13" s="6" t="inlineStr">
         <is>
-          <t>45.81</t>
+          <t>1,274.77</t>
         </is>
       </c>
       <c r="L13" s="6" t="inlineStr"/>
@@ -8123,13 +8125,13 @@
       </c>
       <c r="N13" s="6" t="inlineStr">
         <is>
-          <t>KB</t>
+          <t>한국</t>
         </is>
       </c>
       <c r="O13" s="6" t="inlineStr"/>
       <c r="P13" s="7" t="inlineStr">
         <is>
-          <t>2,575</t>
+          <t>330</t>
         </is>
       </c>
       <c r="Q13" s="6" t="inlineStr">
@@ -8146,7 +8148,7 @@
     <row r="14" ht="30" customHeight="1">
       <c r="A14" s="6" t="inlineStr">
         <is>
-          <t>져스텍</t>
+          <t>스트라드비젼</t>
         </is>
       </c>
       <c r="B14" s="18" t="inlineStr">
@@ -8156,32 +8158,32 @@
       </c>
       <c r="C14" s="6" t="inlineStr">
         <is>
-          <t>10,500~12,500</t>
+          <t>12,000~14,000</t>
         </is>
       </c>
       <c r="D14" s="7" t="inlineStr">
         <is>
-          <t>1,600,000</t>
+          <t>7,000,000</t>
         </is>
       </c>
       <c r="E14" s="7" t="inlineStr">
         <is>
-          <t>20,000</t>
+          <t>84,000</t>
         </is>
       </c>
       <c r="F14" s="6" t="inlineStr">
         <is>
-          <t>26.82배 (PER)</t>
+          <t>37.45배 (PER)</t>
         </is>
       </c>
       <c r="G14" s="6" t="n">
-        <v>12500</v>
+        <v>12000</v>
       </c>
       <c r="H14" s="6" t="n">
-        <v>1294.99</v>
+        <v>381.3</v>
       </c>
       <c r="I14" s="6" t="n">
-        <v>2252</v>
+        <v>1604</v>
       </c>
       <c r="J14" s="6" t="inlineStr">
         <is>
@@ -8190,29 +8192,29 @@
       </c>
       <c r="K14" s="6" t="inlineStr">
         <is>
-          <t>2,783.89</t>
+          <t>45.81</t>
         </is>
       </c>
       <c r="L14" s="6" t="inlineStr"/>
       <c r="M14" s="6" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="N14" s="6" t="inlineStr">
         <is>
-          <t>삼성</t>
+          <t>KB</t>
         </is>
       </c>
       <c r="O14" s="6" t="inlineStr"/>
       <c r="P14" s="7" t="inlineStr">
         <is>
-          <t>1,164</t>
+          <t>2,575</t>
         </is>
       </c>
       <c r="Q14" s="6" t="inlineStr">
         <is>
-          <t>5.65%</t>
+          <t>3.00%</t>
         </is>
       </c>
       <c r="R14" s="6" t="inlineStr">
@@ -8224,75 +8226,73 @@
     <row r="15" ht="30" customHeight="1">
       <c r="A15" s="6" t="inlineStr">
         <is>
-          <t>메리츠제2호스팩</t>
-        </is>
-      </c>
-      <c r="B15" s="19" t="inlineStr">
-        <is>
-          <t>해당없음</t>
+          <t>져스텍</t>
+        </is>
+      </c>
+      <c r="B15" s="18" t="inlineStr">
+        <is>
+          <t>수집예정</t>
         </is>
       </c>
       <c r="C15" s="6" t="inlineStr">
         <is>
-          <t>2,000</t>
+          <t>10,500~12,500</t>
         </is>
       </c>
       <c r="D15" s="7" t="inlineStr">
         <is>
-          <t>7,000,000</t>
+          <t>1,600,000</t>
         </is>
       </c>
       <c r="E15" s="7" t="inlineStr">
         <is>
-          <t>14,000</t>
-        </is>
-      </c>
-      <c r="F15" s="19" t="inlineStr">
-        <is>
-          <t>해당없음</t>
-        </is>
-      </c>
-      <c r="G15" s="6" t="inlineStr">
-        <is>
-          <t>2,000</t>
-        </is>
+          <t>20,000</t>
+        </is>
+      </c>
+      <c r="F15" s="6" t="inlineStr">
+        <is>
+          <t>26.82배 (PER)</t>
+        </is>
+      </c>
+      <c r="G15" s="6" t="n">
+        <v>12500</v>
       </c>
       <c r="H15" s="6" t="n">
-        <v>1087.58</v>
+        <v>1294.99</v>
       </c>
       <c r="I15" s="6" t="n">
-        <v>1798</v>
+        <v>2252</v>
       </c>
       <c r="J15" s="6" t="inlineStr">
         <is>
-          <t>2026-06-09~06-10</t>
+          <t>2026-06-18~06-19</t>
         </is>
       </c>
       <c r="K15" s="6" t="inlineStr">
         <is>
-          <t>1,338.66</t>
+          <t>2,783.89</t>
         </is>
       </c>
       <c r="L15" s="6" t="inlineStr"/>
       <c r="M15" s="6" t="inlineStr">
         <is>
-          <t>2026-06-19</t>
+          <t>2026-06-29</t>
         </is>
       </c>
       <c r="N15" s="6" t="inlineStr">
         <is>
-          <t>메리츠</t>
+          <t>삼성</t>
         </is>
       </c>
       <c r="O15" s="6" t="inlineStr"/>
       <c r="P15" s="7" t="inlineStr">
         <is>
-          <t>245</t>
+          <t>1,164</t>
         </is>
       </c>
       <c r="Q15" s="6" t="inlineStr">
         <is>
-          <t>1.75%</t>
+          <t>5.65%</t>
         </is>
       </c>
       <c r="R15" s="6" t="inlineStr">
@@ -8304,77 +8304,75 @@
     <row r="16" ht="30" customHeight="1">
       <c r="A16" s="6" t="inlineStr">
         <is>
-          <t>피스피스스튜디오</t>
-        </is>
-      </c>
-      <c r="B16" s="18" t="inlineStr">
-        <is>
-          <t>수집예정</t>
+          <t>메리츠제2호스팩</t>
+        </is>
+      </c>
+      <c r="B16" s="19" t="inlineStr">
+        <is>
+          <t>해당없음</t>
         </is>
       </c>
       <c r="C16" s="6" t="inlineStr">
         <is>
-          <t>19,000~21,500</t>
+          <t>2,000</t>
         </is>
       </c>
       <c r="D16" s="7" t="inlineStr">
         <is>
-          <t>2,272,637</t>
+          <t>7,000,000</t>
         </is>
       </c>
       <c r="E16" s="7" t="inlineStr">
         <is>
-          <t>48,862</t>
-        </is>
-      </c>
-      <c r="F16" s="6" t="inlineStr">
-        <is>
-          <t>21.48배 (PER)</t>
-        </is>
-      </c>
-      <c r="G16" s="6" t="n">
-        <v>21500</v>
+          <t>14,000</t>
+        </is>
+      </c>
+      <c r="F16" s="19" t="inlineStr">
+        <is>
+          <t>해당없음</t>
+        </is>
+      </c>
+      <c r="G16" s="6" t="inlineStr">
+        <is>
+          <t>2,000</t>
+        </is>
       </c>
       <c r="H16" s="6" t="n">
-        <v>847.76</v>
+        <v>1087.58</v>
       </c>
       <c r="I16" s="6" t="n">
-        <v>2329</v>
+        <v>1798</v>
       </c>
       <c r="J16" s="6" t="inlineStr">
         <is>
-          <t>2026-05-26~05-27</t>
+          <t>2026-06-09~06-10</t>
         </is>
       </c>
       <c r="K16" s="6" t="inlineStr">
         <is>
-          <t>1,191.15</t>
+          <t>1,338.66</t>
         </is>
       </c>
       <c r="L16" s="6" t="inlineStr"/>
       <c r="M16" s="6" t="inlineStr">
         <is>
-          <t>2026-06-08</t>
+          <t>2026-06-19</t>
         </is>
       </c>
       <c r="N16" s="6" t="inlineStr">
         <is>
-          <t>미래</t>
-        </is>
-      </c>
-      <c r="O16" s="6" t="inlineStr">
-        <is>
-          <t>NH</t>
-        </is>
-      </c>
+          <t>메리츠</t>
+        </is>
+      </c>
+      <c r="O16" s="6" t="inlineStr"/>
       <c r="P16" s="7" t="inlineStr">
         <is>
-          <t>1,994</t>
+          <t>245</t>
         </is>
       </c>
       <c r="Q16" s="6" t="inlineStr">
         <is>
-          <t>4.00%</t>
+          <t>1.75%</t>
         </is>
       </c>
       <c r="R16" s="6" t="inlineStr">
@@ -8386,75 +8384,77 @@
     <row r="17" ht="30" customHeight="1">
       <c r="A17" s="6" t="inlineStr">
         <is>
-          <t>대신밸런스제20호스팩</t>
-        </is>
-      </c>
-      <c r="B17" s="19" t="inlineStr">
-        <is>
-          <t>해당없음</t>
+          <t>피스피스스튜디오</t>
+        </is>
+      </c>
+      <c r="B17" s="18" t="inlineStr">
+        <is>
+          <t>수집예정</t>
         </is>
       </c>
       <c r="C17" s="6" t="inlineStr">
         <is>
-          <t>2,000</t>
+          <t>19,000~21,500</t>
         </is>
       </c>
       <c r="D17" s="7" t="inlineStr">
         <is>
-          <t>6,500,000</t>
+          <t>2,272,637</t>
         </is>
       </c>
       <c r="E17" s="7" t="inlineStr">
         <is>
-          <t>13,000</t>
-        </is>
-      </c>
-      <c r="F17" s="19" t="inlineStr">
-        <is>
-          <t>해당없음</t>
-        </is>
-      </c>
-      <c r="G17" s="6" t="inlineStr">
-        <is>
-          <t>2,000</t>
-        </is>
+          <t>48,862</t>
+        </is>
+      </c>
+      <c r="F17" s="6" t="inlineStr">
+        <is>
+          <t>21.48배 (PER)</t>
+        </is>
+      </c>
+      <c r="G17" s="6" t="n">
+        <v>21500</v>
       </c>
       <c r="H17" s="6" t="n">
-        <v>1327.13</v>
+        <v>847.76</v>
       </c>
       <c r="I17" s="6" t="n">
-        <v>2194</v>
+        <v>2329</v>
       </c>
       <c r="J17" s="6" t="inlineStr">
         <is>
-          <t>2026-05-22~05-25</t>
+          <t>2026-05-26~05-27</t>
         </is>
       </c>
       <c r="K17" s="6" t="inlineStr">
         <is>
-          <t>1,486.88</t>
+          <t>1,191.15</t>
         </is>
       </c>
       <c r="L17" s="6" t="inlineStr"/>
       <c r="M17" s="6" t="inlineStr">
         <is>
-          <t>2026-06-05</t>
+          <t>2026-06-08</t>
         </is>
       </c>
       <c r="N17" s="6" t="inlineStr">
         <is>
-          <t>대신</t>
-        </is>
-      </c>
-      <c r="O17" s="6" t="inlineStr"/>
+          <t>미래</t>
+        </is>
+      </c>
+      <c r="O17" s="6" t="inlineStr">
+        <is>
+          <t>NH</t>
+        </is>
+      </c>
       <c r="P17" s="7" t="inlineStr">
         <is>
-          <t>390</t>
+          <t>1,994</t>
         </is>
       </c>
       <c r="Q17" s="6" t="inlineStr">
         <is>
-          <t>3.00%</t>
+          <t>4.00%</t>
         </is>
       </c>
       <c r="R17" s="6" t="inlineStr">
@@ -8466,73 +8466,75 @@
     <row r="18" ht="30" customHeight="1">
       <c r="A18" s="6" t="inlineStr">
         <is>
-          <t>마키나락스</t>
-        </is>
-      </c>
-      <c r="B18" s="18" t="inlineStr">
-        <is>
-          <t>수집예정</t>
+          <t>대신밸런스제20호스팩</t>
+        </is>
+      </c>
+      <c r="B18" s="19" t="inlineStr">
+        <is>
+          <t>해당없음</t>
         </is>
       </c>
       <c r="C18" s="6" t="inlineStr">
         <is>
-          <t>12,500~15,000</t>
+          <t>2,000</t>
         </is>
       </c>
       <c r="D18" s="7" t="inlineStr">
         <is>
-          <t>2,635,000</t>
+          <t>6,500,000</t>
         </is>
       </c>
       <c r="E18" s="7" t="inlineStr">
         <is>
-          <t>39,525</t>
-        </is>
-      </c>
-      <c r="F18" s="6" t="inlineStr">
-        <is>
-          <t>40.5배 (PER)</t>
-        </is>
-      </c>
-      <c r="G18" s="6" t="n">
-        <v>15000</v>
+          <t>13,000</t>
+        </is>
+      </c>
+      <c r="F18" s="19" t="inlineStr">
+        <is>
+          <t>해당없음</t>
+        </is>
+      </c>
+      <c r="G18" s="6" t="inlineStr">
+        <is>
+          <t>2,000</t>
+        </is>
       </c>
       <c r="H18" s="6" t="n">
-        <v>1196.08</v>
+        <v>1327.13</v>
       </c>
       <c r="I18" s="6" t="n">
-        <v>2427</v>
+        <v>2194</v>
       </c>
       <c r="J18" s="6" t="inlineStr">
         <is>
-          <t>2026-05-11~05-12</t>
+          <t>2026-05-22~05-25</t>
         </is>
       </c>
       <c r="K18" s="6" t="inlineStr">
         <is>
-          <t>2,807.79</t>
+          <t>1,486.88</t>
         </is>
       </c>
       <c r="L18" s="6" t="inlineStr"/>
       <c r="M18" s="6" t="inlineStr">
         <is>
-          <t>2026-05-20</t>
+          <t>2026-06-05</t>
         </is>
       </c>
       <c r="N18" s="6" t="inlineStr">
         <is>
-          <t>미래</t>
+          <t>대신</t>
         </is>
       </c>
       <c r="O18" s="6" t="inlineStr"/>
       <c r="P18" s="7" t="inlineStr">
         <is>
-          <t>2,026</t>
+          <t>390</t>
         </is>
       </c>
       <c r="Q18" s="6" t="inlineStr">
         <is>
-          <t>5.00%</t>
+          <t>3.00%</t>
         </is>
       </c>
       <c r="R18" s="6" t="inlineStr">
@@ -8544,7 +8546,7 @@
     <row r="19" ht="30" customHeight="1">
       <c r="A19" s="6" t="inlineStr">
         <is>
-          <t>폴레드</t>
+          <t>마키나락스</t>
         </is>
       </c>
       <c r="B19" s="18" t="inlineStr">
@@ -8554,63 +8556,63 @@
       </c>
       <c r="C19" s="6" t="inlineStr">
         <is>
-          <t>4,100~5,000</t>
+          <t>12,500~15,000</t>
         </is>
       </c>
       <c r="D19" s="7" t="inlineStr">
         <is>
-          <t>2,600,000</t>
+          <t>2,635,000</t>
         </is>
       </c>
       <c r="E19" s="7" t="inlineStr">
         <is>
-          <t>13,000</t>
+          <t>39,525</t>
         </is>
       </c>
       <c r="F19" s="6" t="inlineStr">
         <is>
-          <t>19.05배 (PER)</t>
+          <t>40.5배 (PER)</t>
         </is>
       </c>
       <c r="G19" s="6" t="n">
-        <v>5000</v>
+        <v>15000</v>
       </c>
       <c r="H19" s="6" t="n">
-        <v>1486.66</v>
+        <v>1196.08</v>
       </c>
       <c r="I19" s="6" t="n">
-        <v>2372</v>
+        <v>2427</v>
       </c>
       <c r="J19" s="6" t="inlineStr">
         <is>
-          <t>2026-05-04~05-05</t>
+          <t>2026-05-11~05-12</t>
         </is>
       </c>
       <c r="K19" s="6" t="inlineStr">
         <is>
-          <t>3,169.86</t>
+          <t>2,807.79</t>
         </is>
       </c>
       <c r="L19" s="6" t="inlineStr"/>
       <c r="M19" s="6" t="inlineStr">
         <is>
-          <t>2026-05-14</t>
+          <t>2026-05-20</t>
         </is>
       </c>
       <c r="N19" s="6" t="inlineStr">
         <is>
-          <t>NH</t>
+          <t>미래</t>
         </is>
       </c>
       <c r="O19" s="6" t="inlineStr"/>
       <c r="P19" s="7" t="inlineStr">
         <is>
-          <t>540</t>
+          <t>2,026</t>
         </is>
       </c>
       <c r="Q19" s="6" t="inlineStr">
         <is>
-          <t>4.03%</t>
+          <t>5.00%</t>
         </is>
       </c>
       <c r="R19" s="6" t="inlineStr">
@@ -8622,7 +8624,7 @@
     <row r="20" ht="30" customHeight="1">
       <c r="A20" s="6" t="inlineStr">
         <is>
-          <t>코스모로보틱스</t>
+          <t>폴레드</t>
         </is>
       </c>
       <c r="B20" s="18" t="inlineStr">
@@ -8632,67 +8634,63 @@
       </c>
       <c r="C20" s="6" t="inlineStr">
         <is>
-          <t>5,300~6,000</t>
+          <t>4,100~5,000</t>
         </is>
       </c>
       <c r="D20" s="7" t="inlineStr">
         <is>
-          <t>4,170,000</t>
+          <t>2,600,000</t>
         </is>
       </c>
       <c r="E20" s="7" t="inlineStr">
         <is>
-          <t>25,020</t>
+          <t>13,000</t>
         </is>
       </c>
       <c r="F20" s="6" t="inlineStr">
         <is>
-          <t>47.45배 (PER)</t>
+          <t>19.05배 (PER)</t>
         </is>
       </c>
       <c r="G20" s="6" t="n">
-        <v>6000</v>
+        <v>5000</v>
       </c>
       <c r="H20" s="6" t="n">
-        <v>1140.11</v>
+        <v>1486.66</v>
       </c>
       <c r="I20" s="6" t="n">
-        <v>2257</v>
+        <v>2372</v>
       </c>
       <c r="J20" s="6" t="inlineStr">
         <is>
-          <t>2026-04-27~04-28</t>
+          <t>2026-05-04~05-05</t>
         </is>
       </c>
       <c r="K20" s="6" t="inlineStr">
         <is>
-          <t>2,013.80</t>
+          <t>3,169.86</t>
         </is>
       </c>
       <c r="L20" s="6" t="inlineStr"/>
       <c r="M20" s="6" t="inlineStr">
         <is>
-          <t>2026-05-11</t>
+          <t>2026-05-14</t>
         </is>
       </c>
       <c r="N20" s="6" t="inlineStr">
         <is>
-          <t>유진</t>
-        </is>
-      </c>
-      <c r="O20" s="6" t="inlineStr">
-        <is>
           <t>NH</t>
         </is>
       </c>
+      <c r="O20" s="6" t="inlineStr"/>
       <c r="P20" s="7" t="inlineStr">
         <is>
-          <t>1,289</t>
+          <t>540</t>
         </is>
       </c>
       <c r="Q20" s="6" t="inlineStr">
         <is>
-          <t>3.78%</t>
+          <t>4.03%</t>
         </is>
       </c>
       <c r="R20" s="6" t="inlineStr">
@@ -8704,75 +8702,77 @@
     <row r="21" ht="30" customHeight="1">
       <c r="A21" s="6" t="inlineStr">
         <is>
-          <t>신한스팩18호</t>
-        </is>
-      </c>
-      <c r="B21" s="19" t="inlineStr">
-        <is>
-          <t>해당없음</t>
+          <t>코스모로보틱스</t>
+        </is>
+      </c>
+      <c r="B21" s="18" t="inlineStr">
+        <is>
+          <t>수집예정</t>
         </is>
       </c>
       <c r="C21" s="6" t="inlineStr">
         <is>
-          <t>2,000</t>
+          <t>5,300~6,000</t>
         </is>
       </c>
       <c r="D21" s="7" t="inlineStr">
         <is>
-          <t>5,000,000</t>
+          <t>4,170,000</t>
         </is>
       </c>
       <c r="E21" s="7" t="inlineStr">
         <is>
-          <t>10,000</t>
-        </is>
-      </c>
-      <c r="F21" s="19" t="inlineStr">
-        <is>
-          <t>해당없음</t>
-        </is>
-      </c>
-      <c r="G21" s="6" t="inlineStr">
-        <is>
-          <t>2,000</t>
-        </is>
+          <t>25,020</t>
+        </is>
+      </c>
+      <c r="F21" s="6" t="inlineStr">
+        <is>
+          <t>47.45배 (PER)</t>
+        </is>
+      </c>
+      <c r="G21" s="6" t="n">
+        <v>6000</v>
       </c>
       <c r="H21" s="6" t="n">
-        <v>1388.6</v>
+        <v>1140.11</v>
       </c>
       <c r="I21" s="6" t="n">
-        <v>2044</v>
+        <v>2257</v>
       </c>
       <c r="J21" s="6" t="inlineStr">
         <is>
-          <t>2026-04-20~04-21</t>
+          <t>2026-04-27~04-28</t>
         </is>
       </c>
       <c r="K21" s="6" t="inlineStr">
         <is>
-          <t>1,601.36</t>
+          <t>2,013.80</t>
         </is>
       </c>
       <c r="L21" s="6" t="inlineStr"/>
       <c r="M21" s="6" t="inlineStr">
         <is>
-          <t>2026-04-30</t>
+          <t>2026-05-11</t>
         </is>
       </c>
       <c r="N21" s="6" t="inlineStr">
         <is>
-          <t>신한</t>
-        </is>
-      </c>
-      <c r="O21" s="6" t="inlineStr"/>
+          <t>유진</t>
+        </is>
+      </c>
+      <c r="O21" s="6" t="inlineStr">
+        <is>
+          <t>NH</t>
+        </is>
+      </c>
       <c r="P21" s="7" t="inlineStr">
         <is>
-          <t>350</t>
+          <t>1,289</t>
         </is>
       </c>
       <c r="Q21" s="6" t="inlineStr">
         <is>
-          <t>3.50%</t>
+          <t>3.78%</t>
         </is>
       </c>
       <c r="R21" s="6" t="inlineStr">
@@ -8784,42 +8784,44 @@
     <row r="22" ht="30" customHeight="1">
       <c r="A22" s="6" t="inlineStr">
         <is>
-          <t>채비</t>
-        </is>
-      </c>
-      <c r="B22" s="18" t="inlineStr">
-        <is>
-          <t>수집예정</t>
+          <t>신한스팩18호</t>
+        </is>
+      </c>
+      <c r="B22" s="19" t="inlineStr">
+        <is>
+          <t>해당없음</t>
         </is>
       </c>
       <c r="C22" s="6" t="inlineStr">
         <is>
-          <t>12,300~15,300</t>
+          <t>2,000</t>
         </is>
       </c>
       <c r="D22" s="7" t="inlineStr">
         <is>
-          <t>9,000,000</t>
+          <t>5,000,000</t>
         </is>
       </c>
       <c r="E22" s="7" t="inlineStr">
         <is>
-          <t>110,700</t>
-        </is>
-      </c>
-      <c r="F22" s="6" t="inlineStr">
-        <is>
-          <t>24.0배 (EV/EBITDA)</t>
-        </is>
-      </c>
-      <c r="G22" s="6" t="n">
-        <v>12300</v>
+          <t>10,000</t>
+        </is>
+      </c>
+      <c r="F22" s="19" t="inlineStr">
+        <is>
+          <t>해당없음</t>
+        </is>
+      </c>
+      <c r="G22" s="6" t="inlineStr">
+        <is>
+          <t>2,000</t>
+        </is>
       </c>
       <c r="H22" s="6" t="n">
-        <v>55.23</v>
+        <v>1388.6</v>
       </c>
       <c r="I22" s="6" t="n">
-        <v>751</v>
+        <v>2044</v>
       </c>
       <c r="J22" s="6" t="inlineStr">
         <is>
@@ -8828,33 +8830,29 @@
       </c>
       <c r="K22" s="6" t="inlineStr">
         <is>
-          <t>302.11</t>
+          <t>1,601.36</t>
         </is>
       </c>
       <c r="L22" s="6" t="inlineStr"/>
       <c r="M22" s="6" t="inlineStr">
         <is>
-          <t>2026-04-29</t>
+          <t>2026-04-30</t>
         </is>
       </c>
       <c r="N22" s="6" t="inlineStr">
         <is>
-          <t>KB</t>
-        </is>
-      </c>
-      <c r="O22" s="6" t="inlineStr">
-        <is>
-          <t>삼성</t>
-        </is>
-      </c>
+          <t>신한</t>
+        </is>
+      </c>
+      <c r="O22" s="6" t="inlineStr"/>
       <c r="P22" s="7" t="inlineStr">
         <is>
-          <t>3,384</t>
+          <t>350</t>
         </is>
       </c>
       <c r="Q22" s="6" t="inlineStr">
         <is>
-          <t>3.00%</t>
+          <t>3.50%</t>
         </is>
       </c>
       <c r="R22" s="6" t="inlineStr">
@@ -8866,75 +8864,77 @@
     <row r="23" ht="30" customHeight="1">
       <c r="A23" s="6" t="inlineStr">
         <is>
-          <t>키움히어로스펙2호</t>
-        </is>
-      </c>
-      <c r="B23" s="19" t="inlineStr">
-        <is>
-          <t>해당없음</t>
+          <t>채비</t>
+        </is>
+      </c>
+      <c r="B23" s="18" t="inlineStr">
+        <is>
+          <t>수집예정</t>
         </is>
       </c>
       <c r="C23" s="6" t="inlineStr">
         <is>
-          <t>2,000</t>
+          <t>12,300~15,300</t>
         </is>
       </c>
       <c r="D23" s="7" t="inlineStr">
         <is>
-          <t>6,000,000</t>
+          <t>9,000,000</t>
         </is>
       </c>
       <c r="E23" s="7" t="inlineStr">
         <is>
-          <t>12,000</t>
-        </is>
-      </c>
-      <c r="F23" s="19" t="inlineStr">
-        <is>
-          <t>해당없음</t>
-        </is>
-      </c>
-      <c r="G23" s="6" t="inlineStr">
-        <is>
-          <t>2,000</t>
-        </is>
+          <t>110,700</t>
+        </is>
+      </c>
+      <c r="F23" s="6" t="inlineStr">
+        <is>
+          <t>24.0배 (EV/EBITDA)</t>
+        </is>
+      </c>
+      <c r="G23" s="6" t="n">
+        <v>12300</v>
       </c>
       <c r="H23" s="6" t="n">
-        <v>1271.12</v>
+        <v>55.23</v>
       </c>
       <c r="I23" s="6" t="n">
-        <v>2054</v>
+        <v>751</v>
       </c>
       <c r="J23" s="6" t="inlineStr">
         <is>
-          <t>2026-04-14~04-15</t>
+          <t>2026-04-20~04-21</t>
         </is>
       </c>
       <c r="K23" s="6" t="inlineStr">
         <is>
-          <t>1,727.59</t>
+          <t>302.11</t>
         </is>
       </c>
       <c r="L23" s="6" t="inlineStr"/>
       <c r="M23" s="6" t="inlineStr">
         <is>
-          <t>2026-04-23</t>
+          <t>2026-04-29</t>
         </is>
       </c>
       <c r="N23" s="6" t="inlineStr">
         <is>
-          <t>키움</t>
-        </is>
-      </c>
-      <c r="O23" s="6" t="inlineStr"/>
+          <t>KB</t>
+        </is>
+      </c>
+      <c r="O23" s="6" t="inlineStr">
+        <is>
+          <t>삼성</t>
+        </is>
+      </c>
       <c r="P23" s="7" t="inlineStr">
         <is>
-          <t>300</t>
+          <t>3,384</t>
         </is>
       </c>
       <c r="Q23" s="6" t="inlineStr">
         <is>
-          <t>2.50%</t>
+          <t>3.00%</t>
         </is>
       </c>
       <c r="R23" s="6" t="inlineStr">
@@ -8946,7 +8946,7 @@
     <row r="24" ht="30" customHeight="1">
       <c r="A24" s="6" t="inlineStr">
         <is>
-          <t>교보스팩20호</t>
+          <t>키움히어로스펙2호</t>
         </is>
       </c>
       <c r="B24" s="19" t="inlineStr">
@@ -8961,12 +8961,12 @@
       </c>
       <c r="D24" s="7" t="inlineStr">
         <is>
-          <t>5,400,000</t>
+          <t>6,000,000</t>
         </is>
       </c>
       <c r="E24" s="7" t="inlineStr">
         <is>
-          <t>10,800</t>
+          <t>12,000</t>
         </is>
       </c>
       <c r="F24" s="19" t="inlineStr">
@@ -8980,30 +8980,30 @@
         </is>
       </c>
       <c r="H24" s="6" t="n">
-        <v>1196.99</v>
+        <v>1271.12</v>
       </c>
       <c r="I24" s="6" t="n">
-        <v>1855</v>
+        <v>2054</v>
       </c>
       <c r="J24" s="6" t="inlineStr">
         <is>
-          <t>2026-03-23~03-24</t>
+          <t>2026-04-14~04-15</t>
         </is>
       </c>
       <c r="K24" s="6" t="inlineStr">
         <is>
-          <t>747.00</t>
+          <t>1,727.59</t>
         </is>
       </c>
       <c r="L24" s="6" t="inlineStr"/>
       <c r="M24" s="6" t="inlineStr">
         <is>
-          <t>2026-04-02</t>
+          <t>2026-04-23</t>
         </is>
       </c>
       <c r="N24" s="6" t="inlineStr">
         <is>
-          <t>교보</t>
+          <t>키움</t>
         </is>
       </c>
       <c r="O24" s="6" t="inlineStr"/>
@@ -9014,7 +9014,7 @@
       </c>
       <c r="Q24" s="6" t="inlineStr">
         <is>
-          <t>2.78%</t>
+          <t>2.50%</t>
         </is>
       </c>
       <c r="R24" s="6" t="inlineStr">
@@ -9026,42 +9026,44 @@
     <row r="25" ht="30" customHeight="1">
       <c r="A25" s="6" t="inlineStr">
         <is>
-          <t>인벤테라</t>
-        </is>
-      </c>
-      <c r="B25" s="18" t="inlineStr">
-        <is>
-          <t>수집예정</t>
+          <t>교보스팩20호</t>
+        </is>
+      </c>
+      <c r="B25" s="19" t="inlineStr">
+        <is>
+          <t>해당없음</t>
         </is>
       </c>
       <c r="C25" s="6" t="inlineStr">
         <is>
-          <t>12,100~16,600</t>
+          <t>2,000</t>
         </is>
       </c>
       <c r="D25" s="7" t="inlineStr">
         <is>
-          <t>1,180,000</t>
+          <t>5,400,000</t>
         </is>
       </c>
       <c r="E25" s="7" t="inlineStr">
         <is>
-          <t>19,588</t>
-        </is>
-      </c>
-      <c r="F25" s="6" t="inlineStr">
-        <is>
-          <t>24.34배 (PER)</t>
-        </is>
-      </c>
-      <c r="G25" s="6" t="n">
-        <v>16600</v>
+          <t>10,800</t>
+        </is>
+      </c>
+      <c r="F25" s="19" t="inlineStr">
+        <is>
+          <t>해당없음</t>
+        </is>
+      </c>
+      <c r="G25" s="6" t="inlineStr">
+        <is>
+          <t>2,000</t>
+        </is>
       </c>
       <c r="H25" s="6" t="n">
-        <v>1328.82</v>
+        <v>1196.99</v>
       </c>
       <c r="I25" s="6" t="n">
-        <v>2309</v>
+        <v>1855</v>
       </c>
       <c r="J25" s="6" t="inlineStr">
         <is>
@@ -9070,7 +9072,7 @@
       </c>
       <c r="K25" s="6" t="inlineStr">
         <is>
-          <t>1,913.00</t>
+          <t>747.00</t>
         </is>
       </c>
       <c r="L25" s="6" t="inlineStr"/>
@@ -9081,18 +9083,18 @@
       </c>
       <c r="N25" s="6" t="inlineStr">
         <is>
-          <t>NH</t>
+          <t>교보</t>
         </is>
       </c>
       <c r="O25" s="6" t="inlineStr"/>
       <c r="P25" s="7" t="inlineStr">
         <is>
-          <t>1,211</t>
+          <t>300</t>
         </is>
       </c>
       <c r="Q25" s="6" t="inlineStr">
         <is>
-          <t>6.00%</t>
+          <t>2.78%</t>
         </is>
       </c>
       <c r="R25" s="6" t="inlineStr">
@@ -9104,75 +9106,73 @@
     <row r="26" ht="30" customHeight="1">
       <c r="A26" s="6" t="inlineStr">
         <is>
-          <t>신한스팩17호</t>
-        </is>
-      </c>
-      <c r="B26" s="19" t="inlineStr">
-        <is>
-          <t>해당없음</t>
+          <t>인벤테라</t>
+        </is>
+      </c>
+      <c r="B26" s="18" t="inlineStr">
+        <is>
+          <t>수집예정</t>
         </is>
       </c>
       <c r="C26" s="6" t="inlineStr">
         <is>
-          <t>2,000</t>
+          <t>12,100~16,600</t>
         </is>
       </c>
       <c r="D26" s="7" t="inlineStr">
         <is>
-          <t>5,000,000</t>
+          <t>1,180,000</t>
         </is>
       </c>
       <c r="E26" s="7" t="inlineStr">
         <is>
-          <t>10,000</t>
-        </is>
-      </c>
-      <c r="F26" s="19" t="inlineStr">
-        <is>
-          <t>해당없음</t>
-        </is>
-      </c>
-      <c r="G26" s="6" t="inlineStr">
-        <is>
-          <t>2,000</t>
-        </is>
+          <t>19,588</t>
+        </is>
+      </c>
+      <c r="F26" s="6" t="inlineStr">
+        <is>
+          <t>24.34배 (PER)</t>
+        </is>
+      </c>
+      <c r="G26" s="6" t="n">
+        <v>16600</v>
       </c>
       <c r="H26" s="6" t="n">
-        <v>1343.8</v>
+        <v>1328.82</v>
       </c>
       <c r="I26" s="6" t="n">
-        <v>2022</v>
+        <v>2309</v>
       </c>
       <c r="J26" s="6" t="inlineStr">
         <is>
-          <t>2026-03-19~03-20</t>
+          <t>2026-03-23~03-24</t>
         </is>
       </c>
       <c r="K26" s="6" t="inlineStr">
         <is>
-          <t>1,403.74</t>
+          <t>1,913.00</t>
         </is>
       </c>
       <c r="L26" s="6" t="inlineStr"/>
       <c r="M26" s="6" t="inlineStr">
         <is>
-          <t>2026-04-01</t>
+          <t>2026-04-02</t>
         </is>
       </c>
       <c r="N26" s="6" t="inlineStr">
         <is>
-          <t>신한</t>
+          <t>NH</t>
         </is>
       </c>
       <c r="O26" s="6" t="inlineStr"/>
       <c r="P26" s="7" t="inlineStr">
         <is>
-          <t>350</t>
+          <t>1,211</t>
         </is>
       </c>
       <c r="Q26" s="6" t="inlineStr">
         <is>
-          <t>3.50%</t>
+          <t>6.00%</t>
         </is>
       </c>
       <c r="R26" s="6" t="inlineStr">
@@ -9184,42 +9184,44 @@
     <row r="27" ht="30" customHeight="1">
       <c r="A27" s="6" t="inlineStr">
         <is>
-          <t>리센스메디컬</t>
-        </is>
-      </c>
-      <c r="B27" s="18" t="inlineStr">
-        <is>
-          <t>수집예정</t>
+          <t>신한스팩17호</t>
+        </is>
+      </c>
+      <c r="B27" s="19" t="inlineStr">
+        <is>
+          <t>해당없음</t>
         </is>
       </c>
       <c r="C27" s="6" t="inlineStr">
         <is>
-          <t>9,000~11,000</t>
+          <t>2,000</t>
         </is>
       </c>
       <c r="D27" s="7" t="inlineStr">
         <is>
-          <t>1,400,000</t>
+          <t>5,000,000</t>
         </is>
       </c>
       <c r="E27" s="7" t="inlineStr">
         <is>
-          <t>15,400</t>
-        </is>
-      </c>
-      <c r="F27" s="6" t="inlineStr">
-        <is>
-          <t>31.33배 (PER)</t>
-        </is>
-      </c>
-      <c r="G27" s="6" t="n">
-        <v>11000</v>
+          <t>10,000</t>
+        </is>
+      </c>
+      <c r="F27" s="19" t="inlineStr">
+        <is>
+          <t>해당없음</t>
+        </is>
+      </c>
+      <c r="G27" s="6" t="inlineStr">
+        <is>
+          <t>2,000</t>
+        </is>
       </c>
       <c r="H27" s="6" t="n">
-        <v>1352.63</v>
+        <v>1343.8</v>
       </c>
       <c r="I27" s="6" t="n">
-        <v>2261</v>
+        <v>2022</v>
       </c>
       <c r="J27" s="6" t="inlineStr">
         <is>
@@ -9228,33 +9230,29 @@
       </c>
       <c r="K27" s="6" t="inlineStr">
         <is>
-          <t>2,097.68</t>
+          <t>1,403.74</t>
         </is>
       </c>
       <c r="L27" s="6" t="inlineStr"/>
       <c r="M27" s="6" t="inlineStr">
         <is>
-          <t>2026-03-31</t>
+          <t>2026-04-01</t>
         </is>
       </c>
       <c r="N27" s="6" t="inlineStr">
         <is>
-          <t>한국</t>
-        </is>
-      </c>
-      <c r="O27" s="6" t="inlineStr">
-        <is>
-          <t>KB</t>
-        </is>
-      </c>
+          <t>신한</t>
+        </is>
+      </c>
+      <c r="O27" s="6" t="inlineStr"/>
       <c r="P27" s="7" t="inlineStr">
         <is>
-          <t>916</t>
+          <t>350</t>
         </is>
       </c>
       <c r="Q27" s="6" t="inlineStr">
         <is>
-          <t>5.77%</t>
+          <t>3.50%</t>
         </is>
       </c>
       <c r="R27" s="6" t="inlineStr">
@@ -9266,75 +9264,77 @@
     <row r="28" ht="30" customHeight="1">
       <c r="A28" s="6" t="inlineStr">
         <is>
-          <t>NH스팩33호</t>
-        </is>
-      </c>
-      <c r="B28" s="19" t="inlineStr">
-        <is>
-          <t>해당없음</t>
+          <t>리센스메디컬</t>
+        </is>
+      </c>
+      <c r="B28" s="18" t="inlineStr">
+        <is>
+          <t>수집예정</t>
         </is>
       </c>
       <c r="C28" s="6" t="inlineStr">
         <is>
-          <t>2,000</t>
+          <t>9,000~11,000</t>
         </is>
       </c>
       <c r="D28" s="7" t="inlineStr">
         <is>
-          <t>6,350,000</t>
+          <t>1,400,000</t>
         </is>
       </c>
       <c r="E28" s="7" t="inlineStr">
         <is>
-          <t>12,700</t>
-        </is>
-      </c>
-      <c r="F28" s="19" t="inlineStr">
-        <is>
-          <t>해당없음</t>
-        </is>
-      </c>
-      <c r="G28" s="6" t="inlineStr">
-        <is>
-          <t>2,000</t>
-        </is>
+          <t>15,400</t>
+        </is>
+      </c>
+      <c r="F28" s="6" t="inlineStr">
+        <is>
+          <t>31.33배 (PER)</t>
+        </is>
+      </c>
+      <c r="G28" s="6" t="n">
+        <v>11000</v>
       </c>
       <c r="H28" s="6" t="n">
-        <v>1228.71</v>
+        <v>1352.63</v>
       </c>
       <c r="I28" s="6" t="n">
-        <v>2058</v>
+        <v>2261</v>
       </c>
       <c r="J28" s="6" t="inlineStr">
         <is>
-          <t>2026-03-17~03-18</t>
+          <t>2026-03-19~03-20</t>
         </is>
       </c>
       <c r="K28" s="6" t="inlineStr">
         <is>
-          <t>569.27</t>
+          <t>2,097.68</t>
         </is>
       </c>
       <c r="L28" s="6" t="inlineStr"/>
       <c r="M28" s="6" t="inlineStr">
         <is>
-          <t>2026-03-27</t>
+          <t>2026-03-31</t>
         </is>
       </c>
       <c r="N28" s="6" t="inlineStr">
         <is>
-          <t>NH</t>
-        </is>
-      </c>
-      <c r="O28" s="6" t="inlineStr"/>
+          <t>한국</t>
+        </is>
+      </c>
+      <c r="O28" s="6" t="inlineStr">
+        <is>
+          <t>KB</t>
+        </is>
+      </c>
       <c r="P28" s="7" t="inlineStr">
         <is>
-          <t>381</t>
+          <t>916</t>
         </is>
       </c>
       <c r="Q28" s="6" t="inlineStr">
         <is>
-          <t>3.00%</t>
+          <t>5.77%</t>
         </is>
       </c>
       <c r="R28" s="6" t="inlineStr">
@@ -9346,73 +9346,75 @@
     <row r="29" ht="30" customHeight="1">
       <c r="A29" s="6" t="inlineStr">
         <is>
-          <t>메쥬</t>
-        </is>
-      </c>
-      <c r="B29" s="18" t="inlineStr">
-        <is>
-          <t>수집예정</t>
+          <t>NH스팩33호</t>
+        </is>
+      </c>
+      <c r="B29" s="19" t="inlineStr">
+        <is>
+          <t>해당없음</t>
         </is>
       </c>
       <c r="C29" s="6" t="inlineStr">
         <is>
-          <t>16,700~21,600</t>
+          <t>2,000</t>
         </is>
       </c>
       <c r="D29" s="7" t="inlineStr">
         <is>
-          <t>1,345,000</t>
+          <t>6,350,000</t>
         </is>
       </c>
       <c r="E29" s="7" t="inlineStr">
         <is>
-          <t>29,052</t>
-        </is>
-      </c>
-      <c r="F29" s="6" t="inlineStr">
-        <is>
-          <t>20.66배 (PER)</t>
-        </is>
-      </c>
-      <c r="G29" s="6" t="n">
-        <v>21600</v>
+          <t>12,700</t>
+        </is>
+      </c>
+      <c r="F29" s="19" t="inlineStr">
+        <is>
+          <t>해당없음</t>
+        </is>
+      </c>
+      <c r="G29" s="6" t="inlineStr">
+        <is>
+          <t>2,000</t>
+        </is>
       </c>
       <c r="H29" s="6" t="n">
-        <v>1108.93</v>
+        <v>1228.71</v>
       </c>
       <c r="I29" s="6" t="n">
-        <v>2320</v>
+        <v>2058</v>
       </c>
       <c r="J29" s="6" t="inlineStr">
         <is>
-          <t>2026-03-16~03-17</t>
+          <t>2026-03-17~03-18</t>
         </is>
       </c>
       <c r="K29" s="6" t="inlineStr">
         <is>
-          <t>2,428.25</t>
+          <t>569.27</t>
         </is>
       </c>
       <c r="L29" s="6" t="inlineStr"/>
       <c r="M29" s="6" t="inlineStr">
         <is>
-          <t>2026-03-26</t>
+          <t>2026-03-27</t>
         </is>
       </c>
       <c r="N29" s="6" t="inlineStr">
         <is>
-          <t>신한</t>
+          <t>NH</t>
         </is>
       </c>
       <c r="O29" s="6" t="inlineStr"/>
       <c r="P29" s="7" t="inlineStr">
         <is>
-          <t>1,496</t>
+          <t>381</t>
         </is>
       </c>
       <c r="Q29" s="6" t="inlineStr">
         <is>
-          <t>5.00%</t>
+          <t>3.00%</t>
         </is>
       </c>
       <c r="R29" s="6" t="inlineStr">
@@ -9424,7 +9426,7 @@
     <row r="30" ht="30" customHeight="1">
       <c r="A30" s="6" t="inlineStr">
         <is>
-          <t>한패스</t>
+          <t>메쥬</t>
         </is>
       </c>
       <c r="B30" s="18" t="inlineStr">
@@ -9434,32 +9436,32 @@
       </c>
       <c r="C30" s="6" t="inlineStr">
         <is>
-          <t>17,000~19,000</t>
+          <t>16,700~21,600</t>
         </is>
       </c>
       <c r="D30" s="7" t="inlineStr">
         <is>
-          <t>1,100,000</t>
+          <t>1,345,000</t>
         </is>
       </c>
       <c r="E30" s="7" t="inlineStr">
         <is>
-          <t>20,900</t>
+          <t>29,052</t>
         </is>
       </c>
       <c r="F30" s="6" t="inlineStr">
         <is>
-          <t>29.09배 (PER)</t>
+          <t>20.66배 (PER)</t>
         </is>
       </c>
       <c r="G30" s="6" t="n">
-        <v>19000</v>
+        <v>21600</v>
       </c>
       <c r="H30" s="6" t="n">
-        <v>1172.59</v>
+        <v>1108.93</v>
       </c>
       <c r="I30" s="6" t="n">
-        <v>2229</v>
+        <v>2320</v>
       </c>
       <c r="J30" s="6" t="inlineStr">
         <is>
@@ -9468,29 +9470,29 @@
       </c>
       <c r="K30" s="6" t="inlineStr">
         <is>
-          <t>1,673.04</t>
+          <t>2,428.25</t>
         </is>
       </c>
       <c r="L30" s="6" t="inlineStr"/>
       <c r="M30" s="6" t="inlineStr">
         <is>
-          <t>2026-03-25</t>
+          <t>2026-03-26</t>
         </is>
       </c>
       <c r="N30" s="6" t="inlineStr">
         <is>
-          <t>한국</t>
+          <t>신한</t>
         </is>
       </c>
       <c r="O30" s="6" t="inlineStr"/>
       <c r="P30" s="7" t="inlineStr">
         <is>
-          <t>753</t>
+          <t>1,496</t>
         </is>
       </c>
       <c r="Q30" s="6" t="inlineStr">
         <is>
-          <t>3.50%</t>
+          <t>5.00%</t>
         </is>
       </c>
       <c r="R30" s="6" t="inlineStr">
@@ -9502,7 +9504,7 @@
     <row r="31" ht="30" customHeight="1">
       <c r="A31" s="6" t="inlineStr">
         <is>
-          <t>아이엠바이오로직스</t>
+          <t>한패스</t>
         </is>
       </c>
       <c r="B31" s="18" t="inlineStr">
@@ -9512,47 +9514,47 @@
       </c>
       <c r="C31" s="6" t="inlineStr">
         <is>
-          <t>19,000~26,000</t>
+          <t>17,000~19,000</t>
         </is>
       </c>
       <c r="D31" s="7" t="inlineStr">
         <is>
-          <t>2,000,000</t>
+          <t>1,100,000</t>
         </is>
       </c>
       <c r="E31" s="7" t="inlineStr">
         <is>
-          <t>52,000</t>
+          <t>20,900</t>
         </is>
       </c>
       <c r="F31" s="6" t="inlineStr">
         <is>
-          <t>21.46배 (PER)</t>
+          <t>29.09배 (PER)</t>
         </is>
       </c>
       <c r="G31" s="6" t="n">
-        <v>26000</v>
+        <v>19000</v>
       </c>
       <c r="H31" s="6" t="n">
-        <v>839.23</v>
+        <v>1172.59</v>
       </c>
       <c r="I31" s="6" t="n">
-        <v>2333</v>
+        <v>2229</v>
       </c>
       <c r="J31" s="6" t="inlineStr">
         <is>
-          <t>2026-03-11~03-12</t>
+          <t>2026-03-16~03-17</t>
         </is>
       </c>
       <c r="K31" s="6" t="inlineStr">
         <is>
-          <t>1,806.00</t>
+          <t>1,673.04</t>
         </is>
       </c>
       <c r="L31" s="6" t="inlineStr"/>
       <c r="M31" s="6" t="inlineStr">
         <is>
-          <t>2026-03-20</t>
+          <t>2026-03-25</t>
         </is>
       </c>
       <c r="N31" s="6" t="inlineStr">
@@ -9563,12 +9565,12 @@
       <c r="O31" s="6" t="inlineStr"/>
       <c r="P31" s="7" t="inlineStr">
         <is>
-          <t>2,650</t>
+          <t>753</t>
         </is>
       </c>
       <c r="Q31" s="6" t="inlineStr">
         <is>
-          <t>5.00%</t>
+          <t>3.50%</t>
         </is>
       </c>
       <c r="R31" s="6" t="inlineStr">
@@ -9580,7 +9582,7 @@
     <row r="32" ht="30" customHeight="1">
       <c r="A32" s="6" t="inlineStr">
         <is>
-          <t>카나프테라퓨틱스</t>
+          <t>아이엠바이오로직스</t>
         </is>
       </c>
       <c r="B32" s="18" t="inlineStr">
@@ -9590,7 +9592,7 @@
       </c>
       <c r="C32" s="6" t="inlineStr">
         <is>
-          <t>16,000~20,000</t>
+          <t>19,000~26,000</t>
         </is>
       </c>
       <c r="D32" s="7" t="inlineStr">
@@ -9600,37 +9602,37 @@
       </c>
       <c r="E32" s="7" t="inlineStr">
         <is>
-          <t>40,000</t>
+          <t>52,000</t>
         </is>
       </c>
       <c r="F32" s="6" t="inlineStr">
         <is>
-          <t>23.59배 (PER)</t>
+          <t>21.46배 (PER)</t>
         </is>
       </c>
       <c r="G32" s="6" t="n">
-        <v>20000</v>
+        <v>26000</v>
       </c>
       <c r="H32" s="6" t="n">
-        <v>962.1</v>
+        <v>839.23</v>
       </c>
       <c r="I32" s="6" t="n">
-        <v>2327</v>
+        <v>2333</v>
       </c>
       <c r="J32" s="6" t="inlineStr">
         <is>
-          <t>2026-03-05~03-06</t>
+          <t>2026-03-11~03-12</t>
         </is>
       </c>
       <c r="K32" s="6" t="inlineStr">
         <is>
-          <t>1,899.29</t>
+          <t>1,806.00</t>
         </is>
       </c>
       <c r="L32" s="6" t="inlineStr"/>
       <c r="M32" s="6" t="inlineStr">
         <is>
-          <t>2026-03-16</t>
+          <t>2026-03-20</t>
         </is>
       </c>
       <c r="N32" s="6" t="inlineStr">
@@ -9641,7 +9643,7 @@
       <c r="O32" s="6" t="inlineStr"/>
       <c r="P32" s="7" t="inlineStr">
         <is>
-          <t>2,050</t>
+          <t>2,650</t>
         </is>
       </c>
       <c r="Q32" s="6" t="inlineStr">
@@ -9658,7 +9660,7 @@
     <row r="33" ht="30" customHeight="1">
       <c r="A33" s="6" t="inlineStr">
         <is>
-          <t>액스비스</t>
+          <t>카나프테라퓨틱스</t>
         </is>
       </c>
       <c r="B33" s="18" t="inlineStr">
@@ -9668,63 +9670,63 @@
       </c>
       <c r="C33" s="6" t="inlineStr">
         <is>
-          <t>10,100~11,500</t>
+          <t>16,000~20,000</t>
         </is>
       </c>
       <c r="D33" s="7" t="inlineStr">
         <is>
-          <t>2,300,000</t>
+          <t>2,000,000</t>
         </is>
       </c>
       <c r="E33" s="7" t="inlineStr">
         <is>
-          <t>26,450</t>
+          <t>40,000</t>
         </is>
       </c>
       <c r="F33" s="6" t="inlineStr">
         <is>
-          <t>27.60배 (PER)</t>
+          <t>23.59배 (PER)</t>
         </is>
       </c>
       <c r="G33" s="6" t="n">
-        <v>11500</v>
+        <v>20000</v>
       </c>
       <c r="H33" s="6" t="n">
-        <v>1124.21</v>
+        <v>962.1</v>
       </c>
       <c r="I33" s="6" t="n">
-        <v>2411</v>
+        <v>2327</v>
       </c>
       <c r="J33" s="6" t="inlineStr">
         <is>
-          <t>2026-02-23~02-24</t>
+          <t>2026-03-05~03-06</t>
         </is>
       </c>
       <c r="K33" s="6" t="inlineStr">
         <is>
-          <t>1,960.87</t>
+          <t>1,899.29</t>
         </is>
       </c>
       <c r="L33" s="6" t="inlineStr"/>
       <c r="M33" s="6" t="inlineStr">
         <is>
-          <t>2026-03-09</t>
+          <t>2026-03-16</t>
         </is>
       </c>
       <c r="N33" s="6" t="inlineStr">
         <is>
-          <t>미래</t>
+          <t>한국</t>
         </is>
       </c>
       <c r="O33" s="6" t="inlineStr"/>
       <c r="P33" s="7" t="inlineStr">
         <is>
-          <t>1,090</t>
+          <t>2,050</t>
         </is>
       </c>
       <c r="Q33" s="6" t="inlineStr">
         <is>
-          <t>4.00%</t>
+          <t>5.00%</t>
         </is>
       </c>
       <c r="R33" s="6" t="inlineStr">
@@ -9736,7 +9738,7 @@
     <row r="34" ht="30" customHeight="1">
       <c r="A34" s="6" t="inlineStr">
         <is>
-          <t>에스팀</t>
+          <t>액스비스</t>
         </is>
       </c>
       <c r="B34" s="18" t="inlineStr">
@@ -9746,32 +9748,32 @@
       </c>
       <c r="C34" s="6" t="inlineStr">
         <is>
-          <t>7,000~8,500</t>
+          <t>10,100~11,500</t>
         </is>
       </c>
       <c r="D34" s="7" t="inlineStr">
         <is>
-          <t>1,800,000</t>
+          <t>2,300,000</t>
         </is>
       </c>
       <c r="E34" s="7" t="inlineStr">
         <is>
-          <t>15,300</t>
+          <t>26,450</t>
         </is>
       </c>
       <c r="F34" s="6" t="inlineStr">
         <is>
-          <t>17.71배 (EV/EBITDA)</t>
+          <t>27.60배 (PER)</t>
         </is>
       </c>
       <c r="G34" s="6" t="n">
-        <v>8500</v>
+        <v>11500</v>
       </c>
       <c r="H34" s="6" t="n">
-        <v>1334.91</v>
+        <v>1124.21</v>
       </c>
       <c r="I34" s="6" t="n">
-        <v>2263</v>
+        <v>2411</v>
       </c>
       <c r="J34" s="6" t="inlineStr">
         <is>
@@ -9780,29 +9782,29 @@
       </c>
       <c r="K34" s="6" t="inlineStr">
         <is>
-          <t>1,334.91</t>
+          <t>1,960.87</t>
         </is>
       </c>
       <c r="L34" s="6" t="inlineStr"/>
       <c r="M34" s="6" t="inlineStr">
         <is>
-          <t>2026-03-06</t>
+          <t>2026-03-09</t>
         </is>
       </c>
       <c r="N34" s="6" t="inlineStr">
         <is>
-          <t>한국</t>
+          <t>미래</t>
         </is>
       </c>
       <c r="O34" s="6" t="inlineStr"/>
       <c r="P34" s="7" t="inlineStr">
         <is>
-          <t>788</t>
+          <t>1,090</t>
         </is>
       </c>
       <c r="Q34" s="6" t="inlineStr">
         <is>
-          <t>5.00%</t>
+          <t>4.00%</t>
         </is>
       </c>
       <c r="R34" s="6" t="inlineStr">
@@ -9814,7 +9816,7 @@
     <row r="35" ht="30" customHeight="1">
       <c r="A35" s="6" t="inlineStr">
         <is>
-          <t>케이뱅크 (유가)</t>
+          <t>에스팀</t>
         </is>
       </c>
       <c r="B35" s="18" t="inlineStr">
@@ -9824,67 +9826,63 @@
       </c>
       <c r="C35" s="6" t="inlineStr">
         <is>
-          <t>8,300~9,500</t>
+          <t>7,000~8,500</t>
         </is>
       </c>
       <c r="D35" s="7" t="inlineStr">
         <is>
-          <t>60,000,000</t>
+          <t>1,800,000</t>
         </is>
       </c>
       <c r="E35" s="7" t="inlineStr">
         <is>
-          <t>498,000</t>
+          <t>15,300</t>
         </is>
       </c>
       <c r="F35" s="6" t="inlineStr">
         <is>
-          <t>1.80배 (PBR)</t>
+          <t>17.71배 (EV/EBITDA)</t>
         </is>
       </c>
       <c r="G35" s="6" t="n">
-        <v>8300</v>
+        <v>8500</v>
       </c>
       <c r="H35" s="6" t="n">
-        <v>198.53</v>
+        <v>1334.91</v>
       </c>
       <c r="I35" s="6" t="n">
-        <v>2007</v>
+        <v>2263</v>
       </c>
       <c r="J35" s="6" t="inlineStr">
         <is>
-          <t>2026-02-20~23</t>
+          <t>2026-02-23~02-24</t>
         </is>
       </c>
       <c r="K35" s="6" t="inlineStr">
         <is>
-          <t>134.59</t>
+          <t>1,334.91</t>
         </is>
       </c>
       <c r="L35" s="6" t="inlineStr"/>
       <c r="M35" s="6" t="inlineStr">
         <is>
-          <t>2026-03-05</t>
+          <t>2026-03-06</t>
         </is>
       </c>
       <c r="N35" s="6" t="inlineStr">
         <is>
-          <t>NH</t>
-        </is>
-      </c>
-      <c r="O35" s="6" t="inlineStr">
-        <is>
-          <t>삼성</t>
-        </is>
-      </c>
+          <t>한국</t>
+        </is>
+      </c>
+      <c r="O35" s="6" t="inlineStr"/>
       <c r="P35" s="7" t="inlineStr">
         <is>
-          <t>5,976</t>
+          <t>788</t>
         </is>
       </c>
       <c r="Q35" s="6" t="inlineStr">
         <is>
-          <t>1.2%</t>
+          <t>5.00%</t>
         </is>
       </c>
       <c r="R35" s="6" t="inlineStr">
@@ -9896,63 +9894,57 @@
     <row r="36" ht="30" customHeight="1">
       <c r="A36" s="6" t="inlineStr">
         <is>
-          <t>세미티에스</t>
-        </is>
-      </c>
-      <c r="B36" s="19" t="inlineStr">
-        <is>
-          <t>해당없음</t>
-        </is>
-      </c>
-      <c r="C36" s="19" t="inlineStr">
-        <is>
-          <t>해당없음</t>
-        </is>
-      </c>
-      <c r="D36" s="19" t="inlineStr">
-        <is>
-          <t>해당없음</t>
-        </is>
-      </c>
-      <c r="E36" s="19" t="inlineStr">
-        <is>
-          <t>해당없음</t>
-        </is>
-      </c>
-      <c r="F36" s="19" t="inlineStr">
-        <is>
-          <t>해당없음</t>
-        </is>
-      </c>
-      <c r="G36" s="19" t="inlineStr">
-        <is>
-          <t>해당없음</t>
-        </is>
-      </c>
-      <c r="H36" s="19" t="inlineStr">
-        <is>
-          <t>해당없음</t>
-        </is>
-      </c>
-      <c r="I36" s="19" t="inlineStr">
-        <is>
-          <t>해당없음</t>
-        </is>
-      </c>
-      <c r="J36" s="19" t="inlineStr">
-        <is>
-          <t>해당없음</t>
-        </is>
-      </c>
-      <c r="K36" s="19" t="inlineStr">
-        <is>
-          <t>해당없음</t>
+          <t>케이뱅크 (유가)</t>
+        </is>
+      </c>
+      <c r="B36" s="18" t="inlineStr">
+        <is>
+          <t>수집예정</t>
+        </is>
+      </c>
+      <c r="C36" s="6" t="inlineStr">
+        <is>
+          <t>8,300~9,500</t>
+        </is>
+      </c>
+      <c r="D36" s="7" t="inlineStr">
+        <is>
+          <t>60,000,000</t>
+        </is>
+      </c>
+      <c r="E36" s="7" t="inlineStr">
+        <is>
+          <t>498,000</t>
+        </is>
+      </c>
+      <c r="F36" s="6" t="inlineStr">
+        <is>
+          <t>1.80배 (PBR)</t>
+        </is>
+      </c>
+      <c r="G36" s="6" t="n">
+        <v>8300</v>
+      </c>
+      <c r="H36" s="6" t="n">
+        <v>198.53</v>
+      </c>
+      <c r="I36" s="6" t="n">
+        <v>2007</v>
+      </c>
+      <c r="J36" s="6" t="inlineStr">
+        <is>
+          <t>2026-02-20~23</t>
+        </is>
+      </c>
+      <c r="K36" s="6" t="inlineStr">
+        <is>
+          <t>134.59</t>
         </is>
       </c>
       <c r="L36" s="6" t="inlineStr"/>
       <c r="M36" s="6" t="inlineStr">
         <is>
-          <t>2026-02-05</t>
+          <t>2026-03-05</t>
         </is>
       </c>
       <c r="N36" s="6" t="inlineStr">
@@ -9960,77 +9952,87 @@
           <t>NH</t>
         </is>
       </c>
-      <c r="O36" s="6" t="inlineStr"/>
-      <c r="P36" s="19" t="inlineStr">
-        <is>
-          <t>해당없음</t>
-        </is>
-      </c>
-      <c r="Q36" s="19" t="inlineStr">
-        <is>
-          <t>해당없음</t>
+      <c r="O36" s="6" t="inlineStr">
+        <is>
+          <t>삼성</t>
+        </is>
+      </c>
+      <c r="P36" s="7" t="inlineStr">
+        <is>
+          <t>5,976</t>
+        </is>
+      </c>
+      <c r="Q36" s="6" t="inlineStr">
+        <is>
+          <t>1.2%</t>
         </is>
       </c>
       <c r="R36" s="6" t="inlineStr">
         <is>
-          <t>상장완료(스팩합병)</t>
+          <t>상장완료</t>
         </is>
       </c>
     </row>
     <row r="37" ht="30" customHeight="1">
       <c r="A37" s="6" t="inlineStr">
         <is>
-          <t>덕양에너젠</t>
-        </is>
-      </c>
-      <c r="B37" s="18" t="inlineStr">
-        <is>
-          <t>수집예정</t>
-        </is>
-      </c>
-      <c r="C37" s="6" t="inlineStr">
-        <is>
-          <t>8,500~10,000</t>
-        </is>
-      </c>
-      <c r="D37" s="7" t="inlineStr">
-        <is>
-          <t>7,500,000</t>
-        </is>
-      </c>
-      <c r="E37" s="7" t="inlineStr">
-        <is>
-          <t>75,000</t>
-        </is>
-      </c>
-      <c r="F37" s="6" t="inlineStr">
-        <is>
-          <t>30.32배 (EV/EBITDA)</t>
-        </is>
-      </c>
-      <c r="G37" s="6" t="n">
-        <v>10000</v>
-      </c>
-      <c r="H37" s="6" t="n">
-        <v>650.14</v>
-      </c>
-      <c r="I37" s="6" t="n">
-        <v>2324</v>
-      </c>
-      <c r="J37" s="6" t="inlineStr">
-        <is>
-          <t>2026-01-20~01-21</t>
-        </is>
-      </c>
-      <c r="K37" s="6" t="inlineStr">
-        <is>
-          <t>1,354.00</t>
+          <t>세미티에스</t>
+        </is>
+      </c>
+      <c r="B37" s="19" t="inlineStr">
+        <is>
+          <t>해당없음</t>
+        </is>
+      </c>
+      <c r="C37" s="19" t="inlineStr">
+        <is>
+          <t>해당없음</t>
+        </is>
+      </c>
+      <c r="D37" s="19" t="inlineStr">
+        <is>
+          <t>해당없음</t>
+        </is>
+      </c>
+      <c r="E37" s="19" t="inlineStr">
+        <is>
+          <t>해당없음</t>
+        </is>
+      </c>
+      <c r="F37" s="19" t="inlineStr">
+        <is>
+          <t>해당없음</t>
+        </is>
+      </c>
+      <c r="G37" s="19" t="inlineStr">
+        <is>
+          <t>해당없음</t>
+        </is>
+      </c>
+      <c r="H37" s="19" t="inlineStr">
+        <is>
+          <t>해당없음</t>
+        </is>
+      </c>
+      <c r="I37" s="19" t="inlineStr">
+        <is>
+          <t>해당없음</t>
+        </is>
+      </c>
+      <c r="J37" s="19" t="inlineStr">
+        <is>
+          <t>해당없음</t>
+        </is>
+      </c>
+      <c r="K37" s="19" t="inlineStr">
+        <is>
+          <t>해당없음</t>
         </is>
       </c>
       <c r="L37" s="6" t="inlineStr"/>
       <c r="M37" s="6" t="inlineStr">
         <is>
-          <t>2026-01-30</t>
+          <t>2026-02-05</t>
         </is>
       </c>
       <c r="N37" s="6" t="inlineStr">
@@ -10038,87 +10040,77 @@
           <t>NH</t>
         </is>
       </c>
-      <c r="O37" s="6" t="inlineStr">
-        <is>
-          <t>미래</t>
-        </is>
-      </c>
-      <c r="P37" s="7" t="inlineStr">
-        <is>
-          <t>2,000</t>
-        </is>
-      </c>
-      <c r="Q37" s="6" t="inlineStr">
-        <is>
-          <t>2.92%</t>
+      <c r="O37" s="6" t="inlineStr"/>
+      <c r="P37" s="19" t="inlineStr">
+        <is>
+          <t>해당없음</t>
+        </is>
+      </c>
+      <c r="Q37" s="19" t="inlineStr">
+        <is>
+          <t>해당없음</t>
         </is>
       </c>
       <c r="R37" s="6" t="inlineStr">
         <is>
-          <t>상장완료</t>
+          <t>상장완료(스팩합병)</t>
         </is>
       </c>
     </row>
     <row r="38" ht="30" customHeight="1">
       <c r="A38" s="6" t="inlineStr">
         <is>
-          <t>케이피항공산업</t>
-        </is>
-      </c>
-      <c r="B38" s="19" t="inlineStr">
-        <is>
-          <t>해당없음</t>
-        </is>
-      </c>
-      <c r="C38" s="19" t="inlineStr">
-        <is>
-          <t>해당없음</t>
-        </is>
-      </c>
-      <c r="D38" s="19" t="inlineStr">
-        <is>
-          <t>해당없음</t>
-        </is>
-      </c>
-      <c r="E38" s="19" t="inlineStr">
-        <is>
-          <t>해당없음</t>
-        </is>
-      </c>
-      <c r="F38" s="19" t="inlineStr">
-        <is>
-          <t>해당없음</t>
-        </is>
-      </c>
-      <c r="G38" s="19" t="inlineStr">
-        <is>
-          <t>해당없음</t>
-        </is>
-      </c>
-      <c r="H38" s="19" t="inlineStr">
-        <is>
-          <t>해당없음</t>
-        </is>
-      </c>
-      <c r="I38" s="19" t="inlineStr">
-        <is>
-          <t>해당없음</t>
-        </is>
-      </c>
-      <c r="J38" s="19" t="inlineStr">
-        <is>
-          <t>해당없음</t>
-        </is>
-      </c>
-      <c r="K38" s="19" t="inlineStr">
-        <is>
-          <t>해당없음</t>
+          <t>덕양에너젠</t>
+        </is>
+      </c>
+      <c r="B38" s="18" t="inlineStr">
+        <is>
+          <t>수집예정</t>
+        </is>
+      </c>
+      <c r="C38" s="6" t="inlineStr">
+        <is>
+          <t>8,500~10,000</t>
+        </is>
+      </c>
+      <c r="D38" s="7" t="inlineStr">
+        <is>
+          <t>7,500,000</t>
+        </is>
+      </c>
+      <c r="E38" s="7" t="inlineStr">
+        <is>
+          <t>75,000</t>
+        </is>
+      </c>
+      <c r="F38" s="6" t="inlineStr">
+        <is>
+          <t>30.32배 (EV/EBITDA)</t>
+        </is>
+      </c>
+      <c r="G38" s="6" t="n">
+        <v>10000</v>
+      </c>
+      <c r="H38" s="6" t="n">
+        <v>650.14</v>
+      </c>
+      <c r="I38" s="6" t="n">
+        <v>2324</v>
+      </c>
+      <c r="J38" s="6" t="inlineStr">
+        <is>
+          <t>2026-01-20~01-21</t>
+        </is>
+      </c>
+      <c r="K38" s="6" t="inlineStr">
+        <is>
+          <t>1,354.00</t>
         </is>
       </c>
       <c r="L38" s="6" t="inlineStr"/>
       <c r="M38" s="6" t="inlineStr">
         <is>
-          <t>2026-01-29</t>
+          <t>2026-01-30</t>
         </is>
       </c>
       <c r="N38" s="6" t="inlineStr">
@@ -10126,27 +10118,31 @@
           <t>NH</t>
         </is>
       </c>
-      <c r="O38" s="6" t="inlineStr"/>
-      <c r="P38" s="19" t="inlineStr">
-        <is>
-          <t>해당없음</t>
-        </is>
-      </c>
-      <c r="Q38" s="19" t="inlineStr">
-        <is>
-          <t>해당없음</t>
+      <c r="O38" s="6" t="inlineStr">
+        <is>
+          <t>미래</t>
+        </is>
+      </c>
+      <c r="P38" s="7" t="inlineStr">
+        <is>
+          <t>2,000</t>
+        </is>
+      </c>
+      <c r="Q38" s="6" t="inlineStr">
+        <is>
+          <t>2.92%</t>
         </is>
       </c>
       <c r="R38" s="6" t="inlineStr">
         <is>
-          <t>상장완료(스팩합병)</t>
+          <t>상장완료</t>
         </is>
       </c>
     </row>
     <row r="39" ht="30" customHeight="1">
       <c r="A39" s="6" t="inlineStr">
         <is>
-          <t>삼성스팩13호</t>
+          <t>케이피항공산업</t>
         </is>
       </c>
       <c r="B39" s="19" t="inlineStr">
@@ -10154,19 +10150,19 @@
           <t>해당없음</t>
         </is>
       </c>
-      <c r="C39" s="6" t="inlineStr">
-        <is>
-          <t>2,000</t>
-        </is>
-      </c>
-      <c r="D39" s="7" t="inlineStr">
-        <is>
-          <t>6,000,000</t>
-        </is>
-      </c>
-      <c r="E39" s="7" t="inlineStr">
-        <is>
-          <t>12,000</t>
+      <c r="C39" s="19" t="inlineStr">
+        <is>
+          <t>해당없음</t>
+        </is>
+      </c>
+      <c r="D39" s="19" t="inlineStr">
+        <is>
+          <t>해당없음</t>
+        </is>
+      </c>
+      <c r="E39" s="19" t="inlineStr">
+        <is>
+          <t>해당없음</t>
         </is>
       </c>
       <c r="F39" s="19" t="inlineStr">
@@ -10174,196 +10170,208 @@
           <t>해당없음</t>
         </is>
       </c>
-      <c r="G39" s="6" t="inlineStr">
-        <is>
-          <t>2,000</t>
-        </is>
-      </c>
-      <c r="H39" s="6" t="n">
-        <v>1159.11</v>
-      </c>
-      <c r="I39" s="6" t="n">
-        <v>1892</v>
-      </c>
-      <c r="J39" s="6" t="inlineStr">
-        <is>
-          <t>2026-01-12~01-13</t>
-        </is>
-      </c>
-      <c r="K39" s="6" t="inlineStr">
-        <is>
-          <t>1,870.40</t>
+      <c r="G39" s="19" t="inlineStr">
+        <is>
+          <t>해당없음</t>
+        </is>
+      </c>
+      <c r="H39" s="19" t="inlineStr">
+        <is>
+          <t>해당없음</t>
+        </is>
+      </c>
+      <c r="I39" s="19" t="inlineStr">
+        <is>
+          <t>해당없음</t>
+        </is>
+      </c>
+      <c r="J39" s="19" t="inlineStr">
+        <is>
+          <t>해당없음</t>
+        </is>
+      </c>
+      <c r="K39" s="19" t="inlineStr">
+        <is>
+          <t>해당없음</t>
         </is>
       </c>
       <c r="L39" s="6" t="inlineStr"/>
       <c r="M39" s="6" t="inlineStr">
         <is>
+          <t>2026-01-29</t>
+        </is>
+      </c>
+      <c r="N39" s="6" t="inlineStr">
+        <is>
+          <t>NH</t>
+        </is>
+      </c>
+      <c r="O39" s="6" t="inlineStr"/>
+      <c r="P39" s="19" t="inlineStr">
+        <is>
+          <t>해당없음</t>
+        </is>
+      </c>
+      <c r="Q39" s="19" t="inlineStr">
+        <is>
+          <t>해당없음</t>
+        </is>
+      </c>
+      <c r="R39" s="6" t="inlineStr">
+        <is>
+          <t>상장완료(스팩합병)</t>
+        </is>
+      </c>
+    </row>
+    <row r="40" ht="30" customHeight="1">
+      <c r="A40" s="6" t="inlineStr">
+        <is>
+          <t>삼성스팩13호</t>
+        </is>
+      </c>
+      <c r="B40" s="19" t="inlineStr">
+        <is>
+          <t>해당없음</t>
+        </is>
+      </c>
+      <c r="C40" s="6" t="inlineStr">
+        <is>
+          <t>2,000</t>
+        </is>
+      </c>
+      <c r="D40" s="7" t="inlineStr">
+        <is>
+          <t>6,000,000</t>
+        </is>
+      </c>
+      <c r="E40" s="7" t="inlineStr">
+        <is>
+          <t>12,000</t>
+        </is>
+      </c>
+      <c r="F40" s="19" t="inlineStr">
+        <is>
+          <t>해당없음</t>
+        </is>
+      </c>
+      <c r="G40" s="6" t="inlineStr">
+        <is>
+          <t>2,000</t>
+        </is>
+      </c>
+      <c r="H40" s="6" t="n">
+        <v>1159.11</v>
+      </c>
+      <c r="I40" s="6" t="n">
+        <v>1892</v>
+      </c>
+      <c r="J40" s="6" t="inlineStr">
+        <is>
+          <t>2026-01-12~01-13</t>
+        </is>
+      </c>
+      <c r="K40" s="6" t="inlineStr">
+        <is>
+          <t>1,870.40</t>
+        </is>
+      </c>
+      <c r="L40" s="6" t="inlineStr"/>
+      <c r="M40" s="6" t="inlineStr">
+        <is>
           <t>2026-01-21</t>
         </is>
       </c>
-      <c r="N39" s="6" t="inlineStr">
+      <c r="N40" s="6" t="inlineStr">
         <is>
           <t>삼성</t>
         </is>
       </c>
-      <c r="O39" s="6" t="inlineStr"/>
-      <c r="P39" s="7" t="inlineStr">
+      <c r="O40" s="6" t="inlineStr"/>
+      <c r="P40" s="7" t="inlineStr">
         <is>
           <t>360</t>
         </is>
       </c>
-      <c r="Q39" s="6" t="inlineStr">
+      <c r="Q40" s="6" t="inlineStr">
         <is>
           <t>3.00%</t>
         </is>
       </c>
-      <c r="R39" s="6" t="inlineStr">
+      <c r="R40" s="6" t="inlineStr">
         <is>
           <t>상장완료</t>
         </is>
       </c>
     </row>
-    <row r="41" ht="22" customHeight="1">
-      <c r="A41" s="3" t="inlineStr">
-        <is>
-          <t>■ 공모 진행 (예심 승인법인)  (25건)</t>
-        </is>
-      </c>
-      <c r="B41" s="4" t="n"/>
-      <c r="C41" s="4" t="n"/>
-      <c r="D41" s="4" t="n"/>
-      <c r="E41" s="4" t="n"/>
-      <c r="F41" s="4" t="n"/>
-      <c r="G41" s="4" t="n"/>
-      <c r="H41" s="4" t="n"/>
-      <c r="I41" s="4" t="n"/>
-      <c r="J41" s="4" t="n"/>
-      <c r="K41" s="4" t="n"/>
-      <c r="L41" s="4" t="n"/>
-      <c r="M41" s="4" t="n"/>
-      <c r="N41" s="4" t="n"/>
-      <c r="O41" s="4" t="n"/>
-      <c r="P41" s="4" t="n"/>
-      <c r="Q41" s="4" t="n"/>
-      <c r="R41" s="4" t="n"/>
-    </row>
-    <row r="42" ht="30" customHeight="1">
-      <c r="A42" s="6" t="inlineStr">
-        <is>
-          <t>인제니아테라퓨틱스</t>
-        </is>
-      </c>
-      <c r="B42" s="6" t="inlineStr">
-        <is>
-          <t>07-20~07-24</t>
-        </is>
-      </c>
-      <c r="C42" s="6" t="inlineStr">
-        <is>
-          <t>12,000~14,500</t>
-        </is>
-      </c>
-      <c r="D42" s="7" t="inlineStr">
-        <is>
-          <t>5,000,000</t>
-        </is>
-      </c>
-      <c r="E42" s="7" t="inlineStr">
-        <is>
-          <t>60,000,000,000</t>
-        </is>
-      </c>
-      <c r="F42" s="6" t="inlineStr">
-        <is>
-          <t>22.89배 (PER)</t>
-        </is>
-      </c>
-      <c r="G42" s="6" t="inlineStr">
-        <is>
-          <t>12,000</t>
-        </is>
-      </c>
-      <c r="H42" s="6" t="n">
-        <v>50.4</v>
-      </c>
-      <c r="I42" s="6" t="n">
-        <v>307</v>
-      </c>
-      <c r="J42" s="6" t="inlineStr">
-        <is>
-          <t>07-30~07-31</t>
-        </is>
-      </c>
-      <c r="K42" s="6" t="inlineStr"/>
-      <c r="L42" s="6" t="inlineStr"/>
-      <c r="M42" s="6" t="inlineStr"/>
-      <c r="N42" s="6" t="inlineStr">
-        <is>
-          <t>삼성증권</t>
-        </is>
-      </c>
-      <c r="O42" s="6" t="inlineStr"/>
-      <c r="P42" s="7" t="inlineStr">
-        <is>
-          <t>4,095,000,000</t>
-        </is>
-      </c>
-      <c r="Q42" s="6" t="inlineStr">
-        <is>
-          <t>6.5%</t>
-        </is>
-      </c>
-      <c r="R42" s="6" t="inlineStr">
-        <is>
-          <t>청약완료·상장대기</t>
-        </is>
-      </c>
+    <row r="42" ht="22" customHeight="1">
+      <c r="A42" s="3" t="inlineStr">
+        <is>
+          <t>■ 공모 진행 (예심 승인법인)  (24건)</t>
+        </is>
+      </c>
+      <c r="B42" s="4" t="n"/>
+      <c r="C42" s="4" t="n"/>
+      <c r="D42" s="4" t="n"/>
+      <c r="E42" s="4" t="n"/>
+      <c r="F42" s="4" t="n"/>
+      <c r="G42" s="4" t="n"/>
+      <c r="H42" s="4" t="n"/>
+      <c r="I42" s="4" t="n"/>
+      <c r="J42" s="4" t="n"/>
+      <c r="K42" s="4" t="n"/>
+      <c r="L42" s="4" t="n"/>
+      <c r="M42" s="4" t="n"/>
+      <c r="N42" s="4" t="n"/>
+      <c r="O42" s="4" t="n"/>
+      <c r="P42" s="4" t="n"/>
+      <c r="Q42" s="4" t="n"/>
+      <c r="R42" s="4" t="n"/>
     </row>
     <row r="43" ht="30" customHeight="1">
       <c r="A43" s="6" t="inlineStr">
         <is>
-          <t>케이앤에스아이앤씨</t>
+          <t>인제니아테라퓨틱스</t>
         </is>
       </c>
       <c r="B43" s="6" t="inlineStr">
         <is>
-          <t>07-27~07-31</t>
+          <t>07-20~07-24</t>
         </is>
       </c>
       <c r="C43" s="6" t="inlineStr">
         <is>
-          <t>9,000~11,000</t>
+          <t>12,000~14,500</t>
         </is>
       </c>
       <c r="D43" s="7" t="inlineStr">
         <is>
-          <t>2,400,000</t>
+          <t>5,000,000</t>
         </is>
       </c>
       <c r="E43" s="7" t="inlineStr">
         <is>
-          <t>26,400,000,000</t>
+          <t>60,000,000,000</t>
         </is>
       </c>
       <c r="F43" s="6" t="inlineStr">
         <is>
-          <t>42.08배 (PER)</t>
+          <t>22.89배 (PER)</t>
         </is>
       </c>
       <c r="G43" s="6" t="inlineStr">
         <is>
-          <t>11,000</t>
+          <t>12,000</t>
         </is>
       </c>
       <c r="H43" s="6" t="n">
-        <v>938.24</v>
+        <v>50.4</v>
       </c>
       <c r="I43" s="6" t="n">
-        <v>2024</v>
+        <v>307</v>
       </c>
       <c r="J43" s="6" t="inlineStr">
         <is>
-          <t>08-04~08-05</t>
+          <t>07-30~07-31</t>
         </is>
       </c>
       <c r="K43" s="6" t="inlineStr"/>
@@ -10371,18 +10379,18 @@
       <c r="M43" s="6" t="inlineStr"/>
       <c r="N43" s="6" t="inlineStr">
         <is>
-          <t>아이비케이투자증권</t>
+          <t>삼성증권</t>
         </is>
       </c>
       <c r="O43" s="6" t="inlineStr"/>
       <c r="P43" s="7" t="inlineStr">
         <is>
-          <t>1,500,000,000</t>
+          <t>4,095,000,000</t>
         </is>
       </c>
       <c r="Q43" s="6" t="inlineStr">
         <is>
-          <t>3.5%</t>
+          <t>6.5%</t>
         </is>
       </c>
       <c r="R43" s="6" t="inlineStr">
@@ -10738,17 +10746,17 @@
     <row r="49" ht="30" customHeight="1">
       <c r="A49" s="6" t="inlineStr">
         <is>
-          <t>빅웨이브로보틱스</t>
+          <t>네오사피엔스</t>
         </is>
       </c>
       <c r="B49" s="6" t="inlineStr">
         <is>
-          <t>09-07~09-11</t>
+          <t>08-31~09-04</t>
         </is>
       </c>
       <c r="C49" s="6" t="inlineStr">
         <is>
-          <t>20,000~24,000</t>
+          <t>13,800~15,800</t>
         </is>
       </c>
       <c r="D49" s="7" t="inlineStr">
@@ -10758,12 +10766,12 @@
       </c>
       <c r="E49" s="7" t="inlineStr">
         <is>
-          <t>40,000,000,000</t>
+          <t>27,600,000,000</t>
         </is>
       </c>
       <c r="F49" s="6" t="inlineStr">
         <is>
-          <t>15.41 (PSR)</t>
+          <t>26.76배 (PER)</t>
         </is>
       </c>
       <c r="G49" s="6" t="inlineStr"/>
@@ -10771,7 +10779,7 @@
       <c r="I49" s="6" t="inlineStr"/>
       <c r="J49" s="6" t="inlineStr">
         <is>
-          <t>09-16~09-17</t>
+          <t>09-08~09-09</t>
         </is>
       </c>
       <c r="K49" s="6" t="inlineStr"/>
@@ -10779,22 +10787,18 @@
       <c r="M49" s="6" t="inlineStr"/>
       <c r="N49" s="6" t="inlineStr">
         <is>
-          <t>유진투자증권</t>
-        </is>
-      </c>
-      <c r="O49" s="6" t="inlineStr">
-        <is>
-          <t>미래</t>
-        </is>
-      </c>
+          <t>대신증권</t>
+        </is>
+      </c>
+      <c r="O49" s="6" t="inlineStr"/>
       <c r="P49" s="7" t="inlineStr">
         <is>
-          <t>627,300,000</t>
+          <t>1,080,264,000</t>
         </is>
       </c>
       <c r="Q49" s="6" t="inlineStr">
         <is>
-          <t>3.0%</t>
+          <t>3.8%</t>
         </is>
       </c>
       <c r="R49" s="6" t="inlineStr">
@@ -10806,32 +10810,32 @@
     <row r="50" ht="30" customHeight="1">
       <c r="A50" s="6" t="inlineStr">
         <is>
-          <t>덕산넵코어스</t>
+          <t>빅웨이브로보틱스</t>
         </is>
       </c>
       <c r="B50" s="6" t="inlineStr">
         <is>
-          <t>09-08~09-14</t>
+          <t>09-07~09-11</t>
         </is>
       </c>
       <c r="C50" s="6" t="inlineStr">
         <is>
-          <t>12,400~14,600</t>
+          <t>20,000~24,000</t>
         </is>
       </c>
       <c r="D50" s="7" t="inlineStr">
         <is>
-          <t>3,000,000</t>
+          <t>2,000,000</t>
         </is>
       </c>
       <c r="E50" s="7" t="inlineStr">
         <is>
-          <t>37,200,000,000</t>
+          <t>40,000,000,000</t>
         </is>
       </c>
       <c r="F50" s="6" t="inlineStr">
         <is>
-          <t>34.08배 (PER)</t>
+          <t>15.41 (PSR)</t>
         </is>
       </c>
       <c r="G50" s="6" t="inlineStr"/>
@@ -10847,18 +10851,22 @@
       <c r="M50" s="6" t="inlineStr"/>
       <c r="N50" s="6" t="inlineStr">
         <is>
-          <t>대신증권</t>
-        </is>
-      </c>
-      <c r="O50" s="6" t="inlineStr"/>
+          <t>유진투자증권</t>
+        </is>
+      </c>
+      <c r="O50" s="6" t="inlineStr">
+        <is>
+          <t>미래</t>
+        </is>
+      </c>
       <c r="P50" s="7" t="inlineStr">
         <is>
-          <t>1,413,399,926</t>
+          <t>627,300,000</t>
         </is>
       </c>
       <c r="Q50" s="6" t="inlineStr">
         <is>
-          <t>3.7%</t>
+          <t>3.0%</t>
         </is>
       </c>
       <c r="R50" s="6" t="inlineStr">
@@ -10870,32 +10878,32 @@
     <row r="51" ht="30" customHeight="1">
       <c r="A51" s="6" t="inlineStr">
         <is>
-          <t>엔에이치스팩34호</t>
+          <t>덕산넵코어스</t>
         </is>
       </c>
       <c r="B51" s="6" t="inlineStr">
         <is>
-          <t>08-24~08-25</t>
-        </is>
-      </c>
-      <c r="C51" s="18" t="inlineStr">
-        <is>
-          <t>수집예정</t>
-        </is>
-      </c>
-      <c r="D51" s="18" t="inlineStr">
-        <is>
-          <t>수집예정</t>
-        </is>
-      </c>
-      <c r="E51" s="18" t="inlineStr">
-        <is>
-          <t>수집예정</t>
-        </is>
-      </c>
-      <c r="F51" s="18" t="inlineStr">
-        <is>
-          <t>수집예정</t>
+          <t>09-08~09-14</t>
+        </is>
+      </c>
+      <c r="C51" s="6" t="inlineStr">
+        <is>
+          <t>12,400~14,600</t>
+        </is>
+      </c>
+      <c r="D51" s="7" t="inlineStr">
+        <is>
+          <t>3,000,000</t>
+        </is>
+      </c>
+      <c r="E51" s="7" t="inlineStr">
+        <is>
+          <t>37,200,000,000</t>
+        </is>
+      </c>
+      <c r="F51" s="6" t="inlineStr">
+        <is>
+          <t>34.08배 (PER)</t>
         </is>
       </c>
       <c r="G51" s="6" t="inlineStr"/>
@@ -10903,127 +10911,127 @@
       <c r="I51" s="6" t="inlineStr"/>
       <c r="J51" s="6" t="inlineStr">
         <is>
-          <t>09-01~09-02</t>
+          <t>09-16~09-17</t>
         </is>
       </c>
       <c r="K51" s="6" t="inlineStr"/>
       <c r="L51" s="6" t="inlineStr"/>
       <c r="M51" s="6" t="inlineStr"/>
-      <c r="N51" s="18" t="inlineStr">
-        <is>
-          <t>수집예정</t>
+      <c r="N51" s="6" t="inlineStr">
+        <is>
+          <t>대신증권</t>
         </is>
       </c>
       <c r="O51" s="6" t="inlineStr"/>
-      <c r="P51" s="18" t="inlineStr">
-        <is>
-          <t>수집예정</t>
+      <c r="P51" s="7" t="inlineStr">
+        <is>
+          <t>1,413,399,926</t>
         </is>
       </c>
       <c r="Q51" s="6" t="inlineStr">
         <is>
-          <t>50%</t>
+          <t>3.7%</t>
         </is>
       </c>
       <c r="R51" s="6" t="inlineStr">
         <is>
-          <t>최초</t>
+          <t>정정</t>
         </is>
       </c>
     </row>
     <row r="52" ht="30" customHeight="1">
       <c r="A52" s="6" t="inlineStr">
         <is>
-          <t>네오사피엔스</t>
-        </is>
-      </c>
-      <c r="B52" s="6" t="inlineStr">
-        <is>
-          <t>08-31~09-04</t>
-        </is>
-      </c>
-      <c r="C52" s="6" t="inlineStr">
-        <is>
-          <t>13,800~15,800</t>
-        </is>
-      </c>
-      <c r="D52" s="7" t="inlineStr">
-        <is>
-          <t>2,000,000</t>
-        </is>
-      </c>
-      <c r="E52" s="7" t="inlineStr">
-        <is>
-          <t>27,600,000,000</t>
-        </is>
-      </c>
-      <c r="F52" s="6" t="inlineStr">
-        <is>
-          <t>26.76배 (PER)</t>
+          <t>케이비제34호스팩</t>
+        </is>
+      </c>
+      <c r="B52" s="18" t="inlineStr">
+        <is>
+          <t>수집예정</t>
+        </is>
+      </c>
+      <c r="C52" s="18" t="inlineStr">
+        <is>
+          <t>수집예정</t>
+        </is>
+      </c>
+      <c r="D52" s="18" t="inlineStr">
+        <is>
+          <t>수집예정</t>
+        </is>
+      </c>
+      <c r="E52" s="18" t="inlineStr">
+        <is>
+          <t>수집예정</t>
+        </is>
+      </c>
+      <c r="F52" s="18" t="inlineStr">
+        <is>
+          <t>수집예정</t>
         </is>
       </c>
       <c r="G52" s="6" t="inlineStr"/>
       <c r="H52" s="6" t="inlineStr"/>
       <c r="I52" s="6" t="inlineStr"/>
-      <c r="J52" s="6" t="inlineStr">
-        <is>
-          <t>09-08~09-09</t>
+      <c r="J52" s="18" t="inlineStr">
+        <is>
+          <t>수집예정</t>
         </is>
       </c>
       <c r="K52" s="6" t="inlineStr"/>
       <c r="L52" s="6" t="inlineStr"/>
       <c r="M52" s="6" t="inlineStr"/>
-      <c r="N52" s="6" t="inlineStr">
-        <is>
-          <t>대신증권</t>
+      <c r="N52" s="18" t="inlineStr">
+        <is>
+          <t>수집예정</t>
         </is>
       </c>
       <c r="O52" s="6" t="inlineStr"/>
-      <c r="P52" s="7" t="inlineStr">
-        <is>
-          <t>1,080,264,000</t>
-        </is>
-      </c>
-      <c r="Q52" s="6" t="inlineStr">
-        <is>
-          <t>3.8%</t>
+      <c r="P52" s="18" t="inlineStr">
+        <is>
+          <t>수집예정</t>
+        </is>
+      </c>
+      <c r="Q52" s="18" t="inlineStr">
+        <is>
+          <t>수집예정</t>
         </is>
       </c>
       <c r="R52" s="6" t="inlineStr">
         <is>
-          <t>최초</t>
+          <t>정정</t>
         </is>
       </c>
     </row>
     <row r="53" ht="30" customHeight="1">
       <c r="A53" s="6" t="inlineStr">
         <is>
-          <t>와이즈플래닛컴퍼니</t>
+          <t>엔에이치스팩34호</t>
         </is>
       </c>
       <c r="B53" s="6" t="inlineStr">
         <is>
-          <t>09-04~09-10</t>
-        </is>
-      </c>
-      <c r="C53" s="6" t="inlineStr">
-        <is>
-          <t>10,000~12,000</t>
-        </is>
-      </c>
-      <c r="D53" s="7" t="inlineStr">
-        <is>
-          <t>1,600,000</t>
-        </is>
-      </c>
-      <c r="E53" s="7" t="inlineStr">
-        <is>
-          <t>16,000,000,000</t>
-        </is>
-      </c>
-      <c r="F53" s="6" t="inlineStr">
-        <is>
-          <t>21.59배 (PER)</t>
+          <t>08-24~08-25</t>
+        </is>
+      </c>
+      <c r="C53" s="18" t="inlineStr">
+        <is>
+          <t>수집예정</t>
+        </is>
+      </c>
+      <c r="D53" s="18" t="inlineStr">
+        <is>
+          <t>수집예정</t>
+        </is>
+      </c>
+      <c r="E53" s="18" t="inlineStr">
+        <is>
+          <t>수집예정</t>
+        </is>
+      </c>
+      <c r="F53" s="18" t="inlineStr">
+        <is>
+          <t>수집예정</t>
         </is>
       </c>
       <c r="G53" s="6" t="inlineStr"/>
@@ -11031,26 +11039,26 @@
       <c r="I53" s="6" t="inlineStr"/>
       <c r="J53" s="6" t="inlineStr">
         <is>
-          <t>09-14~09-15</t>
+          <t>09-01~09-02</t>
         </is>
       </c>
       <c r="K53" s="6" t="inlineStr"/>
       <c r="L53" s="6" t="inlineStr"/>
       <c r="M53" s="6" t="inlineStr"/>
-      <c r="N53" s="6" t="inlineStr">
-        <is>
-          <t>대신증권</t>
+      <c r="N53" s="18" t="inlineStr">
+        <is>
+          <t>수집예정</t>
         </is>
       </c>
       <c r="O53" s="6" t="inlineStr"/>
-      <c r="P53" s="7" t="inlineStr">
-        <is>
-          <t>494,400,000</t>
+      <c r="P53" s="18" t="inlineStr">
+        <is>
+          <t>수집예정</t>
         </is>
       </c>
       <c r="Q53" s="6" t="inlineStr">
         <is>
-          <t>3.0%</t>
+          <t>50%</t>
         </is>
       </c>
       <c r="R53" s="6" t="inlineStr">
@@ -11062,32 +11070,32 @@
     <row r="54" ht="30" customHeight="1">
       <c r="A54" s="6" t="inlineStr">
         <is>
-          <t>글로벌테크놀로지</t>
+          <t>와이즈플래닛컴퍼니</t>
         </is>
       </c>
       <c r="B54" s="6" t="inlineStr">
         <is>
-          <t>09-07~09-11</t>
+          <t>09-04~09-10</t>
         </is>
       </c>
       <c r="C54" s="6" t="inlineStr">
         <is>
-          <t>13,000~15,000</t>
+          <t>10,000~12,000</t>
         </is>
       </c>
       <c r="D54" s="7" t="inlineStr">
         <is>
-          <t>4,000,000</t>
+          <t>1,600,000</t>
         </is>
       </c>
       <c r="E54" s="7" t="inlineStr">
         <is>
-          <t>52,000,000,000</t>
+          <t>16,000,000,000</t>
         </is>
       </c>
       <c r="F54" s="6" t="inlineStr">
         <is>
-          <t>20.77배 (PER)</t>
+          <t>21.59배 (PER)</t>
         </is>
       </c>
       <c r="G54" s="6" t="inlineStr"/>
@@ -11095,7 +11103,7 @@
       <c r="I54" s="6" t="inlineStr"/>
       <c r="J54" s="6" t="inlineStr">
         <is>
-          <t>09-16~09-17</t>
+          <t>09-14~09-15</t>
         </is>
       </c>
       <c r="K54" s="6" t="inlineStr"/>
@@ -11103,18 +11111,18 @@
       <c r="M54" s="6" t="inlineStr"/>
       <c r="N54" s="6" t="inlineStr">
         <is>
-          <t>한국투자증권</t>
+          <t>대신증권</t>
         </is>
       </c>
       <c r="O54" s="6" t="inlineStr"/>
       <c r="P54" s="7" t="inlineStr">
         <is>
-          <t>2,119,999,960</t>
-        </is>
-      </c>
-      <c r="Q54" s="18" t="inlineStr">
-        <is>
-          <t>수집예정</t>
+          <t>494,400,000</t>
+        </is>
+      </c>
+      <c r="Q54" s="6" t="inlineStr">
+        <is>
+          <t>3.0%</t>
         </is>
       </c>
       <c r="R54" s="6" t="inlineStr">
@@ -11126,54 +11134,54 @@
     <row r="55" ht="30" customHeight="1">
       <c r="A55" s="6" t="inlineStr">
         <is>
-          <t>엠에스바이오</t>
-        </is>
-      </c>
-      <c r="B55" s="18" t="inlineStr">
-        <is>
-          <t>수집예정</t>
-        </is>
-      </c>
-      <c r="C55" s="18" t="inlineStr">
-        <is>
-          <t>수집예정</t>
-        </is>
-      </c>
-      <c r="D55" s="18" t="inlineStr">
-        <is>
-          <t>수집예정</t>
-        </is>
-      </c>
-      <c r="E55" s="18" t="inlineStr">
-        <is>
-          <t>수집예정</t>
-        </is>
-      </c>
-      <c r="F55" s="18" t="inlineStr">
-        <is>
-          <t>수집예정</t>
+          <t>글로벌테크놀로지</t>
+        </is>
+      </c>
+      <c r="B55" s="6" t="inlineStr">
+        <is>
+          <t>09-07~09-11</t>
+        </is>
+      </c>
+      <c r="C55" s="6" t="inlineStr">
+        <is>
+          <t>13,000~15,000</t>
+        </is>
+      </c>
+      <c r="D55" s="7" t="inlineStr">
+        <is>
+          <t>4,000,000</t>
+        </is>
+      </c>
+      <c r="E55" s="7" t="inlineStr">
+        <is>
+          <t>52,000,000,000</t>
+        </is>
+      </c>
+      <c r="F55" s="6" t="inlineStr">
+        <is>
+          <t>20.77배 (PER)</t>
         </is>
       </c>
       <c r="G55" s="6" t="inlineStr"/>
       <c r="H55" s="6" t="inlineStr"/>
       <c r="I55" s="6" t="inlineStr"/>
-      <c r="J55" s="18" t="inlineStr">
-        <is>
-          <t>수집예정</t>
+      <c r="J55" s="6" t="inlineStr">
+        <is>
+          <t>09-16~09-17</t>
         </is>
       </c>
       <c r="K55" s="6" t="inlineStr"/>
       <c r="L55" s="6" t="inlineStr"/>
       <c r="M55" s="6" t="inlineStr"/>
-      <c r="N55" s="18" t="inlineStr">
-        <is>
-          <t>수집예정</t>
+      <c r="N55" s="6" t="inlineStr">
+        <is>
+          <t>한국투자증권</t>
         </is>
       </c>
       <c r="O55" s="6" t="inlineStr"/>
-      <c r="P55" s="18" t="inlineStr">
-        <is>
-          <t>수집예정</t>
+      <c r="P55" s="7" t="inlineStr">
+        <is>
+          <t>2,119,999,960</t>
         </is>
       </c>
       <c r="Q55" s="18" t="inlineStr">
@@ -11183,14 +11191,14 @@
       </c>
       <c r="R55" s="6" t="inlineStr">
         <is>
-          <t>신고서 대기</t>
+          <t>최초</t>
         </is>
       </c>
     </row>
     <row r="56" ht="30" customHeight="1">
       <c r="A56" s="6" t="inlineStr">
         <is>
-          <t>디티에스</t>
+          <t>엠에스바이오</t>
         </is>
       </c>
       <c r="B56" s="18" t="inlineStr">
@@ -11254,7 +11262,7 @@
     <row r="57" ht="30" customHeight="1">
       <c r="A57" s="6" t="inlineStr">
         <is>
-          <t>에스케이증권제14호기업인수목적</t>
+          <t>디티에스</t>
         </is>
       </c>
       <c r="B57" s="18" t="inlineStr">
@@ -11318,7 +11326,7 @@
     <row r="58" ht="30" customHeight="1">
       <c r="A58" s="6" t="inlineStr">
         <is>
-          <t>케이비제34호스팩</t>
+          <t>에스케이증권제14호기업인수목적</t>
         </is>
       </c>
       <c r="B58" s="18" t="inlineStr">
@@ -12169,7 +12177,7 @@
         <v>0</v>
       </c>
       <c r="E13" s="6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F13" s="21">
         <f>IF((C13+D13)=0,"-",C13/(C13+D13))</f>
@@ -12292,30 +12300,30 @@
     <row r="22">
       <c r="A22" s="6" t="inlineStr">
         <is>
-          <t>미래에셋증권</t>
+          <t>아이비케이투자증권</t>
         </is>
       </c>
       <c r="B22" s="6" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="C22" s="6" t="inlineStr">
         <is>
-          <t>48,280,000,000</t>
+          <t>72,600,000,000</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="6" t="inlineStr">
         <is>
-          <t>아이비케이투자증권</t>
+          <t>미래에셋증권</t>
         </is>
       </c>
       <c r="B23" s="6" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C23" s="6" t="inlineStr">
         <is>
-          <t>46,200,000,000</t>
+          <t>48,280,000,000</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore: update IPO data 2026-08-15
</commit_message>
<xml_diff>
--- a/IPO_analysis.xlsx
+++ b/IPO_analysis.xlsx
@@ -618,7 +618,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>기준일 2026-08-14 · 청구일 직전 사업연도 · 별도/개별 재무제표 · 단위 백만원(별도 표기 시 USD)</t>
+          <t>기준일 2026-08-15 · 청구일 직전 사업연도 · 별도/개별 재무제표 · 단위 백만원(별도 표기 시 USD)</t>
         </is>
       </c>
     </row>
@@ -10808,7 +10808,7 @@
       </c>
       <c r="B49" s="6" t="inlineStr">
         <is>
-          <t>08-31~09-04</t>
+          <t>09-02~09-08</t>
         </is>
       </c>
       <c r="C49" s="6" t="inlineStr">
@@ -10836,7 +10836,7 @@
       <c r="I49" s="6" t="inlineStr"/>
       <c r="J49" s="6" t="inlineStr">
         <is>
-          <t>09-08~09-09</t>
+          <t>09-10~09-11</t>
         </is>
       </c>
       <c r="K49" s="6" t="inlineStr"/>
@@ -11191,32 +11191,32 @@
     <row r="55" ht="30" customHeight="1">
       <c r="A55" s="6" t="inlineStr">
         <is>
-          <t>글로벌테크놀로지</t>
+          <t>한국제17호스팩</t>
         </is>
       </c>
       <c r="B55" s="6" t="inlineStr">
         <is>
-          <t>09-07~09-11</t>
-        </is>
-      </c>
-      <c r="C55" s="6" t="inlineStr">
-        <is>
-          <t>13,000~15,000</t>
+          <t>09-07~09-08</t>
+        </is>
+      </c>
+      <c r="C55" s="18" t="inlineStr">
+        <is>
+          <t>수집예정</t>
         </is>
       </c>
       <c r="D55" s="7" t="inlineStr">
         <is>
-          <t>4,000,000</t>
+          <t>7,000,000</t>
         </is>
       </c>
       <c r="E55" s="7" t="inlineStr">
         <is>
-          <t>52,000,000,000</t>
-        </is>
-      </c>
-      <c r="F55" s="6" t="inlineStr">
-        <is>
-          <t>20.77배 (PER)</t>
+          <t>14,000,000,000</t>
+        </is>
+      </c>
+      <c r="F55" s="18" t="inlineStr">
+        <is>
+          <t>수집예정</t>
         </is>
       </c>
       <c r="G55" s="6" t="inlineStr"/>
@@ -11224,26 +11224,26 @@
       <c r="I55" s="6" t="inlineStr"/>
       <c r="J55" s="6" t="inlineStr">
         <is>
-          <t>09-16~09-17</t>
+          <t>09-10~09-11</t>
         </is>
       </c>
       <c r="K55" s="6" t="inlineStr"/>
       <c r="L55" s="6" t="inlineStr"/>
       <c r="M55" s="6" t="inlineStr"/>
-      <c r="N55" s="6" t="inlineStr">
-        <is>
-          <t>한국투자증권</t>
+      <c r="N55" s="18" t="inlineStr">
+        <is>
+          <t>수집예정</t>
         </is>
       </c>
       <c r="O55" s="6" t="inlineStr"/>
-      <c r="P55" s="7" t="inlineStr">
-        <is>
-          <t>2,119,999,960</t>
-        </is>
-      </c>
-      <c r="Q55" s="18" t="inlineStr">
-        <is>
-          <t>수집예정</t>
+      <c r="P55" s="18" t="inlineStr">
+        <is>
+          <t>수집예정</t>
+        </is>
+      </c>
+      <c r="Q55" s="6" t="inlineStr">
+        <is>
+          <t>3.0%</t>
         </is>
       </c>
       <c r="R55" s="6" t="inlineStr">
@@ -11255,54 +11255,54 @@
     <row r="56" ht="30" customHeight="1">
       <c r="A56" s="6" t="inlineStr">
         <is>
-          <t>한국제17호스팩</t>
-        </is>
-      </c>
-      <c r="B56" s="18" t="inlineStr">
-        <is>
-          <t>수집예정</t>
-        </is>
-      </c>
-      <c r="C56" s="18" t="inlineStr">
-        <is>
-          <t>수집예정</t>
-        </is>
-      </c>
-      <c r="D56" s="18" t="inlineStr">
-        <is>
-          <t>수집예정</t>
-        </is>
-      </c>
-      <c r="E56" s="18" t="inlineStr">
-        <is>
-          <t>수집예정</t>
-        </is>
-      </c>
-      <c r="F56" s="18" t="inlineStr">
-        <is>
-          <t>수집예정</t>
+          <t>글로벌테크놀로지</t>
+        </is>
+      </c>
+      <c r="B56" s="6" t="inlineStr">
+        <is>
+          <t>09-07~09-11</t>
+        </is>
+      </c>
+      <c r="C56" s="6" t="inlineStr">
+        <is>
+          <t>13,000~15,000</t>
+        </is>
+      </c>
+      <c r="D56" s="7" t="inlineStr">
+        <is>
+          <t>4,000,000</t>
+        </is>
+      </c>
+      <c r="E56" s="7" t="inlineStr">
+        <is>
+          <t>52,000,000,000</t>
+        </is>
+      </c>
+      <c r="F56" s="6" t="inlineStr">
+        <is>
+          <t>20.77배 (PER)</t>
         </is>
       </c>
       <c r="G56" s="6" t="inlineStr"/>
       <c r="H56" s="6" t="inlineStr"/>
       <c r="I56" s="6" t="inlineStr"/>
-      <c r="J56" s="18" t="inlineStr">
-        <is>
-          <t>수집예정</t>
+      <c r="J56" s="6" t="inlineStr">
+        <is>
+          <t>09-16~09-17</t>
         </is>
       </c>
       <c r="K56" s="6" t="inlineStr"/>
       <c r="L56" s="6" t="inlineStr"/>
       <c r="M56" s="6" t="inlineStr"/>
-      <c r="N56" s="18" t="inlineStr">
-        <is>
-          <t>수집예정</t>
+      <c r="N56" s="6" t="inlineStr">
+        <is>
+          <t>한국투자증권</t>
         </is>
       </c>
       <c r="O56" s="6" t="inlineStr"/>
-      <c r="P56" s="18" t="inlineStr">
-        <is>
-          <t>수집예정</t>
+      <c r="P56" s="7" t="inlineStr">
+        <is>
+          <t>2,119,999,960</t>
         </is>
       </c>
       <c r="Q56" s="18" t="inlineStr">

</xml_diff>

<commit_message>
chore: update IPO data 2026-08-19
</commit_message>
<xml_diff>
--- a/IPO_analysis.xlsx
+++ b/IPO_analysis.xlsx
@@ -618,7 +618,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>기준일 2026-08-18 · 청구일 직전 사업연도 · 별도/개별 재무제표 · 단위 백만원(별도 표기 시 USD)</t>
+          <t>기준일 2026-08-19 · 청구일 직전 사업연도 · 별도/개별 재무제표 · 단위 백만원(별도 표기 시 USD)</t>
         </is>
       </c>
     </row>
@@ -11128,32 +11128,32 @@
     <row r="53" ht="30" customHeight="1">
       <c r="A53" s="6" t="inlineStr">
         <is>
-          <t>덕산넵코어스</t>
+          <t>글로벌테크놀로지</t>
         </is>
       </c>
       <c r="B53" s="6" t="inlineStr">
         <is>
-          <t>09-08~09-14</t>
+          <t>09-07~09-11</t>
         </is>
       </c>
       <c r="C53" s="6" t="inlineStr">
         <is>
-          <t>12,400~14,600</t>
+          <t>13,000~15,000</t>
         </is>
       </c>
       <c r="D53" s="7" t="inlineStr">
         <is>
-          <t>3,000,000</t>
+          <t>4,000,000</t>
         </is>
       </c>
       <c r="E53" s="7" t="inlineStr">
         <is>
-          <t>37,200,000,000</t>
+          <t>52,000,000,000</t>
         </is>
       </c>
       <c r="F53" s="6" t="inlineStr">
         <is>
-          <t>34.08배 (PER)</t>
+          <t>20.77배 (PER)</t>
         </is>
       </c>
       <c r="G53" s="6" t="inlineStr"/>
@@ -11169,18 +11169,18 @@
       <c r="M53" s="6" t="inlineStr"/>
       <c r="N53" s="6" t="inlineStr">
         <is>
-          <t>대신증권</t>
+          <t>한국투자증권</t>
         </is>
       </c>
       <c r="O53" s="6" t="inlineStr"/>
       <c r="P53" s="7" t="inlineStr">
         <is>
-          <t>1,413,399,926</t>
-        </is>
-      </c>
-      <c r="Q53" s="6" t="inlineStr">
-        <is>
-          <t>3.7%</t>
+          <t>2,119,999,960</t>
+        </is>
+      </c>
+      <c r="Q53" s="18" t="inlineStr">
+        <is>
+          <t>수집예정</t>
         </is>
       </c>
       <c r="R53" s="6" t="inlineStr">
@@ -11192,32 +11192,32 @@
     <row r="54" ht="30" customHeight="1">
       <c r="A54" s="6" t="inlineStr">
         <is>
-          <t>엔에이치스팩34호</t>
+          <t>덕산넵코어스</t>
         </is>
       </c>
       <c r="B54" s="6" t="inlineStr">
         <is>
-          <t>08-24~08-25</t>
-        </is>
-      </c>
-      <c r="C54" s="18" t="inlineStr">
-        <is>
-          <t>수집예정</t>
-        </is>
-      </c>
-      <c r="D54" s="18" t="inlineStr">
-        <is>
-          <t>수집예정</t>
-        </is>
-      </c>
-      <c r="E54" s="18" t="inlineStr">
-        <is>
-          <t>수집예정</t>
-        </is>
-      </c>
-      <c r="F54" s="18" t="inlineStr">
-        <is>
-          <t>수집예정</t>
+          <t>09-08~09-14</t>
+        </is>
+      </c>
+      <c r="C54" s="6" t="inlineStr">
+        <is>
+          <t>12,400~14,600</t>
+        </is>
+      </c>
+      <c r="D54" s="7" t="inlineStr">
+        <is>
+          <t>3,000,000</t>
+        </is>
+      </c>
+      <c r="E54" s="7" t="inlineStr">
+        <is>
+          <t>37,200,000,000</t>
+        </is>
+      </c>
+      <c r="F54" s="6" t="inlineStr">
+        <is>
+          <t>34.08배 (PER)</t>
         </is>
       </c>
       <c r="G54" s="6" t="inlineStr"/>
@@ -11225,43 +11225,43 @@
       <c r="I54" s="6" t="inlineStr"/>
       <c r="J54" s="6" t="inlineStr">
         <is>
-          <t>09-01~09-02</t>
+          <t>09-16~09-17</t>
         </is>
       </c>
       <c r="K54" s="6" t="inlineStr"/>
       <c r="L54" s="6" t="inlineStr"/>
       <c r="M54" s="6" t="inlineStr"/>
-      <c r="N54" s="18" t="inlineStr">
-        <is>
-          <t>수집예정</t>
+      <c r="N54" s="6" t="inlineStr">
+        <is>
+          <t>대신증권</t>
         </is>
       </c>
       <c r="O54" s="6" t="inlineStr"/>
-      <c r="P54" s="18" t="inlineStr">
-        <is>
-          <t>수집예정</t>
+      <c r="P54" s="7" t="inlineStr">
+        <is>
+          <t>1,413,399,926</t>
         </is>
       </c>
       <c r="Q54" s="6" t="inlineStr">
         <is>
-          <t>50%</t>
+          <t>3.7%</t>
         </is>
       </c>
       <c r="R54" s="6" t="inlineStr">
         <is>
-          <t>최초</t>
+          <t>정정</t>
         </is>
       </c>
     </row>
     <row r="55" ht="30" customHeight="1">
       <c r="A55" s="6" t="inlineStr">
         <is>
-          <t>한국제17호스팩</t>
+          <t>엔에이치스팩34호</t>
         </is>
       </c>
       <c r="B55" s="6" t="inlineStr">
         <is>
-          <t>09-07~09-08</t>
+          <t>08-24~08-25</t>
         </is>
       </c>
       <c r="C55" s="18" t="inlineStr">
@@ -11269,14 +11269,14 @@
           <t>수집예정</t>
         </is>
       </c>
-      <c r="D55" s="7" t="inlineStr">
-        <is>
-          <t>7,000,000</t>
-        </is>
-      </c>
-      <c r="E55" s="7" t="inlineStr">
-        <is>
-          <t>14,000,000,000</t>
+      <c r="D55" s="18" t="inlineStr">
+        <is>
+          <t>수집예정</t>
+        </is>
+      </c>
+      <c r="E55" s="18" t="inlineStr">
+        <is>
+          <t>수집예정</t>
         </is>
       </c>
       <c r="F55" s="18" t="inlineStr">
@@ -11289,7 +11289,7 @@
       <c r="I55" s="6" t="inlineStr"/>
       <c r="J55" s="6" t="inlineStr">
         <is>
-          <t>09-10~09-11</t>
+          <t>09-01~09-02</t>
         </is>
       </c>
       <c r="K55" s="6" t="inlineStr"/>
@@ -11308,7 +11308,7 @@
       </c>
       <c r="Q55" s="6" t="inlineStr">
         <is>
-          <t>3.0%</t>
+          <t>50%</t>
         </is>
       </c>
       <c r="R55" s="6" t="inlineStr">
@@ -11320,32 +11320,32 @@
     <row r="56" ht="30" customHeight="1">
       <c r="A56" s="6" t="inlineStr">
         <is>
-          <t>글로벌테크놀로지</t>
+          <t>한국제17호스팩</t>
         </is>
       </c>
       <c r="B56" s="6" t="inlineStr">
         <is>
-          <t>09-07~09-11</t>
-        </is>
-      </c>
-      <c r="C56" s="6" t="inlineStr">
-        <is>
-          <t>13,000~15,000</t>
+          <t>09-07~09-08</t>
+        </is>
+      </c>
+      <c r="C56" s="18" t="inlineStr">
+        <is>
+          <t>수집예정</t>
         </is>
       </c>
       <c r="D56" s="7" t="inlineStr">
         <is>
-          <t>4,000,000</t>
+          <t>7,000,000</t>
         </is>
       </c>
       <c r="E56" s="7" t="inlineStr">
         <is>
-          <t>52,000,000,000</t>
-        </is>
-      </c>
-      <c r="F56" s="6" t="inlineStr">
-        <is>
-          <t>20.77배 (PER)</t>
+          <t>14,000,000,000</t>
+        </is>
+      </c>
+      <c r="F56" s="18" t="inlineStr">
+        <is>
+          <t>수집예정</t>
         </is>
       </c>
       <c r="G56" s="6" t="inlineStr"/>
@@ -11353,26 +11353,26 @@
       <c r="I56" s="6" t="inlineStr"/>
       <c r="J56" s="6" t="inlineStr">
         <is>
-          <t>09-16~09-17</t>
+          <t>09-10~09-11</t>
         </is>
       </c>
       <c r="K56" s="6" t="inlineStr"/>
       <c r="L56" s="6" t="inlineStr"/>
       <c r="M56" s="6" t="inlineStr"/>
-      <c r="N56" s="6" t="inlineStr">
-        <is>
-          <t>한국투자증권</t>
+      <c r="N56" s="18" t="inlineStr">
+        <is>
+          <t>수집예정</t>
         </is>
       </c>
       <c r="O56" s="6" t="inlineStr"/>
-      <c r="P56" s="7" t="inlineStr">
-        <is>
-          <t>2,119,999,960</t>
-        </is>
-      </c>
-      <c r="Q56" s="18" t="inlineStr">
-        <is>
-          <t>수집예정</t>
+      <c r="P56" s="18" t="inlineStr">
+        <is>
+          <t>수집예정</t>
+        </is>
+      </c>
+      <c r="Q56" s="6" t="inlineStr">
+        <is>
+          <t>3.0%</t>
         </is>
       </c>
       <c r="R56" s="6" t="inlineStr">

</xml_diff>

<commit_message>
chore: update IPO data 2026-08-21
</commit_message>
<xml_diff>
--- a/IPO_analysis.xlsx
+++ b/IPO_analysis.xlsx
@@ -618,7 +618,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>기준일 2026-08-20 · 청구일 직전 사업연도 · 별도/개별 재무제표 · 단위 백만원(별도 표기 시 USD)</t>
+          <t>기준일 2026-08-21 · 청구일 직전 사업연도 · 별도/개별 재무제표 · 단위 백만원(별도 표기 시 USD)</t>
         </is>
       </c>
     </row>
@@ -4594,7 +4594,7 @@
       </c>
       <c r="K76" s="6" t="inlineStr">
         <is>
-          <t>상장승인(상장예정)</t>
+          <t>상장완료 (2026-08-21)</t>
         </is>
       </c>
     </row>
@@ -4822,7 +4822,7 @@
       </c>
       <c r="K80" s="6" t="inlineStr">
         <is>
-          <t>상장전</t>
+          <t>상장승인(상장예정)</t>
         </is>
       </c>
     </row>
@@ -7621,7 +7621,7 @@
     <row r="6" ht="22" customHeight="1">
       <c r="A6" s="3" t="inlineStr">
         <is>
-          <t>■ 상장 완료 (2026)  (35건)</t>
+          <t>■ 상장 완료 (2026)  (36건)</t>
         </is>
       </c>
       <c r="B6" s="4" t="n"/>
@@ -7645,44 +7645,44 @@
     <row r="7" ht="30" customHeight="1">
       <c r="A7" s="6" t="inlineStr">
         <is>
-          <t>인제니아테라퓨틱스</t>
+          <t>기도산업</t>
         </is>
       </c>
       <c r="B7" s="6" t="inlineStr">
         <is>
-          <t>07-20~07-24</t>
+          <t>07-31~08-06</t>
         </is>
       </c>
       <c r="C7" s="6" t="inlineStr">
         <is>
-          <t>12,000~14,500</t>
+          <t>24,800~28,400</t>
         </is>
       </c>
       <c r="D7" s="7" t="inlineStr">
         <is>
-          <t>5,000,000</t>
+          <t>1,700,000</t>
         </is>
       </c>
       <c r="E7" s="7" t="inlineStr">
         <is>
-          <t>60,000,000,000</t>
+          <t>48,280,000,000</t>
         </is>
       </c>
       <c r="F7" s="6" t="inlineStr">
         <is>
-          <t>22.89배 (PER)</t>
+          <t>10.01배 (PER)</t>
         </is>
       </c>
       <c r="G7" s="6" t="inlineStr">
         <is>
-          <t>12,000</t>
+          <t>28,400</t>
         </is>
       </c>
       <c r="H7" s="6" t="n">
-        <v>50.4</v>
+        <v>213.31</v>
       </c>
       <c r="I7" s="6" t="n">
-        <v>307</v>
+        <v>637</v>
       </c>
       <c r="J7" s="18" t="inlineStr">
         <is>
@@ -7697,23 +7697,23 @@
       <c r="L7" s="6" t="inlineStr"/>
       <c r="M7" s="6" t="inlineStr">
         <is>
-          <t>2026-08-18</t>
+          <t>2026-08-21</t>
         </is>
       </c>
       <c r="N7" s="6" t="inlineStr">
         <is>
-          <t>삼성증권</t>
+          <t>미래에셋증권</t>
         </is>
       </c>
       <c r="O7" s="6" t="inlineStr"/>
       <c r="P7" s="7" t="inlineStr">
         <is>
-          <t>4,095,000,000</t>
+          <t>716,720,000</t>
         </is>
       </c>
       <c r="Q7" s="6" t="inlineStr">
         <is>
-          <t>6.5%</t>
+          <t>1.0%</t>
         </is>
       </c>
       <c r="R7" s="6" t="inlineStr">
@@ -7725,44 +7725,44 @@
     <row r="8" ht="30" customHeight="1">
       <c r="A8" s="6" t="inlineStr">
         <is>
-          <t>케이앤에스아이앤씨</t>
+          <t>인제니아테라퓨틱스</t>
         </is>
       </c>
       <c r="B8" s="6" t="inlineStr">
         <is>
-          <t>07-27~07-31</t>
+          <t>07-20~07-24</t>
         </is>
       </c>
       <c r="C8" s="6" t="inlineStr">
         <is>
-          <t>9,000~11,000</t>
+          <t>12,000~14,500</t>
         </is>
       </c>
       <c r="D8" s="7" t="inlineStr">
         <is>
-          <t>2,400,000</t>
+          <t>5,000,000</t>
         </is>
       </c>
       <c r="E8" s="7" t="inlineStr">
         <is>
-          <t>26,400,000,000</t>
+          <t>60,000,000,000</t>
         </is>
       </c>
       <c r="F8" s="6" t="inlineStr">
         <is>
-          <t>42.08배 (PER)</t>
+          <t>22.89배 (PER)</t>
         </is>
       </c>
       <c r="G8" s="6" t="inlineStr">
         <is>
-          <t>11,000</t>
+          <t>12,000</t>
         </is>
       </c>
       <c r="H8" s="6" t="n">
-        <v>938.24</v>
+        <v>50.4</v>
       </c>
       <c r="I8" s="6" t="n">
-        <v>2024</v>
+        <v>307</v>
       </c>
       <c r="J8" s="18" t="inlineStr">
         <is>
@@ -7777,23 +7777,23 @@
       <c r="L8" s="6" t="inlineStr"/>
       <c r="M8" s="6" t="inlineStr">
         <is>
-          <t>2026-08-13</t>
+          <t>2026-08-18</t>
         </is>
       </c>
       <c r="N8" s="6" t="inlineStr">
         <is>
-          <t>아이비케이투자증권</t>
+          <t>삼성증권</t>
         </is>
       </c>
       <c r="O8" s="6" t="inlineStr"/>
       <c r="P8" s="7" t="inlineStr">
         <is>
-          <t>1,500,000,000</t>
+          <t>4,095,000,000</t>
         </is>
       </c>
       <c r="Q8" s="6" t="inlineStr">
         <is>
-          <t>3.5%</t>
+          <t>6.5%</t>
         </is>
       </c>
       <c r="R8" s="6" t="inlineStr">
@@ -7805,44 +7805,44 @@
     <row r="9" ht="30" customHeight="1">
       <c r="A9" s="6" t="inlineStr">
         <is>
-          <t>딜리셔스</t>
+          <t>케이앤에스아이앤씨</t>
         </is>
       </c>
       <c r="B9" s="6" t="inlineStr">
         <is>
-          <t>07-23~07-29</t>
+          <t>07-27~07-31</t>
         </is>
       </c>
       <c r="C9" s="6" t="inlineStr">
         <is>
-          <t>5,000~7,000</t>
+          <t>9,000~11,000</t>
         </is>
       </c>
       <c r="D9" s="7" t="inlineStr">
         <is>
-          <t>2,200,000</t>
+          <t>2,400,000</t>
         </is>
       </c>
       <c r="E9" s="7" t="inlineStr">
         <is>
-          <t>15,400,000,000</t>
+          <t>26,400,000,000</t>
         </is>
       </c>
       <c r="F9" s="6" t="inlineStr">
         <is>
-          <t>23.93배 (PER)</t>
+          <t>42.08배 (PER)</t>
         </is>
       </c>
       <c r="G9" s="6" t="inlineStr">
         <is>
-          <t>7,000</t>
+          <t>11,000</t>
         </is>
       </c>
       <c r="H9" s="6" t="n">
-        <v>184.06</v>
+        <v>938.24</v>
       </c>
       <c r="I9" s="6" t="n">
-        <v>441</v>
+        <v>2024</v>
       </c>
       <c r="J9" s="18" t="inlineStr">
         <is>
@@ -7857,23 +7857,23 @@
       <c r="L9" s="6" t="inlineStr"/>
       <c r="M9" s="6" t="inlineStr">
         <is>
-          <t>2026-08-12</t>
+          <t>2026-08-13</t>
         </is>
       </c>
       <c r="N9" s="6" t="inlineStr">
         <is>
-          <t>한국투자증권</t>
+          <t>아이비케이투자증권</t>
         </is>
       </c>
       <c r="O9" s="6" t="inlineStr"/>
       <c r="P9" s="7" t="inlineStr">
         <is>
-          <t>566,500,000</t>
+          <t>1,500,000,000</t>
         </is>
       </c>
       <c r="Q9" s="6" t="inlineStr">
         <is>
-          <t>5.0%</t>
+          <t>3.5%</t>
         </is>
       </c>
       <c r="R9" s="6" t="inlineStr">
@@ -7885,44 +7885,44 @@
     <row r="10" ht="30" customHeight="1">
       <c r="A10" s="6" t="inlineStr">
         <is>
-          <t>에이치엘지노믹스</t>
+          <t>딜리셔스</t>
         </is>
       </c>
       <c r="B10" s="6" t="inlineStr">
         <is>
-          <t>07-02~07-08</t>
+          <t>07-23~07-29</t>
         </is>
       </c>
       <c r="C10" s="6" t="inlineStr">
         <is>
-          <t>18,500~21,500</t>
+          <t>5,000~7,000</t>
         </is>
       </c>
       <c r="D10" s="7" t="inlineStr">
         <is>
-          <t>2,565,000</t>
+          <t>2,200,000</t>
         </is>
       </c>
       <c r="E10" s="7" t="inlineStr">
         <is>
-          <t>55,147,500,000</t>
+          <t>15,400,000,000</t>
         </is>
       </c>
       <c r="F10" s="6" t="inlineStr">
         <is>
-          <t>12.85배 (EV/EBITDA)</t>
+          <t>23.93배 (PER)</t>
         </is>
       </c>
       <c r="G10" s="6" t="inlineStr">
         <is>
-          <t>21,500</t>
+          <t>7,000</t>
         </is>
       </c>
       <c r="H10" s="6" t="n">
-        <v>714.52</v>
+        <v>184.06</v>
       </c>
       <c r="I10" s="6" t="n">
-        <v>2148</v>
+        <v>441</v>
       </c>
       <c r="J10" s="18" t="inlineStr">
         <is>
@@ -7937,27 +7937,23 @@
       <c r="L10" s="6" t="inlineStr"/>
       <c r="M10" s="6" t="inlineStr">
         <is>
-          <t>2026-07-24</t>
+          <t>2026-08-12</t>
         </is>
       </c>
       <c r="N10" s="6" t="inlineStr">
         <is>
-          <t>KB</t>
-        </is>
-      </c>
-      <c r="O10" s="6" t="inlineStr">
-        <is>
-          <t>아이비케이투자증권, IBK투자증권, IBK투자증권, IBK투자증권, IBK투자증권, IBK투자증권㈜, 보통주, IBK투자증권㈜</t>
-        </is>
-      </c>
+          <t>한국투자증권</t>
+        </is>
+      </c>
+      <c r="O10" s="6" t="inlineStr"/>
       <c r="P10" s="7" t="inlineStr">
         <is>
-          <t>1,211</t>
+          <t>566,500,000</t>
         </is>
       </c>
       <c r="Q10" s="6" t="inlineStr">
         <is>
-          <t>2.5%</t>
+          <t>5.0%</t>
         </is>
       </c>
       <c r="R10" s="6" t="inlineStr">
@@ -7969,63 +7965,59 @@
     <row r="11" ht="30" customHeight="1">
       <c r="A11" s="6" t="inlineStr">
         <is>
-          <t>레메디</t>
-        </is>
-      </c>
-      <c r="B11" s="18" t="inlineStr">
-        <is>
-          <t>수집예정</t>
+          <t>에이치엘지노믹스</t>
+        </is>
+      </c>
+      <c r="B11" s="6" t="inlineStr">
+        <is>
+          <t>07-02~07-08</t>
         </is>
       </c>
       <c r="C11" s="6" t="inlineStr">
         <is>
-          <t>17,800~20,700</t>
+          <t>18,500~21,500</t>
         </is>
       </c>
       <c r="D11" s="7" t="inlineStr">
         <is>
-          <t>1,200,000</t>
+          <t>2,565,000</t>
         </is>
       </c>
       <c r="E11" s="7" t="inlineStr">
         <is>
-          <t>24,840,000,000</t>
+          <t>55,147,500,000</t>
         </is>
       </c>
       <c r="F11" s="6" t="inlineStr">
         <is>
-          <t>21.95배 (PER)</t>
+          <t>12.85배 (EV/EBITDA)</t>
         </is>
       </c>
       <c r="G11" s="6" t="inlineStr">
         <is>
-          <t>20,700</t>
-        </is>
-      </c>
-      <c r="H11" s="6" t="inlineStr">
-        <is>
-          <t>1,146.41</t>
-        </is>
-      </c>
-      <c r="I11" s="6" t="inlineStr">
-        <is>
-          <t>2,246</t>
-        </is>
+          <t>21,500</t>
+        </is>
+      </c>
+      <c r="H11" s="6" t="n">
+        <v>714.52</v>
+      </c>
+      <c r="I11" s="6" t="n">
+        <v>2148</v>
       </c>
       <c r="J11" s="18" t="inlineStr">
         <is>
           <t>수집예정</t>
         </is>
       </c>
-      <c r="K11" s="6" t="inlineStr">
-        <is>
-          <t>1,706.71</t>
+      <c r="K11" s="18" t="inlineStr">
+        <is>
+          <t>수집예정</t>
         </is>
       </c>
       <c r="L11" s="6" t="inlineStr"/>
       <c r="M11" s="6" t="inlineStr">
         <is>
-          <t>2026-07-13</t>
+          <t>2026-07-24</t>
         </is>
       </c>
       <c r="N11" s="6" t="inlineStr">
@@ -8033,15 +8025,19 @@
           <t>KB</t>
         </is>
       </c>
-      <c r="O11" s="6" t="inlineStr"/>
+      <c r="O11" s="6" t="inlineStr">
+        <is>
+          <t>아이비케이투자증권, IBK투자증권, IBK투자증권, IBK투자증권, IBK투자증권, IBK투자증권㈜, 보통주, IBK투자증권㈜</t>
+        </is>
+      </c>
       <c r="P11" s="7" t="inlineStr">
         <is>
-          <t>1,279</t>
+          <t>1,211</t>
         </is>
       </c>
       <c r="Q11" s="6" t="inlineStr">
         <is>
-          <t>5.0%</t>
+          <t>2.5%</t>
         </is>
       </c>
       <c r="R11" s="6" t="inlineStr">
@@ -8053,7 +8049,7 @@
     <row r="12" ht="30" customHeight="1">
       <c r="A12" s="6" t="inlineStr">
         <is>
-          <t>레몬헬스케어</t>
+          <t>레메디</t>
         </is>
       </c>
       <c r="B12" s="18" t="inlineStr">
@@ -8063,45 +8059,53 @@
       </c>
       <c r="C12" s="6" t="inlineStr">
         <is>
-          <t>7,500~10,000</t>
+          <t>17,800~20,700</t>
         </is>
       </c>
       <c r="D12" s="7" t="inlineStr">
         <is>
-          <t>2,000,000</t>
+          <t>1,200,000</t>
         </is>
       </c>
       <c r="E12" s="7" t="inlineStr">
         <is>
-          <t>20,000</t>
+          <t>24,840,000,000</t>
         </is>
       </c>
       <c r="F12" s="6" t="inlineStr">
         <is>
-          <t>25.48배 (PER)</t>
-        </is>
-      </c>
-      <c r="G12" s="6" t="n">
-        <v>10000</v>
-      </c>
-      <c r="H12" s="6" t="n">
-        <v>1238</v>
-      </c>
-      <c r="I12" s="6" t="n">
-        <v>2233</v>
-      </c>
-      <c r="J12" s="6" t="inlineStr">
-        <is>
-          <t>2026-06-24~25</t>
-        </is>
-      </c>
-      <c r="K12" s="6" t="n">
-        <v>1510.57</v>
+          <t>21.95배 (PER)</t>
+        </is>
+      </c>
+      <c r="G12" s="6" t="inlineStr">
+        <is>
+          <t>20,700</t>
+        </is>
+      </c>
+      <c r="H12" s="6" t="inlineStr">
+        <is>
+          <t>1,146.41</t>
+        </is>
+      </c>
+      <c r="I12" s="6" t="inlineStr">
+        <is>
+          <t>2,246</t>
+        </is>
+      </c>
+      <c r="J12" s="18" t="inlineStr">
+        <is>
+          <t>수집예정</t>
+        </is>
+      </c>
+      <c r="K12" s="6" t="inlineStr">
+        <is>
+          <t>1,706.71</t>
+        </is>
       </c>
       <c r="L12" s="6" t="inlineStr"/>
       <c r="M12" s="6" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-07-13</t>
         </is>
       </c>
       <c r="N12" s="6" t="inlineStr">
@@ -8112,12 +8116,12 @@
       <c r="O12" s="6" t="inlineStr"/>
       <c r="P12" s="7" t="inlineStr">
         <is>
-          <t>824</t>
+          <t>1,279</t>
         </is>
       </c>
       <c r="Q12" s="6" t="inlineStr">
         <is>
-          <t>4.0%</t>
+          <t>5.0%</t>
         </is>
       </c>
       <c r="R12" s="6" t="inlineStr">
@@ -8129,7 +8133,7 @@
     <row r="13" ht="30" customHeight="1">
       <c r="A13" s="6" t="inlineStr">
         <is>
-          <t>매드업</t>
+          <t>레몬헬스케어</t>
         </is>
       </c>
       <c r="B13" s="18" t="inlineStr">
@@ -8139,7 +8143,7 @@
       </c>
       <c r="C13" s="6" t="inlineStr">
         <is>
-          <t>7,000~8,000</t>
+          <t>7,500~10,000</t>
         </is>
       </c>
       <c r="D13" s="7" t="inlineStr">
@@ -8149,51 +8153,51 @@
       </c>
       <c r="E13" s="7" t="inlineStr">
         <is>
-          <t>16,000</t>
+          <t>20,000</t>
         </is>
       </c>
       <c r="F13" s="6" t="inlineStr">
         <is>
-          <t>24.57배 (PER)</t>
+          <t>25.48배 (PER)</t>
         </is>
       </c>
       <c r="G13" s="6" t="n">
-        <v>8000</v>
+        <v>10000</v>
       </c>
       <c r="H13" s="6" t="n">
-        <v>1396.29</v>
+        <v>1238</v>
       </c>
       <c r="I13" s="6" t="n">
-        <v>2392</v>
+        <v>2233</v>
       </c>
       <c r="J13" s="6" t="inlineStr">
         <is>
-          <t>2026-06-23~24</t>
+          <t>2026-06-24~25</t>
         </is>
       </c>
       <c r="K13" s="6" t="n">
-        <v>3304.76</v>
+        <v>1510.57</v>
       </c>
       <c r="L13" s="6" t="inlineStr"/>
       <c r="M13" s="6" t="inlineStr">
         <is>
-          <t>2026-07-01</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="N13" s="6" t="inlineStr">
         <is>
-          <t>미래</t>
+          <t>KB</t>
         </is>
       </c>
       <c r="O13" s="6" t="inlineStr"/>
       <c r="P13" s="7" t="inlineStr">
         <is>
-          <t>742</t>
+          <t>824</t>
         </is>
       </c>
       <c r="Q13" s="6" t="inlineStr">
         <is>
-          <t>4.5%</t>
+          <t>4.0%</t>
         </is>
       </c>
       <c r="R13" s="6" t="inlineStr">
@@ -8205,75 +8209,71 @@
     <row r="14" ht="30" customHeight="1">
       <c r="A14" s="6" t="inlineStr">
         <is>
-          <t>한국제16호스팩</t>
-        </is>
-      </c>
-      <c r="B14" s="19" t="inlineStr">
-        <is>
-          <t>해당없음</t>
+          <t>매드업</t>
+        </is>
+      </c>
+      <c r="B14" s="18" t="inlineStr">
+        <is>
+          <t>수집예정</t>
         </is>
       </c>
       <c r="C14" s="6" t="inlineStr">
         <is>
-          <t>2,000</t>
+          <t>7,000~8,000</t>
         </is>
       </c>
       <c r="D14" s="7" t="inlineStr">
         <is>
-          <t>5,500,000</t>
+          <t>2,000,000</t>
         </is>
       </c>
       <c r="E14" s="7" t="inlineStr">
         <is>
-          <t>11,000</t>
-        </is>
-      </c>
-      <c r="F14" s="19" t="inlineStr">
-        <is>
-          <t>해당없음</t>
-        </is>
-      </c>
-      <c r="G14" s="6" t="inlineStr">
-        <is>
-          <t>2,000</t>
-        </is>
+          <t>16,000</t>
+        </is>
+      </c>
+      <c r="F14" s="6" t="inlineStr">
+        <is>
+          <t>24.57배 (PER)</t>
+        </is>
+      </c>
+      <c r="G14" s="6" t="n">
+        <v>8000</v>
       </c>
       <c r="H14" s="6" t="n">
-        <v>1364.09</v>
+        <v>1396.29</v>
       </c>
       <c r="I14" s="6" t="n">
-        <v>2089</v>
+        <v>2392</v>
       </c>
       <c r="J14" s="6" t="inlineStr">
         <is>
-          <t>2026-06-22~06-23</t>
-        </is>
-      </c>
-      <c r="K14" s="6" t="inlineStr">
-        <is>
-          <t>1,274.77</t>
-        </is>
+          <t>2026-06-23~24</t>
+        </is>
+      </c>
+      <c r="K14" s="6" t="n">
+        <v>3304.76</v>
       </c>
       <c r="L14" s="6" t="inlineStr"/>
       <c r="M14" s="6" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-07-01</t>
         </is>
       </c>
       <c r="N14" s="6" t="inlineStr">
         <is>
-          <t>한국</t>
+          <t>미래</t>
         </is>
       </c>
       <c r="O14" s="6" t="inlineStr"/>
       <c r="P14" s="7" t="inlineStr">
         <is>
-          <t>330</t>
+          <t>742</t>
         </is>
       </c>
       <c r="Q14" s="6" t="inlineStr">
         <is>
-          <t>3.00%</t>
+          <t>4.5%</t>
         </is>
       </c>
       <c r="R14" s="6" t="inlineStr">
@@ -8285,51 +8285,53 @@
     <row r="15" ht="30" customHeight="1">
       <c r="A15" s="6" t="inlineStr">
         <is>
-          <t>스트라드비젼</t>
-        </is>
-      </c>
-      <c r="B15" s="18" t="inlineStr">
-        <is>
-          <t>수집예정</t>
+          <t>한국제16호스팩</t>
+        </is>
+      </c>
+      <c r="B15" s="19" t="inlineStr">
+        <is>
+          <t>해당없음</t>
         </is>
       </c>
       <c r="C15" s="6" t="inlineStr">
         <is>
-          <t>12,000~14,000</t>
+          <t>2,000</t>
         </is>
       </c>
       <c r="D15" s="7" t="inlineStr">
         <is>
-          <t>7,000,000</t>
+          <t>5,500,000</t>
         </is>
       </c>
       <c r="E15" s="7" t="inlineStr">
         <is>
-          <t>84,000</t>
-        </is>
-      </c>
-      <c r="F15" s="6" t="inlineStr">
-        <is>
-          <t>37.45배 (PER)</t>
-        </is>
-      </c>
-      <c r="G15" s="6" t="n">
-        <v>12000</v>
+          <t>11,000</t>
+        </is>
+      </c>
+      <c r="F15" s="19" t="inlineStr">
+        <is>
+          <t>해당없음</t>
+        </is>
+      </c>
+      <c r="G15" s="6" t="inlineStr">
+        <is>
+          <t>2,000</t>
+        </is>
       </c>
       <c r="H15" s="6" t="n">
-        <v>381.3</v>
+        <v>1364.09</v>
       </c>
       <c r="I15" s="6" t="n">
-        <v>1604</v>
+        <v>2089</v>
       </c>
       <c r="J15" s="6" t="inlineStr">
         <is>
-          <t>2026-06-18~06-19</t>
+          <t>2026-06-22~06-23</t>
         </is>
       </c>
       <c r="K15" s="6" t="inlineStr">
         <is>
-          <t>45.81</t>
+          <t>1,274.77</t>
         </is>
       </c>
       <c r="L15" s="6" t="inlineStr"/>
@@ -8340,13 +8342,13 @@
       </c>
       <c r="N15" s="6" t="inlineStr">
         <is>
-          <t>KB</t>
+          <t>한국</t>
         </is>
       </c>
       <c r="O15" s="6" t="inlineStr"/>
       <c r="P15" s="7" t="inlineStr">
         <is>
-          <t>2,575</t>
+          <t>330</t>
         </is>
       </c>
       <c r="Q15" s="6" t="inlineStr">
@@ -8363,7 +8365,7 @@
     <row r="16" ht="30" customHeight="1">
       <c r="A16" s="6" t="inlineStr">
         <is>
-          <t>져스텍</t>
+          <t>스트라드비젼</t>
         </is>
       </c>
       <c r="B16" s="18" t="inlineStr">
@@ -8373,32 +8375,32 @@
       </c>
       <c r="C16" s="6" t="inlineStr">
         <is>
-          <t>10,500~12,500</t>
+          <t>12,000~14,000</t>
         </is>
       </c>
       <c r="D16" s="7" t="inlineStr">
         <is>
-          <t>1,600,000</t>
+          <t>7,000,000</t>
         </is>
       </c>
       <c r="E16" s="7" t="inlineStr">
         <is>
-          <t>20,000</t>
+          <t>84,000</t>
         </is>
       </c>
       <c r="F16" s="6" t="inlineStr">
         <is>
-          <t>26.82배 (PER)</t>
+          <t>37.45배 (PER)</t>
         </is>
       </c>
       <c r="G16" s="6" t="n">
-        <v>12500</v>
+        <v>12000</v>
       </c>
       <c r="H16" s="6" t="n">
-        <v>1294.99</v>
+        <v>381.3</v>
       </c>
       <c r="I16" s="6" t="n">
-        <v>2252</v>
+        <v>1604</v>
       </c>
       <c r="J16" s="6" t="inlineStr">
         <is>
@@ -8407,29 +8409,29 @@
       </c>
       <c r="K16" s="6" t="inlineStr">
         <is>
-          <t>2,783.89</t>
+          <t>45.81</t>
         </is>
       </c>
       <c r="L16" s="6" t="inlineStr"/>
       <c r="M16" s="6" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="N16" s="6" t="inlineStr">
         <is>
-          <t>삼성</t>
+          <t>KB</t>
         </is>
       </c>
       <c r="O16" s="6" t="inlineStr"/>
       <c r="P16" s="7" t="inlineStr">
         <is>
-          <t>1,164</t>
+          <t>2,575</t>
         </is>
       </c>
       <c r="Q16" s="6" t="inlineStr">
         <is>
-          <t>5.65%</t>
+          <t>3.00%</t>
         </is>
       </c>
       <c r="R16" s="6" t="inlineStr">
@@ -8441,75 +8443,73 @@
     <row r="17" ht="30" customHeight="1">
       <c r="A17" s="6" t="inlineStr">
         <is>
-          <t>메리츠제2호스팩</t>
-        </is>
-      </c>
-      <c r="B17" s="19" t="inlineStr">
-        <is>
-          <t>해당없음</t>
+          <t>져스텍</t>
+        </is>
+      </c>
+      <c r="B17" s="18" t="inlineStr">
+        <is>
+          <t>수집예정</t>
         </is>
       </c>
       <c r="C17" s="6" t="inlineStr">
         <is>
-          <t>2,000</t>
+          <t>10,500~12,500</t>
         </is>
       </c>
       <c r="D17" s="7" t="inlineStr">
         <is>
-          <t>7,000,000</t>
+          <t>1,600,000</t>
         </is>
       </c>
       <c r="E17" s="7" t="inlineStr">
         <is>
-          <t>14,000</t>
-        </is>
-      </c>
-      <c r="F17" s="19" t="inlineStr">
-        <is>
-          <t>해당없음</t>
-        </is>
-      </c>
-      <c r="G17" s="6" t="inlineStr">
-        <is>
-          <t>2,000</t>
-        </is>
+          <t>20,000</t>
+        </is>
+      </c>
+      <c r="F17" s="6" t="inlineStr">
+        <is>
+          <t>26.82배 (PER)</t>
+        </is>
+      </c>
+      <c r="G17" s="6" t="n">
+        <v>12500</v>
       </c>
       <c r="H17" s="6" t="n">
-        <v>1087.58</v>
+        <v>1294.99</v>
       </c>
       <c r="I17" s="6" t="n">
-        <v>1798</v>
+        <v>2252</v>
       </c>
       <c r="J17" s="6" t="inlineStr">
         <is>
-          <t>2026-06-09~06-10</t>
+          <t>2026-06-18~06-19</t>
         </is>
       </c>
       <c r="K17" s="6" t="inlineStr">
         <is>
-          <t>1,338.66</t>
+          <t>2,783.89</t>
         </is>
       </c>
       <c r="L17" s="6" t="inlineStr"/>
       <c r="M17" s="6" t="inlineStr">
         <is>
-          <t>2026-06-19</t>
+          <t>2026-06-29</t>
         </is>
       </c>
       <c r="N17" s="6" t="inlineStr">
         <is>
-          <t>메리츠</t>
+          <t>삼성</t>
         </is>
       </c>
       <c r="O17" s="6" t="inlineStr"/>
       <c r="P17" s="7" t="inlineStr">
         <is>
-          <t>245</t>
+          <t>1,164</t>
         </is>
       </c>
       <c r="Q17" s="6" t="inlineStr">
         <is>
-          <t>1.75%</t>
+          <t>5.65%</t>
         </is>
       </c>
       <c r="R17" s="6" t="inlineStr">
@@ -8521,77 +8521,75 @@
     <row r="18" ht="30" customHeight="1">
       <c r="A18" s="6" t="inlineStr">
         <is>
-          <t>피스피스스튜디오</t>
-        </is>
-      </c>
-      <c r="B18" s="18" t="inlineStr">
-        <is>
-          <t>수집예정</t>
+          <t>메리츠제2호스팩</t>
+        </is>
+      </c>
+      <c r="B18" s="19" t="inlineStr">
+        <is>
+          <t>해당없음</t>
         </is>
       </c>
       <c r="C18" s="6" t="inlineStr">
         <is>
-          <t>19,000~21,500</t>
+          <t>2,000</t>
         </is>
       </c>
       <c r="D18" s="7" t="inlineStr">
         <is>
-          <t>2,272,637</t>
+          <t>7,000,000</t>
         </is>
       </c>
       <c r="E18" s="7" t="inlineStr">
         <is>
-          <t>48,862</t>
-        </is>
-      </c>
-      <c r="F18" s="6" t="inlineStr">
-        <is>
-          <t>21.48배 (PER)</t>
-        </is>
-      </c>
-      <c r="G18" s="6" t="n">
-        <v>21500</v>
+          <t>14,000</t>
+        </is>
+      </c>
+      <c r="F18" s="19" t="inlineStr">
+        <is>
+          <t>해당없음</t>
+        </is>
+      </c>
+      <c r="G18" s="6" t="inlineStr">
+        <is>
+          <t>2,000</t>
+        </is>
       </c>
       <c r="H18" s="6" t="n">
-        <v>847.76</v>
+        <v>1087.58</v>
       </c>
       <c r="I18" s="6" t="n">
-        <v>2329</v>
+        <v>1798</v>
       </c>
       <c r="J18" s="6" t="inlineStr">
         <is>
-          <t>2026-05-26~05-27</t>
+          <t>2026-06-09~06-10</t>
         </is>
       </c>
       <c r="K18" s="6" t="inlineStr">
         <is>
-          <t>1,191.15</t>
+          <t>1,338.66</t>
         </is>
       </c>
       <c r="L18" s="6" t="inlineStr"/>
       <c r="M18" s="6" t="inlineStr">
         <is>
-          <t>2026-06-08</t>
+          <t>2026-06-19</t>
         </is>
       </c>
       <c r="N18" s="6" t="inlineStr">
         <is>
-          <t>미래</t>
-        </is>
-      </c>
-      <c r="O18" s="6" t="inlineStr">
-        <is>
-          <t>NH</t>
-        </is>
-      </c>
+          <t>메리츠</t>
+        </is>
+      </c>
+      <c r="O18" s="6" t="inlineStr"/>
       <c r="P18" s="7" t="inlineStr">
         <is>
-          <t>1,994</t>
+          <t>245</t>
         </is>
       </c>
       <c r="Q18" s="6" t="inlineStr">
         <is>
-          <t>4.00%</t>
+          <t>1.75%</t>
         </is>
       </c>
       <c r="R18" s="6" t="inlineStr">
@@ -8603,75 +8601,77 @@
     <row r="19" ht="30" customHeight="1">
       <c r="A19" s="6" t="inlineStr">
         <is>
-          <t>대신밸런스제20호스팩</t>
-        </is>
-      </c>
-      <c r="B19" s="19" t="inlineStr">
-        <is>
-          <t>해당없음</t>
+          <t>피스피스스튜디오</t>
+        </is>
+      </c>
+      <c r="B19" s="18" t="inlineStr">
+        <is>
+          <t>수집예정</t>
         </is>
       </c>
       <c r="C19" s="6" t="inlineStr">
         <is>
-          <t>2,000</t>
+          <t>19,000~21,500</t>
         </is>
       </c>
       <c r="D19" s="7" t="inlineStr">
         <is>
-          <t>6,500,000</t>
+          <t>2,272,637</t>
         </is>
       </c>
       <c r="E19" s="7" t="inlineStr">
         <is>
-          <t>13,000</t>
-        </is>
-      </c>
-      <c r="F19" s="19" t="inlineStr">
-        <is>
-          <t>해당없음</t>
-        </is>
-      </c>
-      <c r="G19" s="6" t="inlineStr">
-        <is>
-          <t>2,000</t>
-        </is>
+          <t>48,862</t>
+        </is>
+      </c>
+      <c r="F19" s="6" t="inlineStr">
+        <is>
+          <t>21.48배 (PER)</t>
+        </is>
+      </c>
+      <c r="G19" s="6" t="n">
+        <v>21500</v>
       </c>
       <c r="H19" s="6" t="n">
-        <v>1327.13</v>
+        <v>847.76</v>
       </c>
       <c r="I19" s="6" t="n">
-        <v>2194</v>
+        <v>2329</v>
       </c>
       <c r="J19" s="6" t="inlineStr">
         <is>
-          <t>2026-05-22~05-25</t>
+          <t>2026-05-26~05-27</t>
         </is>
       </c>
       <c r="K19" s="6" t="inlineStr">
         <is>
-          <t>1,486.88</t>
+          <t>1,191.15</t>
         </is>
       </c>
       <c r="L19" s="6" t="inlineStr"/>
       <c r="M19" s="6" t="inlineStr">
         <is>
-          <t>2026-06-05</t>
+          <t>2026-06-08</t>
         </is>
       </c>
       <c r="N19" s="6" t="inlineStr">
         <is>
-          <t>대신</t>
-        </is>
-      </c>
-      <c r="O19" s="6" t="inlineStr"/>
+          <t>미래</t>
+        </is>
+      </c>
+      <c r="O19" s="6" t="inlineStr">
+        <is>
+          <t>NH</t>
+        </is>
+      </c>
       <c r="P19" s="7" t="inlineStr">
         <is>
-          <t>390</t>
+          <t>1,994</t>
         </is>
       </c>
       <c r="Q19" s="6" t="inlineStr">
         <is>
-          <t>3.00%</t>
+          <t>4.00%</t>
         </is>
       </c>
       <c r="R19" s="6" t="inlineStr">
@@ -8683,73 +8683,75 @@
     <row r="20" ht="30" customHeight="1">
       <c r="A20" s="6" t="inlineStr">
         <is>
-          <t>마키나락스</t>
-        </is>
-      </c>
-      <c r="B20" s="18" t="inlineStr">
-        <is>
-          <t>수집예정</t>
+          <t>대신밸런스제20호스팩</t>
+        </is>
+      </c>
+      <c r="B20" s="19" t="inlineStr">
+        <is>
+          <t>해당없음</t>
         </is>
       </c>
       <c r="C20" s="6" t="inlineStr">
         <is>
-          <t>12,500~15,000</t>
+          <t>2,000</t>
         </is>
       </c>
       <c r="D20" s="7" t="inlineStr">
         <is>
-          <t>2,635,000</t>
+          <t>6,500,000</t>
         </is>
       </c>
       <c r="E20" s="7" t="inlineStr">
         <is>
-          <t>39,525</t>
-        </is>
-      </c>
-      <c r="F20" s="6" t="inlineStr">
-        <is>
-          <t>40.5배 (PER)</t>
-        </is>
-      </c>
-      <c r="G20" s="6" t="n">
-        <v>15000</v>
+          <t>13,000</t>
+        </is>
+      </c>
+      <c r="F20" s="19" t="inlineStr">
+        <is>
+          <t>해당없음</t>
+        </is>
+      </c>
+      <c r="G20" s="6" t="inlineStr">
+        <is>
+          <t>2,000</t>
+        </is>
       </c>
       <c r="H20" s="6" t="n">
-        <v>1196.08</v>
+        <v>1327.13</v>
       </c>
       <c r="I20" s="6" t="n">
-        <v>2427</v>
+        <v>2194</v>
       </c>
       <c r="J20" s="6" t="inlineStr">
         <is>
-          <t>2026-05-11~05-12</t>
+          <t>2026-05-22~05-25</t>
         </is>
       </c>
       <c r="K20" s="6" t="inlineStr">
         <is>
-          <t>2,807.79</t>
+          <t>1,486.88</t>
         </is>
       </c>
       <c r="L20" s="6" t="inlineStr"/>
       <c r="M20" s="6" t="inlineStr">
         <is>
-          <t>2026-05-20</t>
+          <t>2026-06-05</t>
         </is>
       </c>
       <c r="N20" s="6" t="inlineStr">
         <is>
-          <t>미래</t>
+          <t>대신</t>
         </is>
       </c>
       <c r="O20" s="6" t="inlineStr"/>
       <c r="P20" s="7" t="inlineStr">
         <is>
-          <t>2,026</t>
+          <t>390</t>
         </is>
       </c>
       <c r="Q20" s="6" t="inlineStr">
         <is>
-          <t>5.00%</t>
+          <t>3.00%</t>
         </is>
       </c>
       <c r="R20" s="6" t="inlineStr">
@@ -8761,7 +8763,7 @@
     <row r="21" ht="30" customHeight="1">
       <c r="A21" s="6" t="inlineStr">
         <is>
-          <t>폴레드</t>
+          <t>마키나락스</t>
         </is>
       </c>
       <c r="B21" s="18" t="inlineStr">
@@ -8771,63 +8773,63 @@
       </c>
       <c r="C21" s="6" t="inlineStr">
         <is>
-          <t>4,100~5,000</t>
+          <t>12,500~15,000</t>
         </is>
       </c>
       <c r="D21" s="7" t="inlineStr">
         <is>
-          <t>2,600,000</t>
+          <t>2,635,000</t>
         </is>
       </c>
       <c r="E21" s="7" t="inlineStr">
         <is>
-          <t>13,000</t>
+          <t>39,525</t>
         </is>
       </c>
       <c r="F21" s="6" t="inlineStr">
         <is>
-          <t>19.05배 (PER)</t>
+          <t>40.5배 (PER)</t>
         </is>
       </c>
       <c r="G21" s="6" t="n">
-        <v>5000</v>
+        <v>15000</v>
       </c>
       <c r="H21" s="6" t="n">
-        <v>1486.66</v>
+        <v>1196.08</v>
       </c>
       <c r="I21" s="6" t="n">
-        <v>2372</v>
+        <v>2427</v>
       </c>
       <c r="J21" s="6" t="inlineStr">
         <is>
-          <t>2026-05-04~05-05</t>
+          <t>2026-05-11~05-12</t>
         </is>
       </c>
       <c r="K21" s="6" t="inlineStr">
         <is>
-          <t>3,169.86</t>
+          <t>2,807.79</t>
         </is>
       </c>
       <c r="L21" s="6" t="inlineStr"/>
       <c r="M21" s="6" t="inlineStr">
         <is>
-          <t>2026-05-14</t>
+          <t>2026-05-20</t>
         </is>
       </c>
       <c r="N21" s="6" t="inlineStr">
         <is>
-          <t>NH</t>
+          <t>미래</t>
         </is>
       </c>
       <c r="O21" s="6" t="inlineStr"/>
       <c r="P21" s="7" t="inlineStr">
         <is>
-          <t>540</t>
+          <t>2,026</t>
         </is>
       </c>
       <c r="Q21" s="6" t="inlineStr">
         <is>
-          <t>4.03%</t>
+          <t>5.00%</t>
         </is>
       </c>
       <c r="R21" s="6" t="inlineStr">
@@ -8839,7 +8841,7 @@
     <row r="22" ht="30" customHeight="1">
       <c r="A22" s="6" t="inlineStr">
         <is>
-          <t>코스모로보틱스</t>
+          <t>폴레드</t>
         </is>
       </c>
       <c r="B22" s="18" t="inlineStr">
@@ -8849,67 +8851,63 @@
       </c>
       <c r="C22" s="6" t="inlineStr">
         <is>
-          <t>5,300~6,000</t>
+          <t>4,100~5,000</t>
         </is>
       </c>
       <c r="D22" s="7" t="inlineStr">
         <is>
-          <t>4,170,000</t>
+          <t>2,600,000</t>
         </is>
       </c>
       <c r="E22" s="7" t="inlineStr">
         <is>
-          <t>25,020</t>
+          <t>13,000</t>
         </is>
       </c>
       <c r="F22" s="6" t="inlineStr">
         <is>
-          <t>47.45배 (PER)</t>
+          <t>19.05배 (PER)</t>
         </is>
       </c>
       <c r="G22" s="6" t="n">
-        <v>6000</v>
+        <v>5000</v>
       </c>
       <c r="H22" s="6" t="n">
-        <v>1140.11</v>
+        <v>1486.66</v>
       </c>
       <c r="I22" s="6" t="n">
-        <v>2257</v>
+        <v>2372</v>
       </c>
       <c r="J22" s="6" t="inlineStr">
         <is>
-          <t>2026-04-27~04-28</t>
+          <t>2026-05-04~05-05</t>
         </is>
       </c>
       <c r="K22" s="6" t="inlineStr">
         <is>
-          <t>2,013.80</t>
+          <t>3,169.86</t>
         </is>
       </c>
       <c r="L22" s="6" t="inlineStr"/>
       <c r="M22" s="6" t="inlineStr">
         <is>
-          <t>2026-05-11</t>
+          <t>2026-05-14</t>
         </is>
       </c>
       <c r="N22" s="6" t="inlineStr">
         <is>
-          <t>유진</t>
-        </is>
-      </c>
-      <c r="O22" s="6" t="inlineStr">
-        <is>
           <t>NH</t>
         </is>
       </c>
+      <c r="O22" s="6" t="inlineStr"/>
       <c r="P22" s="7" t="inlineStr">
         <is>
-          <t>1,289</t>
+          <t>540</t>
         </is>
       </c>
       <c r="Q22" s="6" t="inlineStr">
         <is>
-          <t>3.78%</t>
+          <t>4.03%</t>
         </is>
       </c>
       <c r="R22" s="6" t="inlineStr">
@@ -8921,75 +8919,77 @@
     <row r="23" ht="30" customHeight="1">
       <c r="A23" s="6" t="inlineStr">
         <is>
-          <t>신한스팩18호</t>
-        </is>
-      </c>
-      <c r="B23" s="19" t="inlineStr">
-        <is>
-          <t>해당없음</t>
+          <t>코스모로보틱스</t>
+        </is>
+      </c>
+      <c r="B23" s="18" t="inlineStr">
+        <is>
+          <t>수집예정</t>
         </is>
       </c>
       <c r="C23" s="6" t="inlineStr">
         <is>
-          <t>2,000</t>
+          <t>5,300~6,000</t>
         </is>
       </c>
       <c r="D23" s="7" t="inlineStr">
         <is>
-          <t>5,000,000</t>
+          <t>4,170,000</t>
         </is>
       </c>
       <c r="E23" s="7" t="inlineStr">
         <is>
-          <t>10,000</t>
-        </is>
-      </c>
-      <c r="F23" s="19" t="inlineStr">
-        <is>
-          <t>해당없음</t>
-        </is>
-      </c>
-      <c r="G23" s="6" t="inlineStr">
-        <is>
-          <t>2,000</t>
-        </is>
+          <t>25,020</t>
+        </is>
+      </c>
+      <c r="F23" s="6" t="inlineStr">
+        <is>
+          <t>47.45배 (PER)</t>
+        </is>
+      </c>
+      <c r="G23" s="6" t="n">
+        <v>6000</v>
       </c>
       <c r="H23" s="6" t="n">
-        <v>1388.6</v>
+        <v>1140.11</v>
       </c>
       <c r="I23" s="6" t="n">
-        <v>2044</v>
+        <v>2257</v>
       </c>
       <c r="J23" s="6" t="inlineStr">
         <is>
-          <t>2026-04-20~04-21</t>
+          <t>2026-04-27~04-28</t>
         </is>
       </c>
       <c r="K23" s="6" t="inlineStr">
         <is>
-          <t>1,601.36</t>
+          <t>2,013.80</t>
         </is>
       </c>
       <c r="L23" s="6" t="inlineStr"/>
       <c r="M23" s="6" t="inlineStr">
         <is>
-          <t>2026-04-30</t>
+          <t>2026-05-11</t>
         </is>
       </c>
       <c r="N23" s="6" t="inlineStr">
         <is>
-          <t>신한</t>
-        </is>
-      </c>
-      <c r="O23" s="6" t="inlineStr"/>
+          <t>유진</t>
+        </is>
+      </c>
+      <c r="O23" s="6" t="inlineStr">
+        <is>
+          <t>NH</t>
+        </is>
+      </c>
       <c r="P23" s="7" t="inlineStr">
         <is>
-          <t>350</t>
+          <t>1,289</t>
         </is>
       </c>
       <c r="Q23" s="6" t="inlineStr">
         <is>
-          <t>3.50%</t>
+          <t>3.78%</t>
         </is>
       </c>
       <c r="R23" s="6" t="inlineStr">
@@ -9001,42 +9001,44 @@
     <row r="24" ht="30" customHeight="1">
       <c r="A24" s="6" t="inlineStr">
         <is>
-          <t>채비</t>
-        </is>
-      </c>
-      <c r="B24" s="18" t="inlineStr">
-        <is>
-          <t>수집예정</t>
+          <t>신한스팩18호</t>
+        </is>
+      </c>
+      <c r="B24" s="19" t="inlineStr">
+        <is>
+          <t>해당없음</t>
         </is>
       </c>
       <c r="C24" s="6" t="inlineStr">
         <is>
-          <t>12,300~15,300</t>
+          <t>2,000</t>
         </is>
       </c>
       <c r="D24" s="7" t="inlineStr">
         <is>
-          <t>9,000,000</t>
+          <t>5,000,000</t>
         </is>
       </c>
       <c r="E24" s="7" t="inlineStr">
         <is>
-          <t>110,700</t>
-        </is>
-      </c>
-      <c r="F24" s="6" t="inlineStr">
-        <is>
-          <t>24.0배 (EV/EBITDA)</t>
-        </is>
-      </c>
-      <c r="G24" s="6" t="n">
-        <v>12300</v>
+          <t>10,000</t>
+        </is>
+      </c>
+      <c r="F24" s="19" t="inlineStr">
+        <is>
+          <t>해당없음</t>
+        </is>
+      </c>
+      <c r="G24" s="6" t="inlineStr">
+        <is>
+          <t>2,000</t>
+        </is>
       </c>
       <c r="H24" s="6" t="n">
-        <v>55.23</v>
+        <v>1388.6</v>
       </c>
       <c r="I24" s="6" t="n">
-        <v>751</v>
+        <v>2044</v>
       </c>
       <c r="J24" s="6" t="inlineStr">
         <is>
@@ -9045,33 +9047,29 @@
       </c>
       <c r="K24" s="6" t="inlineStr">
         <is>
-          <t>302.11</t>
+          <t>1,601.36</t>
         </is>
       </c>
       <c r="L24" s="6" t="inlineStr"/>
       <c r="M24" s="6" t="inlineStr">
         <is>
-          <t>2026-04-29</t>
+          <t>2026-04-30</t>
         </is>
       </c>
       <c r="N24" s="6" t="inlineStr">
         <is>
-          <t>KB</t>
-        </is>
-      </c>
-      <c r="O24" s="6" t="inlineStr">
-        <is>
-          <t>삼성</t>
-        </is>
-      </c>
+          <t>신한</t>
+        </is>
+      </c>
+      <c r="O24" s="6" t="inlineStr"/>
       <c r="P24" s="7" t="inlineStr">
         <is>
-          <t>3,384</t>
+          <t>350</t>
         </is>
       </c>
       <c r="Q24" s="6" t="inlineStr">
         <is>
-          <t>3.00%</t>
+          <t>3.50%</t>
         </is>
       </c>
       <c r="R24" s="6" t="inlineStr">
@@ -9083,75 +9081,77 @@
     <row r="25" ht="30" customHeight="1">
       <c r="A25" s="6" t="inlineStr">
         <is>
-          <t>키움히어로스펙2호</t>
-        </is>
-      </c>
-      <c r="B25" s="19" t="inlineStr">
-        <is>
-          <t>해당없음</t>
+          <t>채비</t>
+        </is>
+      </c>
+      <c r="B25" s="18" t="inlineStr">
+        <is>
+          <t>수집예정</t>
         </is>
       </c>
       <c r="C25" s="6" t="inlineStr">
         <is>
-          <t>2,000</t>
+          <t>12,300~15,300</t>
         </is>
       </c>
       <c r="D25" s="7" t="inlineStr">
         <is>
-          <t>6,000,000</t>
+          <t>9,000,000</t>
         </is>
       </c>
       <c r="E25" s="7" t="inlineStr">
         <is>
-          <t>12,000</t>
-        </is>
-      </c>
-      <c r="F25" s="19" t="inlineStr">
-        <is>
-          <t>해당없음</t>
-        </is>
-      </c>
-      <c r="G25" s="6" t="inlineStr">
-        <is>
-          <t>2,000</t>
-        </is>
+          <t>110,700</t>
+        </is>
+      </c>
+      <c r="F25" s="6" t="inlineStr">
+        <is>
+          <t>24.0배 (EV/EBITDA)</t>
+        </is>
+      </c>
+      <c r="G25" s="6" t="n">
+        <v>12300</v>
       </c>
       <c r="H25" s="6" t="n">
-        <v>1271.12</v>
+        <v>55.23</v>
       </c>
       <c r="I25" s="6" t="n">
-        <v>2054</v>
+        <v>751</v>
       </c>
       <c r="J25" s="6" t="inlineStr">
         <is>
-          <t>2026-04-14~04-15</t>
+          <t>2026-04-20~04-21</t>
         </is>
       </c>
       <c r="K25" s="6" t="inlineStr">
         <is>
-          <t>1,727.59</t>
+          <t>302.11</t>
         </is>
       </c>
       <c r="L25" s="6" t="inlineStr"/>
       <c r="M25" s="6" t="inlineStr">
         <is>
-          <t>2026-04-23</t>
+          <t>2026-04-29</t>
         </is>
       </c>
       <c r="N25" s="6" t="inlineStr">
         <is>
-          <t>키움</t>
-        </is>
-      </c>
-      <c r="O25" s="6" t="inlineStr"/>
+          <t>KB</t>
+        </is>
+      </c>
+      <c r="O25" s="6" t="inlineStr">
+        <is>
+          <t>삼성</t>
+        </is>
+      </c>
       <c r="P25" s="7" t="inlineStr">
         <is>
-          <t>300</t>
+          <t>3,384</t>
         </is>
       </c>
       <c r="Q25" s="6" t="inlineStr">
         <is>
-          <t>2.50%</t>
+          <t>3.00%</t>
         </is>
       </c>
       <c r="R25" s="6" t="inlineStr">
@@ -9163,7 +9163,7 @@
     <row r="26" ht="30" customHeight="1">
       <c r="A26" s="6" t="inlineStr">
         <is>
-          <t>교보스팩20호</t>
+          <t>키움히어로스펙2호</t>
         </is>
       </c>
       <c r="B26" s="19" t="inlineStr">
@@ -9178,12 +9178,12 @@
       </c>
       <c r="D26" s="7" t="inlineStr">
         <is>
-          <t>5,400,000</t>
+          <t>6,000,000</t>
         </is>
       </c>
       <c r="E26" s="7" t="inlineStr">
         <is>
-          <t>10,800</t>
+          <t>12,000</t>
         </is>
       </c>
       <c r="F26" s="19" t="inlineStr">
@@ -9197,30 +9197,30 @@
         </is>
       </c>
       <c r="H26" s="6" t="n">
-        <v>1196.99</v>
+        <v>1271.12</v>
       </c>
       <c r="I26" s="6" t="n">
-        <v>1855</v>
+        <v>2054</v>
       </c>
       <c r="J26" s="6" t="inlineStr">
         <is>
-          <t>2026-03-23~03-24</t>
+          <t>2026-04-14~04-15</t>
         </is>
       </c>
       <c r="K26" s="6" t="inlineStr">
         <is>
-          <t>747.00</t>
+          <t>1,727.59</t>
         </is>
       </c>
       <c r="L26" s="6" t="inlineStr"/>
       <c r="M26" s="6" t="inlineStr">
         <is>
-          <t>2026-04-02</t>
+          <t>2026-04-23</t>
         </is>
       </c>
       <c r="N26" s="6" t="inlineStr">
         <is>
-          <t>교보</t>
+          <t>키움</t>
         </is>
       </c>
       <c r="O26" s="6" t="inlineStr"/>
@@ -9231,7 +9231,7 @@
       </c>
       <c r="Q26" s="6" t="inlineStr">
         <is>
-          <t>2.78%</t>
+          <t>2.50%</t>
         </is>
       </c>
       <c r="R26" s="6" t="inlineStr">
@@ -9243,42 +9243,44 @@
     <row r="27" ht="30" customHeight="1">
       <c r="A27" s="6" t="inlineStr">
         <is>
-          <t>인벤테라</t>
-        </is>
-      </c>
-      <c r="B27" s="18" t="inlineStr">
-        <is>
-          <t>수집예정</t>
+          <t>교보스팩20호</t>
+        </is>
+      </c>
+      <c r="B27" s="19" t="inlineStr">
+        <is>
+          <t>해당없음</t>
         </is>
       </c>
       <c r="C27" s="6" t="inlineStr">
         <is>
-          <t>12,100~16,600</t>
+          <t>2,000</t>
         </is>
       </c>
       <c r="D27" s="7" t="inlineStr">
         <is>
-          <t>1,180,000</t>
+          <t>5,400,000</t>
         </is>
       </c>
       <c r="E27" s="7" t="inlineStr">
         <is>
-          <t>19,588</t>
-        </is>
-      </c>
-      <c r="F27" s="6" t="inlineStr">
-        <is>
-          <t>24.34배 (PER)</t>
-        </is>
-      </c>
-      <c r="G27" s="6" t="n">
-        <v>16600</v>
+          <t>10,800</t>
+        </is>
+      </c>
+      <c r="F27" s="19" t="inlineStr">
+        <is>
+          <t>해당없음</t>
+        </is>
+      </c>
+      <c r="G27" s="6" t="inlineStr">
+        <is>
+          <t>2,000</t>
+        </is>
       </c>
       <c r="H27" s="6" t="n">
-        <v>1328.82</v>
+        <v>1196.99</v>
       </c>
       <c r="I27" s="6" t="n">
-        <v>2309</v>
+        <v>1855</v>
       </c>
       <c r="J27" s="6" t="inlineStr">
         <is>
@@ -9287,7 +9289,7 @@
       </c>
       <c r="K27" s="6" t="inlineStr">
         <is>
-          <t>1,913.00</t>
+          <t>747.00</t>
         </is>
       </c>
       <c r="L27" s="6" t="inlineStr"/>
@@ -9298,18 +9300,18 @@
       </c>
       <c r="N27" s="6" t="inlineStr">
         <is>
-          <t>NH</t>
+          <t>교보</t>
         </is>
       </c>
       <c r="O27" s="6" t="inlineStr"/>
       <c r="P27" s="7" t="inlineStr">
         <is>
-          <t>1,211</t>
+          <t>300</t>
         </is>
       </c>
       <c r="Q27" s="6" t="inlineStr">
         <is>
-          <t>6.00%</t>
+          <t>2.78%</t>
         </is>
       </c>
       <c r="R27" s="6" t="inlineStr">
@@ -9321,75 +9323,73 @@
     <row r="28" ht="30" customHeight="1">
       <c r="A28" s="6" t="inlineStr">
         <is>
-          <t>신한스팩17호</t>
-        </is>
-      </c>
-      <c r="B28" s="19" t="inlineStr">
-        <is>
-          <t>해당없음</t>
+          <t>인벤테라</t>
+        </is>
+      </c>
+      <c r="B28" s="18" t="inlineStr">
+        <is>
+          <t>수집예정</t>
         </is>
       </c>
       <c r="C28" s="6" t="inlineStr">
         <is>
-          <t>2,000</t>
+          <t>12,100~16,600</t>
         </is>
       </c>
       <c r="D28" s="7" t="inlineStr">
         <is>
-          <t>5,000,000</t>
+          <t>1,180,000</t>
         </is>
       </c>
       <c r="E28" s="7" t="inlineStr">
         <is>
-          <t>10,000</t>
-        </is>
-      </c>
-      <c r="F28" s="19" t="inlineStr">
-        <is>
-          <t>해당없음</t>
-        </is>
-      </c>
-      <c r="G28" s="6" t="inlineStr">
-        <is>
-          <t>2,000</t>
-        </is>
+          <t>19,588</t>
+        </is>
+      </c>
+      <c r="F28" s="6" t="inlineStr">
+        <is>
+          <t>24.34배 (PER)</t>
+        </is>
+      </c>
+      <c r="G28" s="6" t="n">
+        <v>16600</v>
       </c>
       <c r="H28" s="6" t="n">
-        <v>1343.8</v>
+        <v>1328.82</v>
       </c>
       <c r="I28" s="6" t="n">
-        <v>2022</v>
+        <v>2309</v>
       </c>
       <c r="J28" s="6" t="inlineStr">
         <is>
-          <t>2026-03-19~03-20</t>
+          <t>2026-03-23~03-24</t>
         </is>
       </c>
       <c r="K28" s="6" t="inlineStr">
         <is>
-          <t>1,403.74</t>
+          <t>1,913.00</t>
         </is>
       </c>
       <c r="L28" s="6" t="inlineStr"/>
       <c r="M28" s="6" t="inlineStr">
         <is>
-          <t>2026-04-01</t>
+          <t>2026-04-02</t>
         </is>
       </c>
       <c r="N28" s="6" t="inlineStr">
         <is>
-          <t>신한</t>
+          <t>NH</t>
         </is>
       </c>
       <c r="O28" s="6" t="inlineStr"/>
       <c r="P28" s="7" t="inlineStr">
         <is>
-          <t>350</t>
+          <t>1,211</t>
         </is>
       </c>
       <c r="Q28" s="6" t="inlineStr">
         <is>
-          <t>3.50%</t>
+          <t>6.00%</t>
         </is>
       </c>
       <c r="R28" s="6" t="inlineStr">
@@ -9401,42 +9401,44 @@
     <row r="29" ht="30" customHeight="1">
       <c r="A29" s="6" t="inlineStr">
         <is>
-          <t>리센스메디컬</t>
-        </is>
-      </c>
-      <c r="B29" s="18" t="inlineStr">
-        <is>
-          <t>수집예정</t>
+          <t>신한스팩17호</t>
+        </is>
+      </c>
+      <c r="B29" s="19" t="inlineStr">
+        <is>
+          <t>해당없음</t>
         </is>
       </c>
       <c r="C29" s="6" t="inlineStr">
         <is>
-          <t>9,000~11,000</t>
+          <t>2,000</t>
         </is>
       </c>
       <c r="D29" s="7" t="inlineStr">
         <is>
-          <t>1,400,000</t>
+          <t>5,000,000</t>
         </is>
       </c>
       <c r="E29" s="7" t="inlineStr">
         <is>
-          <t>15,400</t>
-        </is>
-      </c>
-      <c r="F29" s="6" t="inlineStr">
-        <is>
-          <t>31.33배 (PER)</t>
-        </is>
-      </c>
-      <c r="G29" s="6" t="n">
-        <v>11000</v>
+          <t>10,000</t>
+        </is>
+      </c>
+      <c r="F29" s="19" t="inlineStr">
+        <is>
+          <t>해당없음</t>
+        </is>
+      </c>
+      <c r="G29" s="6" t="inlineStr">
+        <is>
+          <t>2,000</t>
+        </is>
       </c>
       <c r="H29" s="6" t="n">
-        <v>1352.63</v>
+        <v>1343.8</v>
       </c>
       <c r="I29" s="6" t="n">
-        <v>2261</v>
+        <v>2022</v>
       </c>
       <c r="J29" s="6" t="inlineStr">
         <is>
@@ -9445,33 +9447,29 @@
       </c>
       <c r="K29" s="6" t="inlineStr">
         <is>
-          <t>2,097.68</t>
+          <t>1,403.74</t>
         </is>
       </c>
       <c r="L29" s="6" t="inlineStr"/>
       <c r="M29" s="6" t="inlineStr">
         <is>
-          <t>2026-03-31</t>
+          <t>2026-04-01</t>
         </is>
       </c>
       <c r="N29" s="6" t="inlineStr">
         <is>
-          <t>한국</t>
-        </is>
-      </c>
-      <c r="O29" s="6" t="inlineStr">
-        <is>
-          <t>KB</t>
-        </is>
-      </c>
+          <t>신한</t>
+        </is>
+      </c>
+      <c r="O29" s="6" t="inlineStr"/>
       <c r="P29" s="7" t="inlineStr">
         <is>
-          <t>916</t>
+          <t>350</t>
         </is>
       </c>
       <c r="Q29" s="6" t="inlineStr">
         <is>
-          <t>5.77%</t>
+          <t>3.50%</t>
         </is>
       </c>
       <c r="R29" s="6" t="inlineStr">
@@ -9483,75 +9481,77 @@
     <row r="30" ht="30" customHeight="1">
       <c r="A30" s="6" t="inlineStr">
         <is>
-          <t>NH스팩33호</t>
-        </is>
-      </c>
-      <c r="B30" s="19" t="inlineStr">
-        <is>
-          <t>해당없음</t>
+          <t>리센스메디컬</t>
+        </is>
+      </c>
+      <c r="B30" s="18" t="inlineStr">
+        <is>
+          <t>수집예정</t>
         </is>
       </c>
       <c r="C30" s="6" t="inlineStr">
         <is>
-          <t>2,000</t>
+          <t>9,000~11,000</t>
         </is>
       </c>
       <c r="D30" s="7" t="inlineStr">
         <is>
-          <t>6,350,000</t>
+          <t>1,400,000</t>
         </is>
       </c>
       <c r="E30" s="7" t="inlineStr">
         <is>
-          <t>12,700</t>
-        </is>
-      </c>
-      <c r="F30" s="19" t="inlineStr">
-        <is>
-          <t>해당없음</t>
-        </is>
-      </c>
-      <c r="G30" s="6" t="inlineStr">
-        <is>
-          <t>2,000</t>
-        </is>
+          <t>15,400</t>
+        </is>
+      </c>
+      <c r="F30" s="6" t="inlineStr">
+        <is>
+          <t>31.33배 (PER)</t>
+        </is>
+      </c>
+      <c r="G30" s="6" t="n">
+        <v>11000</v>
       </c>
       <c r="H30" s="6" t="n">
-        <v>1228.71</v>
+        <v>1352.63</v>
       </c>
       <c r="I30" s="6" t="n">
-        <v>2058</v>
+        <v>2261</v>
       </c>
       <c r="J30" s="6" t="inlineStr">
         <is>
-          <t>2026-03-17~03-18</t>
+          <t>2026-03-19~03-20</t>
         </is>
       </c>
       <c r="K30" s="6" t="inlineStr">
         <is>
-          <t>569.27</t>
+          <t>2,097.68</t>
         </is>
       </c>
       <c r="L30" s="6" t="inlineStr"/>
       <c r="M30" s="6" t="inlineStr">
         <is>
-          <t>2026-03-27</t>
+          <t>2026-03-31</t>
         </is>
       </c>
       <c r="N30" s="6" t="inlineStr">
         <is>
-          <t>NH</t>
-        </is>
-      </c>
-      <c r="O30" s="6" t="inlineStr"/>
+          <t>한국</t>
+        </is>
+      </c>
+      <c r="O30" s="6" t="inlineStr">
+        <is>
+          <t>KB</t>
+        </is>
+      </c>
       <c r="P30" s="7" t="inlineStr">
         <is>
-          <t>381</t>
+          <t>916</t>
         </is>
       </c>
       <c r="Q30" s="6" t="inlineStr">
         <is>
-          <t>3.00%</t>
+          <t>5.77%</t>
         </is>
       </c>
       <c r="R30" s="6" t="inlineStr">
@@ -9563,73 +9563,75 @@
     <row r="31" ht="30" customHeight="1">
       <c r="A31" s="6" t="inlineStr">
         <is>
-          <t>메쥬</t>
-        </is>
-      </c>
-      <c r="B31" s="18" t="inlineStr">
-        <is>
-          <t>수집예정</t>
+          <t>NH스팩33호</t>
+        </is>
+      </c>
+      <c r="B31" s="19" t="inlineStr">
+        <is>
+          <t>해당없음</t>
         </is>
       </c>
       <c r="C31" s="6" t="inlineStr">
         <is>
-          <t>16,700~21,600</t>
+          <t>2,000</t>
         </is>
       </c>
       <c r="D31" s="7" t="inlineStr">
         <is>
-          <t>1,345,000</t>
+          <t>6,350,000</t>
         </is>
       </c>
       <c r="E31" s="7" t="inlineStr">
         <is>
-          <t>29,052</t>
-        </is>
-      </c>
-      <c r="F31" s="6" t="inlineStr">
-        <is>
-          <t>20.66배 (PER)</t>
-        </is>
-      </c>
-      <c r="G31" s="6" t="n">
-        <v>21600</v>
+          <t>12,700</t>
+        </is>
+      </c>
+      <c r="F31" s="19" t="inlineStr">
+        <is>
+          <t>해당없음</t>
+        </is>
+      </c>
+      <c r="G31" s="6" t="inlineStr">
+        <is>
+          <t>2,000</t>
+        </is>
       </c>
       <c r="H31" s="6" t="n">
-        <v>1108.93</v>
+        <v>1228.71</v>
       </c>
       <c r="I31" s="6" t="n">
-        <v>2320</v>
+        <v>2058</v>
       </c>
       <c r="J31" s="6" t="inlineStr">
         <is>
-          <t>2026-03-16~03-17</t>
+          <t>2026-03-17~03-18</t>
         </is>
       </c>
       <c r="K31" s="6" t="inlineStr">
         <is>
-          <t>2,428.25</t>
+          <t>569.27</t>
         </is>
       </c>
       <c r="L31" s="6" t="inlineStr"/>
       <c r="M31" s="6" t="inlineStr">
         <is>
-          <t>2026-03-26</t>
+          <t>2026-03-27</t>
         </is>
       </c>
       <c r="N31" s="6" t="inlineStr">
         <is>
-          <t>신한</t>
+          <t>NH</t>
         </is>
       </c>
       <c r="O31" s="6" t="inlineStr"/>
       <c r="P31" s="7" t="inlineStr">
         <is>
-          <t>1,496</t>
+          <t>381</t>
         </is>
       </c>
       <c r="Q31" s="6" t="inlineStr">
         <is>
-          <t>5.00%</t>
+          <t>3.00%</t>
         </is>
       </c>
       <c r="R31" s="6" t="inlineStr">
@@ -9641,7 +9643,7 @@
     <row r="32" ht="30" customHeight="1">
       <c r="A32" s="6" t="inlineStr">
         <is>
-          <t>한패스</t>
+          <t>메쥬</t>
         </is>
       </c>
       <c r="B32" s="18" t="inlineStr">
@@ -9651,32 +9653,32 @@
       </c>
       <c r="C32" s="6" t="inlineStr">
         <is>
-          <t>17,000~19,000</t>
+          <t>16,700~21,600</t>
         </is>
       </c>
       <c r="D32" s="7" t="inlineStr">
         <is>
-          <t>1,100,000</t>
+          <t>1,345,000</t>
         </is>
       </c>
       <c r="E32" s="7" t="inlineStr">
         <is>
-          <t>20,900</t>
+          <t>29,052</t>
         </is>
       </c>
       <c r="F32" s="6" t="inlineStr">
         <is>
-          <t>29.09배 (PER)</t>
+          <t>20.66배 (PER)</t>
         </is>
       </c>
       <c r="G32" s="6" t="n">
-        <v>19000</v>
+        <v>21600</v>
       </c>
       <c r="H32" s="6" t="n">
-        <v>1172.59</v>
+        <v>1108.93</v>
       </c>
       <c r="I32" s="6" t="n">
-        <v>2229</v>
+        <v>2320</v>
       </c>
       <c r="J32" s="6" t="inlineStr">
         <is>
@@ -9685,29 +9687,29 @@
       </c>
       <c r="K32" s="6" t="inlineStr">
         <is>
-          <t>1,673.04</t>
+          <t>2,428.25</t>
         </is>
       </c>
       <c r="L32" s="6" t="inlineStr"/>
       <c r="M32" s="6" t="inlineStr">
         <is>
-          <t>2026-03-25</t>
+          <t>2026-03-26</t>
         </is>
       </c>
       <c r="N32" s="6" t="inlineStr">
         <is>
-          <t>한국</t>
+          <t>신한</t>
         </is>
       </c>
       <c r="O32" s="6" t="inlineStr"/>
       <c r="P32" s="7" t="inlineStr">
         <is>
-          <t>753</t>
+          <t>1,496</t>
         </is>
       </c>
       <c r="Q32" s="6" t="inlineStr">
         <is>
-          <t>3.50%</t>
+          <t>5.00%</t>
         </is>
       </c>
       <c r="R32" s="6" t="inlineStr">
@@ -9719,7 +9721,7 @@
     <row r="33" ht="30" customHeight="1">
       <c r="A33" s="6" t="inlineStr">
         <is>
-          <t>아이엠바이오로직스</t>
+          <t>한패스</t>
         </is>
       </c>
       <c r="B33" s="18" t="inlineStr">
@@ -9729,47 +9731,47 @@
       </c>
       <c r="C33" s="6" t="inlineStr">
         <is>
-          <t>19,000~26,000</t>
+          <t>17,000~19,000</t>
         </is>
       </c>
       <c r="D33" s="7" t="inlineStr">
         <is>
-          <t>2,000,000</t>
+          <t>1,100,000</t>
         </is>
       </c>
       <c r="E33" s="7" t="inlineStr">
         <is>
-          <t>52,000</t>
+          <t>20,900</t>
         </is>
       </c>
       <c r="F33" s="6" t="inlineStr">
         <is>
-          <t>21.46배 (PER)</t>
+          <t>29.09배 (PER)</t>
         </is>
       </c>
       <c r="G33" s="6" t="n">
-        <v>26000</v>
+        <v>19000</v>
       </c>
       <c r="H33" s="6" t="n">
-        <v>839.23</v>
+        <v>1172.59</v>
       </c>
       <c r="I33" s="6" t="n">
-        <v>2333</v>
+        <v>2229</v>
       </c>
       <c r="J33" s="6" t="inlineStr">
         <is>
-          <t>2026-03-11~03-12</t>
+          <t>2026-03-16~03-17</t>
         </is>
       </c>
       <c r="K33" s="6" t="inlineStr">
         <is>
-          <t>1,806.00</t>
+          <t>1,673.04</t>
         </is>
       </c>
       <c r="L33" s="6" t="inlineStr"/>
       <c r="M33" s="6" t="inlineStr">
         <is>
-          <t>2026-03-20</t>
+          <t>2026-03-25</t>
         </is>
       </c>
       <c r="N33" s="6" t="inlineStr">
@@ -9780,12 +9782,12 @@
       <c r="O33" s="6" t="inlineStr"/>
       <c r="P33" s="7" t="inlineStr">
         <is>
-          <t>2,650</t>
+          <t>753</t>
         </is>
       </c>
       <c r="Q33" s="6" t="inlineStr">
         <is>
-          <t>5.00%</t>
+          <t>3.50%</t>
         </is>
       </c>
       <c r="R33" s="6" t="inlineStr">
@@ -9797,7 +9799,7 @@
     <row r="34" ht="30" customHeight="1">
       <c r="A34" s="6" t="inlineStr">
         <is>
-          <t>카나프테라퓨틱스</t>
+          <t>아이엠바이오로직스</t>
         </is>
       </c>
       <c r="B34" s="18" t="inlineStr">
@@ -9807,7 +9809,7 @@
       </c>
       <c r="C34" s="6" t="inlineStr">
         <is>
-          <t>16,000~20,000</t>
+          <t>19,000~26,000</t>
         </is>
       </c>
       <c r="D34" s="7" t="inlineStr">
@@ -9817,37 +9819,37 @@
       </c>
       <c r="E34" s="7" t="inlineStr">
         <is>
-          <t>40,000</t>
+          <t>52,000</t>
         </is>
       </c>
       <c r="F34" s="6" t="inlineStr">
         <is>
-          <t>23.59배 (PER)</t>
+          <t>21.46배 (PER)</t>
         </is>
       </c>
       <c r="G34" s="6" t="n">
-        <v>20000</v>
+        <v>26000</v>
       </c>
       <c r="H34" s="6" t="n">
-        <v>962.1</v>
+        <v>839.23</v>
       </c>
       <c r="I34" s="6" t="n">
-        <v>2327</v>
+        <v>2333</v>
       </c>
       <c r="J34" s="6" t="inlineStr">
         <is>
-          <t>2026-03-05~03-06</t>
+          <t>2026-03-11~03-12</t>
         </is>
       </c>
       <c r="K34" s="6" t="inlineStr">
         <is>
-          <t>1,899.29</t>
+          <t>1,806.00</t>
         </is>
       </c>
       <c r="L34" s="6" t="inlineStr"/>
       <c r="M34" s="6" t="inlineStr">
         <is>
-          <t>2026-03-16</t>
+          <t>2026-03-20</t>
         </is>
       </c>
       <c r="N34" s="6" t="inlineStr">
@@ -9858,7 +9860,7 @@
       <c r="O34" s="6" t="inlineStr"/>
       <c r="P34" s="7" t="inlineStr">
         <is>
-          <t>2,050</t>
+          <t>2,650</t>
         </is>
       </c>
       <c r="Q34" s="6" t="inlineStr">
@@ -9875,7 +9877,7 @@
     <row r="35" ht="30" customHeight="1">
       <c r="A35" s="6" t="inlineStr">
         <is>
-          <t>액스비스</t>
+          <t>카나프테라퓨틱스</t>
         </is>
       </c>
       <c r="B35" s="18" t="inlineStr">
@@ -9885,63 +9887,63 @@
       </c>
       <c r="C35" s="6" t="inlineStr">
         <is>
-          <t>10,100~11,500</t>
+          <t>16,000~20,000</t>
         </is>
       </c>
       <c r="D35" s="7" t="inlineStr">
         <is>
-          <t>2,300,000</t>
+          <t>2,000,000</t>
         </is>
       </c>
       <c r="E35" s="7" t="inlineStr">
         <is>
-          <t>26,450</t>
+          <t>40,000</t>
         </is>
       </c>
       <c r="F35" s="6" t="inlineStr">
         <is>
-          <t>27.60배 (PER)</t>
+          <t>23.59배 (PER)</t>
         </is>
       </c>
       <c r="G35" s="6" t="n">
-        <v>11500</v>
+        <v>20000</v>
       </c>
       <c r="H35" s="6" t="n">
-        <v>1124.21</v>
+        <v>962.1</v>
       </c>
       <c r="I35" s="6" t="n">
-        <v>2411</v>
+        <v>2327</v>
       </c>
       <c r="J35" s="6" t="inlineStr">
         <is>
-          <t>2026-02-23~02-24</t>
+          <t>2026-03-05~03-06</t>
         </is>
       </c>
       <c r="K35" s="6" t="inlineStr">
         <is>
-          <t>1,960.87</t>
+          <t>1,899.29</t>
         </is>
       </c>
       <c r="L35" s="6" t="inlineStr"/>
       <c r="M35" s="6" t="inlineStr">
         <is>
-          <t>2026-03-09</t>
+          <t>2026-03-16</t>
         </is>
       </c>
       <c r="N35" s="6" t="inlineStr">
         <is>
-          <t>미래</t>
+          <t>한국</t>
         </is>
       </c>
       <c r="O35" s="6" t="inlineStr"/>
       <c r="P35" s="7" t="inlineStr">
         <is>
-          <t>1,090</t>
+          <t>2,050</t>
         </is>
       </c>
       <c r="Q35" s="6" t="inlineStr">
         <is>
-          <t>4.00%</t>
+          <t>5.00%</t>
         </is>
       </c>
       <c r="R35" s="6" t="inlineStr">
@@ -9953,7 +9955,7 @@
     <row r="36" ht="30" customHeight="1">
       <c r="A36" s="6" t="inlineStr">
         <is>
-          <t>에스팀</t>
+          <t>액스비스</t>
         </is>
       </c>
       <c r="B36" s="18" t="inlineStr">
@@ -9963,32 +9965,32 @@
       </c>
       <c r="C36" s="6" t="inlineStr">
         <is>
-          <t>7,000~8,500</t>
+          <t>10,100~11,500</t>
         </is>
       </c>
       <c r="D36" s="7" t="inlineStr">
         <is>
-          <t>1,800,000</t>
+          <t>2,300,000</t>
         </is>
       </c>
       <c r="E36" s="7" t="inlineStr">
         <is>
-          <t>15,300</t>
+          <t>26,450</t>
         </is>
       </c>
       <c r="F36" s="6" t="inlineStr">
         <is>
-          <t>17.71배 (EV/EBITDA)</t>
+          <t>27.60배 (PER)</t>
         </is>
       </c>
       <c r="G36" s="6" t="n">
-        <v>8500</v>
+        <v>11500</v>
       </c>
       <c r="H36" s="6" t="n">
-        <v>1334.91</v>
+        <v>1124.21</v>
       </c>
       <c r="I36" s="6" t="n">
-        <v>2263</v>
+        <v>2411</v>
       </c>
       <c r="J36" s="6" t="inlineStr">
         <is>
@@ -9997,29 +9999,29 @@
       </c>
       <c r="K36" s="6" t="inlineStr">
         <is>
-          <t>1,334.91</t>
+          <t>1,960.87</t>
         </is>
       </c>
       <c r="L36" s="6" t="inlineStr"/>
       <c r="M36" s="6" t="inlineStr">
         <is>
-          <t>2026-03-06</t>
+          <t>2026-03-09</t>
         </is>
       </c>
       <c r="N36" s="6" t="inlineStr">
         <is>
-          <t>한국</t>
+          <t>미래</t>
         </is>
       </c>
       <c r="O36" s="6" t="inlineStr"/>
       <c r="P36" s="7" t="inlineStr">
         <is>
-          <t>788</t>
+          <t>1,090</t>
         </is>
       </c>
       <c r="Q36" s="6" t="inlineStr">
         <is>
-          <t>5.00%</t>
+          <t>4.00%</t>
         </is>
       </c>
       <c r="R36" s="6" t="inlineStr">
@@ -10031,7 +10033,7 @@
     <row r="37" ht="30" customHeight="1">
       <c r="A37" s="6" t="inlineStr">
         <is>
-          <t>케이뱅크 (유가)</t>
+          <t>에스팀</t>
         </is>
       </c>
       <c r="B37" s="18" t="inlineStr">
@@ -10041,67 +10043,63 @@
       </c>
       <c r="C37" s="6" t="inlineStr">
         <is>
-          <t>8,300~9,500</t>
+          <t>7,000~8,500</t>
         </is>
       </c>
       <c r="D37" s="7" t="inlineStr">
         <is>
-          <t>60,000,000</t>
+          <t>1,800,000</t>
         </is>
       </c>
       <c r="E37" s="7" t="inlineStr">
         <is>
-          <t>498,000</t>
+          <t>15,300</t>
         </is>
       </c>
       <c r="F37" s="6" t="inlineStr">
         <is>
-          <t>1.80배 (PBR)</t>
+          <t>17.71배 (EV/EBITDA)</t>
         </is>
       </c>
       <c r="G37" s="6" t="n">
-        <v>8300</v>
+        <v>8500</v>
       </c>
       <c r="H37" s="6" t="n">
-        <v>198.53</v>
+        <v>1334.91</v>
       </c>
       <c r="I37" s="6" t="n">
-        <v>2007</v>
+        <v>2263</v>
       </c>
       <c r="J37" s="6" t="inlineStr">
         <is>
-          <t>2026-02-20~23</t>
+          <t>2026-02-23~02-24</t>
         </is>
       </c>
       <c r="K37" s="6" t="inlineStr">
         <is>
-          <t>134.59</t>
+          <t>1,334.91</t>
         </is>
       </c>
       <c r="L37" s="6" t="inlineStr"/>
       <c r="M37" s="6" t="inlineStr">
         <is>
-          <t>2026-03-05</t>
+          <t>2026-03-06</t>
         </is>
       </c>
       <c r="N37" s="6" t="inlineStr">
         <is>
-          <t>NH</t>
-        </is>
-      </c>
-      <c r="O37" s="6" t="inlineStr">
-        <is>
-          <t>삼성</t>
-        </is>
-      </c>
+          <t>한국</t>
+        </is>
+      </c>
+      <c r="O37" s="6" t="inlineStr"/>
       <c r="P37" s="7" t="inlineStr">
         <is>
-          <t>5,976</t>
+          <t>788</t>
         </is>
       </c>
       <c r="Q37" s="6" t="inlineStr">
         <is>
-          <t>1.2%</t>
+          <t>5.00%</t>
         </is>
       </c>
       <c r="R37" s="6" t="inlineStr">
@@ -10113,63 +10111,57 @@
     <row r="38" ht="30" customHeight="1">
       <c r="A38" s="6" t="inlineStr">
         <is>
-          <t>세미티에스</t>
-        </is>
-      </c>
-      <c r="B38" s="19" t="inlineStr">
-        <is>
-          <t>해당없음</t>
-        </is>
-      </c>
-      <c r="C38" s="19" t="inlineStr">
-        <is>
-          <t>해당없음</t>
-        </is>
-      </c>
-      <c r="D38" s="19" t="inlineStr">
-        <is>
-          <t>해당없음</t>
-        </is>
-      </c>
-      <c r="E38" s="19" t="inlineStr">
-        <is>
-          <t>해당없음</t>
-        </is>
-      </c>
-      <c r="F38" s="19" t="inlineStr">
-        <is>
-          <t>해당없음</t>
-        </is>
-      </c>
-      <c r="G38" s="19" t="inlineStr">
-        <is>
-          <t>해당없음</t>
-        </is>
-      </c>
-      <c r="H38" s="19" t="inlineStr">
-        <is>
-          <t>해당없음</t>
-        </is>
-      </c>
-      <c r="I38" s="19" t="inlineStr">
-        <is>
-          <t>해당없음</t>
-        </is>
-      </c>
-      <c r="J38" s="19" t="inlineStr">
-        <is>
-          <t>해당없음</t>
-        </is>
-      </c>
-      <c r="K38" s="19" t="inlineStr">
-        <is>
-          <t>해당없음</t>
+          <t>케이뱅크 (유가)</t>
+        </is>
+      </c>
+      <c r="B38" s="18" t="inlineStr">
+        <is>
+          <t>수집예정</t>
+        </is>
+      </c>
+      <c r="C38" s="6" t="inlineStr">
+        <is>
+          <t>8,300~9,500</t>
+        </is>
+      </c>
+      <c r="D38" s="7" t="inlineStr">
+        <is>
+          <t>60,000,000</t>
+        </is>
+      </c>
+      <c r="E38" s="7" t="inlineStr">
+        <is>
+          <t>498,000</t>
+        </is>
+      </c>
+      <c r="F38" s="6" t="inlineStr">
+        <is>
+          <t>1.80배 (PBR)</t>
+        </is>
+      </c>
+      <c r="G38" s="6" t="n">
+        <v>8300</v>
+      </c>
+      <c r="H38" s="6" t="n">
+        <v>198.53</v>
+      </c>
+      <c r="I38" s="6" t="n">
+        <v>2007</v>
+      </c>
+      <c r="J38" s="6" t="inlineStr">
+        <is>
+          <t>2026-02-20~23</t>
+        </is>
+      </c>
+      <c r="K38" s="6" t="inlineStr">
+        <is>
+          <t>134.59</t>
         </is>
       </c>
       <c r="L38" s="6" t="inlineStr"/>
       <c r="M38" s="6" t="inlineStr">
         <is>
-          <t>2026-02-05</t>
+          <t>2026-03-05</t>
         </is>
       </c>
       <c r="N38" s="6" t="inlineStr">
@@ -10177,77 +10169,87 @@
           <t>NH</t>
         </is>
       </c>
-      <c r="O38" s="6" t="inlineStr"/>
-      <c r="P38" s="19" t="inlineStr">
-        <is>
-          <t>해당없음</t>
-        </is>
-      </c>
-      <c r="Q38" s="19" t="inlineStr">
-        <is>
-          <t>해당없음</t>
+      <c r="O38" s="6" t="inlineStr">
+        <is>
+          <t>삼성</t>
+        </is>
+      </c>
+      <c r="P38" s="7" t="inlineStr">
+        <is>
+          <t>5,976</t>
+        </is>
+      </c>
+      <c r="Q38" s="6" t="inlineStr">
+        <is>
+          <t>1.2%</t>
         </is>
       </c>
       <c r="R38" s="6" t="inlineStr">
         <is>
-          <t>상장완료(스팩합병)</t>
+          <t>상장완료</t>
         </is>
       </c>
     </row>
     <row r="39" ht="30" customHeight="1">
       <c r="A39" s="6" t="inlineStr">
         <is>
-          <t>덕양에너젠</t>
-        </is>
-      </c>
-      <c r="B39" s="18" t="inlineStr">
-        <is>
-          <t>수집예정</t>
-        </is>
-      </c>
-      <c r="C39" s="6" t="inlineStr">
-        <is>
-          <t>8,500~10,000</t>
-        </is>
-      </c>
-      <c r="D39" s="7" t="inlineStr">
-        <is>
-          <t>7,500,000</t>
-        </is>
-      </c>
-      <c r="E39" s="7" t="inlineStr">
-        <is>
-          <t>75,000</t>
-        </is>
-      </c>
-      <c r="F39" s="6" t="inlineStr">
-        <is>
-          <t>30.32배 (EV/EBITDA)</t>
-        </is>
-      </c>
-      <c r="G39" s="6" t="n">
-        <v>10000</v>
-      </c>
-      <c r="H39" s="6" t="n">
-        <v>650.14</v>
-      </c>
-      <c r="I39" s="6" t="n">
-        <v>2324</v>
-      </c>
-      <c r="J39" s="6" t="inlineStr">
-        <is>
-          <t>2026-01-20~01-21</t>
-        </is>
-      </c>
-      <c r="K39" s="6" t="inlineStr">
-        <is>
-          <t>1,354.00</t>
+          <t>세미티에스</t>
+        </is>
+      </c>
+      <c r="B39" s="19" t="inlineStr">
+        <is>
+          <t>해당없음</t>
+        </is>
+      </c>
+      <c r="C39" s="19" t="inlineStr">
+        <is>
+          <t>해당없음</t>
+        </is>
+      </c>
+      <c r="D39" s="19" t="inlineStr">
+        <is>
+          <t>해당없음</t>
+        </is>
+      </c>
+      <c r="E39" s="19" t="inlineStr">
+        <is>
+          <t>해당없음</t>
+        </is>
+      </c>
+      <c r="F39" s="19" t="inlineStr">
+        <is>
+          <t>해당없음</t>
+        </is>
+      </c>
+      <c r="G39" s="19" t="inlineStr">
+        <is>
+          <t>해당없음</t>
+        </is>
+      </c>
+      <c r="H39" s="19" t="inlineStr">
+        <is>
+          <t>해당없음</t>
+        </is>
+      </c>
+      <c r="I39" s="19" t="inlineStr">
+        <is>
+          <t>해당없음</t>
+        </is>
+      </c>
+      <c r="J39" s="19" t="inlineStr">
+        <is>
+          <t>해당없음</t>
+        </is>
+      </c>
+      <c r="K39" s="19" t="inlineStr">
+        <is>
+          <t>해당없음</t>
         </is>
       </c>
       <c r="L39" s="6" t="inlineStr"/>
       <c r="M39" s="6" t="inlineStr">
         <is>
-          <t>2026-01-30</t>
+          <t>2026-02-05</t>
         </is>
       </c>
       <c r="N39" s="6" t="inlineStr">
@@ -10255,87 +10257,77 @@
           <t>NH</t>
         </is>
       </c>
-      <c r="O39" s="6" t="inlineStr">
-        <is>
-          <t>미래</t>
-        </is>
-      </c>
-      <c r="P39" s="7" t="inlineStr">
-        <is>
-          <t>2,000</t>
-        </is>
-      </c>
-      <c r="Q39" s="6" t="inlineStr">
-        <is>
-          <t>2.92%</t>
+      <c r="O39" s="6" t="inlineStr"/>
+      <c r="P39" s="19" t="inlineStr">
+        <is>
+          <t>해당없음</t>
+        </is>
+      </c>
+      <c r="Q39" s="19" t="inlineStr">
+        <is>
+          <t>해당없음</t>
         </is>
       </c>
       <c r="R39" s="6" t="inlineStr">
         <is>
-          <t>상장완료</t>
+          <t>상장완료(스팩합병)</t>
         </is>
       </c>
     </row>
     <row r="40" ht="30" customHeight="1">
       <c r="A40" s="6" t="inlineStr">
         <is>
-          <t>케이피항공산업</t>
-        </is>
-      </c>
-      <c r="B40" s="19" t="inlineStr">
-        <is>
-          <t>해당없음</t>
-        </is>
-      </c>
-      <c r="C40" s="19" t="inlineStr">
-        <is>
-          <t>해당없음</t>
-        </is>
-      </c>
-      <c r="D40" s="19" t="inlineStr">
-        <is>
-          <t>해당없음</t>
-        </is>
-      </c>
-      <c r="E40" s="19" t="inlineStr">
-        <is>
-          <t>해당없음</t>
-        </is>
-      </c>
-      <c r="F40" s="19" t="inlineStr">
-        <is>
-          <t>해당없음</t>
-        </is>
-      </c>
-      <c r="G40" s="19" t="inlineStr">
-        <is>
-          <t>해당없음</t>
-        </is>
-      </c>
-      <c r="H40" s="19" t="inlineStr">
-        <is>
-          <t>해당없음</t>
-        </is>
-      </c>
-      <c r="I40" s="19" t="inlineStr">
-        <is>
-          <t>해당없음</t>
-        </is>
-      </c>
-      <c r="J40" s="19" t="inlineStr">
-        <is>
-          <t>해당없음</t>
-        </is>
-      </c>
-      <c r="K40" s="19" t="inlineStr">
-        <is>
-          <t>해당없음</t>
+          <t>덕양에너젠</t>
+        </is>
+      </c>
+      <c r="B40" s="18" t="inlineStr">
+        <is>
+          <t>수집예정</t>
+        </is>
+      </c>
+      <c r="C40" s="6" t="inlineStr">
+        <is>
+          <t>8,500~10,000</t>
+        </is>
+      </c>
+      <c r="D40" s="7" t="inlineStr">
+        <is>
+          <t>7,500,000</t>
+        </is>
+      </c>
+      <c r="E40" s="7" t="inlineStr">
+        <is>
+          <t>75,000</t>
+        </is>
+      </c>
+      <c r="F40" s="6" t="inlineStr">
+        <is>
+          <t>30.32배 (EV/EBITDA)</t>
+        </is>
+      </c>
+      <c r="G40" s="6" t="n">
+        <v>10000</v>
+      </c>
+      <c r="H40" s="6" t="n">
+        <v>650.14</v>
+      </c>
+      <c r="I40" s="6" t="n">
+        <v>2324</v>
+      </c>
+      <c r="J40" s="6" t="inlineStr">
+        <is>
+          <t>2026-01-20~01-21</t>
+        </is>
+      </c>
+      <c r="K40" s="6" t="inlineStr">
+        <is>
+          <t>1,354.00</t>
         </is>
       </c>
       <c r="L40" s="6" t="inlineStr"/>
       <c r="M40" s="6" t="inlineStr">
         <is>
-          <t>2026-01-29</t>
+          <t>2026-01-30</t>
         </is>
       </c>
       <c r="N40" s="6" t="inlineStr">
@@ -10343,27 +10335,31 @@
           <t>NH</t>
         </is>
       </c>
-      <c r="O40" s="6" t="inlineStr"/>
-      <c r="P40" s="19" t="inlineStr">
-        <is>
-          <t>해당없음</t>
-        </is>
-      </c>
-      <c r="Q40" s="19" t="inlineStr">
-        <is>
-          <t>해당없음</t>
+      <c r="O40" s="6" t="inlineStr">
+        <is>
+          <t>미래</t>
+        </is>
+      </c>
+      <c r="P40" s="7" t="inlineStr">
+        <is>
+          <t>2,000</t>
+        </is>
+      </c>
+      <c r="Q40" s="6" t="inlineStr">
+        <is>
+          <t>2.92%</t>
         </is>
       </c>
       <c r="R40" s="6" t="inlineStr">
         <is>
-          <t>상장완료(스팩합병)</t>
+          <t>상장완료</t>
         </is>
       </c>
     </row>
     <row r="41" ht="30" customHeight="1">
       <c r="A41" s="6" t="inlineStr">
         <is>
-          <t>삼성스팩13호</t>
+          <t>케이피항공산업</t>
         </is>
       </c>
       <c r="B41" s="19" t="inlineStr">
@@ -10371,19 +10367,19 @@
           <t>해당없음</t>
         </is>
       </c>
-      <c r="C41" s="6" t="inlineStr">
-        <is>
-          <t>2,000</t>
-        </is>
-      </c>
-      <c r="D41" s="7" t="inlineStr">
-        <is>
-          <t>6,000,000</t>
-        </is>
-      </c>
-      <c r="E41" s="7" t="inlineStr">
-        <is>
-          <t>12,000</t>
+      <c r="C41" s="19" t="inlineStr">
+        <is>
+          <t>해당없음</t>
+        </is>
+      </c>
+      <c r="D41" s="19" t="inlineStr">
+        <is>
+          <t>해당없음</t>
+        </is>
+      </c>
+      <c r="E41" s="19" t="inlineStr">
+        <is>
+          <t>해당없음</t>
         </is>
       </c>
       <c r="F41" s="19" t="inlineStr">
@@ -10391,150 +10387,162 @@
           <t>해당없음</t>
         </is>
       </c>
-      <c r="G41" s="6" t="inlineStr">
-        <is>
-          <t>2,000</t>
-        </is>
-      </c>
-      <c r="H41" s="6" t="n">
-        <v>1159.11</v>
-      </c>
-      <c r="I41" s="6" t="n">
-        <v>1892</v>
-      </c>
-      <c r="J41" s="6" t="inlineStr">
-        <is>
-          <t>2026-01-12~01-13</t>
-        </is>
-      </c>
-      <c r="K41" s="6" t="inlineStr">
-        <is>
-          <t>1,870.40</t>
+      <c r="G41" s="19" t="inlineStr">
+        <is>
+          <t>해당없음</t>
+        </is>
+      </c>
+      <c r="H41" s="19" t="inlineStr">
+        <is>
+          <t>해당없음</t>
+        </is>
+      </c>
+      <c r="I41" s="19" t="inlineStr">
+        <is>
+          <t>해당없음</t>
+        </is>
+      </c>
+      <c r="J41" s="19" t="inlineStr">
+        <is>
+          <t>해당없음</t>
+        </is>
+      </c>
+      <c r="K41" s="19" t="inlineStr">
+        <is>
+          <t>해당없음</t>
         </is>
       </c>
       <c r="L41" s="6" t="inlineStr"/>
       <c r="M41" s="6" t="inlineStr">
         <is>
+          <t>2026-01-29</t>
+        </is>
+      </c>
+      <c r="N41" s="6" t="inlineStr">
+        <is>
+          <t>NH</t>
+        </is>
+      </c>
+      <c r="O41" s="6" t="inlineStr"/>
+      <c r="P41" s="19" t="inlineStr">
+        <is>
+          <t>해당없음</t>
+        </is>
+      </c>
+      <c r="Q41" s="19" t="inlineStr">
+        <is>
+          <t>해당없음</t>
+        </is>
+      </c>
+      <c r="R41" s="6" t="inlineStr">
+        <is>
+          <t>상장완료(스팩합병)</t>
+        </is>
+      </c>
+    </row>
+    <row r="42" ht="30" customHeight="1">
+      <c r="A42" s="6" t="inlineStr">
+        <is>
+          <t>삼성스팩13호</t>
+        </is>
+      </c>
+      <c r="B42" s="19" t="inlineStr">
+        <is>
+          <t>해당없음</t>
+        </is>
+      </c>
+      <c r="C42" s="6" t="inlineStr">
+        <is>
+          <t>2,000</t>
+        </is>
+      </c>
+      <c r="D42" s="7" t="inlineStr">
+        <is>
+          <t>6,000,000</t>
+        </is>
+      </c>
+      <c r="E42" s="7" t="inlineStr">
+        <is>
+          <t>12,000</t>
+        </is>
+      </c>
+      <c r="F42" s="19" t="inlineStr">
+        <is>
+          <t>해당없음</t>
+        </is>
+      </c>
+      <c r="G42" s="6" t="inlineStr">
+        <is>
+          <t>2,000</t>
+        </is>
+      </c>
+      <c r="H42" s="6" t="n">
+        <v>1159.11</v>
+      </c>
+      <c r="I42" s="6" t="n">
+        <v>1892</v>
+      </c>
+      <c r="J42" s="6" t="inlineStr">
+        <is>
+          <t>2026-01-12~01-13</t>
+        </is>
+      </c>
+      <c r="K42" s="6" t="inlineStr">
+        <is>
+          <t>1,870.40</t>
+        </is>
+      </c>
+      <c r="L42" s="6" t="inlineStr"/>
+      <c r="M42" s="6" t="inlineStr">
+        <is>
           <t>2026-01-21</t>
         </is>
       </c>
-      <c r="N41" s="6" t="inlineStr">
+      <c r="N42" s="6" t="inlineStr">
         <is>
           <t>삼성</t>
         </is>
       </c>
-      <c r="O41" s="6" t="inlineStr"/>
-      <c r="P41" s="7" t="inlineStr">
+      <c r="O42" s="6" t="inlineStr"/>
+      <c r="P42" s="7" t="inlineStr">
         <is>
           <t>360</t>
         </is>
       </c>
-      <c r="Q41" s="6" t="inlineStr">
+      <c r="Q42" s="6" t="inlineStr">
         <is>
           <t>3.00%</t>
         </is>
       </c>
-      <c r="R41" s="6" t="inlineStr">
+      <c r="R42" s="6" t="inlineStr">
         <is>
           <t>상장완료</t>
         </is>
       </c>
     </row>
-    <row r="43" ht="22" customHeight="1">
-      <c r="A43" s="3" t="inlineStr">
-        <is>
-          <t>■ 공모 진행 (예심 승인법인)  (25건)</t>
-        </is>
-      </c>
-      <c r="B43" s="4" t="n"/>
-      <c r="C43" s="4" t="n"/>
-      <c r="D43" s="4" t="n"/>
-      <c r="E43" s="4" t="n"/>
-      <c r="F43" s="4" t="n"/>
-      <c r="G43" s="4" t="n"/>
-      <c r="H43" s="4" t="n"/>
-      <c r="I43" s="4" t="n"/>
-      <c r="J43" s="4" t="n"/>
-      <c r="K43" s="4" t="n"/>
-      <c r="L43" s="4" t="n"/>
-      <c r="M43" s="4" t="n"/>
-      <c r="N43" s="4" t="n"/>
-      <c r="O43" s="4" t="n"/>
-      <c r="P43" s="4" t="n"/>
-      <c r="Q43" s="4" t="n"/>
-      <c r="R43" s="4" t="n"/>
-    </row>
-    <row r="44" ht="30" customHeight="1">
-      <c r="A44" s="6" t="inlineStr">
-        <is>
-          <t>기도산업</t>
-        </is>
-      </c>
-      <c r="B44" s="6" t="inlineStr">
-        <is>
-          <t>07-31~08-06</t>
-        </is>
-      </c>
-      <c r="C44" s="6" t="inlineStr">
-        <is>
-          <t>24,800~28,400</t>
-        </is>
-      </c>
-      <c r="D44" s="7" t="inlineStr">
-        <is>
-          <t>1,700,000</t>
-        </is>
-      </c>
-      <c r="E44" s="7" t="inlineStr">
-        <is>
-          <t>48,280,000,000</t>
-        </is>
-      </c>
-      <c r="F44" s="6" t="inlineStr">
-        <is>
-          <t>10.01배 (PER)</t>
-        </is>
-      </c>
-      <c r="G44" s="6" t="inlineStr">
-        <is>
-          <t>28,400</t>
-        </is>
-      </c>
-      <c r="H44" s="6" t="n">
-        <v>213.31</v>
-      </c>
-      <c r="I44" s="6" t="n">
-        <v>637</v>
-      </c>
-      <c r="J44" s="6" t="inlineStr">
-        <is>
-          <t>08-11~08-12</t>
-        </is>
-      </c>
-      <c r="K44" s="6" t="inlineStr"/>
-      <c r="L44" s="6" t="inlineStr"/>
-      <c r="M44" s="6" t="inlineStr"/>
-      <c r="N44" s="6" t="inlineStr">
-        <is>
-          <t>미래에셋증권</t>
-        </is>
-      </c>
-      <c r="O44" s="6" t="inlineStr"/>
-      <c r="P44" s="7" t="inlineStr">
-        <is>
-          <t>716,720,000</t>
-        </is>
-      </c>
-      <c r="Q44" s="6" t="inlineStr">
-        <is>
-          <t>1.0%</t>
-        </is>
-      </c>
-      <c r="R44" s="6" t="inlineStr">
-        <is>
-          <t>청약완료·상장대기</t>
-        </is>
-      </c>
+    <row r="44" ht="22" customHeight="1">
+      <c r="A44" s="3" t="inlineStr">
+        <is>
+          <t>■ 공모 진행 (예심 승인법인)  (24건)</t>
+        </is>
+      </c>
+      <c r="B44" s="4" t="n"/>
+      <c r="C44" s="4" t="n"/>
+      <c r="D44" s="4" t="n"/>
+      <c r="E44" s="4" t="n"/>
+      <c r="F44" s="4" t="n"/>
+      <c r="G44" s="4" t="n"/>
+      <c r="H44" s="4" t="n"/>
+      <c r="I44" s="4" t="n"/>
+      <c r="J44" s="4" t="n"/>
+      <c r="K44" s="4" t="n"/>
+      <c r="L44" s="4" t="n"/>
+      <c r="M44" s="4" t="n"/>
+      <c r="N44" s="4" t="n"/>
+      <c r="O44" s="4" t="n"/>
+      <c r="P44" s="4" t="n"/>
+      <c r="Q44" s="4" t="n"/>
+      <c r="R44" s="4" t="n"/>
     </row>
     <row r="45" ht="30" customHeight="1">
       <c r="A45" s="6" t="inlineStr">
@@ -11013,7 +11021,7 @@
       </c>
       <c r="C52" s="6" t="inlineStr">
         <is>
-          <t>20,000~24,000</t>
+          <t>15,000~18,000</t>
         </is>
       </c>
       <c r="D52" s="7" t="inlineStr">
@@ -11028,7 +11036,7 @@
       </c>
       <c r="F52" s="6" t="inlineStr">
         <is>
-          <t>15.41 (PSR)</t>
+          <t>11.15 (PSR)</t>
         </is>
       </c>
       <c r="G52" s="6" t="inlineStr"/>
@@ -11036,7 +11044,7 @@
       <c r="I52" s="6" t="inlineStr"/>
       <c r="J52" s="6" t="inlineStr">
         <is>
-          <t>09-16~09-17</t>
+          <t>09-15~09-16</t>
         </is>
       </c>
       <c r="K52" s="6" t="inlineStr"/>
@@ -11054,7 +11062,7 @@
       </c>
       <c r="P52" s="7" t="inlineStr">
         <is>
-          <t>627,300,000</t>
+          <t>378,216,000</t>
         </is>
       </c>
       <c r="Q52" s="6" t="inlineStr">
@@ -11327,17 +11335,17 @@
     <row r="57" ht="30" customHeight="1">
       <c r="A57" s="6" t="inlineStr">
         <is>
-          <t>엠에스바이오</t>
-        </is>
-      </c>
-      <c r="B57" s="18" t="inlineStr">
-        <is>
-          <t>수집예정</t>
-        </is>
-      </c>
-      <c r="C57" s="18" t="inlineStr">
-        <is>
-          <t>수집예정</t>
+          <t>엘리스그룹</t>
+        </is>
+      </c>
+      <c r="B57" s="6" t="inlineStr">
+        <is>
+          <t>09-09~09-15</t>
+        </is>
+      </c>
+      <c r="C57" s="6" t="inlineStr">
+        <is>
+          <t>70,400~90,500</t>
         </is>
       </c>
       <c r="D57" s="18" t="inlineStr">
@@ -11350,58 +11358,62 @@
           <t>수집예정</t>
         </is>
       </c>
-      <c r="F57" s="18" t="inlineStr">
-        <is>
-          <t>수집예정</t>
+      <c r="F57" s="6" t="inlineStr">
+        <is>
+          <t>27.13배 (EV/EBITDA)</t>
         </is>
       </c>
       <c r="G57" s="6" t="inlineStr"/>
       <c r="H57" s="6" t="inlineStr"/>
       <c r="I57" s="6" t="inlineStr"/>
-      <c r="J57" s="18" t="inlineStr">
-        <is>
-          <t>수집예정</t>
+      <c r="J57" s="6" t="inlineStr">
+        <is>
+          <t>09-18~09-21</t>
         </is>
       </c>
       <c r="K57" s="6" t="inlineStr"/>
       <c r="L57" s="6" t="inlineStr"/>
       <c r="M57" s="6" t="inlineStr"/>
-      <c r="N57" s="18" t="inlineStr">
-        <is>
-          <t>수집예정</t>
-        </is>
-      </c>
-      <c r="O57" s="6" t="inlineStr"/>
-      <c r="P57" s="18" t="inlineStr">
-        <is>
-          <t>수집예정</t>
-        </is>
-      </c>
-      <c r="Q57" s="18" t="inlineStr">
-        <is>
-          <t>수집예정</t>
+      <c r="N57" s="6" t="inlineStr">
+        <is>
+          <t>미래에셋증권㈜</t>
+        </is>
+      </c>
+      <c r="O57" s="6" t="inlineStr">
+        <is>
+          <t>삼성</t>
+        </is>
+      </c>
+      <c r="P57" s="7" t="inlineStr">
+        <is>
+          <t>1,889,144,928</t>
+        </is>
+      </c>
+      <c r="Q57" s="6" t="inlineStr">
+        <is>
+          <t>1.5%</t>
         </is>
       </c>
       <c r="R57" s="6" t="inlineStr">
         <is>
-          <t>신고서 대기</t>
+          <t>최초</t>
         </is>
       </c>
     </row>
     <row r="58" ht="30" customHeight="1">
       <c r="A58" s="6" t="inlineStr">
         <is>
-          <t>디티에스</t>
-        </is>
-      </c>
-      <c r="B58" s="18" t="inlineStr">
-        <is>
-          <t>수집예정</t>
-        </is>
-      </c>
-      <c r="C58" s="18" t="inlineStr">
-        <is>
-          <t>수집예정</t>
+          <t>멜콘</t>
+        </is>
+      </c>
+      <c r="B58" s="6" t="inlineStr">
+        <is>
+          <t>09-16~09-22</t>
+        </is>
+      </c>
+      <c r="C58" s="6" t="inlineStr">
+        <is>
+          <t>10,700~12,300</t>
         </is>
       </c>
       <c r="D58" s="18" t="inlineStr">
@@ -11414,48 +11426,48 @@
           <t>수집예정</t>
         </is>
       </c>
-      <c r="F58" s="18" t="inlineStr">
-        <is>
-          <t>수집예정</t>
+      <c r="F58" s="6" t="inlineStr">
+        <is>
+          <t>26.18배 (PER)</t>
         </is>
       </c>
       <c r="G58" s="6" t="inlineStr"/>
       <c r="H58" s="6" t="inlineStr"/>
       <c r="I58" s="6" t="inlineStr"/>
-      <c r="J58" s="18" t="inlineStr">
-        <is>
-          <t>수집예정</t>
+      <c r="J58" s="6" t="inlineStr">
+        <is>
+          <t>10-01~10-02</t>
         </is>
       </c>
       <c r="K58" s="6" t="inlineStr"/>
       <c r="L58" s="6" t="inlineStr"/>
       <c r="M58" s="6" t="inlineStr"/>
-      <c r="N58" s="18" t="inlineStr">
-        <is>
-          <t>수집예정</t>
+      <c r="N58" s="6" t="inlineStr">
+        <is>
+          <t>대신증권</t>
         </is>
       </c>
       <c r="O58" s="6" t="inlineStr"/>
-      <c r="P58" s="18" t="inlineStr">
-        <is>
-          <t>수집예정</t>
-        </is>
-      </c>
-      <c r="Q58" s="18" t="inlineStr">
-        <is>
-          <t>수집예정</t>
+      <c r="P58" s="7" t="inlineStr">
+        <is>
+          <t>826,575,000</t>
+        </is>
+      </c>
+      <c r="Q58" s="6" t="inlineStr">
+        <is>
+          <t>3.0%</t>
         </is>
       </c>
       <c r="R58" s="6" t="inlineStr">
         <is>
-          <t>신고서 대기</t>
+          <t>최초</t>
         </is>
       </c>
     </row>
     <row r="59" ht="30" customHeight="1">
       <c r="A59" s="6" t="inlineStr">
         <is>
-          <t>에스케이증권제14호기업인수목적</t>
+          <t>엠에스바이오</t>
         </is>
       </c>
       <c r="B59" s="18" t="inlineStr">
@@ -11519,7 +11531,7 @@
     <row r="60" ht="30" customHeight="1">
       <c r="A60" s="6" t="inlineStr">
         <is>
-          <t>한화플러스제6호스팩</t>
+          <t>디티에스</t>
         </is>
       </c>
       <c r="B60" s="18" t="inlineStr">
@@ -11583,7 +11595,7 @@
     <row r="61" ht="30" customHeight="1">
       <c r="A61" s="6" t="inlineStr">
         <is>
-          <t>래블업</t>
+          <t>에스케이증권제14호기업인수목적</t>
         </is>
       </c>
       <c r="B61" s="18" t="inlineStr">
@@ -11647,7 +11659,7 @@
     <row r="62" ht="30" customHeight="1">
       <c r="A62" s="6" t="inlineStr">
         <is>
-          <t>엠비디</t>
+          <t>한화플러스제6호스팩</t>
         </is>
       </c>
       <c r="B62" s="18" t="inlineStr">
@@ -11711,7 +11723,7 @@
     <row r="63" ht="30" customHeight="1">
       <c r="A63" s="6" t="inlineStr">
         <is>
-          <t>멜콘</t>
+          <t>래블업</t>
         </is>
       </c>
       <c r="B63" s="18" t="inlineStr">
@@ -11775,7 +11787,7 @@
     <row r="64" ht="30" customHeight="1">
       <c r="A64" s="6" t="inlineStr">
         <is>
-          <t>진코스텍</t>
+          <t>엠비디</t>
         </is>
       </c>
       <c r="B64" s="18" t="inlineStr">
@@ -11839,7 +11851,7 @@
     <row r="65" ht="30" customHeight="1">
       <c r="A65" s="6" t="inlineStr">
         <is>
-          <t>바로팜</t>
+          <t>진코스텍</t>
         </is>
       </c>
       <c r="B65" s="18" t="inlineStr">
@@ -11903,7 +11915,7 @@
     <row r="66" ht="30" customHeight="1">
       <c r="A66" s="6" t="inlineStr">
         <is>
-          <t>크리에이츠</t>
+          <t>바로팜</t>
         </is>
       </c>
       <c r="B66" s="18" t="inlineStr">
@@ -11967,7 +11979,7 @@
     <row r="67" ht="30" customHeight="1">
       <c r="A67" s="6" t="inlineStr">
         <is>
-          <t>티앤이코리아</t>
+          <t>크리에이츠</t>
         </is>
       </c>
       <c r="B67" s="18" t="inlineStr">
@@ -12031,7 +12043,7 @@
     <row r="68" ht="30" customHeight="1">
       <c r="A68" s="6" t="inlineStr">
         <is>
-          <t>엘리스그룹</t>
+          <t>티앤이코리아</t>
         </is>
       </c>
       <c r="B68" s="18" t="inlineStr">
@@ -12124,7 +12136,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F35"/>
+  <dimension ref="A1:F36"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -12361,7 +12373,7 @@
         </is>
       </c>
       <c r="B13" s="6" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="C13" s="6" t="n">
         <v>5</v>
@@ -12370,7 +12382,7 @@
         <v>0</v>
       </c>
       <c r="E13" s="6" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="F13" s="21">
         <f>IF((C13+D13)=0,"-",C13/(C13+D13))</f>
@@ -12478,45 +12490,45 @@
     <row r="21">
       <c r="A21" s="6" t="inlineStr">
         <is>
-          <t>대신증권</t>
+          <t>미래에셋증권</t>
         </is>
       </c>
       <c r="B21" s="6" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="C21" s="6" t="inlineStr">
         <is>
-          <t>80,800,000,000</t>
+          <t>96,560,000,000</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="6" t="inlineStr">
         <is>
-          <t>아이비케이투자증권</t>
+          <t>대신증권</t>
         </is>
       </c>
       <c r="B22" s="6" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="C22" s="6" t="inlineStr">
         <is>
-          <t>72,600,000,000</t>
+          <t>80,800,000,000</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="6" t="inlineStr">
         <is>
-          <t>미래에셋증권</t>
+          <t>아이비케이투자증권</t>
         </is>
       </c>
       <c r="B23" s="6" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="C23" s="6" t="inlineStr">
         <is>
-          <t>48,280,000,000</t>
+          <t>72,600,000,000</t>
         </is>
       </c>
     </row>
@@ -12699,6 +12711,17 @@
           <t>10,800</t>
         </is>
       </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="6" t="inlineStr">
+        <is>
+          <t>미래에셋증권㈜</t>
+        </is>
+      </c>
+      <c r="B36" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="C36" s="6" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
chore: update IPO data 2026-08-24
</commit_message>
<xml_diff>
--- a/IPO_analysis.xlsx
+++ b/IPO_analysis.xlsx
@@ -618,7 +618,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>기준일 2026-08-23 · 청구일 직전 사업연도 · 별도/개별 재무제표 · 단위 백만원(별도 표기 시 USD)</t>
+          <t>기준일 2026-08-24 · 청구일 직전 사업연도 · 별도/개별 재무제표 · 단위 백만원(별도 표기 시 USD)</t>
         </is>
       </c>
     </row>
@@ -4765,7 +4765,7 @@
       </c>
       <c r="K79" s="6" t="inlineStr">
         <is>
-          <t>상장승인(상장예정)</t>
+          <t>상장완료 (2026-08-24)</t>
         </is>
       </c>
     </row>
@@ -7621,7 +7621,7 @@
     <row r="6" ht="22" customHeight="1">
       <c r="A6" s="3" t="inlineStr">
         <is>
-          <t>■ 상장 완료 (2026)  (36건)</t>
+          <t>■ 상장 완료 (2026)  (37건)</t>
         </is>
       </c>
       <c r="B6" s="4" t="n"/>
@@ -7645,44 +7645,44 @@
     <row r="7" ht="30" customHeight="1">
       <c r="A7" s="6" t="inlineStr">
         <is>
-          <t>기도산업</t>
+          <t>니어스랩</t>
         </is>
       </c>
       <c r="B7" s="6" t="inlineStr">
         <is>
-          <t>07-31~08-06</t>
+          <t>08-03~08-07</t>
         </is>
       </c>
       <c r="C7" s="6" t="inlineStr">
         <is>
-          <t>24,800~28,400</t>
+          <t>30,000~41,200</t>
         </is>
       </c>
       <c r="D7" s="7" t="inlineStr">
         <is>
-          <t>1,700,000</t>
+          <t>910,000</t>
         </is>
       </c>
       <c r="E7" s="7" t="inlineStr">
         <is>
-          <t>48,280,000,000</t>
+          <t>37,492,000,000</t>
         </is>
       </c>
       <c r="F7" s="6" t="inlineStr">
         <is>
-          <t>10.01배 (PER)</t>
+          <t>44.41배 (PER)</t>
         </is>
       </c>
       <c r="G7" s="6" t="inlineStr">
         <is>
-          <t>28,400</t>
+          <t>41,200</t>
         </is>
       </c>
       <c r="H7" s="6" t="n">
-        <v>213.31</v>
+        <v>743.49</v>
       </c>
       <c r="I7" s="6" t="n">
-        <v>637</v>
+        <v>1795</v>
       </c>
       <c r="J7" s="18" t="inlineStr">
         <is>
@@ -7697,23 +7697,23 @@
       <c r="L7" s="6" t="inlineStr"/>
       <c r="M7" s="6" t="inlineStr">
         <is>
-          <t>2026-08-21</t>
+          <t>2026-08-24</t>
         </is>
       </c>
       <c r="N7" s="6" t="inlineStr">
         <is>
-          <t>미래에셋증권</t>
+          <t>삼성증권</t>
         </is>
       </c>
       <c r="O7" s="6" t="inlineStr"/>
       <c r="P7" s="7" t="inlineStr">
         <is>
-          <t>716,720,000</t>
+          <t>1,265,355,000</t>
         </is>
       </c>
       <c r="Q7" s="6" t="inlineStr">
         <is>
-          <t>1.0%</t>
+          <t>4.50%</t>
         </is>
       </c>
       <c r="R7" s="6" t="inlineStr">
@@ -7725,44 +7725,44 @@
     <row r="8" ht="30" customHeight="1">
       <c r="A8" s="6" t="inlineStr">
         <is>
-          <t>인제니아테라퓨틱스</t>
+          <t>기도산업</t>
         </is>
       </c>
       <c r="B8" s="6" t="inlineStr">
         <is>
-          <t>07-20~07-24</t>
+          <t>07-31~08-06</t>
         </is>
       </c>
       <c r="C8" s="6" t="inlineStr">
         <is>
-          <t>12,000~14,500</t>
+          <t>24,800~28,400</t>
         </is>
       </c>
       <c r="D8" s="7" t="inlineStr">
         <is>
-          <t>5,000,000</t>
+          <t>1,700,000</t>
         </is>
       </c>
       <c r="E8" s="7" t="inlineStr">
         <is>
-          <t>60,000,000,000</t>
+          <t>48,280,000,000</t>
         </is>
       </c>
       <c r="F8" s="6" t="inlineStr">
         <is>
-          <t>22.89배 (PER)</t>
+          <t>10.01배 (PER)</t>
         </is>
       </c>
       <c r="G8" s="6" t="inlineStr">
         <is>
-          <t>12,000</t>
+          <t>28,400</t>
         </is>
       </c>
       <c r="H8" s="6" t="n">
-        <v>50.4</v>
+        <v>213.31</v>
       </c>
       <c r="I8" s="6" t="n">
-        <v>307</v>
+        <v>637</v>
       </c>
       <c r="J8" s="18" t="inlineStr">
         <is>
@@ -7777,23 +7777,23 @@
       <c r="L8" s="6" t="inlineStr"/>
       <c r="M8" s="6" t="inlineStr">
         <is>
-          <t>2026-08-18</t>
+          <t>2026-08-21</t>
         </is>
       </c>
       <c r="N8" s="6" t="inlineStr">
         <is>
-          <t>삼성증권</t>
+          <t>미래에셋증권</t>
         </is>
       </c>
       <c r="O8" s="6" t="inlineStr"/>
       <c r="P8" s="7" t="inlineStr">
         <is>
-          <t>4,095,000,000</t>
+          <t>716,720,000</t>
         </is>
       </c>
       <c r="Q8" s="6" t="inlineStr">
         <is>
-          <t>6.5%</t>
+          <t>1.0%</t>
         </is>
       </c>
       <c r="R8" s="6" t="inlineStr">
@@ -7805,44 +7805,44 @@
     <row r="9" ht="30" customHeight="1">
       <c r="A9" s="6" t="inlineStr">
         <is>
-          <t>케이앤에스아이앤씨</t>
+          <t>인제니아테라퓨틱스</t>
         </is>
       </c>
       <c r="B9" s="6" t="inlineStr">
         <is>
-          <t>07-27~07-31</t>
+          <t>07-20~07-24</t>
         </is>
       </c>
       <c r="C9" s="6" t="inlineStr">
         <is>
-          <t>9,000~11,000</t>
+          <t>12,000~14,500</t>
         </is>
       </c>
       <c r="D9" s="7" t="inlineStr">
         <is>
-          <t>2,400,000</t>
+          <t>5,000,000</t>
         </is>
       </c>
       <c r="E9" s="7" t="inlineStr">
         <is>
-          <t>26,400,000,000</t>
+          <t>60,000,000,000</t>
         </is>
       </c>
       <c r="F9" s="6" t="inlineStr">
         <is>
-          <t>42.08배 (PER)</t>
+          <t>22.89배 (PER)</t>
         </is>
       </c>
       <c r="G9" s="6" t="inlineStr">
         <is>
-          <t>11,000</t>
+          <t>12,000</t>
         </is>
       </c>
       <c r="H9" s="6" t="n">
-        <v>938.24</v>
+        <v>50.4</v>
       </c>
       <c r="I9" s="6" t="n">
-        <v>2024</v>
+        <v>307</v>
       </c>
       <c r="J9" s="18" t="inlineStr">
         <is>
@@ -7857,23 +7857,23 @@
       <c r="L9" s="6" t="inlineStr"/>
       <c r="M9" s="6" t="inlineStr">
         <is>
-          <t>2026-08-13</t>
+          <t>2026-08-18</t>
         </is>
       </c>
       <c r="N9" s="6" t="inlineStr">
         <is>
-          <t>아이비케이투자증권</t>
+          <t>삼성증권</t>
         </is>
       </c>
       <c r="O9" s="6" t="inlineStr"/>
       <c r="P9" s="7" t="inlineStr">
         <is>
-          <t>1,500,000,000</t>
+          <t>4,095,000,000</t>
         </is>
       </c>
       <c r="Q9" s="6" t="inlineStr">
         <is>
-          <t>3.5%</t>
+          <t>6.5%</t>
         </is>
       </c>
       <c r="R9" s="6" t="inlineStr">
@@ -7885,44 +7885,44 @@
     <row r="10" ht="30" customHeight="1">
       <c r="A10" s="6" t="inlineStr">
         <is>
-          <t>딜리셔스</t>
+          <t>케이앤에스아이앤씨</t>
         </is>
       </c>
       <c r="B10" s="6" t="inlineStr">
         <is>
-          <t>07-23~07-29</t>
+          <t>07-27~07-31</t>
         </is>
       </c>
       <c r="C10" s="6" t="inlineStr">
         <is>
-          <t>5,000~7,000</t>
+          <t>9,000~11,000</t>
         </is>
       </c>
       <c r="D10" s="7" t="inlineStr">
         <is>
-          <t>2,200,000</t>
+          <t>2,400,000</t>
         </is>
       </c>
       <c r="E10" s="7" t="inlineStr">
         <is>
-          <t>15,400,000,000</t>
+          <t>26,400,000,000</t>
         </is>
       </c>
       <c r="F10" s="6" t="inlineStr">
         <is>
-          <t>23.93배 (PER)</t>
+          <t>42.08배 (PER)</t>
         </is>
       </c>
       <c r="G10" s="6" t="inlineStr">
         <is>
-          <t>7,000</t>
+          <t>11,000</t>
         </is>
       </c>
       <c r="H10" s="6" t="n">
-        <v>184.06</v>
+        <v>938.24</v>
       </c>
       <c r="I10" s="6" t="n">
-        <v>441</v>
+        <v>2024</v>
       </c>
       <c r="J10" s="18" t="inlineStr">
         <is>
@@ -7937,23 +7937,23 @@
       <c r="L10" s="6" t="inlineStr"/>
       <c r="M10" s="6" t="inlineStr">
         <is>
-          <t>2026-08-12</t>
+          <t>2026-08-13</t>
         </is>
       </c>
       <c r="N10" s="6" t="inlineStr">
         <is>
-          <t>한국투자증권</t>
+          <t>아이비케이투자증권</t>
         </is>
       </c>
       <c r="O10" s="6" t="inlineStr"/>
       <c r="P10" s="7" t="inlineStr">
         <is>
-          <t>566,500,000</t>
+          <t>1,500,000,000</t>
         </is>
       </c>
       <c r="Q10" s="6" t="inlineStr">
         <is>
-          <t>5.0%</t>
+          <t>3.5%</t>
         </is>
       </c>
       <c r="R10" s="6" t="inlineStr">
@@ -7965,44 +7965,44 @@
     <row r="11" ht="30" customHeight="1">
       <c r="A11" s="6" t="inlineStr">
         <is>
-          <t>에이치엘지노믹스</t>
+          <t>딜리셔스</t>
         </is>
       </c>
       <c r="B11" s="6" t="inlineStr">
         <is>
-          <t>07-02~07-08</t>
+          <t>07-23~07-29</t>
         </is>
       </c>
       <c r="C11" s="6" t="inlineStr">
         <is>
-          <t>18,500~21,500</t>
+          <t>5,000~7,000</t>
         </is>
       </c>
       <c r="D11" s="7" t="inlineStr">
         <is>
-          <t>2,565,000</t>
+          <t>2,200,000</t>
         </is>
       </c>
       <c r="E11" s="7" t="inlineStr">
         <is>
-          <t>55,147,500,000</t>
+          <t>15,400,000,000</t>
         </is>
       </c>
       <c r="F11" s="6" t="inlineStr">
         <is>
-          <t>12.85배 (EV/EBITDA)</t>
+          <t>23.93배 (PER)</t>
         </is>
       </c>
       <c r="G11" s="6" t="inlineStr">
         <is>
-          <t>21,500</t>
+          <t>7,000</t>
         </is>
       </c>
       <c r="H11" s="6" t="n">
-        <v>714.52</v>
+        <v>184.06</v>
       </c>
       <c r="I11" s="6" t="n">
-        <v>2148</v>
+        <v>441</v>
       </c>
       <c r="J11" s="18" t="inlineStr">
         <is>
@@ -8017,27 +8017,23 @@
       <c r="L11" s="6" t="inlineStr"/>
       <c r="M11" s="6" t="inlineStr">
         <is>
-          <t>2026-07-24</t>
+          <t>2026-08-12</t>
         </is>
       </c>
       <c r="N11" s="6" t="inlineStr">
         <is>
-          <t>KB</t>
-        </is>
-      </c>
-      <c r="O11" s="6" t="inlineStr">
-        <is>
-          <t>아이비케이투자증권, IBK투자증권, IBK투자증권, IBK투자증권, IBK투자증권, IBK투자증권㈜, 보통주, IBK투자증권㈜</t>
-        </is>
-      </c>
+          <t>한국투자증권</t>
+        </is>
+      </c>
+      <c r="O11" s="6" t="inlineStr"/>
       <c r="P11" s="7" t="inlineStr">
         <is>
-          <t>1,211</t>
+          <t>566,500,000</t>
         </is>
       </c>
       <c r="Q11" s="6" t="inlineStr">
         <is>
-          <t>2.5%</t>
+          <t>5.0%</t>
         </is>
       </c>
       <c r="R11" s="6" t="inlineStr">
@@ -8049,63 +8045,59 @@
     <row r="12" ht="30" customHeight="1">
       <c r="A12" s="6" t="inlineStr">
         <is>
-          <t>레메디</t>
-        </is>
-      </c>
-      <c r="B12" s="18" t="inlineStr">
-        <is>
-          <t>수집예정</t>
+          <t>에이치엘지노믹스</t>
+        </is>
+      </c>
+      <c r="B12" s="6" t="inlineStr">
+        <is>
+          <t>07-02~07-08</t>
         </is>
       </c>
       <c r="C12" s="6" t="inlineStr">
         <is>
-          <t>17,800~20,700</t>
+          <t>18,500~21,500</t>
         </is>
       </c>
       <c r="D12" s="7" t="inlineStr">
         <is>
-          <t>1,200,000</t>
+          <t>2,565,000</t>
         </is>
       </c>
       <c r="E12" s="7" t="inlineStr">
         <is>
-          <t>24,840,000,000</t>
+          <t>55,147,500,000</t>
         </is>
       </c>
       <c r="F12" s="6" t="inlineStr">
         <is>
-          <t>21.95배 (PER)</t>
+          <t>12.85배 (EV/EBITDA)</t>
         </is>
       </c>
       <c r="G12" s="6" t="inlineStr">
         <is>
-          <t>20,700</t>
-        </is>
-      </c>
-      <c r="H12" s="6" t="inlineStr">
-        <is>
-          <t>1,146.41</t>
-        </is>
-      </c>
-      <c r="I12" s="6" t="inlineStr">
-        <is>
-          <t>2,246</t>
-        </is>
+          <t>21,500</t>
+        </is>
+      </c>
+      <c r="H12" s="6" t="n">
+        <v>714.52</v>
+      </c>
+      <c r="I12" s="6" t="n">
+        <v>2148</v>
       </c>
       <c r="J12" s="18" t="inlineStr">
         <is>
           <t>수집예정</t>
         </is>
       </c>
-      <c r="K12" s="6" t="inlineStr">
-        <is>
-          <t>1,706.71</t>
+      <c r="K12" s="18" t="inlineStr">
+        <is>
+          <t>수집예정</t>
         </is>
       </c>
       <c r="L12" s="6" t="inlineStr"/>
       <c r="M12" s="6" t="inlineStr">
         <is>
-          <t>2026-07-13</t>
+          <t>2026-07-24</t>
         </is>
       </c>
       <c r="N12" s="6" t="inlineStr">
@@ -8113,15 +8105,19 @@
           <t>KB</t>
         </is>
       </c>
-      <c r="O12" s="6" t="inlineStr"/>
+      <c r="O12" s="6" t="inlineStr">
+        <is>
+          <t>아이비케이투자증권, IBK투자증권, IBK투자증권, IBK투자증권, IBK투자증권, IBK투자증권㈜, 보통주, IBK투자증권㈜</t>
+        </is>
+      </c>
       <c r="P12" s="7" t="inlineStr">
         <is>
-          <t>1,279</t>
+          <t>1,211</t>
         </is>
       </c>
       <c r="Q12" s="6" t="inlineStr">
         <is>
-          <t>5.0%</t>
+          <t>2.5%</t>
         </is>
       </c>
       <c r="R12" s="6" t="inlineStr">
@@ -8133,7 +8129,7 @@
     <row r="13" ht="30" customHeight="1">
       <c r="A13" s="6" t="inlineStr">
         <is>
-          <t>레몬헬스케어</t>
+          <t>레메디</t>
         </is>
       </c>
       <c r="B13" s="18" t="inlineStr">
@@ -8143,45 +8139,53 @@
       </c>
       <c r="C13" s="6" t="inlineStr">
         <is>
-          <t>7,500~10,000</t>
+          <t>17,800~20,700</t>
         </is>
       </c>
       <c r="D13" s="7" t="inlineStr">
         <is>
-          <t>2,000,000</t>
+          <t>1,200,000</t>
         </is>
       </c>
       <c r="E13" s="7" t="inlineStr">
         <is>
-          <t>20,000</t>
+          <t>24,840,000,000</t>
         </is>
       </c>
       <c r="F13" s="6" t="inlineStr">
         <is>
-          <t>25.48배 (PER)</t>
-        </is>
-      </c>
-      <c r="G13" s="6" t="n">
-        <v>10000</v>
-      </c>
-      <c r="H13" s="6" t="n">
-        <v>1238</v>
-      </c>
-      <c r="I13" s="6" t="n">
-        <v>2233</v>
-      </c>
-      <c r="J13" s="6" t="inlineStr">
-        <is>
-          <t>2026-06-24~25</t>
-        </is>
-      </c>
-      <c r="K13" s="6" t="n">
-        <v>1510.57</v>
+          <t>21.95배 (PER)</t>
+        </is>
+      </c>
+      <c r="G13" s="6" t="inlineStr">
+        <is>
+          <t>20,700</t>
+        </is>
+      </c>
+      <c r="H13" s="6" t="inlineStr">
+        <is>
+          <t>1,146.41</t>
+        </is>
+      </c>
+      <c r="I13" s="6" t="inlineStr">
+        <is>
+          <t>2,246</t>
+        </is>
+      </c>
+      <c r="J13" s="18" t="inlineStr">
+        <is>
+          <t>수집예정</t>
+        </is>
+      </c>
+      <c r="K13" s="6" t="inlineStr">
+        <is>
+          <t>1,706.71</t>
+        </is>
       </c>
       <c r="L13" s="6" t="inlineStr"/>
       <c r="M13" s="6" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-07-13</t>
         </is>
       </c>
       <c r="N13" s="6" t="inlineStr">
@@ -8192,12 +8196,12 @@
       <c r="O13" s="6" t="inlineStr"/>
       <c r="P13" s="7" t="inlineStr">
         <is>
-          <t>824</t>
+          <t>1,279</t>
         </is>
       </c>
       <c r="Q13" s="6" t="inlineStr">
         <is>
-          <t>4.0%</t>
+          <t>5.0%</t>
         </is>
       </c>
       <c r="R13" s="6" t="inlineStr">
@@ -8209,7 +8213,7 @@
     <row r="14" ht="30" customHeight="1">
       <c r="A14" s="6" t="inlineStr">
         <is>
-          <t>매드업</t>
+          <t>레몬헬스케어</t>
         </is>
       </c>
       <c r="B14" s="18" t="inlineStr">
@@ -8219,7 +8223,7 @@
       </c>
       <c r="C14" s="6" t="inlineStr">
         <is>
-          <t>7,000~8,000</t>
+          <t>7,500~10,000</t>
         </is>
       </c>
       <c r="D14" s="7" t="inlineStr">
@@ -8229,51 +8233,51 @@
       </c>
       <c r="E14" s="7" t="inlineStr">
         <is>
-          <t>16,000</t>
+          <t>20,000</t>
         </is>
       </c>
       <c r="F14" s="6" t="inlineStr">
         <is>
-          <t>24.57배 (PER)</t>
+          <t>25.48배 (PER)</t>
         </is>
       </c>
       <c r="G14" s="6" t="n">
-        <v>8000</v>
+        <v>10000</v>
       </c>
       <c r="H14" s="6" t="n">
-        <v>1396.29</v>
+        <v>1238</v>
       </c>
       <c r="I14" s="6" t="n">
-        <v>2392</v>
+        <v>2233</v>
       </c>
       <c r="J14" s="6" t="inlineStr">
         <is>
-          <t>2026-06-23~24</t>
+          <t>2026-06-24~25</t>
         </is>
       </c>
       <c r="K14" s="6" t="n">
-        <v>3304.76</v>
+        <v>1510.57</v>
       </c>
       <c r="L14" s="6" t="inlineStr"/>
       <c r="M14" s="6" t="inlineStr">
         <is>
-          <t>2026-07-01</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="N14" s="6" t="inlineStr">
         <is>
-          <t>미래</t>
+          <t>KB</t>
         </is>
       </c>
       <c r="O14" s="6" t="inlineStr"/>
       <c r="P14" s="7" t="inlineStr">
         <is>
-          <t>742</t>
+          <t>824</t>
         </is>
       </c>
       <c r="Q14" s="6" t="inlineStr">
         <is>
-          <t>4.5%</t>
+          <t>4.0%</t>
         </is>
       </c>
       <c r="R14" s="6" t="inlineStr">
@@ -8285,75 +8289,71 @@
     <row r="15" ht="30" customHeight="1">
       <c r="A15" s="6" t="inlineStr">
         <is>
-          <t>한국제16호스팩</t>
-        </is>
-      </c>
-      <c r="B15" s="19" t="inlineStr">
-        <is>
-          <t>해당없음</t>
+          <t>매드업</t>
+        </is>
+      </c>
+      <c r="B15" s="18" t="inlineStr">
+        <is>
+          <t>수집예정</t>
         </is>
       </c>
       <c r="C15" s="6" t="inlineStr">
         <is>
-          <t>2,000</t>
+          <t>7,000~8,000</t>
         </is>
       </c>
       <c r="D15" s="7" t="inlineStr">
         <is>
-          <t>5,500,000</t>
+          <t>2,000,000</t>
         </is>
       </c>
       <c r="E15" s="7" t="inlineStr">
         <is>
-          <t>11,000</t>
-        </is>
-      </c>
-      <c r="F15" s="19" t="inlineStr">
-        <is>
-          <t>해당없음</t>
-        </is>
-      </c>
-      <c r="G15" s="6" t="inlineStr">
-        <is>
-          <t>2,000</t>
-        </is>
+          <t>16,000</t>
+        </is>
+      </c>
+      <c r="F15" s="6" t="inlineStr">
+        <is>
+          <t>24.57배 (PER)</t>
+        </is>
+      </c>
+      <c r="G15" s="6" t="n">
+        <v>8000</v>
       </c>
       <c r="H15" s="6" t="n">
-        <v>1364.09</v>
+        <v>1396.29</v>
       </c>
       <c r="I15" s="6" t="n">
-        <v>2089</v>
+        <v>2392</v>
       </c>
       <c r="J15" s="6" t="inlineStr">
         <is>
-          <t>2026-06-22~06-23</t>
-        </is>
-      </c>
-      <c r="K15" s="6" t="inlineStr">
-        <is>
-          <t>1,274.77</t>
-        </is>
+          <t>2026-06-23~24</t>
+        </is>
+      </c>
+      <c r="K15" s="6" t="n">
+        <v>3304.76</v>
       </c>
       <c r="L15" s="6" t="inlineStr"/>
       <c r="M15" s="6" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-07-01</t>
         </is>
       </c>
       <c r="N15" s="6" t="inlineStr">
         <is>
-          <t>한국</t>
+          <t>미래</t>
         </is>
       </c>
       <c r="O15" s="6" t="inlineStr"/>
       <c r="P15" s="7" t="inlineStr">
         <is>
-          <t>330</t>
+          <t>742</t>
         </is>
       </c>
       <c r="Q15" s="6" t="inlineStr">
         <is>
-          <t>3.00%</t>
+          <t>4.5%</t>
         </is>
       </c>
       <c r="R15" s="6" t="inlineStr">
@@ -8365,51 +8365,53 @@
     <row r="16" ht="30" customHeight="1">
       <c r="A16" s="6" t="inlineStr">
         <is>
-          <t>스트라드비젼</t>
-        </is>
-      </c>
-      <c r="B16" s="18" t="inlineStr">
-        <is>
-          <t>수집예정</t>
+          <t>한국제16호스팩</t>
+        </is>
+      </c>
+      <c r="B16" s="19" t="inlineStr">
+        <is>
+          <t>해당없음</t>
         </is>
       </c>
       <c r="C16" s="6" t="inlineStr">
         <is>
-          <t>12,000~14,000</t>
+          <t>2,000</t>
         </is>
       </c>
       <c r="D16" s="7" t="inlineStr">
         <is>
-          <t>7,000,000</t>
+          <t>5,500,000</t>
         </is>
       </c>
       <c r="E16" s="7" t="inlineStr">
         <is>
-          <t>84,000</t>
-        </is>
-      </c>
-      <c r="F16" s="6" t="inlineStr">
-        <is>
-          <t>37.45배 (PER)</t>
-        </is>
-      </c>
-      <c r="G16" s="6" t="n">
-        <v>12000</v>
+          <t>11,000</t>
+        </is>
+      </c>
+      <c r="F16" s="19" t="inlineStr">
+        <is>
+          <t>해당없음</t>
+        </is>
+      </c>
+      <c r="G16" s="6" t="inlineStr">
+        <is>
+          <t>2,000</t>
+        </is>
       </c>
       <c r="H16" s="6" t="n">
-        <v>381.3</v>
+        <v>1364.09</v>
       </c>
       <c r="I16" s="6" t="n">
-        <v>1604</v>
+        <v>2089</v>
       </c>
       <c r="J16" s="6" t="inlineStr">
         <is>
-          <t>2026-06-18~06-19</t>
+          <t>2026-06-22~06-23</t>
         </is>
       </c>
       <c r="K16" s="6" t="inlineStr">
         <is>
-          <t>45.81</t>
+          <t>1,274.77</t>
         </is>
       </c>
       <c r="L16" s="6" t="inlineStr"/>
@@ -8420,13 +8422,13 @@
       </c>
       <c r="N16" s="6" t="inlineStr">
         <is>
-          <t>KB</t>
+          <t>한국</t>
         </is>
       </c>
       <c r="O16" s="6" t="inlineStr"/>
       <c r="P16" s="7" t="inlineStr">
         <is>
-          <t>2,575</t>
+          <t>330</t>
         </is>
       </c>
       <c r="Q16" s="6" t="inlineStr">
@@ -8443,7 +8445,7 @@
     <row r="17" ht="30" customHeight="1">
       <c r="A17" s="6" t="inlineStr">
         <is>
-          <t>져스텍</t>
+          <t>스트라드비젼</t>
         </is>
       </c>
       <c r="B17" s="18" t="inlineStr">
@@ -8453,32 +8455,32 @@
       </c>
       <c r="C17" s="6" t="inlineStr">
         <is>
-          <t>10,500~12,500</t>
+          <t>12,000~14,000</t>
         </is>
       </c>
       <c r="D17" s="7" t="inlineStr">
         <is>
-          <t>1,600,000</t>
+          <t>7,000,000</t>
         </is>
       </c>
       <c r="E17" s="7" t="inlineStr">
         <is>
-          <t>20,000</t>
+          <t>84,000</t>
         </is>
       </c>
       <c r="F17" s="6" t="inlineStr">
         <is>
-          <t>26.82배 (PER)</t>
+          <t>37.45배 (PER)</t>
         </is>
       </c>
       <c r="G17" s="6" t="n">
-        <v>12500</v>
+        <v>12000</v>
       </c>
       <c r="H17" s="6" t="n">
-        <v>1294.99</v>
+        <v>381.3</v>
       </c>
       <c r="I17" s="6" t="n">
-        <v>2252</v>
+        <v>1604</v>
       </c>
       <c r="J17" s="6" t="inlineStr">
         <is>
@@ -8487,29 +8489,29 @@
       </c>
       <c r="K17" s="6" t="inlineStr">
         <is>
-          <t>2,783.89</t>
+          <t>45.81</t>
         </is>
       </c>
       <c r="L17" s="6" t="inlineStr"/>
       <c r="M17" s="6" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="N17" s="6" t="inlineStr">
         <is>
-          <t>삼성</t>
+          <t>KB</t>
         </is>
       </c>
       <c r="O17" s="6" t="inlineStr"/>
       <c r="P17" s="7" t="inlineStr">
         <is>
-          <t>1,164</t>
+          <t>2,575</t>
         </is>
       </c>
       <c r="Q17" s="6" t="inlineStr">
         <is>
-          <t>5.65%</t>
+          <t>3.00%</t>
         </is>
       </c>
       <c r="R17" s="6" t="inlineStr">
@@ -8521,75 +8523,73 @@
     <row r="18" ht="30" customHeight="1">
       <c r="A18" s="6" t="inlineStr">
         <is>
-          <t>메리츠제2호스팩</t>
-        </is>
-      </c>
-      <c r="B18" s="19" t="inlineStr">
-        <is>
-          <t>해당없음</t>
+          <t>져스텍</t>
+        </is>
+      </c>
+      <c r="B18" s="18" t="inlineStr">
+        <is>
+          <t>수집예정</t>
         </is>
       </c>
       <c r="C18" s="6" t="inlineStr">
         <is>
-          <t>2,000</t>
+          <t>10,500~12,500</t>
         </is>
       </c>
       <c r="D18" s="7" t="inlineStr">
         <is>
-          <t>7,000,000</t>
+          <t>1,600,000</t>
         </is>
       </c>
       <c r="E18" s="7" t="inlineStr">
         <is>
-          <t>14,000</t>
-        </is>
-      </c>
-      <c r="F18" s="19" t="inlineStr">
-        <is>
-          <t>해당없음</t>
-        </is>
-      </c>
-      <c r="G18" s="6" t="inlineStr">
-        <is>
-          <t>2,000</t>
-        </is>
+          <t>20,000</t>
+        </is>
+      </c>
+      <c r="F18" s="6" t="inlineStr">
+        <is>
+          <t>26.82배 (PER)</t>
+        </is>
+      </c>
+      <c r="G18" s="6" t="n">
+        <v>12500</v>
       </c>
       <c r="H18" s="6" t="n">
-        <v>1087.58</v>
+        <v>1294.99</v>
       </c>
       <c r="I18" s="6" t="n">
-        <v>1798</v>
+        <v>2252</v>
       </c>
       <c r="J18" s="6" t="inlineStr">
         <is>
-          <t>2026-06-09~06-10</t>
+          <t>2026-06-18~06-19</t>
         </is>
       </c>
       <c r="K18" s="6" t="inlineStr">
         <is>
-          <t>1,338.66</t>
+          <t>2,783.89</t>
         </is>
       </c>
       <c r="L18" s="6" t="inlineStr"/>
       <c r="M18" s="6" t="inlineStr">
         <is>
-          <t>2026-06-19</t>
+          <t>2026-06-29</t>
         </is>
       </c>
       <c r="N18" s="6" t="inlineStr">
         <is>
-          <t>메리츠</t>
+          <t>삼성</t>
         </is>
       </c>
       <c r="O18" s="6" t="inlineStr"/>
       <c r="P18" s="7" t="inlineStr">
         <is>
-          <t>245</t>
+          <t>1,164</t>
         </is>
       </c>
       <c r="Q18" s="6" t="inlineStr">
         <is>
-          <t>1.75%</t>
+          <t>5.65%</t>
         </is>
       </c>
       <c r="R18" s="6" t="inlineStr">
@@ -8601,77 +8601,75 @@
     <row r="19" ht="30" customHeight="1">
       <c r="A19" s="6" t="inlineStr">
         <is>
-          <t>피스피스스튜디오</t>
-        </is>
-      </c>
-      <c r="B19" s="18" t="inlineStr">
-        <is>
-          <t>수집예정</t>
+          <t>메리츠제2호스팩</t>
+        </is>
+      </c>
+      <c r="B19" s="19" t="inlineStr">
+        <is>
+          <t>해당없음</t>
         </is>
       </c>
       <c r="C19" s="6" t="inlineStr">
         <is>
-          <t>19,000~21,500</t>
+          <t>2,000</t>
         </is>
       </c>
       <c r="D19" s="7" t="inlineStr">
         <is>
-          <t>2,272,637</t>
+          <t>7,000,000</t>
         </is>
       </c>
       <c r="E19" s="7" t="inlineStr">
         <is>
-          <t>48,862</t>
-        </is>
-      </c>
-      <c r="F19" s="6" t="inlineStr">
-        <is>
-          <t>21.48배 (PER)</t>
-        </is>
-      </c>
-      <c r="G19" s="6" t="n">
-        <v>21500</v>
+          <t>14,000</t>
+        </is>
+      </c>
+      <c r="F19" s="19" t="inlineStr">
+        <is>
+          <t>해당없음</t>
+        </is>
+      </c>
+      <c r="G19" s="6" t="inlineStr">
+        <is>
+          <t>2,000</t>
+        </is>
       </c>
       <c r="H19" s="6" t="n">
-        <v>847.76</v>
+        <v>1087.58</v>
       </c>
       <c r="I19" s="6" t="n">
-        <v>2329</v>
+        <v>1798</v>
       </c>
       <c r="J19" s="6" t="inlineStr">
         <is>
-          <t>2026-05-26~05-27</t>
+          <t>2026-06-09~06-10</t>
         </is>
       </c>
       <c r="K19" s="6" t="inlineStr">
         <is>
-          <t>1,191.15</t>
+          <t>1,338.66</t>
         </is>
       </c>
       <c r="L19" s="6" t="inlineStr"/>
       <c r="M19" s="6" t="inlineStr">
         <is>
-          <t>2026-06-08</t>
+          <t>2026-06-19</t>
         </is>
       </c>
       <c r="N19" s="6" t="inlineStr">
         <is>
-          <t>미래</t>
-        </is>
-      </c>
-      <c r="O19" s="6" t="inlineStr">
-        <is>
-          <t>NH</t>
-        </is>
-      </c>
+          <t>메리츠</t>
+        </is>
+      </c>
+      <c r="O19" s="6" t="inlineStr"/>
       <c r="P19" s="7" t="inlineStr">
         <is>
-          <t>1,994</t>
+          <t>245</t>
         </is>
       </c>
       <c r="Q19" s="6" t="inlineStr">
         <is>
-          <t>4.00%</t>
+          <t>1.75%</t>
         </is>
       </c>
       <c r="R19" s="6" t="inlineStr">
@@ -8683,75 +8681,77 @@
     <row r="20" ht="30" customHeight="1">
       <c r="A20" s="6" t="inlineStr">
         <is>
-          <t>대신밸런스제20호스팩</t>
-        </is>
-      </c>
-      <c r="B20" s="19" t="inlineStr">
-        <is>
-          <t>해당없음</t>
+          <t>피스피스스튜디오</t>
+        </is>
+      </c>
+      <c r="B20" s="18" t="inlineStr">
+        <is>
+          <t>수집예정</t>
         </is>
       </c>
       <c r="C20" s="6" t="inlineStr">
         <is>
-          <t>2,000</t>
+          <t>19,000~21,500</t>
         </is>
       </c>
       <c r="D20" s="7" t="inlineStr">
         <is>
-          <t>6,500,000</t>
+          <t>2,272,637</t>
         </is>
       </c>
       <c r="E20" s="7" t="inlineStr">
         <is>
-          <t>13,000</t>
-        </is>
-      </c>
-      <c r="F20" s="19" t="inlineStr">
-        <is>
-          <t>해당없음</t>
-        </is>
-      </c>
-      <c r="G20" s="6" t="inlineStr">
-        <is>
-          <t>2,000</t>
-        </is>
+          <t>48,862</t>
+        </is>
+      </c>
+      <c r="F20" s="6" t="inlineStr">
+        <is>
+          <t>21.48배 (PER)</t>
+        </is>
+      </c>
+      <c r="G20" s="6" t="n">
+        <v>21500</v>
       </c>
       <c r="H20" s="6" t="n">
-        <v>1327.13</v>
+        <v>847.76</v>
       </c>
       <c r="I20" s="6" t="n">
-        <v>2194</v>
+        <v>2329</v>
       </c>
       <c r="J20" s="6" t="inlineStr">
         <is>
-          <t>2026-05-22~05-25</t>
+          <t>2026-05-26~05-27</t>
         </is>
       </c>
       <c r="K20" s="6" t="inlineStr">
         <is>
-          <t>1,486.88</t>
+          <t>1,191.15</t>
         </is>
       </c>
       <c r="L20" s="6" t="inlineStr"/>
       <c r="M20" s="6" t="inlineStr">
         <is>
-          <t>2026-06-05</t>
+          <t>2026-06-08</t>
         </is>
       </c>
       <c r="N20" s="6" t="inlineStr">
         <is>
-          <t>대신</t>
-        </is>
-      </c>
-      <c r="O20" s="6" t="inlineStr"/>
+          <t>미래</t>
+        </is>
+      </c>
+      <c r="O20" s="6" t="inlineStr">
+        <is>
+          <t>NH</t>
+        </is>
+      </c>
       <c r="P20" s="7" t="inlineStr">
         <is>
-          <t>390</t>
+          <t>1,994</t>
         </is>
       </c>
       <c r="Q20" s="6" t="inlineStr">
         <is>
-          <t>3.00%</t>
+          <t>4.00%</t>
         </is>
       </c>
       <c r="R20" s="6" t="inlineStr">
@@ -8763,73 +8763,75 @@
     <row r="21" ht="30" customHeight="1">
       <c r="A21" s="6" t="inlineStr">
         <is>
-          <t>마키나락스</t>
-        </is>
-      </c>
-      <c r="B21" s="18" t="inlineStr">
-        <is>
-          <t>수집예정</t>
+          <t>대신밸런스제20호스팩</t>
+        </is>
+      </c>
+      <c r="B21" s="19" t="inlineStr">
+        <is>
+          <t>해당없음</t>
         </is>
       </c>
       <c r="C21" s="6" t="inlineStr">
         <is>
-          <t>12,500~15,000</t>
+          <t>2,000</t>
         </is>
       </c>
       <c r="D21" s="7" t="inlineStr">
         <is>
-          <t>2,635,000</t>
+          <t>6,500,000</t>
         </is>
       </c>
       <c r="E21" s="7" t="inlineStr">
         <is>
-          <t>39,525</t>
-        </is>
-      </c>
-      <c r="F21" s="6" t="inlineStr">
-        <is>
-          <t>40.5배 (PER)</t>
-        </is>
-      </c>
-      <c r="G21" s="6" t="n">
-        <v>15000</v>
+          <t>13,000</t>
+        </is>
+      </c>
+      <c r="F21" s="19" t="inlineStr">
+        <is>
+          <t>해당없음</t>
+        </is>
+      </c>
+      <c r="G21" s="6" t="inlineStr">
+        <is>
+          <t>2,000</t>
+        </is>
       </c>
       <c r="H21" s="6" t="n">
-        <v>1196.08</v>
+        <v>1327.13</v>
       </c>
       <c r="I21" s="6" t="n">
-        <v>2427</v>
+        <v>2194</v>
       </c>
       <c r="J21" s="6" t="inlineStr">
         <is>
-          <t>2026-05-11~05-12</t>
+          <t>2026-05-22~05-25</t>
         </is>
       </c>
       <c r="K21" s="6" t="inlineStr">
         <is>
-          <t>2,807.79</t>
+          <t>1,486.88</t>
         </is>
       </c>
       <c r="L21" s="6" t="inlineStr"/>
       <c r="M21" s="6" t="inlineStr">
         <is>
-          <t>2026-05-20</t>
+          <t>2026-06-05</t>
         </is>
       </c>
       <c r="N21" s="6" t="inlineStr">
         <is>
-          <t>미래</t>
+          <t>대신</t>
         </is>
       </c>
       <c r="O21" s="6" t="inlineStr"/>
       <c r="P21" s="7" t="inlineStr">
         <is>
-          <t>2,026</t>
+          <t>390</t>
         </is>
       </c>
       <c r="Q21" s="6" t="inlineStr">
         <is>
-          <t>5.00%</t>
+          <t>3.00%</t>
         </is>
       </c>
       <c r="R21" s="6" t="inlineStr">
@@ -8841,7 +8843,7 @@
     <row r="22" ht="30" customHeight="1">
       <c r="A22" s="6" t="inlineStr">
         <is>
-          <t>폴레드</t>
+          <t>마키나락스</t>
         </is>
       </c>
       <c r="B22" s="18" t="inlineStr">
@@ -8851,63 +8853,63 @@
       </c>
       <c r="C22" s="6" t="inlineStr">
         <is>
-          <t>4,100~5,000</t>
+          <t>12,500~15,000</t>
         </is>
       </c>
       <c r="D22" s="7" t="inlineStr">
         <is>
-          <t>2,600,000</t>
+          <t>2,635,000</t>
         </is>
       </c>
       <c r="E22" s="7" t="inlineStr">
         <is>
-          <t>13,000</t>
+          <t>39,525</t>
         </is>
       </c>
       <c r="F22" s="6" t="inlineStr">
         <is>
-          <t>19.05배 (PER)</t>
+          <t>40.5배 (PER)</t>
         </is>
       </c>
       <c r="G22" s="6" t="n">
-        <v>5000</v>
+        <v>15000</v>
       </c>
       <c r="H22" s="6" t="n">
-        <v>1486.66</v>
+        <v>1196.08</v>
       </c>
       <c r="I22" s="6" t="n">
-        <v>2372</v>
+        <v>2427</v>
       </c>
       <c r="J22" s="6" t="inlineStr">
         <is>
-          <t>2026-05-04~05-05</t>
+          <t>2026-05-11~05-12</t>
         </is>
       </c>
       <c r="K22" s="6" t="inlineStr">
         <is>
-          <t>3,169.86</t>
+          <t>2,807.79</t>
         </is>
       </c>
       <c r="L22" s="6" t="inlineStr"/>
       <c r="M22" s="6" t="inlineStr">
         <is>
-          <t>2026-05-14</t>
+          <t>2026-05-20</t>
         </is>
       </c>
       <c r="N22" s="6" t="inlineStr">
         <is>
-          <t>NH</t>
+          <t>미래</t>
         </is>
       </c>
       <c r="O22" s="6" t="inlineStr"/>
       <c r="P22" s="7" t="inlineStr">
         <is>
-          <t>540</t>
+          <t>2,026</t>
         </is>
       </c>
       <c r="Q22" s="6" t="inlineStr">
         <is>
-          <t>4.03%</t>
+          <t>5.00%</t>
         </is>
       </c>
       <c r="R22" s="6" t="inlineStr">
@@ -8919,7 +8921,7 @@
     <row r="23" ht="30" customHeight="1">
       <c r="A23" s="6" t="inlineStr">
         <is>
-          <t>코스모로보틱스</t>
+          <t>폴레드</t>
         </is>
       </c>
       <c r="B23" s="18" t="inlineStr">
@@ -8929,67 +8931,63 @@
       </c>
       <c r="C23" s="6" t="inlineStr">
         <is>
-          <t>5,300~6,000</t>
+          <t>4,100~5,000</t>
         </is>
       </c>
       <c r="D23" s="7" t="inlineStr">
         <is>
-          <t>4,170,000</t>
+          <t>2,600,000</t>
         </is>
       </c>
       <c r="E23" s="7" t="inlineStr">
         <is>
-          <t>25,020</t>
+          <t>13,000</t>
         </is>
       </c>
       <c r="F23" s="6" t="inlineStr">
         <is>
-          <t>47.45배 (PER)</t>
+          <t>19.05배 (PER)</t>
         </is>
       </c>
       <c r="G23" s="6" t="n">
-        <v>6000</v>
+        <v>5000</v>
       </c>
       <c r="H23" s="6" t="n">
-        <v>1140.11</v>
+        <v>1486.66</v>
       </c>
       <c r="I23" s="6" t="n">
-        <v>2257</v>
+        <v>2372</v>
       </c>
       <c r="J23" s="6" t="inlineStr">
         <is>
-          <t>2026-04-27~04-28</t>
+          <t>2026-05-04~05-05</t>
         </is>
       </c>
       <c r="K23" s="6" t="inlineStr">
         <is>
-          <t>2,013.80</t>
+          <t>3,169.86</t>
         </is>
       </c>
       <c r="L23" s="6" t="inlineStr"/>
       <c r="M23" s="6" t="inlineStr">
         <is>
-          <t>2026-05-11</t>
+          <t>2026-05-14</t>
         </is>
       </c>
       <c r="N23" s="6" t="inlineStr">
         <is>
-          <t>유진</t>
-        </is>
-      </c>
-      <c r="O23" s="6" t="inlineStr">
-        <is>
           <t>NH</t>
         </is>
       </c>
+      <c r="O23" s="6" t="inlineStr"/>
       <c r="P23" s="7" t="inlineStr">
         <is>
-          <t>1,289</t>
+          <t>540</t>
         </is>
       </c>
       <c r="Q23" s="6" t="inlineStr">
         <is>
-          <t>3.78%</t>
+          <t>4.03%</t>
         </is>
       </c>
       <c r="R23" s="6" t="inlineStr">
@@ -9001,75 +8999,77 @@
     <row r="24" ht="30" customHeight="1">
       <c r="A24" s="6" t="inlineStr">
         <is>
-          <t>신한스팩18호</t>
-        </is>
-      </c>
-      <c r="B24" s="19" t="inlineStr">
-        <is>
-          <t>해당없음</t>
+          <t>코스모로보틱스</t>
+        </is>
+      </c>
+      <c r="B24" s="18" t="inlineStr">
+        <is>
+          <t>수집예정</t>
         </is>
       </c>
       <c r="C24" s="6" t="inlineStr">
         <is>
-          <t>2,000</t>
+          <t>5,300~6,000</t>
         </is>
       </c>
       <c r="D24" s="7" t="inlineStr">
         <is>
-          <t>5,000,000</t>
+          <t>4,170,000</t>
         </is>
       </c>
       <c r="E24" s="7" t="inlineStr">
         <is>
-          <t>10,000</t>
-        </is>
-      </c>
-      <c r="F24" s="19" t="inlineStr">
-        <is>
-          <t>해당없음</t>
-        </is>
-      </c>
-      <c r="G24" s="6" t="inlineStr">
-        <is>
-          <t>2,000</t>
-        </is>
+          <t>25,020</t>
+        </is>
+      </c>
+      <c r="F24" s="6" t="inlineStr">
+        <is>
+          <t>47.45배 (PER)</t>
+        </is>
+      </c>
+      <c r="G24" s="6" t="n">
+        <v>6000</v>
       </c>
       <c r="H24" s="6" t="n">
-        <v>1388.6</v>
+        <v>1140.11</v>
       </c>
       <c r="I24" s="6" t="n">
-        <v>2044</v>
+        <v>2257</v>
       </c>
       <c r="J24" s="6" t="inlineStr">
         <is>
-          <t>2026-04-20~04-21</t>
+          <t>2026-04-27~04-28</t>
         </is>
       </c>
       <c r="K24" s="6" t="inlineStr">
         <is>
-          <t>1,601.36</t>
+          <t>2,013.80</t>
         </is>
       </c>
       <c r="L24" s="6" t="inlineStr"/>
       <c r="M24" s="6" t="inlineStr">
         <is>
-          <t>2026-04-30</t>
+          <t>2026-05-11</t>
         </is>
       </c>
       <c r="N24" s="6" t="inlineStr">
         <is>
-          <t>신한</t>
-        </is>
-      </c>
-      <c r="O24" s="6" t="inlineStr"/>
+          <t>유진</t>
+        </is>
+      </c>
+      <c r="O24" s="6" t="inlineStr">
+        <is>
+          <t>NH</t>
+        </is>
+      </c>
       <c r="P24" s="7" t="inlineStr">
         <is>
-          <t>350</t>
+          <t>1,289</t>
         </is>
       </c>
       <c r="Q24" s="6" t="inlineStr">
         <is>
-          <t>3.50%</t>
+          <t>3.78%</t>
         </is>
       </c>
       <c r="R24" s="6" t="inlineStr">
@@ -9081,42 +9081,44 @@
     <row r="25" ht="30" customHeight="1">
       <c r="A25" s="6" t="inlineStr">
         <is>
-          <t>채비</t>
-        </is>
-      </c>
-      <c r="B25" s="18" t="inlineStr">
-        <is>
-          <t>수집예정</t>
+          <t>신한스팩18호</t>
+        </is>
+      </c>
+      <c r="B25" s="19" t="inlineStr">
+        <is>
+          <t>해당없음</t>
         </is>
       </c>
       <c r="C25" s="6" t="inlineStr">
         <is>
-          <t>12,300~15,300</t>
+          <t>2,000</t>
         </is>
       </c>
       <c r="D25" s="7" t="inlineStr">
         <is>
-          <t>9,000,000</t>
+          <t>5,000,000</t>
         </is>
       </c>
       <c r="E25" s="7" t="inlineStr">
         <is>
-          <t>110,700</t>
-        </is>
-      </c>
-      <c r="F25" s="6" t="inlineStr">
-        <is>
-          <t>24.0배 (EV/EBITDA)</t>
-        </is>
-      </c>
-      <c r="G25" s="6" t="n">
-        <v>12300</v>
+          <t>10,000</t>
+        </is>
+      </c>
+      <c r="F25" s="19" t="inlineStr">
+        <is>
+          <t>해당없음</t>
+        </is>
+      </c>
+      <c r="G25" s="6" t="inlineStr">
+        <is>
+          <t>2,000</t>
+        </is>
       </c>
       <c r="H25" s="6" t="n">
-        <v>55.23</v>
+        <v>1388.6</v>
       </c>
       <c r="I25" s="6" t="n">
-        <v>751</v>
+        <v>2044</v>
       </c>
       <c r="J25" s="6" t="inlineStr">
         <is>
@@ -9125,33 +9127,29 @@
       </c>
       <c r="K25" s="6" t="inlineStr">
         <is>
-          <t>302.11</t>
+          <t>1,601.36</t>
         </is>
       </c>
       <c r="L25" s="6" t="inlineStr"/>
       <c r="M25" s="6" t="inlineStr">
         <is>
-          <t>2026-04-29</t>
+          <t>2026-04-30</t>
         </is>
       </c>
       <c r="N25" s="6" t="inlineStr">
         <is>
-          <t>KB</t>
-        </is>
-      </c>
-      <c r="O25" s="6" t="inlineStr">
-        <is>
-          <t>삼성</t>
-        </is>
-      </c>
+          <t>신한</t>
+        </is>
+      </c>
+      <c r="O25" s="6" t="inlineStr"/>
       <c r="P25" s="7" t="inlineStr">
         <is>
-          <t>3,384</t>
+          <t>350</t>
         </is>
       </c>
       <c r="Q25" s="6" t="inlineStr">
         <is>
-          <t>3.00%</t>
+          <t>3.50%</t>
         </is>
       </c>
       <c r="R25" s="6" t="inlineStr">
@@ -9163,75 +9161,77 @@
     <row r="26" ht="30" customHeight="1">
       <c r="A26" s="6" t="inlineStr">
         <is>
-          <t>키움히어로스펙2호</t>
-        </is>
-      </c>
-      <c r="B26" s="19" t="inlineStr">
-        <is>
-          <t>해당없음</t>
+          <t>채비</t>
+        </is>
+      </c>
+      <c r="B26" s="18" t="inlineStr">
+        <is>
+          <t>수집예정</t>
         </is>
       </c>
       <c r="C26" s="6" t="inlineStr">
         <is>
-          <t>2,000</t>
+          <t>12,300~15,300</t>
         </is>
       </c>
       <c r="D26" s="7" t="inlineStr">
         <is>
-          <t>6,000,000</t>
+          <t>9,000,000</t>
         </is>
       </c>
       <c r="E26" s="7" t="inlineStr">
         <is>
-          <t>12,000</t>
-        </is>
-      </c>
-      <c r="F26" s="19" t="inlineStr">
-        <is>
-          <t>해당없음</t>
-        </is>
-      </c>
-      <c r="G26" s="6" t="inlineStr">
-        <is>
-          <t>2,000</t>
-        </is>
+          <t>110,700</t>
+        </is>
+      </c>
+      <c r="F26" s="6" t="inlineStr">
+        <is>
+          <t>24.0배 (EV/EBITDA)</t>
+        </is>
+      </c>
+      <c r="G26" s="6" t="n">
+        <v>12300</v>
       </c>
       <c r="H26" s="6" t="n">
-        <v>1271.12</v>
+        <v>55.23</v>
       </c>
       <c r="I26" s="6" t="n">
-        <v>2054</v>
+        <v>751</v>
       </c>
       <c r="J26" s="6" t="inlineStr">
         <is>
-          <t>2026-04-14~04-15</t>
+          <t>2026-04-20~04-21</t>
         </is>
       </c>
       <c r="K26" s="6" t="inlineStr">
         <is>
-          <t>1,727.59</t>
+          <t>302.11</t>
         </is>
       </c>
       <c r="L26" s="6" t="inlineStr"/>
       <c r="M26" s="6" t="inlineStr">
         <is>
-          <t>2026-04-23</t>
+          <t>2026-04-29</t>
         </is>
       </c>
       <c r="N26" s="6" t="inlineStr">
         <is>
-          <t>키움</t>
-        </is>
-      </c>
-      <c r="O26" s="6" t="inlineStr"/>
+          <t>KB</t>
+        </is>
+      </c>
+      <c r="O26" s="6" t="inlineStr">
+        <is>
+          <t>삼성</t>
+        </is>
+      </c>
       <c r="P26" s="7" t="inlineStr">
         <is>
-          <t>300</t>
+          <t>3,384</t>
         </is>
       </c>
       <c r="Q26" s="6" t="inlineStr">
         <is>
-          <t>2.50%</t>
+          <t>3.00%</t>
         </is>
       </c>
       <c r="R26" s="6" t="inlineStr">
@@ -9243,7 +9243,7 @@
     <row r="27" ht="30" customHeight="1">
       <c r="A27" s="6" t="inlineStr">
         <is>
-          <t>교보스팩20호</t>
+          <t>키움히어로스펙2호</t>
         </is>
       </c>
       <c r="B27" s="19" t="inlineStr">
@@ -9258,12 +9258,12 @@
       </c>
       <c r="D27" s="7" t="inlineStr">
         <is>
-          <t>5,400,000</t>
+          <t>6,000,000</t>
         </is>
       </c>
       <c r="E27" s="7" t="inlineStr">
         <is>
-          <t>10,800</t>
+          <t>12,000</t>
         </is>
       </c>
       <c r="F27" s="19" t="inlineStr">
@@ -9277,30 +9277,30 @@
         </is>
       </c>
       <c r="H27" s="6" t="n">
-        <v>1196.99</v>
+        <v>1271.12</v>
       </c>
       <c r="I27" s="6" t="n">
-        <v>1855</v>
+        <v>2054</v>
       </c>
       <c r="J27" s="6" t="inlineStr">
         <is>
-          <t>2026-03-23~03-24</t>
+          <t>2026-04-14~04-15</t>
         </is>
       </c>
       <c r="K27" s="6" t="inlineStr">
         <is>
-          <t>747.00</t>
+          <t>1,727.59</t>
         </is>
       </c>
       <c r="L27" s="6" t="inlineStr"/>
       <c r="M27" s="6" t="inlineStr">
         <is>
-          <t>2026-04-02</t>
+          <t>2026-04-23</t>
         </is>
       </c>
       <c r="N27" s="6" t="inlineStr">
         <is>
-          <t>교보</t>
+          <t>키움</t>
         </is>
       </c>
       <c r="O27" s="6" t="inlineStr"/>
@@ -9311,7 +9311,7 @@
       </c>
       <c r="Q27" s="6" t="inlineStr">
         <is>
-          <t>2.78%</t>
+          <t>2.50%</t>
         </is>
       </c>
       <c r="R27" s="6" t="inlineStr">
@@ -9323,42 +9323,44 @@
     <row r="28" ht="30" customHeight="1">
       <c r="A28" s="6" t="inlineStr">
         <is>
-          <t>인벤테라</t>
-        </is>
-      </c>
-      <c r="B28" s="18" t="inlineStr">
-        <is>
-          <t>수집예정</t>
+          <t>교보스팩20호</t>
+        </is>
+      </c>
+      <c r="B28" s="19" t="inlineStr">
+        <is>
+          <t>해당없음</t>
         </is>
       </c>
       <c r="C28" s="6" t="inlineStr">
         <is>
-          <t>12,100~16,600</t>
+          <t>2,000</t>
         </is>
       </c>
       <c r="D28" s="7" t="inlineStr">
         <is>
-          <t>1,180,000</t>
+          <t>5,400,000</t>
         </is>
       </c>
       <c r="E28" s="7" t="inlineStr">
         <is>
-          <t>19,588</t>
-        </is>
-      </c>
-      <c r="F28" s="6" t="inlineStr">
-        <is>
-          <t>24.34배 (PER)</t>
-        </is>
-      </c>
-      <c r="G28" s="6" t="n">
-        <v>16600</v>
+          <t>10,800</t>
+        </is>
+      </c>
+      <c r="F28" s="19" t="inlineStr">
+        <is>
+          <t>해당없음</t>
+        </is>
+      </c>
+      <c r="G28" s="6" t="inlineStr">
+        <is>
+          <t>2,000</t>
+        </is>
       </c>
       <c r="H28" s="6" t="n">
-        <v>1328.82</v>
+        <v>1196.99</v>
       </c>
       <c r="I28" s="6" t="n">
-        <v>2309</v>
+        <v>1855</v>
       </c>
       <c r="J28" s="6" t="inlineStr">
         <is>
@@ -9367,7 +9369,7 @@
       </c>
       <c r="K28" s="6" t="inlineStr">
         <is>
-          <t>1,913.00</t>
+          <t>747.00</t>
         </is>
       </c>
       <c r="L28" s="6" t="inlineStr"/>
@@ -9378,18 +9380,18 @@
       </c>
       <c r="N28" s="6" t="inlineStr">
         <is>
-          <t>NH</t>
+          <t>교보</t>
         </is>
       </c>
       <c r="O28" s="6" t="inlineStr"/>
       <c r="P28" s="7" t="inlineStr">
         <is>
-          <t>1,211</t>
+          <t>300</t>
         </is>
       </c>
       <c r="Q28" s="6" t="inlineStr">
         <is>
-          <t>6.00%</t>
+          <t>2.78%</t>
         </is>
       </c>
       <c r="R28" s="6" t="inlineStr">
@@ -9401,75 +9403,73 @@
     <row r="29" ht="30" customHeight="1">
       <c r="A29" s="6" t="inlineStr">
         <is>
-          <t>신한스팩17호</t>
-        </is>
-      </c>
-      <c r="B29" s="19" t="inlineStr">
-        <is>
-          <t>해당없음</t>
+          <t>인벤테라</t>
+        </is>
+      </c>
+      <c r="B29" s="18" t="inlineStr">
+        <is>
+          <t>수집예정</t>
         </is>
       </c>
       <c r="C29" s="6" t="inlineStr">
         <is>
-          <t>2,000</t>
+          <t>12,100~16,600</t>
         </is>
       </c>
       <c r="D29" s="7" t="inlineStr">
         <is>
-          <t>5,000,000</t>
+          <t>1,180,000</t>
         </is>
       </c>
       <c r="E29" s="7" t="inlineStr">
         <is>
-          <t>10,000</t>
-        </is>
-      </c>
-      <c r="F29" s="19" t="inlineStr">
-        <is>
-          <t>해당없음</t>
-        </is>
-      </c>
-      <c r="G29" s="6" t="inlineStr">
-        <is>
-          <t>2,000</t>
-        </is>
+          <t>19,588</t>
+        </is>
+      </c>
+      <c r="F29" s="6" t="inlineStr">
+        <is>
+          <t>24.34배 (PER)</t>
+        </is>
+      </c>
+      <c r="G29" s="6" t="n">
+        <v>16600</v>
       </c>
       <c r="H29" s="6" t="n">
-        <v>1343.8</v>
+        <v>1328.82</v>
       </c>
       <c r="I29" s="6" t="n">
-        <v>2022</v>
+        <v>2309</v>
       </c>
       <c r="J29" s="6" t="inlineStr">
         <is>
-          <t>2026-03-19~03-20</t>
+          <t>2026-03-23~03-24</t>
         </is>
       </c>
       <c r="K29" s="6" t="inlineStr">
         <is>
-          <t>1,403.74</t>
+          <t>1,913.00</t>
         </is>
       </c>
       <c r="L29" s="6" t="inlineStr"/>
       <c r="M29" s="6" t="inlineStr">
         <is>
-          <t>2026-04-01</t>
+          <t>2026-04-02</t>
         </is>
       </c>
       <c r="N29" s="6" t="inlineStr">
         <is>
-          <t>신한</t>
+          <t>NH</t>
         </is>
       </c>
       <c r="O29" s="6" t="inlineStr"/>
       <c r="P29" s="7" t="inlineStr">
         <is>
-          <t>350</t>
+          <t>1,211</t>
         </is>
       </c>
       <c r="Q29" s="6" t="inlineStr">
         <is>
-          <t>3.50%</t>
+          <t>6.00%</t>
         </is>
       </c>
       <c r="R29" s="6" t="inlineStr">
@@ -9481,42 +9481,44 @@
     <row r="30" ht="30" customHeight="1">
       <c r="A30" s="6" t="inlineStr">
         <is>
-          <t>리센스메디컬</t>
-        </is>
-      </c>
-      <c r="B30" s="18" t="inlineStr">
-        <is>
-          <t>수집예정</t>
+          <t>신한스팩17호</t>
+        </is>
+      </c>
+      <c r="B30" s="19" t="inlineStr">
+        <is>
+          <t>해당없음</t>
         </is>
       </c>
       <c r="C30" s="6" t="inlineStr">
         <is>
-          <t>9,000~11,000</t>
+          <t>2,000</t>
         </is>
       </c>
       <c r="D30" s="7" t="inlineStr">
         <is>
-          <t>1,400,000</t>
+          <t>5,000,000</t>
         </is>
       </c>
       <c r="E30" s="7" t="inlineStr">
         <is>
-          <t>15,400</t>
-        </is>
-      </c>
-      <c r="F30" s="6" t="inlineStr">
-        <is>
-          <t>31.33배 (PER)</t>
-        </is>
-      </c>
-      <c r="G30" s="6" t="n">
-        <v>11000</v>
+          <t>10,000</t>
+        </is>
+      </c>
+      <c r="F30" s="19" t="inlineStr">
+        <is>
+          <t>해당없음</t>
+        </is>
+      </c>
+      <c r="G30" s="6" t="inlineStr">
+        <is>
+          <t>2,000</t>
+        </is>
       </c>
       <c r="H30" s="6" t="n">
-        <v>1352.63</v>
+        <v>1343.8</v>
       </c>
       <c r="I30" s="6" t="n">
-        <v>2261</v>
+        <v>2022</v>
       </c>
       <c r="J30" s="6" t="inlineStr">
         <is>
@@ -9525,33 +9527,29 @@
       </c>
       <c r="K30" s="6" t="inlineStr">
         <is>
-          <t>2,097.68</t>
+          <t>1,403.74</t>
         </is>
       </c>
       <c r="L30" s="6" t="inlineStr"/>
       <c r="M30" s="6" t="inlineStr">
         <is>
-          <t>2026-03-31</t>
+          <t>2026-04-01</t>
         </is>
       </c>
       <c r="N30" s="6" t="inlineStr">
         <is>
-          <t>한국</t>
-        </is>
-      </c>
-      <c r="O30" s="6" t="inlineStr">
-        <is>
-          <t>KB</t>
-        </is>
-      </c>
+          <t>신한</t>
+        </is>
+      </c>
+      <c r="O30" s="6" t="inlineStr"/>
       <c r="P30" s="7" t="inlineStr">
         <is>
-          <t>916</t>
+          <t>350</t>
         </is>
       </c>
       <c r="Q30" s="6" t="inlineStr">
         <is>
-          <t>5.77%</t>
+          <t>3.50%</t>
         </is>
       </c>
       <c r="R30" s="6" t="inlineStr">
@@ -9563,75 +9561,77 @@
     <row r="31" ht="30" customHeight="1">
       <c r="A31" s="6" t="inlineStr">
         <is>
-          <t>NH스팩33호</t>
-        </is>
-      </c>
-      <c r="B31" s="19" t="inlineStr">
-        <is>
-          <t>해당없음</t>
+          <t>리센스메디컬</t>
+        </is>
+      </c>
+      <c r="B31" s="18" t="inlineStr">
+        <is>
+          <t>수집예정</t>
         </is>
       </c>
       <c r="C31" s="6" t="inlineStr">
         <is>
-          <t>2,000</t>
+          <t>9,000~11,000</t>
         </is>
       </c>
       <c r="D31" s="7" t="inlineStr">
         <is>
-          <t>6,350,000</t>
+          <t>1,400,000</t>
         </is>
       </c>
       <c r="E31" s="7" t="inlineStr">
         <is>
-          <t>12,700</t>
-        </is>
-      </c>
-      <c r="F31" s="19" t="inlineStr">
-        <is>
-          <t>해당없음</t>
-        </is>
-      </c>
-      <c r="G31" s="6" t="inlineStr">
-        <is>
-          <t>2,000</t>
-        </is>
+          <t>15,400</t>
+        </is>
+      </c>
+      <c r="F31" s="6" t="inlineStr">
+        <is>
+          <t>31.33배 (PER)</t>
+        </is>
+      </c>
+      <c r="G31" s="6" t="n">
+        <v>11000</v>
       </c>
       <c r="H31" s="6" t="n">
-        <v>1228.71</v>
+        <v>1352.63</v>
       </c>
       <c r="I31" s="6" t="n">
-        <v>2058</v>
+        <v>2261</v>
       </c>
       <c r="J31" s="6" t="inlineStr">
         <is>
-          <t>2026-03-17~03-18</t>
+          <t>2026-03-19~03-20</t>
         </is>
       </c>
       <c r="K31" s="6" t="inlineStr">
         <is>
-          <t>569.27</t>
+          <t>2,097.68</t>
         </is>
       </c>
       <c r="L31" s="6" t="inlineStr"/>
       <c r="M31" s="6" t="inlineStr">
         <is>
-          <t>2026-03-27</t>
+          <t>2026-03-31</t>
         </is>
       </c>
       <c r="N31" s="6" t="inlineStr">
         <is>
-          <t>NH</t>
-        </is>
-      </c>
-      <c r="O31" s="6" t="inlineStr"/>
+          <t>한국</t>
+        </is>
+      </c>
+      <c r="O31" s="6" t="inlineStr">
+        <is>
+          <t>KB</t>
+        </is>
+      </c>
       <c r="P31" s="7" t="inlineStr">
         <is>
-          <t>381</t>
+          <t>916</t>
         </is>
       </c>
       <c r="Q31" s="6" t="inlineStr">
         <is>
-          <t>3.00%</t>
+          <t>5.77%</t>
         </is>
       </c>
       <c r="R31" s="6" t="inlineStr">
@@ -9643,73 +9643,75 @@
     <row r="32" ht="30" customHeight="1">
       <c r="A32" s="6" t="inlineStr">
         <is>
-          <t>메쥬</t>
-        </is>
-      </c>
-      <c r="B32" s="18" t="inlineStr">
-        <is>
-          <t>수집예정</t>
+          <t>NH스팩33호</t>
+        </is>
+      </c>
+      <c r="B32" s="19" t="inlineStr">
+        <is>
+          <t>해당없음</t>
         </is>
       </c>
       <c r="C32" s="6" t="inlineStr">
         <is>
-          <t>16,700~21,600</t>
+          <t>2,000</t>
         </is>
       </c>
       <c r="D32" s="7" t="inlineStr">
         <is>
-          <t>1,345,000</t>
+          <t>6,350,000</t>
         </is>
       </c>
       <c r="E32" s="7" t="inlineStr">
         <is>
-          <t>29,052</t>
-        </is>
-      </c>
-      <c r="F32" s="6" t="inlineStr">
-        <is>
-          <t>20.66배 (PER)</t>
-        </is>
-      </c>
-      <c r="G32" s="6" t="n">
-        <v>21600</v>
+          <t>12,700</t>
+        </is>
+      </c>
+      <c r="F32" s="19" t="inlineStr">
+        <is>
+          <t>해당없음</t>
+        </is>
+      </c>
+      <c r="G32" s="6" t="inlineStr">
+        <is>
+          <t>2,000</t>
+        </is>
       </c>
       <c r="H32" s="6" t="n">
-        <v>1108.93</v>
+        <v>1228.71</v>
       </c>
       <c r="I32" s="6" t="n">
-        <v>2320</v>
+        <v>2058</v>
       </c>
       <c r="J32" s="6" t="inlineStr">
         <is>
-          <t>2026-03-16~03-17</t>
+          <t>2026-03-17~03-18</t>
         </is>
       </c>
       <c r="K32" s="6" t="inlineStr">
         <is>
-          <t>2,428.25</t>
+          <t>569.27</t>
         </is>
       </c>
       <c r="L32" s="6" t="inlineStr"/>
       <c r="M32" s="6" t="inlineStr">
         <is>
-          <t>2026-03-26</t>
+          <t>2026-03-27</t>
         </is>
       </c>
       <c r="N32" s="6" t="inlineStr">
         <is>
-          <t>신한</t>
+          <t>NH</t>
         </is>
       </c>
       <c r="O32" s="6" t="inlineStr"/>
       <c r="P32" s="7" t="inlineStr">
         <is>
-          <t>1,496</t>
+          <t>381</t>
         </is>
       </c>
       <c r="Q32" s="6" t="inlineStr">
         <is>
-          <t>5.00%</t>
+          <t>3.00%</t>
         </is>
       </c>
       <c r="R32" s="6" t="inlineStr">
@@ -9721,7 +9723,7 @@
     <row r="33" ht="30" customHeight="1">
       <c r="A33" s="6" t="inlineStr">
         <is>
-          <t>한패스</t>
+          <t>메쥬</t>
         </is>
       </c>
       <c r="B33" s="18" t="inlineStr">
@@ -9731,32 +9733,32 @@
       </c>
       <c r="C33" s="6" t="inlineStr">
         <is>
-          <t>17,000~19,000</t>
+          <t>16,700~21,600</t>
         </is>
       </c>
       <c r="D33" s="7" t="inlineStr">
         <is>
-          <t>1,100,000</t>
+          <t>1,345,000</t>
         </is>
       </c>
       <c r="E33" s="7" t="inlineStr">
         <is>
-          <t>20,900</t>
+          <t>29,052</t>
         </is>
       </c>
       <c r="F33" s="6" t="inlineStr">
         <is>
-          <t>29.09배 (PER)</t>
+          <t>20.66배 (PER)</t>
         </is>
       </c>
       <c r="G33" s="6" t="n">
-        <v>19000</v>
+        <v>21600</v>
       </c>
       <c r="H33" s="6" t="n">
-        <v>1172.59</v>
+        <v>1108.93</v>
       </c>
       <c r="I33" s="6" t="n">
-        <v>2229</v>
+        <v>2320</v>
       </c>
       <c r="J33" s="6" t="inlineStr">
         <is>
@@ -9765,29 +9767,29 @@
       </c>
       <c r="K33" s="6" t="inlineStr">
         <is>
-          <t>1,673.04</t>
+          <t>2,428.25</t>
         </is>
       </c>
       <c r="L33" s="6" t="inlineStr"/>
       <c r="M33" s="6" t="inlineStr">
         <is>
-          <t>2026-03-25</t>
+          <t>2026-03-26</t>
         </is>
       </c>
       <c r="N33" s="6" t="inlineStr">
         <is>
-          <t>한국</t>
+          <t>신한</t>
         </is>
       </c>
       <c r="O33" s="6" t="inlineStr"/>
       <c r="P33" s="7" t="inlineStr">
         <is>
-          <t>753</t>
+          <t>1,496</t>
         </is>
       </c>
       <c r="Q33" s="6" t="inlineStr">
         <is>
-          <t>3.50%</t>
+          <t>5.00%</t>
         </is>
       </c>
       <c r="R33" s="6" t="inlineStr">
@@ -9799,7 +9801,7 @@
     <row r="34" ht="30" customHeight="1">
       <c r="A34" s="6" t="inlineStr">
         <is>
-          <t>아이엠바이오로직스</t>
+          <t>한패스</t>
         </is>
       </c>
       <c r="B34" s="18" t="inlineStr">
@@ -9809,47 +9811,47 @@
       </c>
       <c r="C34" s="6" t="inlineStr">
         <is>
-          <t>19,000~26,000</t>
+          <t>17,000~19,000</t>
         </is>
       </c>
       <c r="D34" s="7" t="inlineStr">
         <is>
-          <t>2,000,000</t>
+          <t>1,100,000</t>
         </is>
       </c>
       <c r="E34" s="7" t="inlineStr">
         <is>
-          <t>52,000</t>
+          <t>20,900</t>
         </is>
       </c>
       <c r="F34" s="6" t="inlineStr">
         <is>
-          <t>21.46배 (PER)</t>
+          <t>29.09배 (PER)</t>
         </is>
       </c>
       <c r="G34" s="6" t="n">
-        <v>26000</v>
+        <v>19000</v>
       </c>
       <c r="H34" s="6" t="n">
-        <v>839.23</v>
+        <v>1172.59</v>
       </c>
       <c r="I34" s="6" t="n">
-        <v>2333</v>
+        <v>2229</v>
       </c>
       <c r="J34" s="6" t="inlineStr">
         <is>
-          <t>2026-03-11~03-12</t>
+          <t>2026-03-16~03-17</t>
         </is>
       </c>
       <c r="K34" s="6" t="inlineStr">
         <is>
-          <t>1,806.00</t>
+          <t>1,673.04</t>
         </is>
       </c>
       <c r="L34" s="6" t="inlineStr"/>
       <c r="M34" s="6" t="inlineStr">
         <is>
-          <t>2026-03-20</t>
+          <t>2026-03-25</t>
         </is>
       </c>
       <c r="N34" s="6" t="inlineStr">
@@ -9860,12 +9862,12 @@
       <c r="O34" s="6" t="inlineStr"/>
       <c r="P34" s="7" t="inlineStr">
         <is>
-          <t>2,650</t>
+          <t>753</t>
         </is>
       </c>
       <c r="Q34" s="6" t="inlineStr">
         <is>
-          <t>5.00%</t>
+          <t>3.50%</t>
         </is>
       </c>
       <c r="R34" s="6" t="inlineStr">
@@ -9877,7 +9879,7 @@
     <row r="35" ht="30" customHeight="1">
       <c r="A35" s="6" t="inlineStr">
         <is>
-          <t>카나프테라퓨틱스</t>
+          <t>아이엠바이오로직스</t>
         </is>
       </c>
       <c r="B35" s="18" t="inlineStr">
@@ -9887,7 +9889,7 @@
       </c>
       <c r="C35" s="6" t="inlineStr">
         <is>
-          <t>16,000~20,000</t>
+          <t>19,000~26,000</t>
         </is>
       </c>
       <c r="D35" s="7" t="inlineStr">
@@ -9897,37 +9899,37 @@
       </c>
       <c r="E35" s="7" t="inlineStr">
         <is>
-          <t>40,000</t>
+          <t>52,000</t>
         </is>
       </c>
       <c r="F35" s="6" t="inlineStr">
         <is>
-          <t>23.59배 (PER)</t>
+          <t>21.46배 (PER)</t>
         </is>
       </c>
       <c r="G35" s="6" t="n">
-        <v>20000</v>
+        <v>26000</v>
       </c>
       <c r="H35" s="6" t="n">
-        <v>962.1</v>
+        <v>839.23</v>
       </c>
       <c r="I35" s="6" t="n">
-        <v>2327</v>
+        <v>2333</v>
       </c>
       <c r="J35" s="6" t="inlineStr">
         <is>
-          <t>2026-03-05~03-06</t>
+          <t>2026-03-11~03-12</t>
         </is>
       </c>
       <c r="K35" s="6" t="inlineStr">
         <is>
-          <t>1,899.29</t>
+          <t>1,806.00</t>
         </is>
       </c>
       <c r="L35" s="6" t="inlineStr"/>
       <c r="M35" s="6" t="inlineStr">
         <is>
-          <t>2026-03-16</t>
+          <t>2026-03-20</t>
         </is>
       </c>
       <c r="N35" s="6" t="inlineStr">
@@ -9938,7 +9940,7 @@
       <c r="O35" s="6" t="inlineStr"/>
       <c r="P35" s="7" t="inlineStr">
         <is>
-          <t>2,050</t>
+          <t>2,650</t>
         </is>
       </c>
       <c r="Q35" s="6" t="inlineStr">
@@ -9955,7 +9957,7 @@
     <row r="36" ht="30" customHeight="1">
       <c r="A36" s="6" t="inlineStr">
         <is>
-          <t>액스비스</t>
+          <t>카나프테라퓨틱스</t>
         </is>
       </c>
       <c r="B36" s="18" t="inlineStr">
@@ -9965,63 +9967,63 @@
       </c>
       <c r="C36" s="6" t="inlineStr">
         <is>
-          <t>10,100~11,500</t>
+          <t>16,000~20,000</t>
         </is>
       </c>
       <c r="D36" s="7" t="inlineStr">
         <is>
-          <t>2,300,000</t>
+          <t>2,000,000</t>
         </is>
       </c>
       <c r="E36" s="7" t="inlineStr">
         <is>
-          <t>26,450</t>
+          <t>40,000</t>
         </is>
       </c>
       <c r="F36" s="6" t="inlineStr">
         <is>
-          <t>27.60배 (PER)</t>
+          <t>23.59배 (PER)</t>
         </is>
       </c>
       <c r="G36" s="6" t="n">
-        <v>11500</v>
+        <v>20000</v>
       </c>
       <c r="H36" s="6" t="n">
-        <v>1124.21</v>
+        <v>962.1</v>
       </c>
       <c r="I36" s="6" t="n">
-        <v>2411</v>
+        <v>2327</v>
       </c>
       <c r="J36" s="6" t="inlineStr">
         <is>
-          <t>2026-02-23~02-24</t>
+          <t>2026-03-05~03-06</t>
         </is>
       </c>
       <c r="K36" s="6" t="inlineStr">
         <is>
-          <t>1,960.87</t>
+          <t>1,899.29</t>
         </is>
       </c>
       <c r="L36" s="6" t="inlineStr"/>
       <c r="M36" s="6" t="inlineStr">
         <is>
-          <t>2026-03-09</t>
+          <t>2026-03-16</t>
         </is>
       </c>
       <c r="N36" s="6" t="inlineStr">
         <is>
-          <t>미래</t>
+          <t>한국</t>
         </is>
       </c>
       <c r="O36" s="6" t="inlineStr"/>
       <c r="P36" s="7" t="inlineStr">
         <is>
-          <t>1,090</t>
+          <t>2,050</t>
         </is>
       </c>
       <c r="Q36" s="6" t="inlineStr">
         <is>
-          <t>4.00%</t>
+          <t>5.00%</t>
         </is>
       </c>
       <c r="R36" s="6" t="inlineStr">
@@ -10033,7 +10035,7 @@
     <row r="37" ht="30" customHeight="1">
       <c r="A37" s="6" t="inlineStr">
         <is>
-          <t>에스팀</t>
+          <t>액스비스</t>
         </is>
       </c>
       <c r="B37" s="18" t="inlineStr">
@@ -10043,32 +10045,32 @@
       </c>
       <c r="C37" s="6" t="inlineStr">
         <is>
-          <t>7,000~8,500</t>
+          <t>10,100~11,500</t>
         </is>
       </c>
       <c r="D37" s="7" t="inlineStr">
         <is>
-          <t>1,800,000</t>
+          <t>2,300,000</t>
         </is>
       </c>
       <c r="E37" s="7" t="inlineStr">
         <is>
-          <t>15,300</t>
+          <t>26,450</t>
         </is>
       </c>
       <c r="F37" s="6" t="inlineStr">
         <is>
-          <t>17.71배 (EV/EBITDA)</t>
+          <t>27.60배 (PER)</t>
         </is>
       </c>
       <c r="G37" s="6" t="n">
-        <v>8500</v>
+        <v>11500</v>
       </c>
       <c r="H37" s="6" t="n">
-        <v>1334.91</v>
+        <v>1124.21</v>
       </c>
       <c r="I37" s="6" t="n">
-        <v>2263</v>
+        <v>2411</v>
       </c>
       <c r="J37" s="6" t="inlineStr">
         <is>
@@ -10077,29 +10079,29 @@
       </c>
       <c r="K37" s="6" t="inlineStr">
         <is>
-          <t>1,334.91</t>
+          <t>1,960.87</t>
         </is>
       </c>
       <c r="L37" s="6" t="inlineStr"/>
       <c r="M37" s="6" t="inlineStr">
         <is>
-          <t>2026-03-06</t>
+          <t>2026-03-09</t>
         </is>
       </c>
       <c r="N37" s="6" t="inlineStr">
         <is>
-          <t>한국</t>
+          <t>미래</t>
         </is>
       </c>
       <c r="O37" s="6" t="inlineStr"/>
       <c r="P37" s="7" t="inlineStr">
         <is>
-          <t>788</t>
+          <t>1,090</t>
         </is>
       </c>
       <c r="Q37" s="6" t="inlineStr">
         <is>
-          <t>5.00%</t>
+          <t>4.00%</t>
         </is>
       </c>
       <c r="R37" s="6" t="inlineStr">
@@ -10111,7 +10113,7 @@
     <row r="38" ht="30" customHeight="1">
       <c r="A38" s="6" t="inlineStr">
         <is>
-          <t>케이뱅크 (유가)</t>
+          <t>에스팀</t>
         </is>
       </c>
       <c r="B38" s="18" t="inlineStr">
@@ -10121,67 +10123,63 @@
       </c>
       <c r="C38" s="6" t="inlineStr">
         <is>
-          <t>8,300~9,500</t>
+          <t>7,000~8,500</t>
         </is>
       </c>
       <c r="D38" s="7" t="inlineStr">
         <is>
-          <t>60,000,000</t>
+          <t>1,800,000</t>
         </is>
       </c>
       <c r="E38" s="7" t="inlineStr">
         <is>
-          <t>498,000</t>
+          <t>15,300</t>
         </is>
       </c>
       <c r="F38" s="6" t="inlineStr">
         <is>
-          <t>1.80배 (PBR)</t>
+          <t>17.71배 (EV/EBITDA)</t>
         </is>
       </c>
       <c r="G38" s="6" t="n">
-        <v>8300</v>
+        <v>8500</v>
       </c>
       <c r="H38" s="6" t="n">
-        <v>198.53</v>
+        <v>1334.91</v>
       </c>
       <c r="I38" s="6" t="n">
-        <v>2007</v>
+        <v>2263</v>
       </c>
       <c r="J38" s="6" t="inlineStr">
         <is>
-          <t>2026-02-20~23</t>
+          <t>2026-02-23~02-24</t>
         </is>
       </c>
       <c r="K38" s="6" t="inlineStr">
         <is>
-          <t>134.59</t>
+          <t>1,334.91</t>
         </is>
       </c>
       <c r="L38" s="6" t="inlineStr"/>
       <c r="M38" s="6" t="inlineStr">
         <is>
-          <t>2026-03-05</t>
+          <t>2026-03-06</t>
         </is>
       </c>
       <c r="N38" s="6" t="inlineStr">
         <is>
-          <t>NH</t>
-        </is>
-      </c>
-      <c r="O38" s="6" t="inlineStr">
-        <is>
-          <t>삼성</t>
-        </is>
-      </c>
+          <t>한국</t>
+        </is>
+      </c>
+      <c r="O38" s="6" t="inlineStr"/>
       <c r="P38" s="7" t="inlineStr">
         <is>
-          <t>5,976</t>
+          <t>788</t>
         </is>
       </c>
       <c r="Q38" s="6" t="inlineStr">
         <is>
-          <t>1.2%</t>
+          <t>5.00%</t>
         </is>
       </c>
       <c r="R38" s="6" t="inlineStr">
@@ -10193,63 +10191,57 @@
     <row r="39" ht="30" customHeight="1">
       <c r="A39" s="6" t="inlineStr">
         <is>
-          <t>세미티에스</t>
-        </is>
-      </c>
-      <c r="B39" s="19" t="inlineStr">
-        <is>
-          <t>해당없음</t>
-        </is>
-      </c>
-      <c r="C39" s="19" t="inlineStr">
-        <is>
-          <t>해당없음</t>
-        </is>
-      </c>
-      <c r="D39" s="19" t="inlineStr">
-        <is>
-          <t>해당없음</t>
-        </is>
-      </c>
-      <c r="E39" s="19" t="inlineStr">
-        <is>
-          <t>해당없음</t>
-        </is>
-      </c>
-      <c r="F39" s="19" t="inlineStr">
-        <is>
-          <t>해당없음</t>
-        </is>
-      </c>
-      <c r="G39" s="19" t="inlineStr">
-        <is>
-          <t>해당없음</t>
-        </is>
-      </c>
-      <c r="H39" s="19" t="inlineStr">
-        <is>
-          <t>해당없음</t>
-        </is>
-      </c>
-      <c r="I39" s="19" t="inlineStr">
-        <is>
-          <t>해당없음</t>
-        </is>
-      </c>
-      <c r="J39" s="19" t="inlineStr">
-        <is>
-          <t>해당없음</t>
-        </is>
-      </c>
-      <c r="K39" s="19" t="inlineStr">
-        <is>
-          <t>해당없음</t>
+          <t>케이뱅크 (유가)</t>
+        </is>
+      </c>
+      <c r="B39" s="18" t="inlineStr">
+        <is>
+          <t>수집예정</t>
+        </is>
+      </c>
+      <c r="C39" s="6" t="inlineStr">
+        <is>
+          <t>8,300~9,500</t>
+        </is>
+      </c>
+      <c r="D39" s="7" t="inlineStr">
+        <is>
+          <t>60,000,000</t>
+        </is>
+      </c>
+      <c r="E39" s="7" t="inlineStr">
+        <is>
+          <t>498,000</t>
+        </is>
+      </c>
+      <c r="F39" s="6" t="inlineStr">
+        <is>
+          <t>1.80배 (PBR)</t>
+        </is>
+      </c>
+      <c r="G39" s="6" t="n">
+        <v>8300</v>
+      </c>
+      <c r="H39" s="6" t="n">
+        <v>198.53</v>
+      </c>
+      <c r="I39" s="6" t="n">
+        <v>2007</v>
+      </c>
+      <c r="J39" s="6" t="inlineStr">
+        <is>
+          <t>2026-02-20~23</t>
+        </is>
+      </c>
+      <c r="K39" s="6" t="inlineStr">
+        <is>
+          <t>134.59</t>
         </is>
       </c>
       <c r="L39" s="6" t="inlineStr"/>
       <c r="M39" s="6" t="inlineStr">
         <is>
-          <t>2026-02-05</t>
+          <t>2026-03-05</t>
         </is>
       </c>
       <c r="N39" s="6" t="inlineStr">
@@ -10257,77 +10249,87 @@
           <t>NH</t>
         </is>
       </c>
-      <c r="O39" s="6" t="inlineStr"/>
-      <c r="P39" s="19" t="inlineStr">
-        <is>
-          <t>해당없음</t>
-        </is>
-      </c>
-      <c r="Q39" s="19" t="inlineStr">
-        <is>
-          <t>해당없음</t>
+      <c r="O39" s="6" t="inlineStr">
+        <is>
+          <t>삼성</t>
+        </is>
+      </c>
+      <c r="P39" s="7" t="inlineStr">
+        <is>
+          <t>5,976</t>
+        </is>
+      </c>
+      <c r="Q39" s="6" t="inlineStr">
+        <is>
+          <t>1.2%</t>
         </is>
       </c>
       <c r="R39" s="6" t="inlineStr">
         <is>
-          <t>상장완료(스팩합병)</t>
+          <t>상장완료</t>
         </is>
       </c>
     </row>
     <row r="40" ht="30" customHeight="1">
       <c r="A40" s="6" t="inlineStr">
         <is>
-          <t>덕양에너젠</t>
-        </is>
-      </c>
-      <c r="B40" s="18" t="inlineStr">
-        <is>
-          <t>수집예정</t>
-        </is>
-      </c>
-      <c r="C40" s="6" t="inlineStr">
-        <is>
-          <t>8,500~10,000</t>
-        </is>
-      </c>
-      <c r="D40" s="7" t="inlineStr">
-        <is>
-          <t>7,500,000</t>
-        </is>
-      </c>
-      <c r="E40" s="7" t="inlineStr">
-        <is>
-          <t>75,000</t>
-        </is>
-      </c>
-      <c r="F40" s="6" t="inlineStr">
-        <is>
-          <t>30.32배 (EV/EBITDA)</t>
-        </is>
-      </c>
-      <c r="G40" s="6" t="n">
-        <v>10000</v>
-      </c>
-      <c r="H40" s="6" t="n">
-        <v>650.14</v>
-      </c>
-      <c r="I40" s="6" t="n">
-        <v>2324</v>
-      </c>
-      <c r="J40" s="6" t="inlineStr">
-        <is>
-          <t>2026-01-20~01-21</t>
-        </is>
-      </c>
-      <c r="K40" s="6" t="inlineStr">
-        <is>
-          <t>1,354.00</t>
+          <t>세미티에스</t>
+        </is>
+      </c>
+      <c r="B40" s="19" t="inlineStr">
+        <is>
+          <t>해당없음</t>
+        </is>
+      </c>
+      <c r="C40" s="19" t="inlineStr">
+        <is>
+          <t>해당없음</t>
+        </is>
+      </c>
+      <c r="D40" s="19" t="inlineStr">
+        <is>
+          <t>해당없음</t>
+        </is>
+      </c>
+      <c r="E40" s="19" t="inlineStr">
+        <is>
+          <t>해당없음</t>
+        </is>
+      </c>
+      <c r="F40" s="19" t="inlineStr">
+        <is>
+          <t>해당없음</t>
+        </is>
+      </c>
+      <c r="G40" s="19" t="inlineStr">
+        <is>
+          <t>해당없음</t>
+        </is>
+      </c>
+      <c r="H40" s="19" t="inlineStr">
+        <is>
+          <t>해당없음</t>
+        </is>
+      </c>
+      <c r="I40" s="19" t="inlineStr">
+        <is>
+          <t>해당없음</t>
+        </is>
+      </c>
+      <c r="J40" s="19" t="inlineStr">
+        <is>
+          <t>해당없음</t>
+        </is>
+      </c>
+      <c r="K40" s="19" t="inlineStr">
+        <is>
+          <t>해당없음</t>
         </is>
       </c>
       <c r="L40" s="6" t="inlineStr"/>
       <c r="M40" s="6" t="inlineStr">
         <is>
-          <t>2026-01-30</t>
+          <t>2026-02-05</t>
         </is>
       </c>
       <c r="N40" s="6" t="inlineStr">
@@ -10335,87 +10337,77 @@
           <t>NH</t>
         </is>
       </c>
-      <c r="O40" s="6" t="inlineStr">
-        <is>
-          <t>미래</t>
-        </is>
-      </c>
-      <c r="P40" s="7" t="inlineStr">
-        <is>
-          <t>2,000</t>
-        </is>
-      </c>
-      <c r="Q40" s="6" t="inlineStr">
-        <is>
-          <t>2.92%</t>
+      <c r="O40" s="6" t="inlineStr"/>
+      <c r="P40" s="19" t="inlineStr">
+        <is>
+          <t>해당없음</t>
+        </is>
+      </c>
+      <c r="Q40" s="19" t="inlineStr">
+        <is>
+          <t>해당없음</t>
         </is>
       </c>
       <c r="R40" s="6" t="inlineStr">
         <is>
-          <t>상장완료</t>
+          <t>상장완료(스팩합병)</t>
         </is>
       </c>
     </row>
     <row r="41" ht="30" customHeight="1">
       <c r="A41" s="6" t="inlineStr">
         <is>
-          <t>케이피항공산업</t>
-        </is>
-      </c>
-      <c r="B41" s="19" t="inlineStr">
-        <is>
-          <t>해당없음</t>
-        </is>
-      </c>
-      <c r="C41" s="19" t="inlineStr">
-        <is>
-          <t>해당없음</t>
-        </is>
-      </c>
-      <c r="D41" s="19" t="inlineStr">
-        <is>
-          <t>해당없음</t>
-        </is>
-      </c>
-      <c r="E41" s="19" t="inlineStr">
-        <is>
-          <t>해당없음</t>
-        </is>
-      </c>
-      <c r="F41" s="19" t="inlineStr">
-        <is>
-          <t>해당없음</t>
-        </is>
-      </c>
-      <c r="G41" s="19" t="inlineStr">
-        <is>
-          <t>해당없음</t>
-        </is>
-      </c>
-      <c r="H41" s="19" t="inlineStr">
-        <is>
-          <t>해당없음</t>
-        </is>
-      </c>
-      <c r="I41" s="19" t="inlineStr">
-        <is>
-          <t>해당없음</t>
-        </is>
-      </c>
-      <c r="J41" s="19" t="inlineStr">
-        <is>
-          <t>해당없음</t>
-        </is>
-      </c>
-      <c r="K41" s="19" t="inlineStr">
-        <is>
-          <t>해당없음</t>
+          <t>덕양에너젠</t>
+        </is>
+      </c>
+      <c r="B41" s="18" t="inlineStr">
+        <is>
+          <t>수집예정</t>
+        </is>
+      </c>
+      <c r="C41" s="6" t="inlineStr">
+        <is>
+          <t>8,500~10,000</t>
+        </is>
+      </c>
+      <c r="D41" s="7" t="inlineStr">
+        <is>
+          <t>7,500,000</t>
+        </is>
+      </c>
+      <c r="E41" s="7" t="inlineStr">
+        <is>
+          <t>75,000</t>
+        </is>
+      </c>
+      <c r="F41" s="6" t="inlineStr">
+        <is>
+          <t>30.32배 (EV/EBITDA)</t>
+        </is>
+      </c>
+      <c r="G41" s="6" t="n">
+        <v>10000</v>
+      </c>
+      <c r="H41" s="6" t="n">
+        <v>650.14</v>
+      </c>
+      <c r="I41" s="6" t="n">
+        <v>2324</v>
+      </c>
+      <c r="J41" s="6" t="inlineStr">
+        <is>
+          <t>2026-01-20~01-21</t>
+        </is>
+      </c>
+      <c r="K41" s="6" t="inlineStr">
+        <is>
+          <t>1,354.00</t>
         </is>
       </c>
       <c r="L41" s="6" t="inlineStr"/>
       <c r="M41" s="6" t="inlineStr">
         <is>
-          <t>2026-01-29</t>
+          <t>2026-01-30</t>
         </is>
       </c>
       <c r="N41" s="6" t="inlineStr">
@@ -10423,27 +10415,31 @@
           <t>NH</t>
         </is>
       </c>
-      <c r="O41" s="6" t="inlineStr"/>
-      <c r="P41" s="19" t="inlineStr">
-        <is>
-          <t>해당없음</t>
-        </is>
-      </c>
-      <c r="Q41" s="19" t="inlineStr">
-        <is>
-          <t>해당없음</t>
+      <c r="O41" s="6" t="inlineStr">
+        <is>
+          <t>미래</t>
+        </is>
+      </c>
+      <c r="P41" s="7" t="inlineStr">
+        <is>
+          <t>2,000</t>
+        </is>
+      </c>
+      <c r="Q41" s="6" t="inlineStr">
+        <is>
+          <t>2.92%</t>
         </is>
       </c>
       <c r="R41" s="6" t="inlineStr">
         <is>
-          <t>상장완료(스팩합병)</t>
+          <t>상장완료</t>
         </is>
       </c>
     </row>
     <row r="42" ht="30" customHeight="1">
       <c r="A42" s="6" t="inlineStr">
         <is>
-          <t>삼성스팩13호</t>
+          <t>케이피항공산업</t>
         </is>
       </c>
       <c r="B42" s="19" t="inlineStr">
@@ -10451,19 +10447,19 @@
           <t>해당없음</t>
         </is>
       </c>
-      <c r="C42" s="6" t="inlineStr">
-        <is>
-          <t>2,000</t>
-        </is>
-      </c>
-      <c r="D42" s="7" t="inlineStr">
-        <is>
-          <t>6,000,000</t>
-        </is>
-      </c>
-      <c r="E42" s="7" t="inlineStr">
-        <is>
-          <t>12,000</t>
+      <c r="C42" s="19" t="inlineStr">
+        <is>
+          <t>해당없음</t>
+        </is>
+      </c>
+      <c r="D42" s="19" t="inlineStr">
+        <is>
+          <t>해당없음</t>
+        </is>
+      </c>
+      <c r="E42" s="19" t="inlineStr">
+        <is>
+          <t>해당없음</t>
         </is>
       </c>
       <c r="F42" s="19" t="inlineStr">
@@ -10471,150 +10467,162 @@
           <t>해당없음</t>
         </is>
       </c>
-      <c r="G42" s="6" t="inlineStr">
-        <is>
-          <t>2,000</t>
-        </is>
-      </c>
-      <c r="H42" s="6" t="n">
-        <v>1159.11</v>
-      </c>
-      <c r="I42" s="6" t="n">
-        <v>1892</v>
-      </c>
-      <c r="J42" s="6" t="inlineStr">
-        <is>
-          <t>2026-01-12~01-13</t>
-        </is>
-      </c>
-      <c r="K42" s="6" t="inlineStr">
-        <is>
-          <t>1,870.40</t>
+      <c r="G42" s="19" t="inlineStr">
+        <is>
+          <t>해당없음</t>
+        </is>
+      </c>
+      <c r="H42" s="19" t="inlineStr">
+        <is>
+          <t>해당없음</t>
+        </is>
+      </c>
+      <c r="I42" s="19" t="inlineStr">
+        <is>
+          <t>해당없음</t>
+        </is>
+      </c>
+      <c r="J42" s="19" t="inlineStr">
+        <is>
+          <t>해당없음</t>
+        </is>
+      </c>
+      <c r="K42" s="19" t="inlineStr">
+        <is>
+          <t>해당없음</t>
         </is>
       </c>
       <c r="L42" s="6" t="inlineStr"/>
       <c r="M42" s="6" t="inlineStr">
         <is>
+          <t>2026-01-29</t>
+        </is>
+      </c>
+      <c r="N42" s="6" t="inlineStr">
+        <is>
+          <t>NH</t>
+        </is>
+      </c>
+      <c r="O42" s="6" t="inlineStr"/>
+      <c r="P42" s="19" t="inlineStr">
+        <is>
+          <t>해당없음</t>
+        </is>
+      </c>
+      <c r="Q42" s="19" t="inlineStr">
+        <is>
+          <t>해당없음</t>
+        </is>
+      </c>
+      <c r="R42" s="6" t="inlineStr">
+        <is>
+          <t>상장완료(스팩합병)</t>
+        </is>
+      </c>
+    </row>
+    <row r="43" ht="30" customHeight="1">
+      <c r="A43" s="6" t="inlineStr">
+        <is>
+          <t>삼성스팩13호</t>
+        </is>
+      </c>
+      <c r="B43" s="19" t="inlineStr">
+        <is>
+          <t>해당없음</t>
+        </is>
+      </c>
+      <c r="C43" s="6" t="inlineStr">
+        <is>
+          <t>2,000</t>
+        </is>
+      </c>
+      <c r="D43" s="7" t="inlineStr">
+        <is>
+          <t>6,000,000</t>
+        </is>
+      </c>
+      <c r="E43" s="7" t="inlineStr">
+        <is>
+          <t>12,000</t>
+        </is>
+      </c>
+      <c r="F43" s="19" t="inlineStr">
+        <is>
+          <t>해당없음</t>
+        </is>
+      </c>
+      <c r="G43" s="6" t="inlineStr">
+        <is>
+          <t>2,000</t>
+        </is>
+      </c>
+      <c r="H43" s="6" t="n">
+        <v>1159.11</v>
+      </c>
+      <c r="I43" s="6" t="n">
+        <v>1892</v>
+      </c>
+      <c r="J43" s="6" t="inlineStr">
+        <is>
+          <t>2026-01-12~01-13</t>
+        </is>
+      </c>
+      <c r="K43" s="6" t="inlineStr">
+        <is>
+          <t>1,870.40</t>
+        </is>
+      </c>
+      <c r="L43" s="6" t="inlineStr"/>
+      <c r="M43" s="6" t="inlineStr">
+        <is>
           <t>2026-01-21</t>
         </is>
       </c>
-      <c r="N42" s="6" t="inlineStr">
+      <c r="N43" s="6" t="inlineStr">
         <is>
           <t>삼성</t>
         </is>
       </c>
-      <c r="O42" s="6" t="inlineStr"/>
-      <c r="P42" s="7" t="inlineStr">
+      <c r="O43" s="6" t="inlineStr"/>
+      <c r="P43" s="7" t="inlineStr">
         <is>
           <t>360</t>
         </is>
       </c>
-      <c r="Q42" s="6" t="inlineStr">
+      <c r="Q43" s="6" t="inlineStr">
         <is>
           <t>3.00%</t>
         </is>
       </c>
-      <c r="R42" s="6" t="inlineStr">
+      <c r="R43" s="6" t="inlineStr">
         <is>
           <t>상장완료</t>
         </is>
       </c>
     </row>
-    <row r="44" ht="22" customHeight="1">
-      <c r="A44" s="3" t="inlineStr">
-        <is>
-          <t>■ 공모 진행 (예심 승인법인)  (24건)</t>
-        </is>
-      </c>
-      <c r="B44" s="4" t="n"/>
-      <c r="C44" s="4" t="n"/>
-      <c r="D44" s="4" t="n"/>
-      <c r="E44" s="4" t="n"/>
-      <c r="F44" s="4" t="n"/>
-      <c r="G44" s="4" t="n"/>
-      <c r="H44" s="4" t="n"/>
-      <c r="I44" s="4" t="n"/>
-      <c r="J44" s="4" t="n"/>
-      <c r="K44" s="4" t="n"/>
-      <c r="L44" s="4" t="n"/>
-      <c r="M44" s="4" t="n"/>
-      <c r="N44" s="4" t="n"/>
-      <c r="O44" s="4" t="n"/>
-      <c r="P44" s="4" t="n"/>
-      <c r="Q44" s="4" t="n"/>
-      <c r="R44" s="4" t="n"/>
-    </row>
-    <row r="45" ht="30" customHeight="1">
-      <c r="A45" s="6" t="inlineStr">
-        <is>
-          <t>니어스랩</t>
-        </is>
-      </c>
-      <c r="B45" s="6" t="inlineStr">
-        <is>
-          <t>08-03~08-07</t>
-        </is>
-      </c>
-      <c r="C45" s="6" t="inlineStr">
-        <is>
-          <t>30,000~41,200</t>
-        </is>
-      </c>
-      <c r="D45" s="7" t="inlineStr">
-        <is>
-          <t>910,000</t>
-        </is>
-      </c>
-      <c r="E45" s="7" t="inlineStr">
-        <is>
-          <t>37,492,000,000</t>
-        </is>
-      </c>
-      <c r="F45" s="6" t="inlineStr">
-        <is>
-          <t>44.41배 (PER)</t>
-        </is>
-      </c>
-      <c r="G45" s="6" t="inlineStr">
-        <is>
-          <t>41,200</t>
-        </is>
-      </c>
-      <c r="H45" s="6" t="n">
-        <v>743.49</v>
-      </c>
-      <c r="I45" s="6" t="n">
-        <v>1795</v>
-      </c>
-      <c r="J45" s="6" t="inlineStr">
-        <is>
-          <t>08-12~08-13</t>
-        </is>
-      </c>
-      <c r="K45" s="6" t="inlineStr"/>
-      <c r="L45" s="6" t="inlineStr"/>
-      <c r="M45" s="6" t="inlineStr"/>
-      <c r="N45" s="6" t="inlineStr">
-        <is>
-          <t>삼성증권</t>
-        </is>
-      </c>
-      <c r="O45" s="6" t="inlineStr"/>
-      <c r="P45" s="7" t="inlineStr">
-        <is>
-          <t>1,265,355,000</t>
-        </is>
-      </c>
-      <c r="Q45" s="6" t="inlineStr">
-        <is>
-          <t>4.50%</t>
-        </is>
-      </c>
-      <c r="R45" s="6" t="inlineStr">
-        <is>
-          <t>청약완료·상장대기</t>
-        </is>
-      </c>
+    <row r="45" ht="22" customHeight="1">
+      <c r="A45" s="3" t="inlineStr">
+        <is>
+          <t>■ 공모 진행 (예심 승인법인)  (23건)</t>
+        </is>
+      </c>
+      <c r="B45" s="4" t="n"/>
+      <c r="C45" s="4" t="n"/>
+      <c r="D45" s="4" t="n"/>
+      <c r="E45" s="4" t="n"/>
+      <c r="F45" s="4" t="n"/>
+      <c r="G45" s="4" t="n"/>
+      <c r="H45" s="4" t="n"/>
+      <c r="I45" s="4" t="n"/>
+      <c r="J45" s="4" t="n"/>
+      <c r="K45" s="4" t="n"/>
+      <c r="L45" s="4" t="n"/>
+      <c r="M45" s="4" t="n"/>
+      <c r="N45" s="4" t="n"/>
+      <c r="O45" s="4" t="n"/>
+      <c r="P45" s="4" t="n"/>
+      <c r="Q45" s="4" t="n"/>
+      <c r="R45" s="4" t="n"/>
     </row>
     <row r="46" ht="30" customHeight="1">
       <c r="A46" s="6" t="inlineStr">
@@ -12382,7 +12390,7 @@
         <v>0</v>
       </c>
       <c r="E13" s="6" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="F13" s="21">
         <f>IF((C13+D13)=0,"-",C13/(C13+D13))</f>
@@ -12449,11 +12457,11 @@
         </is>
       </c>
       <c r="B18" s="6" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="C18" s="6" t="inlineStr">
         <is>
-          <t>157,492,000,000</t>
+          <t>194,984,000,000</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore: update IPO data 2026-08-26
</commit_message>
<xml_diff>
--- a/IPO_analysis.xlsx
+++ b/IPO_analysis.xlsx
@@ -618,7 +618,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>기준일 2026-08-25 · 청구일 직전 사업연도 · 별도/개별 재무제표 · 단위 백만원(별도 표기 시 USD)</t>
+          <t>기준일 2026-08-26 · 청구일 직전 사업연도 · 별도/개별 재무제표 · 단위 백만원(별도 표기 시 USD)</t>
         </is>
       </c>
     </row>
@@ -756,7 +756,7 @@
     <row r="7">
       <c r="A7" s="6" t="inlineStr">
         <is>
-          <t>2026-08-21</t>
+          <t>2026-08-25</t>
         </is>
       </c>
       <c r="B7" s="6" t="inlineStr">
@@ -796,7 +796,7 @@
       </c>
       <c r="I7" s="6" t="inlineStr">
         <is>
-          <t>금융 지원 서비스업</t>
+          <t>기타 금융업</t>
         </is>
       </c>
       <c r="J7" s="6" t="inlineStr">
@@ -11726,12 +11726,12 @@
     <row r="60" ht="30" customHeight="1">
       <c r="A60" s="6" t="inlineStr">
         <is>
-          <t>엠에스바이오</t>
-        </is>
-      </c>
-      <c r="B60" s="18" t="inlineStr">
-        <is>
-          <t>수집예정</t>
+          <t>에스케이증권제14호기업인수목적</t>
+        </is>
+      </c>
+      <c r="B60" s="6" t="inlineStr">
+        <is>
+          <t>10-12~10-13</t>
         </is>
       </c>
       <c r="C60" s="18" t="inlineStr">
@@ -11739,14 +11739,14 @@
           <t>수집예정</t>
         </is>
       </c>
-      <c r="D60" s="18" t="inlineStr">
-        <is>
-          <t>수집예정</t>
-        </is>
-      </c>
-      <c r="E60" s="18" t="inlineStr">
-        <is>
-          <t>수집예정</t>
+      <c r="D60" s="7" t="inlineStr">
+        <is>
+          <t>6,500,000</t>
+        </is>
+      </c>
+      <c r="E60" s="7" t="inlineStr">
+        <is>
+          <t>13,000,000,000</t>
         </is>
       </c>
       <c r="F60" s="18" t="inlineStr">
@@ -11757,9 +11757,9 @@
       <c r="G60" s="6" t="inlineStr"/>
       <c r="H60" s="6" t="inlineStr"/>
       <c r="I60" s="6" t="inlineStr"/>
-      <c r="J60" s="18" t="inlineStr">
-        <is>
-          <t>수집예정</t>
+      <c r="J60" s="6" t="inlineStr">
+        <is>
+          <t>10-15~10-16</t>
         </is>
       </c>
       <c r="K60" s="6" t="inlineStr"/>
@@ -11776,21 +11776,21 @@
           <t>수집예정</t>
         </is>
       </c>
-      <c r="Q60" s="18" t="inlineStr">
-        <is>
-          <t>수집예정</t>
+      <c r="Q60" s="6" t="inlineStr">
+        <is>
+          <t>50%</t>
         </is>
       </c>
       <c r="R60" s="6" t="inlineStr">
         <is>
-          <t>신고서 대기</t>
+          <t>최초</t>
         </is>
       </c>
     </row>
     <row r="61" ht="30" customHeight="1">
       <c r="A61" s="6" t="inlineStr">
         <is>
-          <t>디티에스</t>
+          <t>엠에스바이오</t>
         </is>
       </c>
       <c r="B61" s="18" t="inlineStr">
@@ -11854,7 +11854,7 @@
     <row r="62" ht="30" customHeight="1">
       <c r="A62" s="6" t="inlineStr">
         <is>
-          <t>에스케이증권제14호기업인수목적</t>
+          <t>디티에스</t>
         </is>
       </c>
       <c r="B62" s="18" t="inlineStr">
@@ -12632,7 +12632,7 @@
         </is>
       </c>
       <c r="B13" s="6" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="C13" s="6" t="n">
         <v>6</v>

</xml_diff>

<commit_message>
chore: update IPO data 2026-08-27
</commit_message>
<xml_diff>
--- a/IPO_analysis.xlsx
+++ b/IPO_analysis.xlsx
@@ -618,7 +618,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>기준일 2026-08-26 · 청구일 직전 사업연도 · 별도/개별 재무제표 · 단위 백만원(별도 표기 시 USD)</t>
+          <t>기준일 2026-08-27 · 청구일 직전 사업연도 · 별도/개별 재무제표 · 단위 백만원(별도 표기 시 USD)</t>
         </is>
       </c>
     </row>
@@ -11091,14 +11091,14 @@
           <t>수집예정</t>
         </is>
       </c>
-      <c r="D50" s="18" t="inlineStr">
-        <is>
-          <t>수집예정</t>
-        </is>
-      </c>
-      <c r="E50" s="18" t="inlineStr">
-        <is>
-          <t>수집예정</t>
+      <c r="D50" s="7" t="inlineStr">
+        <is>
+          <t>7,000,000</t>
+        </is>
+      </c>
+      <c r="E50" s="7" t="inlineStr">
+        <is>
+          <t>14,000,000,000</t>
         </is>
       </c>
       <c r="F50" s="18" t="inlineStr">
@@ -11221,12 +11221,12 @@
       </c>
       <c r="D52" s="7" t="inlineStr">
         <is>
-          <t>2,000,000</t>
+          <t>1,600,000</t>
         </is>
       </c>
       <c r="E52" s="7" t="inlineStr">
         <is>
-          <t>40,000,000,000</t>
+          <t>24,000,000,000</t>
         </is>
       </c>
       <c r="F52" s="6" t="inlineStr">
@@ -11363,7 +11363,7 @@
       </c>
       <c r="F54" s="6" t="inlineStr">
         <is>
-          <t>34.08배 (PER)</t>
+          <t>32.57배 (PER)</t>
         </is>
       </c>
       <c r="G54" s="6" t="inlineStr"/>
@@ -11415,14 +11415,14 @@
           <t>수집예정</t>
         </is>
       </c>
-      <c r="D55" s="18" t="inlineStr">
-        <is>
-          <t>수집예정</t>
-        </is>
-      </c>
-      <c r="E55" s="18" t="inlineStr">
-        <is>
-          <t>수집예정</t>
+      <c r="D55" s="7" t="inlineStr">
+        <is>
+          <t>8,500,000</t>
+        </is>
+      </c>
+      <c r="E55" s="7" t="inlineStr">
+        <is>
+          <t>17,000,000,000</t>
         </is>
       </c>
       <c r="F55" s="18" t="inlineStr">
@@ -11543,14 +11543,14 @@
           <t>70,400~90,500</t>
         </is>
       </c>
-      <c r="D57" s="18" t="inlineStr">
-        <is>
-          <t>수집예정</t>
-        </is>
-      </c>
-      <c r="E57" s="18" t="inlineStr">
-        <is>
-          <t>수집예정</t>
+      <c r="D57" s="7" t="inlineStr">
+        <is>
+          <t>2,222,000</t>
+        </is>
+      </c>
+      <c r="E57" s="7" t="inlineStr">
+        <is>
+          <t>156,428,800,000</t>
         </is>
       </c>
       <c r="F57" s="6" t="inlineStr">
@@ -11611,14 +11611,14 @@
           <t>10,700~12,300</t>
         </is>
       </c>
-      <c r="D58" s="18" t="inlineStr">
-        <is>
-          <t>수집예정</t>
-        </is>
-      </c>
-      <c r="E58" s="18" t="inlineStr">
-        <is>
-          <t>수집예정</t>
+      <c r="D58" s="7" t="inlineStr">
+        <is>
+          <t>2,500,000</t>
+        </is>
+      </c>
+      <c r="E58" s="7" t="inlineStr">
+        <is>
+          <t>26,750,000,000</t>
         </is>
       </c>
       <c r="F58" s="6" t="inlineStr">
@@ -11662,32 +11662,32 @@
     <row r="59" ht="30" customHeight="1">
       <c r="A59" s="6" t="inlineStr">
         <is>
-          <t>래블업</t>
+          <t>진코스텍</t>
         </is>
       </c>
       <c r="B59" s="6" t="inlineStr">
         <is>
-          <t>09-28~10-02</t>
+          <t>09-16~09-22</t>
         </is>
       </c>
       <c r="C59" s="6" t="inlineStr">
         <is>
-          <t>20,000~23,000</t>
-        </is>
-      </c>
-      <c r="D59" s="18" t="inlineStr">
-        <is>
-          <t>수집예정</t>
-        </is>
-      </c>
-      <c r="E59" s="18" t="inlineStr">
-        <is>
-          <t>수집예정</t>
+          <t>19,500~23,500</t>
+        </is>
+      </c>
+      <c r="D59" s="7" t="inlineStr">
+        <is>
+          <t>852,000</t>
+        </is>
+      </c>
+      <c r="E59" s="7" t="inlineStr">
+        <is>
+          <t>16,614,000,000</t>
         </is>
       </c>
       <c r="F59" s="6" t="inlineStr">
         <is>
-          <t>33.6배 (PER)</t>
+          <t>17.61배 (PER)</t>
         </is>
       </c>
       <c r="G59" s="6" t="inlineStr"/>
@@ -11695,7 +11695,7 @@
       <c r="I59" s="6" t="inlineStr"/>
       <c r="J59" s="6" t="inlineStr">
         <is>
-          <t>10-12~10-13</t>
+          <t>10-02~10-06</t>
         </is>
       </c>
       <c r="K59" s="6" t="inlineStr"/>
@@ -11703,18 +11703,18 @@
       <c r="M59" s="6" t="inlineStr"/>
       <c r="N59" s="6" t="inlineStr">
         <is>
-          <t>NH투자증권</t>
+          <t>하나증권</t>
         </is>
       </c>
       <c r="O59" s="6" t="inlineStr"/>
       <c r="P59" s="7" t="inlineStr">
         <is>
-          <t>2,007,000,000</t>
+          <t>697,788,000</t>
         </is>
       </c>
       <c r="Q59" s="6" t="inlineStr">
         <is>
-          <t>4.5%</t>
+          <t>4.0%</t>
         </is>
       </c>
       <c r="R59" s="6" t="inlineStr">
@@ -11726,32 +11726,32 @@
     <row r="60" ht="30" customHeight="1">
       <c r="A60" s="6" t="inlineStr">
         <is>
-          <t>에스케이증권제14호기업인수목적</t>
+          <t>래블업</t>
         </is>
       </c>
       <c r="B60" s="6" t="inlineStr">
         <is>
-          <t>10-12~10-13</t>
-        </is>
-      </c>
-      <c r="C60" s="18" t="inlineStr">
-        <is>
-          <t>수집예정</t>
+          <t>09-28~10-02</t>
+        </is>
+      </c>
+      <c r="C60" s="6" t="inlineStr">
+        <is>
+          <t>20,000~23,000</t>
         </is>
       </c>
       <c r="D60" s="7" t="inlineStr">
         <is>
-          <t>6,500,000</t>
+          <t>2,180,000</t>
         </is>
       </c>
       <c r="E60" s="7" t="inlineStr">
         <is>
-          <t>13,000,000,000</t>
-        </is>
-      </c>
-      <c r="F60" s="18" t="inlineStr">
-        <is>
-          <t>수집예정</t>
+          <t>43,600,000,000</t>
+        </is>
+      </c>
+      <c r="F60" s="6" t="inlineStr">
+        <is>
+          <t>33.6배 (PER)</t>
         </is>
       </c>
       <c r="G60" s="6" t="inlineStr"/>
@@ -11759,26 +11759,26 @@
       <c r="I60" s="6" t="inlineStr"/>
       <c r="J60" s="6" t="inlineStr">
         <is>
-          <t>10-15~10-16</t>
+          <t>10-12~10-13</t>
         </is>
       </c>
       <c r="K60" s="6" t="inlineStr"/>
       <c r="L60" s="6" t="inlineStr"/>
       <c r="M60" s="6" t="inlineStr"/>
-      <c r="N60" s="18" t="inlineStr">
-        <is>
-          <t>수집예정</t>
+      <c r="N60" s="6" t="inlineStr">
+        <is>
+          <t>NH투자증권</t>
         </is>
       </c>
       <c r="O60" s="6" t="inlineStr"/>
-      <c r="P60" s="18" t="inlineStr">
-        <is>
-          <t>수집예정</t>
+      <c r="P60" s="7" t="inlineStr">
+        <is>
+          <t>2,007,000,000</t>
         </is>
       </c>
       <c r="Q60" s="6" t="inlineStr">
         <is>
-          <t>50%</t>
+          <t>4.5%</t>
         </is>
       </c>
       <c r="R60" s="6" t="inlineStr">
@@ -11790,27 +11790,27 @@
     <row r="61" ht="30" customHeight="1">
       <c r="A61" s="6" t="inlineStr">
         <is>
-          <t>엠에스바이오</t>
-        </is>
-      </c>
-      <c r="B61" s="18" t="inlineStr">
+          <t>에스케이증권제14호기업인수목적</t>
+        </is>
+      </c>
+      <c r="B61" s="6" t="inlineStr">
+        <is>
+          <t>10-12~10-13</t>
+        </is>
+      </c>
+      <c r="C61" s="18" t="inlineStr">
         <is>
           <t>수집예정</t>
         </is>
       </c>
-      <c r="C61" s="18" t="inlineStr">
-        <is>
-          <t>수집예정</t>
-        </is>
-      </c>
-      <c r="D61" s="18" t="inlineStr">
-        <is>
-          <t>수집예정</t>
-        </is>
-      </c>
-      <c r="E61" s="18" t="inlineStr">
-        <is>
-          <t>수집예정</t>
+      <c r="D61" s="7" t="inlineStr">
+        <is>
+          <t>6,500,000</t>
+        </is>
+      </c>
+      <c r="E61" s="7" t="inlineStr">
+        <is>
+          <t>13,000,000,000</t>
         </is>
       </c>
       <c r="F61" s="18" t="inlineStr">
@@ -11821,9 +11821,9 @@
       <c r="G61" s="6" t="inlineStr"/>
       <c r="H61" s="6" t="inlineStr"/>
       <c r="I61" s="6" t="inlineStr"/>
-      <c r="J61" s="18" t="inlineStr">
-        <is>
-          <t>수집예정</t>
+      <c r="J61" s="6" t="inlineStr">
+        <is>
+          <t>10-15~10-16</t>
         </is>
       </c>
       <c r="K61" s="6" t="inlineStr"/>
@@ -11840,21 +11840,21 @@
           <t>수집예정</t>
         </is>
       </c>
-      <c r="Q61" s="18" t="inlineStr">
-        <is>
-          <t>수집예정</t>
+      <c r="Q61" s="6" t="inlineStr">
+        <is>
+          <t>50%</t>
         </is>
       </c>
       <c r="R61" s="6" t="inlineStr">
         <is>
-          <t>신고서 대기</t>
+          <t>최초</t>
         </is>
       </c>
     </row>
     <row r="62" ht="30" customHeight="1">
       <c r="A62" s="6" t="inlineStr">
         <is>
-          <t>디티에스</t>
+          <t>엠에스바이오</t>
         </is>
       </c>
       <c r="B62" s="18" t="inlineStr">
@@ -11918,7 +11918,7 @@
     <row r="63" ht="30" customHeight="1">
       <c r="A63" s="6" t="inlineStr">
         <is>
-          <t>한화플러스제6호스팩</t>
+          <t>디티에스</t>
         </is>
       </c>
       <c r="B63" s="18" t="inlineStr">
@@ -11982,7 +11982,7 @@
     <row r="64" ht="30" customHeight="1">
       <c r="A64" s="6" t="inlineStr">
         <is>
-          <t>엠비디</t>
+          <t>한화플러스제6호스팩</t>
         </is>
       </c>
       <c r="B64" s="18" t="inlineStr">
@@ -12046,7 +12046,7 @@
     <row r="65" ht="30" customHeight="1">
       <c r="A65" s="6" t="inlineStr">
         <is>
-          <t>진코스텍</t>
+          <t>엠비디</t>
         </is>
       </c>
       <c r="B65" s="18" t="inlineStr">
@@ -12395,7 +12395,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F37"/>
+  <dimension ref="A1:F38"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -12719,52 +12719,52 @@
     <row r="19">
       <c r="A19" s="6" t="inlineStr">
         <is>
-          <t>KB</t>
+          <t>미래에셋증권㈜</t>
         </is>
       </c>
       <c r="B19" s="6" t="n">
-        <v>7</v>
+        <v>1</v>
       </c>
       <c r="C19" s="6" t="inlineStr">
         <is>
-          <t>135,135,239,540</t>
+          <t>156,428,800,000</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="6" t="inlineStr">
         <is>
-          <t>한국투자증권</t>
+          <t>KB</t>
         </is>
       </c>
       <c r="B20" s="6" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="C20" s="6" t="inlineStr">
         <is>
-          <t>102,800,000,000</t>
+          <t>135,135,239,540</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="6" t="inlineStr">
         <is>
-          <t>미래에셋증권</t>
+          <t>대신증권</t>
         </is>
       </c>
       <c r="B21" s="6" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="C21" s="6" t="inlineStr">
         <is>
-          <t>96,560,000,000</t>
+          <t>107,550,000,000</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="6" t="inlineStr">
         <is>
-          <t>대신증권</t>
+          <t>한국투자증권</t>
         </is>
       </c>
       <c r="B22" s="6" t="n">
@@ -12772,179 +12772,179 @@
       </c>
       <c r="C22" s="6" t="inlineStr">
         <is>
-          <t>80,800,000,000</t>
+          <t>102,800,000,000</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="6" t="inlineStr">
         <is>
-          <t>아이비케이투자증권</t>
+          <t>미래에셋증권</t>
         </is>
       </c>
       <c r="B23" s="6" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="C23" s="6" t="inlineStr">
         <is>
-          <t>72,600,000,000</t>
+          <t>96,560,000,000</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="6" t="inlineStr">
         <is>
-          <t>DB증권</t>
+          <t>아이비케이투자증권</t>
         </is>
       </c>
       <c r="B24" s="6" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C24" s="6" t="inlineStr">
         <is>
-          <t>46,000,000,000</t>
+          <t>72,600,000,000</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="6" t="inlineStr">
         <is>
-          <t>유진투자증권</t>
+          <t>DB증권</t>
         </is>
       </c>
       <c r="B25" s="6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C25" s="6" t="inlineStr">
         <is>
-          <t>40,000,000,000</t>
+          <t>46,000,000,000</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="6" t="inlineStr">
         <is>
-          <t>NH</t>
+          <t>NH투자증권</t>
         </is>
       </c>
       <c r="B26" s="6" t="n">
-        <v>7</v>
+        <v>1</v>
       </c>
       <c r="C26" s="6" t="inlineStr">
         <is>
-          <t>618,288</t>
+          <t>43,600,000,000</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="6" t="inlineStr">
         <is>
-          <t>한국</t>
+          <t>유진투자증권</t>
         </is>
       </c>
       <c r="B27" s="6" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="C27" s="6" t="inlineStr">
         <is>
-          <t>154,600</t>
+          <t>24,000,000,000</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="6" t="inlineStr">
         <is>
-          <t>미래</t>
+          <t>하나증권</t>
         </is>
       </c>
       <c r="B28" s="6" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="C28" s="6" t="inlineStr">
         <is>
-          <t>130,837</t>
+          <t>16,614,000,000</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="6" t="inlineStr">
         <is>
-          <t>신한</t>
+          <t>NH</t>
         </is>
       </c>
       <c r="B29" s="6" t="n">
-        <v>3</v>
+        <v>7</v>
       </c>
       <c r="C29" s="6" t="inlineStr">
         <is>
-          <t>49,052</t>
+          <t>618,288</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="6" t="inlineStr">
         <is>
-          <t>삼성</t>
+          <t>한국</t>
         </is>
       </c>
       <c r="B30" s="6" t="n">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="C30" s="6" t="inlineStr">
         <is>
-          <t>32,000</t>
+          <t>154,600</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="6" t="inlineStr">
         <is>
-          <t>유진</t>
+          <t>미래</t>
         </is>
       </c>
       <c r="B31" s="6" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="C31" s="6" t="inlineStr">
         <is>
-          <t>25,020</t>
+          <t>130,837</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="6" t="inlineStr">
         <is>
-          <t>메리츠</t>
+          <t>신한</t>
         </is>
       </c>
       <c r="B32" s="6" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="C32" s="6" t="inlineStr">
         <is>
-          <t>14,000</t>
+          <t>49,052</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="6" t="inlineStr">
         <is>
-          <t>대신</t>
+          <t>삼성</t>
         </is>
       </c>
       <c r="B33" s="6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C33" s="6" t="inlineStr">
         <is>
-          <t>13,000</t>
+          <t>32,000</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="6" t="inlineStr">
         <is>
-          <t>키움</t>
+          <t>유진</t>
         </is>
       </c>
       <c r="B34" s="6" t="n">
@@ -12952,14 +12952,14 @@
       </c>
       <c r="C34" s="6" t="inlineStr">
         <is>
-          <t>12,000</t>
+          <t>25,020</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="6" t="inlineStr">
         <is>
-          <t>교보</t>
+          <t>메리츠</t>
         </is>
       </c>
       <c r="B35" s="6" t="n">
@@ -12967,31 +12967,54 @@
       </c>
       <c r="C35" s="6" t="inlineStr">
         <is>
-          <t>10,800</t>
+          <t>14,000</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="6" t="inlineStr">
         <is>
-          <t>NH투자증권</t>
+          <t>대신</t>
         </is>
       </c>
       <c r="B36" s="6" t="n">
         <v>1</v>
       </c>
-      <c r="C36" s="6" t="inlineStr"/>
+      <c r="C36" s="6" t="inlineStr">
+        <is>
+          <t>13,000</t>
+        </is>
+      </c>
     </row>
     <row r="37">
       <c r="A37" s="6" t="inlineStr">
         <is>
-          <t>미래에셋증권㈜</t>
+          <t>키움</t>
         </is>
       </c>
       <c r="B37" s="6" t="n">
         <v>1</v>
       </c>
-      <c r="C37" s="6" t="inlineStr"/>
+      <c r="C37" s="6" t="inlineStr">
+        <is>
+          <t>12,000</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="6" t="inlineStr">
+        <is>
+          <t>교보</t>
+        </is>
+      </c>
+      <c r="B38" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="C38" s="6" t="inlineStr">
+        <is>
+          <t>10,800</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
chore: update IPO data 2026-08-29
</commit_message>
<xml_diff>
--- a/IPO_analysis.xlsx
+++ b/IPO_analysis.xlsx
@@ -618,7 +618,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>기준일 2026-08-28 · 청구일 직전 사업연도 · 별도/개별 재무제표 · 단위 백만원(별도 표기 시 USD)</t>
+          <t>기준일 2026-08-29 · 청구일 직전 사업연도 · 별도/개별 재무제표 · 단위 백만원(별도 표기 시 USD)</t>
         </is>
       </c>
     </row>
@@ -10893,96 +10893,104 @@
     <row r="48" ht="30" customHeight="1">
       <c r="A48" s="6" t="inlineStr">
         <is>
-          <t>브릴스</t>
+          <t>엔에이치스팩34호</t>
         </is>
       </c>
       <c r="B48" s="6" t="inlineStr">
         <is>
-          <t>08-31~09-04</t>
-        </is>
-      </c>
-      <c r="C48" s="6" t="inlineStr">
-        <is>
-          <t>16,500~19,500</t>
+          <t>08-24~08-25</t>
+        </is>
+      </c>
+      <c r="C48" s="18" t="inlineStr">
+        <is>
+          <t>수집예정</t>
         </is>
       </c>
       <c r="D48" s="7" t="inlineStr">
         <is>
-          <t>1,200,000</t>
+          <t>8,500,000</t>
         </is>
       </c>
       <c r="E48" s="7" t="inlineStr">
         <is>
-          <t>19,800,000,000</t>
-        </is>
-      </c>
-      <c r="F48" s="6" t="inlineStr">
-        <is>
-          <t>13.44 (PSR)</t>
-        </is>
-      </c>
-      <c r="G48" s="6" t="inlineStr"/>
-      <c r="H48" s="6" t="inlineStr"/>
-      <c r="I48" s="6" t="inlineStr"/>
+          <t>17,000,000,000</t>
+        </is>
+      </c>
+      <c r="F48" s="18" t="inlineStr">
+        <is>
+          <t>수집예정</t>
+        </is>
+      </c>
+      <c r="G48" s="6" t="inlineStr">
+        <is>
+          <t>2,000</t>
+        </is>
+      </c>
+      <c r="H48" s="6" t="n">
+        <v>1160.7</v>
+      </c>
+      <c r="I48" s="6" t="n">
+        <v>2050</v>
+      </c>
       <c r="J48" s="6" t="inlineStr">
         <is>
-          <t>09-08~09-09</t>
+          <t>09-01~09-02</t>
         </is>
       </c>
       <c r="K48" s="6" t="inlineStr"/>
       <c r="L48" s="6" t="inlineStr"/>
       <c r="M48" s="6" t="inlineStr"/>
-      <c r="N48" s="6" t="inlineStr">
-        <is>
-          <t>아이비케이투자증권</t>
+      <c r="N48" s="18" t="inlineStr">
+        <is>
+          <t>수집예정</t>
         </is>
       </c>
       <c r="O48" s="6" t="inlineStr"/>
-      <c r="P48" s="7" t="inlineStr">
-        <is>
-          <t>713,790,000</t>
+      <c r="P48" s="18" t="inlineStr">
+        <is>
+          <t>수집예정</t>
         </is>
       </c>
       <c r="Q48" s="6" t="inlineStr">
         <is>
-          <t>3.5%</t>
+          <t>50%</t>
         </is>
       </c>
       <c r="R48" s="6" t="inlineStr">
         <is>
-          <t>정정</t>
+          <t>발행조건확정</t>
         </is>
       </c>
     </row>
     <row r="49" ht="30" customHeight="1">
       <c r="A49" s="6" t="inlineStr">
         <is>
-          <t>네오사피엔스</t>
+          <t>브릴스</t>
         </is>
       </c>
       <c r="B49" s="6" t="inlineStr">
         <is>
-          <t>09-02~09-08</t>
+          <t>08-31~09-04</t>
         </is>
       </c>
       <c r="C49" s="6" t="inlineStr">
         <is>
-          <t>13,800~15,800</t>
+          <t>16,500~19,500</t>
         </is>
       </c>
       <c r="D49" s="7" t="inlineStr">
         <is>
-          <t>2,000,000</t>
+          <t>1,200,000</t>
         </is>
       </c>
       <c r="E49" s="7" t="inlineStr">
         <is>
-          <t>27,600,000,000</t>
+          <t>19,800,000,000</t>
         </is>
       </c>
       <c r="F49" s="6" t="inlineStr">
         <is>
-          <t>26.76배 (PER)</t>
+          <t>13.44 (PSR)</t>
         </is>
       </c>
       <c r="G49" s="6" t="inlineStr"/>
@@ -10990,7 +10998,7 @@
       <c r="I49" s="6" t="inlineStr"/>
       <c r="J49" s="6" t="inlineStr">
         <is>
-          <t>09-10~09-11</t>
+          <t>09-08~09-09</t>
         </is>
       </c>
       <c r="K49" s="6" t="inlineStr"/>
@@ -10998,18 +11006,18 @@
       <c r="M49" s="6" t="inlineStr"/>
       <c r="N49" s="6" t="inlineStr">
         <is>
-          <t>대신증권</t>
+          <t>아이비케이투자증권</t>
         </is>
       </c>
       <c r="O49" s="6" t="inlineStr"/>
       <c r="P49" s="7" t="inlineStr">
         <is>
-          <t>1,080,264,000</t>
+          <t>713,790,000</t>
         </is>
       </c>
       <c r="Q49" s="6" t="inlineStr">
         <is>
-          <t>3.8%</t>
+          <t>3.5%</t>
         </is>
       </c>
       <c r="R49" s="6" t="inlineStr">
@@ -11021,32 +11029,32 @@
     <row r="50" ht="30" customHeight="1">
       <c r="A50" s="6" t="inlineStr">
         <is>
-          <t>케이비제34호스팩</t>
+          <t>네오사피엔스</t>
         </is>
       </c>
       <c r="B50" s="6" t="inlineStr">
         <is>
-          <t>09-04~09-07</t>
-        </is>
-      </c>
-      <c r="C50" s="18" t="inlineStr">
-        <is>
-          <t>수집예정</t>
+          <t>09-02~09-08</t>
+        </is>
+      </c>
+      <c r="C50" s="6" t="inlineStr">
+        <is>
+          <t>13,800~15,800</t>
         </is>
       </c>
       <c r="D50" s="7" t="inlineStr">
         <is>
-          <t>7,000,000</t>
+          <t>2,000,000</t>
         </is>
       </c>
       <c r="E50" s="7" t="inlineStr">
         <is>
-          <t>14,000,000,000</t>
-        </is>
-      </c>
-      <c r="F50" s="18" t="inlineStr">
-        <is>
-          <t>수집예정</t>
+          <t>27,600,000,000</t>
+        </is>
+      </c>
+      <c r="F50" s="6" t="inlineStr">
+        <is>
+          <t>26.76배 (PER)</t>
         </is>
       </c>
       <c r="G50" s="6" t="inlineStr"/>
@@ -11060,20 +11068,20 @@
       <c r="K50" s="6" t="inlineStr"/>
       <c r="L50" s="6" t="inlineStr"/>
       <c r="M50" s="6" t="inlineStr"/>
-      <c r="N50" s="18" t="inlineStr">
-        <is>
-          <t>수집예정</t>
+      <c r="N50" s="6" t="inlineStr">
+        <is>
+          <t>대신증권</t>
         </is>
       </c>
       <c r="O50" s="6" t="inlineStr"/>
-      <c r="P50" s="18" t="inlineStr">
-        <is>
-          <t>수집예정</t>
+      <c r="P50" s="7" t="inlineStr">
+        <is>
+          <t>1,080,264,000</t>
         </is>
       </c>
       <c r="Q50" s="6" t="inlineStr">
         <is>
-          <t>3.5%</t>
+          <t>3.8%</t>
         </is>
       </c>
       <c r="R50" s="6" t="inlineStr">
@@ -11085,32 +11093,32 @@
     <row r="51" ht="30" customHeight="1">
       <c r="A51" s="6" t="inlineStr">
         <is>
-          <t>와이즈플래닛컴퍼니</t>
+          <t>케이비제34호스팩</t>
         </is>
       </c>
       <c r="B51" s="6" t="inlineStr">
         <is>
-          <t>09-04~09-10</t>
-        </is>
-      </c>
-      <c r="C51" s="6" t="inlineStr">
-        <is>
-          <t>10,000~12,000</t>
+          <t>09-04~09-07</t>
+        </is>
+      </c>
+      <c r="C51" s="18" t="inlineStr">
+        <is>
+          <t>수집예정</t>
         </is>
       </c>
       <c r="D51" s="7" t="inlineStr">
         <is>
-          <t>1,600,000</t>
+          <t>7,000,000</t>
         </is>
       </c>
       <c r="E51" s="7" t="inlineStr">
         <is>
-          <t>16,000,000,000</t>
-        </is>
-      </c>
-      <c r="F51" s="6" t="inlineStr">
-        <is>
-          <t>21.59배 (PER)</t>
+          <t>14,000,000,000</t>
+        </is>
+      </c>
+      <c r="F51" s="18" t="inlineStr">
+        <is>
+          <t>수집예정</t>
         </is>
       </c>
       <c r="G51" s="6" t="inlineStr"/>
@@ -11118,26 +11126,26 @@
       <c r="I51" s="6" t="inlineStr"/>
       <c r="J51" s="6" t="inlineStr">
         <is>
-          <t>09-14~09-15</t>
+          <t>09-10~09-11</t>
         </is>
       </c>
       <c r="K51" s="6" t="inlineStr"/>
       <c r="L51" s="6" t="inlineStr"/>
       <c r="M51" s="6" t="inlineStr"/>
-      <c r="N51" s="6" t="inlineStr">
-        <is>
-          <t>대신증권</t>
+      <c r="N51" s="18" t="inlineStr">
+        <is>
+          <t>수집예정</t>
         </is>
       </c>
       <c r="O51" s="6" t="inlineStr"/>
-      <c r="P51" s="7" t="inlineStr">
-        <is>
-          <t>494,400,000</t>
+      <c r="P51" s="18" t="inlineStr">
+        <is>
+          <t>수집예정</t>
         </is>
       </c>
       <c r="Q51" s="6" t="inlineStr">
         <is>
-          <t>3.0%</t>
+          <t>3.5%</t>
         </is>
       </c>
       <c r="R51" s="6" t="inlineStr">
@@ -11149,32 +11157,32 @@
     <row r="52" ht="30" customHeight="1">
       <c r="A52" s="6" t="inlineStr">
         <is>
-          <t>한국제17호스팩</t>
+          <t>와이즈플래닛컴퍼니</t>
         </is>
       </c>
       <c r="B52" s="6" t="inlineStr">
         <is>
-          <t>09-07~09-08</t>
-        </is>
-      </c>
-      <c r="C52" s="18" t="inlineStr">
-        <is>
-          <t>수집예정</t>
+          <t>09-04~09-10</t>
+        </is>
+      </c>
+      <c r="C52" s="6" t="inlineStr">
+        <is>
+          <t>10,000~12,000</t>
         </is>
       </c>
       <c r="D52" s="7" t="inlineStr">
         <is>
-          <t>7,000,000</t>
+          <t>1,600,000</t>
         </is>
       </c>
       <c r="E52" s="7" t="inlineStr">
         <is>
-          <t>14,000,000,000</t>
-        </is>
-      </c>
-      <c r="F52" s="18" t="inlineStr">
-        <is>
-          <t>수집예정</t>
+          <t>16,000,000,000</t>
+        </is>
+      </c>
+      <c r="F52" s="6" t="inlineStr">
+        <is>
+          <t>21.59배 (PER)</t>
         </is>
       </c>
       <c r="G52" s="6" t="inlineStr"/>
@@ -11182,21 +11190,21 @@
       <c r="I52" s="6" t="inlineStr"/>
       <c r="J52" s="6" t="inlineStr">
         <is>
-          <t>09-10~09-11</t>
+          <t>09-14~09-15</t>
         </is>
       </c>
       <c r="K52" s="6" t="inlineStr"/>
       <c r="L52" s="6" t="inlineStr"/>
       <c r="M52" s="6" t="inlineStr"/>
-      <c r="N52" s="18" t="inlineStr">
-        <is>
-          <t>수집예정</t>
+      <c r="N52" s="6" t="inlineStr">
+        <is>
+          <t>대신증권</t>
         </is>
       </c>
       <c r="O52" s="6" t="inlineStr"/>
-      <c r="P52" s="18" t="inlineStr">
-        <is>
-          <t>수집예정</t>
+      <c r="P52" s="7" t="inlineStr">
+        <is>
+          <t>494,400,000</t>
         </is>
       </c>
       <c r="Q52" s="6" t="inlineStr">
@@ -11213,32 +11221,32 @@
     <row r="53" ht="30" customHeight="1">
       <c r="A53" s="6" t="inlineStr">
         <is>
-          <t>빅웨이브로보틱스</t>
+          <t>한국제17호스팩</t>
         </is>
       </c>
       <c r="B53" s="6" t="inlineStr">
         <is>
-          <t>09-07~09-11</t>
-        </is>
-      </c>
-      <c r="C53" s="6" t="inlineStr">
-        <is>
-          <t>15,000~18,000</t>
+          <t>09-07~09-08</t>
+        </is>
+      </c>
+      <c r="C53" s="18" t="inlineStr">
+        <is>
+          <t>수집예정</t>
         </is>
       </c>
       <c r="D53" s="7" t="inlineStr">
         <is>
-          <t>1,600,000</t>
+          <t>7,000,000</t>
         </is>
       </c>
       <c r="E53" s="7" t="inlineStr">
         <is>
-          <t>24,000,000,000</t>
-        </is>
-      </c>
-      <c r="F53" s="6" t="inlineStr">
-        <is>
-          <t>11.15 (PSR)</t>
+          <t>14,000,000,000</t>
+        </is>
+      </c>
+      <c r="F53" s="18" t="inlineStr">
+        <is>
+          <t>수집예정</t>
         </is>
       </c>
       <c r="G53" s="6" t="inlineStr"/>
@@ -11246,25 +11254,21 @@
       <c r="I53" s="6" t="inlineStr"/>
       <c r="J53" s="6" t="inlineStr">
         <is>
-          <t>09-15~09-16</t>
+          <t>09-10~09-11</t>
         </is>
       </c>
       <c r="K53" s="6" t="inlineStr"/>
       <c r="L53" s="6" t="inlineStr"/>
       <c r="M53" s="6" t="inlineStr"/>
-      <c r="N53" s="6" t="inlineStr">
-        <is>
-          <t>유진투자증권</t>
-        </is>
-      </c>
-      <c r="O53" s="6" t="inlineStr">
-        <is>
-          <t>미래</t>
-        </is>
-      </c>
-      <c r="P53" s="7" t="inlineStr">
-        <is>
-          <t>378,216,000</t>
+      <c r="N53" s="18" t="inlineStr">
+        <is>
+          <t>수집예정</t>
+        </is>
+      </c>
+      <c r="O53" s="6" t="inlineStr"/>
+      <c r="P53" s="18" t="inlineStr">
+        <is>
+          <t>수집예정</t>
         </is>
       </c>
       <c r="Q53" s="6" t="inlineStr">
@@ -11281,7 +11285,7 @@
     <row r="54" ht="30" customHeight="1">
       <c r="A54" s="6" t="inlineStr">
         <is>
-          <t>글로벌테크놀로지</t>
+          <t>빅웨이브로보틱스</t>
         </is>
       </c>
       <c r="B54" s="6" t="inlineStr">
@@ -11291,22 +11295,22 @@
       </c>
       <c r="C54" s="6" t="inlineStr">
         <is>
-          <t>13,000~15,000</t>
+          <t>15,000~18,000</t>
         </is>
       </c>
       <c r="D54" s="7" t="inlineStr">
         <is>
-          <t>4,000,000</t>
+          <t>1,600,000</t>
         </is>
       </c>
       <c r="E54" s="7" t="inlineStr">
         <is>
-          <t>52,000,000,000</t>
+          <t>24,000,000,000</t>
         </is>
       </c>
       <c r="F54" s="6" t="inlineStr">
         <is>
-          <t>20.77배 (PER)</t>
+          <t>11.15 (PSR)</t>
         </is>
       </c>
       <c r="G54" s="6" t="inlineStr"/>
@@ -11314,7 +11318,7 @@
       <c r="I54" s="6" t="inlineStr"/>
       <c r="J54" s="6" t="inlineStr">
         <is>
-          <t>09-16~09-17</t>
+          <t>09-15~09-16</t>
         </is>
       </c>
       <c r="K54" s="6" t="inlineStr"/>
@@ -11322,18 +11326,22 @@
       <c r="M54" s="6" t="inlineStr"/>
       <c r="N54" s="6" t="inlineStr">
         <is>
-          <t>한국투자증권</t>
-        </is>
-      </c>
-      <c r="O54" s="6" t="inlineStr"/>
+          <t>유진투자증권</t>
+        </is>
+      </c>
+      <c r="O54" s="6" t="inlineStr">
+        <is>
+          <t>미래</t>
+        </is>
+      </c>
       <c r="P54" s="7" t="inlineStr">
         <is>
-          <t>2,119,999,960</t>
-        </is>
-      </c>
-      <c r="Q54" s="18" t="inlineStr">
-        <is>
-          <t>수집예정</t>
+          <t>378,216,000</t>
+        </is>
+      </c>
+      <c r="Q54" s="6" t="inlineStr">
+        <is>
+          <t>3.0%</t>
         </is>
       </c>
       <c r="R54" s="6" t="inlineStr">
@@ -11345,32 +11353,32 @@
     <row r="55" ht="30" customHeight="1">
       <c r="A55" s="6" t="inlineStr">
         <is>
-          <t>덕산넵코어스</t>
+          <t>글로벌테크놀로지</t>
         </is>
       </c>
       <c r="B55" s="6" t="inlineStr">
         <is>
-          <t>09-08~09-14</t>
+          <t>09-07~09-11</t>
         </is>
       </c>
       <c r="C55" s="6" t="inlineStr">
         <is>
-          <t>12,400~14,600</t>
+          <t>13,000~15,000</t>
         </is>
       </c>
       <c r="D55" s="7" t="inlineStr">
         <is>
-          <t>3,000,000</t>
+          <t>4,000,000</t>
         </is>
       </c>
       <c r="E55" s="7" t="inlineStr">
         <is>
-          <t>37,200,000,000</t>
+          <t>52,000,000,000</t>
         </is>
       </c>
       <c r="F55" s="6" t="inlineStr">
         <is>
-          <t>32.57배 (PER)</t>
+          <t>20.77배 (PER)</t>
         </is>
       </c>
       <c r="G55" s="6" t="inlineStr"/>
@@ -11386,18 +11394,18 @@
       <c r="M55" s="6" t="inlineStr"/>
       <c r="N55" s="6" t="inlineStr">
         <is>
-          <t>대신증권</t>
+          <t>한국투자증권</t>
         </is>
       </c>
       <c r="O55" s="6" t="inlineStr"/>
       <c r="P55" s="7" t="inlineStr">
         <is>
-          <t>1,413,399,926</t>
-        </is>
-      </c>
-      <c r="Q55" s="6" t="inlineStr">
-        <is>
-          <t>3.7%</t>
+          <t>2,119,999,960</t>
+        </is>
+      </c>
+      <c r="Q55" s="18" t="inlineStr">
+        <is>
+          <t>수집예정</t>
         </is>
       </c>
       <c r="R55" s="6" t="inlineStr">
@@ -11409,32 +11417,32 @@
     <row r="56" ht="30" customHeight="1">
       <c r="A56" s="6" t="inlineStr">
         <is>
-          <t>엔에이치스팩34호</t>
+          <t>덕산넵코어스</t>
         </is>
       </c>
       <c r="B56" s="6" t="inlineStr">
         <is>
-          <t>08-24~08-25</t>
-        </is>
-      </c>
-      <c r="C56" s="18" t="inlineStr">
-        <is>
-          <t>수집예정</t>
+          <t>09-08~09-14</t>
+        </is>
+      </c>
+      <c r="C56" s="6" t="inlineStr">
+        <is>
+          <t>12,400~14,600</t>
         </is>
       </c>
       <c r="D56" s="7" t="inlineStr">
         <is>
-          <t>8,500,000</t>
+          <t>3,000,000</t>
         </is>
       </c>
       <c r="E56" s="7" t="inlineStr">
         <is>
-          <t>17,000,000,000</t>
-        </is>
-      </c>
-      <c r="F56" s="18" t="inlineStr">
-        <is>
-          <t>수집예정</t>
+          <t>37,200,000,000</t>
+        </is>
+      </c>
+      <c r="F56" s="6" t="inlineStr">
+        <is>
+          <t>32.57배 (PER)</t>
         </is>
       </c>
       <c r="G56" s="6" t="inlineStr"/>
@@ -11442,31 +11450,31 @@
       <c r="I56" s="6" t="inlineStr"/>
       <c r="J56" s="6" t="inlineStr">
         <is>
-          <t>09-01~09-02</t>
+          <t>09-16~09-17</t>
         </is>
       </c>
       <c r="K56" s="6" t="inlineStr"/>
       <c r="L56" s="6" t="inlineStr"/>
       <c r="M56" s="6" t="inlineStr"/>
-      <c r="N56" s="18" t="inlineStr">
-        <is>
-          <t>수집예정</t>
+      <c r="N56" s="6" t="inlineStr">
+        <is>
+          <t>대신증권</t>
         </is>
       </c>
       <c r="O56" s="6" t="inlineStr"/>
-      <c r="P56" s="18" t="inlineStr">
-        <is>
-          <t>수집예정</t>
+      <c r="P56" s="7" t="inlineStr">
+        <is>
+          <t>1,413,399,926</t>
         </is>
       </c>
       <c r="Q56" s="6" t="inlineStr">
         <is>
-          <t>50%</t>
+          <t>3.7%</t>
         </is>
       </c>
       <c r="R56" s="6" t="inlineStr">
         <is>
-          <t>최초</t>
+          <t>정정</t>
         </is>
       </c>
     </row>
@@ -11669,32 +11677,32 @@
     <row r="60" ht="30" customHeight="1">
       <c r="A60" s="6" t="inlineStr">
         <is>
-          <t>래블업</t>
+          <t>엠비디</t>
         </is>
       </c>
       <c r="B60" s="6" t="inlineStr">
         <is>
-          <t>09-28~10-02</t>
+          <t>09-21~09-29</t>
         </is>
       </c>
       <c r="C60" s="6" t="inlineStr">
         <is>
-          <t>20,000~23,000</t>
+          <t>9,400~11,500</t>
         </is>
       </c>
       <c r="D60" s="7" t="inlineStr">
         <is>
-          <t>2,180,000</t>
+          <t>2,000,000</t>
         </is>
       </c>
       <c r="E60" s="7" t="inlineStr">
         <is>
-          <t>43,600,000,000</t>
+          <t>18,800,000,000</t>
         </is>
       </c>
       <c r="F60" s="6" t="inlineStr">
         <is>
-          <t>33.6배 (PER)</t>
+          <t>26.87배 (PER)</t>
         </is>
       </c>
       <c r="G60" s="6" t="inlineStr"/>
@@ -11702,7 +11710,7 @@
       <c r="I60" s="6" t="inlineStr"/>
       <c r="J60" s="6" t="inlineStr">
         <is>
-          <t>10-12~10-13</t>
+          <t>10-06~10-07</t>
         </is>
       </c>
       <c r="K60" s="6" t="inlineStr"/>
@@ -11710,18 +11718,18 @@
       <c r="M60" s="6" t="inlineStr"/>
       <c r="N60" s="6" t="inlineStr">
         <is>
-          <t>NH투자증권</t>
+          <t>하나증권</t>
         </is>
       </c>
       <c r="O60" s="6" t="inlineStr"/>
       <c r="P60" s="7" t="inlineStr">
         <is>
-          <t>2,007,000,000</t>
+          <t>968,200,000</t>
         </is>
       </c>
       <c r="Q60" s="6" t="inlineStr">
         <is>
-          <t>4.5%</t>
+          <t>5.0%</t>
         </is>
       </c>
       <c r="R60" s="6" t="inlineStr">
@@ -11733,32 +11741,32 @@
     <row r="61" ht="30" customHeight="1">
       <c r="A61" s="6" t="inlineStr">
         <is>
-          <t>에스케이증권제14호기업인수목적</t>
+          <t>래블업</t>
         </is>
       </c>
       <c r="B61" s="6" t="inlineStr">
         <is>
-          <t>10-12~10-13</t>
-        </is>
-      </c>
-      <c r="C61" s="18" t="inlineStr">
-        <is>
-          <t>수집예정</t>
+          <t>09-28~10-02</t>
+        </is>
+      </c>
+      <c r="C61" s="6" t="inlineStr">
+        <is>
+          <t>20,000~23,000</t>
         </is>
       </c>
       <c r="D61" s="7" t="inlineStr">
         <is>
-          <t>6,500,000</t>
+          <t>2,180,000</t>
         </is>
       </c>
       <c r="E61" s="7" t="inlineStr">
         <is>
-          <t>13,000,000,000</t>
-        </is>
-      </c>
-      <c r="F61" s="18" t="inlineStr">
-        <is>
-          <t>수집예정</t>
+          <t>43,600,000,000</t>
+        </is>
+      </c>
+      <c r="F61" s="6" t="inlineStr">
+        <is>
+          <t>33.6배 (PER)</t>
         </is>
       </c>
       <c r="G61" s="6" t="inlineStr"/>
@@ -11766,26 +11774,26 @@
       <c r="I61" s="6" t="inlineStr"/>
       <c r="J61" s="6" t="inlineStr">
         <is>
-          <t>10-15~10-16</t>
+          <t>10-12~10-13</t>
         </is>
       </c>
       <c r="K61" s="6" t="inlineStr"/>
       <c r="L61" s="6" t="inlineStr"/>
       <c r="M61" s="6" t="inlineStr"/>
-      <c r="N61" s="18" t="inlineStr">
-        <is>
-          <t>수집예정</t>
+      <c r="N61" s="6" t="inlineStr">
+        <is>
+          <t>NH투자증권</t>
         </is>
       </c>
       <c r="O61" s="6" t="inlineStr"/>
-      <c r="P61" s="18" t="inlineStr">
-        <is>
-          <t>수집예정</t>
+      <c r="P61" s="7" t="inlineStr">
+        <is>
+          <t>2,007,000,000</t>
         </is>
       </c>
       <c r="Q61" s="6" t="inlineStr">
         <is>
-          <t>50%</t>
+          <t>4.5%</t>
         </is>
       </c>
       <c r="R61" s="6" t="inlineStr">
@@ -11797,27 +11805,27 @@
     <row r="62" ht="30" customHeight="1">
       <c r="A62" s="6" t="inlineStr">
         <is>
-          <t>엠비디</t>
-        </is>
-      </c>
-      <c r="B62" s="18" t="inlineStr">
+          <t>에스케이증권제14호기업인수목적</t>
+        </is>
+      </c>
+      <c r="B62" s="6" t="inlineStr">
+        <is>
+          <t>10-12~10-13</t>
+        </is>
+      </c>
+      <c r="C62" s="18" t="inlineStr">
         <is>
           <t>수집예정</t>
         </is>
       </c>
-      <c r="C62" s="18" t="inlineStr">
-        <is>
-          <t>수집예정</t>
-        </is>
-      </c>
-      <c r="D62" s="18" t="inlineStr">
-        <is>
-          <t>수집예정</t>
-        </is>
-      </c>
-      <c r="E62" s="18" t="inlineStr">
-        <is>
-          <t>수집예정</t>
+      <c r="D62" s="7" t="inlineStr">
+        <is>
+          <t>6,500,000</t>
+        </is>
+      </c>
+      <c r="E62" s="7" t="inlineStr">
+        <is>
+          <t>13,000,000,000</t>
         </is>
       </c>
       <c r="F62" s="18" t="inlineStr">
@@ -11828,9 +11836,9 @@
       <c r="G62" s="6" t="inlineStr"/>
       <c r="H62" s="6" t="inlineStr"/>
       <c r="I62" s="6" t="inlineStr"/>
-      <c r="J62" s="18" t="inlineStr">
-        <is>
-          <t>수집예정</t>
+      <c r="J62" s="6" t="inlineStr">
+        <is>
+          <t>10-15~10-16</t>
         </is>
       </c>
       <c r="K62" s="6" t="inlineStr"/>
@@ -11847,9 +11855,9 @@
           <t>수집예정</t>
         </is>
       </c>
-      <c r="Q62" s="18" t="inlineStr">
-        <is>
-          <t>수집예정</t>
+      <c r="Q62" s="6" t="inlineStr">
+        <is>
+          <t>50%</t>
         </is>
       </c>
       <c r="R62" s="6" t="inlineStr">
@@ -11861,7 +11869,7 @@
     <row r="63" ht="30" customHeight="1">
       <c r="A63" s="6" t="inlineStr">
         <is>
-          <t>다비오</t>
+          <t>엠에스바이오</t>
         </is>
       </c>
       <c r="B63" s="18" t="inlineStr">
@@ -11918,14 +11926,14 @@
       </c>
       <c r="R63" s="6" t="inlineStr">
         <is>
-          <t>corp_code 미확보(수동확인)</t>
+          <t>신고서 대기</t>
         </is>
       </c>
     </row>
     <row r="64" ht="30" customHeight="1">
       <c r="A64" s="6" t="inlineStr">
         <is>
-          <t>엠에스바이오</t>
+          <t>디티에스</t>
         </is>
       </c>
       <c r="B64" s="18" t="inlineStr">
@@ -11989,7 +11997,7 @@
     <row r="65" ht="30" customHeight="1">
       <c r="A65" s="6" t="inlineStr">
         <is>
-          <t>디티에스</t>
+          <t>한화플러스제6호스팩</t>
         </is>
       </c>
       <c r="B65" s="18" t="inlineStr">
@@ -12053,7 +12061,7 @@
     <row r="66" ht="30" customHeight="1">
       <c r="A66" s="6" t="inlineStr">
         <is>
-          <t>한화플러스제6호스팩</t>
+          <t>바로팜</t>
         </is>
       </c>
       <c r="B66" s="18" t="inlineStr">
@@ -12117,7 +12125,7 @@
     <row r="67" ht="30" customHeight="1">
       <c r="A67" s="6" t="inlineStr">
         <is>
-          <t>바로팜</t>
+          <t>크리에이츠</t>
         </is>
       </c>
       <c r="B67" s="18" t="inlineStr">
@@ -12181,7 +12189,7 @@
     <row r="68" ht="30" customHeight="1">
       <c r="A68" s="6" t="inlineStr">
         <is>
-          <t>크리에이츠</t>
+          <t>티앤이코리아</t>
         </is>
       </c>
       <c r="B68" s="18" t="inlineStr">
@@ -12245,7 +12253,7 @@
     <row r="69" ht="30" customHeight="1">
       <c r="A69" s="6" t="inlineStr">
         <is>
-          <t>티앤이코리아</t>
+          <t>유캐스트</t>
         </is>
       </c>
       <c r="B69" s="18" t="inlineStr">
@@ -12309,7 +12317,7 @@
     <row r="70" ht="30" customHeight="1">
       <c r="A70" s="6" t="inlineStr">
         <is>
-          <t>유캐스트</t>
+          <t>다비오</t>
         </is>
       </c>
       <c r="B70" s="18" t="inlineStr">
@@ -12846,22 +12854,22 @@
     <row r="27">
       <c r="A27" s="6" t="inlineStr">
         <is>
-          <t>유진투자증권</t>
+          <t>하나증권</t>
         </is>
       </c>
       <c r="B27" s="6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C27" s="6" t="inlineStr">
         <is>
-          <t>24,000,000,000</t>
+          <t>35,414,000,000</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="6" t="inlineStr">
         <is>
-          <t>하나증권</t>
+          <t>유진투자증권</t>
         </is>
       </c>
       <c r="B28" s="6" t="n">
@@ -12869,7 +12877,7 @@
       </c>
       <c r="C28" s="6" t="inlineStr">
         <is>
-          <t>16,614,000,000</t>
+          <t>24,000,000,000</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore: update IPO data 2026-08-31
</commit_message>
<xml_diff>
--- a/IPO_analysis.xlsx
+++ b/IPO_analysis.xlsx
@@ -618,7 +618,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>기준일 2026-08-30 · 청구일 직전 사업연도 · 별도/개별 재무제표 · 단위 백만원(별도 표기 시 USD)</t>
+          <t>기준일 2026-08-31 · 청구일 직전 사업연도 · 별도/개별 재무제표 · 단위 백만원(별도 표기 시 USD)</t>
         </is>
       </c>
     </row>
@@ -10865,7 +10865,11 @@
           <t>08-26~08-27</t>
         </is>
       </c>
-      <c r="K47" s="6" t="inlineStr"/>
+      <c r="K47" s="6" t="inlineStr">
+        <is>
+          <t>88.20</t>
+        </is>
+      </c>
       <c r="L47" s="6" t="inlineStr"/>
       <c r="M47" s="6" t="inlineStr"/>
       <c r="N47" s="6" t="inlineStr">
@@ -10886,7 +10890,7 @@
       </c>
       <c r="R47" s="6" t="inlineStr">
         <is>
-          <t>발행조건확정</t>
+          <t>청약완료·상장대기</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore: update IPO data 2026-09-01
</commit_message>
<xml_diff>
--- a/IPO_analysis.xlsx
+++ b/IPO_analysis.xlsx
@@ -618,14 +618,14 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>기준일 2026-08-31 · 청구일 직전 사업연도 · 별도/개별 재무제표 · 단위 백만원(별도 표기 시 USD)</t>
+          <t>기준일 2026-09-01 · 청구일 직전 사업연도 · 별도/개별 재무제표 · 단위 백만원(별도 표기 시 USD)</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
-          <t>■ 심사 신청(진행중)  (49건)</t>
+          <t>■ 심사 신청(진행중)  (48건)</t>
         </is>
       </c>
       <c r="B4" s="4" t="n"/>
@@ -3216,12 +3216,12 @@
     <row r="51">
       <c r="A51" s="6" t="inlineStr">
         <is>
-          <t>2026-04-30</t>
+          <t>2026-04-08</t>
         </is>
       </c>
       <c r="B51" s="6" t="inlineStr">
         <is>
-          <t>텔레픽스</t>
+          <t>옵토닉스</t>
         </is>
       </c>
       <c r="C51" s="6" t="inlineStr">
@@ -3241,27 +3241,27 @@
       </c>
       <c r="F51" s="7" t="inlineStr">
         <is>
-          <t>4,896</t>
+          <t>25,368</t>
         </is>
       </c>
       <c r="G51" s="7" t="inlineStr">
         <is>
-          <t>-16,214</t>
+          <t>1,901</t>
         </is>
       </c>
       <c r="H51" s="7" t="inlineStr">
         <is>
-          <t>9,146</t>
+          <t>730</t>
         </is>
       </c>
       <c r="I51" s="6" t="inlineStr">
         <is>
-          <t>소프트웨어 개발 및 공급업</t>
+          <t>광학렌즈 및 광학요소 제조업</t>
         </is>
       </c>
       <c r="J51" s="6" t="inlineStr">
         <is>
-          <t>미래</t>
+          <t>한국</t>
         </is>
       </c>
       <c r="K51" s="6" t="inlineStr">
@@ -3273,12 +3273,12 @@
     <row r="52">
       <c r="A52" s="6" t="inlineStr">
         <is>
-          <t>2026-04-08</t>
+          <t>2026-03-24</t>
         </is>
       </c>
       <c r="B52" s="6" t="inlineStr">
         <is>
-          <t>옵토닉스</t>
+          <t>인텔리빅스</t>
         </is>
       </c>
       <c r="C52" s="6" t="inlineStr">
@@ -3298,27 +3298,27 @@
       </c>
       <c r="F52" s="7" t="inlineStr">
         <is>
-          <t>25,368</t>
+          <t>46,644</t>
         </is>
       </c>
       <c r="G52" s="7" t="inlineStr">
         <is>
-          <t>1,901</t>
+          <t>5,357</t>
         </is>
       </c>
       <c r="H52" s="7" t="inlineStr">
         <is>
-          <t>730</t>
+          <t>1,048</t>
         </is>
       </c>
       <c r="I52" s="6" t="inlineStr">
         <is>
-          <t>광학렌즈 및 광학요소 제조업</t>
+          <t>소프트웨어 개발 및 공급업</t>
         </is>
       </c>
       <c r="J52" s="6" t="inlineStr">
         <is>
-          <t>한국</t>
+          <t>미래</t>
         </is>
       </c>
       <c r="K52" s="6" t="inlineStr">
@@ -3330,12 +3330,12 @@
     <row r="53">
       <c r="A53" s="6" t="inlineStr">
         <is>
-          <t>2026-03-24</t>
+          <t>2026-02-27</t>
         </is>
       </c>
       <c r="B53" s="6" t="inlineStr">
         <is>
-          <t>인텔리빅스</t>
+          <t>피지티</t>
         </is>
       </c>
       <c r="C53" s="6" t="inlineStr">
@@ -3355,175 +3355,175 @@
       </c>
       <c r="F53" s="7" t="inlineStr">
         <is>
-          <t>46,644</t>
+          <t>40,141</t>
         </is>
       </c>
       <c r="G53" s="7" t="inlineStr">
         <is>
-          <t>5,357</t>
+          <t>-69,722</t>
         </is>
       </c>
       <c r="H53" s="7" t="inlineStr">
         <is>
-          <t>1,048</t>
+          <t>6,029</t>
         </is>
       </c>
       <c r="I53" s="6" t="inlineStr">
         <is>
+          <t>기타 화학제품 제조업</t>
+        </is>
+      </c>
+      <c r="J53" s="6" t="inlineStr">
+        <is>
+          <t>한국</t>
+        </is>
+      </c>
+      <c r="K53" s="6" t="inlineStr">
+        <is>
+          <t>예심 진행중</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="3" t="inlineStr">
+        <is>
+          <t>■ 심사 승인  (54건)</t>
+        </is>
+      </c>
+      <c r="B55" s="4" t="n"/>
+      <c r="C55" s="4" t="n"/>
+      <c r="D55" s="4" t="n"/>
+      <c r="E55" s="4" t="n"/>
+      <c r="F55" s="4" t="n"/>
+      <c r="G55" s="4" t="n"/>
+      <c r="H55" s="4" t="n"/>
+      <c r="I55" s="4" t="n"/>
+      <c r="J55" s="4" t="n"/>
+      <c r="K55" s="4" t="n"/>
+    </row>
+    <row r="56">
+      <c r="A56" s="5" t="inlineStr">
+        <is>
+          <t>일자</t>
+        </is>
+      </c>
+      <c r="B56" s="5" t="inlineStr">
+        <is>
+          <t>회사명</t>
+        </is>
+      </c>
+      <c r="C56" s="5" t="inlineStr">
+        <is>
+          <t>시장</t>
+        </is>
+      </c>
+      <c r="D56" s="5" t="inlineStr">
+        <is>
+          <t>상장유형</t>
+        </is>
+      </c>
+      <c r="E56" s="5" t="inlineStr">
+        <is>
+          <t>기준연도</t>
+        </is>
+      </c>
+      <c r="F56" s="5" t="inlineStr">
+        <is>
+          <t>매출액</t>
+        </is>
+      </c>
+      <c r="G56" s="5" t="inlineStr">
+        <is>
+          <t>순이익</t>
+        </is>
+      </c>
+      <c r="H56" s="5" t="inlineStr">
+        <is>
+          <t>자기자본</t>
+        </is>
+      </c>
+      <c r="I56" s="5" t="inlineStr">
+        <is>
+          <t>업종</t>
+        </is>
+      </c>
+      <c r="J56" s="5" t="inlineStr">
+        <is>
+          <t>대표주관사</t>
+        </is>
+      </c>
+      <c r="K56" s="5" t="inlineStr">
+        <is>
+          <t>현황</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="6" t="inlineStr">
+        <is>
+          <t>2026-08-28</t>
+        </is>
+      </c>
+      <c r="B57" s="6" t="inlineStr">
+        <is>
+          <t>다비오</t>
+        </is>
+      </c>
+      <c r="C57" s="6" t="inlineStr">
+        <is>
+          <t>코스닥</t>
+        </is>
+      </c>
+      <c r="D57" s="6" t="inlineStr">
+        <is>
+          <t>신규상장</t>
+        </is>
+      </c>
+      <c r="E57" s="6" t="inlineStr">
+        <is>
+          <t>FY25</t>
+        </is>
+      </c>
+      <c r="F57" s="7" t="inlineStr">
+        <is>
+          <t>9,251</t>
+        </is>
+      </c>
+      <c r="G57" s="7" t="inlineStr">
+        <is>
+          <t>-3,473</t>
+        </is>
+      </c>
+      <c r="H57" s="7" t="inlineStr">
+        <is>
+          <t>300</t>
+        </is>
+      </c>
+      <c r="I57" s="6" t="inlineStr">
+        <is>
           <t>소프트웨어 개발 및 공급업</t>
         </is>
       </c>
-      <c r="J53" s="6" t="inlineStr">
-        <is>
-          <t>미래</t>
-        </is>
-      </c>
-      <c r="K53" s="6" t="inlineStr">
-        <is>
-          <t>예심 진행중</t>
-        </is>
-      </c>
-    </row>
-    <row r="54">
-      <c r="A54" s="6" t="inlineStr">
-        <is>
-          <t>2026-02-27</t>
-        </is>
-      </c>
-      <c r="B54" s="6" t="inlineStr">
-        <is>
-          <t>피지티</t>
-        </is>
-      </c>
-      <c r="C54" s="6" t="inlineStr">
-        <is>
-          <t>코스닥</t>
-        </is>
-      </c>
-      <c r="D54" s="6" t="inlineStr">
-        <is>
-          <t>신규상장</t>
-        </is>
-      </c>
-      <c r="E54" s="6" t="inlineStr">
-        <is>
-          <t>FY25</t>
-        </is>
-      </c>
-      <c r="F54" s="7" t="inlineStr">
-        <is>
-          <t>40,141</t>
-        </is>
-      </c>
-      <c r="G54" s="7" t="inlineStr">
-        <is>
-          <t>-69,722</t>
-        </is>
-      </c>
-      <c r="H54" s="7" t="inlineStr">
-        <is>
-          <t>6,029</t>
-        </is>
-      </c>
-      <c r="I54" s="6" t="inlineStr">
-        <is>
-          <t>기타 화학제품 제조업</t>
-        </is>
-      </c>
-      <c r="J54" s="6" t="inlineStr">
-        <is>
-          <t>한국</t>
-        </is>
-      </c>
-      <c r="K54" s="6" t="inlineStr">
-        <is>
-          <t>예심 진행중</t>
-        </is>
-      </c>
-    </row>
-    <row r="56">
-      <c r="A56" s="3" t="inlineStr">
-        <is>
-          <t>■ 심사 승인  (54건)</t>
-        </is>
-      </c>
-      <c r="B56" s="4" t="n"/>
-      <c r="C56" s="4" t="n"/>
-      <c r="D56" s="4" t="n"/>
-      <c r="E56" s="4" t="n"/>
-      <c r="F56" s="4" t="n"/>
-      <c r="G56" s="4" t="n"/>
-      <c r="H56" s="4" t="n"/>
-      <c r="I56" s="4" t="n"/>
-      <c r="J56" s="4" t="n"/>
-      <c r="K56" s="4" t="n"/>
-    </row>
-    <row r="57">
-      <c r="A57" s="5" t="inlineStr">
-        <is>
-          <t>일자</t>
-        </is>
-      </c>
-      <c r="B57" s="5" t="inlineStr">
-        <is>
-          <t>회사명</t>
-        </is>
-      </c>
-      <c r="C57" s="5" t="inlineStr">
-        <is>
-          <t>시장</t>
-        </is>
-      </c>
-      <c r="D57" s="5" t="inlineStr">
-        <is>
-          <t>상장유형</t>
-        </is>
-      </c>
-      <c r="E57" s="5" t="inlineStr">
-        <is>
-          <t>기준연도</t>
-        </is>
-      </c>
-      <c r="F57" s="5" t="inlineStr">
-        <is>
-          <t>매출액</t>
-        </is>
-      </c>
-      <c r="G57" s="5" t="inlineStr">
-        <is>
-          <t>순이익</t>
-        </is>
-      </c>
-      <c r="H57" s="5" t="inlineStr">
-        <is>
-          <t>자기자본</t>
-        </is>
-      </c>
-      <c r="I57" s="5" t="inlineStr">
-        <is>
-          <t>업종</t>
-        </is>
-      </c>
-      <c r="J57" s="5" t="inlineStr">
-        <is>
-          <t>대표주관사</t>
-        </is>
-      </c>
-      <c r="K57" s="5" t="inlineStr">
-        <is>
-          <t>현황</t>
+      <c r="J57" s="6" t="inlineStr">
+        <is>
+          <t>대신</t>
+        </is>
+      </c>
+      <c r="K57" s="6" t="inlineStr">
+        <is>
+          <t>상장전</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" s="6" t="inlineStr">
         <is>
-          <t>2026-08-28</t>
+          <t>2026-08-20</t>
         </is>
       </c>
       <c r="B58" s="6" t="inlineStr">
         <is>
-          <t>다비오</t>
+          <t>티앤이코리아</t>
         </is>
       </c>
       <c r="C58" s="6" t="inlineStr">
@@ -3543,27 +3543,27 @@
       </c>
       <c r="F58" s="7" t="inlineStr">
         <is>
-          <t>9,251</t>
+          <t>22,339</t>
         </is>
       </c>
       <c r="G58" s="7" t="inlineStr">
         <is>
-          <t>-3,473</t>
+          <t>-7,091</t>
         </is>
       </c>
       <c r="H58" s="7" t="inlineStr">
         <is>
-          <t>300</t>
+          <t>481</t>
         </is>
       </c>
       <c r="I58" s="6" t="inlineStr">
         <is>
-          <t>소프트웨어 개발 및 공급업</t>
+          <t>일반 목적용 기계 제조업</t>
         </is>
       </c>
       <c r="J58" s="6" t="inlineStr">
         <is>
-          <t>대신</t>
+          <t>신한</t>
         </is>
       </c>
       <c r="K58" s="6" t="inlineStr">
@@ -3580,7 +3580,7 @@
       </c>
       <c r="B59" s="6" t="inlineStr">
         <is>
-          <t>티앤이코리아</t>
+          <t>유캐스트</t>
         </is>
       </c>
       <c r="C59" s="6" t="inlineStr">
@@ -3600,27 +3600,27 @@
       </c>
       <c r="F59" s="7" t="inlineStr">
         <is>
-          <t>22,339</t>
+          <t>5,934</t>
         </is>
       </c>
       <c r="G59" s="7" t="inlineStr">
         <is>
-          <t>-7,091</t>
+          <t>-3,557</t>
         </is>
       </c>
       <c r="H59" s="7" t="inlineStr">
         <is>
-          <t>481</t>
+          <t>1,881</t>
         </is>
       </c>
       <c r="I59" s="6" t="inlineStr">
         <is>
-          <t>일반 목적용 기계 제조업</t>
+          <t>통신 및 방송 장비 제조업</t>
         </is>
       </c>
       <c r="J59" s="6" t="inlineStr">
         <is>
-          <t>신한</t>
+          <t>유진</t>
         </is>
       </c>
       <c r="K59" s="6" t="inlineStr">
@@ -3637,7 +3637,7 @@
       </c>
       <c r="B60" s="6" t="inlineStr">
         <is>
-          <t>유캐스트</t>
+          <t>엘리스그룹</t>
         </is>
       </c>
       <c r="C60" s="6" t="inlineStr">
@@ -3657,27 +3657,27 @@
       </c>
       <c r="F60" s="7" t="inlineStr">
         <is>
-          <t>5,934</t>
+          <t>39,513</t>
         </is>
       </c>
       <c r="G60" s="7" t="inlineStr">
         <is>
-          <t>-3,557</t>
+          <t>15,666</t>
         </is>
       </c>
       <c r="H60" s="7" t="inlineStr">
         <is>
-          <t>1,881</t>
+          <t>85,400</t>
         </is>
       </c>
       <c r="I60" s="6" t="inlineStr">
         <is>
-          <t>통신 및 방송 장비 제조업</t>
+          <t>소프트웨어 개발 및 공급업</t>
         </is>
       </c>
       <c r="J60" s="6" t="inlineStr">
         <is>
-          <t>유진</t>
+          <t>미래, 삼성</t>
         </is>
       </c>
       <c r="K60" s="6" t="inlineStr">
@@ -3689,12 +3689,12 @@
     <row r="61">
       <c r="A61" s="6" t="inlineStr">
         <is>
-          <t>2026-08-20</t>
+          <t>2026-08-12</t>
         </is>
       </c>
       <c r="B61" s="6" t="inlineStr">
         <is>
-          <t>엘리스그룹</t>
+          <t>진코스텍</t>
         </is>
       </c>
       <c r="C61" s="6" t="inlineStr">
@@ -3704,7 +3704,7 @@
       </c>
       <c r="D61" s="6" t="inlineStr">
         <is>
-          <t>신규상장</t>
+          <t>이전상장</t>
         </is>
       </c>
       <c r="E61" s="6" t="inlineStr">
@@ -3714,27 +3714,27 @@
       </c>
       <c r="F61" s="7" t="inlineStr">
         <is>
-          <t>39,513</t>
+          <t>48,646</t>
         </is>
       </c>
       <c r="G61" s="7" t="inlineStr">
         <is>
-          <t>15,666</t>
+          <t>6,017</t>
         </is>
       </c>
       <c r="H61" s="7" t="inlineStr">
         <is>
-          <t>85,400</t>
+          <t>18,795</t>
         </is>
       </c>
       <c r="I61" s="6" t="inlineStr">
         <is>
-          <t>소프트웨어 개발 및 공급업</t>
+          <t>기타 화학제품 제조업</t>
         </is>
       </c>
       <c r="J61" s="6" t="inlineStr">
         <is>
-          <t>미래, 삼성</t>
+          <t>하나</t>
         </is>
       </c>
       <c r="K61" s="6" t="inlineStr">
@@ -3751,7 +3751,7 @@
       </c>
       <c r="B62" s="6" t="inlineStr">
         <is>
-          <t>진코스텍</t>
+          <t>바로팜</t>
         </is>
       </c>
       <c r="C62" s="6" t="inlineStr">
@@ -3761,7 +3761,7 @@
       </c>
       <c r="D62" s="6" t="inlineStr">
         <is>
-          <t>이전상장</t>
+          <t>신규상장</t>
         </is>
       </c>
       <c r="E62" s="6" t="inlineStr">
@@ -3771,27 +3771,27 @@
       </c>
       <c r="F62" s="7" t="inlineStr">
         <is>
-          <t>48,646</t>
+          <t>96,724</t>
         </is>
       </c>
       <c r="G62" s="7" t="inlineStr">
         <is>
-          <t>6,017</t>
+          <t>-9,679</t>
         </is>
       </c>
       <c r="H62" s="7" t="inlineStr">
         <is>
-          <t>18,795</t>
+          <t>30,673</t>
         </is>
       </c>
       <c r="I62" s="6" t="inlineStr">
         <is>
-          <t>기타 화학제품 제조업</t>
+          <t>상품 중개업</t>
         </is>
       </c>
       <c r="J62" s="6" t="inlineStr">
         <is>
-          <t>하나</t>
+          <t>미래</t>
         </is>
       </c>
       <c r="K62" s="6" t="inlineStr">
@@ -3808,7 +3808,7 @@
       </c>
       <c r="B63" s="6" t="inlineStr">
         <is>
-          <t>바로팜</t>
+          <t>크리에이츠</t>
         </is>
       </c>
       <c r="C63" s="6" t="inlineStr">
@@ -3828,27 +3828,27 @@
       </c>
       <c r="F63" s="7" t="inlineStr">
         <is>
-          <t>96,724</t>
+          <t>76,395</t>
         </is>
       </c>
       <c r="G63" s="7" t="inlineStr">
         <is>
-          <t>-9,679</t>
+          <t>23,749</t>
         </is>
       </c>
       <c r="H63" s="7" t="inlineStr">
         <is>
-          <t>30,673</t>
+          <t>2,335</t>
         </is>
       </c>
       <c r="I63" s="6" t="inlineStr">
         <is>
-          <t>상품 중개업</t>
+          <t>그외 기타 제품 제조업</t>
         </is>
       </c>
       <c r="J63" s="6" t="inlineStr">
         <is>
-          <t>미래</t>
+          <t>삼성</t>
         </is>
       </c>
       <c r="K63" s="6" t="inlineStr">
@@ -3860,12 +3860,12 @@
     <row r="64">
       <c r="A64" s="6" t="inlineStr">
         <is>
-          <t>2026-08-12</t>
+          <t>2026-07-30</t>
         </is>
       </c>
       <c r="B64" s="6" t="inlineStr">
         <is>
-          <t>크리에이츠</t>
+          <t>래블업</t>
         </is>
       </c>
       <c r="C64" s="6" t="inlineStr">
@@ -3885,27 +3885,27 @@
       </c>
       <c r="F64" s="7" t="inlineStr">
         <is>
-          <t>76,395</t>
+          <t>6,712</t>
         </is>
       </c>
       <c r="G64" s="7" t="inlineStr">
         <is>
-          <t>23,749</t>
+          <t>-1,526</t>
         </is>
       </c>
       <c r="H64" s="7" t="inlineStr">
         <is>
-          <t>2,335</t>
+          <t>373</t>
         </is>
       </c>
       <c r="I64" s="6" t="inlineStr">
         <is>
-          <t>그외 기타 제품 제조업</t>
+          <t>데이터베이스 및 온라인정보 제공업</t>
         </is>
       </c>
       <c r="J64" s="6" t="inlineStr">
         <is>
-          <t>삼성</t>
+          <t>NH</t>
         </is>
       </c>
       <c r="K64" s="6" t="inlineStr">
@@ -3922,7 +3922,7 @@
       </c>
       <c r="B65" s="6" t="inlineStr">
         <is>
-          <t>래블업</t>
+          <t>멜콘</t>
         </is>
       </c>
       <c r="C65" s="6" t="inlineStr">
@@ -3942,27 +3942,27 @@
       </c>
       <c r="F65" s="7" t="inlineStr">
         <is>
-          <t>6,712</t>
+          <t>39,319</t>
         </is>
       </c>
       <c r="G65" s="7" t="inlineStr">
         <is>
-          <t>-1,526</t>
+          <t>4,739</t>
         </is>
       </c>
       <c r="H65" s="7" t="inlineStr">
         <is>
-          <t>373</t>
+          <t>1,250</t>
         </is>
       </c>
       <c r="I65" s="6" t="inlineStr">
         <is>
-          <t>데이터베이스 및 온라인정보 제공업</t>
+          <t>특수 목적용 기계 제조업</t>
         </is>
       </c>
       <c r="J65" s="6" t="inlineStr">
         <is>
-          <t>NH</t>
+          <t>대신</t>
         </is>
       </c>
       <c r="K65" s="6" t="inlineStr">
@@ -3979,7 +3979,7 @@
       </c>
       <c r="B66" s="6" t="inlineStr">
         <is>
-          <t>멜콘</t>
+          <t>엠비디</t>
         </is>
       </c>
       <c r="C66" s="6" t="inlineStr">
@@ -3999,27 +3999,27 @@
       </c>
       <c r="F66" s="7" t="inlineStr">
         <is>
-          <t>39,319</t>
+          <t>1,524</t>
         </is>
       </c>
       <c r="G66" s="7" t="inlineStr">
         <is>
-          <t>4,739</t>
+          <t>-2,125</t>
         </is>
       </c>
       <c r="H66" s="7" t="inlineStr">
         <is>
-          <t>1,250</t>
+          <t>2,753</t>
         </is>
       </c>
       <c r="I66" s="6" t="inlineStr">
         <is>
-          <t>특수 목적용 기계 제조업</t>
+          <t>물질 검사, 측정 및 분석기구 제조업</t>
         </is>
       </c>
       <c r="J66" s="6" t="inlineStr">
         <is>
-          <t>대신</t>
+          <t>하나</t>
         </is>
       </c>
       <c r="K66" s="6" t="inlineStr">
@@ -4031,12 +4031,12 @@
     <row r="67">
       <c r="A67" s="6" t="inlineStr">
         <is>
-          <t>2026-07-30</t>
+          <t>2026-07-29</t>
         </is>
       </c>
       <c r="B67" s="6" t="inlineStr">
         <is>
-          <t>엠비디</t>
+          <t>에스케이증권제14호기업인수목적</t>
         </is>
       </c>
       <c r="C67" s="6" t="inlineStr">
@@ -4056,27 +4056,27 @@
       </c>
       <c r="F67" s="7" t="inlineStr">
         <is>
-          <t>1,524</t>
+          <t>-</t>
         </is>
       </c>
       <c r="G67" s="7" t="inlineStr">
         <is>
-          <t>-2,125</t>
+          <t>-</t>
         </is>
       </c>
       <c r="H67" s="7" t="inlineStr">
         <is>
-          <t>2,753</t>
+          <t>17</t>
         </is>
       </c>
       <c r="I67" s="6" t="inlineStr">
         <is>
-          <t>물질 검사, 측정 및 분석기구 제조업</t>
+          <t>기타 금융업</t>
         </is>
       </c>
       <c r="J67" s="6" t="inlineStr">
         <is>
-          <t>하나</t>
+          <t>SK</t>
         </is>
       </c>
       <c r="K67" s="6" t="inlineStr">
@@ -4093,7 +4093,7 @@
       </c>
       <c r="B68" s="6" t="inlineStr">
         <is>
-          <t>에스케이증권제14호기업인수목적</t>
+          <t>케이비제34호스팩</t>
         </is>
       </c>
       <c r="C68" s="6" t="inlineStr">
@@ -4123,7 +4123,7 @@
       </c>
       <c r="H68" s="7" t="inlineStr">
         <is>
-          <t>17</t>
+          <t>21</t>
         </is>
       </c>
       <c r="I68" s="6" t="inlineStr">
@@ -4133,7 +4133,7 @@
       </c>
       <c r="J68" s="6" t="inlineStr">
         <is>
-          <t>SK</t>
+          <t>KB</t>
         </is>
       </c>
       <c r="K68" s="6" t="inlineStr">
@@ -4150,7 +4150,7 @@
       </c>
       <c r="B69" s="6" t="inlineStr">
         <is>
-          <t>케이비제34호스팩</t>
+          <t>한국제17호스팩</t>
         </is>
       </c>
       <c r="C69" s="6" t="inlineStr">
@@ -4180,7 +4180,7 @@
       </c>
       <c r="H69" s="7" t="inlineStr">
         <is>
-          <t>21</t>
+          <t>170</t>
         </is>
       </c>
       <c r="I69" s="6" t="inlineStr">
@@ -4190,7 +4190,7 @@
       </c>
       <c r="J69" s="6" t="inlineStr">
         <is>
-          <t>KB</t>
+          <t>한국</t>
         </is>
       </c>
       <c r="K69" s="6" t="inlineStr">
@@ -4207,7 +4207,7 @@
       </c>
       <c r="B70" s="6" t="inlineStr">
         <is>
-          <t>한국제17호스팩</t>
+          <t>한화플러스제6호스팩</t>
         </is>
       </c>
       <c r="C70" s="6" t="inlineStr">
@@ -4237,7 +4237,7 @@
       </c>
       <c r="H70" s="7" t="inlineStr">
         <is>
-          <t>170</t>
+          <t>41</t>
         </is>
       </c>
       <c r="I70" s="6" t="inlineStr">
@@ -4247,7 +4247,7 @@
       </c>
       <c r="J70" s="6" t="inlineStr">
         <is>
-          <t>한국</t>
+          <t>한화</t>
         </is>
       </c>
       <c r="K70" s="6" t="inlineStr">
@@ -4259,12 +4259,12 @@
     <row r="71">
       <c r="A71" s="6" t="inlineStr">
         <is>
-          <t>2026-07-29</t>
+          <t>2026-07-22</t>
         </is>
       </c>
       <c r="B71" s="6" t="inlineStr">
         <is>
-          <t>한화플러스제6호스팩</t>
+          <t>엔에이치스팩34호</t>
         </is>
       </c>
       <c r="C71" s="6" t="inlineStr">
@@ -4294,17 +4294,17 @@
       </c>
       <c r="H71" s="7" t="inlineStr">
         <is>
-          <t>41</t>
+          <t>55</t>
         </is>
       </c>
       <c r="I71" s="6" t="inlineStr">
         <is>
-          <t>기타 금융업</t>
+          <t>금융 지원 서비스업</t>
         </is>
       </c>
       <c r="J71" s="6" t="inlineStr">
         <is>
-          <t>한화</t>
+          <t>NH</t>
         </is>
       </c>
       <c r="K71" s="6" t="inlineStr">
@@ -4316,12 +4316,12 @@
     <row r="72">
       <c r="A72" s="6" t="inlineStr">
         <is>
-          <t>2026-07-22</t>
+          <t>2026-07-20</t>
         </is>
       </c>
       <c r="B72" s="6" t="inlineStr">
         <is>
-          <t>엔에이치스팩34호</t>
+          <t>글로벌테크놀로지</t>
         </is>
       </c>
       <c r="C72" s="6" t="inlineStr">
@@ -4341,27 +4341,27 @@
       </c>
       <c r="F72" s="7" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>29,689</t>
         </is>
       </c>
       <c r="G72" s="7" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>-25,889</t>
         </is>
       </c>
       <c r="H72" s="7" t="inlineStr">
         <is>
-          <t>55</t>
+          <t>6,402</t>
         </is>
       </c>
       <c r="I72" s="6" t="inlineStr">
         <is>
-          <t>금융 지원 서비스업</t>
+          <t>반도체 제조업</t>
         </is>
       </c>
       <c r="J72" s="6" t="inlineStr">
         <is>
-          <t>NH</t>
+          <t>한국</t>
         </is>
       </c>
       <c r="K72" s="6" t="inlineStr">
@@ -4378,7 +4378,7 @@
       </c>
       <c r="B73" s="6" t="inlineStr">
         <is>
-          <t>글로벌테크놀로지</t>
+          <t>덕산넵코어스</t>
         </is>
       </c>
       <c r="C73" s="6" t="inlineStr">
@@ -4393,32 +4393,32 @@
       </c>
       <c r="E73" s="6" t="inlineStr">
         <is>
-          <t>FY25</t>
+          <t>FY24</t>
         </is>
       </c>
       <c r="F73" s="7" t="inlineStr">
         <is>
-          <t>29,689</t>
+          <t>48,504</t>
         </is>
       </c>
       <c r="G73" s="7" t="inlineStr">
         <is>
-          <t>-25,889</t>
+          <t>3,668</t>
         </is>
       </c>
       <c r="H73" s="7" t="inlineStr">
         <is>
-          <t>6,402</t>
+          <t>8,448</t>
         </is>
       </c>
       <c r="I73" s="6" t="inlineStr">
         <is>
-          <t>반도체 제조업</t>
+          <t>항공기,우주선 및 부품 제조업</t>
         </is>
       </c>
       <c r="J73" s="6" t="inlineStr">
         <is>
-          <t>한국</t>
+          <t>대신</t>
         </is>
       </c>
       <c r="K73" s="6" t="inlineStr">
@@ -4435,7 +4435,7 @@
       </c>
       <c r="B74" s="6" t="inlineStr">
         <is>
-          <t>덕산넵코어스</t>
+          <t>디티에스</t>
         </is>
       </c>
       <c r="C74" s="6" t="inlineStr">
@@ -4455,22 +4455,22 @@
       </c>
       <c r="F74" s="7" t="inlineStr">
         <is>
-          <t>48,504</t>
+          <t>142,718</t>
         </is>
       </c>
       <c r="G74" s="7" t="inlineStr">
         <is>
-          <t>3,668</t>
+          <t>18,765</t>
         </is>
       </c>
       <c r="H74" s="7" t="inlineStr">
         <is>
-          <t>8,448</t>
+          <t>63,153</t>
         </is>
       </c>
       <c r="I74" s="6" t="inlineStr">
         <is>
-          <t>항공기,우주선 및 부품 제조업</t>
+          <t>특수 목적용 기계 제조업</t>
         </is>
       </c>
       <c r="J74" s="6" t="inlineStr">
@@ -4487,12 +4487,12 @@
     <row r="75">
       <c r="A75" s="6" t="inlineStr">
         <is>
-          <t>2026-07-20</t>
+          <t>2026-07-10</t>
         </is>
       </c>
       <c r="B75" s="6" t="inlineStr">
         <is>
-          <t>디티에스</t>
+          <t>네오사피엔스</t>
         </is>
       </c>
       <c r="C75" s="6" t="inlineStr">
@@ -4507,27 +4507,27 @@
       </c>
       <c r="E75" s="6" t="inlineStr">
         <is>
-          <t>FY24</t>
+          <t>FY25</t>
         </is>
       </c>
       <c r="F75" s="7" t="inlineStr">
         <is>
-          <t>142,718</t>
+          <t>10,649</t>
         </is>
       </c>
       <c r="G75" s="7" t="inlineStr">
         <is>
-          <t>18,765</t>
+          <t>-6,994</t>
         </is>
       </c>
       <c r="H75" s="7" t="inlineStr">
         <is>
-          <t>63,153</t>
+          <t>-39,962</t>
         </is>
       </c>
       <c r="I75" s="6" t="inlineStr">
         <is>
-          <t>특수 목적용 기계 제조업</t>
+          <t>소프트웨어 개발 및 공급업</t>
         </is>
       </c>
       <c r="J75" s="6" t="inlineStr">
@@ -4549,7 +4549,7 @@
       </c>
       <c r="B76" s="6" t="inlineStr">
         <is>
-          <t>네오사피엔스</t>
+          <t>엠에스바이오</t>
         </is>
       </c>
       <c r="C76" s="6" t="inlineStr">
@@ -4569,27 +4569,27 @@
       </c>
       <c r="F76" s="7" t="inlineStr">
         <is>
-          <t>10,649</t>
+          <t>23,787</t>
         </is>
       </c>
       <c r="G76" s="7" t="inlineStr">
         <is>
-          <t>-6,994</t>
+          <t>7,288</t>
         </is>
       </c>
       <c r="H76" s="7" t="inlineStr">
         <is>
-          <t>-39,962</t>
+          <t>1,942</t>
         </is>
       </c>
       <c r="I76" s="6" t="inlineStr">
         <is>
-          <t>소프트웨어 개발 및 공급업</t>
+          <t>의료용 기기 제조업</t>
         </is>
       </c>
       <c r="J76" s="6" t="inlineStr">
         <is>
-          <t>대신</t>
+          <t>KB</t>
         </is>
       </c>
       <c r="K76" s="6" t="inlineStr">
@@ -4601,12 +4601,12 @@
     <row r="77">
       <c r="A77" s="6" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
+          <t>2026-06-25</t>
         </is>
       </c>
       <c r="B77" s="6" t="inlineStr">
         <is>
-          <t>엠에스바이오</t>
+          <t>기도산업</t>
         </is>
       </c>
       <c r="C77" s="6" t="inlineStr">
@@ -4626,32 +4626,32 @@
       </c>
       <c r="F77" s="7" t="inlineStr">
         <is>
-          <t>23,787</t>
+          <t>346,551</t>
         </is>
       </c>
       <c r="G77" s="7" t="inlineStr">
         <is>
-          <t>7,288</t>
+          <t>35,334</t>
         </is>
       </c>
       <c r="H77" s="7" t="inlineStr">
         <is>
-          <t>1,942</t>
+          <t>145,991</t>
         </is>
       </c>
       <c r="I77" s="6" t="inlineStr">
         <is>
-          <t>의료용 기기 제조업</t>
+          <t>봉제의복 제조업</t>
         </is>
       </c>
       <c r="J77" s="6" t="inlineStr">
         <is>
-          <t>KB</t>
+          <t>미래</t>
         </is>
       </c>
       <c r="K77" s="6" t="inlineStr">
         <is>
-          <t>상장전</t>
+          <t>상장완료 (2026-08-21)</t>
         </is>
       </c>
     </row>
@@ -4663,7 +4663,7 @@
       </c>
       <c r="B78" s="6" t="inlineStr">
         <is>
-          <t>기도산업</t>
+          <t>브릴스</t>
         </is>
       </c>
       <c r="C78" s="6" t="inlineStr">
@@ -4683,32 +4683,32 @@
       </c>
       <c r="F78" s="7" t="inlineStr">
         <is>
-          <t>346,551</t>
+          <t>23,759</t>
         </is>
       </c>
       <c r="G78" s="7" t="inlineStr">
         <is>
-          <t>35,334</t>
+          <t>1,744</t>
         </is>
       </c>
       <c r="H78" s="7" t="inlineStr">
         <is>
-          <t>145,991</t>
+          <t>4,785</t>
         </is>
       </c>
       <c r="I78" s="6" t="inlineStr">
         <is>
-          <t>봉제의복 제조업</t>
+          <t>특수 목적용 기계 제조업</t>
         </is>
       </c>
       <c r="J78" s="6" t="inlineStr">
         <is>
-          <t>미래</t>
+          <t>IBK</t>
         </is>
       </c>
       <c r="K78" s="6" t="inlineStr">
         <is>
-          <t>상장완료 (2026-08-21)</t>
+          <t>상장전</t>
         </is>
       </c>
     </row>
@@ -4720,7 +4720,7 @@
       </c>
       <c r="B79" s="6" t="inlineStr">
         <is>
-          <t>브릴스</t>
+          <t>와이즈플래닛컴퍼니</t>
         </is>
       </c>
       <c r="C79" s="6" t="inlineStr">
@@ -4740,27 +4740,27 @@
       </c>
       <c r="F79" s="7" t="inlineStr">
         <is>
-          <t>23,759</t>
+          <t>44,578</t>
         </is>
       </c>
       <c r="G79" s="7" t="inlineStr">
         <is>
-          <t>1,744</t>
+          <t>7,748</t>
         </is>
       </c>
       <c r="H79" s="7" t="inlineStr">
         <is>
-          <t>4,785</t>
+          <t>959</t>
         </is>
       </c>
       <c r="I79" s="6" t="inlineStr">
         <is>
-          <t>특수 목적용 기계 제조업</t>
+          <t>광고물 문안, 도안, 설계 등 작성업</t>
         </is>
       </c>
       <c r="J79" s="6" t="inlineStr">
         <is>
-          <t>IBK</t>
+          <t>대신</t>
         </is>
       </c>
       <c r="K79" s="6" t="inlineStr">
@@ -4772,12 +4772,12 @@
     <row r="80">
       <c r="A80" s="6" t="inlineStr">
         <is>
-          <t>2026-06-25</t>
+          <t>2026-06-24</t>
         </is>
       </c>
       <c r="B80" s="6" t="inlineStr">
         <is>
-          <t>와이즈플래닛컴퍼니</t>
+          <t>니어스랩</t>
         </is>
       </c>
       <c r="C80" s="6" t="inlineStr">
@@ -4797,32 +4797,32 @@
       </c>
       <c r="F80" s="7" t="inlineStr">
         <is>
-          <t>44,578</t>
+          <t>6,361</t>
         </is>
       </c>
       <c r="G80" s="7" t="inlineStr">
         <is>
-          <t>7,748</t>
+          <t>-7,287</t>
         </is>
       </c>
       <c r="H80" s="7" t="inlineStr">
         <is>
-          <t>959</t>
+          <t>127</t>
         </is>
       </c>
       <c r="I80" s="6" t="inlineStr">
         <is>
-          <t>광고물 문안, 도안, 설계 등 작성업</t>
+          <t>소프트웨어 개발 및 공급업</t>
         </is>
       </c>
       <c r="J80" s="6" t="inlineStr">
         <is>
-          <t>대신</t>
+          <t>삼성</t>
         </is>
       </c>
       <c r="K80" s="6" t="inlineStr">
         <is>
-          <t>상장전</t>
+          <t>상장완료 (2026-08-24)</t>
         </is>
       </c>
     </row>
@@ -4834,7 +4834,7 @@
       </c>
       <c r="B81" s="6" t="inlineStr">
         <is>
-          <t>니어스랩</t>
+          <t>해치텍</t>
         </is>
       </c>
       <c r="C81" s="6" t="inlineStr">
@@ -4854,32 +4854,32 @@
       </c>
       <c r="F81" s="7" t="inlineStr">
         <is>
-          <t>6,361</t>
+          <t>14,079</t>
         </is>
       </c>
       <c r="G81" s="7" t="inlineStr">
         <is>
-          <t>-7,287</t>
+          <t>-8,009</t>
         </is>
       </c>
       <c r="H81" s="7" t="inlineStr">
         <is>
-          <t>127</t>
+          <t>2,229</t>
         </is>
       </c>
       <c r="I81" s="6" t="inlineStr">
         <is>
-          <t>소프트웨어 개발 및 공급업</t>
+          <t>반도체 제조업</t>
         </is>
       </c>
       <c r="J81" s="6" t="inlineStr">
         <is>
-          <t>삼성</t>
+          <t>DB</t>
         </is>
       </c>
       <c r="K81" s="6" t="inlineStr">
         <is>
-          <t>상장완료 (2026-08-24)</t>
+          <t>상장완료 (2026-08-25)</t>
         </is>
       </c>
     </row>
@@ -4891,7 +4891,7 @@
       </c>
       <c r="B82" s="6" t="inlineStr">
         <is>
-          <t>해치텍</t>
+          <t>스카이랩스</t>
         </is>
       </c>
       <c r="C82" s="6" t="inlineStr">
@@ -4911,44 +4911,44 @@
       </c>
       <c r="F82" s="7" t="inlineStr">
         <is>
-          <t>14,079</t>
+          <t>7,936</t>
         </is>
       </c>
       <c r="G82" s="7" t="inlineStr">
         <is>
-          <t>-8,009</t>
+          <t>-62,995</t>
         </is>
       </c>
       <c r="H82" s="7" t="inlineStr">
         <is>
-          <t>2,229</t>
+          <t>8,341</t>
         </is>
       </c>
       <c r="I82" s="6" t="inlineStr">
         <is>
-          <t>반도체 제조업</t>
+          <t>의료용 기기 제조업</t>
         </is>
       </c>
       <c r="J82" s="6" t="inlineStr">
         <is>
-          <t>DB</t>
+          <t>한국</t>
         </is>
       </c>
       <c r="K82" s="6" t="inlineStr">
         <is>
-          <t>상장완료 (2026-08-25)</t>
+          <t>상장전</t>
         </is>
       </c>
     </row>
     <row r="83">
       <c r="A83" s="6" t="inlineStr">
         <is>
-          <t>2026-06-24</t>
+          <t>2026-06-15</t>
         </is>
       </c>
       <c r="B83" s="6" t="inlineStr">
         <is>
-          <t>스카이랩스</t>
+          <t>에이치엘지노믹스</t>
         </is>
       </c>
       <c r="C83" s="6" t="inlineStr">
@@ -4968,32 +4968,32 @@
       </c>
       <c r="F83" s="7" t="inlineStr">
         <is>
-          <t>7,936</t>
+          <t>28,877</t>
         </is>
       </c>
       <c r="G83" s="7" t="inlineStr">
         <is>
-          <t>-62,995</t>
+          <t>8,452</t>
         </is>
       </c>
       <c r="H83" s="7" t="inlineStr">
         <is>
-          <t>8,341</t>
+          <t>83,552</t>
         </is>
       </c>
       <c r="I83" s="6" t="inlineStr">
         <is>
-          <t>의료용 기기 제조업</t>
+          <t>기초 의약물질 제조업</t>
         </is>
       </c>
       <c r="J83" s="6" t="inlineStr">
         <is>
-          <t>한국</t>
+          <t>KB, IBK</t>
         </is>
       </c>
       <c r="K83" s="6" t="inlineStr">
         <is>
-          <t>상장전</t>
+          <t>상장완료 (2026-07-24)</t>
         </is>
       </c>
     </row>
@@ -5005,7 +5005,7 @@
       </c>
       <c r="B84" s="6" t="inlineStr">
         <is>
-          <t>에이치엘지노믹스</t>
+          <t>딜리셔스</t>
         </is>
       </c>
       <c r="C84" s="6" t="inlineStr">
@@ -5025,44 +5025,44 @@
       </c>
       <c r="F84" s="7" t="inlineStr">
         <is>
-          <t>28,877</t>
+          <t>25,149</t>
         </is>
       </c>
       <c r="G84" s="7" t="inlineStr">
         <is>
-          <t>8,452</t>
+          <t>-20,419</t>
         </is>
       </c>
       <c r="H84" s="7" t="inlineStr">
         <is>
-          <t>83,552</t>
+          <t>-114,384</t>
         </is>
       </c>
       <c r="I84" s="6" t="inlineStr">
         <is>
-          <t>기초 의약물질 제조업</t>
+          <t>무점포 소매업</t>
         </is>
       </c>
       <c r="J84" s="6" t="inlineStr">
         <is>
-          <t>KB, IBK</t>
+          <t>한국</t>
         </is>
       </c>
       <c r="K84" s="6" t="inlineStr">
         <is>
-          <t>상장완료 (2026-07-24)</t>
+          <t>상장완료 (2026-08-12)</t>
         </is>
       </c>
     </row>
     <row r="85">
       <c r="A85" s="6" t="inlineStr">
         <is>
-          <t>2026-06-15</t>
+          <t>2026-05-21</t>
         </is>
       </c>
       <c r="B85" s="6" t="inlineStr">
         <is>
-          <t>딜리셔스</t>
+          <t>인제니아테라퓨틱스</t>
         </is>
       </c>
       <c r="C85" s="6" t="inlineStr">
@@ -5082,44 +5082,44 @@
       </c>
       <c r="F85" s="7" t="inlineStr">
         <is>
-          <t>25,149</t>
+          <t>2,588,400</t>
         </is>
       </c>
       <c r="G85" s="7" t="inlineStr">
         <is>
-          <t>-20,419</t>
+          <t>15,755,864</t>
         </is>
       </c>
       <c r="H85" s="7" t="inlineStr">
         <is>
-          <t>-114,384</t>
+          <t>30,841,690</t>
         </is>
       </c>
       <c r="I85" s="6" t="inlineStr">
         <is>
-          <t>무점포 소매업</t>
+          <t>자연과학 및 공학 연구개발업</t>
         </is>
       </c>
       <c r="J85" s="6" t="inlineStr">
         <is>
-          <t>한국</t>
+          <t>삼성</t>
         </is>
       </c>
       <c r="K85" s="6" t="inlineStr">
         <is>
-          <t>상장완료 (2026-08-12)</t>
+          <t>상장완료 (2026-08-18)</t>
         </is>
       </c>
     </row>
     <row r="86">
       <c r="A86" s="6" t="inlineStr">
         <is>
-          <t>2026-05-21</t>
+          <t>2026-05-20</t>
         </is>
       </c>
       <c r="B86" s="6" t="inlineStr">
         <is>
-          <t>인제니아테라퓨틱스</t>
+          <t>한국제16호스팩</t>
         </is>
       </c>
       <c r="C86" s="6" t="inlineStr">
@@ -5137,46 +5137,30 @@
           <t>FY25</t>
         </is>
       </c>
-      <c r="F86" s="7" t="inlineStr">
-        <is>
-          <t>2,588,400</t>
-        </is>
-      </c>
-      <c r="G86" s="7" t="inlineStr">
-        <is>
-          <t>15,755,864</t>
-        </is>
-      </c>
-      <c r="H86" s="7" t="inlineStr">
-        <is>
-          <t>30,841,690</t>
-        </is>
-      </c>
-      <c r="I86" s="6" t="inlineStr">
-        <is>
-          <t>자연과학 및 공학 연구개발업</t>
-        </is>
-      </c>
+      <c r="F86" s="7" t="inlineStr"/>
+      <c r="G86" s="7" t="inlineStr"/>
+      <c r="H86" s="7" t="inlineStr"/>
+      <c r="I86" s="6" t="inlineStr"/>
       <c r="J86" s="6" t="inlineStr">
         <is>
-          <t>삼성</t>
+          <t>한국</t>
         </is>
       </c>
       <c r="K86" s="6" t="inlineStr">
         <is>
-          <t>상장완료 (2026-08-18)</t>
+          <t>상장완료 (2026-06-30)</t>
         </is>
       </c>
     </row>
     <row r="87">
       <c r="A87" s="6" t="inlineStr">
         <is>
-          <t>2026-05-20</t>
+          <t>2026-05-07</t>
         </is>
       </c>
       <c r="B87" s="6" t="inlineStr">
         <is>
-          <t>한국제16호스팩</t>
+          <t>레메디</t>
         </is>
       </c>
       <c r="C87" s="6" t="inlineStr">
@@ -5194,18 +5178,34 @@
           <t>FY25</t>
         </is>
       </c>
-      <c r="F87" s="7" t="inlineStr"/>
-      <c r="G87" s="7" t="inlineStr"/>
-      <c r="H87" s="7" t="inlineStr"/>
-      <c r="I87" s="6" t="inlineStr"/>
+      <c r="F87" s="7" t="inlineStr">
+        <is>
+          <t>13,441</t>
+        </is>
+      </c>
+      <c r="G87" s="7" t="inlineStr">
+        <is>
+          <t>741</t>
+        </is>
+      </c>
+      <c r="H87" s="7" t="inlineStr">
+        <is>
+          <t>5,870</t>
+        </is>
+      </c>
+      <c r="I87" s="6" t="inlineStr">
+        <is>
+          <t>의료용 기기 제조업</t>
+        </is>
+      </c>
       <c r="J87" s="6" t="inlineStr">
         <is>
-          <t>한국</t>
+          <t>KB</t>
         </is>
       </c>
       <c r="K87" s="6" t="inlineStr">
         <is>
-          <t>상장완료 (2026-06-30)</t>
+          <t>상장완료 (2026-07-13)</t>
         </is>
       </c>
     </row>
@@ -5217,7 +5217,7 @@
       </c>
       <c r="B88" s="6" t="inlineStr">
         <is>
-          <t>레메디</t>
+          <t>케이앤에스아이앤씨</t>
         </is>
       </c>
       <c r="C88" s="6" t="inlineStr">
@@ -5237,44 +5237,44 @@
       </c>
       <c r="F88" s="7" t="inlineStr">
         <is>
-          <t>13,441</t>
+          <t>13,482</t>
         </is>
       </c>
       <c r="G88" s="7" t="inlineStr">
         <is>
-          <t>741</t>
+          <t>-2,213</t>
         </is>
       </c>
       <c r="H88" s="7" t="inlineStr">
         <is>
-          <t>5,870</t>
+          <t>4,273</t>
         </is>
       </c>
       <c r="I88" s="6" t="inlineStr">
         <is>
-          <t>의료용 기기 제조업</t>
+          <t>통신 및 방송 장비 제조업</t>
         </is>
       </c>
       <c r="J88" s="6" t="inlineStr">
         <is>
-          <t>KB</t>
+          <t>IBK</t>
         </is>
       </c>
       <c r="K88" s="6" t="inlineStr">
         <is>
-          <t>상장완료 (2026-07-13)</t>
+          <t>상장완료 (2026-08-13)</t>
         </is>
       </c>
     </row>
     <row r="89">
       <c r="A89" s="6" t="inlineStr">
         <is>
-          <t>2026-05-07</t>
+          <t>2026-04-27</t>
         </is>
       </c>
       <c r="B89" s="6" t="inlineStr">
         <is>
-          <t>케이앤에스아이앤씨</t>
+          <t>메리츠제2호스팩</t>
         </is>
       </c>
       <c r="C89" s="6" t="inlineStr">
@@ -5292,46 +5292,30 @@
           <t>FY25</t>
         </is>
       </c>
-      <c r="F89" s="7" t="inlineStr">
-        <is>
-          <t>13,482</t>
-        </is>
-      </c>
-      <c r="G89" s="7" t="inlineStr">
-        <is>
-          <t>-2,213</t>
-        </is>
-      </c>
-      <c r="H89" s="7" t="inlineStr">
-        <is>
-          <t>4,273</t>
-        </is>
-      </c>
-      <c r="I89" s="6" t="inlineStr">
-        <is>
-          <t>통신 및 방송 장비 제조업</t>
-        </is>
-      </c>
+      <c r="F89" s="7" t="inlineStr"/>
+      <c r="G89" s="7" t="inlineStr"/>
+      <c r="H89" s="7" t="inlineStr"/>
+      <c r="I89" s="6" t="inlineStr"/>
       <c r="J89" s="6" t="inlineStr">
         <is>
-          <t>IBK</t>
+          <t>메리츠</t>
         </is>
       </c>
       <c r="K89" s="6" t="inlineStr">
         <is>
-          <t>상장완료 (2026-08-13)</t>
+          <t>상장완료 (2026-06-19)</t>
         </is>
       </c>
     </row>
     <row r="90">
       <c r="A90" s="6" t="inlineStr">
         <is>
-          <t>2026-04-27</t>
+          <t>2026-04-23</t>
         </is>
       </c>
       <c r="B90" s="6" t="inlineStr">
         <is>
-          <t>메리츠제2호스팩</t>
+          <t>빅웨이브로보틱스</t>
         </is>
       </c>
       <c r="C90" s="6" t="inlineStr">
@@ -5346,33 +5330,49 @@
       </c>
       <c r="E90" s="6" t="inlineStr">
         <is>
-          <t>FY25</t>
-        </is>
-      </c>
-      <c r="F90" s="7" t="inlineStr"/>
-      <c r="G90" s="7" t="inlineStr"/>
-      <c r="H90" s="7" t="inlineStr"/>
-      <c r="I90" s="6" t="inlineStr"/>
+          <t>FY24</t>
+        </is>
+      </c>
+      <c r="F90" s="7" t="inlineStr">
+        <is>
+          <t>13,851</t>
+        </is>
+      </c>
+      <c r="G90" s="7" t="inlineStr">
+        <is>
+          <t>-5,856</t>
+        </is>
+      </c>
+      <c r="H90" s="7" t="inlineStr">
+        <is>
+          <t>9,470</t>
+        </is>
+      </c>
+      <c r="I90" s="6" t="inlineStr">
+        <is>
+          <t>소프트웨어 개발 및 공급업</t>
+        </is>
+      </c>
       <c r="J90" s="6" t="inlineStr">
         <is>
-          <t>메리츠</t>
+          <t>유진, 미래</t>
         </is>
       </c>
       <c r="K90" s="6" t="inlineStr">
         <is>
-          <t>상장완료 (2026-06-19)</t>
+          <t>상장전</t>
         </is>
       </c>
     </row>
     <row r="91">
       <c r="A91" s="6" t="inlineStr">
         <is>
-          <t>2026-04-23</t>
+          <t>2026-04-09</t>
         </is>
       </c>
       <c r="B91" s="6" t="inlineStr">
         <is>
-          <t>빅웨이브로보틱스</t>
+          <t>매드업</t>
         </is>
       </c>
       <c r="C91" s="6" t="inlineStr">
@@ -5392,44 +5392,44 @@
       </c>
       <c r="F91" s="7" t="inlineStr">
         <is>
-          <t>13,851</t>
+          <t>34,989</t>
         </is>
       </c>
       <c r="G91" s="7" t="inlineStr">
         <is>
-          <t>-5,856</t>
+          <t>-2,747</t>
         </is>
       </c>
       <c r="H91" s="7" t="inlineStr">
         <is>
-          <t>9,470</t>
+          <t>-15,766</t>
         </is>
       </c>
       <c r="I91" s="6" t="inlineStr">
         <is>
-          <t>소프트웨어 개발 및 공급업</t>
+          <t>광고</t>
         </is>
       </c>
       <c r="J91" s="6" t="inlineStr">
         <is>
-          <t>유진, 미래</t>
+          <t>미래</t>
         </is>
       </c>
       <c r="K91" s="6" t="inlineStr">
         <is>
-          <t>상장전</t>
+          <t>상장완료 (2026-07-01)</t>
         </is>
       </c>
     </row>
     <row r="92">
       <c r="A92" s="6" t="inlineStr">
         <is>
-          <t>2026-04-09</t>
+          <t>2026-04-02</t>
         </is>
       </c>
       <c r="B92" s="6" t="inlineStr">
         <is>
-          <t>매드업</t>
+          <t>져스텍</t>
         </is>
       </c>
       <c r="C92" s="6" t="inlineStr">
@@ -5449,32 +5449,32 @@
       </c>
       <c r="F92" s="7" t="inlineStr">
         <is>
-          <t>34,989</t>
+          <t>19,851</t>
         </is>
       </c>
       <c r="G92" s="7" t="inlineStr">
         <is>
-          <t>-2,747</t>
+          <t>444</t>
         </is>
       </c>
       <c r="H92" s="7" t="inlineStr">
         <is>
-          <t>-15,766</t>
+          <t>10,953</t>
         </is>
       </c>
       <c r="I92" s="6" t="inlineStr">
         <is>
-          <t>광고</t>
+          <t>기계</t>
         </is>
       </c>
       <c r="J92" s="6" t="inlineStr">
         <is>
-          <t>미래</t>
+          <t>삼성</t>
         </is>
       </c>
       <c r="K92" s="6" t="inlineStr">
         <is>
-          <t>상장완료 (2026-07-01)</t>
+          <t>상장완료 (2026-06-29)</t>
         </is>
       </c>
     </row>
@@ -5486,7 +5486,7 @@
       </c>
       <c r="B93" s="6" t="inlineStr">
         <is>
-          <t>져스텍</t>
+          <t>스트라드비젼</t>
         </is>
       </c>
       <c r="C93" s="6" t="inlineStr">
@@ -5506,44 +5506,44 @@
       </c>
       <c r="F93" s="7" t="inlineStr">
         <is>
-          <t>19,851</t>
+          <t>11,539</t>
         </is>
       </c>
       <c r="G93" s="7" t="inlineStr">
         <is>
-          <t>444</t>
+          <t>-65,529</t>
         </is>
       </c>
       <c r="H93" s="7" t="inlineStr">
         <is>
-          <t>10,953</t>
+          <t>-245,151</t>
         </is>
       </c>
       <c r="I93" s="6" t="inlineStr">
         <is>
-          <t>기계</t>
+          <t>소프트웨어</t>
         </is>
       </c>
       <c r="J93" s="6" t="inlineStr">
         <is>
-          <t>삼성</t>
+          <t>KB</t>
         </is>
       </c>
       <c r="K93" s="6" t="inlineStr">
         <is>
-          <t>상장완료 (2026-06-29)</t>
+          <t>상장완료 (2026-06-30)</t>
         </is>
       </c>
     </row>
     <row r="94">
       <c r="A94" s="6" t="inlineStr">
         <is>
-          <t>2026-04-02</t>
+          <t>2026-03-30</t>
         </is>
       </c>
       <c r="B94" s="6" t="inlineStr">
         <is>
-          <t>스트라드비젼</t>
+          <t>대신밸런스제20호스팩</t>
         </is>
       </c>
       <c r="C94" s="6" t="inlineStr">
@@ -5558,49 +5558,33 @@
       </c>
       <c r="E94" s="6" t="inlineStr">
         <is>
-          <t>FY24</t>
-        </is>
-      </c>
-      <c r="F94" s="7" t="inlineStr">
-        <is>
-          <t>11,539</t>
-        </is>
-      </c>
-      <c r="G94" s="7" t="inlineStr">
-        <is>
-          <t>-65,529</t>
-        </is>
-      </c>
-      <c r="H94" s="7" t="inlineStr">
-        <is>
-          <t>-245,151</t>
-        </is>
-      </c>
-      <c r="I94" s="6" t="inlineStr">
-        <is>
-          <t>소프트웨어</t>
-        </is>
-      </c>
+          <t>FY25</t>
+        </is>
+      </c>
+      <c r="F94" s="7" t="inlineStr"/>
+      <c r="G94" s="7" t="inlineStr"/>
+      <c r="H94" s="7" t="inlineStr"/>
+      <c r="I94" s="6" t="inlineStr"/>
       <c r="J94" s="6" t="inlineStr">
         <is>
-          <t>KB</t>
+          <t>대신</t>
         </is>
       </c>
       <c r="K94" s="6" t="inlineStr">
         <is>
-          <t>상장완료 (2026-06-30)</t>
+          <t>상장완료 (2026-06-05)</t>
         </is>
       </c>
     </row>
     <row r="95">
       <c r="A95" s="6" t="inlineStr">
         <is>
-          <t>2026-03-30</t>
+          <t>2026-03-26</t>
         </is>
       </c>
       <c r="B95" s="6" t="inlineStr">
         <is>
-          <t>대신밸런스제20호스팩</t>
+          <t>피스피스스튜디오</t>
         </is>
       </c>
       <c r="C95" s="6" t="inlineStr">
@@ -5615,21 +5599,37 @@
       </c>
       <c r="E95" s="6" t="inlineStr">
         <is>
-          <t>FY25</t>
-        </is>
-      </c>
-      <c r="F95" s="7" t="inlineStr"/>
-      <c r="G95" s="7" t="inlineStr"/>
-      <c r="H95" s="7" t="inlineStr"/>
-      <c r="I95" s="6" t="inlineStr"/>
+          <t>FY24</t>
+        </is>
+      </c>
+      <c r="F95" s="7" t="inlineStr">
+        <is>
+          <t>113,777</t>
+        </is>
+      </c>
+      <c r="G95" s="7" t="inlineStr">
+        <is>
+          <t>17,603</t>
+        </is>
+      </c>
+      <c r="H95" s="7" t="inlineStr">
+        <is>
+          <t>55,861</t>
+        </is>
+      </c>
+      <c r="I95" s="6" t="inlineStr">
+        <is>
+          <t>섬유,의류,신발,호화품</t>
+        </is>
+      </c>
       <c r="J95" s="6" t="inlineStr">
         <is>
-          <t>대신</t>
+          <t>NH, 미래</t>
         </is>
       </c>
       <c r="K95" s="6" t="inlineStr">
         <is>
-          <t>상장완료 (2026-06-05)</t>
+          <t>상장완료 (2026-06-08)</t>
         </is>
       </c>
     </row>
@@ -5641,7 +5641,7 @@
       </c>
       <c r="B96" s="6" t="inlineStr">
         <is>
-          <t>피스피스스튜디오</t>
+          <t>폴레드</t>
         </is>
       </c>
       <c r="C96" s="6" t="inlineStr">
@@ -5661,32 +5661,32 @@
       </c>
       <c r="F96" s="7" t="inlineStr">
         <is>
-          <t>113,777</t>
+          <t>52,808</t>
         </is>
       </c>
       <c r="G96" s="7" t="inlineStr">
         <is>
-          <t>17,603</t>
+          <t>543</t>
         </is>
       </c>
       <c r="H96" s="7" t="inlineStr">
         <is>
-          <t>55,861</t>
+          <t>25,416</t>
         </is>
       </c>
       <c r="I96" s="6" t="inlineStr">
         <is>
-          <t>섬유,의류,신발,호화품</t>
+          <t>가정용기기와용품</t>
         </is>
       </c>
       <c r="J96" s="6" t="inlineStr">
         <is>
-          <t>NH, 미래</t>
+          <t>NH</t>
         </is>
       </c>
       <c r="K96" s="6" t="inlineStr">
         <is>
-          <t>상장완료 (2026-06-08)</t>
+          <t>상장완료 (2026-05-14)</t>
         </is>
       </c>
     </row>
@@ -5698,7 +5698,7 @@
       </c>
       <c r="B97" s="6" t="inlineStr">
         <is>
-          <t>폴레드</t>
+          <t>레몬헬스케어</t>
         </is>
       </c>
       <c r="C97" s="6" t="inlineStr">
@@ -5718,44 +5718,44 @@
       </c>
       <c r="F97" s="7" t="inlineStr">
         <is>
-          <t>52,808</t>
+          <t>14,877</t>
         </is>
       </c>
       <c r="G97" s="7" t="inlineStr">
         <is>
-          <t>543</t>
+          <t>-2,898</t>
         </is>
       </c>
       <c r="H97" s="7" t="inlineStr">
         <is>
-          <t>25,416</t>
+          <t>-31,162</t>
         </is>
       </c>
       <c r="I97" s="6" t="inlineStr">
         <is>
-          <t>가정용기기와용품</t>
+          <t>건강관리업체및서비스</t>
         </is>
       </c>
       <c r="J97" s="6" t="inlineStr">
         <is>
-          <t>NH</t>
+          <t>KB</t>
         </is>
       </c>
       <c r="K97" s="6" t="inlineStr">
         <is>
-          <t>상장완료 (2026-05-14)</t>
+          <t>상장완료 (2026-07-06)</t>
         </is>
       </c>
     </row>
     <row r="98">
       <c r="A98" s="6" t="inlineStr">
         <is>
-          <t>2026-03-26</t>
+          <t>2026-02-27</t>
         </is>
       </c>
       <c r="B98" s="6" t="inlineStr">
         <is>
-          <t>레몬헬스케어</t>
+          <t>마키나락스</t>
         </is>
       </c>
       <c r="C98" s="6" t="inlineStr">
@@ -5775,32 +5775,32 @@
       </c>
       <c r="F98" s="7" t="inlineStr">
         <is>
-          <t>14,877</t>
+          <t>8,294</t>
         </is>
       </c>
       <c r="G98" s="7" t="inlineStr">
         <is>
-          <t>-2,898</t>
+          <t>-6,073</t>
         </is>
       </c>
       <c r="H98" s="7" t="inlineStr">
         <is>
-          <t>-31,162</t>
+          <t>2,680</t>
         </is>
       </c>
       <c r="I98" s="6" t="inlineStr">
         <is>
-          <t>건강관리업체및서비스</t>
+          <t>소프트웨어</t>
         </is>
       </c>
       <c r="J98" s="6" t="inlineStr">
         <is>
-          <t>KB</t>
+          <t>미래</t>
         </is>
       </c>
       <c r="K98" s="6" t="inlineStr">
         <is>
-          <t>상장완료 (2026-07-06)</t>
+          <t>상장완료 (2026-05-20)</t>
         </is>
       </c>
     </row>
@@ -5812,7 +5812,7 @@
       </c>
       <c r="B99" s="6" t="inlineStr">
         <is>
-          <t>마키나락스</t>
+          <t>채비</t>
         </is>
       </c>
       <c r="C99" s="6" t="inlineStr">
@@ -5832,44 +5832,44 @@
       </c>
       <c r="F99" s="7" t="inlineStr">
         <is>
-          <t>8,294</t>
+          <t>85,082</t>
         </is>
       </c>
       <c r="G99" s="7" t="inlineStr">
         <is>
-          <t>-6,073</t>
+          <t>-54,495</t>
         </is>
       </c>
       <c r="H99" s="7" t="inlineStr">
         <is>
-          <t>2,680</t>
+          <t>96,866</t>
         </is>
       </c>
       <c r="I99" s="6" t="inlineStr">
         <is>
-          <t>소프트웨어</t>
+          <t>전기제품</t>
         </is>
       </c>
       <c r="J99" s="6" t="inlineStr">
         <is>
-          <t>미래</t>
+          <t>KB, 삼성, 대신, 하나</t>
         </is>
       </c>
       <c r="K99" s="6" t="inlineStr">
         <is>
-          <t>상장완료 (2026-05-20)</t>
+          <t>상장완료 (2026-04-29)</t>
         </is>
       </c>
     </row>
     <row r="100">
       <c r="A100" s="6" t="inlineStr">
         <is>
-          <t>2026-02-27</t>
+          <t>2026-02-10</t>
         </is>
       </c>
       <c r="B100" s="6" t="inlineStr">
         <is>
-          <t>채비</t>
+          <t>키움히어로제2호스팩</t>
         </is>
       </c>
       <c r="C100" s="6" t="inlineStr">
@@ -5887,46 +5887,30 @@
           <t>FY24</t>
         </is>
       </c>
-      <c r="F100" s="7" t="inlineStr">
-        <is>
-          <t>85,082</t>
-        </is>
-      </c>
-      <c r="G100" s="7" t="inlineStr">
-        <is>
-          <t>-54,495</t>
-        </is>
-      </c>
-      <c r="H100" s="7" t="inlineStr">
-        <is>
-          <t>96,866</t>
-        </is>
-      </c>
-      <c r="I100" s="6" t="inlineStr">
-        <is>
-          <t>전기제품</t>
-        </is>
-      </c>
+      <c r="F100" s="7" t="inlineStr"/>
+      <c r="G100" s="7" t="inlineStr"/>
+      <c r="H100" s="7" t="inlineStr"/>
+      <c r="I100" s="6" t="inlineStr"/>
       <c r="J100" s="6" t="inlineStr">
         <is>
-          <t>KB, 삼성, 대신, 하나</t>
+          <t>키움</t>
         </is>
       </c>
       <c r="K100" s="6" t="inlineStr">
         <is>
-          <t>상장완료 (2026-04-29)</t>
+          <t>상장완료 (2026-04-23)</t>
         </is>
       </c>
     </row>
     <row r="101">
       <c r="A101" s="6" t="inlineStr">
         <is>
-          <t>2026-02-10</t>
+          <t>2026-02-05</t>
         </is>
       </c>
       <c r="B101" s="6" t="inlineStr">
         <is>
-          <t>키움히어로제2호스팩</t>
+          <t>세미티에스</t>
         </is>
       </c>
       <c r="C101" s="6" t="inlineStr">
@@ -5936,7 +5920,7 @@
       </c>
       <c r="D101" s="6" t="inlineStr">
         <is>
-          <t>신규상장</t>
+          <t>스팩 소멸합병</t>
         </is>
       </c>
       <c r="E101" s="6" t="inlineStr">
@@ -5944,30 +5928,46 @@
           <t>FY24</t>
         </is>
       </c>
-      <c r="F101" s="7" t="inlineStr"/>
-      <c r="G101" s="7" t="inlineStr"/>
-      <c r="H101" s="7" t="inlineStr"/>
-      <c r="I101" s="6" t="inlineStr"/>
+      <c r="F101" s="7" t="inlineStr">
+        <is>
+          <t>20,808</t>
+        </is>
+      </c>
+      <c r="G101" s="7" t="inlineStr">
+        <is>
+          <t>7,337</t>
+        </is>
+      </c>
+      <c r="H101" s="7" t="inlineStr">
+        <is>
+          <t>26,616</t>
+        </is>
+      </c>
+      <c r="I101" s="6" t="inlineStr">
+        <is>
+          <t>반도체와반도체장비</t>
+        </is>
+      </c>
       <c r="J101" s="6" t="inlineStr">
         <is>
-          <t>키움</t>
+          <t>NH</t>
         </is>
       </c>
       <c r="K101" s="6" t="inlineStr">
         <is>
-          <t>상장완료 (2026-04-23)</t>
+          <t>상장완료 (2026-02-05)</t>
         </is>
       </c>
     </row>
     <row r="102">
       <c r="A102" s="6" t="inlineStr">
         <is>
-          <t>2026-02-05</t>
+          <t>2026-02-02</t>
         </is>
       </c>
       <c r="B102" s="6" t="inlineStr">
         <is>
-          <t>세미티에스</t>
+          <t>교보20호스팩</t>
         </is>
       </c>
       <c r="C102" s="6" t="inlineStr">
@@ -5977,7 +5977,7 @@
       </c>
       <c r="D102" s="6" t="inlineStr">
         <is>
-          <t>스팩 소멸합병</t>
+          <t>신규상장</t>
         </is>
       </c>
       <c r="E102" s="6" t="inlineStr">
@@ -5985,46 +5985,30 @@
           <t>FY24</t>
         </is>
       </c>
-      <c r="F102" s="7" t="inlineStr">
-        <is>
-          <t>20,808</t>
-        </is>
-      </c>
-      <c r="G102" s="7" t="inlineStr">
-        <is>
-          <t>7,337</t>
-        </is>
-      </c>
-      <c r="H102" s="7" t="inlineStr">
-        <is>
-          <t>26,616</t>
-        </is>
-      </c>
-      <c r="I102" s="6" t="inlineStr">
-        <is>
-          <t>반도체와반도체장비</t>
-        </is>
-      </c>
+      <c r="F102" s="7" t="inlineStr"/>
+      <c r="G102" s="7" t="inlineStr"/>
+      <c r="H102" s="7" t="inlineStr"/>
+      <c r="I102" s="6" t="inlineStr"/>
       <c r="J102" s="6" t="inlineStr">
         <is>
-          <t>NH</t>
+          <t>교보</t>
         </is>
       </c>
       <c r="K102" s="6" t="inlineStr">
         <is>
-          <t>상장완료 (2026-02-05)</t>
+          <t>상장완료 (2026-04-02)</t>
         </is>
       </c>
     </row>
     <row r="103">
       <c r="A103" s="6" t="inlineStr">
         <is>
-          <t>2026-02-02</t>
+          <t>2026-01-29</t>
         </is>
       </c>
       <c r="B103" s="6" t="inlineStr">
         <is>
-          <t>교보20호스팩</t>
+          <t>케이피항공산업</t>
         </is>
       </c>
       <c r="C103" s="6" t="inlineStr">
@@ -6034,7 +6018,7 @@
       </c>
       <c r="D103" s="6" t="inlineStr">
         <is>
-          <t>신규상장</t>
+          <t>스팩 소멸합병</t>
         </is>
       </c>
       <c r="E103" s="6" t="inlineStr">
@@ -6042,18 +6026,34 @@
           <t>FY24</t>
         </is>
       </c>
-      <c r="F103" s="7" t="inlineStr"/>
-      <c r="G103" s="7" t="inlineStr"/>
-      <c r="H103" s="7" t="inlineStr"/>
-      <c r="I103" s="6" t="inlineStr"/>
+      <c r="F103" s="7" t="inlineStr">
+        <is>
+          <t>49,651</t>
+        </is>
+      </c>
+      <c r="G103" s="7" t="inlineStr">
+        <is>
+          <t>3,018</t>
+        </is>
+      </c>
+      <c r="H103" s="7" t="inlineStr">
+        <is>
+          <t>15,901</t>
+        </is>
+      </c>
+      <c r="I103" s="6" t="inlineStr">
+        <is>
+          <t>우주항공과국방</t>
+        </is>
+      </c>
       <c r="J103" s="6" t="inlineStr">
         <is>
-          <t>교보</t>
+          <t>NH</t>
         </is>
       </c>
       <c r="K103" s="6" t="inlineStr">
         <is>
-          <t>상장완료 (2026-04-02)</t>
+          <t>상장완료 (2026-01-29)</t>
         </is>
       </c>
     </row>
@@ -6065,7 +6065,7 @@
       </c>
       <c r="B104" s="6" t="inlineStr">
         <is>
-          <t>케이피항공산업</t>
+          <t>한패스</t>
         </is>
       </c>
       <c r="C104" s="6" t="inlineStr">
@@ -6075,7 +6075,7 @@
       </c>
       <c r="D104" s="6" t="inlineStr">
         <is>
-          <t>스팩 소멸합병</t>
+          <t>신규상장</t>
         </is>
       </c>
       <c r="E104" s="6" t="inlineStr">
@@ -6085,44 +6085,44 @@
       </c>
       <c r="F104" s="7" t="inlineStr">
         <is>
-          <t>49,651</t>
+          <t>55,297</t>
         </is>
       </c>
       <c r="G104" s="7" t="inlineStr">
         <is>
-          <t>3,018</t>
+          <t>4,403</t>
         </is>
       </c>
       <c r="H104" s="7" t="inlineStr">
         <is>
-          <t>15,901</t>
+          <t>-28,065</t>
         </is>
       </c>
       <c r="I104" s="6" t="inlineStr">
         <is>
-          <t>우주항공과국방</t>
+          <t>IT서비스</t>
         </is>
       </c>
       <c r="J104" s="6" t="inlineStr">
         <is>
-          <t>NH</t>
+          <t>한국, 대신</t>
         </is>
       </c>
       <c r="K104" s="6" t="inlineStr">
         <is>
-          <t>상장완료 (2026-01-29)</t>
+          <t>상장완료 (2026-03-25)</t>
         </is>
       </c>
     </row>
     <row r="105">
       <c r="A105" s="6" t="inlineStr">
         <is>
-          <t>2026-01-29</t>
+          <t>2026-01-22</t>
         </is>
       </c>
       <c r="B105" s="6" t="inlineStr">
         <is>
-          <t>한패스</t>
+          <t>신한제18호스팩</t>
         </is>
       </c>
       <c r="C105" s="6" t="inlineStr">
@@ -6140,46 +6140,30 @@
           <t>FY24</t>
         </is>
       </c>
-      <c r="F105" s="7" t="inlineStr">
-        <is>
-          <t>55,297</t>
-        </is>
-      </c>
-      <c r="G105" s="7" t="inlineStr">
-        <is>
-          <t>4,403</t>
-        </is>
-      </c>
-      <c r="H105" s="7" t="inlineStr">
-        <is>
-          <t>-28,065</t>
-        </is>
-      </c>
-      <c r="I105" s="6" t="inlineStr">
-        <is>
-          <t>IT서비스</t>
-        </is>
-      </c>
+      <c r="F105" s="7" t="inlineStr"/>
+      <c r="G105" s="7" t="inlineStr"/>
+      <c r="H105" s="7" t="inlineStr"/>
+      <c r="I105" s="6" t="inlineStr"/>
       <c r="J105" s="6" t="inlineStr">
         <is>
-          <t>한국, 대신</t>
+          <t>신한</t>
         </is>
       </c>
       <c r="K105" s="6" t="inlineStr">
         <is>
-          <t>상장완료 (2026-03-25)</t>
+          <t>상장완료 (2026-04-30)</t>
         </is>
       </c>
     </row>
     <row r="106">
       <c r="A106" s="6" t="inlineStr">
         <is>
-          <t>2026-01-22</t>
+          <t>2026-01-20</t>
         </is>
       </c>
       <c r="B106" s="6" t="inlineStr">
         <is>
-          <t>신한제18호스팩</t>
+          <t>엔에이치스팩33호</t>
         </is>
       </c>
       <c r="C106" s="6" t="inlineStr">
@@ -6203,24 +6187,24 @@
       <c r="I106" s="6" t="inlineStr"/>
       <c r="J106" s="6" t="inlineStr">
         <is>
-          <t>신한</t>
+          <t>NH</t>
         </is>
       </c>
       <c r="K106" s="6" t="inlineStr">
         <is>
-          <t>상장완료 (2026-04-30)</t>
+          <t>상장완료 (2026-03-27)</t>
         </is>
       </c>
     </row>
     <row r="107">
       <c r="A107" s="6" t="inlineStr">
         <is>
-          <t>2026-01-20</t>
+          <t>2026-01-19</t>
         </is>
       </c>
       <c r="B107" s="6" t="inlineStr">
         <is>
-          <t>엔에이치스팩33호</t>
+          <t>신한제17호스팩</t>
         </is>
       </c>
       <c r="C107" s="6" t="inlineStr">
@@ -6244,24 +6228,24 @@
       <c r="I107" s="6" t="inlineStr"/>
       <c r="J107" s="6" t="inlineStr">
         <is>
-          <t>NH</t>
+          <t>신한</t>
         </is>
       </c>
       <c r="K107" s="6" t="inlineStr">
         <is>
-          <t>상장완료 (2026-03-27)</t>
+          <t>상장완료 (2026-04-01)</t>
         </is>
       </c>
     </row>
     <row r="108">
       <c r="A108" s="6" t="inlineStr">
         <is>
-          <t>2026-01-19</t>
+          <t>2026-01-16</t>
         </is>
       </c>
       <c r="B108" s="6" t="inlineStr">
         <is>
-          <t>신한제17호스팩</t>
+          <t>아이엠바이오로직스</t>
         </is>
       </c>
       <c r="C108" s="6" t="inlineStr">
@@ -6279,18 +6263,34 @@
           <t>FY24</t>
         </is>
       </c>
-      <c r="F108" s="7" t="inlineStr"/>
-      <c r="G108" s="7" t="inlineStr"/>
-      <c r="H108" s="7" t="inlineStr"/>
-      <c r="I108" s="6" t="inlineStr"/>
+      <c r="F108" s="7" t="inlineStr">
+        <is>
+          <t>27,594</t>
+        </is>
+      </c>
+      <c r="G108" s="7" t="inlineStr">
+        <is>
+          <t>-11,884</t>
+        </is>
+      </c>
+      <c r="H108" s="7" t="inlineStr">
+        <is>
+          <t>-77,202</t>
+        </is>
+      </c>
+      <c r="I108" s="6" t="inlineStr">
+        <is>
+          <t>제약</t>
+        </is>
+      </c>
       <c r="J108" s="6" t="inlineStr">
         <is>
-          <t>신한</t>
+          <t>한국, 신한</t>
         </is>
       </c>
       <c r="K108" s="6" t="inlineStr">
         <is>
-          <t>상장완료 (2026-04-01)</t>
+          <t>상장완료 (2026-03-20)</t>
         </is>
       </c>
     </row>
@@ -6302,7 +6302,7 @@
       </c>
       <c r="B109" s="6" t="inlineStr">
         <is>
-          <t>아이엠바이오로직스</t>
+          <t>에스팀</t>
         </is>
       </c>
       <c r="C109" s="6" t="inlineStr">
@@ -6322,220 +6322,220 @@
       </c>
       <c r="F109" s="7" t="inlineStr">
         <is>
-          <t>27,594</t>
+          <t>35,574</t>
         </is>
       </c>
       <c r="G109" s="7" t="inlineStr">
         <is>
-          <t>-11,884</t>
+          <t>1,372</t>
         </is>
       </c>
       <c r="H109" s="7" t="inlineStr">
         <is>
-          <t>-77,202</t>
+          <t>12,331</t>
         </is>
       </c>
       <c r="I109" s="6" t="inlineStr">
         <is>
-          <t>제약</t>
+          <t>광고</t>
         </is>
       </c>
       <c r="J109" s="6" t="inlineStr">
         <is>
-          <t>한국, 신한</t>
+          <t>한국</t>
         </is>
       </c>
       <c r="K109" s="6" t="inlineStr">
         <is>
-          <t>상장완료 (2026-03-20)</t>
+          <t>상장완료 (2026-03-06)</t>
         </is>
       </c>
     </row>
     <row r="110">
       <c r="A110" s="6" t="inlineStr">
         <is>
-          <t>2026-01-16</t>
+          <t>2026-01-12</t>
         </is>
       </c>
       <c r="B110" s="6" t="inlineStr">
         <is>
-          <t>에스팀</t>
+          <t>케이뱅크</t>
         </is>
       </c>
       <c r="C110" s="6" t="inlineStr">
         <is>
+          <t>유가</t>
+        </is>
+      </c>
+      <c r="D110" s="6" t="inlineStr">
+        <is>
+          <t>신규상장</t>
+        </is>
+      </c>
+      <c r="E110" s="6" t="inlineStr">
+        <is>
+          <t>FY24</t>
+        </is>
+      </c>
+      <c r="F110" s="7" t="inlineStr">
+        <is>
+          <t>1,228,501</t>
+        </is>
+      </c>
+      <c r="G110" s="7" t="inlineStr">
+        <is>
+          <t>128,053</t>
+        </is>
+      </c>
+      <c r="H110" s="7" t="inlineStr">
+        <is>
+          <t>1,995,845</t>
+        </is>
+      </c>
+      <c r="I110" s="6" t="inlineStr">
+        <is>
+          <t>은행</t>
+        </is>
+      </c>
+      <c r="J110" s="6" t="inlineStr">
+        <is>
+          <t>NH, 삼성</t>
+        </is>
+      </c>
+      <c r="K110" s="6" t="inlineStr">
+        <is>
+          <t>상장완료 (2026-03-05)</t>
+        </is>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" s="3" t="inlineStr">
+        <is>
+          <t>■ 철회·미승인  (18건)</t>
+        </is>
+      </c>
+      <c r="B112" s="4" t="n"/>
+      <c r="C112" s="4" t="n"/>
+      <c r="D112" s="4" t="n"/>
+      <c r="E112" s="4" t="n"/>
+      <c r="F112" s="4" t="n"/>
+      <c r="G112" s="4" t="n"/>
+      <c r="H112" s="4" t="n"/>
+      <c r="I112" s="4" t="n"/>
+      <c r="J112" s="4" t="n"/>
+      <c r="K112" s="4" t="n"/>
+    </row>
+    <row r="113">
+      <c r="A113" s="5" t="inlineStr">
+        <is>
+          <t>일자</t>
+        </is>
+      </c>
+      <c r="B113" s="5" t="inlineStr">
+        <is>
+          <t>회사명</t>
+        </is>
+      </c>
+      <c r="C113" s="5" t="inlineStr">
+        <is>
+          <t>시장</t>
+        </is>
+      </c>
+      <c r="D113" s="5" t="inlineStr">
+        <is>
+          <t>상장유형</t>
+        </is>
+      </c>
+      <c r="E113" s="5" t="inlineStr">
+        <is>
+          <t>기준연도</t>
+        </is>
+      </c>
+      <c r="F113" s="5" t="inlineStr">
+        <is>
+          <t>매출액</t>
+        </is>
+      </c>
+      <c r="G113" s="5" t="inlineStr">
+        <is>
+          <t>순이익</t>
+        </is>
+      </c>
+      <c r="H113" s="5" t="inlineStr">
+        <is>
+          <t>자기자본</t>
+        </is>
+      </c>
+      <c r="I113" s="5" t="inlineStr">
+        <is>
+          <t>업종</t>
+        </is>
+      </c>
+      <c r="J113" s="5" t="inlineStr">
+        <is>
+          <t>대표주관사</t>
+        </is>
+      </c>
+      <c r="K113" s="5" t="inlineStr">
+        <is>
+          <t>현황</t>
+        </is>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114" s="6" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="B114" s="6" t="inlineStr">
+        <is>
+          <t>텔레픽스</t>
+        </is>
+      </c>
+      <c r="C114" s="6" t="inlineStr">
+        <is>
           <t>코스닥</t>
         </is>
       </c>
-      <c r="D110" s="6" t="inlineStr">
+      <c r="D114" s="6" t="inlineStr">
         <is>
           <t>신규상장</t>
         </is>
       </c>
-      <c r="E110" s="6" t="inlineStr">
-        <is>
-          <t>FY24</t>
-        </is>
-      </c>
-      <c r="F110" s="7" t="inlineStr">
-        <is>
-          <t>35,574</t>
-        </is>
-      </c>
-      <c r="G110" s="7" t="inlineStr">
-        <is>
-          <t>1,372</t>
-        </is>
-      </c>
-      <c r="H110" s="7" t="inlineStr">
-        <is>
-          <t>12,331</t>
-        </is>
-      </c>
-      <c r="I110" s="6" t="inlineStr">
-        <is>
-          <t>광고</t>
-        </is>
-      </c>
-      <c r="J110" s="6" t="inlineStr">
-        <is>
-          <t>한국</t>
-        </is>
-      </c>
-      <c r="K110" s="6" t="inlineStr">
-        <is>
-          <t>상장완료 (2026-03-06)</t>
-        </is>
-      </c>
-    </row>
-    <row r="111">
-      <c r="A111" s="6" t="inlineStr">
-        <is>
-          <t>2026-01-12</t>
-        </is>
-      </c>
-      <c r="B111" s="6" t="inlineStr">
-        <is>
-          <t>케이뱅크</t>
-        </is>
-      </c>
-      <c r="C111" s="6" t="inlineStr">
-        <is>
-          <t>유가</t>
-        </is>
-      </c>
-      <c r="D111" s="6" t="inlineStr">
-        <is>
-          <t>신규상장</t>
-        </is>
-      </c>
-      <c r="E111" s="6" t="inlineStr">
-        <is>
-          <t>FY24</t>
-        </is>
-      </c>
-      <c r="F111" s="7" t="inlineStr">
-        <is>
-          <t>1,228,501</t>
-        </is>
-      </c>
-      <c r="G111" s="7" t="inlineStr">
-        <is>
-          <t>128,053</t>
-        </is>
-      </c>
-      <c r="H111" s="7" t="inlineStr">
-        <is>
-          <t>1,995,845</t>
-        </is>
-      </c>
-      <c r="I111" s="6" t="inlineStr">
-        <is>
-          <t>은행</t>
-        </is>
-      </c>
-      <c r="J111" s="6" t="inlineStr">
-        <is>
-          <t>NH, 삼성</t>
-        </is>
-      </c>
-      <c r="K111" s="6" t="inlineStr">
-        <is>
-          <t>상장완료 (2026-03-05)</t>
-        </is>
-      </c>
-    </row>
-    <row r="113">
-      <c r="A113" s="3" t="inlineStr">
-        <is>
-          <t>■ 철회·미승인  (17건)</t>
-        </is>
-      </c>
-      <c r="B113" s="4" t="n"/>
-      <c r="C113" s="4" t="n"/>
-      <c r="D113" s="4" t="n"/>
-      <c r="E113" s="4" t="n"/>
-      <c r="F113" s="4" t="n"/>
-      <c r="G113" s="4" t="n"/>
-      <c r="H113" s="4" t="n"/>
-      <c r="I113" s="4" t="n"/>
-      <c r="J113" s="4" t="n"/>
-      <c r="K113" s="4" t="n"/>
-    </row>
-    <row r="114">
-      <c r="A114" s="5" t="inlineStr">
-        <is>
-          <t>일자</t>
-        </is>
-      </c>
-      <c r="B114" s="5" t="inlineStr">
-        <is>
-          <t>회사명</t>
-        </is>
-      </c>
-      <c r="C114" s="5" t="inlineStr">
-        <is>
-          <t>시장</t>
-        </is>
-      </c>
-      <c r="D114" s="5" t="inlineStr">
-        <is>
-          <t>상장유형</t>
-        </is>
-      </c>
-      <c r="E114" s="5" t="inlineStr">
-        <is>
-          <t>기준연도</t>
-        </is>
-      </c>
-      <c r="F114" s="5" t="inlineStr">
-        <is>
-          <t>매출액</t>
-        </is>
-      </c>
-      <c r="G114" s="5" t="inlineStr">
-        <is>
-          <t>순이익</t>
-        </is>
-      </c>
-      <c r="H114" s="5" t="inlineStr">
-        <is>
-          <t>자기자본</t>
-        </is>
-      </c>
-      <c r="I114" s="5" t="inlineStr">
-        <is>
-          <t>업종</t>
-        </is>
-      </c>
-      <c r="J114" s="5" t="inlineStr">
-        <is>
-          <t>대표주관사</t>
-        </is>
-      </c>
-      <c r="K114" s="5" t="inlineStr">
-        <is>
-          <t>현황</t>
+      <c r="E114" s="6" t="inlineStr">
+        <is>
+          <t>FY25</t>
+        </is>
+      </c>
+      <c r="F114" s="7" t="inlineStr">
+        <is>
+          <t>4,896</t>
+        </is>
+      </c>
+      <c r="G114" s="7" t="inlineStr">
+        <is>
+          <t>-16,214</t>
+        </is>
+      </c>
+      <c r="H114" s="7" t="inlineStr">
+        <is>
+          <t>9,146</t>
+        </is>
+      </c>
+      <c r="I114" s="6" t="inlineStr">
+        <is>
+          <t>소프트웨어 개발 및 공급업</t>
+        </is>
+      </c>
+      <c r="J114" s="6" t="inlineStr">
+        <is>
+          <t>미래</t>
+        </is>
+      </c>
+      <c r="K114" s="6" t="inlineStr">
+        <is>
+          <t>심사 철회</t>
         </is>
       </c>
     </row>
@@ -12657,7 +12657,7 @@
         <v>7</v>
       </c>
       <c r="D13" s="6" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E13" s="6" t="n">
         <v>6</v>

</xml_diff>

<commit_message>
chore: update IPO data 2026-09-02
</commit_message>
<xml_diff>
--- a/IPO_analysis.xlsx
+++ b/IPO_analysis.xlsx
@@ -592,7 +592,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K131"/>
+  <dimension ref="A1:K132"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -618,7 +618,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>기준일 2026-09-01 · 청구일 직전 사업연도 · 별도/개별 재무제표 · 단위 백만원(별도 표기 시 USD)</t>
+          <t>기준일 2026-09-02 · 청구일 직전 사업연도 · 별도/개별 재무제표 · 단위 백만원(별도 표기 시 USD)</t>
         </is>
       </c>
     </row>
@@ -3387,7 +3387,7 @@
     <row r="55">
       <c r="A55" s="3" t="inlineStr">
         <is>
-          <t>■ 심사 승인  (54건)</t>
+          <t>■ 심사 승인  (55건)</t>
         </is>
       </c>
       <c r="B55" s="4" t="n"/>
@@ -3466,7 +3466,7 @@
       </c>
       <c r="B57" s="6" t="inlineStr">
         <is>
-          <t>다비오</t>
+          <t>하나에어로다이내믹스</t>
         </is>
       </c>
       <c r="C57" s="6" t="inlineStr">
@@ -3486,27 +3486,27 @@
       </c>
       <c r="F57" s="7" t="inlineStr">
         <is>
-          <t>9,251</t>
+          <t>33,286</t>
         </is>
       </c>
       <c r="G57" s="7" t="inlineStr">
         <is>
-          <t>-3,473</t>
+          <t>2,420</t>
         </is>
       </c>
       <c r="H57" s="7" t="inlineStr">
         <is>
-          <t>300</t>
+          <t>890</t>
         </is>
       </c>
       <c r="I57" s="6" t="inlineStr">
         <is>
-          <t>소프트웨어 개발 및 공급업</t>
+          <t>항공기,우주선 및 부품 제조업</t>
         </is>
       </c>
       <c r="J57" s="6" t="inlineStr">
         <is>
-          <t>대신</t>
+          <t>IBK</t>
         </is>
       </c>
       <c r="K57" s="6" t="inlineStr">
@@ -3518,12 +3518,12 @@
     <row r="58">
       <c r="A58" s="6" t="inlineStr">
         <is>
-          <t>2026-08-20</t>
+          <t>2026-08-28</t>
         </is>
       </c>
       <c r="B58" s="6" t="inlineStr">
         <is>
-          <t>티앤이코리아</t>
+          <t>다비오</t>
         </is>
       </c>
       <c r="C58" s="6" t="inlineStr">
@@ -3543,27 +3543,27 @@
       </c>
       <c r="F58" s="7" t="inlineStr">
         <is>
-          <t>22,339</t>
+          <t>9,251</t>
         </is>
       </c>
       <c r="G58" s="7" t="inlineStr">
         <is>
-          <t>-7,091</t>
+          <t>-3,473</t>
         </is>
       </c>
       <c r="H58" s="7" t="inlineStr">
         <is>
-          <t>481</t>
+          <t>300</t>
         </is>
       </c>
       <c r="I58" s="6" t="inlineStr">
         <is>
-          <t>일반 목적용 기계 제조업</t>
+          <t>소프트웨어 개발 및 공급업</t>
         </is>
       </c>
       <c r="J58" s="6" t="inlineStr">
         <is>
-          <t>신한</t>
+          <t>대신</t>
         </is>
       </c>
       <c r="K58" s="6" t="inlineStr">
@@ -3580,7 +3580,7 @@
       </c>
       <c r="B59" s="6" t="inlineStr">
         <is>
-          <t>유캐스트</t>
+          <t>티앤이코리아</t>
         </is>
       </c>
       <c r="C59" s="6" t="inlineStr">
@@ -3600,27 +3600,27 @@
       </c>
       <c r="F59" s="7" t="inlineStr">
         <is>
-          <t>5,934</t>
+          <t>22,339</t>
         </is>
       </c>
       <c r="G59" s="7" t="inlineStr">
         <is>
-          <t>-3,557</t>
+          <t>-7,091</t>
         </is>
       </c>
       <c r="H59" s="7" t="inlineStr">
         <is>
-          <t>1,881</t>
+          <t>481</t>
         </is>
       </c>
       <c r="I59" s="6" t="inlineStr">
         <is>
-          <t>통신 및 방송 장비 제조업</t>
+          <t>일반 목적용 기계 제조업</t>
         </is>
       </c>
       <c r="J59" s="6" t="inlineStr">
         <is>
-          <t>유진</t>
+          <t>신한</t>
         </is>
       </c>
       <c r="K59" s="6" t="inlineStr">
@@ -3637,7 +3637,7 @@
       </c>
       <c r="B60" s="6" t="inlineStr">
         <is>
-          <t>엘리스그룹</t>
+          <t>유캐스트</t>
         </is>
       </c>
       <c r="C60" s="6" t="inlineStr">
@@ -3657,27 +3657,27 @@
       </c>
       <c r="F60" s="7" t="inlineStr">
         <is>
-          <t>39,513</t>
+          <t>5,934</t>
         </is>
       </c>
       <c r="G60" s="7" t="inlineStr">
         <is>
-          <t>15,666</t>
+          <t>-3,557</t>
         </is>
       </c>
       <c r="H60" s="7" t="inlineStr">
         <is>
-          <t>85,400</t>
+          <t>1,881</t>
         </is>
       </c>
       <c r="I60" s="6" t="inlineStr">
         <is>
-          <t>소프트웨어 개발 및 공급업</t>
+          <t>통신 및 방송 장비 제조업</t>
         </is>
       </c>
       <c r="J60" s="6" t="inlineStr">
         <is>
-          <t>미래, 삼성</t>
+          <t>유진</t>
         </is>
       </c>
       <c r="K60" s="6" t="inlineStr">
@@ -3689,12 +3689,12 @@
     <row r="61">
       <c r="A61" s="6" t="inlineStr">
         <is>
-          <t>2026-08-12</t>
+          <t>2026-08-20</t>
         </is>
       </c>
       <c r="B61" s="6" t="inlineStr">
         <is>
-          <t>진코스텍</t>
+          <t>엘리스그룹</t>
         </is>
       </c>
       <c r="C61" s="6" t="inlineStr">
@@ -3704,7 +3704,7 @@
       </c>
       <c r="D61" s="6" t="inlineStr">
         <is>
-          <t>이전상장</t>
+          <t>신규상장</t>
         </is>
       </c>
       <c r="E61" s="6" t="inlineStr">
@@ -3714,27 +3714,27 @@
       </c>
       <c r="F61" s="7" t="inlineStr">
         <is>
-          <t>48,646</t>
+          <t>39,513</t>
         </is>
       </c>
       <c r="G61" s="7" t="inlineStr">
         <is>
-          <t>6,017</t>
+          <t>15,666</t>
         </is>
       </c>
       <c r="H61" s="7" t="inlineStr">
         <is>
-          <t>18,795</t>
+          <t>85,400</t>
         </is>
       </c>
       <c r="I61" s="6" t="inlineStr">
         <is>
-          <t>기타 화학제품 제조업</t>
+          <t>소프트웨어 개발 및 공급업</t>
         </is>
       </c>
       <c r="J61" s="6" t="inlineStr">
         <is>
-          <t>하나</t>
+          <t>미래, 삼성</t>
         </is>
       </c>
       <c r="K61" s="6" t="inlineStr">
@@ -3751,7 +3751,7 @@
       </c>
       <c r="B62" s="6" t="inlineStr">
         <is>
-          <t>바로팜</t>
+          <t>진코스텍</t>
         </is>
       </c>
       <c r="C62" s="6" t="inlineStr">
@@ -3761,7 +3761,7 @@
       </c>
       <c r="D62" s="6" t="inlineStr">
         <is>
-          <t>신규상장</t>
+          <t>이전상장</t>
         </is>
       </c>
       <c r="E62" s="6" t="inlineStr">
@@ -3771,27 +3771,27 @@
       </c>
       <c r="F62" s="7" t="inlineStr">
         <is>
-          <t>96,724</t>
+          <t>48,646</t>
         </is>
       </c>
       <c r="G62" s="7" t="inlineStr">
         <is>
-          <t>-9,679</t>
+          <t>6,017</t>
         </is>
       </c>
       <c r="H62" s="7" t="inlineStr">
         <is>
-          <t>30,673</t>
+          <t>18,795</t>
         </is>
       </c>
       <c r="I62" s="6" t="inlineStr">
         <is>
-          <t>상품 중개업</t>
+          <t>기타 화학제품 제조업</t>
         </is>
       </c>
       <c r="J62" s="6" t="inlineStr">
         <is>
-          <t>미래</t>
+          <t>하나</t>
         </is>
       </c>
       <c r="K62" s="6" t="inlineStr">
@@ -3808,7 +3808,7 @@
       </c>
       <c r="B63" s="6" t="inlineStr">
         <is>
-          <t>크리에이츠</t>
+          <t>바로팜</t>
         </is>
       </c>
       <c r="C63" s="6" t="inlineStr">
@@ -3828,27 +3828,27 @@
       </c>
       <c r="F63" s="7" t="inlineStr">
         <is>
-          <t>76,395</t>
+          <t>96,724</t>
         </is>
       </c>
       <c r="G63" s="7" t="inlineStr">
         <is>
-          <t>23,749</t>
+          <t>-9,679</t>
         </is>
       </c>
       <c r="H63" s="7" t="inlineStr">
         <is>
-          <t>2,335</t>
+          <t>30,673</t>
         </is>
       </c>
       <c r="I63" s="6" t="inlineStr">
         <is>
-          <t>그외 기타 제품 제조업</t>
+          <t>상품 중개업</t>
         </is>
       </c>
       <c r="J63" s="6" t="inlineStr">
         <is>
-          <t>삼성</t>
+          <t>미래</t>
         </is>
       </c>
       <c r="K63" s="6" t="inlineStr">
@@ -3860,12 +3860,12 @@
     <row r="64">
       <c r="A64" s="6" t="inlineStr">
         <is>
-          <t>2026-07-30</t>
+          <t>2026-08-12</t>
         </is>
       </c>
       <c r="B64" s="6" t="inlineStr">
         <is>
-          <t>래블업</t>
+          <t>크리에이츠</t>
         </is>
       </c>
       <c r="C64" s="6" t="inlineStr">
@@ -3885,27 +3885,27 @@
       </c>
       <c r="F64" s="7" t="inlineStr">
         <is>
-          <t>6,712</t>
+          <t>76,395</t>
         </is>
       </c>
       <c r="G64" s="7" t="inlineStr">
         <is>
-          <t>-1,526</t>
+          <t>23,749</t>
         </is>
       </c>
       <c r="H64" s="7" t="inlineStr">
         <is>
-          <t>373</t>
+          <t>2,335</t>
         </is>
       </c>
       <c r="I64" s="6" t="inlineStr">
         <is>
-          <t>데이터베이스 및 온라인정보 제공업</t>
+          <t>그외 기타 제품 제조업</t>
         </is>
       </c>
       <c r="J64" s="6" t="inlineStr">
         <is>
-          <t>NH</t>
+          <t>삼성</t>
         </is>
       </c>
       <c r="K64" s="6" t="inlineStr">
@@ -3922,7 +3922,7 @@
       </c>
       <c r="B65" s="6" t="inlineStr">
         <is>
-          <t>멜콘</t>
+          <t>래블업</t>
         </is>
       </c>
       <c r="C65" s="6" t="inlineStr">
@@ -3942,27 +3942,27 @@
       </c>
       <c r="F65" s="7" t="inlineStr">
         <is>
-          <t>39,319</t>
+          <t>6,712</t>
         </is>
       </c>
       <c r="G65" s="7" t="inlineStr">
         <is>
-          <t>4,739</t>
+          <t>-1,526</t>
         </is>
       </c>
       <c r="H65" s="7" t="inlineStr">
         <is>
-          <t>1,250</t>
+          <t>373</t>
         </is>
       </c>
       <c r="I65" s="6" t="inlineStr">
         <is>
-          <t>특수 목적용 기계 제조업</t>
+          <t>데이터베이스 및 온라인정보 제공업</t>
         </is>
       </c>
       <c r="J65" s="6" t="inlineStr">
         <is>
-          <t>대신</t>
+          <t>NH</t>
         </is>
       </c>
       <c r="K65" s="6" t="inlineStr">
@@ -3979,7 +3979,7 @@
       </c>
       <c r="B66" s="6" t="inlineStr">
         <is>
-          <t>엠비디</t>
+          <t>멜콘</t>
         </is>
       </c>
       <c r="C66" s="6" t="inlineStr">
@@ -3999,27 +3999,27 @@
       </c>
       <c r="F66" s="7" t="inlineStr">
         <is>
-          <t>1,524</t>
+          <t>39,319</t>
         </is>
       </c>
       <c r="G66" s="7" t="inlineStr">
         <is>
-          <t>-2,125</t>
+          <t>4,739</t>
         </is>
       </c>
       <c r="H66" s="7" t="inlineStr">
         <is>
-          <t>2,753</t>
+          <t>1,250</t>
         </is>
       </c>
       <c r="I66" s="6" t="inlineStr">
         <is>
-          <t>물질 검사, 측정 및 분석기구 제조업</t>
+          <t>특수 목적용 기계 제조업</t>
         </is>
       </c>
       <c r="J66" s="6" t="inlineStr">
         <is>
-          <t>하나</t>
+          <t>대신</t>
         </is>
       </c>
       <c r="K66" s="6" t="inlineStr">
@@ -4031,12 +4031,12 @@
     <row r="67">
       <c r="A67" s="6" t="inlineStr">
         <is>
-          <t>2026-07-29</t>
+          <t>2026-07-30</t>
         </is>
       </c>
       <c r="B67" s="6" t="inlineStr">
         <is>
-          <t>에스케이증권제14호기업인수목적</t>
+          <t>엠비디</t>
         </is>
       </c>
       <c r="C67" s="6" t="inlineStr">
@@ -4056,27 +4056,27 @@
       </c>
       <c r="F67" s="7" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>1,524</t>
         </is>
       </c>
       <c r="G67" s="7" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>-2,125</t>
         </is>
       </c>
       <c r="H67" s="7" t="inlineStr">
         <is>
-          <t>17</t>
+          <t>2,753</t>
         </is>
       </c>
       <c r="I67" s="6" t="inlineStr">
         <is>
-          <t>기타 금융업</t>
+          <t>물질 검사, 측정 및 분석기구 제조업</t>
         </is>
       </c>
       <c r="J67" s="6" t="inlineStr">
         <is>
-          <t>SK</t>
+          <t>하나</t>
         </is>
       </c>
       <c r="K67" s="6" t="inlineStr">
@@ -4093,7 +4093,7 @@
       </c>
       <c r="B68" s="6" t="inlineStr">
         <is>
-          <t>케이비제34호스팩</t>
+          <t>에스케이증권제14호기업인수목적</t>
         </is>
       </c>
       <c r="C68" s="6" t="inlineStr">
@@ -4123,7 +4123,7 @@
       </c>
       <c r="H68" s="7" t="inlineStr">
         <is>
-          <t>21</t>
+          <t>17</t>
         </is>
       </c>
       <c r="I68" s="6" t="inlineStr">
@@ -4133,7 +4133,7 @@
       </c>
       <c r="J68" s="6" t="inlineStr">
         <is>
-          <t>KB</t>
+          <t>SK</t>
         </is>
       </c>
       <c r="K68" s="6" t="inlineStr">
@@ -4150,7 +4150,7 @@
       </c>
       <c r="B69" s="6" t="inlineStr">
         <is>
-          <t>한국제17호스팩</t>
+          <t>케이비제34호스팩</t>
         </is>
       </c>
       <c r="C69" s="6" t="inlineStr">
@@ -4180,7 +4180,7 @@
       </c>
       <c r="H69" s="7" t="inlineStr">
         <is>
-          <t>170</t>
+          <t>21</t>
         </is>
       </c>
       <c r="I69" s="6" t="inlineStr">
@@ -4190,7 +4190,7 @@
       </c>
       <c r="J69" s="6" t="inlineStr">
         <is>
-          <t>한국</t>
+          <t>KB</t>
         </is>
       </c>
       <c r="K69" s="6" t="inlineStr">
@@ -4207,7 +4207,7 @@
       </c>
       <c r="B70" s="6" t="inlineStr">
         <is>
-          <t>한화플러스제6호스팩</t>
+          <t>한국제17호스팩</t>
         </is>
       </c>
       <c r="C70" s="6" t="inlineStr">
@@ -4237,7 +4237,7 @@
       </c>
       <c r="H70" s="7" t="inlineStr">
         <is>
-          <t>41</t>
+          <t>170</t>
         </is>
       </c>
       <c r="I70" s="6" t="inlineStr">
@@ -4247,7 +4247,7 @@
       </c>
       <c r="J70" s="6" t="inlineStr">
         <is>
-          <t>한화</t>
+          <t>한국</t>
         </is>
       </c>
       <c r="K70" s="6" t="inlineStr">
@@ -4259,12 +4259,12 @@
     <row r="71">
       <c r="A71" s="6" t="inlineStr">
         <is>
-          <t>2026-07-22</t>
+          <t>2026-07-29</t>
         </is>
       </c>
       <c r="B71" s="6" t="inlineStr">
         <is>
-          <t>엔에이치스팩34호</t>
+          <t>한화플러스제6호스팩</t>
         </is>
       </c>
       <c r="C71" s="6" t="inlineStr">
@@ -4294,17 +4294,17 @@
       </c>
       <c r="H71" s="7" t="inlineStr">
         <is>
-          <t>55</t>
+          <t>41</t>
         </is>
       </c>
       <c r="I71" s="6" t="inlineStr">
         <is>
-          <t>금융 지원 서비스업</t>
+          <t>기타 금융업</t>
         </is>
       </c>
       <c r="J71" s="6" t="inlineStr">
         <is>
-          <t>NH</t>
+          <t>한화</t>
         </is>
       </c>
       <c r="K71" s="6" t="inlineStr">
@@ -4316,12 +4316,12 @@
     <row r="72">
       <c r="A72" s="6" t="inlineStr">
         <is>
-          <t>2026-07-20</t>
+          <t>2026-07-22</t>
         </is>
       </c>
       <c r="B72" s="6" t="inlineStr">
         <is>
-          <t>글로벌테크놀로지</t>
+          <t>엔에이치스팩34호</t>
         </is>
       </c>
       <c r="C72" s="6" t="inlineStr">
@@ -4341,27 +4341,27 @@
       </c>
       <c r="F72" s="7" t="inlineStr">
         <is>
-          <t>29,689</t>
+          <t>-</t>
         </is>
       </c>
       <c r="G72" s="7" t="inlineStr">
         <is>
-          <t>-25,889</t>
+          <t>-</t>
         </is>
       </c>
       <c r="H72" s="7" t="inlineStr">
         <is>
-          <t>6,402</t>
+          <t>55</t>
         </is>
       </c>
       <c r="I72" s="6" t="inlineStr">
         <is>
-          <t>반도체 제조업</t>
+          <t>금융 지원 서비스업</t>
         </is>
       </c>
       <c r="J72" s="6" t="inlineStr">
         <is>
-          <t>한국</t>
+          <t>NH</t>
         </is>
       </c>
       <c r="K72" s="6" t="inlineStr">
@@ -4378,7 +4378,7 @@
       </c>
       <c r="B73" s="6" t="inlineStr">
         <is>
-          <t>덕산넵코어스</t>
+          <t>글로벌테크놀로지</t>
         </is>
       </c>
       <c r="C73" s="6" t="inlineStr">
@@ -4393,32 +4393,32 @@
       </c>
       <c r="E73" s="6" t="inlineStr">
         <is>
-          <t>FY24</t>
+          <t>FY25</t>
         </is>
       </c>
       <c r="F73" s="7" t="inlineStr">
         <is>
-          <t>48,504</t>
+          <t>29,689</t>
         </is>
       </c>
       <c r="G73" s="7" t="inlineStr">
         <is>
-          <t>3,668</t>
+          <t>-25,889</t>
         </is>
       </c>
       <c r="H73" s="7" t="inlineStr">
         <is>
-          <t>8,448</t>
+          <t>6,402</t>
         </is>
       </c>
       <c r="I73" s="6" t="inlineStr">
         <is>
-          <t>항공기,우주선 및 부품 제조업</t>
+          <t>반도체 제조업</t>
         </is>
       </c>
       <c r="J73" s="6" t="inlineStr">
         <is>
-          <t>대신</t>
+          <t>한국</t>
         </is>
       </c>
       <c r="K73" s="6" t="inlineStr">
@@ -4435,7 +4435,7 @@
       </c>
       <c r="B74" s="6" t="inlineStr">
         <is>
-          <t>디티에스</t>
+          <t>덕산넵코어스</t>
         </is>
       </c>
       <c r="C74" s="6" t="inlineStr">
@@ -4455,22 +4455,22 @@
       </c>
       <c r="F74" s="7" t="inlineStr">
         <is>
-          <t>142,718</t>
+          <t>48,504</t>
         </is>
       </c>
       <c r="G74" s="7" t="inlineStr">
         <is>
-          <t>18,765</t>
+          <t>3,668</t>
         </is>
       </c>
       <c r="H74" s="7" t="inlineStr">
         <is>
-          <t>63,153</t>
+          <t>8,448</t>
         </is>
       </c>
       <c r="I74" s="6" t="inlineStr">
         <is>
-          <t>특수 목적용 기계 제조업</t>
+          <t>항공기,우주선 및 부품 제조업</t>
         </is>
       </c>
       <c r="J74" s="6" t="inlineStr">
@@ -4487,12 +4487,12 @@
     <row r="75">
       <c r="A75" s="6" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
+          <t>2026-07-20</t>
         </is>
       </c>
       <c r="B75" s="6" t="inlineStr">
         <is>
-          <t>네오사피엔스</t>
+          <t>디티에스</t>
         </is>
       </c>
       <c r="C75" s="6" t="inlineStr">
@@ -4507,27 +4507,27 @@
       </c>
       <c r="E75" s="6" t="inlineStr">
         <is>
-          <t>FY25</t>
+          <t>FY24</t>
         </is>
       </c>
       <c r="F75" s="7" t="inlineStr">
         <is>
-          <t>10,649</t>
+          <t>142,718</t>
         </is>
       </c>
       <c r="G75" s="7" t="inlineStr">
         <is>
-          <t>-6,994</t>
+          <t>18,765</t>
         </is>
       </c>
       <c r="H75" s="7" t="inlineStr">
         <is>
-          <t>-39,962</t>
+          <t>63,153</t>
         </is>
       </c>
       <c r="I75" s="6" t="inlineStr">
         <is>
-          <t>소프트웨어 개발 및 공급업</t>
+          <t>특수 목적용 기계 제조업</t>
         </is>
       </c>
       <c r="J75" s="6" t="inlineStr">
@@ -4549,7 +4549,7 @@
       </c>
       <c r="B76" s="6" t="inlineStr">
         <is>
-          <t>엠에스바이오</t>
+          <t>네오사피엔스</t>
         </is>
       </c>
       <c r="C76" s="6" t="inlineStr">
@@ -4569,27 +4569,27 @@
       </c>
       <c r="F76" s="7" t="inlineStr">
         <is>
-          <t>23,787</t>
+          <t>10,649</t>
         </is>
       </c>
       <c r="G76" s="7" t="inlineStr">
         <is>
-          <t>7,288</t>
+          <t>-6,994</t>
         </is>
       </c>
       <c r="H76" s="7" t="inlineStr">
         <is>
-          <t>1,942</t>
+          <t>-39,962</t>
         </is>
       </c>
       <c r="I76" s="6" t="inlineStr">
         <is>
-          <t>의료용 기기 제조업</t>
+          <t>소프트웨어 개발 및 공급업</t>
         </is>
       </c>
       <c r="J76" s="6" t="inlineStr">
         <is>
-          <t>KB</t>
+          <t>대신</t>
         </is>
       </c>
       <c r="K76" s="6" t="inlineStr">
@@ -4601,12 +4601,12 @@
     <row r="77">
       <c r="A77" s="6" t="inlineStr">
         <is>
-          <t>2026-06-25</t>
+          <t>2026-07-10</t>
         </is>
       </c>
       <c r="B77" s="6" t="inlineStr">
         <is>
-          <t>기도산업</t>
+          <t>엠에스바이오</t>
         </is>
       </c>
       <c r="C77" s="6" t="inlineStr">
@@ -4626,32 +4626,32 @@
       </c>
       <c r="F77" s="7" t="inlineStr">
         <is>
-          <t>346,551</t>
+          <t>23,787</t>
         </is>
       </c>
       <c r="G77" s="7" t="inlineStr">
         <is>
-          <t>35,334</t>
+          <t>7,288</t>
         </is>
       </c>
       <c r="H77" s="7" t="inlineStr">
         <is>
-          <t>145,991</t>
+          <t>1,942</t>
         </is>
       </c>
       <c r="I77" s="6" t="inlineStr">
         <is>
-          <t>봉제의복 제조업</t>
+          <t>의료용 기기 제조업</t>
         </is>
       </c>
       <c r="J77" s="6" t="inlineStr">
         <is>
-          <t>미래</t>
+          <t>KB</t>
         </is>
       </c>
       <c r="K77" s="6" t="inlineStr">
         <is>
-          <t>상장완료 (2026-08-21)</t>
+          <t>상장전</t>
         </is>
       </c>
     </row>
@@ -4663,7 +4663,7 @@
       </c>
       <c r="B78" s="6" t="inlineStr">
         <is>
-          <t>브릴스</t>
+          <t>기도산업</t>
         </is>
       </c>
       <c r="C78" s="6" t="inlineStr">
@@ -4683,32 +4683,32 @@
       </c>
       <c r="F78" s="7" t="inlineStr">
         <is>
-          <t>23,759</t>
+          <t>346,551</t>
         </is>
       </c>
       <c r="G78" s="7" t="inlineStr">
         <is>
-          <t>1,744</t>
+          <t>35,334</t>
         </is>
       </c>
       <c r="H78" s="7" t="inlineStr">
         <is>
-          <t>4,785</t>
+          <t>145,991</t>
         </is>
       </c>
       <c r="I78" s="6" t="inlineStr">
         <is>
-          <t>특수 목적용 기계 제조업</t>
+          <t>봉제의복 제조업</t>
         </is>
       </c>
       <c r="J78" s="6" t="inlineStr">
         <is>
-          <t>IBK</t>
+          <t>미래</t>
         </is>
       </c>
       <c r="K78" s="6" t="inlineStr">
         <is>
-          <t>상장전</t>
+          <t>상장완료 (2026-08-21)</t>
         </is>
       </c>
     </row>
@@ -4720,7 +4720,7 @@
       </c>
       <c r="B79" s="6" t="inlineStr">
         <is>
-          <t>와이즈플래닛컴퍼니</t>
+          <t>브릴스</t>
         </is>
       </c>
       <c r="C79" s="6" t="inlineStr">
@@ -4740,27 +4740,27 @@
       </c>
       <c r="F79" s="7" t="inlineStr">
         <is>
-          <t>44,578</t>
+          <t>23,759</t>
         </is>
       </c>
       <c r="G79" s="7" t="inlineStr">
         <is>
-          <t>7,748</t>
+          <t>1,744</t>
         </is>
       </c>
       <c r="H79" s="7" t="inlineStr">
         <is>
-          <t>959</t>
+          <t>4,785</t>
         </is>
       </c>
       <c r="I79" s="6" t="inlineStr">
         <is>
-          <t>광고물 문안, 도안, 설계 등 작성업</t>
+          <t>특수 목적용 기계 제조업</t>
         </is>
       </c>
       <c r="J79" s="6" t="inlineStr">
         <is>
-          <t>대신</t>
+          <t>IBK</t>
         </is>
       </c>
       <c r="K79" s="6" t="inlineStr">
@@ -4772,12 +4772,12 @@
     <row r="80">
       <c r="A80" s="6" t="inlineStr">
         <is>
-          <t>2026-06-24</t>
+          <t>2026-06-25</t>
         </is>
       </c>
       <c r="B80" s="6" t="inlineStr">
         <is>
-          <t>니어스랩</t>
+          <t>와이즈플래닛컴퍼니</t>
         </is>
       </c>
       <c r="C80" s="6" t="inlineStr">
@@ -4797,32 +4797,32 @@
       </c>
       <c r="F80" s="7" t="inlineStr">
         <is>
-          <t>6,361</t>
+          <t>44,578</t>
         </is>
       </c>
       <c r="G80" s="7" t="inlineStr">
         <is>
-          <t>-7,287</t>
+          <t>7,748</t>
         </is>
       </c>
       <c r="H80" s="7" t="inlineStr">
         <is>
-          <t>127</t>
+          <t>959</t>
         </is>
       </c>
       <c r="I80" s="6" t="inlineStr">
         <is>
-          <t>소프트웨어 개발 및 공급업</t>
+          <t>광고물 문안, 도안, 설계 등 작성업</t>
         </is>
       </c>
       <c r="J80" s="6" t="inlineStr">
         <is>
-          <t>삼성</t>
+          <t>대신</t>
         </is>
       </c>
       <c r="K80" s="6" t="inlineStr">
         <is>
-          <t>상장완료 (2026-08-24)</t>
+          <t>상장전</t>
         </is>
       </c>
     </row>
@@ -4834,7 +4834,7 @@
       </c>
       <c r="B81" s="6" t="inlineStr">
         <is>
-          <t>해치텍</t>
+          <t>니어스랩</t>
         </is>
       </c>
       <c r="C81" s="6" t="inlineStr">
@@ -4854,32 +4854,32 @@
       </c>
       <c r="F81" s="7" t="inlineStr">
         <is>
-          <t>14,079</t>
+          <t>6,361</t>
         </is>
       </c>
       <c r="G81" s="7" t="inlineStr">
         <is>
-          <t>-8,009</t>
+          <t>-7,287</t>
         </is>
       </c>
       <c r="H81" s="7" t="inlineStr">
         <is>
-          <t>2,229</t>
+          <t>127</t>
         </is>
       </c>
       <c r="I81" s="6" t="inlineStr">
         <is>
-          <t>반도체 제조업</t>
+          <t>소프트웨어 개발 및 공급업</t>
         </is>
       </c>
       <c r="J81" s="6" t="inlineStr">
         <is>
-          <t>DB</t>
+          <t>삼성</t>
         </is>
       </c>
       <c r="K81" s="6" t="inlineStr">
         <is>
-          <t>상장완료 (2026-08-25)</t>
+          <t>상장완료 (2026-08-24)</t>
         </is>
       </c>
     </row>
@@ -4891,7 +4891,7 @@
       </c>
       <c r="B82" s="6" t="inlineStr">
         <is>
-          <t>스카이랩스</t>
+          <t>해치텍</t>
         </is>
       </c>
       <c r="C82" s="6" t="inlineStr">
@@ -4911,44 +4911,44 @@
       </c>
       <c r="F82" s="7" t="inlineStr">
         <is>
-          <t>7,936</t>
+          <t>14,079</t>
         </is>
       </c>
       <c r="G82" s="7" t="inlineStr">
         <is>
-          <t>-62,995</t>
+          <t>-8,009</t>
         </is>
       </c>
       <c r="H82" s="7" t="inlineStr">
         <is>
-          <t>8,341</t>
+          <t>2,229</t>
         </is>
       </c>
       <c r="I82" s="6" t="inlineStr">
         <is>
-          <t>의료용 기기 제조업</t>
+          <t>반도체 제조업</t>
         </is>
       </c>
       <c r="J82" s="6" t="inlineStr">
         <is>
-          <t>한국</t>
+          <t>DB</t>
         </is>
       </c>
       <c r="K82" s="6" t="inlineStr">
         <is>
-          <t>상장전</t>
+          <t>상장완료 (2026-08-25)</t>
         </is>
       </c>
     </row>
     <row r="83">
       <c r="A83" s="6" t="inlineStr">
         <is>
-          <t>2026-06-15</t>
+          <t>2026-06-24</t>
         </is>
       </c>
       <c r="B83" s="6" t="inlineStr">
         <is>
-          <t>에이치엘지노믹스</t>
+          <t>스카이랩스</t>
         </is>
       </c>
       <c r="C83" s="6" t="inlineStr">
@@ -4968,32 +4968,32 @@
       </c>
       <c r="F83" s="7" t="inlineStr">
         <is>
-          <t>28,877</t>
+          <t>7,936</t>
         </is>
       </c>
       <c r="G83" s="7" t="inlineStr">
         <is>
-          <t>8,452</t>
+          <t>-62,995</t>
         </is>
       </c>
       <c r="H83" s="7" t="inlineStr">
         <is>
-          <t>83,552</t>
+          <t>8,341</t>
         </is>
       </c>
       <c r="I83" s="6" t="inlineStr">
         <is>
-          <t>기초 의약물질 제조업</t>
+          <t>의료용 기기 제조업</t>
         </is>
       </c>
       <c r="J83" s="6" t="inlineStr">
         <is>
-          <t>KB, IBK</t>
+          <t>한국</t>
         </is>
       </c>
       <c r="K83" s="6" t="inlineStr">
         <is>
-          <t>상장완료 (2026-07-24)</t>
+          <t>상장승인(상장예정)</t>
         </is>
       </c>
     </row>
@@ -5005,7 +5005,7 @@
       </c>
       <c r="B84" s="6" t="inlineStr">
         <is>
-          <t>딜리셔스</t>
+          <t>에이치엘지노믹스</t>
         </is>
       </c>
       <c r="C84" s="6" t="inlineStr">
@@ -5025,44 +5025,44 @@
       </c>
       <c r="F84" s="7" t="inlineStr">
         <is>
-          <t>25,149</t>
+          <t>28,877</t>
         </is>
       </c>
       <c r="G84" s="7" t="inlineStr">
         <is>
-          <t>-20,419</t>
+          <t>8,452</t>
         </is>
       </c>
       <c r="H84" s="7" t="inlineStr">
         <is>
-          <t>-114,384</t>
+          <t>83,552</t>
         </is>
       </c>
       <c r="I84" s="6" t="inlineStr">
         <is>
-          <t>무점포 소매업</t>
+          <t>기초 의약물질 제조업</t>
         </is>
       </c>
       <c r="J84" s="6" t="inlineStr">
         <is>
-          <t>한국</t>
+          <t>KB, IBK</t>
         </is>
       </c>
       <c r="K84" s="6" t="inlineStr">
         <is>
-          <t>상장완료 (2026-08-12)</t>
+          <t>상장완료 (2026-07-24)</t>
         </is>
       </c>
     </row>
     <row r="85">
       <c r="A85" s="6" t="inlineStr">
         <is>
-          <t>2026-05-21</t>
+          <t>2026-06-15</t>
         </is>
       </c>
       <c r="B85" s="6" t="inlineStr">
         <is>
-          <t>인제니아테라퓨틱스</t>
+          <t>딜리셔스</t>
         </is>
       </c>
       <c r="C85" s="6" t="inlineStr">
@@ -5082,44 +5082,44 @@
       </c>
       <c r="F85" s="7" t="inlineStr">
         <is>
-          <t>2,588,400</t>
+          <t>25,149</t>
         </is>
       </c>
       <c r="G85" s="7" t="inlineStr">
         <is>
-          <t>15,755,864</t>
+          <t>-20,419</t>
         </is>
       </c>
       <c r="H85" s="7" t="inlineStr">
         <is>
-          <t>30,841,690</t>
+          <t>-114,384</t>
         </is>
       </c>
       <c r="I85" s="6" t="inlineStr">
         <is>
-          <t>자연과학 및 공학 연구개발업</t>
+          <t>무점포 소매업</t>
         </is>
       </c>
       <c r="J85" s="6" t="inlineStr">
         <is>
-          <t>삼성</t>
+          <t>한국</t>
         </is>
       </c>
       <c r="K85" s="6" t="inlineStr">
         <is>
-          <t>상장완료 (2026-08-18)</t>
+          <t>상장완료 (2026-08-12)</t>
         </is>
       </c>
     </row>
     <row r="86">
       <c r="A86" s="6" t="inlineStr">
         <is>
-          <t>2026-05-20</t>
+          <t>2026-05-21</t>
         </is>
       </c>
       <c r="B86" s="6" t="inlineStr">
         <is>
-          <t>한국제16호스팩</t>
+          <t>인제니아테라퓨틱스</t>
         </is>
       </c>
       <c r="C86" s="6" t="inlineStr">
@@ -5137,30 +5137,46 @@
           <t>FY25</t>
         </is>
       </c>
-      <c r="F86" s="7" t="inlineStr"/>
-      <c r="G86" s="7" t="inlineStr"/>
-      <c r="H86" s="7" t="inlineStr"/>
-      <c r="I86" s="6" t="inlineStr"/>
+      <c r="F86" s="7" t="inlineStr">
+        <is>
+          <t>2,588,400</t>
+        </is>
+      </c>
+      <c r="G86" s="7" t="inlineStr">
+        <is>
+          <t>15,755,864</t>
+        </is>
+      </c>
+      <c r="H86" s="7" t="inlineStr">
+        <is>
+          <t>30,841,690</t>
+        </is>
+      </c>
+      <c r="I86" s="6" t="inlineStr">
+        <is>
+          <t>자연과학 및 공학 연구개발업</t>
+        </is>
+      </c>
       <c r="J86" s="6" t="inlineStr">
         <is>
-          <t>한국</t>
+          <t>삼성</t>
         </is>
       </c>
       <c r="K86" s="6" t="inlineStr">
         <is>
-          <t>상장완료 (2026-06-30)</t>
+          <t>상장완료 (2026-08-18)</t>
         </is>
       </c>
     </row>
     <row r="87">
       <c r="A87" s="6" t="inlineStr">
         <is>
-          <t>2026-05-07</t>
+          <t>2026-05-20</t>
         </is>
       </c>
       <c r="B87" s="6" t="inlineStr">
         <is>
-          <t>레메디</t>
+          <t>한국제16호스팩</t>
         </is>
       </c>
       <c r="C87" s="6" t="inlineStr">
@@ -5178,34 +5194,18 @@
           <t>FY25</t>
         </is>
       </c>
-      <c r="F87" s="7" t="inlineStr">
-        <is>
-          <t>13,441</t>
-        </is>
-      </c>
-      <c r="G87" s="7" t="inlineStr">
-        <is>
-          <t>741</t>
-        </is>
-      </c>
-      <c r="H87" s="7" t="inlineStr">
-        <is>
-          <t>5,870</t>
-        </is>
-      </c>
-      <c r="I87" s="6" t="inlineStr">
-        <is>
-          <t>의료용 기기 제조업</t>
-        </is>
-      </c>
+      <c r="F87" s="7" t="inlineStr"/>
+      <c r="G87" s="7" t="inlineStr"/>
+      <c r="H87" s="7" t="inlineStr"/>
+      <c r="I87" s="6" t="inlineStr"/>
       <c r="J87" s="6" t="inlineStr">
         <is>
-          <t>KB</t>
+          <t>한국</t>
         </is>
       </c>
       <c r="K87" s="6" t="inlineStr">
         <is>
-          <t>상장완료 (2026-07-13)</t>
+          <t>상장완료 (2026-06-30)</t>
         </is>
       </c>
     </row>
@@ -5217,7 +5217,7 @@
       </c>
       <c r="B88" s="6" t="inlineStr">
         <is>
-          <t>케이앤에스아이앤씨</t>
+          <t>레메디</t>
         </is>
       </c>
       <c r="C88" s="6" t="inlineStr">
@@ -5237,44 +5237,44 @@
       </c>
       <c r="F88" s="7" t="inlineStr">
         <is>
-          <t>13,482</t>
+          <t>13,441</t>
         </is>
       </c>
       <c r="G88" s="7" t="inlineStr">
         <is>
-          <t>-2,213</t>
+          <t>741</t>
         </is>
       </c>
       <c r="H88" s="7" t="inlineStr">
         <is>
-          <t>4,273</t>
+          <t>5,870</t>
         </is>
       </c>
       <c r="I88" s="6" t="inlineStr">
         <is>
-          <t>통신 및 방송 장비 제조업</t>
+          <t>의료용 기기 제조업</t>
         </is>
       </c>
       <c r="J88" s="6" t="inlineStr">
         <is>
-          <t>IBK</t>
+          <t>KB</t>
         </is>
       </c>
       <c r="K88" s="6" t="inlineStr">
         <is>
-          <t>상장완료 (2026-08-13)</t>
+          <t>상장완료 (2026-07-13)</t>
         </is>
       </c>
     </row>
     <row r="89">
       <c r="A89" s="6" t="inlineStr">
         <is>
-          <t>2026-04-27</t>
+          <t>2026-05-07</t>
         </is>
       </c>
       <c r="B89" s="6" t="inlineStr">
         <is>
-          <t>메리츠제2호스팩</t>
+          <t>케이앤에스아이앤씨</t>
         </is>
       </c>
       <c r="C89" s="6" t="inlineStr">
@@ -5292,30 +5292,46 @@
           <t>FY25</t>
         </is>
       </c>
-      <c r="F89" s="7" t="inlineStr"/>
-      <c r="G89" s="7" t="inlineStr"/>
-      <c r="H89" s="7" t="inlineStr"/>
-      <c r="I89" s="6" t="inlineStr"/>
+      <c r="F89" s="7" t="inlineStr">
+        <is>
+          <t>13,482</t>
+        </is>
+      </c>
+      <c r="G89" s="7" t="inlineStr">
+        <is>
+          <t>-2,213</t>
+        </is>
+      </c>
+      <c r="H89" s="7" t="inlineStr">
+        <is>
+          <t>4,273</t>
+        </is>
+      </c>
+      <c r="I89" s="6" t="inlineStr">
+        <is>
+          <t>통신 및 방송 장비 제조업</t>
+        </is>
+      </c>
       <c r="J89" s="6" t="inlineStr">
         <is>
-          <t>메리츠</t>
+          <t>IBK</t>
         </is>
       </c>
       <c r="K89" s="6" t="inlineStr">
         <is>
-          <t>상장완료 (2026-06-19)</t>
+          <t>상장완료 (2026-08-13)</t>
         </is>
       </c>
     </row>
     <row r="90">
       <c r="A90" s="6" t="inlineStr">
         <is>
-          <t>2026-04-23</t>
+          <t>2026-04-27</t>
         </is>
       </c>
       <c r="B90" s="6" t="inlineStr">
         <is>
-          <t>빅웨이브로보틱스</t>
+          <t>메리츠제2호스팩</t>
         </is>
       </c>
       <c r="C90" s="6" t="inlineStr">
@@ -5330,49 +5346,33 @@
       </c>
       <c r="E90" s="6" t="inlineStr">
         <is>
-          <t>FY24</t>
-        </is>
-      </c>
-      <c r="F90" s="7" t="inlineStr">
-        <is>
-          <t>13,851</t>
-        </is>
-      </c>
-      <c r="G90" s="7" t="inlineStr">
-        <is>
-          <t>-5,856</t>
-        </is>
-      </c>
-      <c r="H90" s="7" t="inlineStr">
-        <is>
-          <t>9,470</t>
-        </is>
-      </c>
-      <c r="I90" s="6" t="inlineStr">
-        <is>
-          <t>소프트웨어 개발 및 공급업</t>
-        </is>
-      </c>
+          <t>FY25</t>
+        </is>
+      </c>
+      <c r="F90" s="7" t="inlineStr"/>
+      <c r="G90" s="7" t="inlineStr"/>
+      <c r="H90" s="7" t="inlineStr"/>
+      <c r="I90" s="6" t="inlineStr"/>
       <c r="J90" s="6" t="inlineStr">
         <is>
-          <t>유진, 미래</t>
+          <t>메리츠</t>
         </is>
       </c>
       <c r="K90" s="6" t="inlineStr">
         <is>
-          <t>상장전</t>
+          <t>상장완료 (2026-06-19)</t>
         </is>
       </c>
     </row>
     <row r="91">
       <c r="A91" s="6" t="inlineStr">
         <is>
-          <t>2026-04-09</t>
+          <t>2026-04-23</t>
         </is>
       </c>
       <c r="B91" s="6" t="inlineStr">
         <is>
-          <t>매드업</t>
+          <t>빅웨이브로보틱스</t>
         </is>
       </c>
       <c r="C91" s="6" t="inlineStr">
@@ -5392,44 +5392,44 @@
       </c>
       <c r="F91" s="7" t="inlineStr">
         <is>
-          <t>34,989</t>
+          <t>13,851</t>
         </is>
       </c>
       <c r="G91" s="7" t="inlineStr">
         <is>
-          <t>-2,747</t>
+          <t>-5,856</t>
         </is>
       </c>
       <c r="H91" s="7" t="inlineStr">
         <is>
-          <t>-15,766</t>
+          <t>9,470</t>
         </is>
       </c>
       <c r="I91" s="6" t="inlineStr">
         <is>
-          <t>광고</t>
+          <t>소프트웨어 개발 및 공급업</t>
         </is>
       </c>
       <c r="J91" s="6" t="inlineStr">
         <is>
-          <t>미래</t>
+          <t>유진, 미래</t>
         </is>
       </c>
       <c r="K91" s="6" t="inlineStr">
         <is>
-          <t>상장완료 (2026-07-01)</t>
+          <t>상장전</t>
         </is>
       </c>
     </row>
     <row r="92">
       <c r="A92" s="6" t="inlineStr">
         <is>
-          <t>2026-04-02</t>
+          <t>2026-04-09</t>
         </is>
       </c>
       <c r="B92" s="6" t="inlineStr">
         <is>
-          <t>져스텍</t>
+          <t>매드업</t>
         </is>
       </c>
       <c r="C92" s="6" t="inlineStr">
@@ -5449,32 +5449,32 @@
       </c>
       <c r="F92" s="7" t="inlineStr">
         <is>
-          <t>19,851</t>
+          <t>34,989</t>
         </is>
       </c>
       <c r="G92" s="7" t="inlineStr">
         <is>
-          <t>444</t>
+          <t>-2,747</t>
         </is>
       </c>
       <c r="H92" s="7" t="inlineStr">
         <is>
-          <t>10,953</t>
+          <t>-15,766</t>
         </is>
       </c>
       <c r="I92" s="6" t="inlineStr">
         <is>
-          <t>기계</t>
+          <t>광고</t>
         </is>
       </c>
       <c r="J92" s="6" t="inlineStr">
         <is>
-          <t>삼성</t>
+          <t>미래</t>
         </is>
       </c>
       <c r="K92" s="6" t="inlineStr">
         <is>
-          <t>상장완료 (2026-06-29)</t>
+          <t>상장완료 (2026-07-01)</t>
         </is>
       </c>
     </row>
@@ -5486,7 +5486,7 @@
       </c>
       <c r="B93" s="6" t="inlineStr">
         <is>
-          <t>스트라드비젼</t>
+          <t>져스텍</t>
         </is>
       </c>
       <c r="C93" s="6" t="inlineStr">
@@ -5506,44 +5506,44 @@
       </c>
       <c r="F93" s="7" t="inlineStr">
         <is>
-          <t>11,539</t>
+          <t>19,851</t>
         </is>
       </c>
       <c r="G93" s="7" t="inlineStr">
         <is>
-          <t>-65,529</t>
+          <t>444</t>
         </is>
       </c>
       <c r="H93" s="7" t="inlineStr">
         <is>
-          <t>-245,151</t>
+          <t>10,953</t>
         </is>
       </c>
       <c r="I93" s="6" t="inlineStr">
         <is>
-          <t>소프트웨어</t>
+          <t>기계</t>
         </is>
       </c>
       <c r="J93" s="6" t="inlineStr">
         <is>
-          <t>KB</t>
+          <t>삼성</t>
         </is>
       </c>
       <c r="K93" s="6" t="inlineStr">
         <is>
-          <t>상장완료 (2026-06-30)</t>
+          <t>상장완료 (2026-06-29)</t>
         </is>
       </c>
     </row>
     <row r="94">
       <c r="A94" s="6" t="inlineStr">
         <is>
-          <t>2026-03-30</t>
+          <t>2026-04-02</t>
         </is>
       </c>
       <c r="B94" s="6" t="inlineStr">
         <is>
-          <t>대신밸런스제20호스팩</t>
+          <t>스트라드비젼</t>
         </is>
       </c>
       <c r="C94" s="6" t="inlineStr">
@@ -5558,33 +5558,49 @@
       </c>
       <c r="E94" s="6" t="inlineStr">
         <is>
-          <t>FY25</t>
-        </is>
-      </c>
-      <c r="F94" s="7" t="inlineStr"/>
-      <c r="G94" s="7" t="inlineStr"/>
-      <c r="H94" s="7" t="inlineStr"/>
-      <c r="I94" s="6" t="inlineStr"/>
+          <t>FY24</t>
+        </is>
+      </c>
+      <c r="F94" s="7" t="inlineStr">
+        <is>
+          <t>11,539</t>
+        </is>
+      </c>
+      <c r="G94" s="7" t="inlineStr">
+        <is>
+          <t>-65,529</t>
+        </is>
+      </c>
+      <c r="H94" s="7" t="inlineStr">
+        <is>
+          <t>-245,151</t>
+        </is>
+      </c>
+      <c r="I94" s="6" t="inlineStr">
+        <is>
+          <t>소프트웨어</t>
+        </is>
+      </c>
       <c r="J94" s="6" t="inlineStr">
         <is>
-          <t>대신</t>
+          <t>KB</t>
         </is>
       </c>
       <c r="K94" s="6" t="inlineStr">
         <is>
-          <t>상장완료 (2026-06-05)</t>
+          <t>상장완료 (2026-06-30)</t>
         </is>
       </c>
     </row>
     <row r="95">
       <c r="A95" s="6" t="inlineStr">
         <is>
-          <t>2026-03-26</t>
+          <t>2026-03-30</t>
         </is>
       </c>
       <c r="B95" s="6" t="inlineStr">
         <is>
-          <t>피스피스스튜디오</t>
+          <t>대신밸런스제20호스팩</t>
         </is>
       </c>
       <c r="C95" s="6" t="inlineStr">
@@ -5599,37 +5615,21 @@
       </c>
       <c r="E95" s="6" t="inlineStr">
         <is>
-          <t>FY24</t>
-        </is>
-      </c>
-      <c r="F95" s="7" t="inlineStr">
-        <is>
-          <t>113,777</t>
-        </is>
-      </c>
-      <c r="G95" s="7" t="inlineStr">
-        <is>
-          <t>17,603</t>
-        </is>
-      </c>
-      <c r="H95" s="7" t="inlineStr">
-        <is>
-          <t>55,861</t>
-        </is>
-      </c>
-      <c r="I95" s="6" t="inlineStr">
-        <is>
-          <t>섬유,의류,신발,호화품</t>
-        </is>
-      </c>
+          <t>FY25</t>
+        </is>
+      </c>
+      <c r="F95" s="7" t="inlineStr"/>
+      <c r="G95" s="7" t="inlineStr"/>
+      <c r="H95" s="7" t="inlineStr"/>
+      <c r="I95" s="6" t="inlineStr"/>
       <c r="J95" s="6" t="inlineStr">
         <is>
-          <t>NH, 미래</t>
+          <t>대신</t>
         </is>
       </c>
       <c r="K95" s="6" t="inlineStr">
         <is>
-          <t>상장완료 (2026-06-08)</t>
+          <t>상장완료 (2026-06-05)</t>
         </is>
       </c>
     </row>
@@ -5641,7 +5641,7 @@
       </c>
       <c r="B96" s="6" t="inlineStr">
         <is>
-          <t>폴레드</t>
+          <t>피스피스스튜디오</t>
         </is>
       </c>
       <c r="C96" s="6" t="inlineStr">
@@ -5661,32 +5661,32 @@
       </c>
       <c r="F96" s="7" t="inlineStr">
         <is>
-          <t>52,808</t>
+          <t>113,777</t>
         </is>
       </c>
       <c r="G96" s="7" t="inlineStr">
         <is>
-          <t>543</t>
+          <t>17,603</t>
         </is>
       </c>
       <c r="H96" s="7" t="inlineStr">
         <is>
-          <t>25,416</t>
+          <t>55,861</t>
         </is>
       </c>
       <c r="I96" s="6" t="inlineStr">
         <is>
-          <t>가정용기기와용품</t>
+          <t>섬유,의류,신발,호화품</t>
         </is>
       </c>
       <c r="J96" s="6" t="inlineStr">
         <is>
-          <t>NH</t>
+          <t>NH, 미래</t>
         </is>
       </c>
       <c r="K96" s="6" t="inlineStr">
         <is>
-          <t>상장완료 (2026-05-14)</t>
+          <t>상장완료 (2026-06-08)</t>
         </is>
       </c>
     </row>
@@ -5698,7 +5698,7 @@
       </c>
       <c r="B97" s="6" t="inlineStr">
         <is>
-          <t>레몬헬스케어</t>
+          <t>폴레드</t>
         </is>
       </c>
       <c r="C97" s="6" t="inlineStr">
@@ -5718,44 +5718,44 @@
       </c>
       <c r="F97" s="7" t="inlineStr">
         <is>
-          <t>14,877</t>
+          <t>52,808</t>
         </is>
       </c>
       <c r="G97" s="7" t="inlineStr">
         <is>
-          <t>-2,898</t>
+          <t>543</t>
         </is>
       </c>
       <c r="H97" s="7" t="inlineStr">
         <is>
-          <t>-31,162</t>
+          <t>25,416</t>
         </is>
       </c>
       <c r="I97" s="6" t="inlineStr">
         <is>
-          <t>건강관리업체및서비스</t>
+          <t>가정용기기와용품</t>
         </is>
       </c>
       <c r="J97" s="6" t="inlineStr">
         <is>
-          <t>KB</t>
+          <t>NH</t>
         </is>
       </c>
       <c r="K97" s="6" t="inlineStr">
         <is>
-          <t>상장완료 (2026-07-06)</t>
+          <t>상장완료 (2026-05-14)</t>
         </is>
       </c>
     </row>
     <row r="98">
       <c r="A98" s="6" t="inlineStr">
         <is>
-          <t>2026-02-27</t>
+          <t>2026-03-26</t>
         </is>
       </c>
       <c r="B98" s="6" t="inlineStr">
         <is>
-          <t>마키나락스</t>
+          <t>레몬헬스케어</t>
         </is>
       </c>
       <c r="C98" s="6" t="inlineStr">
@@ -5775,32 +5775,32 @@
       </c>
       <c r="F98" s="7" t="inlineStr">
         <is>
-          <t>8,294</t>
+          <t>14,877</t>
         </is>
       </c>
       <c r="G98" s="7" t="inlineStr">
         <is>
-          <t>-6,073</t>
+          <t>-2,898</t>
         </is>
       </c>
       <c r="H98" s="7" t="inlineStr">
         <is>
-          <t>2,680</t>
+          <t>-31,162</t>
         </is>
       </c>
       <c r="I98" s="6" t="inlineStr">
         <is>
-          <t>소프트웨어</t>
+          <t>건강관리업체및서비스</t>
         </is>
       </c>
       <c r="J98" s="6" t="inlineStr">
         <is>
-          <t>미래</t>
+          <t>KB</t>
         </is>
       </c>
       <c r="K98" s="6" t="inlineStr">
         <is>
-          <t>상장완료 (2026-05-20)</t>
+          <t>상장완료 (2026-07-06)</t>
         </is>
       </c>
     </row>
@@ -5812,7 +5812,7 @@
       </c>
       <c r="B99" s="6" t="inlineStr">
         <is>
-          <t>채비</t>
+          <t>마키나락스</t>
         </is>
       </c>
       <c r="C99" s="6" t="inlineStr">
@@ -5832,44 +5832,44 @@
       </c>
       <c r="F99" s="7" t="inlineStr">
         <is>
-          <t>85,082</t>
+          <t>8,294</t>
         </is>
       </c>
       <c r="G99" s="7" t="inlineStr">
         <is>
-          <t>-54,495</t>
+          <t>-6,073</t>
         </is>
       </c>
       <c r="H99" s="7" t="inlineStr">
         <is>
-          <t>96,866</t>
+          <t>2,680</t>
         </is>
       </c>
       <c r="I99" s="6" t="inlineStr">
         <is>
-          <t>전기제품</t>
+          <t>소프트웨어</t>
         </is>
       </c>
       <c r="J99" s="6" t="inlineStr">
         <is>
-          <t>KB, 삼성, 대신, 하나</t>
+          <t>미래</t>
         </is>
       </c>
       <c r="K99" s="6" t="inlineStr">
         <is>
-          <t>상장완료 (2026-04-29)</t>
+          <t>상장완료 (2026-05-20)</t>
         </is>
       </c>
     </row>
     <row r="100">
       <c r="A100" s="6" t="inlineStr">
         <is>
-          <t>2026-02-10</t>
+          <t>2026-02-27</t>
         </is>
       </c>
       <c r="B100" s="6" t="inlineStr">
         <is>
-          <t>키움히어로제2호스팩</t>
+          <t>채비</t>
         </is>
       </c>
       <c r="C100" s="6" t="inlineStr">
@@ -5887,30 +5887,46 @@
           <t>FY24</t>
         </is>
       </c>
-      <c r="F100" s="7" t="inlineStr"/>
-      <c r="G100" s="7" t="inlineStr"/>
-      <c r="H100" s="7" t="inlineStr"/>
-      <c r="I100" s="6" t="inlineStr"/>
+      <c r="F100" s="7" t="inlineStr">
+        <is>
+          <t>85,082</t>
+        </is>
+      </c>
+      <c r="G100" s="7" t="inlineStr">
+        <is>
+          <t>-54,495</t>
+        </is>
+      </c>
+      <c r="H100" s="7" t="inlineStr">
+        <is>
+          <t>96,866</t>
+        </is>
+      </c>
+      <c r="I100" s="6" t="inlineStr">
+        <is>
+          <t>전기제품</t>
+        </is>
+      </c>
       <c r="J100" s="6" t="inlineStr">
         <is>
-          <t>키움</t>
+          <t>KB, 삼성, 대신, 하나</t>
         </is>
       </c>
       <c r="K100" s="6" t="inlineStr">
         <is>
-          <t>상장완료 (2026-04-23)</t>
+          <t>상장완료 (2026-04-29)</t>
         </is>
       </c>
     </row>
     <row r="101">
       <c r="A101" s="6" t="inlineStr">
         <is>
-          <t>2026-02-05</t>
+          <t>2026-02-10</t>
         </is>
       </c>
       <c r="B101" s="6" t="inlineStr">
         <is>
-          <t>세미티에스</t>
+          <t>키움히어로제2호스팩</t>
         </is>
       </c>
       <c r="C101" s="6" t="inlineStr">
@@ -5920,7 +5936,7 @@
       </c>
       <c r="D101" s="6" t="inlineStr">
         <is>
-          <t>스팩 소멸합병</t>
+          <t>신규상장</t>
         </is>
       </c>
       <c r="E101" s="6" t="inlineStr">
@@ -5928,46 +5944,30 @@
           <t>FY24</t>
         </is>
       </c>
-      <c r="F101" s="7" t="inlineStr">
-        <is>
-          <t>20,808</t>
-        </is>
-      </c>
-      <c r="G101" s="7" t="inlineStr">
-        <is>
-          <t>7,337</t>
-        </is>
-      </c>
-      <c r="H101" s="7" t="inlineStr">
-        <is>
-          <t>26,616</t>
-        </is>
-      </c>
-      <c r="I101" s="6" t="inlineStr">
-        <is>
-          <t>반도체와반도체장비</t>
-        </is>
-      </c>
+      <c r="F101" s="7" t="inlineStr"/>
+      <c r="G101" s="7" t="inlineStr"/>
+      <c r="H101" s="7" t="inlineStr"/>
+      <c r="I101" s="6" t="inlineStr"/>
       <c r="J101" s="6" t="inlineStr">
         <is>
-          <t>NH</t>
+          <t>키움</t>
         </is>
       </c>
       <c r="K101" s="6" t="inlineStr">
         <is>
-          <t>상장완료 (2026-02-05)</t>
+          <t>상장완료 (2026-04-23)</t>
         </is>
       </c>
     </row>
     <row r="102">
       <c r="A102" s="6" t="inlineStr">
         <is>
-          <t>2026-02-02</t>
+          <t>2026-02-05</t>
         </is>
       </c>
       <c r="B102" s="6" t="inlineStr">
         <is>
-          <t>교보20호스팩</t>
+          <t>세미티에스</t>
         </is>
       </c>
       <c r="C102" s="6" t="inlineStr">
@@ -5977,7 +5977,7 @@
       </c>
       <c r="D102" s="6" t="inlineStr">
         <is>
-          <t>신규상장</t>
+          <t>스팩 소멸합병</t>
         </is>
       </c>
       <c r="E102" s="6" t="inlineStr">
@@ -5985,30 +5985,46 @@
           <t>FY24</t>
         </is>
       </c>
-      <c r="F102" s="7" t="inlineStr"/>
-      <c r="G102" s="7" t="inlineStr"/>
-      <c r="H102" s="7" t="inlineStr"/>
-      <c r="I102" s="6" t="inlineStr"/>
+      <c r="F102" s="7" t="inlineStr">
+        <is>
+          <t>20,808</t>
+        </is>
+      </c>
+      <c r="G102" s="7" t="inlineStr">
+        <is>
+          <t>7,337</t>
+        </is>
+      </c>
+      <c r="H102" s="7" t="inlineStr">
+        <is>
+          <t>26,616</t>
+        </is>
+      </c>
+      <c r="I102" s="6" t="inlineStr">
+        <is>
+          <t>반도체와반도체장비</t>
+        </is>
+      </c>
       <c r="J102" s="6" t="inlineStr">
         <is>
-          <t>교보</t>
+          <t>NH</t>
         </is>
       </c>
       <c r="K102" s="6" t="inlineStr">
         <is>
-          <t>상장완료 (2026-04-02)</t>
+          <t>상장완료 (2026-02-05)</t>
         </is>
       </c>
     </row>
     <row r="103">
       <c r="A103" s="6" t="inlineStr">
         <is>
-          <t>2026-01-29</t>
+          <t>2026-02-02</t>
         </is>
       </c>
       <c r="B103" s="6" t="inlineStr">
         <is>
-          <t>케이피항공산업</t>
+          <t>교보20호스팩</t>
         </is>
       </c>
       <c r="C103" s="6" t="inlineStr">
@@ -6018,7 +6034,7 @@
       </c>
       <c r="D103" s="6" t="inlineStr">
         <is>
-          <t>스팩 소멸합병</t>
+          <t>신규상장</t>
         </is>
       </c>
       <c r="E103" s="6" t="inlineStr">
@@ -6026,34 +6042,18 @@
           <t>FY24</t>
         </is>
       </c>
-      <c r="F103" s="7" t="inlineStr">
-        <is>
-          <t>49,651</t>
-        </is>
-      </c>
-      <c r="G103" s="7" t="inlineStr">
-        <is>
-          <t>3,018</t>
-        </is>
-      </c>
-      <c r="H103" s="7" t="inlineStr">
-        <is>
-          <t>15,901</t>
-        </is>
-      </c>
-      <c r="I103" s="6" t="inlineStr">
-        <is>
-          <t>우주항공과국방</t>
-        </is>
-      </c>
+      <c r="F103" s="7" t="inlineStr"/>
+      <c r="G103" s="7" t="inlineStr"/>
+      <c r="H103" s="7" t="inlineStr"/>
+      <c r="I103" s="6" t="inlineStr"/>
       <c r="J103" s="6" t="inlineStr">
         <is>
-          <t>NH</t>
+          <t>교보</t>
         </is>
       </c>
       <c r="K103" s="6" t="inlineStr">
         <is>
-          <t>상장완료 (2026-01-29)</t>
+          <t>상장완료 (2026-04-02)</t>
         </is>
       </c>
     </row>
@@ -6065,7 +6065,7 @@
       </c>
       <c r="B104" s="6" t="inlineStr">
         <is>
-          <t>한패스</t>
+          <t>케이피항공산업</t>
         </is>
       </c>
       <c r="C104" s="6" t="inlineStr">
@@ -6075,7 +6075,7 @@
       </c>
       <c r="D104" s="6" t="inlineStr">
         <is>
-          <t>신규상장</t>
+          <t>스팩 소멸합병</t>
         </is>
       </c>
       <c r="E104" s="6" t="inlineStr">
@@ -6085,44 +6085,44 @@
       </c>
       <c r="F104" s="7" t="inlineStr">
         <is>
-          <t>55,297</t>
+          <t>49,651</t>
         </is>
       </c>
       <c r="G104" s="7" t="inlineStr">
         <is>
-          <t>4,403</t>
+          <t>3,018</t>
         </is>
       </c>
       <c r="H104" s="7" t="inlineStr">
         <is>
-          <t>-28,065</t>
+          <t>15,901</t>
         </is>
       </c>
       <c r="I104" s="6" t="inlineStr">
         <is>
-          <t>IT서비스</t>
+          <t>우주항공과국방</t>
         </is>
       </c>
       <c r="J104" s="6" t="inlineStr">
         <is>
-          <t>한국, 대신</t>
+          <t>NH</t>
         </is>
       </c>
       <c r="K104" s="6" t="inlineStr">
         <is>
-          <t>상장완료 (2026-03-25)</t>
+          <t>상장완료 (2026-01-29)</t>
         </is>
       </c>
     </row>
     <row r="105">
       <c r="A105" s="6" t="inlineStr">
         <is>
-          <t>2026-01-22</t>
+          <t>2026-01-29</t>
         </is>
       </c>
       <c r="B105" s="6" t="inlineStr">
         <is>
-          <t>신한제18호스팩</t>
+          <t>한패스</t>
         </is>
       </c>
       <c r="C105" s="6" t="inlineStr">
@@ -6140,30 +6140,46 @@
           <t>FY24</t>
         </is>
       </c>
-      <c r="F105" s="7" t="inlineStr"/>
-      <c r="G105" s="7" t="inlineStr"/>
-      <c r="H105" s="7" t="inlineStr"/>
-      <c r="I105" s="6" t="inlineStr"/>
+      <c r="F105" s="7" t="inlineStr">
+        <is>
+          <t>55,297</t>
+        </is>
+      </c>
+      <c r="G105" s="7" t="inlineStr">
+        <is>
+          <t>4,403</t>
+        </is>
+      </c>
+      <c r="H105" s="7" t="inlineStr">
+        <is>
+          <t>-28,065</t>
+        </is>
+      </c>
+      <c r="I105" s="6" t="inlineStr">
+        <is>
+          <t>IT서비스</t>
+        </is>
+      </c>
       <c r="J105" s="6" t="inlineStr">
         <is>
-          <t>신한</t>
+          <t>한국, 대신</t>
         </is>
       </c>
       <c r="K105" s="6" t="inlineStr">
         <is>
-          <t>상장완료 (2026-04-30)</t>
+          <t>상장완료 (2026-03-25)</t>
         </is>
       </c>
     </row>
     <row r="106">
       <c r="A106" s="6" t="inlineStr">
         <is>
-          <t>2026-01-20</t>
+          <t>2026-01-22</t>
         </is>
       </c>
       <c r="B106" s="6" t="inlineStr">
         <is>
-          <t>엔에이치스팩33호</t>
+          <t>신한제18호스팩</t>
         </is>
       </c>
       <c r="C106" s="6" t="inlineStr">
@@ -6187,24 +6203,24 @@
       <c r="I106" s="6" t="inlineStr"/>
       <c r="J106" s="6" t="inlineStr">
         <is>
-          <t>NH</t>
+          <t>신한</t>
         </is>
       </c>
       <c r="K106" s="6" t="inlineStr">
         <is>
-          <t>상장완료 (2026-03-27)</t>
+          <t>상장완료 (2026-04-30)</t>
         </is>
       </c>
     </row>
     <row r="107">
       <c r="A107" s="6" t="inlineStr">
         <is>
-          <t>2026-01-19</t>
+          <t>2026-01-20</t>
         </is>
       </c>
       <c r="B107" s="6" t="inlineStr">
         <is>
-          <t>신한제17호스팩</t>
+          <t>엔에이치스팩33호</t>
         </is>
       </c>
       <c r="C107" s="6" t="inlineStr">
@@ -6228,24 +6244,24 @@
       <c r="I107" s="6" t="inlineStr"/>
       <c r="J107" s="6" t="inlineStr">
         <is>
-          <t>신한</t>
+          <t>NH</t>
         </is>
       </c>
       <c r="K107" s="6" t="inlineStr">
         <is>
-          <t>상장완료 (2026-04-01)</t>
+          <t>상장완료 (2026-03-27)</t>
         </is>
       </c>
     </row>
     <row r="108">
       <c r="A108" s="6" t="inlineStr">
         <is>
-          <t>2026-01-16</t>
+          <t>2026-01-19</t>
         </is>
       </c>
       <c r="B108" s="6" t="inlineStr">
         <is>
-          <t>아이엠바이오로직스</t>
+          <t>신한제17호스팩</t>
         </is>
       </c>
       <c r="C108" s="6" t="inlineStr">
@@ -6263,34 +6279,18 @@
           <t>FY24</t>
         </is>
       </c>
-      <c r="F108" s="7" t="inlineStr">
-        <is>
-          <t>27,594</t>
-        </is>
-      </c>
-      <c r="G108" s="7" t="inlineStr">
-        <is>
-          <t>-11,884</t>
-        </is>
-      </c>
-      <c r="H108" s="7" t="inlineStr">
-        <is>
-          <t>-77,202</t>
-        </is>
-      </c>
-      <c r="I108" s="6" t="inlineStr">
-        <is>
-          <t>제약</t>
-        </is>
-      </c>
+      <c r="F108" s="7" t="inlineStr"/>
+      <c r="G108" s="7" t="inlineStr"/>
+      <c r="H108" s="7" t="inlineStr"/>
+      <c r="I108" s="6" t="inlineStr"/>
       <c r="J108" s="6" t="inlineStr">
         <is>
-          <t>한국, 신한</t>
+          <t>신한</t>
         </is>
       </c>
       <c r="K108" s="6" t="inlineStr">
         <is>
-          <t>상장완료 (2026-03-20)</t>
+          <t>상장완료 (2026-04-01)</t>
         </is>
       </c>
     </row>
@@ -6302,7 +6302,7 @@
       </c>
       <c r="B109" s="6" t="inlineStr">
         <is>
-          <t>에스팀</t>
+          <t>아이엠바이오로직스</t>
         </is>
       </c>
       <c r="C109" s="6" t="inlineStr">
@@ -6322,232 +6322,232 @@
       </c>
       <c r="F109" s="7" t="inlineStr">
         <is>
-          <t>35,574</t>
+          <t>27,594</t>
         </is>
       </c>
       <c r="G109" s="7" t="inlineStr">
         <is>
-          <t>1,372</t>
+          <t>-11,884</t>
         </is>
       </c>
       <c r="H109" s="7" t="inlineStr">
         <is>
-          <t>12,331</t>
+          <t>-77,202</t>
         </is>
       </c>
       <c r="I109" s="6" t="inlineStr">
         <is>
-          <t>광고</t>
+          <t>제약</t>
         </is>
       </c>
       <c r="J109" s="6" t="inlineStr">
         <is>
-          <t>한국</t>
+          <t>한국, 신한</t>
         </is>
       </c>
       <c r="K109" s="6" t="inlineStr">
         <is>
-          <t>상장완료 (2026-03-06)</t>
+          <t>상장완료 (2026-03-20)</t>
         </is>
       </c>
     </row>
     <row r="110">
       <c r="A110" s="6" t="inlineStr">
         <is>
+          <t>2026-01-16</t>
+        </is>
+      </c>
+      <c r="B110" s="6" t="inlineStr">
+        <is>
+          <t>에스팀</t>
+        </is>
+      </c>
+      <c r="C110" s="6" t="inlineStr">
+        <is>
+          <t>코스닥</t>
+        </is>
+      </c>
+      <c r="D110" s="6" t="inlineStr">
+        <is>
+          <t>신규상장</t>
+        </is>
+      </c>
+      <c r="E110" s="6" t="inlineStr">
+        <is>
+          <t>FY24</t>
+        </is>
+      </c>
+      <c r="F110" s="7" t="inlineStr">
+        <is>
+          <t>35,574</t>
+        </is>
+      </c>
+      <c r="G110" s="7" t="inlineStr">
+        <is>
+          <t>1,372</t>
+        </is>
+      </c>
+      <c r="H110" s="7" t="inlineStr">
+        <is>
+          <t>12,331</t>
+        </is>
+      </c>
+      <c r="I110" s="6" t="inlineStr">
+        <is>
+          <t>광고</t>
+        </is>
+      </c>
+      <c r="J110" s="6" t="inlineStr">
+        <is>
+          <t>한국</t>
+        </is>
+      </c>
+      <c r="K110" s="6" t="inlineStr">
+        <is>
+          <t>상장완료 (2026-03-06)</t>
+        </is>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" s="6" t="inlineStr">
+        <is>
           <t>2026-01-12</t>
         </is>
       </c>
-      <c r="B110" s="6" t="inlineStr">
+      <c r="B111" s="6" t="inlineStr">
         <is>
           <t>케이뱅크</t>
         </is>
       </c>
-      <c r="C110" s="6" t="inlineStr">
+      <c r="C111" s="6" t="inlineStr">
         <is>
           <t>유가</t>
         </is>
       </c>
-      <c r="D110" s="6" t="inlineStr">
+      <c r="D111" s="6" t="inlineStr">
         <is>
           <t>신규상장</t>
         </is>
       </c>
-      <c r="E110" s="6" t="inlineStr">
+      <c r="E111" s="6" t="inlineStr">
         <is>
           <t>FY24</t>
         </is>
       </c>
-      <c r="F110" s="7" t="inlineStr">
+      <c r="F111" s="7" t="inlineStr">
         <is>
           <t>1,228,501</t>
         </is>
       </c>
-      <c r="G110" s="7" t="inlineStr">
+      <c r="G111" s="7" t="inlineStr">
         <is>
           <t>128,053</t>
         </is>
       </c>
-      <c r="H110" s="7" t="inlineStr">
+      <c r="H111" s="7" t="inlineStr">
         <is>
           <t>1,995,845</t>
         </is>
       </c>
-      <c r="I110" s="6" t="inlineStr">
+      <c r="I111" s="6" t="inlineStr">
         <is>
           <t>은행</t>
         </is>
       </c>
-      <c r="J110" s="6" t="inlineStr">
+      <c r="J111" s="6" t="inlineStr">
         <is>
           <t>NH, 삼성</t>
         </is>
       </c>
-      <c r="K110" s="6" t="inlineStr">
+      <c r="K111" s="6" t="inlineStr">
         <is>
           <t>상장완료 (2026-03-05)</t>
         </is>
       </c>
     </row>
-    <row r="112">
-      <c r="A112" s="3" t="inlineStr">
+    <row r="113">
+      <c r="A113" s="3" t="inlineStr">
         <is>
           <t>■ 철회·미승인  (18건)</t>
         </is>
       </c>
-      <c r="B112" s="4" t="n"/>
-      <c r="C112" s="4" t="n"/>
-      <c r="D112" s="4" t="n"/>
-      <c r="E112" s="4" t="n"/>
-      <c r="F112" s="4" t="n"/>
-      <c r="G112" s="4" t="n"/>
-      <c r="H112" s="4" t="n"/>
-      <c r="I112" s="4" t="n"/>
-      <c r="J112" s="4" t="n"/>
-      <c r="K112" s="4" t="n"/>
-    </row>
-    <row r="113">
-      <c r="A113" s="5" t="inlineStr">
+      <c r="B113" s="4" t="n"/>
+      <c r="C113" s="4" t="n"/>
+      <c r="D113" s="4" t="n"/>
+      <c r="E113" s="4" t="n"/>
+      <c r="F113" s="4" t="n"/>
+      <c r="G113" s="4" t="n"/>
+      <c r="H113" s="4" t="n"/>
+      <c r="I113" s="4" t="n"/>
+      <c r="J113" s="4" t="n"/>
+      <c r="K113" s="4" t="n"/>
+    </row>
+    <row r="114">
+      <c r="A114" s="5" t="inlineStr">
         <is>
           <t>일자</t>
         </is>
       </c>
-      <c r="B113" s="5" t="inlineStr">
+      <c r="B114" s="5" t="inlineStr">
         <is>
           <t>회사명</t>
         </is>
       </c>
-      <c r="C113" s="5" t="inlineStr">
+      <c r="C114" s="5" t="inlineStr">
         <is>
           <t>시장</t>
         </is>
       </c>
-      <c r="D113" s="5" t="inlineStr">
+      <c r="D114" s="5" t="inlineStr">
         <is>
           <t>상장유형</t>
         </is>
       </c>
-      <c r="E113" s="5" t="inlineStr">
+      <c r="E114" s="5" t="inlineStr">
         <is>
           <t>기준연도</t>
         </is>
       </c>
-      <c r="F113" s="5" t="inlineStr">
+      <c r="F114" s="5" t="inlineStr">
         <is>
           <t>매출액</t>
         </is>
       </c>
-      <c r="G113" s="5" t="inlineStr">
+      <c r="G114" s="5" t="inlineStr">
         <is>
           <t>순이익</t>
         </is>
       </c>
-      <c r="H113" s="5" t="inlineStr">
+      <c r="H114" s="5" t="inlineStr">
         <is>
           <t>자기자본</t>
         </is>
       </c>
-      <c r="I113" s="5" t="inlineStr">
+      <c r="I114" s="5" t="inlineStr">
         <is>
           <t>업종</t>
         </is>
       </c>
-      <c r="J113" s="5" t="inlineStr">
+      <c r="J114" s="5" t="inlineStr">
         <is>
           <t>대표주관사</t>
         </is>
       </c>
-      <c r="K113" s="5" t="inlineStr">
+      <c r="K114" s="5" t="inlineStr">
         <is>
           <t>현황</t>
-        </is>
-      </c>
-    </row>
-    <row r="114">
-      <c r="A114" s="6" t="inlineStr">
-        <is>
-          <t>2026-08-31</t>
-        </is>
-      </c>
-      <c r="B114" s="6" t="inlineStr">
-        <is>
-          <t>텔레픽스</t>
-        </is>
-      </c>
-      <c r="C114" s="6" t="inlineStr">
-        <is>
-          <t>코스닥</t>
-        </is>
-      </c>
-      <c r="D114" s="6" t="inlineStr">
-        <is>
-          <t>신규상장</t>
-        </is>
-      </c>
-      <c r="E114" s="6" t="inlineStr">
-        <is>
-          <t>FY25</t>
-        </is>
-      </c>
-      <c r="F114" s="7" t="inlineStr">
-        <is>
-          <t>4,896</t>
-        </is>
-      </c>
-      <c r="G114" s="7" t="inlineStr">
-        <is>
-          <t>-16,214</t>
-        </is>
-      </c>
-      <c r="H114" s="7" t="inlineStr">
-        <is>
-          <t>9,146</t>
-        </is>
-      </c>
-      <c r="I114" s="6" t="inlineStr">
-        <is>
-          <t>소프트웨어 개발 및 공급업</t>
-        </is>
-      </c>
-      <c r="J114" s="6" t="inlineStr">
-        <is>
-          <t>미래</t>
-        </is>
-      </c>
-      <c r="K114" s="6" t="inlineStr">
-        <is>
-          <t>심사 철회</t>
         </is>
       </c>
     </row>
     <row r="115">
       <c r="A115" s="6" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-31</t>
         </is>
       </c>
       <c r="B115" s="6" t="inlineStr">
         <is>
-          <t>씨엠디엘</t>
+          <t>텔레픽스</t>
         </is>
       </c>
       <c r="C115" s="6" t="inlineStr">
@@ -6557,37 +6557,37 @@
       </c>
       <c r="D115" s="6" t="inlineStr">
         <is>
-          <t>스팩 소멸합병</t>
+          <t>신규상장</t>
         </is>
       </c>
       <c r="E115" s="6" t="inlineStr">
         <is>
-          <t>FY24</t>
+          <t>FY25</t>
         </is>
       </c>
       <c r="F115" s="7" t="inlineStr">
         <is>
-          <t>39,991</t>
+          <t>4,896</t>
         </is>
       </c>
       <c r="G115" s="7" t="inlineStr">
         <is>
-          <t>3,541</t>
+          <t>-16,214</t>
         </is>
       </c>
       <c r="H115" s="7" t="inlineStr">
         <is>
-          <t>503</t>
+          <t>9,146</t>
         </is>
       </c>
       <c r="I115" s="6" t="inlineStr">
         <is>
-          <t>기타 기초 유기 화학물질 제조업</t>
+          <t>소프트웨어 개발 및 공급업</t>
         </is>
       </c>
       <c r="J115" s="6" t="inlineStr">
         <is>
-          <t>교보</t>
+          <t>미래</t>
         </is>
       </c>
       <c r="K115" s="6" t="inlineStr">
@@ -6599,12 +6599,12 @@
     <row r="116">
       <c r="A116" s="6" t="inlineStr">
         <is>
-          <t>2026-07-23</t>
+          <t>2026-07-31</t>
         </is>
       </c>
       <c r="B116" s="6" t="inlineStr">
         <is>
-          <t>모비어스</t>
+          <t>씨엠디엘</t>
         </is>
       </c>
       <c r="C116" s="6" t="inlineStr">
@@ -6614,37 +6614,37 @@
       </c>
       <c r="D116" s="6" t="inlineStr">
         <is>
-          <t>신규상장</t>
+          <t>스팩 소멸합병</t>
         </is>
       </c>
       <c r="E116" s="6" t="inlineStr">
         <is>
-          <t>FY25</t>
+          <t>FY24</t>
         </is>
       </c>
       <c r="F116" s="7" t="inlineStr">
         <is>
-          <t>31,989</t>
+          <t>39,991</t>
         </is>
       </c>
       <c r="G116" s="7" t="inlineStr">
         <is>
-          <t>-45,307</t>
+          <t>3,541</t>
         </is>
       </c>
       <c r="H116" s="7" t="inlineStr">
         <is>
-          <t>-96,707</t>
+          <t>503</t>
         </is>
       </c>
       <c r="I116" s="6" t="inlineStr">
         <is>
-          <t>컴퓨터 프로그래밍, 시스템 통합 및 관리업</t>
+          <t>기타 기초 유기 화학물질 제조업</t>
         </is>
       </c>
       <c r="J116" s="6" t="inlineStr">
         <is>
-          <t>미래</t>
+          <t>교보</t>
         </is>
       </c>
       <c r="K116" s="6" t="inlineStr">
@@ -6656,12 +6656,12 @@
     <row r="117">
       <c r="A117" s="6" t="inlineStr">
         <is>
-          <t>2026-06-16</t>
+          <t>2026-07-23</t>
         </is>
       </c>
       <c r="B117" s="6" t="inlineStr">
         <is>
-          <t>넥스트젠바이오</t>
+          <t>모비어스</t>
         </is>
       </c>
       <c r="C117" s="6" t="inlineStr">
@@ -6676,32 +6676,32 @@
       </c>
       <c r="E117" s="6" t="inlineStr">
         <is>
-          <t>FY24</t>
+          <t>FY25</t>
         </is>
       </c>
       <c r="F117" s="7" t="inlineStr">
         <is>
-          <t>100</t>
+          <t>31,989</t>
         </is>
       </c>
       <c r="G117" s="7" t="inlineStr">
         <is>
-          <t>69</t>
+          <t>-45,307</t>
         </is>
       </c>
       <c r="H117" s="7" t="inlineStr">
         <is>
-          <t>4,792</t>
+          <t>-96,707</t>
         </is>
       </c>
       <c r="I117" s="6" t="inlineStr">
         <is>
-          <t>자연과학 및 공학 연구개발업</t>
+          <t>컴퓨터 프로그래밍, 시스템 통합 및 관리업</t>
         </is>
       </c>
       <c r="J117" s="6" t="inlineStr">
         <is>
-          <t>한국</t>
+          <t>미래</t>
         </is>
       </c>
       <c r="K117" s="6" t="inlineStr">
@@ -6713,12 +6713,12 @@
     <row r="118">
       <c r="A118" s="6" t="inlineStr">
         <is>
-          <t>2026-06-15</t>
+          <t>2026-06-16</t>
         </is>
       </c>
       <c r="B118" s="6" t="inlineStr">
         <is>
-          <t>파워큐브세미</t>
+          <t>넥스트젠바이오</t>
         </is>
       </c>
       <c r="C118" s="6" t="inlineStr">
@@ -6733,32 +6733,32 @@
       </c>
       <c r="E118" s="6" t="inlineStr">
         <is>
-          <t>FY25</t>
+          <t>FY24</t>
         </is>
       </c>
       <c r="F118" s="7" t="inlineStr">
         <is>
-          <t>10,341</t>
+          <t>100</t>
         </is>
       </c>
       <c r="G118" s="7" t="inlineStr">
         <is>
-          <t>-10,837</t>
+          <t>69</t>
         </is>
       </c>
       <c r="H118" s="7" t="inlineStr">
         <is>
-          <t>841</t>
+          <t>4,792</t>
         </is>
       </c>
       <c r="I118" s="6" t="inlineStr">
         <is>
-          <t>반도체 제조업</t>
+          <t>자연과학 및 공학 연구개발업</t>
         </is>
       </c>
       <c r="J118" s="6" t="inlineStr">
         <is>
-          <t>하나, BNK</t>
+          <t>한국</t>
         </is>
       </c>
       <c r="K118" s="6" t="inlineStr">
@@ -6770,12 +6770,12 @@
     <row r="119">
       <c r="A119" s="6" t="inlineStr">
         <is>
-          <t>2026-05-29</t>
+          <t>2026-06-15</t>
         </is>
       </c>
       <c r="B119" s="6" t="inlineStr">
         <is>
-          <t>제이피이노베이션</t>
+          <t>파워큐브세미</t>
         </is>
       </c>
       <c r="C119" s="6" t="inlineStr">
@@ -6795,27 +6795,27 @@
       </c>
       <c r="F119" s="7" t="inlineStr">
         <is>
-          <t>56,324</t>
+          <t>10,341</t>
         </is>
       </c>
       <c r="G119" s="7" t="inlineStr">
         <is>
-          <t>5,588</t>
+          <t>-10,837</t>
         </is>
       </c>
       <c r="H119" s="7" t="inlineStr">
         <is>
-          <t>3,684</t>
+          <t>841</t>
         </is>
       </c>
       <c r="I119" s="6" t="inlineStr">
         <is>
-          <t>특수 목적용 기계 제조업</t>
+          <t>반도체 제조업</t>
         </is>
       </c>
       <c r="J119" s="6" t="inlineStr">
         <is>
-          <t>삼성</t>
+          <t>하나, BNK</t>
         </is>
       </c>
       <c r="K119" s="6" t="inlineStr">
@@ -6827,12 +6827,12 @@
     <row r="120">
       <c r="A120" s="6" t="inlineStr">
         <is>
-          <t>2026-05-26</t>
+          <t>2026-05-29</t>
         </is>
       </c>
       <c r="B120" s="6" t="inlineStr">
         <is>
-          <t>케이솔루션</t>
+          <t>제이피이노베이션</t>
         </is>
       </c>
       <c r="C120" s="6" t="inlineStr">
@@ -6842,7 +6842,7 @@
       </c>
       <c r="D120" s="6" t="inlineStr">
         <is>
-          <t>스팩 존속합병</t>
+          <t>신규상장</t>
         </is>
       </c>
       <c r="E120" s="6" t="inlineStr">
@@ -6852,27 +6852,27 @@
       </c>
       <c r="F120" s="7" t="inlineStr">
         <is>
-          <t>34,565</t>
+          <t>56,324</t>
         </is>
       </c>
       <c r="G120" s="7" t="inlineStr">
         <is>
-          <t>1,158</t>
+          <t>5,588</t>
         </is>
       </c>
       <c r="H120" s="7" t="inlineStr">
         <is>
-          <t>653</t>
+          <t>3,684</t>
         </is>
       </c>
       <c r="I120" s="6" t="inlineStr">
         <is>
-          <t>차체 및 특장차 제조업</t>
+          <t>특수 목적용 기계 제조업</t>
         </is>
       </c>
       <c r="J120" s="6" t="inlineStr">
         <is>
-          <t>DB</t>
+          <t>삼성</t>
         </is>
       </c>
       <c r="K120" s="6" t="inlineStr">
@@ -6884,12 +6884,12 @@
     <row r="121">
       <c r="A121" s="6" t="inlineStr">
         <is>
-          <t>2026-04-30</t>
+          <t>2026-05-26</t>
         </is>
       </c>
       <c r="B121" s="6" t="inlineStr">
         <is>
-          <t>디토닉</t>
+          <t>케이솔루션</t>
         </is>
       </c>
       <c r="C121" s="6" t="inlineStr">
@@ -6899,37 +6899,37 @@
       </c>
       <c r="D121" s="6" t="inlineStr">
         <is>
-          <t>신규상장</t>
+          <t>스팩 존속합병</t>
         </is>
       </c>
       <c r="E121" s="6" t="inlineStr">
         <is>
-          <t>FY24</t>
+          <t>FY25</t>
         </is>
       </c>
       <c r="F121" s="7" t="inlineStr">
         <is>
-          <t>31,293</t>
+          <t>34,565</t>
         </is>
       </c>
       <c r="G121" s="7" t="inlineStr">
         <is>
-          <t>-1,633</t>
+          <t>1,158</t>
         </is>
       </c>
       <c r="H121" s="7" t="inlineStr">
         <is>
-          <t>-21,926</t>
+          <t>653</t>
         </is>
       </c>
       <c r="I121" s="6" t="inlineStr">
         <is>
-          <t>소프트웨어 개발 및 공급업</t>
+          <t>차체 및 특장차 제조업</t>
         </is>
       </c>
       <c r="J121" s="6" t="inlineStr">
         <is>
-          <t>NH</t>
+          <t>DB</t>
         </is>
       </c>
       <c r="K121" s="6" t="inlineStr">
@@ -6941,12 +6941,12 @@
     <row r="122">
       <c r="A122" s="6" t="inlineStr">
         <is>
-          <t>2026-04-22</t>
+          <t>2026-04-30</t>
         </is>
       </c>
       <c r="B122" s="6" t="inlineStr">
         <is>
-          <t>에스케이팩</t>
+          <t>디토닉</t>
         </is>
       </c>
       <c r="C122" s="6" t="inlineStr">
@@ -6956,7 +6956,7 @@
       </c>
       <c r="D122" s="6" t="inlineStr">
         <is>
-          <t>스팩 소멸합병</t>
+          <t>신규상장</t>
         </is>
       </c>
       <c r="E122" s="6" t="inlineStr">
@@ -6966,27 +6966,27 @@
       </c>
       <c r="F122" s="7" t="inlineStr">
         <is>
-          <t>27,310</t>
+          <t>31,293</t>
         </is>
       </c>
       <c r="G122" s="7" t="inlineStr">
         <is>
-          <t>2,257</t>
+          <t>-1,633</t>
         </is>
       </c>
       <c r="H122" s="7" t="inlineStr">
         <is>
-          <t>3,207</t>
+          <t>-21,926</t>
         </is>
       </c>
       <c r="I122" s="6" t="inlineStr">
         <is>
-          <t>용기 세척, 포장 및 충전기 제조업</t>
+          <t>소프트웨어 개발 및 공급업</t>
         </is>
       </c>
       <c r="J122" s="6" t="inlineStr">
         <is>
-          <t>교보</t>
+          <t>NH</t>
         </is>
       </c>
       <c r="K122" s="6" t="inlineStr">
@@ -6998,12 +6998,12 @@
     <row r="123">
       <c r="A123" s="6" t="inlineStr">
         <is>
-          <t>2026-04-20</t>
+          <t>2026-04-22</t>
         </is>
       </c>
       <c r="B123" s="6" t="inlineStr">
         <is>
-          <t>메타넷엑스</t>
+          <t>에스케이팩</t>
         </is>
       </c>
       <c r="C123" s="6" t="inlineStr">
@@ -7013,7 +7013,7 @@
       </c>
       <c r="D123" s="6" t="inlineStr">
         <is>
-          <t>신규상장</t>
+          <t>스팩 소멸합병</t>
         </is>
       </c>
       <c r="E123" s="6" t="inlineStr">
@@ -7023,27 +7023,27 @@
       </c>
       <c r="F123" s="7" t="inlineStr">
         <is>
-          <t>244,130</t>
+          <t>27,310</t>
         </is>
       </c>
       <c r="G123" s="7" t="inlineStr">
         <is>
-          <t>13,455</t>
+          <t>2,257</t>
         </is>
       </c>
       <c r="H123" s="7" t="inlineStr">
         <is>
-          <t>9,995</t>
+          <t>3,207</t>
         </is>
       </c>
       <c r="I123" s="6" t="inlineStr">
         <is>
-          <t>컴퓨터 프로그래밍, 시스템 통합 및 관리업</t>
+          <t>용기 세척, 포장 및 충전기 제조업</t>
         </is>
       </c>
       <c r="J123" s="6" t="inlineStr">
         <is>
-          <t>NH</t>
+          <t>교보</t>
         </is>
       </c>
       <c r="K123" s="6" t="inlineStr">
@@ -7055,12 +7055,12 @@
     <row r="124">
       <c r="A124" s="6" t="inlineStr">
         <is>
-          <t>2026-03-17</t>
+          <t>2026-04-20</t>
         </is>
       </c>
       <c r="B124" s="6" t="inlineStr">
         <is>
-          <t>무아스</t>
+          <t>메타넷엑스</t>
         </is>
       </c>
       <c r="C124" s="6" t="inlineStr">
@@ -7070,7 +7070,7 @@
       </c>
       <c r="D124" s="6" t="inlineStr">
         <is>
-          <t>스팩 소멸합병</t>
+          <t>신규상장</t>
         </is>
       </c>
       <c r="E124" s="6" t="inlineStr">
@@ -7080,27 +7080,27 @@
       </c>
       <c r="F124" s="7" t="inlineStr">
         <is>
-          <t>41,813</t>
+          <t>244,130</t>
         </is>
       </c>
       <c r="G124" s="7" t="inlineStr">
         <is>
-          <t>3,903</t>
+          <t>13,455</t>
         </is>
       </c>
       <c r="H124" s="7" t="inlineStr">
         <is>
-          <t>532</t>
+          <t>9,995</t>
         </is>
       </c>
       <c r="I124" s="6" t="inlineStr">
         <is>
-          <t>가정용 전기기기 제조업</t>
+          <t>컴퓨터 프로그래밍, 시스템 통합 및 관리업</t>
         </is>
       </c>
       <c r="J124" s="6" t="inlineStr">
         <is>
-          <t>신한</t>
+          <t>NH</t>
         </is>
       </c>
       <c r="K124" s="6" t="inlineStr">
@@ -7117,7 +7117,7 @@
       </c>
       <c r="B125" s="6" t="inlineStr">
         <is>
-          <t>유빅스테라퓨틱스</t>
+          <t>무아스</t>
         </is>
       </c>
       <c r="C125" s="6" t="inlineStr">
@@ -7127,7 +7127,7 @@
       </c>
       <c r="D125" s="6" t="inlineStr">
         <is>
-          <t>신규상장</t>
+          <t>스팩 소멸합병</t>
         </is>
       </c>
       <c r="E125" s="6" t="inlineStr">
@@ -7137,27 +7137,27 @@
       </c>
       <c r="F125" s="7" t="inlineStr">
         <is>
-          <t>1,071</t>
+          <t>41,813</t>
         </is>
       </c>
       <c r="G125" s="7" t="inlineStr">
         <is>
-          <t>-15,145</t>
+          <t>3,903</t>
         </is>
       </c>
       <c r="H125" s="7" t="inlineStr">
         <is>
-          <t>5,489</t>
+          <t>532</t>
         </is>
       </c>
       <c r="I125" s="6" t="inlineStr">
         <is>
-          <t>자연과학 및 공학 연구개발업</t>
+          <t>가정용 전기기기 제조업</t>
         </is>
       </c>
       <c r="J125" s="6" t="inlineStr">
         <is>
-          <t>대신</t>
+          <t>신한</t>
         </is>
       </c>
       <c r="K125" s="6" t="inlineStr">
@@ -7169,12 +7169,12 @@
     <row r="126">
       <c r="A126" s="6" t="inlineStr">
         <is>
-          <t>2026-03-16</t>
+          <t>2026-03-17</t>
         </is>
       </c>
       <c r="B126" s="6" t="inlineStr">
         <is>
-          <t>코드잇</t>
+          <t>유빅스테라퓨틱스</t>
         </is>
       </c>
       <c r="C126" s="6" t="inlineStr">
@@ -7194,27 +7194,27 @@
       </c>
       <c r="F126" s="7" t="inlineStr">
         <is>
-          <t>30,747</t>
+          <t>1,071</t>
         </is>
       </c>
       <c r="G126" s="7" t="inlineStr">
         <is>
-          <t>6,652</t>
+          <t>-15,145</t>
         </is>
       </c>
       <c r="H126" s="7" t="inlineStr">
         <is>
-          <t>2,403</t>
+          <t>5,489</t>
         </is>
       </c>
       <c r="I126" s="6" t="inlineStr">
         <is>
-          <t>교육지원 서비스업</t>
+          <t>자연과학 및 공학 연구개발업</t>
         </is>
       </c>
       <c r="J126" s="6" t="inlineStr">
         <is>
-          <t>미래</t>
+          <t>대신</t>
         </is>
       </c>
       <c r="K126" s="6" t="inlineStr">
@@ -7226,12 +7226,12 @@
     <row r="127">
       <c r="A127" s="6" t="inlineStr">
         <is>
-          <t>2026-02-05</t>
+          <t>2026-03-16</t>
         </is>
       </c>
       <c r="B127" s="6" t="inlineStr">
         <is>
-          <t>한컴인스페이스</t>
+          <t>코드잇</t>
         </is>
       </c>
       <c r="C127" s="6" t="inlineStr">
@@ -7251,44 +7251,44 @@
       </c>
       <c r="F127" s="7" t="inlineStr">
         <is>
-          <t>23,492</t>
+          <t>30,747</t>
         </is>
       </c>
       <c r="G127" s="7" t="inlineStr">
         <is>
-          <t>-3,104</t>
+          <t>6,652</t>
         </is>
       </c>
       <c r="H127" s="7" t="inlineStr">
         <is>
-          <t>5,815</t>
+          <t>2,403</t>
         </is>
       </c>
       <c r="I127" s="6" t="inlineStr">
         <is>
-          <t>소프트웨어 개발 및 공급업</t>
+          <t>교육지원 서비스업</t>
         </is>
       </c>
       <c r="J127" s="6" t="inlineStr">
         <is>
-          <t>대신</t>
+          <t>미래</t>
         </is>
       </c>
       <c r="K127" s="6" t="inlineStr">
         <is>
-          <t>심사 미승인</t>
+          <t>심사 철회</t>
         </is>
       </c>
     </row>
     <row r="128">
       <c r="A128" s="6" t="inlineStr">
         <is>
-          <t>2026-01-28</t>
+          <t>2026-02-05</t>
         </is>
       </c>
       <c r="B128" s="6" t="inlineStr">
         <is>
-          <t>크몽</t>
+          <t>한컴인스페이스</t>
         </is>
       </c>
       <c r="C128" s="6" t="inlineStr">
@@ -7308,44 +7308,44 @@
       </c>
       <c r="F128" s="7" t="inlineStr">
         <is>
-          <t>48,572</t>
+          <t>23,492</t>
         </is>
       </c>
       <c r="G128" s="7" t="inlineStr">
         <is>
-          <t>3,988</t>
+          <t>-3,104</t>
         </is>
       </c>
       <c r="H128" s="7" t="inlineStr">
         <is>
-          <t>4,930</t>
+          <t>5,815</t>
         </is>
       </c>
       <c r="I128" s="6" t="inlineStr">
         <is>
-          <t>기타 정보 서비스업</t>
+          <t>소프트웨어 개발 및 공급업</t>
         </is>
       </c>
       <c r="J128" s="6" t="inlineStr">
         <is>
-          <t>삼성</t>
+          <t>대신</t>
         </is>
       </c>
       <c r="K128" s="6" t="inlineStr">
         <is>
-          <t>심사 철회</t>
+          <t>심사 미승인</t>
         </is>
       </c>
     </row>
     <row r="129">
       <c r="A129" s="6" t="inlineStr">
         <is>
-          <t>2026-01-27</t>
+          <t>2026-01-28</t>
         </is>
       </c>
       <c r="B129" s="6" t="inlineStr">
         <is>
-          <t>한화플러스제6호스팩</t>
+          <t>크몽</t>
         </is>
       </c>
       <c r="C129" s="6" t="inlineStr">
@@ -7365,27 +7365,27 @@
       </c>
       <c r="F129" s="7" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>48,572</t>
         </is>
       </c>
       <c r="G129" s="7" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>3,988</t>
         </is>
       </c>
       <c r="H129" s="7" t="inlineStr">
         <is>
-          <t>41</t>
+          <t>4,930</t>
         </is>
       </c>
       <c r="I129" s="6" t="inlineStr">
         <is>
-          <t>기타 금융업</t>
+          <t>기타 정보 서비스업</t>
         </is>
       </c>
       <c r="J129" s="6" t="inlineStr">
         <is>
-          <t>한화</t>
+          <t>삼성</t>
         </is>
       </c>
       <c r="K129" s="6" t="inlineStr">
@@ -7397,17 +7397,17 @@
     <row r="130">
       <c r="A130" s="6" t="inlineStr">
         <is>
-          <t>2026-01-26</t>
+          <t>2026-01-27</t>
         </is>
       </c>
       <c r="B130" s="6" t="inlineStr">
         <is>
-          <t>에식스솔루션즈</t>
+          <t>한화플러스제6호스팩</t>
         </is>
       </c>
       <c r="C130" s="6" t="inlineStr">
         <is>
-          <t>유가</t>
+          <t>코스닥</t>
         </is>
       </c>
       <c r="D130" s="6" t="inlineStr">
@@ -7422,27 +7422,27 @@
       </c>
       <c r="F130" s="7" t="inlineStr">
         <is>
-          <t>2,461</t>
+          <t>-</t>
         </is>
       </c>
       <c r="G130" s="7" t="inlineStr">
         <is>
-          <t>46</t>
+          <t>-</t>
         </is>
       </c>
       <c r="H130" s="7" t="inlineStr">
         <is>
-          <t>200</t>
+          <t>41</t>
         </is>
       </c>
       <c r="I130" s="6" t="inlineStr">
         <is>
-          <t>절연선 및 케이블 제조업</t>
+          <t>기타 금융업</t>
         </is>
       </c>
       <c r="J130" s="6" t="inlineStr">
         <is>
-          <t>한국, 미래</t>
+          <t>한화</t>
         </is>
       </c>
       <c r="K130" s="6" t="inlineStr">
@@ -7454,55 +7454,112 @@
     <row r="131">
       <c r="A131" s="6" t="inlineStr">
         <is>
+          <t>2026-01-26</t>
+        </is>
+      </c>
+      <c r="B131" s="6" t="inlineStr">
+        <is>
+          <t>에식스솔루션즈</t>
+        </is>
+      </c>
+      <c r="C131" s="6" t="inlineStr">
+        <is>
+          <t>유가</t>
+        </is>
+      </c>
+      <c r="D131" s="6" t="inlineStr">
+        <is>
+          <t>신규상장</t>
+        </is>
+      </c>
+      <c r="E131" s="6" t="inlineStr">
+        <is>
+          <t>FY24</t>
+        </is>
+      </c>
+      <c r="F131" s="7" t="inlineStr">
+        <is>
+          <t>2,461</t>
+        </is>
+      </c>
+      <c r="G131" s="7" t="inlineStr">
+        <is>
+          <t>46</t>
+        </is>
+      </c>
+      <c r="H131" s="7" t="inlineStr">
+        <is>
+          <t>200</t>
+        </is>
+      </c>
+      <c r="I131" s="6" t="inlineStr">
+        <is>
+          <t>절연선 및 케이블 제조업</t>
+        </is>
+      </c>
+      <c r="J131" s="6" t="inlineStr">
+        <is>
+          <t>한국, 미래</t>
+        </is>
+      </c>
+      <c r="K131" s="6" t="inlineStr">
+        <is>
+          <t>심사 철회</t>
+        </is>
+      </c>
+    </row>
+    <row r="132">
+      <c r="A132" s="6" t="inlineStr">
+        <is>
           <t>2026-01-23</t>
         </is>
       </c>
-      <c r="B131" s="6" t="inlineStr">
+      <c r="B132" s="6" t="inlineStr">
         <is>
           <t>에코크레이션</t>
         </is>
       </c>
-      <c r="C131" s="6" t="inlineStr">
+      <c r="C132" s="6" t="inlineStr">
         <is>
           <t>코스닥</t>
         </is>
       </c>
-      <c r="D131" s="6" t="inlineStr">
+      <c r="D132" s="6" t="inlineStr">
         <is>
           <t>신규상장</t>
         </is>
       </c>
-      <c r="E131" s="6" t="inlineStr">
+      <c r="E132" s="6" t="inlineStr">
         <is>
           <t>FY24</t>
         </is>
       </c>
-      <c r="F131" s="7" t="inlineStr">
+      <c r="F132" s="7" t="inlineStr">
         <is>
           <t>18,544</t>
         </is>
       </c>
-      <c r="G131" s="7" t="inlineStr">
+      <c r="G132" s="7" t="inlineStr">
         <is>
           <t>-15,634</t>
         </is>
       </c>
-      <c r="H131" s="7" t="inlineStr">
+      <c r="H132" s="7" t="inlineStr">
         <is>
           <t>4,550</t>
         </is>
       </c>
-      <c r="I131" s="6" t="inlineStr">
+      <c r="I132" s="6" t="inlineStr">
         <is>
           <t>일반 목적용 기계 제조업</t>
         </is>
       </c>
-      <c r="J131" s="6" t="inlineStr">
+      <c r="J132" s="6" t="inlineStr">
         <is>
           <t>키움</t>
         </is>
       </c>
-      <c r="K131" s="6" t="inlineStr">
+      <c r="K132" s="6" t="inlineStr">
         <is>
           <t>심사 철회</t>
         </is>
@@ -7519,7 +7576,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R74"/>
+  <dimension ref="A1:R75"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="1"/>
@@ -10797,7 +10854,7 @@
     <row r="46" ht="22" customHeight="1">
       <c r="A46" s="3" t="inlineStr">
         <is>
-          <t>■ 공모 진행 (예심 승인법인)  (24건)</t>
+          <t>■ 공모 진행 (예심 승인법인)  (25건)</t>
         </is>
       </c>
       <c r="B46" s="4" t="n"/>
@@ -12382,22 +12439,86 @@
         </is>
       </c>
     </row>
-    <row r="72">
-      <c r="A72" s="20" t="inlineStr">
-        <is>
-          <t>※ 상장 완료 = KIND 신규상장 페이지 기준(스팩합병 포함) · 스팩 공모상장은 밴드·밸류에이션 등 해당없음(공모가 2,000원 고정).</t>
+    <row r="71" ht="30" customHeight="1">
+      <c r="A71" s="6" t="inlineStr">
+        <is>
+          <t>하나에어로다이내믹스</t>
+        </is>
+      </c>
+      <c r="B71" s="18" t="inlineStr">
+        <is>
+          <t>수집예정</t>
+        </is>
+      </c>
+      <c r="C71" s="18" t="inlineStr">
+        <is>
+          <t>수집예정</t>
+        </is>
+      </c>
+      <c r="D71" s="18" t="inlineStr">
+        <is>
+          <t>수집예정</t>
+        </is>
+      </c>
+      <c r="E71" s="18" t="inlineStr">
+        <is>
+          <t>수집예정</t>
+        </is>
+      </c>
+      <c r="F71" s="18" t="inlineStr">
+        <is>
+          <t>수집예정</t>
+        </is>
+      </c>
+      <c r="G71" s="6" t="inlineStr"/>
+      <c r="H71" s="6" t="inlineStr"/>
+      <c r="I71" s="6" t="inlineStr"/>
+      <c r="J71" s="18" t="inlineStr">
+        <is>
+          <t>수집예정</t>
+        </is>
+      </c>
+      <c r="K71" s="6" t="inlineStr"/>
+      <c r="L71" s="6" t="inlineStr"/>
+      <c r="M71" s="6" t="inlineStr"/>
+      <c r="N71" s="18" t="inlineStr">
+        <is>
+          <t>수집예정</t>
+        </is>
+      </c>
+      <c r="O71" s="6" t="inlineStr"/>
+      <c r="P71" s="18" t="inlineStr">
+        <is>
+          <t>수집예정</t>
+        </is>
+      </c>
+      <c r="Q71" s="18" t="inlineStr">
+        <is>
+          <t>수집예정</t>
+        </is>
+      </c>
+      <c r="R71" s="6" t="inlineStr">
+        <is>
+          <t>신고서 대기</t>
         </is>
       </c>
     </row>
     <row r="73">
       <c r="A73" s="20" t="inlineStr">
         <is>
-          <t>※ 기재정정 신고서 내 정정 전·후 병존 → 자동수집은 "정정 후" 값만 취함.</t>
+          <t>※ 상장 완료 = KIND 신규상장 페이지 기준(스팩합병 포함) · 스팩 공모상장은 밴드·밸류에이션 등 해당없음(공모가 2,000원 고정).</t>
         </is>
       </c>
     </row>
     <row r="74">
       <c r="A74" s="20" t="inlineStr">
+        <is>
+          <t>※ 기재정정 신고서 내 정정 전·후 병존 → 자동수집은 "정정 후" 값만 취함.</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" s="20" t="inlineStr">
         <is>
           <t>※ 청약경쟁률=일반투자자 청약수량÷최종배정수량 · "MM-DD~"는 종료일 자동수집 예정.</t>
         </is>
@@ -12585,7 +12706,7 @@
         <v>15</v>
       </c>
       <c r="C10" s="6" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D10" s="6" t="n">
         <v>2</v>
@@ -12654,7 +12775,7 @@
         <v>10</v>
       </c>
       <c r="C13" s="6" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="D13" s="6" t="n">
         <v>1</v>

</xml_diff>

<commit_message>
chore: update IPO data 2026-09-03
</commit_message>
<xml_diff>
--- a/IPO_analysis.xlsx
+++ b/IPO_analysis.xlsx
@@ -618,14 +618,14 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>기준일 2026-09-02 · 청구일 직전 사업연도 · 별도/개별 재무제표 · 단위 백만원(별도 표기 시 USD)</t>
+          <t>기준일 2026-09-03 · 청구일 직전 사업연도 · 별도/개별 재무제표 · 단위 백만원(별도 표기 시 USD)</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
-          <t>■ 심사 신청(진행중)  (48건)</t>
+          <t>■ 심사 신청(진행중)  (46건)</t>
         </is>
       </c>
       <c r="B4" s="4" t="n"/>
@@ -3045,12 +3045,12 @@
     <row r="48">
       <c r="A48" s="6" t="inlineStr">
         <is>
-          <t>2026-05-21</t>
+          <t>2026-05-12</t>
         </is>
       </c>
       <c r="B48" s="6" t="inlineStr">
         <is>
-          <t>에이엔에이치스트럭쳐</t>
+          <t>오토핸즈</t>
         </is>
       </c>
       <c r="C48" s="6" t="inlineStr">
@@ -3060,7 +3060,7 @@
       </c>
       <c r="D48" s="6" t="inlineStr">
         <is>
-          <t>신규상장</t>
+          <t>스팩 소멸합병</t>
         </is>
       </c>
       <c r="E48" s="6" t="inlineStr">
@@ -3070,27 +3070,27 @@
       </c>
       <c r="F48" s="7" t="inlineStr">
         <is>
-          <t>19,784</t>
+          <t>238,564</t>
         </is>
       </c>
       <c r="G48" s="7" t="inlineStr">
         <is>
-          <t>-4,296</t>
+          <t>6,047</t>
         </is>
       </c>
       <c r="H48" s="7" t="inlineStr">
         <is>
-          <t>24,561</t>
+          <t>6,129</t>
         </is>
       </c>
       <c r="I48" s="6" t="inlineStr">
         <is>
-          <t>건축기술, 엔지니어링 및 관련 기술 서비스업</t>
+          <t>자동차 판매업</t>
         </is>
       </c>
       <c r="J48" s="6" t="inlineStr">
         <is>
-          <t>NH</t>
+          <t>미래</t>
         </is>
       </c>
       <c r="K48" s="6" t="inlineStr">
@@ -3102,12 +3102,12 @@
     <row r="49">
       <c r="A49" s="6" t="inlineStr">
         <is>
-          <t>2026-05-12</t>
+          <t>2026-05-06</t>
         </is>
       </c>
       <c r="B49" s="6" t="inlineStr">
         <is>
-          <t>오토핸즈</t>
+          <t>아이벡스메디칼시스템즈</t>
         </is>
       </c>
       <c r="C49" s="6" t="inlineStr">
@@ -3117,7 +3117,7 @@
       </c>
       <c r="D49" s="6" t="inlineStr">
         <is>
-          <t>스팩 소멸합병</t>
+          <t>신규상장</t>
         </is>
       </c>
       <c r="E49" s="6" t="inlineStr">
@@ -3127,27 +3127,27 @@
       </c>
       <c r="F49" s="7" t="inlineStr">
         <is>
-          <t>238,564</t>
+          <t>15,282</t>
         </is>
       </c>
       <c r="G49" s="7" t="inlineStr">
         <is>
-          <t>6,047</t>
+          <t>-7,227</t>
         </is>
       </c>
       <c r="H49" s="7" t="inlineStr">
         <is>
-          <t>6,129</t>
+          <t>744</t>
         </is>
       </c>
       <c r="I49" s="6" t="inlineStr">
         <is>
-          <t>자동차 판매업</t>
+          <t>의료용 기기 제조업</t>
         </is>
       </c>
       <c r="J49" s="6" t="inlineStr">
         <is>
-          <t>미래</t>
+          <t>NH</t>
         </is>
       </c>
       <c r="K49" s="6" t="inlineStr">
@@ -3159,12 +3159,12 @@
     <row r="50">
       <c r="A50" s="6" t="inlineStr">
         <is>
-          <t>2026-05-06</t>
+          <t>2026-04-08</t>
         </is>
       </c>
       <c r="B50" s="6" t="inlineStr">
         <is>
-          <t>아이벡스메디칼시스템즈</t>
+          <t>옵토닉스</t>
         </is>
       </c>
       <c r="C50" s="6" t="inlineStr">
@@ -3184,27 +3184,27 @@
       </c>
       <c r="F50" s="7" t="inlineStr">
         <is>
-          <t>15,282</t>
+          <t>25,368</t>
         </is>
       </c>
       <c r="G50" s="7" t="inlineStr">
         <is>
-          <t>-7,227</t>
+          <t>1,901</t>
         </is>
       </c>
       <c r="H50" s="7" t="inlineStr">
         <is>
-          <t>744</t>
+          <t>730</t>
         </is>
       </c>
       <c r="I50" s="6" t="inlineStr">
         <is>
-          <t>의료용 기기 제조업</t>
+          <t>광학렌즈 및 광학요소 제조업</t>
         </is>
       </c>
       <c r="J50" s="6" t="inlineStr">
         <is>
-          <t>NH</t>
+          <t>한국</t>
         </is>
       </c>
       <c r="K50" s="6" t="inlineStr">
@@ -3216,12 +3216,12 @@
     <row r="51">
       <c r="A51" s="6" t="inlineStr">
         <is>
-          <t>2026-04-08</t>
+          <t>2026-02-27</t>
         </is>
       </c>
       <c r="B51" s="6" t="inlineStr">
         <is>
-          <t>옵토닉스</t>
+          <t>피지티</t>
         </is>
       </c>
       <c r="C51" s="6" t="inlineStr">
@@ -3241,22 +3241,22 @@
       </c>
       <c r="F51" s="7" t="inlineStr">
         <is>
-          <t>25,368</t>
+          <t>40,141</t>
         </is>
       </c>
       <c r="G51" s="7" t="inlineStr">
         <is>
-          <t>1,901</t>
+          <t>-69,722</t>
         </is>
       </c>
       <c r="H51" s="7" t="inlineStr">
         <is>
-          <t>730</t>
+          <t>6,029</t>
         </is>
       </c>
       <c r="I51" s="6" t="inlineStr">
         <is>
-          <t>광학렌즈 및 광학요소 제조업</t>
+          <t>기타 화학제품 제조업</t>
         </is>
       </c>
       <c r="J51" s="6" t="inlineStr">
@@ -3270,191 +3270,191 @@
         </is>
       </c>
     </row>
-    <row r="52">
-      <c r="A52" s="6" t="inlineStr">
-        <is>
-          <t>2026-03-24</t>
-        </is>
-      </c>
-      <c r="B52" s="6" t="inlineStr">
+    <row r="53">
+      <c r="A53" s="3" t="inlineStr">
+        <is>
+          <t>■ 심사 승인  (57건)</t>
+        </is>
+      </c>
+      <c r="B53" s="4" t="n"/>
+      <c r="C53" s="4" t="n"/>
+      <c r="D53" s="4" t="n"/>
+      <c r="E53" s="4" t="n"/>
+      <c r="F53" s="4" t="n"/>
+      <c r="G53" s="4" t="n"/>
+      <c r="H53" s="4" t="n"/>
+      <c r="I53" s="4" t="n"/>
+      <c r="J53" s="4" t="n"/>
+      <c r="K53" s="4" t="n"/>
+    </row>
+    <row r="54">
+      <c r="A54" s="5" t="inlineStr">
+        <is>
+          <t>일자</t>
+        </is>
+      </c>
+      <c r="B54" s="5" t="inlineStr">
+        <is>
+          <t>회사명</t>
+        </is>
+      </c>
+      <c r="C54" s="5" t="inlineStr">
+        <is>
+          <t>시장</t>
+        </is>
+      </c>
+      <c r="D54" s="5" t="inlineStr">
+        <is>
+          <t>상장유형</t>
+        </is>
+      </c>
+      <c r="E54" s="5" t="inlineStr">
+        <is>
+          <t>기준연도</t>
+        </is>
+      </c>
+      <c r="F54" s="5" t="inlineStr">
+        <is>
+          <t>매출액</t>
+        </is>
+      </c>
+      <c r="G54" s="5" t="inlineStr">
+        <is>
+          <t>순이익</t>
+        </is>
+      </c>
+      <c r="H54" s="5" t="inlineStr">
+        <is>
+          <t>자기자본</t>
+        </is>
+      </c>
+      <c r="I54" s="5" t="inlineStr">
+        <is>
+          <t>업종</t>
+        </is>
+      </c>
+      <c r="J54" s="5" t="inlineStr">
+        <is>
+          <t>대표주관사</t>
+        </is>
+      </c>
+      <c r="K54" s="5" t="inlineStr">
+        <is>
+          <t>현황</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="6" t="inlineStr">
+        <is>
+          <t>2026-09-03</t>
+        </is>
+      </c>
+      <c r="B55" s="6" t="inlineStr">
+        <is>
+          <t>에이엔에이치스트럭쳐</t>
+        </is>
+      </c>
+      <c r="C55" s="6" t="inlineStr">
+        <is>
+          <t>코스닥</t>
+        </is>
+      </c>
+      <c r="D55" s="6" t="inlineStr">
+        <is>
+          <t>신규상장</t>
+        </is>
+      </c>
+      <c r="E55" s="6" t="inlineStr">
+        <is>
+          <t>FY25</t>
+        </is>
+      </c>
+      <c r="F55" s="7" t="inlineStr">
+        <is>
+          <t>19,784</t>
+        </is>
+      </c>
+      <c r="G55" s="7" t="inlineStr">
+        <is>
+          <t>-4,296</t>
+        </is>
+      </c>
+      <c r="H55" s="7" t="inlineStr">
+        <is>
+          <t>24,561</t>
+        </is>
+      </c>
+      <c r="I55" s="6" t="inlineStr">
+        <is>
+          <t>건축기술, 엔지니어링 및 관련 기술 서비스업</t>
+        </is>
+      </c>
+      <c r="J55" s="6" t="inlineStr">
+        <is>
+          <t>NH</t>
+        </is>
+      </c>
+      <c r="K55" s="6" t="inlineStr">
+        <is>
+          <t>상장전</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="6" t="inlineStr">
+        <is>
+          <t>2026-09-03</t>
+        </is>
+      </c>
+      <c r="B56" s="6" t="inlineStr">
         <is>
           <t>인텔리빅스</t>
         </is>
       </c>
-      <c r="C52" s="6" t="inlineStr">
+      <c r="C56" s="6" t="inlineStr">
         <is>
           <t>코스닥</t>
         </is>
       </c>
-      <c r="D52" s="6" t="inlineStr">
+      <c r="D56" s="6" t="inlineStr">
         <is>
           <t>신규상장</t>
         </is>
       </c>
-      <c r="E52" s="6" t="inlineStr">
+      <c r="E56" s="6" t="inlineStr">
         <is>
           <t>FY25</t>
         </is>
       </c>
-      <c r="F52" s="7" t="inlineStr">
+      <c r="F56" s="7" t="inlineStr">
         <is>
           <t>46,644</t>
         </is>
       </c>
-      <c r="G52" s="7" t="inlineStr">
+      <c r="G56" s="7" t="inlineStr">
         <is>
           <t>5,357</t>
         </is>
       </c>
-      <c r="H52" s="7" t="inlineStr">
+      <c r="H56" s="7" t="inlineStr">
         <is>
           <t>1,048</t>
         </is>
       </c>
-      <c r="I52" s="6" t="inlineStr">
+      <c r="I56" s="6" t="inlineStr">
         <is>
           <t>소프트웨어 개발 및 공급업</t>
         </is>
       </c>
-      <c r="J52" s="6" t="inlineStr">
+      <c r="J56" s="6" t="inlineStr">
         <is>
           <t>미래</t>
         </is>
       </c>
-      <c r="K52" s="6" t="inlineStr">
-        <is>
-          <t>예심 진행중</t>
-        </is>
-      </c>
-    </row>
-    <row r="53">
-      <c r="A53" s="6" t="inlineStr">
-        <is>
-          <t>2026-02-27</t>
-        </is>
-      </c>
-      <c r="B53" s="6" t="inlineStr">
-        <is>
-          <t>피지티</t>
-        </is>
-      </c>
-      <c r="C53" s="6" t="inlineStr">
-        <is>
-          <t>코스닥</t>
-        </is>
-      </c>
-      <c r="D53" s="6" t="inlineStr">
-        <is>
-          <t>신규상장</t>
-        </is>
-      </c>
-      <c r="E53" s="6" t="inlineStr">
-        <is>
-          <t>FY25</t>
-        </is>
-      </c>
-      <c r="F53" s="7" t="inlineStr">
-        <is>
-          <t>40,141</t>
-        </is>
-      </c>
-      <c r="G53" s="7" t="inlineStr">
-        <is>
-          <t>-69,722</t>
-        </is>
-      </c>
-      <c r="H53" s="7" t="inlineStr">
-        <is>
-          <t>6,029</t>
-        </is>
-      </c>
-      <c r="I53" s="6" t="inlineStr">
-        <is>
-          <t>기타 화학제품 제조업</t>
-        </is>
-      </c>
-      <c r="J53" s="6" t="inlineStr">
-        <is>
-          <t>한국</t>
-        </is>
-      </c>
-      <c r="K53" s="6" t="inlineStr">
-        <is>
-          <t>예심 진행중</t>
-        </is>
-      </c>
-    </row>
-    <row r="55">
-      <c r="A55" s="3" t="inlineStr">
-        <is>
-          <t>■ 심사 승인  (55건)</t>
-        </is>
-      </c>
-      <c r="B55" s="4" t="n"/>
-      <c r="C55" s="4" t="n"/>
-      <c r="D55" s="4" t="n"/>
-      <c r="E55" s="4" t="n"/>
-      <c r="F55" s="4" t="n"/>
-      <c r="G55" s="4" t="n"/>
-      <c r="H55" s="4" t="n"/>
-      <c r="I55" s="4" t="n"/>
-      <c r="J55" s="4" t="n"/>
-      <c r="K55" s="4" t="n"/>
-    </row>
-    <row r="56">
-      <c r="A56" s="5" t="inlineStr">
-        <is>
-          <t>일자</t>
-        </is>
-      </c>
-      <c r="B56" s="5" t="inlineStr">
-        <is>
-          <t>회사명</t>
-        </is>
-      </c>
-      <c r="C56" s="5" t="inlineStr">
-        <is>
-          <t>시장</t>
-        </is>
-      </c>
-      <c r="D56" s="5" t="inlineStr">
-        <is>
-          <t>상장유형</t>
-        </is>
-      </c>
-      <c r="E56" s="5" t="inlineStr">
-        <is>
-          <t>기준연도</t>
-        </is>
-      </c>
-      <c r="F56" s="5" t="inlineStr">
-        <is>
-          <t>매출액</t>
-        </is>
-      </c>
-      <c r="G56" s="5" t="inlineStr">
-        <is>
-          <t>순이익</t>
-        </is>
-      </c>
-      <c r="H56" s="5" t="inlineStr">
-        <is>
-          <t>자기자본</t>
-        </is>
-      </c>
-      <c r="I56" s="5" t="inlineStr">
-        <is>
-          <t>업종</t>
-        </is>
-      </c>
-      <c r="J56" s="5" t="inlineStr">
-        <is>
-          <t>대표주관사</t>
-        </is>
-      </c>
-      <c r="K56" s="5" t="inlineStr">
-        <is>
-          <t>현황</t>
+      <c r="K56" s="6" t="inlineStr">
+        <is>
+          <t>상장전</t>
         </is>
       </c>
     </row>
@@ -7576,7 +7576,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R75"/>
+  <dimension ref="A1:R77"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="1"/>
@@ -10854,7 +10854,7 @@
     <row r="46" ht="22" customHeight="1">
       <c r="A46" s="3" t="inlineStr">
         <is>
-          <t>■ 공모 진행 (예심 승인법인)  (25건)</t>
+          <t>■ 공모 진행 (예심 승인법인)  (27건)</t>
         </is>
       </c>
       <c r="B46" s="4" t="n"/>
@@ -11243,7 +11243,7 @@
       </c>
       <c r="F52" s="6" t="inlineStr">
         <is>
-          <t>21.59배 (PER)</t>
+          <t>20.04배 (PER)</t>
         </is>
       </c>
       <c r="G52" s="6" t="inlineStr"/>
@@ -11866,32 +11866,32 @@
     <row r="62" ht="30" customHeight="1">
       <c r="A62" s="6" t="inlineStr">
         <is>
-          <t>에스케이증권제14호기업인수목적</t>
+          <t>티앤이코리아</t>
         </is>
       </c>
       <c r="B62" s="6" t="inlineStr">
         <is>
-          <t>10-12~10-13</t>
-        </is>
-      </c>
-      <c r="C62" s="18" t="inlineStr">
-        <is>
-          <t>수집예정</t>
+          <t>10-07~10-14</t>
+        </is>
+      </c>
+      <c r="C62" s="6" t="inlineStr">
+        <is>
+          <t>12,600~15,300</t>
         </is>
       </c>
       <c r="D62" s="7" t="inlineStr">
         <is>
-          <t>6,500,000</t>
+          <t>2,400,000</t>
         </is>
       </c>
       <c r="E62" s="7" t="inlineStr">
         <is>
-          <t>13,000,000,000</t>
-        </is>
-      </c>
-      <c r="F62" s="18" t="inlineStr">
-        <is>
-          <t>수집예정</t>
+          <t>30,240,000,000</t>
+        </is>
+      </c>
+      <c r="F62" s="6" t="inlineStr">
+        <is>
+          <t>19.48배 (PER)</t>
         </is>
       </c>
       <c r="G62" s="6" t="inlineStr"/>
@@ -11899,26 +11899,26 @@
       <c r="I62" s="6" t="inlineStr"/>
       <c r="J62" s="6" t="inlineStr">
         <is>
-          <t>10-15~10-16</t>
+          <t>10-20~10-21</t>
         </is>
       </c>
       <c r="K62" s="6" t="inlineStr"/>
       <c r="L62" s="6" t="inlineStr"/>
       <c r="M62" s="6" t="inlineStr"/>
-      <c r="N62" s="18" t="inlineStr">
-        <is>
-          <t>수집예정</t>
+      <c r="N62" s="6" t="inlineStr">
+        <is>
+          <t>신한투자증권</t>
         </is>
       </c>
       <c r="O62" s="6" t="inlineStr"/>
-      <c r="P62" s="18" t="inlineStr">
-        <is>
-          <t>수집예정</t>
+      <c r="P62" s="7" t="inlineStr">
+        <is>
+          <t>1,245,888,000</t>
         </is>
       </c>
       <c r="Q62" s="6" t="inlineStr">
         <is>
-          <t>50%</t>
+          <t>4.0%</t>
         </is>
       </c>
       <c r="R62" s="6" t="inlineStr">
@@ -11930,12 +11930,12 @@
     <row r="63" ht="30" customHeight="1">
       <c r="A63" s="6" t="inlineStr">
         <is>
-          <t>엠에스바이오</t>
-        </is>
-      </c>
-      <c r="B63" s="18" t="inlineStr">
-        <is>
-          <t>수집예정</t>
+          <t>에스케이증권제14호기업인수목적</t>
+        </is>
+      </c>
+      <c r="B63" s="6" t="inlineStr">
+        <is>
+          <t>10-12~10-13</t>
         </is>
       </c>
       <c r="C63" s="18" t="inlineStr">
@@ -11943,14 +11943,14 @@
           <t>수집예정</t>
         </is>
       </c>
-      <c r="D63" s="18" t="inlineStr">
-        <is>
-          <t>수집예정</t>
-        </is>
-      </c>
-      <c r="E63" s="18" t="inlineStr">
-        <is>
-          <t>수집예정</t>
+      <c r="D63" s="7" t="inlineStr">
+        <is>
+          <t>6,500,000</t>
+        </is>
+      </c>
+      <c r="E63" s="7" t="inlineStr">
+        <is>
+          <t>13,000,000,000</t>
         </is>
       </c>
       <c r="F63" s="18" t="inlineStr">
@@ -11961,9 +11961,9 @@
       <c r="G63" s="6" t="inlineStr"/>
       <c r="H63" s="6" t="inlineStr"/>
       <c r="I63" s="6" t="inlineStr"/>
-      <c r="J63" s="18" t="inlineStr">
-        <is>
-          <t>수집예정</t>
+      <c r="J63" s="6" t="inlineStr">
+        <is>
+          <t>10-15~10-16</t>
         </is>
       </c>
       <c r="K63" s="6" t="inlineStr"/>
@@ -11980,21 +11980,21 @@
           <t>수집예정</t>
         </is>
       </c>
-      <c r="Q63" s="18" t="inlineStr">
-        <is>
-          <t>수집예정</t>
+      <c r="Q63" s="6" t="inlineStr">
+        <is>
+          <t>50%</t>
         </is>
       </c>
       <c r="R63" s="6" t="inlineStr">
         <is>
-          <t>신고서 대기</t>
+          <t>최초</t>
         </is>
       </c>
     </row>
     <row r="64" ht="30" customHeight="1">
       <c r="A64" s="6" t="inlineStr">
         <is>
-          <t>디티에스</t>
+          <t>엠에스바이오</t>
         </is>
       </c>
       <c r="B64" s="18" t="inlineStr">
@@ -12058,7 +12058,7 @@
     <row r="65" ht="30" customHeight="1">
       <c r="A65" s="6" t="inlineStr">
         <is>
-          <t>한화플러스제6호스팩</t>
+          <t>디티에스</t>
         </is>
       </c>
       <c r="B65" s="18" t="inlineStr">
@@ -12122,7 +12122,7 @@
     <row r="66" ht="30" customHeight="1">
       <c r="A66" s="6" t="inlineStr">
         <is>
-          <t>바로팜</t>
+          <t>한화플러스제6호스팩</t>
         </is>
       </c>
       <c r="B66" s="18" t="inlineStr">
@@ -12186,7 +12186,7 @@
     <row r="67" ht="30" customHeight="1">
       <c r="A67" s="6" t="inlineStr">
         <is>
-          <t>크리에이츠</t>
+          <t>바로팜</t>
         </is>
       </c>
       <c r="B67" s="18" t="inlineStr">
@@ -12250,7 +12250,7 @@
     <row r="68" ht="30" customHeight="1">
       <c r="A68" s="6" t="inlineStr">
         <is>
-          <t>티앤이코리아</t>
+          <t>크리에이츠</t>
         </is>
       </c>
       <c r="B68" s="18" t="inlineStr">
@@ -12503,22 +12503,150 @@
         </is>
       </c>
     </row>
-    <row r="73">
-      <c r="A73" s="20" t="inlineStr">
-        <is>
-          <t>※ 상장 완료 = KIND 신규상장 페이지 기준(스팩합병 포함) · 스팩 공모상장은 밴드·밸류에이션 등 해당없음(공모가 2,000원 고정).</t>
-        </is>
-      </c>
-    </row>
-    <row r="74">
-      <c r="A74" s="20" t="inlineStr">
-        <is>
-          <t>※ 기재정정 신고서 내 정정 전·후 병존 → 자동수집은 "정정 후" 값만 취함.</t>
+    <row r="72" ht="30" customHeight="1">
+      <c r="A72" s="6" t="inlineStr">
+        <is>
+          <t>에이엔에이치스트럭쳐</t>
+        </is>
+      </c>
+      <c r="B72" s="18" t="inlineStr">
+        <is>
+          <t>수집예정</t>
+        </is>
+      </c>
+      <c r="C72" s="18" t="inlineStr">
+        <is>
+          <t>수집예정</t>
+        </is>
+      </c>
+      <c r="D72" s="18" t="inlineStr">
+        <is>
+          <t>수집예정</t>
+        </is>
+      </c>
+      <c r="E72" s="18" t="inlineStr">
+        <is>
+          <t>수집예정</t>
+        </is>
+      </c>
+      <c r="F72" s="18" t="inlineStr">
+        <is>
+          <t>수집예정</t>
+        </is>
+      </c>
+      <c r="G72" s="6" t="inlineStr"/>
+      <c r="H72" s="6" t="inlineStr"/>
+      <c r="I72" s="6" t="inlineStr"/>
+      <c r="J72" s="18" t="inlineStr">
+        <is>
+          <t>수집예정</t>
+        </is>
+      </c>
+      <c r="K72" s="6" t="inlineStr"/>
+      <c r="L72" s="6" t="inlineStr"/>
+      <c r="M72" s="6" t="inlineStr"/>
+      <c r="N72" s="18" t="inlineStr">
+        <is>
+          <t>수집예정</t>
+        </is>
+      </c>
+      <c r="O72" s="6" t="inlineStr"/>
+      <c r="P72" s="18" t="inlineStr">
+        <is>
+          <t>수집예정</t>
+        </is>
+      </c>
+      <c r="Q72" s="18" t="inlineStr">
+        <is>
+          <t>수집예정</t>
+        </is>
+      </c>
+      <c r="R72" s="6" t="inlineStr">
+        <is>
+          <t>신고서 대기</t>
+        </is>
+      </c>
+    </row>
+    <row r="73" ht="30" customHeight="1">
+      <c r="A73" s="6" t="inlineStr">
+        <is>
+          <t>인텔리빅스</t>
+        </is>
+      </c>
+      <c r="B73" s="18" t="inlineStr">
+        <is>
+          <t>수집예정</t>
+        </is>
+      </c>
+      <c r="C73" s="18" t="inlineStr">
+        <is>
+          <t>수집예정</t>
+        </is>
+      </c>
+      <c r="D73" s="18" t="inlineStr">
+        <is>
+          <t>수집예정</t>
+        </is>
+      </c>
+      <c r="E73" s="18" t="inlineStr">
+        <is>
+          <t>수집예정</t>
+        </is>
+      </c>
+      <c r="F73" s="18" t="inlineStr">
+        <is>
+          <t>수집예정</t>
+        </is>
+      </c>
+      <c r="G73" s="6" t="inlineStr"/>
+      <c r="H73" s="6" t="inlineStr"/>
+      <c r="I73" s="6" t="inlineStr"/>
+      <c r="J73" s="18" t="inlineStr">
+        <is>
+          <t>수집예정</t>
+        </is>
+      </c>
+      <c r="K73" s="6" t="inlineStr"/>
+      <c r="L73" s="6" t="inlineStr"/>
+      <c r="M73" s="6" t="inlineStr"/>
+      <c r="N73" s="18" t="inlineStr">
+        <is>
+          <t>수집예정</t>
+        </is>
+      </c>
+      <c r="O73" s="6" t="inlineStr"/>
+      <c r="P73" s="18" t="inlineStr">
+        <is>
+          <t>수집예정</t>
+        </is>
+      </c>
+      <c r="Q73" s="18" t="inlineStr">
+        <is>
+          <t>수집예정</t>
+        </is>
+      </c>
+      <c r="R73" s="6" t="inlineStr">
+        <is>
+          <t>신고서 대기</t>
         </is>
       </c>
     </row>
     <row r="75">
       <c r="A75" s="20" t="inlineStr">
+        <is>
+          <t>※ 상장 완료 = KIND 신규상장 페이지 기준(스팩합병 포함) · 스팩 공모상장은 밴드·밸류에이션 등 해당없음(공모가 2,000원 고정).</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" s="20" t="inlineStr">
+        <is>
+          <t>※ 기재정정 신고서 내 정정 전·후 병존 → 자동수집은 "정정 후" 값만 취함.</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" s="20" t="inlineStr">
         <is>
           <t>※ 청약경쟁률=일반투자자 청약수량÷최종배정수량 · "MM-DD~"는 종료일 자동수집 예정.</t>
         </is>
@@ -12535,7 +12663,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F38"/>
+  <dimension ref="A1:F40"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -12789,122 +12917,130 @@
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="22" t="inlineStr">
-        <is>
-          <t>합계</t>
-        </is>
-      </c>
-      <c r="B14" s="22">
-        <f>SUM(B6:B13)</f>
-        <v/>
-      </c>
-      <c r="C14" s="22">
-        <f>SUM(C6:C13)</f>
-        <v/>
-      </c>
-      <c r="D14" s="22">
-        <f>SUM(D6:D13)</f>
-        <v/>
-      </c>
-      <c r="E14" s="22">
-        <f>SUM(E6:E13)</f>
-        <v/>
-      </c>
-      <c r="F14" s="23">
+      <c r="A14" s="6" t="inlineStr">
+        <is>
+          <t>2026-09</t>
+        </is>
+      </c>
+      <c r="B14" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="C14" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="D14" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="E14" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="F14" s="21">
         <f>IF((C14+D14)=0,"-",C14/(C14+D14))</f>
         <v/>
       </c>
     </row>
-    <row r="16">
-      <c r="A16" s="3" t="inlineStr">
+    <row r="15">
+      <c r="A15" s="22" t="inlineStr">
+        <is>
+          <t>합계</t>
+        </is>
+      </c>
+      <c r="B15" s="22">
+        <f>SUM(B6:B14)</f>
+        <v/>
+      </c>
+      <c r="C15" s="22">
+        <f>SUM(C6:C14)</f>
+        <v/>
+      </c>
+      <c r="D15" s="22">
+        <f>SUM(D6:D14)</f>
+        <v/>
+      </c>
+      <c r="E15" s="22">
+        <f>SUM(E6:E14)</f>
+        <v/>
+      </c>
+      <c r="F15" s="23">
+        <f>IF((C15+D15)=0,"-",C15/(C15+D15))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="3" t="inlineStr">
         <is>
           <t>② 주관사별 점유율 (공모 확보분)</t>
         </is>
       </c>
-      <c r="B16" s="4" t="n"/>
-      <c r="C16" s="4" t="n"/>
-    </row>
-    <row r="17">
-      <c r="A17" s="5" t="inlineStr">
+      <c r="B17" s="4" t="n"/>
+      <c r="C17" s="4" t="n"/>
+    </row>
+    <row r="18">
+      <c r="A18" s="5" t="inlineStr">
         <is>
           <t>대표주관사</t>
         </is>
       </c>
-      <c r="B17" s="5" t="inlineStr">
+      <c r="B18" s="5" t="inlineStr">
         <is>
           <t>건수</t>
         </is>
       </c>
-      <c r="C17" s="5" t="inlineStr">
+      <c r="C18" s="5" t="inlineStr">
         <is>
           <t>공모금액(백만원)</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" s="6" t="inlineStr">
-        <is>
-          <t>삼성증권</t>
-        </is>
-      </c>
-      <c r="B18" s="6" t="n">
-        <v>4</v>
-      </c>
-      <c r="C18" s="6" t="inlineStr">
-        <is>
-          <t>194,984,000,000</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="6" t="inlineStr">
         <is>
-          <t>미래에셋증권㈜</t>
+          <t>삼성증권</t>
         </is>
       </c>
       <c r="B19" s="6" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="C19" s="6" t="inlineStr">
         <is>
-          <t>156,428,800,000</t>
+          <t>194,984,000,000</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="6" t="inlineStr">
         <is>
-          <t>KB</t>
+          <t>미래에셋증권㈜</t>
         </is>
       </c>
       <c r="B20" s="6" t="n">
-        <v>7</v>
+        <v>1</v>
       </c>
       <c r="C20" s="6" t="inlineStr">
         <is>
-          <t>135,135,239,540</t>
+          <t>156,428,800,000</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="6" t="inlineStr">
         <is>
-          <t>대신증권</t>
+          <t>KB</t>
         </is>
       </c>
       <c r="B21" s="6" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="C21" s="6" t="inlineStr">
         <is>
-          <t>107,550,000,000</t>
+          <t>135,135,239,540</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="6" t="inlineStr">
         <is>
-          <t>한국투자증권</t>
+          <t>대신증권</t>
         </is>
       </c>
       <c r="B22" s="6" t="n">
@@ -12912,209 +13048,209 @@
       </c>
       <c r="C22" s="6" t="inlineStr">
         <is>
-          <t>102,800,000,000</t>
+          <t>107,550,000,000</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="6" t="inlineStr">
         <is>
-          <t>미래에셋증권</t>
+          <t>한국투자증권</t>
         </is>
       </c>
       <c r="B23" s="6" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="C23" s="6" t="inlineStr">
         <is>
-          <t>96,560,000,000</t>
+          <t>102,800,000,000</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="6" t="inlineStr">
         <is>
-          <t>아이비케이투자증권</t>
+          <t>미래에셋증권</t>
         </is>
       </c>
       <c r="B24" s="6" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="C24" s="6" t="inlineStr">
         <is>
-          <t>72,600,000,000</t>
+          <t>96,560,000,000</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="6" t="inlineStr">
         <is>
-          <t>DB증권</t>
+          <t>아이비케이투자증권</t>
         </is>
       </c>
       <c r="B25" s="6" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C25" s="6" t="inlineStr">
         <is>
-          <t>46,000,000,000</t>
+          <t>72,600,000,000</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="6" t="inlineStr">
         <is>
-          <t>NH투자증권</t>
+          <t>DB증권</t>
         </is>
       </c>
       <c r="B26" s="6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C26" s="6" t="inlineStr">
         <is>
-          <t>43,600,000,000</t>
+          <t>46,000,000,000</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="6" t="inlineStr">
         <is>
-          <t>하나증권</t>
+          <t>NH투자증권</t>
         </is>
       </c>
       <c r="B27" s="6" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C27" s="6" t="inlineStr">
         <is>
-          <t>35,414,000,000</t>
+          <t>43,600,000,000</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="6" t="inlineStr">
         <is>
-          <t>유진투자증권</t>
+          <t>하나증권</t>
         </is>
       </c>
       <c r="B28" s="6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C28" s="6" t="inlineStr">
         <is>
-          <t>24,000,000,000</t>
+          <t>35,414,000,000</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="6" t="inlineStr">
         <is>
-          <t>NH</t>
+          <t>신한투자증권</t>
         </is>
       </c>
       <c r="B29" s="6" t="n">
-        <v>7</v>
+        <v>1</v>
       </c>
       <c r="C29" s="6" t="inlineStr">
         <is>
-          <t>618,288</t>
+          <t>30,240,000,000</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="6" t="inlineStr">
         <is>
-          <t>한국</t>
+          <t>유진투자증권</t>
         </is>
       </c>
       <c r="B30" s="6" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="C30" s="6" t="inlineStr">
         <is>
-          <t>154,600</t>
+          <t>24,000,000,000</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="6" t="inlineStr">
         <is>
-          <t>미래</t>
+          <t>NH</t>
         </is>
       </c>
       <c r="B31" s="6" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="C31" s="6" t="inlineStr">
         <is>
-          <t>130,837</t>
+          <t>618,288</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="6" t="inlineStr">
         <is>
-          <t>신한</t>
+          <t>한국</t>
         </is>
       </c>
       <c r="B32" s="6" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="C32" s="6" t="inlineStr">
         <is>
-          <t>49,052</t>
+          <t>154,600</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="6" t="inlineStr">
         <is>
-          <t>삼성</t>
+          <t>미래</t>
         </is>
       </c>
       <c r="B33" s="6" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="C33" s="6" t="inlineStr">
         <is>
-          <t>32,000</t>
+          <t>130,837</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="6" t="inlineStr">
         <is>
-          <t>유진</t>
+          <t>신한</t>
         </is>
       </c>
       <c r="B34" s="6" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="C34" s="6" t="inlineStr">
         <is>
-          <t>25,020</t>
+          <t>49,052</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="6" t="inlineStr">
         <is>
-          <t>메리츠</t>
+          <t>삼성</t>
         </is>
       </c>
       <c r="B35" s="6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C35" s="6" t="inlineStr">
         <is>
-          <t>14,000</t>
+          <t>32,000</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="6" t="inlineStr">
         <is>
-          <t>대신</t>
+          <t>유진</t>
         </is>
       </c>
       <c r="B36" s="6" t="n">
@@ -13122,14 +13258,14 @@
       </c>
       <c r="C36" s="6" t="inlineStr">
         <is>
-          <t>13,000</t>
+          <t>25,020</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="6" t="inlineStr">
         <is>
-          <t>키움</t>
+          <t>메리츠</t>
         </is>
       </c>
       <c r="B37" s="6" t="n">
@@ -13137,20 +13273,50 @@
       </c>
       <c r="C37" s="6" t="inlineStr">
         <is>
-          <t>12,000</t>
+          <t>14,000</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="6" t="inlineStr">
         <is>
-          <t>교보</t>
+          <t>대신</t>
         </is>
       </c>
       <c r="B38" s="6" t="n">
         <v>1</v>
       </c>
       <c r="C38" s="6" t="inlineStr">
+        <is>
+          <t>13,000</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="6" t="inlineStr">
+        <is>
+          <t>키움</t>
+        </is>
+      </c>
+      <c r="B39" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="C39" s="6" t="inlineStr">
+        <is>
+          <t>12,000</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="6" t="inlineStr">
+        <is>
+          <t>교보</t>
+        </is>
+      </c>
+      <c r="B40" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="C40" s="6" t="inlineStr">
         <is>
           <t>10,800</t>
         </is>

</xml_diff>

<commit_message>
chore: update IPO data 2026-09-04
</commit_message>
<xml_diff>
--- a/IPO_analysis.xlsx
+++ b/IPO_analysis.xlsx
@@ -618,7 +618,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>기준일 2026-09-03 · 청구일 직전 사업연도 · 별도/개별 재무제표 · 단위 백만원(별도 표기 시 USD)</t>
+          <t>기준일 2026-09-04 · 청구일 직전 사업연도 · 별도/개별 재무제표 · 단위 백만원(별도 표기 시 USD)</t>
         </is>
       </c>
     </row>
@@ -4993,7 +4993,7 @@
       </c>
       <c r="K83" s="6" t="inlineStr">
         <is>
-          <t>상장승인(상장예정)</t>
+          <t>상장완료 (2026-09-04)</t>
         </is>
       </c>
     </row>
@@ -7792,7 +7792,7 @@
     <row r="6" ht="22" customHeight="1">
       <c r="A6" s="3" t="inlineStr">
         <is>
-          <t>■ 상장 완료 (2026)  (38건)</t>
+          <t>■ 상장 완료 (2026)  (39건)</t>
         </is>
       </c>
       <c r="B6" s="4" t="n"/>
@@ -7816,75 +7816,75 @@
     <row r="7" ht="30" customHeight="1">
       <c r="A7" s="6" t="inlineStr">
         <is>
-          <t>해치텍</t>
+          <t>스카이랩스</t>
         </is>
       </c>
       <c r="B7" s="6" t="inlineStr">
         <is>
-          <t>08-03~08-07</t>
+          <t>08-14~08-21</t>
         </is>
       </c>
       <c r="C7" s="6" t="inlineStr">
         <is>
-          <t>23,000~28,000</t>
+          <t>13,000~16,000</t>
         </is>
       </c>
       <c r="D7" s="7" t="inlineStr">
         <is>
-          <t>1,000,000</t>
+          <t>2,000,000</t>
         </is>
       </c>
       <c r="E7" s="7" t="inlineStr">
         <is>
-          <t>23,000,000,000</t>
+          <t>20,000,000,000</t>
         </is>
       </c>
       <c r="F7" s="6" t="inlineStr">
         <is>
-          <t>36.99배 (PER)</t>
+          <t>29.52배 (PER)</t>
         </is>
       </c>
       <c r="G7" s="6" t="inlineStr">
         <is>
-          <t>23,000</t>
+          <t>10,000</t>
         </is>
       </c>
       <c r="H7" s="6" t="n">
-        <v>101.91</v>
+        <v>63.41</v>
       </c>
       <c r="I7" s="6" t="n">
-        <v>321</v>
+        <v>246</v>
       </c>
       <c r="J7" s="18" t="inlineStr">
         <is>
           <t>수집예정</t>
         </is>
       </c>
-      <c r="K7" s="18" t="inlineStr">
-        <is>
-          <t>수집예정</t>
+      <c r="K7" s="6" t="inlineStr">
+        <is>
+          <t>88.20</t>
         </is>
       </c>
       <c r="L7" s="6" t="inlineStr"/>
       <c r="M7" s="6" t="inlineStr">
         <is>
-          <t>2026-08-25</t>
+          <t>2026-09-04</t>
         </is>
       </c>
       <c r="N7" s="6" t="inlineStr">
         <is>
-          <t>DB증권</t>
+          <t>한국투자증권</t>
         </is>
       </c>
       <c r="O7" s="6" t="inlineStr"/>
       <c r="P7" s="7" t="inlineStr">
         <is>
-          <t>1,302,950,000</t>
-        </is>
-      </c>
-      <c r="Q7" s="6" t="inlineStr">
-        <is>
-          <t>5.5%</t>
+          <t>1,071,200,000</t>
+        </is>
+      </c>
+      <c r="Q7" s="18" t="inlineStr">
+        <is>
+          <t>수집예정</t>
         </is>
       </c>
       <c r="R7" s="6" t="inlineStr">
@@ -7896,7 +7896,7 @@
     <row r="8" ht="30" customHeight="1">
       <c r="A8" s="6" t="inlineStr">
         <is>
-          <t>니어스랩</t>
+          <t>해치텍</t>
         </is>
       </c>
       <c r="B8" s="6" t="inlineStr">
@@ -7906,34 +7906,34 @@
       </c>
       <c r="C8" s="6" t="inlineStr">
         <is>
-          <t>30,000~41,200</t>
+          <t>23,000~28,000</t>
         </is>
       </c>
       <c r="D8" s="7" t="inlineStr">
         <is>
-          <t>910,000</t>
+          <t>1,000,000</t>
         </is>
       </c>
       <c r="E8" s="7" t="inlineStr">
         <is>
-          <t>37,492,000,000</t>
+          <t>23,000,000,000</t>
         </is>
       </c>
       <c r="F8" s="6" t="inlineStr">
         <is>
-          <t>44.41배 (PER)</t>
+          <t>36.99배 (PER)</t>
         </is>
       </c>
       <c r="G8" s="6" t="inlineStr">
         <is>
-          <t>41,200</t>
+          <t>23,000</t>
         </is>
       </c>
       <c r="H8" s="6" t="n">
-        <v>743.49</v>
+        <v>101.91</v>
       </c>
       <c r="I8" s="6" t="n">
-        <v>1795</v>
+        <v>321</v>
       </c>
       <c r="J8" s="18" t="inlineStr">
         <is>
@@ -7948,23 +7948,23 @@
       <c r="L8" s="6" t="inlineStr"/>
       <c r="M8" s="6" t="inlineStr">
         <is>
-          <t>2026-08-24</t>
+          <t>2026-08-25</t>
         </is>
       </c>
       <c r="N8" s="6" t="inlineStr">
         <is>
-          <t>삼성증권</t>
+          <t>DB증권</t>
         </is>
       </c>
       <c r="O8" s="6" t="inlineStr"/>
       <c r="P8" s="7" t="inlineStr">
         <is>
-          <t>1,265,355,000</t>
+          <t>1,302,950,000</t>
         </is>
       </c>
       <c r="Q8" s="6" t="inlineStr">
         <is>
-          <t>4.50%</t>
+          <t>5.5%</t>
         </is>
       </c>
       <c r="R8" s="6" t="inlineStr">
@@ -7976,44 +7976,44 @@
     <row r="9" ht="30" customHeight="1">
       <c r="A9" s="6" t="inlineStr">
         <is>
-          <t>기도산업</t>
+          <t>니어스랩</t>
         </is>
       </c>
       <c r="B9" s="6" t="inlineStr">
         <is>
-          <t>07-31~08-06</t>
+          <t>08-03~08-07</t>
         </is>
       </c>
       <c r="C9" s="6" t="inlineStr">
         <is>
-          <t>24,800~28,400</t>
+          <t>30,000~41,200</t>
         </is>
       </c>
       <c r="D9" s="7" t="inlineStr">
         <is>
-          <t>1,700,000</t>
+          <t>910,000</t>
         </is>
       </c>
       <c r="E9" s="7" t="inlineStr">
         <is>
-          <t>48,280,000,000</t>
+          <t>37,492,000,000</t>
         </is>
       </c>
       <c r="F9" s="6" t="inlineStr">
         <is>
-          <t>10.01배 (PER)</t>
+          <t>44.41배 (PER)</t>
         </is>
       </c>
       <c r="G9" s="6" t="inlineStr">
         <is>
-          <t>28,400</t>
+          <t>41,200</t>
         </is>
       </c>
       <c r="H9" s="6" t="n">
-        <v>213.31</v>
+        <v>743.49</v>
       </c>
       <c r="I9" s="6" t="n">
-        <v>637</v>
+        <v>1795</v>
       </c>
       <c r="J9" s="18" t="inlineStr">
         <is>
@@ -8028,23 +8028,23 @@
       <c r="L9" s="6" t="inlineStr"/>
       <c r="M9" s="6" t="inlineStr">
         <is>
-          <t>2026-08-21</t>
+          <t>2026-08-24</t>
         </is>
       </c>
       <c r="N9" s="6" t="inlineStr">
         <is>
-          <t>미래에셋증권</t>
+          <t>삼성증권</t>
         </is>
       </c>
       <c r="O9" s="6" t="inlineStr"/>
       <c r="P9" s="7" t="inlineStr">
         <is>
-          <t>716,720,000</t>
+          <t>1,265,355,000</t>
         </is>
       </c>
       <c r="Q9" s="6" t="inlineStr">
         <is>
-          <t>1.0%</t>
+          <t>4.50%</t>
         </is>
       </c>
       <c r="R9" s="6" t="inlineStr">
@@ -8056,44 +8056,44 @@
     <row r="10" ht="30" customHeight="1">
       <c r="A10" s="6" t="inlineStr">
         <is>
-          <t>인제니아테라퓨틱스</t>
+          <t>기도산업</t>
         </is>
       </c>
       <c r="B10" s="6" t="inlineStr">
         <is>
-          <t>07-20~07-24</t>
+          <t>07-31~08-06</t>
         </is>
       </c>
       <c r="C10" s="6" t="inlineStr">
         <is>
-          <t>12,000~14,500</t>
+          <t>24,800~28,400</t>
         </is>
       </c>
       <c r="D10" s="7" t="inlineStr">
         <is>
-          <t>5,000,000</t>
+          <t>1,700,000</t>
         </is>
       </c>
       <c r="E10" s="7" t="inlineStr">
         <is>
-          <t>60,000,000,000</t>
+          <t>48,280,000,000</t>
         </is>
       </c>
       <c r="F10" s="6" t="inlineStr">
         <is>
-          <t>22.89배 (PER)</t>
+          <t>10.01배 (PER)</t>
         </is>
       </c>
       <c r="G10" s="6" t="inlineStr">
         <is>
-          <t>12,000</t>
+          <t>28,400</t>
         </is>
       </c>
       <c r="H10" s="6" t="n">
-        <v>50.4</v>
+        <v>213.31</v>
       </c>
       <c r="I10" s="6" t="n">
-        <v>307</v>
+        <v>637</v>
       </c>
       <c r="J10" s="18" t="inlineStr">
         <is>
@@ -8108,23 +8108,23 @@
       <c r="L10" s="6" t="inlineStr"/>
       <c r="M10" s="6" t="inlineStr">
         <is>
-          <t>2026-08-18</t>
+          <t>2026-08-21</t>
         </is>
       </c>
       <c r="N10" s="6" t="inlineStr">
         <is>
-          <t>삼성증권</t>
+          <t>미래에셋증권</t>
         </is>
       </c>
       <c r="O10" s="6" t="inlineStr"/>
       <c r="P10" s="7" t="inlineStr">
         <is>
-          <t>4,095,000,000</t>
+          <t>716,720,000</t>
         </is>
       </c>
       <c r="Q10" s="6" t="inlineStr">
         <is>
-          <t>6.5%</t>
+          <t>1.0%</t>
         </is>
       </c>
       <c r="R10" s="6" t="inlineStr">
@@ -8136,44 +8136,44 @@
     <row r="11" ht="30" customHeight="1">
       <c r="A11" s="6" t="inlineStr">
         <is>
-          <t>케이앤에스아이앤씨</t>
+          <t>인제니아테라퓨틱스</t>
         </is>
       </c>
       <c r="B11" s="6" t="inlineStr">
         <is>
-          <t>07-27~07-31</t>
+          <t>07-20~07-24</t>
         </is>
       </c>
       <c r="C11" s="6" t="inlineStr">
         <is>
-          <t>9,000~11,000</t>
+          <t>12,000~14,500</t>
         </is>
       </c>
       <c r="D11" s="7" t="inlineStr">
         <is>
-          <t>2,400,000</t>
+          <t>5,000,000</t>
         </is>
       </c>
       <c r="E11" s="7" t="inlineStr">
         <is>
-          <t>26,400,000,000</t>
+          <t>60,000,000,000</t>
         </is>
       </c>
       <c r="F11" s="6" t="inlineStr">
         <is>
-          <t>42.08배 (PER)</t>
+          <t>22.89배 (PER)</t>
         </is>
       </c>
       <c r="G11" s="6" t="inlineStr">
         <is>
-          <t>11,000</t>
+          <t>12,000</t>
         </is>
       </c>
       <c r="H11" s="6" t="n">
-        <v>938.24</v>
+        <v>50.4</v>
       </c>
       <c r="I11" s="6" t="n">
-        <v>2024</v>
+        <v>307</v>
       </c>
       <c r="J11" s="18" t="inlineStr">
         <is>
@@ -8188,23 +8188,23 @@
       <c r="L11" s="6" t="inlineStr"/>
       <c r="M11" s="6" t="inlineStr">
         <is>
-          <t>2026-08-13</t>
+          <t>2026-08-18</t>
         </is>
       </c>
       <c r="N11" s="6" t="inlineStr">
         <is>
-          <t>아이비케이투자증권</t>
+          <t>삼성증권</t>
         </is>
       </c>
       <c r="O11" s="6" t="inlineStr"/>
       <c r="P11" s="7" t="inlineStr">
         <is>
-          <t>1,500,000,000</t>
+          <t>4,095,000,000</t>
         </is>
       </c>
       <c r="Q11" s="6" t="inlineStr">
         <is>
-          <t>3.5%</t>
+          <t>6.5%</t>
         </is>
       </c>
       <c r="R11" s="6" t="inlineStr">
@@ -8216,44 +8216,44 @@
     <row r="12" ht="30" customHeight="1">
       <c r="A12" s="6" t="inlineStr">
         <is>
-          <t>딜리셔스</t>
+          <t>케이앤에스아이앤씨</t>
         </is>
       </c>
       <c r="B12" s="6" t="inlineStr">
         <is>
-          <t>07-23~07-29</t>
+          <t>07-27~07-31</t>
         </is>
       </c>
       <c r="C12" s="6" t="inlineStr">
         <is>
-          <t>5,000~7,000</t>
+          <t>9,000~11,000</t>
         </is>
       </c>
       <c r="D12" s="7" t="inlineStr">
         <is>
-          <t>2,200,000</t>
+          <t>2,400,000</t>
         </is>
       </c>
       <c r="E12" s="7" t="inlineStr">
         <is>
-          <t>15,400,000,000</t>
+          <t>26,400,000,000</t>
         </is>
       </c>
       <c r="F12" s="6" t="inlineStr">
         <is>
-          <t>23.93배 (PER)</t>
+          <t>42.08배 (PER)</t>
         </is>
       </c>
       <c r="G12" s="6" t="inlineStr">
         <is>
-          <t>7,000</t>
+          <t>11,000</t>
         </is>
       </c>
       <c r="H12" s="6" t="n">
-        <v>184.06</v>
+        <v>938.24</v>
       </c>
       <c r="I12" s="6" t="n">
-        <v>441</v>
+        <v>2024</v>
       </c>
       <c r="J12" s="18" t="inlineStr">
         <is>
@@ -8268,23 +8268,23 @@
       <c r="L12" s="6" t="inlineStr"/>
       <c r="M12" s="6" t="inlineStr">
         <is>
-          <t>2026-08-12</t>
+          <t>2026-08-13</t>
         </is>
       </c>
       <c r="N12" s="6" t="inlineStr">
         <is>
-          <t>한국투자증권</t>
+          <t>아이비케이투자증권</t>
         </is>
       </c>
       <c r="O12" s="6" t="inlineStr"/>
       <c r="P12" s="7" t="inlineStr">
         <is>
-          <t>566,500,000</t>
+          <t>1,500,000,000</t>
         </is>
       </c>
       <c r="Q12" s="6" t="inlineStr">
         <is>
-          <t>5.0%</t>
+          <t>3.5%</t>
         </is>
       </c>
       <c r="R12" s="6" t="inlineStr">
@@ -8296,44 +8296,44 @@
     <row r="13" ht="30" customHeight="1">
       <c r="A13" s="6" t="inlineStr">
         <is>
-          <t>에이치엘지노믹스</t>
+          <t>딜리셔스</t>
         </is>
       </c>
       <c r="B13" s="6" t="inlineStr">
         <is>
-          <t>07-02~07-08</t>
+          <t>07-23~07-29</t>
         </is>
       </c>
       <c r="C13" s="6" t="inlineStr">
         <is>
-          <t>18,500~21,500</t>
+          <t>5,000~7,000</t>
         </is>
       </c>
       <c r="D13" s="7" t="inlineStr">
         <is>
-          <t>2,565,000</t>
+          <t>2,200,000</t>
         </is>
       </c>
       <c r="E13" s="7" t="inlineStr">
         <is>
-          <t>55,147,500,000</t>
+          <t>15,400,000,000</t>
         </is>
       </c>
       <c r="F13" s="6" t="inlineStr">
         <is>
-          <t>12.85배 (EV/EBITDA)</t>
+          <t>23.93배 (PER)</t>
         </is>
       </c>
       <c r="G13" s="6" t="inlineStr">
         <is>
-          <t>21,500</t>
+          <t>7,000</t>
         </is>
       </c>
       <c r="H13" s="6" t="n">
-        <v>714.52</v>
+        <v>184.06</v>
       </c>
       <c r="I13" s="6" t="n">
-        <v>2148</v>
+        <v>441</v>
       </c>
       <c r="J13" s="18" t="inlineStr">
         <is>
@@ -8348,27 +8348,23 @@
       <c r="L13" s="6" t="inlineStr"/>
       <c r="M13" s="6" t="inlineStr">
         <is>
-          <t>2026-07-24</t>
+          <t>2026-08-12</t>
         </is>
       </c>
       <c r="N13" s="6" t="inlineStr">
         <is>
-          <t>KB</t>
-        </is>
-      </c>
-      <c r="O13" s="6" t="inlineStr">
-        <is>
-          <t>아이비케이투자증권, IBK투자증권, IBK투자증권, IBK투자증권, IBK투자증권, IBK투자증권㈜, 보통주, IBK투자증권㈜</t>
-        </is>
-      </c>
+          <t>한국투자증권</t>
+        </is>
+      </c>
+      <c r="O13" s="6" t="inlineStr"/>
       <c r="P13" s="7" t="inlineStr">
         <is>
-          <t>1,211</t>
+          <t>566,500,000</t>
         </is>
       </c>
       <c r="Q13" s="6" t="inlineStr">
         <is>
-          <t>2.5%</t>
+          <t>5.0%</t>
         </is>
       </c>
       <c r="R13" s="6" t="inlineStr">
@@ -8380,63 +8376,59 @@
     <row r="14" ht="30" customHeight="1">
       <c r="A14" s="6" t="inlineStr">
         <is>
-          <t>레메디</t>
-        </is>
-      </c>
-      <c r="B14" s="18" t="inlineStr">
-        <is>
-          <t>수집예정</t>
+          <t>에이치엘지노믹스</t>
+        </is>
+      </c>
+      <c r="B14" s="6" t="inlineStr">
+        <is>
+          <t>07-02~07-08</t>
         </is>
       </c>
       <c r="C14" s="6" t="inlineStr">
         <is>
-          <t>17,800~20,700</t>
+          <t>18,500~21,500</t>
         </is>
       </c>
       <c r="D14" s="7" t="inlineStr">
         <is>
-          <t>1,200,000</t>
+          <t>2,565,000</t>
         </is>
       </c>
       <c r="E14" s="7" t="inlineStr">
         <is>
-          <t>24,840,000,000</t>
+          <t>55,147,500,000</t>
         </is>
       </c>
       <c r="F14" s="6" t="inlineStr">
         <is>
-          <t>21.95배 (PER)</t>
+          <t>12.85배 (EV/EBITDA)</t>
         </is>
       </c>
       <c r="G14" s="6" t="inlineStr">
         <is>
-          <t>20,700</t>
-        </is>
-      </c>
-      <c r="H14" s="6" t="inlineStr">
-        <is>
-          <t>1,146.41</t>
-        </is>
-      </c>
-      <c r="I14" s="6" t="inlineStr">
-        <is>
-          <t>2,246</t>
-        </is>
+          <t>21,500</t>
+        </is>
+      </c>
+      <c r="H14" s="6" t="n">
+        <v>714.52</v>
+      </c>
+      <c r="I14" s="6" t="n">
+        <v>2148</v>
       </c>
       <c r="J14" s="18" t="inlineStr">
         <is>
           <t>수집예정</t>
         </is>
       </c>
-      <c r="K14" s="6" t="inlineStr">
-        <is>
-          <t>1,706.71</t>
+      <c r="K14" s="18" t="inlineStr">
+        <is>
+          <t>수집예정</t>
         </is>
       </c>
       <c r="L14" s="6" t="inlineStr"/>
       <c r="M14" s="6" t="inlineStr">
         <is>
-          <t>2026-07-13</t>
+          <t>2026-07-24</t>
         </is>
       </c>
       <c r="N14" s="6" t="inlineStr">
@@ -8444,15 +8436,19 @@
           <t>KB</t>
         </is>
       </c>
-      <c r="O14" s="6" t="inlineStr"/>
+      <c r="O14" s="6" t="inlineStr">
+        <is>
+          <t>아이비케이투자증권, IBK투자증권, IBK투자증권, IBK투자증권, IBK투자증권, IBK투자증권㈜, 보통주, IBK투자증권㈜</t>
+        </is>
+      </c>
       <c r="P14" s="7" t="inlineStr">
         <is>
-          <t>1,279</t>
+          <t>1,211</t>
         </is>
       </c>
       <c r="Q14" s="6" t="inlineStr">
         <is>
-          <t>5.0%</t>
+          <t>2.5%</t>
         </is>
       </c>
       <c r="R14" s="6" t="inlineStr">
@@ -8464,7 +8460,7 @@
     <row r="15" ht="30" customHeight="1">
       <c r="A15" s="6" t="inlineStr">
         <is>
-          <t>레몬헬스케어</t>
+          <t>레메디</t>
         </is>
       </c>
       <c r="B15" s="18" t="inlineStr">
@@ -8474,45 +8470,53 @@
       </c>
       <c r="C15" s="6" t="inlineStr">
         <is>
-          <t>7,500~10,000</t>
+          <t>17,800~20,700</t>
         </is>
       </c>
       <c r="D15" s="7" t="inlineStr">
         <is>
-          <t>2,000,000</t>
+          <t>1,200,000</t>
         </is>
       </c>
       <c r="E15" s="7" t="inlineStr">
         <is>
-          <t>20,000</t>
+          <t>24,840,000,000</t>
         </is>
       </c>
       <c r="F15" s="6" t="inlineStr">
         <is>
-          <t>25.48배 (PER)</t>
-        </is>
-      </c>
-      <c r="G15" s="6" t="n">
-        <v>10000</v>
-      </c>
-      <c r="H15" s="6" t="n">
-        <v>1238</v>
-      </c>
-      <c r="I15" s="6" t="n">
-        <v>2233</v>
-      </c>
-      <c r="J15" s="6" t="inlineStr">
-        <is>
-          <t>2026-06-24~25</t>
-        </is>
-      </c>
-      <c r="K15" s="6" t="n">
-        <v>1510.57</v>
+          <t>21.95배 (PER)</t>
+        </is>
+      </c>
+      <c r="G15" s="6" t="inlineStr">
+        <is>
+          <t>20,700</t>
+        </is>
+      </c>
+      <c r="H15" s="6" t="inlineStr">
+        <is>
+          <t>1,146.41</t>
+        </is>
+      </c>
+      <c r="I15" s="6" t="inlineStr">
+        <is>
+          <t>2,246</t>
+        </is>
+      </c>
+      <c r="J15" s="18" t="inlineStr">
+        <is>
+          <t>수집예정</t>
+        </is>
+      </c>
+      <c r="K15" s="6" t="inlineStr">
+        <is>
+          <t>1,706.71</t>
+        </is>
       </c>
       <c r="L15" s="6" t="inlineStr"/>
       <c r="M15" s="6" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-07-13</t>
         </is>
       </c>
       <c r="N15" s="6" t="inlineStr">
@@ -8523,12 +8527,12 @@
       <c r="O15" s="6" t="inlineStr"/>
       <c r="P15" s="7" t="inlineStr">
         <is>
-          <t>824</t>
+          <t>1,279</t>
         </is>
       </c>
       <c r="Q15" s="6" t="inlineStr">
         <is>
-          <t>4.0%</t>
+          <t>5.0%</t>
         </is>
       </c>
       <c r="R15" s="6" t="inlineStr">
@@ -8540,7 +8544,7 @@
     <row r="16" ht="30" customHeight="1">
       <c r="A16" s="6" t="inlineStr">
         <is>
-          <t>매드업</t>
+          <t>레몬헬스케어</t>
         </is>
       </c>
       <c r="B16" s="18" t="inlineStr">
@@ -8550,7 +8554,7 @@
       </c>
       <c r="C16" s="6" t="inlineStr">
         <is>
-          <t>7,000~8,000</t>
+          <t>7,500~10,000</t>
         </is>
       </c>
       <c r="D16" s="7" t="inlineStr">
@@ -8560,51 +8564,51 @@
       </c>
       <c r="E16" s="7" t="inlineStr">
         <is>
-          <t>16,000</t>
+          <t>20,000</t>
         </is>
       </c>
       <c r="F16" s="6" t="inlineStr">
         <is>
-          <t>24.57배 (PER)</t>
+          <t>25.48배 (PER)</t>
         </is>
       </c>
       <c r="G16" s="6" t="n">
-        <v>8000</v>
+        <v>10000</v>
       </c>
       <c r="H16" s="6" t="n">
-        <v>1396.29</v>
+        <v>1238</v>
       </c>
       <c r="I16" s="6" t="n">
-        <v>2392</v>
+        <v>2233</v>
       </c>
       <c r="J16" s="6" t="inlineStr">
         <is>
-          <t>2026-06-23~24</t>
+          <t>2026-06-24~25</t>
         </is>
       </c>
       <c r="K16" s="6" t="n">
-        <v>3304.76</v>
+        <v>1510.57</v>
       </c>
       <c r="L16" s="6" t="inlineStr"/>
       <c r="M16" s="6" t="inlineStr">
         <is>
-          <t>2026-07-01</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="N16" s="6" t="inlineStr">
         <is>
-          <t>미래</t>
+          <t>KB</t>
         </is>
       </c>
       <c r="O16" s="6" t="inlineStr"/>
       <c r="P16" s="7" t="inlineStr">
         <is>
-          <t>742</t>
+          <t>824</t>
         </is>
       </c>
       <c r="Q16" s="6" t="inlineStr">
         <is>
-          <t>4.5%</t>
+          <t>4.0%</t>
         </is>
       </c>
       <c r="R16" s="6" t="inlineStr">
@@ -8616,75 +8620,71 @@
     <row r="17" ht="30" customHeight="1">
       <c r="A17" s="6" t="inlineStr">
         <is>
-          <t>한국제16호스팩</t>
-        </is>
-      </c>
-      <c r="B17" s="19" t="inlineStr">
-        <is>
-          <t>해당없음</t>
+          <t>매드업</t>
+        </is>
+      </c>
+      <c r="B17" s="18" t="inlineStr">
+        <is>
+          <t>수집예정</t>
         </is>
       </c>
       <c r="C17" s="6" t="inlineStr">
         <is>
-          <t>2,000</t>
+          <t>7,000~8,000</t>
         </is>
       </c>
       <c r="D17" s="7" t="inlineStr">
         <is>
-          <t>5,500,000</t>
+          <t>2,000,000</t>
         </is>
       </c>
       <c r="E17" s="7" t="inlineStr">
         <is>
-          <t>11,000</t>
-        </is>
-      </c>
-      <c r="F17" s="19" t="inlineStr">
-        <is>
-          <t>해당없음</t>
-        </is>
-      </c>
-      <c r="G17" s="6" t="inlineStr">
-        <is>
-          <t>2,000</t>
-        </is>
+          <t>16,000</t>
+        </is>
+      </c>
+      <c r="F17" s="6" t="inlineStr">
+        <is>
+          <t>24.57배 (PER)</t>
+        </is>
+      </c>
+      <c r="G17" s="6" t="n">
+        <v>8000</v>
       </c>
       <c r="H17" s="6" t="n">
-        <v>1364.09</v>
+        <v>1396.29</v>
       </c>
       <c r="I17" s="6" t="n">
-        <v>2089</v>
+        <v>2392</v>
       </c>
       <c r="J17" s="6" t="inlineStr">
         <is>
-          <t>2026-06-22~06-23</t>
-        </is>
-      </c>
-      <c r="K17" s="6" t="inlineStr">
-        <is>
-          <t>1,274.77</t>
-        </is>
+          <t>2026-06-23~24</t>
+        </is>
+      </c>
+      <c r="K17" s="6" t="n">
+        <v>3304.76</v>
       </c>
       <c r="L17" s="6" t="inlineStr"/>
       <c r="M17" s="6" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-07-01</t>
         </is>
       </c>
       <c r="N17" s="6" t="inlineStr">
         <is>
-          <t>한국</t>
+          <t>미래</t>
         </is>
       </c>
       <c r="O17" s="6" t="inlineStr"/>
       <c r="P17" s="7" t="inlineStr">
         <is>
-          <t>330</t>
+          <t>742</t>
         </is>
       </c>
       <c r="Q17" s="6" t="inlineStr">
         <is>
-          <t>3.00%</t>
+          <t>4.5%</t>
         </is>
       </c>
       <c r="R17" s="6" t="inlineStr">
@@ -8696,51 +8696,53 @@
     <row r="18" ht="30" customHeight="1">
       <c r="A18" s="6" t="inlineStr">
         <is>
-          <t>스트라드비젼</t>
-        </is>
-      </c>
-      <c r="B18" s="18" t="inlineStr">
-        <is>
-          <t>수집예정</t>
+          <t>한국제16호스팩</t>
+        </is>
+      </c>
+      <c r="B18" s="19" t="inlineStr">
+        <is>
+          <t>해당없음</t>
         </is>
       </c>
       <c r="C18" s="6" t="inlineStr">
         <is>
-          <t>12,000~14,000</t>
+          <t>2,000</t>
         </is>
       </c>
       <c r="D18" s="7" t="inlineStr">
         <is>
-          <t>7,000,000</t>
+          <t>5,500,000</t>
         </is>
       </c>
       <c r="E18" s="7" t="inlineStr">
         <is>
-          <t>84,000</t>
-        </is>
-      </c>
-      <c r="F18" s="6" t="inlineStr">
-        <is>
-          <t>37.45배 (PER)</t>
-        </is>
-      </c>
-      <c r="G18" s="6" t="n">
-        <v>12000</v>
+          <t>11,000</t>
+        </is>
+      </c>
+      <c r="F18" s="19" t="inlineStr">
+        <is>
+          <t>해당없음</t>
+        </is>
+      </c>
+      <c r="G18" s="6" t="inlineStr">
+        <is>
+          <t>2,000</t>
+        </is>
       </c>
       <c r="H18" s="6" t="n">
-        <v>381.3</v>
+        <v>1364.09</v>
       </c>
       <c r="I18" s="6" t="n">
-        <v>1604</v>
+        <v>2089</v>
       </c>
       <c r="J18" s="6" t="inlineStr">
         <is>
-          <t>2026-06-18~06-19</t>
+          <t>2026-06-22~06-23</t>
         </is>
       </c>
       <c r="K18" s="6" t="inlineStr">
         <is>
-          <t>45.81</t>
+          <t>1,274.77</t>
         </is>
       </c>
       <c r="L18" s="6" t="inlineStr"/>
@@ -8751,13 +8753,13 @@
       </c>
       <c r="N18" s="6" t="inlineStr">
         <is>
-          <t>KB</t>
+          <t>한국</t>
         </is>
       </c>
       <c r="O18" s="6" t="inlineStr"/>
       <c r="P18" s="7" t="inlineStr">
         <is>
-          <t>2,575</t>
+          <t>330</t>
         </is>
       </c>
       <c r="Q18" s="6" t="inlineStr">
@@ -8774,7 +8776,7 @@
     <row r="19" ht="30" customHeight="1">
       <c r="A19" s="6" t="inlineStr">
         <is>
-          <t>져스텍</t>
+          <t>스트라드비젼</t>
         </is>
       </c>
       <c r="B19" s="18" t="inlineStr">
@@ -8784,32 +8786,32 @@
       </c>
       <c r="C19" s="6" t="inlineStr">
         <is>
-          <t>10,500~12,500</t>
+          <t>12,000~14,000</t>
         </is>
       </c>
       <c r="D19" s="7" t="inlineStr">
         <is>
-          <t>1,600,000</t>
+          <t>7,000,000</t>
         </is>
       </c>
       <c r="E19" s="7" t="inlineStr">
         <is>
-          <t>20,000</t>
+          <t>84,000</t>
         </is>
       </c>
       <c r="F19" s="6" t="inlineStr">
         <is>
-          <t>26.82배 (PER)</t>
+          <t>37.45배 (PER)</t>
         </is>
       </c>
       <c r="G19" s="6" t="n">
-        <v>12500</v>
+        <v>12000</v>
       </c>
       <c r="H19" s="6" t="n">
-        <v>1294.99</v>
+        <v>381.3</v>
       </c>
       <c r="I19" s="6" t="n">
-        <v>2252</v>
+        <v>1604</v>
       </c>
       <c r="J19" s="6" t="inlineStr">
         <is>
@@ -8818,29 +8820,29 @@
       </c>
       <c r="K19" s="6" t="inlineStr">
         <is>
-          <t>2,783.89</t>
+          <t>45.81</t>
         </is>
       </c>
       <c r="L19" s="6" t="inlineStr"/>
       <c r="M19" s="6" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="N19" s="6" t="inlineStr">
         <is>
-          <t>삼성</t>
+          <t>KB</t>
         </is>
       </c>
       <c r="O19" s="6" t="inlineStr"/>
       <c r="P19" s="7" t="inlineStr">
         <is>
-          <t>1,164</t>
+          <t>2,575</t>
         </is>
       </c>
       <c r="Q19" s="6" t="inlineStr">
         <is>
-          <t>5.65%</t>
+          <t>3.00%</t>
         </is>
       </c>
       <c r="R19" s="6" t="inlineStr">
@@ -8852,75 +8854,73 @@
     <row r="20" ht="30" customHeight="1">
       <c r="A20" s="6" t="inlineStr">
         <is>
-          <t>메리츠제2호스팩</t>
-        </is>
-      </c>
-      <c r="B20" s="19" t="inlineStr">
-        <is>
-          <t>해당없음</t>
+          <t>져스텍</t>
+        </is>
+      </c>
+      <c r="B20" s="18" t="inlineStr">
+        <is>
+          <t>수집예정</t>
         </is>
       </c>
       <c r="C20" s="6" t="inlineStr">
         <is>
-          <t>2,000</t>
+          <t>10,500~12,500</t>
         </is>
       </c>
       <c r="D20" s="7" t="inlineStr">
         <is>
-          <t>7,000,000</t>
+          <t>1,600,000</t>
         </is>
       </c>
       <c r="E20" s="7" t="inlineStr">
         <is>
-          <t>14,000</t>
-        </is>
-      </c>
-      <c r="F20" s="19" t="inlineStr">
-        <is>
-          <t>해당없음</t>
-        </is>
-      </c>
-      <c r="G20" s="6" t="inlineStr">
-        <is>
-          <t>2,000</t>
-        </is>
+          <t>20,000</t>
+        </is>
+      </c>
+      <c r="F20" s="6" t="inlineStr">
+        <is>
+          <t>26.82배 (PER)</t>
+        </is>
+      </c>
+      <c r="G20" s="6" t="n">
+        <v>12500</v>
       </c>
       <c r="H20" s="6" t="n">
-        <v>1087.58</v>
+        <v>1294.99</v>
       </c>
       <c r="I20" s="6" t="n">
-        <v>1798</v>
+        <v>2252</v>
       </c>
       <c r="J20" s="6" t="inlineStr">
         <is>
-          <t>2026-06-09~06-10</t>
+          <t>2026-06-18~06-19</t>
         </is>
       </c>
       <c r="K20" s="6" t="inlineStr">
         <is>
-          <t>1,338.66</t>
+          <t>2,783.89</t>
         </is>
       </c>
       <c r="L20" s="6" t="inlineStr"/>
       <c r="M20" s="6" t="inlineStr">
         <is>
-          <t>2026-06-19</t>
+          <t>2026-06-29</t>
         </is>
       </c>
       <c r="N20" s="6" t="inlineStr">
         <is>
-          <t>메리츠</t>
+          <t>삼성</t>
         </is>
       </c>
       <c r="O20" s="6" t="inlineStr"/>
       <c r="P20" s="7" t="inlineStr">
         <is>
-          <t>245</t>
+          <t>1,164</t>
         </is>
       </c>
       <c r="Q20" s="6" t="inlineStr">
         <is>
-          <t>1.75%</t>
+          <t>5.65%</t>
         </is>
       </c>
       <c r="R20" s="6" t="inlineStr">
@@ -8932,77 +8932,75 @@
     <row r="21" ht="30" customHeight="1">
       <c r="A21" s="6" t="inlineStr">
         <is>
-          <t>피스피스스튜디오</t>
-        </is>
-      </c>
-      <c r="B21" s="18" t="inlineStr">
-        <is>
-          <t>수집예정</t>
+          <t>메리츠제2호스팩</t>
+        </is>
+      </c>
+      <c r="B21" s="19" t="inlineStr">
+        <is>
+          <t>해당없음</t>
         </is>
       </c>
       <c r="C21" s="6" t="inlineStr">
         <is>
-          <t>19,000~21,500</t>
+          <t>2,000</t>
         </is>
       </c>
       <c r="D21" s="7" t="inlineStr">
         <is>
-          <t>2,272,637</t>
+          <t>7,000,000</t>
         </is>
       </c>
       <c r="E21" s="7" t="inlineStr">
         <is>
-          <t>48,862</t>
-        </is>
-      </c>
-      <c r="F21" s="6" t="inlineStr">
-        <is>
-          <t>21.48배 (PER)</t>
-        </is>
-      </c>
-      <c r="G21" s="6" t="n">
-        <v>21500</v>
+          <t>14,000</t>
+        </is>
+      </c>
+      <c r="F21" s="19" t="inlineStr">
+        <is>
+          <t>해당없음</t>
+        </is>
+      </c>
+      <c r="G21" s="6" t="inlineStr">
+        <is>
+          <t>2,000</t>
+        </is>
       </c>
       <c r="H21" s="6" t="n">
-        <v>847.76</v>
+        <v>1087.58</v>
       </c>
       <c r="I21" s="6" t="n">
-        <v>2329</v>
+        <v>1798</v>
       </c>
       <c r="J21" s="6" t="inlineStr">
         <is>
-          <t>2026-05-26~05-27</t>
+          <t>2026-06-09~06-10</t>
         </is>
       </c>
       <c r="K21" s="6" t="inlineStr">
         <is>
-          <t>1,191.15</t>
+          <t>1,338.66</t>
         </is>
       </c>
       <c r="L21" s="6" t="inlineStr"/>
       <c r="M21" s="6" t="inlineStr">
         <is>
-          <t>2026-06-08</t>
+          <t>2026-06-19</t>
         </is>
       </c>
       <c r="N21" s="6" t="inlineStr">
         <is>
-          <t>미래</t>
-        </is>
-      </c>
-      <c r="O21" s="6" t="inlineStr">
-        <is>
-          <t>NH</t>
-        </is>
-      </c>
+          <t>메리츠</t>
+        </is>
+      </c>
+      <c r="O21" s="6" t="inlineStr"/>
       <c r="P21" s="7" t="inlineStr">
         <is>
-          <t>1,994</t>
+          <t>245</t>
         </is>
       </c>
       <c r="Q21" s="6" t="inlineStr">
         <is>
-          <t>4.00%</t>
+          <t>1.75%</t>
         </is>
       </c>
       <c r="R21" s="6" t="inlineStr">
@@ -9014,75 +9012,77 @@
     <row r="22" ht="30" customHeight="1">
       <c r="A22" s="6" t="inlineStr">
         <is>
-          <t>대신밸런스제20호스팩</t>
-        </is>
-      </c>
-      <c r="B22" s="19" t="inlineStr">
-        <is>
-          <t>해당없음</t>
+          <t>피스피스스튜디오</t>
+        </is>
+      </c>
+      <c r="B22" s="18" t="inlineStr">
+        <is>
+          <t>수집예정</t>
         </is>
       </c>
       <c r="C22" s="6" t="inlineStr">
         <is>
-          <t>2,000</t>
+          <t>19,000~21,500</t>
         </is>
       </c>
       <c r="D22" s="7" t="inlineStr">
         <is>
-          <t>6,500,000</t>
+          <t>2,272,637</t>
         </is>
       </c>
       <c r="E22" s="7" t="inlineStr">
         <is>
-          <t>13,000</t>
-        </is>
-      </c>
-      <c r="F22" s="19" t="inlineStr">
-        <is>
-          <t>해당없음</t>
-        </is>
-      </c>
-      <c r="G22" s="6" t="inlineStr">
-        <is>
-          <t>2,000</t>
-        </is>
+          <t>48,862</t>
+        </is>
+      </c>
+      <c r="F22" s="6" t="inlineStr">
+        <is>
+          <t>21.48배 (PER)</t>
+        </is>
+      </c>
+      <c r="G22" s="6" t="n">
+        <v>21500</v>
       </c>
       <c r="H22" s="6" t="n">
-        <v>1327.13</v>
+        <v>847.76</v>
       </c>
       <c r="I22" s="6" t="n">
-        <v>2194</v>
+        <v>2329</v>
       </c>
       <c r="J22" s="6" t="inlineStr">
         <is>
-          <t>2026-05-22~05-25</t>
+          <t>2026-05-26~05-27</t>
         </is>
       </c>
       <c r="K22" s="6" t="inlineStr">
         <is>
-          <t>1,486.88</t>
+          <t>1,191.15</t>
         </is>
       </c>
       <c r="L22" s="6" t="inlineStr"/>
       <c r="M22" s="6" t="inlineStr">
         <is>
-          <t>2026-06-05</t>
+          <t>2026-06-08</t>
         </is>
       </c>
       <c r="N22" s="6" t="inlineStr">
         <is>
-          <t>대신</t>
-        </is>
-      </c>
-      <c r="O22" s="6" t="inlineStr"/>
+          <t>미래</t>
+        </is>
+      </c>
+      <c r="O22" s="6" t="inlineStr">
+        <is>
+          <t>NH</t>
+        </is>
+      </c>
       <c r="P22" s="7" t="inlineStr">
         <is>
-          <t>390</t>
+          <t>1,994</t>
         </is>
       </c>
       <c r="Q22" s="6" t="inlineStr">
         <is>
-          <t>3.00%</t>
+          <t>4.00%</t>
         </is>
       </c>
       <c r="R22" s="6" t="inlineStr">
@@ -9094,73 +9094,75 @@
     <row r="23" ht="30" customHeight="1">
       <c r="A23" s="6" t="inlineStr">
         <is>
-          <t>마키나락스</t>
-        </is>
-      </c>
-      <c r="B23" s="18" t="inlineStr">
-        <is>
-          <t>수집예정</t>
+          <t>대신밸런스제20호스팩</t>
+        </is>
+      </c>
+      <c r="B23" s="19" t="inlineStr">
+        <is>
+          <t>해당없음</t>
         </is>
       </c>
       <c r="C23" s="6" t="inlineStr">
         <is>
-          <t>12,500~15,000</t>
+          <t>2,000</t>
         </is>
       </c>
       <c r="D23" s="7" t="inlineStr">
         <is>
-          <t>2,635,000</t>
+          <t>6,500,000</t>
         </is>
       </c>
       <c r="E23" s="7" t="inlineStr">
         <is>
-          <t>39,525</t>
-        </is>
-      </c>
-      <c r="F23" s="6" t="inlineStr">
-        <is>
-          <t>40.5배 (PER)</t>
-        </is>
-      </c>
-      <c r="G23" s="6" t="n">
-        <v>15000</v>
+          <t>13,000</t>
+        </is>
+      </c>
+      <c r="F23" s="19" t="inlineStr">
+        <is>
+          <t>해당없음</t>
+        </is>
+      </c>
+      <c r="G23" s="6" t="inlineStr">
+        <is>
+          <t>2,000</t>
+        </is>
       </c>
       <c r="H23" s="6" t="n">
-        <v>1196.08</v>
+        <v>1327.13</v>
       </c>
       <c r="I23" s="6" t="n">
-        <v>2427</v>
+        <v>2194</v>
       </c>
       <c r="J23" s="6" t="inlineStr">
         <is>
-          <t>2026-05-11~05-12</t>
+          <t>2026-05-22~05-25</t>
         </is>
       </c>
       <c r="K23" s="6" t="inlineStr">
         <is>
-          <t>2,807.79</t>
+          <t>1,486.88</t>
         </is>
       </c>
       <c r="L23" s="6" t="inlineStr"/>
       <c r="M23" s="6" t="inlineStr">
         <is>
-          <t>2026-05-20</t>
+          <t>2026-06-05</t>
         </is>
       </c>
       <c r="N23" s="6" t="inlineStr">
         <is>
-          <t>미래</t>
+          <t>대신</t>
         </is>
       </c>
       <c r="O23" s="6" t="inlineStr"/>
       <c r="P23" s="7" t="inlineStr">
         <is>
-          <t>2,026</t>
+          <t>390</t>
         </is>
       </c>
       <c r="Q23" s="6" t="inlineStr">
         <is>
-          <t>5.00%</t>
+          <t>3.00%</t>
         </is>
       </c>
       <c r="R23" s="6" t="inlineStr">
@@ -9172,7 +9174,7 @@
     <row r="24" ht="30" customHeight="1">
       <c r="A24" s="6" t="inlineStr">
         <is>
-          <t>폴레드</t>
+          <t>마키나락스</t>
         </is>
       </c>
       <c r="B24" s="18" t="inlineStr">
@@ -9182,63 +9184,63 @@
       </c>
       <c r="C24" s="6" t="inlineStr">
         <is>
-          <t>4,100~5,000</t>
+          <t>12,500~15,000</t>
         </is>
       </c>
       <c r="D24" s="7" t="inlineStr">
         <is>
-          <t>2,600,000</t>
+          <t>2,635,000</t>
         </is>
       </c>
       <c r="E24" s="7" t="inlineStr">
         <is>
-          <t>13,000</t>
+          <t>39,525</t>
         </is>
       </c>
       <c r="F24" s="6" t="inlineStr">
         <is>
-          <t>19.05배 (PER)</t>
+          <t>40.5배 (PER)</t>
         </is>
       </c>
       <c r="G24" s="6" t="n">
-        <v>5000</v>
+        <v>15000</v>
       </c>
       <c r="H24" s="6" t="n">
-        <v>1486.66</v>
+        <v>1196.08</v>
       </c>
       <c r="I24" s="6" t="n">
-        <v>2372</v>
+        <v>2427</v>
       </c>
       <c r="J24" s="6" t="inlineStr">
         <is>
-          <t>2026-05-04~05-05</t>
+          <t>2026-05-11~05-12</t>
         </is>
       </c>
       <c r="K24" s="6" t="inlineStr">
         <is>
-          <t>3,169.86</t>
+          <t>2,807.79</t>
         </is>
       </c>
       <c r="L24" s="6" t="inlineStr"/>
       <c r="M24" s="6" t="inlineStr">
         <is>
-          <t>2026-05-14</t>
+          <t>2026-05-20</t>
         </is>
       </c>
       <c r="N24" s="6" t="inlineStr">
         <is>
-          <t>NH</t>
+          <t>미래</t>
         </is>
       </c>
       <c r="O24" s="6" t="inlineStr"/>
       <c r="P24" s="7" t="inlineStr">
         <is>
-          <t>540</t>
+          <t>2,026</t>
         </is>
       </c>
       <c r="Q24" s="6" t="inlineStr">
         <is>
-          <t>4.03%</t>
+          <t>5.00%</t>
         </is>
       </c>
       <c r="R24" s="6" t="inlineStr">
@@ -9250,7 +9252,7 @@
     <row r="25" ht="30" customHeight="1">
       <c r="A25" s="6" t="inlineStr">
         <is>
-          <t>코스모로보틱스</t>
+          <t>폴레드</t>
         </is>
       </c>
       <c r="B25" s="18" t="inlineStr">
@@ -9260,67 +9262,63 @@
       </c>
       <c r="C25" s="6" t="inlineStr">
         <is>
-          <t>5,300~6,000</t>
+          <t>4,100~5,000</t>
         </is>
       </c>
       <c r="D25" s="7" t="inlineStr">
         <is>
-          <t>4,170,000</t>
+          <t>2,600,000</t>
         </is>
       </c>
       <c r="E25" s="7" t="inlineStr">
         <is>
-          <t>25,020</t>
+          <t>13,000</t>
         </is>
       </c>
       <c r="F25" s="6" t="inlineStr">
         <is>
-          <t>47.45배 (PER)</t>
+          <t>19.05배 (PER)</t>
         </is>
       </c>
       <c r="G25" s="6" t="n">
-        <v>6000</v>
+        <v>5000</v>
       </c>
       <c r="H25" s="6" t="n">
-        <v>1140.11</v>
+        <v>1486.66</v>
       </c>
       <c r="I25" s="6" t="n">
-        <v>2257</v>
+        <v>2372</v>
       </c>
       <c r="J25" s="6" t="inlineStr">
         <is>
-          <t>2026-04-27~04-28</t>
+          <t>2026-05-04~05-05</t>
         </is>
       </c>
       <c r="K25" s="6" t="inlineStr">
         <is>
-          <t>2,013.80</t>
+          <t>3,169.86</t>
         </is>
       </c>
       <c r="L25" s="6" t="inlineStr"/>
       <c r="M25" s="6" t="inlineStr">
         <is>
-          <t>2026-05-11</t>
+          <t>2026-05-14</t>
         </is>
       </c>
       <c r="N25" s="6" t="inlineStr">
         <is>
-          <t>유진</t>
-        </is>
-      </c>
-      <c r="O25" s="6" t="inlineStr">
-        <is>
           <t>NH</t>
         </is>
       </c>
+      <c r="O25" s="6" t="inlineStr"/>
       <c r="P25" s="7" t="inlineStr">
         <is>
-          <t>1,289</t>
+          <t>540</t>
         </is>
       </c>
       <c r="Q25" s="6" t="inlineStr">
         <is>
-          <t>3.78%</t>
+          <t>4.03%</t>
         </is>
       </c>
       <c r="R25" s="6" t="inlineStr">
@@ -9332,75 +9330,77 @@
     <row r="26" ht="30" customHeight="1">
       <c r="A26" s="6" t="inlineStr">
         <is>
-          <t>신한스팩18호</t>
-        </is>
-      </c>
-      <c r="B26" s="19" t="inlineStr">
-        <is>
-          <t>해당없음</t>
+          <t>코스모로보틱스</t>
+        </is>
+      </c>
+      <c r="B26" s="18" t="inlineStr">
+        <is>
+          <t>수집예정</t>
         </is>
       </c>
       <c r="C26" s="6" t="inlineStr">
         <is>
-          <t>2,000</t>
+          <t>5,300~6,000</t>
         </is>
       </c>
       <c r="D26" s="7" t="inlineStr">
         <is>
-          <t>5,000,000</t>
+          <t>4,170,000</t>
         </is>
       </c>
       <c r="E26" s="7" t="inlineStr">
         <is>
-          <t>10,000</t>
-        </is>
-      </c>
-      <c r="F26" s="19" t="inlineStr">
-        <is>
-          <t>해당없음</t>
-        </is>
-      </c>
-      <c r="G26" s="6" t="inlineStr">
-        <is>
-          <t>2,000</t>
-        </is>
+          <t>25,020</t>
+        </is>
+      </c>
+      <c r="F26" s="6" t="inlineStr">
+        <is>
+          <t>47.45배 (PER)</t>
+        </is>
+      </c>
+      <c r="G26" s="6" t="n">
+        <v>6000</v>
       </c>
       <c r="H26" s="6" t="n">
-        <v>1388.6</v>
+        <v>1140.11</v>
       </c>
       <c r="I26" s="6" t="n">
-        <v>2044</v>
+        <v>2257</v>
       </c>
       <c r="J26" s="6" t="inlineStr">
         <is>
-          <t>2026-04-20~04-21</t>
+          <t>2026-04-27~04-28</t>
         </is>
       </c>
       <c r="K26" s="6" t="inlineStr">
         <is>
-          <t>1,601.36</t>
+          <t>2,013.80</t>
         </is>
       </c>
       <c r="L26" s="6" t="inlineStr"/>
       <c r="M26" s="6" t="inlineStr">
         <is>
-          <t>2026-04-30</t>
+          <t>2026-05-11</t>
         </is>
       </c>
       <c r="N26" s="6" t="inlineStr">
         <is>
-          <t>신한</t>
-        </is>
-      </c>
-      <c r="O26" s="6" t="inlineStr"/>
+          <t>유진</t>
+        </is>
+      </c>
+      <c r="O26" s="6" t="inlineStr">
+        <is>
+          <t>NH</t>
+        </is>
+      </c>
       <c r="P26" s="7" t="inlineStr">
         <is>
-          <t>350</t>
+          <t>1,289</t>
         </is>
       </c>
       <c r="Q26" s="6" t="inlineStr">
         <is>
-          <t>3.50%</t>
+          <t>3.78%</t>
         </is>
       </c>
       <c r="R26" s="6" t="inlineStr">
@@ -9412,42 +9412,44 @@
     <row r="27" ht="30" customHeight="1">
       <c r="A27" s="6" t="inlineStr">
         <is>
-          <t>채비</t>
-        </is>
-      </c>
-      <c r="B27" s="18" t="inlineStr">
-        <is>
-          <t>수집예정</t>
+          <t>신한스팩18호</t>
+        </is>
+      </c>
+      <c r="B27" s="19" t="inlineStr">
+        <is>
+          <t>해당없음</t>
         </is>
       </c>
       <c r="C27" s="6" t="inlineStr">
         <is>
-          <t>12,300~15,300</t>
+          <t>2,000</t>
         </is>
       </c>
       <c r="D27" s="7" t="inlineStr">
         <is>
-          <t>9,000,000</t>
+          <t>5,000,000</t>
         </is>
       </c>
       <c r="E27" s="7" t="inlineStr">
         <is>
-          <t>110,700</t>
-        </is>
-      </c>
-      <c r="F27" s="6" t="inlineStr">
-        <is>
-          <t>24.0배 (EV/EBITDA)</t>
-        </is>
-      </c>
-      <c r="G27" s="6" t="n">
-        <v>12300</v>
+          <t>10,000</t>
+        </is>
+      </c>
+      <c r="F27" s="19" t="inlineStr">
+        <is>
+          <t>해당없음</t>
+        </is>
+      </c>
+      <c r="G27" s="6" t="inlineStr">
+        <is>
+          <t>2,000</t>
+        </is>
       </c>
       <c r="H27" s="6" t="n">
-        <v>55.23</v>
+        <v>1388.6</v>
       </c>
       <c r="I27" s="6" t="n">
-        <v>751</v>
+        <v>2044</v>
       </c>
       <c r="J27" s="6" t="inlineStr">
         <is>
@@ -9456,33 +9458,29 @@
       </c>
       <c r="K27" s="6" t="inlineStr">
         <is>
-          <t>302.11</t>
+          <t>1,601.36</t>
         </is>
       </c>
       <c r="L27" s="6" t="inlineStr"/>
       <c r="M27" s="6" t="inlineStr">
         <is>
-          <t>2026-04-29</t>
+          <t>2026-04-30</t>
         </is>
       </c>
       <c r="N27" s="6" t="inlineStr">
         <is>
-          <t>KB</t>
-        </is>
-      </c>
-      <c r="O27" s="6" t="inlineStr">
-        <is>
-          <t>삼성</t>
-        </is>
-      </c>
+          <t>신한</t>
+        </is>
+      </c>
+      <c r="O27" s="6" t="inlineStr"/>
       <c r="P27" s="7" t="inlineStr">
         <is>
-          <t>3,384</t>
+          <t>350</t>
         </is>
       </c>
       <c r="Q27" s="6" t="inlineStr">
         <is>
-          <t>3.00%</t>
+          <t>3.50%</t>
         </is>
       </c>
       <c r="R27" s="6" t="inlineStr">
@@ -9494,75 +9492,77 @@
     <row r="28" ht="30" customHeight="1">
       <c r="A28" s="6" t="inlineStr">
         <is>
-          <t>키움히어로스펙2호</t>
-        </is>
-      </c>
-      <c r="B28" s="19" t="inlineStr">
-        <is>
-          <t>해당없음</t>
+          <t>채비</t>
+        </is>
+      </c>
+      <c r="B28" s="18" t="inlineStr">
+        <is>
+          <t>수집예정</t>
         </is>
       </c>
       <c r="C28" s="6" t="inlineStr">
         <is>
-          <t>2,000</t>
+          <t>12,300~15,300</t>
         </is>
       </c>
       <c r="D28" s="7" t="inlineStr">
         <is>
-          <t>6,000,000</t>
+          <t>9,000,000</t>
         </is>
       </c>
       <c r="E28" s="7" t="inlineStr">
         <is>
-          <t>12,000</t>
-        </is>
-      </c>
-      <c r="F28" s="19" t="inlineStr">
-        <is>
-          <t>해당없음</t>
-        </is>
-      </c>
-      <c r="G28" s="6" t="inlineStr">
-        <is>
-          <t>2,000</t>
-        </is>
+          <t>110,700</t>
+        </is>
+      </c>
+      <c r="F28" s="6" t="inlineStr">
+        <is>
+          <t>24.0배 (EV/EBITDA)</t>
+        </is>
+      </c>
+      <c r="G28" s="6" t="n">
+        <v>12300</v>
       </c>
       <c r="H28" s="6" t="n">
-        <v>1271.12</v>
+        <v>55.23</v>
       </c>
       <c r="I28" s="6" t="n">
-        <v>2054</v>
+        <v>751</v>
       </c>
       <c r="J28" s="6" t="inlineStr">
         <is>
-          <t>2026-04-14~04-15</t>
+          <t>2026-04-20~04-21</t>
         </is>
       </c>
       <c r="K28" s="6" t="inlineStr">
         <is>
-          <t>1,727.59</t>
+          <t>302.11</t>
         </is>
       </c>
       <c r="L28" s="6" t="inlineStr"/>
       <c r="M28" s="6" t="inlineStr">
         <is>
-          <t>2026-04-23</t>
+          <t>2026-04-29</t>
         </is>
       </c>
       <c r="N28" s="6" t="inlineStr">
         <is>
-          <t>키움</t>
-        </is>
-      </c>
-      <c r="O28" s="6" t="inlineStr"/>
+          <t>KB</t>
+        </is>
+      </c>
+      <c r="O28" s="6" t="inlineStr">
+        <is>
+          <t>삼성</t>
+        </is>
+      </c>
       <c r="P28" s="7" t="inlineStr">
         <is>
-          <t>300</t>
+          <t>3,384</t>
         </is>
       </c>
       <c r="Q28" s="6" t="inlineStr">
         <is>
-          <t>2.50%</t>
+          <t>3.00%</t>
         </is>
       </c>
       <c r="R28" s="6" t="inlineStr">
@@ -9574,7 +9574,7 @@
     <row r="29" ht="30" customHeight="1">
       <c r="A29" s="6" t="inlineStr">
         <is>
-          <t>교보스팩20호</t>
+          <t>키움히어로스펙2호</t>
         </is>
       </c>
       <c r="B29" s="19" t="inlineStr">
@@ -9589,12 +9589,12 @@
       </c>
       <c r="D29" s="7" t="inlineStr">
         <is>
-          <t>5,400,000</t>
+          <t>6,000,000</t>
         </is>
       </c>
       <c r="E29" s="7" t="inlineStr">
         <is>
-          <t>10,800</t>
+          <t>12,000</t>
         </is>
       </c>
       <c r="F29" s="19" t="inlineStr">
@@ -9608,30 +9608,30 @@
         </is>
       </c>
       <c r="H29" s="6" t="n">
-        <v>1196.99</v>
+        <v>1271.12</v>
       </c>
       <c r="I29" s="6" t="n">
-        <v>1855</v>
+        <v>2054</v>
       </c>
       <c r="J29" s="6" t="inlineStr">
         <is>
-          <t>2026-03-23~03-24</t>
+          <t>2026-04-14~04-15</t>
         </is>
       </c>
       <c r="K29" s="6" t="inlineStr">
         <is>
-          <t>747.00</t>
+          <t>1,727.59</t>
         </is>
       </c>
       <c r="L29" s="6" t="inlineStr"/>
       <c r="M29" s="6" t="inlineStr">
         <is>
-          <t>2026-04-02</t>
+          <t>2026-04-23</t>
         </is>
       </c>
       <c r="N29" s="6" t="inlineStr">
         <is>
-          <t>교보</t>
+          <t>키움</t>
         </is>
       </c>
       <c r="O29" s="6" t="inlineStr"/>
@@ -9642,7 +9642,7 @@
       </c>
       <c r="Q29" s="6" t="inlineStr">
         <is>
-          <t>2.78%</t>
+          <t>2.50%</t>
         </is>
       </c>
       <c r="R29" s="6" t="inlineStr">
@@ -9654,42 +9654,44 @@
     <row r="30" ht="30" customHeight="1">
       <c r="A30" s="6" t="inlineStr">
         <is>
-          <t>인벤테라</t>
-        </is>
-      </c>
-      <c r="B30" s="18" t="inlineStr">
-        <is>
-          <t>수집예정</t>
+          <t>교보스팩20호</t>
+        </is>
+      </c>
+      <c r="B30" s="19" t="inlineStr">
+        <is>
+          <t>해당없음</t>
         </is>
       </c>
       <c r="C30" s="6" t="inlineStr">
         <is>
-          <t>12,100~16,600</t>
+          <t>2,000</t>
         </is>
       </c>
       <c r="D30" s="7" t="inlineStr">
         <is>
-          <t>1,180,000</t>
+          <t>5,400,000</t>
         </is>
       </c>
       <c r="E30" s="7" t="inlineStr">
         <is>
-          <t>19,588</t>
-        </is>
-      </c>
-      <c r="F30" s="6" t="inlineStr">
-        <is>
-          <t>24.34배 (PER)</t>
-        </is>
-      </c>
-      <c r="G30" s="6" t="n">
-        <v>16600</v>
+          <t>10,800</t>
+        </is>
+      </c>
+      <c r="F30" s="19" t="inlineStr">
+        <is>
+          <t>해당없음</t>
+        </is>
+      </c>
+      <c r="G30" s="6" t="inlineStr">
+        <is>
+          <t>2,000</t>
+        </is>
       </c>
       <c r="H30" s="6" t="n">
-        <v>1328.82</v>
+        <v>1196.99</v>
       </c>
       <c r="I30" s="6" t="n">
-        <v>2309</v>
+        <v>1855</v>
       </c>
       <c r="J30" s="6" t="inlineStr">
         <is>
@@ -9698,7 +9700,7 @@
       </c>
       <c r="K30" s="6" t="inlineStr">
         <is>
-          <t>1,913.00</t>
+          <t>747.00</t>
         </is>
       </c>
       <c r="L30" s="6" t="inlineStr"/>
@@ -9709,18 +9711,18 @@
       </c>
       <c r="N30" s="6" t="inlineStr">
         <is>
-          <t>NH</t>
+          <t>교보</t>
         </is>
       </c>
       <c r="O30" s="6" t="inlineStr"/>
       <c r="P30" s="7" t="inlineStr">
         <is>
-          <t>1,211</t>
+          <t>300</t>
         </is>
       </c>
       <c r="Q30" s="6" t="inlineStr">
         <is>
-          <t>6.00%</t>
+          <t>2.78%</t>
         </is>
       </c>
       <c r="R30" s="6" t="inlineStr">
@@ -9732,75 +9734,73 @@
     <row r="31" ht="30" customHeight="1">
       <c r="A31" s="6" t="inlineStr">
         <is>
-          <t>신한스팩17호</t>
-        </is>
-      </c>
-      <c r="B31" s="19" t="inlineStr">
-        <is>
-          <t>해당없음</t>
+          <t>인벤테라</t>
+        </is>
+      </c>
+      <c r="B31" s="18" t="inlineStr">
+        <is>
+          <t>수집예정</t>
         </is>
       </c>
       <c r="C31" s="6" t="inlineStr">
         <is>
-          <t>2,000</t>
+          <t>12,100~16,600</t>
         </is>
       </c>
       <c r="D31" s="7" t="inlineStr">
         <is>
-          <t>5,000,000</t>
+          <t>1,180,000</t>
         </is>
       </c>
       <c r="E31" s="7" t="inlineStr">
         <is>
-          <t>10,000</t>
-        </is>
-      </c>
-      <c r="F31" s="19" t="inlineStr">
-        <is>
-          <t>해당없음</t>
-        </is>
-      </c>
-      <c r="G31" s="6" t="inlineStr">
-        <is>
-          <t>2,000</t>
-        </is>
+          <t>19,588</t>
+        </is>
+      </c>
+      <c r="F31" s="6" t="inlineStr">
+        <is>
+          <t>24.34배 (PER)</t>
+        </is>
+      </c>
+      <c r="G31" s="6" t="n">
+        <v>16600</v>
       </c>
       <c r="H31" s="6" t="n">
-        <v>1343.8</v>
+        <v>1328.82</v>
       </c>
       <c r="I31" s="6" t="n">
-        <v>2022</v>
+        <v>2309</v>
       </c>
       <c r="J31" s="6" t="inlineStr">
         <is>
-          <t>2026-03-19~03-20</t>
+          <t>2026-03-23~03-24</t>
         </is>
       </c>
       <c r="K31" s="6" t="inlineStr">
         <is>
-          <t>1,403.74</t>
+          <t>1,913.00</t>
         </is>
       </c>
       <c r="L31" s="6" t="inlineStr"/>
       <c r="M31" s="6" t="inlineStr">
         <is>
-          <t>2026-04-01</t>
+          <t>2026-04-02</t>
         </is>
       </c>
       <c r="N31" s="6" t="inlineStr">
         <is>
-          <t>신한</t>
+          <t>NH</t>
         </is>
       </c>
       <c r="O31" s="6" t="inlineStr"/>
       <c r="P31" s="7" t="inlineStr">
         <is>
-          <t>350</t>
+          <t>1,211</t>
         </is>
       </c>
       <c r="Q31" s="6" t="inlineStr">
         <is>
-          <t>3.50%</t>
+          <t>6.00%</t>
         </is>
       </c>
       <c r="R31" s="6" t="inlineStr">
@@ -9812,42 +9812,44 @@
     <row r="32" ht="30" customHeight="1">
       <c r="A32" s="6" t="inlineStr">
         <is>
-          <t>리센스메디컬</t>
-        </is>
-      </c>
-      <c r="B32" s="18" t="inlineStr">
-        <is>
-          <t>수집예정</t>
+          <t>신한스팩17호</t>
+        </is>
+      </c>
+      <c r="B32" s="19" t="inlineStr">
+        <is>
+          <t>해당없음</t>
         </is>
       </c>
       <c r="C32" s="6" t="inlineStr">
         <is>
-          <t>9,000~11,000</t>
+          <t>2,000</t>
         </is>
       </c>
       <c r="D32" s="7" t="inlineStr">
         <is>
-          <t>1,400,000</t>
+          <t>5,000,000</t>
         </is>
       </c>
       <c r="E32" s="7" t="inlineStr">
         <is>
-          <t>15,400</t>
-        </is>
-      </c>
-      <c r="F32" s="6" t="inlineStr">
-        <is>
-          <t>31.33배 (PER)</t>
-        </is>
-      </c>
-      <c r="G32" s="6" t="n">
-        <v>11000</v>
+          <t>10,000</t>
+        </is>
+      </c>
+      <c r="F32" s="19" t="inlineStr">
+        <is>
+          <t>해당없음</t>
+        </is>
+      </c>
+      <c r="G32" s="6" t="inlineStr">
+        <is>
+          <t>2,000</t>
+        </is>
       </c>
       <c r="H32" s="6" t="n">
-        <v>1352.63</v>
+        <v>1343.8</v>
       </c>
       <c r="I32" s="6" t="n">
-        <v>2261</v>
+        <v>2022</v>
       </c>
       <c r="J32" s="6" t="inlineStr">
         <is>
@@ -9856,33 +9858,29 @@
       </c>
       <c r="K32" s="6" t="inlineStr">
         <is>
-          <t>2,097.68</t>
+          <t>1,403.74</t>
         </is>
       </c>
       <c r="L32" s="6" t="inlineStr"/>
       <c r="M32" s="6" t="inlineStr">
         <is>
-          <t>2026-03-31</t>
+          <t>2026-04-01</t>
         </is>
       </c>
       <c r="N32" s="6" t="inlineStr">
         <is>
-          <t>한국</t>
-        </is>
-      </c>
-      <c r="O32" s="6" t="inlineStr">
-        <is>
-          <t>KB</t>
-        </is>
-      </c>
+          <t>신한</t>
+        </is>
+      </c>
+      <c r="O32" s="6" t="inlineStr"/>
       <c r="P32" s="7" t="inlineStr">
         <is>
-          <t>916</t>
+          <t>350</t>
         </is>
       </c>
       <c r="Q32" s="6" t="inlineStr">
         <is>
-          <t>5.77%</t>
+          <t>3.50%</t>
         </is>
       </c>
       <c r="R32" s="6" t="inlineStr">
@@ -9894,75 +9892,77 @@
     <row r="33" ht="30" customHeight="1">
       <c r="A33" s="6" t="inlineStr">
         <is>
-          <t>NH스팩33호</t>
-        </is>
-      </c>
-      <c r="B33" s="19" t="inlineStr">
-        <is>
-          <t>해당없음</t>
+          <t>리센스메디컬</t>
+        </is>
+      </c>
+      <c r="B33" s="18" t="inlineStr">
+        <is>
+          <t>수집예정</t>
         </is>
       </c>
       <c r="C33" s="6" t="inlineStr">
         <is>
-          <t>2,000</t>
+          <t>9,000~11,000</t>
         </is>
       </c>
       <c r="D33" s="7" t="inlineStr">
         <is>
-          <t>6,350,000</t>
+          <t>1,400,000</t>
         </is>
       </c>
       <c r="E33" s="7" t="inlineStr">
         <is>
-          <t>12,700</t>
-        </is>
-      </c>
-      <c r="F33" s="19" t="inlineStr">
-        <is>
-          <t>해당없음</t>
-        </is>
-      </c>
-      <c r="G33" s="6" t="inlineStr">
-        <is>
-          <t>2,000</t>
-        </is>
+          <t>15,400</t>
+        </is>
+      </c>
+      <c r="F33" s="6" t="inlineStr">
+        <is>
+          <t>31.33배 (PER)</t>
+        </is>
+      </c>
+      <c r="G33" s="6" t="n">
+        <v>11000</v>
       </c>
       <c r="H33" s="6" t="n">
-        <v>1228.71</v>
+        <v>1352.63</v>
       </c>
       <c r="I33" s="6" t="n">
-        <v>2058</v>
+        <v>2261</v>
       </c>
       <c r="J33" s="6" t="inlineStr">
         <is>
-          <t>2026-03-17~03-18</t>
+          <t>2026-03-19~03-20</t>
         </is>
       </c>
       <c r="K33" s="6" t="inlineStr">
         <is>
-          <t>569.27</t>
+          <t>2,097.68</t>
         </is>
       </c>
       <c r="L33" s="6" t="inlineStr"/>
       <c r="M33" s="6" t="inlineStr">
         <is>
-          <t>2026-03-27</t>
+          <t>2026-03-31</t>
         </is>
       </c>
       <c r="N33" s="6" t="inlineStr">
         <is>
-          <t>NH</t>
-        </is>
-      </c>
-      <c r="O33" s="6" t="inlineStr"/>
+          <t>한국</t>
+        </is>
+      </c>
+      <c r="O33" s="6" t="inlineStr">
+        <is>
+          <t>KB</t>
+        </is>
+      </c>
       <c r="P33" s="7" t="inlineStr">
         <is>
-          <t>381</t>
+          <t>916</t>
         </is>
       </c>
       <c r="Q33" s="6" t="inlineStr">
         <is>
-          <t>3.00%</t>
+          <t>5.77%</t>
         </is>
       </c>
       <c r="R33" s="6" t="inlineStr">
@@ -9974,73 +9974,75 @@
     <row r="34" ht="30" customHeight="1">
       <c r="A34" s="6" t="inlineStr">
         <is>
-          <t>메쥬</t>
-        </is>
-      </c>
-      <c r="B34" s="18" t="inlineStr">
-        <is>
-          <t>수집예정</t>
+          <t>NH스팩33호</t>
+        </is>
+      </c>
+      <c r="B34" s="19" t="inlineStr">
+        <is>
+          <t>해당없음</t>
         </is>
       </c>
       <c r="C34" s="6" t="inlineStr">
         <is>
-          <t>16,700~21,600</t>
+          <t>2,000</t>
         </is>
       </c>
       <c r="D34" s="7" t="inlineStr">
         <is>
-          <t>1,345,000</t>
+          <t>6,350,000</t>
         </is>
       </c>
       <c r="E34" s="7" t="inlineStr">
         <is>
-          <t>29,052</t>
-        </is>
-      </c>
-      <c r="F34" s="6" t="inlineStr">
-        <is>
-          <t>20.66배 (PER)</t>
-        </is>
-      </c>
-      <c r="G34" s="6" t="n">
-        <v>21600</v>
+          <t>12,700</t>
+        </is>
+      </c>
+      <c r="F34" s="19" t="inlineStr">
+        <is>
+          <t>해당없음</t>
+        </is>
+      </c>
+      <c r="G34" s="6" t="inlineStr">
+        <is>
+          <t>2,000</t>
+        </is>
       </c>
       <c r="H34" s="6" t="n">
-        <v>1108.93</v>
+        <v>1228.71</v>
       </c>
       <c r="I34" s="6" t="n">
-        <v>2320</v>
+        <v>2058</v>
       </c>
       <c r="J34" s="6" t="inlineStr">
         <is>
-          <t>2026-03-16~03-17</t>
+          <t>2026-03-17~03-18</t>
         </is>
       </c>
       <c r="K34" s="6" t="inlineStr">
         <is>
-          <t>2,428.25</t>
+          <t>569.27</t>
         </is>
       </c>
       <c r="L34" s="6" t="inlineStr"/>
       <c r="M34" s="6" t="inlineStr">
         <is>
-          <t>2026-03-26</t>
+          <t>2026-03-27</t>
         </is>
       </c>
       <c r="N34" s="6" t="inlineStr">
         <is>
-          <t>신한</t>
+          <t>NH</t>
         </is>
       </c>
       <c r="O34" s="6" t="inlineStr"/>
       <c r="P34" s="7" t="inlineStr">
         <is>
-          <t>1,496</t>
+          <t>381</t>
         </is>
       </c>
       <c r="Q34" s="6" t="inlineStr">
         <is>
-          <t>5.00%</t>
+          <t>3.00%</t>
         </is>
       </c>
       <c r="R34" s="6" t="inlineStr">
@@ -10052,7 +10054,7 @@
     <row r="35" ht="30" customHeight="1">
       <c r="A35" s="6" t="inlineStr">
         <is>
-          <t>한패스</t>
+          <t>메쥬</t>
         </is>
       </c>
       <c r="B35" s="18" t="inlineStr">
@@ -10062,32 +10064,32 @@
       </c>
       <c r="C35" s="6" t="inlineStr">
         <is>
-          <t>17,000~19,000</t>
+          <t>16,700~21,600</t>
         </is>
       </c>
       <c r="D35" s="7" t="inlineStr">
         <is>
-          <t>1,100,000</t>
+          <t>1,345,000</t>
         </is>
       </c>
       <c r="E35" s="7" t="inlineStr">
         <is>
-          <t>20,900</t>
+          <t>29,052</t>
         </is>
       </c>
       <c r="F35" s="6" t="inlineStr">
         <is>
-          <t>29.09배 (PER)</t>
+          <t>20.66배 (PER)</t>
         </is>
       </c>
       <c r="G35" s="6" t="n">
-        <v>19000</v>
+        <v>21600</v>
       </c>
       <c r="H35" s="6" t="n">
-        <v>1172.59</v>
+        <v>1108.93</v>
       </c>
       <c r="I35" s="6" t="n">
-        <v>2229</v>
+        <v>2320</v>
       </c>
       <c r="J35" s="6" t="inlineStr">
         <is>
@@ -10096,29 +10098,29 @@
       </c>
       <c r="K35" s="6" t="inlineStr">
         <is>
-          <t>1,673.04</t>
+          <t>2,428.25</t>
         </is>
       </c>
       <c r="L35" s="6" t="inlineStr"/>
       <c r="M35" s="6" t="inlineStr">
         <is>
-          <t>2026-03-25</t>
+          <t>2026-03-26</t>
         </is>
       </c>
       <c r="N35" s="6" t="inlineStr">
         <is>
-          <t>한국</t>
+          <t>신한</t>
         </is>
       </c>
       <c r="O35" s="6" t="inlineStr"/>
       <c r="P35" s="7" t="inlineStr">
         <is>
-          <t>753</t>
+          <t>1,496</t>
         </is>
       </c>
       <c r="Q35" s="6" t="inlineStr">
         <is>
-          <t>3.50%</t>
+          <t>5.00%</t>
         </is>
       </c>
       <c r="R35" s="6" t="inlineStr">
@@ -10130,7 +10132,7 @@
     <row r="36" ht="30" customHeight="1">
       <c r="A36" s="6" t="inlineStr">
         <is>
-          <t>아이엠바이오로직스</t>
+          <t>한패스</t>
         </is>
       </c>
       <c r="B36" s="18" t="inlineStr">
@@ -10140,47 +10142,47 @@
       </c>
       <c r="C36" s="6" t="inlineStr">
         <is>
-          <t>19,000~26,000</t>
+          <t>17,000~19,000</t>
         </is>
       </c>
       <c r="D36" s="7" t="inlineStr">
         <is>
-          <t>2,000,000</t>
+          <t>1,100,000</t>
         </is>
       </c>
       <c r="E36" s="7" t="inlineStr">
         <is>
-          <t>52,000</t>
+          <t>20,900</t>
         </is>
       </c>
       <c r="F36" s="6" t="inlineStr">
         <is>
-          <t>21.46배 (PER)</t>
+          <t>29.09배 (PER)</t>
         </is>
       </c>
       <c r="G36" s="6" t="n">
-        <v>26000</v>
+        <v>19000</v>
       </c>
       <c r="H36" s="6" t="n">
-        <v>839.23</v>
+        <v>1172.59</v>
       </c>
       <c r="I36" s="6" t="n">
-        <v>2333</v>
+        <v>2229</v>
       </c>
       <c r="J36" s="6" t="inlineStr">
         <is>
-          <t>2026-03-11~03-12</t>
+          <t>2026-03-16~03-17</t>
         </is>
       </c>
       <c r="K36" s="6" t="inlineStr">
         <is>
-          <t>1,806.00</t>
+          <t>1,673.04</t>
         </is>
       </c>
       <c r="L36" s="6" t="inlineStr"/>
       <c r="M36" s="6" t="inlineStr">
         <is>
-          <t>2026-03-20</t>
+          <t>2026-03-25</t>
         </is>
       </c>
       <c r="N36" s="6" t="inlineStr">
@@ -10191,12 +10193,12 @@
       <c r="O36" s="6" t="inlineStr"/>
       <c r="P36" s="7" t="inlineStr">
         <is>
-          <t>2,650</t>
+          <t>753</t>
         </is>
       </c>
       <c r="Q36" s="6" t="inlineStr">
         <is>
-          <t>5.00%</t>
+          <t>3.50%</t>
         </is>
       </c>
       <c r="R36" s="6" t="inlineStr">
@@ -10208,7 +10210,7 @@
     <row r="37" ht="30" customHeight="1">
       <c r="A37" s="6" t="inlineStr">
         <is>
-          <t>카나프테라퓨틱스</t>
+          <t>아이엠바이오로직스</t>
         </is>
       </c>
       <c r="B37" s="18" t="inlineStr">
@@ -10218,7 +10220,7 @@
       </c>
       <c r="C37" s="6" t="inlineStr">
         <is>
-          <t>16,000~20,000</t>
+          <t>19,000~26,000</t>
         </is>
       </c>
       <c r="D37" s="7" t="inlineStr">
@@ -10228,37 +10230,37 @@
       </c>
       <c r="E37" s="7" t="inlineStr">
         <is>
-          <t>40,000</t>
+          <t>52,000</t>
         </is>
       </c>
       <c r="F37" s="6" t="inlineStr">
         <is>
-          <t>23.59배 (PER)</t>
+          <t>21.46배 (PER)</t>
         </is>
       </c>
       <c r="G37" s="6" t="n">
-        <v>20000</v>
+        <v>26000</v>
       </c>
       <c r="H37" s="6" t="n">
-        <v>962.1</v>
+        <v>839.23</v>
       </c>
       <c r="I37" s="6" t="n">
-        <v>2327</v>
+        <v>2333</v>
       </c>
       <c r="J37" s="6" t="inlineStr">
         <is>
-          <t>2026-03-05~03-06</t>
+          <t>2026-03-11~03-12</t>
         </is>
       </c>
       <c r="K37" s="6" t="inlineStr">
         <is>
-          <t>1,899.29</t>
+          <t>1,806.00</t>
         </is>
       </c>
       <c r="L37" s="6" t="inlineStr"/>
       <c r="M37" s="6" t="inlineStr">
         <is>
-          <t>2026-03-16</t>
+          <t>2026-03-20</t>
         </is>
       </c>
       <c r="N37" s="6" t="inlineStr">
@@ -10269,7 +10271,7 @@
       <c r="O37" s="6" t="inlineStr"/>
       <c r="P37" s="7" t="inlineStr">
         <is>
-          <t>2,050</t>
+          <t>2,650</t>
         </is>
       </c>
       <c r="Q37" s="6" t="inlineStr">
@@ -10286,7 +10288,7 @@
     <row r="38" ht="30" customHeight="1">
       <c r="A38" s="6" t="inlineStr">
         <is>
-          <t>액스비스</t>
+          <t>카나프테라퓨틱스</t>
         </is>
       </c>
       <c r="B38" s="18" t="inlineStr">
@@ -10296,63 +10298,63 @@
       </c>
       <c r="C38" s="6" t="inlineStr">
         <is>
-          <t>10,100~11,500</t>
+          <t>16,000~20,000</t>
         </is>
       </c>
       <c r="D38" s="7" t="inlineStr">
         <is>
-          <t>2,300,000</t>
+          <t>2,000,000</t>
         </is>
       </c>
       <c r="E38" s="7" t="inlineStr">
         <is>
-          <t>26,450</t>
+          <t>40,000</t>
         </is>
       </c>
       <c r="F38" s="6" t="inlineStr">
         <is>
-          <t>27.60배 (PER)</t>
+          <t>23.59배 (PER)</t>
         </is>
       </c>
       <c r="G38" s="6" t="n">
-        <v>11500</v>
+        <v>20000</v>
       </c>
       <c r="H38" s="6" t="n">
-        <v>1124.21</v>
+        <v>962.1</v>
       </c>
       <c r="I38" s="6" t="n">
-        <v>2411</v>
+        <v>2327</v>
       </c>
       <c r="J38" s="6" t="inlineStr">
         <is>
-          <t>2026-02-23~02-24</t>
+          <t>2026-03-05~03-06</t>
         </is>
       </c>
       <c r="K38" s="6" t="inlineStr">
         <is>
-          <t>1,960.87</t>
+          <t>1,899.29</t>
         </is>
       </c>
       <c r="L38" s="6" t="inlineStr"/>
       <c r="M38" s="6" t="inlineStr">
         <is>
-          <t>2026-03-09</t>
+          <t>2026-03-16</t>
         </is>
       </c>
       <c r="N38" s="6" t="inlineStr">
         <is>
-          <t>미래</t>
+          <t>한국</t>
         </is>
       </c>
       <c r="O38" s="6" t="inlineStr"/>
       <c r="P38" s="7" t="inlineStr">
         <is>
-          <t>1,090</t>
+          <t>2,050</t>
         </is>
       </c>
       <c r="Q38" s="6" t="inlineStr">
         <is>
-          <t>4.00%</t>
+          <t>5.00%</t>
         </is>
       </c>
       <c r="R38" s="6" t="inlineStr">
@@ -10364,7 +10366,7 @@
     <row r="39" ht="30" customHeight="1">
       <c r="A39" s="6" t="inlineStr">
         <is>
-          <t>에스팀</t>
+          <t>액스비스</t>
         </is>
       </c>
       <c r="B39" s="18" t="inlineStr">
@@ -10374,32 +10376,32 @@
       </c>
       <c r="C39" s="6" t="inlineStr">
         <is>
-          <t>7,000~8,500</t>
+          <t>10,100~11,500</t>
         </is>
       </c>
       <c r="D39" s="7" t="inlineStr">
         <is>
-          <t>1,800,000</t>
+          <t>2,300,000</t>
         </is>
       </c>
       <c r="E39" s="7" t="inlineStr">
         <is>
-          <t>15,300</t>
+          <t>26,450</t>
         </is>
       </c>
       <c r="F39" s="6" t="inlineStr">
         <is>
-          <t>17.71배 (EV/EBITDA)</t>
+          <t>27.60배 (PER)</t>
         </is>
       </c>
       <c r="G39" s="6" t="n">
-        <v>8500</v>
+        <v>11500</v>
       </c>
       <c r="H39" s="6" t="n">
-        <v>1334.91</v>
+        <v>1124.21</v>
       </c>
       <c r="I39" s="6" t="n">
-        <v>2263</v>
+        <v>2411</v>
       </c>
       <c r="J39" s="6" t="inlineStr">
         <is>
@@ -10408,29 +10410,29 @@
       </c>
       <c r="K39" s="6" t="inlineStr">
         <is>
-          <t>1,334.91</t>
+          <t>1,960.87</t>
         </is>
       </c>
       <c r="L39" s="6" t="inlineStr"/>
       <c r="M39" s="6" t="inlineStr">
         <is>
-          <t>2026-03-06</t>
+          <t>2026-03-09</t>
         </is>
       </c>
       <c r="N39" s="6" t="inlineStr">
         <is>
-          <t>한국</t>
+          <t>미래</t>
         </is>
       </c>
       <c r="O39" s="6" t="inlineStr"/>
       <c r="P39" s="7" t="inlineStr">
         <is>
-          <t>788</t>
+          <t>1,090</t>
         </is>
       </c>
       <c r="Q39" s="6" t="inlineStr">
         <is>
-          <t>5.00%</t>
+          <t>4.00%</t>
         </is>
       </c>
       <c r="R39" s="6" t="inlineStr">
@@ -10442,7 +10444,7 @@
     <row r="40" ht="30" customHeight="1">
       <c r="A40" s="6" t="inlineStr">
         <is>
-          <t>케이뱅크 (유가)</t>
+          <t>에스팀</t>
         </is>
       </c>
       <c r="B40" s="18" t="inlineStr">
@@ -10452,67 +10454,63 @@
       </c>
       <c r="C40" s="6" t="inlineStr">
         <is>
-          <t>8,300~9,500</t>
+          <t>7,000~8,500</t>
         </is>
       </c>
       <c r="D40" s="7" t="inlineStr">
         <is>
-          <t>60,000,000</t>
+          <t>1,800,000</t>
         </is>
       </c>
       <c r="E40" s="7" t="inlineStr">
         <is>
-          <t>498,000</t>
+          <t>15,300</t>
         </is>
       </c>
       <c r="F40" s="6" t="inlineStr">
         <is>
-          <t>1.80배 (PBR)</t>
+          <t>17.71배 (EV/EBITDA)</t>
         </is>
       </c>
       <c r="G40" s="6" t="n">
-        <v>8300</v>
+        <v>8500</v>
       </c>
       <c r="H40" s="6" t="n">
-        <v>198.53</v>
+        <v>1334.91</v>
       </c>
       <c r="I40" s="6" t="n">
-        <v>2007</v>
+        <v>2263</v>
       </c>
       <c r="J40" s="6" t="inlineStr">
         <is>
-          <t>2026-02-20~23</t>
+          <t>2026-02-23~02-24</t>
         </is>
       </c>
       <c r="K40" s="6" t="inlineStr">
         <is>
-          <t>134.59</t>
+          <t>1,334.91</t>
         </is>
       </c>
       <c r="L40" s="6" t="inlineStr"/>
       <c r="M40" s="6" t="inlineStr">
         <is>
-          <t>2026-03-05</t>
+          <t>2026-03-06</t>
         </is>
       </c>
       <c r="N40" s="6" t="inlineStr">
         <is>
-          <t>NH</t>
-        </is>
-      </c>
-      <c r="O40" s="6" t="inlineStr">
-        <is>
-          <t>삼성</t>
-        </is>
-      </c>
+          <t>한국</t>
+        </is>
+      </c>
+      <c r="O40" s="6" t="inlineStr"/>
       <c r="P40" s="7" t="inlineStr">
         <is>
-          <t>5,976</t>
+          <t>788</t>
         </is>
       </c>
       <c r="Q40" s="6" t="inlineStr">
         <is>
-          <t>1.2%</t>
+          <t>5.00%</t>
         </is>
       </c>
       <c r="R40" s="6" t="inlineStr">
@@ -10524,63 +10522,57 @@
     <row r="41" ht="30" customHeight="1">
       <c r="A41" s="6" t="inlineStr">
         <is>
-          <t>세미티에스</t>
-        </is>
-      </c>
-      <c r="B41" s="19" t="inlineStr">
-        <is>
-          <t>해당없음</t>
-        </is>
-      </c>
-      <c r="C41" s="19" t="inlineStr">
-        <is>
-          <t>해당없음</t>
-        </is>
-      </c>
-      <c r="D41" s="19" t="inlineStr">
-        <is>
-          <t>해당없음</t>
-        </is>
-      </c>
-      <c r="E41" s="19" t="inlineStr">
-        <is>
-          <t>해당없음</t>
-        </is>
-      </c>
-      <c r="F41" s="19" t="inlineStr">
-        <is>
-          <t>해당없음</t>
-        </is>
-      </c>
-      <c r="G41" s="19" t="inlineStr">
-        <is>
-          <t>해당없음</t>
-        </is>
-      </c>
-      <c r="H41" s="19" t="inlineStr">
-        <is>
-          <t>해당없음</t>
-        </is>
-      </c>
-      <c r="I41" s="19" t="inlineStr">
-        <is>
-          <t>해당없음</t>
-        </is>
-      </c>
-      <c r="J41" s="19" t="inlineStr">
-        <is>
-          <t>해당없음</t>
-        </is>
-      </c>
-      <c r="K41" s="19" t="inlineStr">
-        <is>
-          <t>해당없음</t>
+          <t>케이뱅크 (유가)</t>
+        </is>
+      </c>
+      <c r="B41" s="18" t="inlineStr">
+        <is>
+          <t>수집예정</t>
+        </is>
+      </c>
+      <c r="C41" s="6" t="inlineStr">
+        <is>
+          <t>8,300~9,500</t>
+        </is>
+      </c>
+      <c r="D41" s="7" t="inlineStr">
+        <is>
+          <t>60,000,000</t>
+        </is>
+      </c>
+      <c r="E41" s="7" t="inlineStr">
+        <is>
+          <t>498,000</t>
+        </is>
+      </c>
+      <c r="F41" s="6" t="inlineStr">
+        <is>
+          <t>1.80배 (PBR)</t>
+        </is>
+      </c>
+      <c r="G41" s="6" t="n">
+        <v>8300</v>
+      </c>
+      <c r="H41" s="6" t="n">
+        <v>198.53</v>
+      </c>
+      <c r="I41" s="6" t="n">
+        <v>2007</v>
+      </c>
+      <c r="J41" s="6" t="inlineStr">
+        <is>
+          <t>2026-02-20~23</t>
+        </is>
+      </c>
+      <c r="K41" s="6" t="inlineStr">
+        <is>
+          <t>134.59</t>
         </is>
       </c>
       <c r="L41" s="6" t="inlineStr"/>
       <c r="M41" s="6" t="inlineStr">
         <is>
-          <t>2026-02-05</t>
+          <t>2026-03-05</t>
         </is>
       </c>
       <c r="N41" s="6" t="inlineStr">
@@ -10588,77 +10580,87 @@
           <t>NH</t>
         </is>
       </c>
-      <c r="O41" s="6" t="inlineStr"/>
-      <c r="P41" s="19" t="inlineStr">
-        <is>
-          <t>해당없음</t>
-        </is>
-      </c>
-      <c r="Q41" s="19" t="inlineStr">
-        <is>
-          <t>해당없음</t>
+      <c r="O41" s="6" t="inlineStr">
+        <is>
+          <t>삼성</t>
+        </is>
+      </c>
+      <c r="P41" s="7" t="inlineStr">
+        <is>
+          <t>5,976</t>
+        </is>
+      </c>
+      <c r="Q41" s="6" t="inlineStr">
+        <is>
+          <t>1.2%</t>
         </is>
       </c>
       <c r="R41" s="6" t="inlineStr">
         <is>
-          <t>상장완료(스팩합병)</t>
+          <t>상장완료</t>
         </is>
       </c>
     </row>
     <row r="42" ht="30" customHeight="1">
       <c r="A42" s="6" t="inlineStr">
         <is>
-          <t>덕양에너젠</t>
-        </is>
-      </c>
-      <c r="B42" s="18" t="inlineStr">
-        <is>
-          <t>수집예정</t>
-        </is>
-      </c>
-      <c r="C42" s="6" t="inlineStr">
-        <is>
-          <t>8,500~10,000</t>
-        </is>
-      </c>
-      <c r="D42" s="7" t="inlineStr">
-        <is>
-          <t>7,500,000</t>
-        </is>
-      </c>
-      <c r="E42" s="7" t="inlineStr">
-        <is>
-          <t>75,000</t>
-        </is>
-      </c>
-      <c r="F42" s="6" t="inlineStr">
-        <is>
-          <t>30.32배 (EV/EBITDA)</t>
-        </is>
-      </c>
-      <c r="G42" s="6" t="n">
-        <v>10000</v>
-      </c>
-      <c r="H42" s="6" t="n">
-        <v>650.14</v>
-      </c>
-      <c r="I42" s="6" t="n">
-        <v>2324</v>
-      </c>
-      <c r="J42" s="6" t="inlineStr">
-        <is>
-          <t>2026-01-20~01-21</t>
-        </is>
-      </c>
-      <c r="K42" s="6" t="inlineStr">
-        <is>
-          <t>1,354.00</t>
+          <t>세미티에스</t>
+        </is>
+      </c>
+      <c r="B42" s="19" t="inlineStr">
+        <is>
+          <t>해당없음</t>
+        </is>
+      </c>
+      <c r="C42" s="19" t="inlineStr">
+        <is>
+          <t>해당없음</t>
+        </is>
+      </c>
+      <c r="D42" s="19" t="inlineStr">
+        <is>
+          <t>해당없음</t>
+        </is>
+      </c>
+      <c r="E42" s="19" t="inlineStr">
+        <is>
+          <t>해당없음</t>
+        </is>
+      </c>
+      <c r="F42" s="19" t="inlineStr">
+        <is>
+          <t>해당없음</t>
+        </is>
+      </c>
+      <c r="G42" s="19" t="inlineStr">
+        <is>
+          <t>해당없음</t>
+        </is>
+      </c>
+      <c r="H42" s="19" t="inlineStr">
+        <is>
+          <t>해당없음</t>
+        </is>
+      </c>
+      <c r="I42" s="19" t="inlineStr">
+        <is>
+          <t>해당없음</t>
+        </is>
+      </c>
+      <c r="J42" s="19" t="inlineStr">
+        <is>
+          <t>해당없음</t>
+        </is>
+      </c>
+      <c r="K42" s="19" t="inlineStr">
+        <is>
+          <t>해당없음</t>
         </is>
       </c>
       <c r="L42" s="6" t="inlineStr"/>
       <c r="M42" s="6" t="inlineStr">
         <is>
-          <t>2026-01-30</t>
+          <t>2026-02-05</t>
         </is>
       </c>
       <c r="N42" s="6" t="inlineStr">
@@ -10666,87 +10668,77 @@
           <t>NH</t>
         </is>
       </c>
-      <c r="O42" s="6" t="inlineStr">
-        <is>
-          <t>미래</t>
-        </is>
-      </c>
-      <c r="P42" s="7" t="inlineStr">
-        <is>
-          <t>2,000</t>
-        </is>
-      </c>
-      <c r="Q42" s="6" t="inlineStr">
-        <is>
-          <t>2.92%</t>
+      <c r="O42" s="6" t="inlineStr"/>
+      <c r="P42" s="19" t="inlineStr">
+        <is>
+          <t>해당없음</t>
+        </is>
+      </c>
+      <c r="Q42" s="19" t="inlineStr">
+        <is>
+          <t>해당없음</t>
         </is>
       </c>
       <c r="R42" s="6" t="inlineStr">
         <is>
-          <t>상장완료</t>
+          <t>상장완료(스팩합병)</t>
         </is>
       </c>
     </row>
     <row r="43" ht="30" customHeight="1">
       <c r="A43" s="6" t="inlineStr">
         <is>
-          <t>케이피항공산업</t>
-        </is>
-      </c>
-      <c r="B43" s="19" t="inlineStr">
-        <is>
-          <t>해당없음</t>
-        </is>
-      </c>
-      <c r="C43" s="19" t="inlineStr">
-        <is>
-          <t>해당없음</t>
-        </is>
-      </c>
-      <c r="D43" s="19" t="inlineStr">
-        <is>
-          <t>해당없음</t>
-        </is>
-      </c>
-      <c r="E43" s="19" t="inlineStr">
-        <is>
-          <t>해당없음</t>
-        </is>
-      </c>
-      <c r="F43" s="19" t="inlineStr">
-        <is>
-          <t>해당없음</t>
-        </is>
-      </c>
-      <c r="G43" s="19" t="inlineStr">
-        <is>
-          <t>해당없음</t>
-        </is>
-      </c>
-      <c r="H43" s="19" t="inlineStr">
-        <is>
-          <t>해당없음</t>
-        </is>
-      </c>
-      <c r="I43" s="19" t="inlineStr">
-        <is>
-          <t>해당없음</t>
-        </is>
-      </c>
-      <c r="J43" s="19" t="inlineStr">
-        <is>
-          <t>해당없음</t>
-        </is>
-      </c>
-      <c r="K43" s="19" t="inlineStr">
-        <is>
-          <t>해당없음</t>
+          <t>덕양에너젠</t>
+        </is>
+      </c>
+      <c r="B43" s="18" t="inlineStr">
+        <is>
+          <t>수집예정</t>
+        </is>
+      </c>
+      <c r="C43" s="6" t="inlineStr">
+        <is>
+          <t>8,500~10,000</t>
+        </is>
+      </c>
+      <c r="D43" s="7" t="inlineStr">
+        <is>
+          <t>7,500,000</t>
+        </is>
+      </c>
+      <c r="E43" s="7" t="inlineStr">
+        <is>
+          <t>75,000</t>
+        </is>
+      </c>
+      <c r="F43" s="6" t="inlineStr">
+        <is>
+          <t>30.32배 (EV/EBITDA)</t>
+        </is>
+      </c>
+      <c r="G43" s="6" t="n">
+        <v>10000</v>
+      </c>
+      <c r="H43" s="6" t="n">
+        <v>650.14</v>
+      </c>
+      <c r="I43" s="6" t="n">
+        <v>2324</v>
+      </c>
+      <c r="J43" s="6" t="inlineStr">
+        <is>
+          <t>2026-01-20~01-21</t>
+        </is>
+      </c>
+      <c r="K43" s="6" t="inlineStr">
+        <is>
+          <t>1,354.00</t>
         </is>
       </c>
       <c r="L43" s="6" t="inlineStr"/>
       <c r="M43" s="6" t="inlineStr">
         <is>
-          <t>2026-01-29</t>
+          <t>2026-01-30</t>
         </is>
       </c>
       <c r="N43" s="6" t="inlineStr">
@@ -10754,27 +10746,31 @@
           <t>NH</t>
         </is>
       </c>
-      <c r="O43" s="6" t="inlineStr"/>
-      <c r="P43" s="19" t="inlineStr">
-        <is>
-          <t>해당없음</t>
-        </is>
-      </c>
-      <c r="Q43" s="19" t="inlineStr">
-        <is>
-          <t>해당없음</t>
+      <c r="O43" s="6" t="inlineStr">
+        <is>
+          <t>미래</t>
+        </is>
+      </c>
+      <c r="P43" s="7" t="inlineStr">
+        <is>
+          <t>2,000</t>
+        </is>
+      </c>
+      <c r="Q43" s="6" t="inlineStr">
+        <is>
+          <t>2.92%</t>
         </is>
       </c>
       <c r="R43" s="6" t="inlineStr">
         <is>
-          <t>상장완료(스팩합병)</t>
+          <t>상장완료</t>
         </is>
       </c>
     </row>
     <row r="44" ht="30" customHeight="1">
       <c r="A44" s="6" t="inlineStr">
         <is>
-          <t>삼성스팩13호</t>
+          <t>케이피항공산업</t>
         </is>
       </c>
       <c r="B44" s="19" t="inlineStr">
@@ -10782,19 +10778,19 @@
           <t>해당없음</t>
         </is>
       </c>
-      <c r="C44" s="6" t="inlineStr">
-        <is>
-          <t>2,000</t>
-        </is>
-      </c>
-      <c r="D44" s="7" t="inlineStr">
-        <is>
-          <t>6,000,000</t>
-        </is>
-      </c>
-      <c r="E44" s="7" t="inlineStr">
-        <is>
-          <t>12,000</t>
+      <c r="C44" s="19" t="inlineStr">
+        <is>
+          <t>해당없음</t>
+        </is>
+      </c>
+      <c r="D44" s="19" t="inlineStr">
+        <is>
+          <t>해당없음</t>
+        </is>
+      </c>
+      <c r="E44" s="19" t="inlineStr">
+        <is>
+          <t>해당없음</t>
         </is>
       </c>
       <c r="F44" s="19" t="inlineStr">
@@ -10802,154 +10798,162 @@
           <t>해당없음</t>
         </is>
       </c>
-      <c r="G44" s="6" t="inlineStr">
-        <is>
-          <t>2,000</t>
-        </is>
-      </c>
-      <c r="H44" s="6" t="n">
-        <v>1159.11</v>
-      </c>
-      <c r="I44" s="6" t="n">
-        <v>1892</v>
-      </c>
-      <c r="J44" s="6" t="inlineStr">
-        <is>
-          <t>2026-01-12~01-13</t>
-        </is>
-      </c>
-      <c r="K44" s="6" t="inlineStr">
-        <is>
-          <t>1,870.40</t>
+      <c r="G44" s="19" t="inlineStr">
+        <is>
+          <t>해당없음</t>
+        </is>
+      </c>
+      <c r="H44" s="19" t="inlineStr">
+        <is>
+          <t>해당없음</t>
+        </is>
+      </c>
+      <c r="I44" s="19" t="inlineStr">
+        <is>
+          <t>해당없음</t>
+        </is>
+      </c>
+      <c r="J44" s="19" t="inlineStr">
+        <is>
+          <t>해당없음</t>
+        </is>
+      </c>
+      <c r="K44" s="19" t="inlineStr">
+        <is>
+          <t>해당없음</t>
         </is>
       </c>
       <c r="L44" s="6" t="inlineStr"/>
       <c r="M44" s="6" t="inlineStr">
         <is>
+          <t>2026-01-29</t>
+        </is>
+      </c>
+      <c r="N44" s="6" t="inlineStr">
+        <is>
+          <t>NH</t>
+        </is>
+      </c>
+      <c r="O44" s="6" t="inlineStr"/>
+      <c r="P44" s="19" t="inlineStr">
+        <is>
+          <t>해당없음</t>
+        </is>
+      </c>
+      <c r="Q44" s="19" t="inlineStr">
+        <is>
+          <t>해당없음</t>
+        </is>
+      </c>
+      <c r="R44" s="6" t="inlineStr">
+        <is>
+          <t>상장완료(스팩합병)</t>
+        </is>
+      </c>
+    </row>
+    <row r="45" ht="30" customHeight="1">
+      <c r="A45" s="6" t="inlineStr">
+        <is>
+          <t>삼성스팩13호</t>
+        </is>
+      </c>
+      <c r="B45" s="19" t="inlineStr">
+        <is>
+          <t>해당없음</t>
+        </is>
+      </c>
+      <c r="C45" s="6" t="inlineStr">
+        <is>
+          <t>2,000</t>
+        </is>
+      </c>
+      <c r="D45" s="7" t="inlineStr">
+        <is>
+          <t>6,000,000</t>
+        </is>
+      </c>
+      <c r="E45" s="7" t="inlineStr">
+        <is>
+          <t>12,000</t>
+        </is>
+      </c>
+      <c r="F45" s="19" t="inlineStr">
+        <is>
+          <t>해당없음</t>
+        </is>
+      </c>
+      <c r="G45" s="6" t="inlineStr">
+        <is>
+          <t>2,000</t>
+        </is>
+      </c>
+      <c r="H45" s="6" t="n">
+        <v>1159.11</v>
+      </c>
+      <c r="I45" s="6" t="n">
+        <v>1892</v>
+      </c>
+      <c r="J45" s="6" t="inlineStr">
+        <is>
+          <t>2026-01-12~01-13</t>
+        </is>
+      </c>
+      <c r="K45" s="6" t="inlineStr">
+        <is>
+          <t>1,870.40</t>
+        </is>
+      </c>
+      <c r="L45" s="6" t="inlineStr"/>
+      <c r="M45" s="6" t="inlineStr">
+        <is>
           <t>2026-01-21</t>
         </is>
       </c>
-      <c r="N44" s="6" t="inlineStr">
+      <c r="N45" s="6" t="inlineStr">
         <is>
           <t>삼성</t>
         </is>
       </c>
-      <c r="O44" s="6" t="inlineStr"/>
-      <c r="P44" s="7" t="inlineStr">
+      <c r="O45" s="6" t="inlineStr"/>
+      <c r="P45" s="7" t="inlineStr">
         <is>
           <t>360</t>
         </is>
       </c>
-      <c r="Q44" s="6" t="inlineStr">
+      <c r="Q45" s="6" t="inlineStr">
         <is>
           <t>3.00%</t>
         </is>
       </c>
-      <c r="R44" s="6" t="inlineStr">
+      <c r="R45" s="6" t="inlineStr">
         <is>
           <t>상장완료</t>
         </is>
       </c>
     </row>
-    <row r="46" ht="22" customHeight="1">
-      <c r="A46" s="3" t="inlineStr">
-        <is>
-          <t>■ 공모 진행 (예심 승인법인)  (27건)</t>
-        </is>
-      </c>
-      <c r="B46" s="4" t="n"/>
-      <c r="C46" s="4" t="n"/>
-      <c r="D46" s="4" t="n"/>
-      <c r="E46" s="4" t="n"/>
-      <c r="F46" s="4" t="n"/>
-      <c r="G46" s="4" t="n"/>
-      <c r="H46" s="4" t="n"/>
-      <c r="I46" s="4" t="n"/>
-      <c r="J46" s="4" t="n"/>
-      <c r="K46" s="4" t="n"/>
-      <c r="L46" s="4" t="n"/>
-      <c r="M46" s="4" t="n"/>
-      <c r="N46" s="4" t="n"/>
-      <c r="O46" s="4" t="n"/>
-      <c r="P46" s="4" t="n"/>
-      <c r="Q46" s="4" t="n"/>
-      <c r="R46" s="4" t="n"/>
-    </row>
-    <row r="47" ht="30" customHeight="1">
-      <c r="A47" s="6" t="inlineStr">
-        <is>
-          <t>스카이랩스</t>
-        </is>
-      </c>
-      <c r="B47" s="6" t="inlineStr">
-        <is>
-          <t>08-14~08-21</t>
-        </is>
-      </c>
-      <c r="C47" s="6" t="inlineStr">
-        <is>
-          <t>13,000~16,000</t>
-        </is>
-      </c>
-      <c r="D47" s="7" t="inlineStr">
-        <is>
-          <t>2,000,000</t>
-        </is>
-      </c>
-      <c r="E47" s="7" t="inlineStr">
-        <is>
-          <t>20,000,000,000</t>
-        </is>
-      </c>
-      <c r="F47" s="6" t="inlineStr">
-        <is>
-          <t>29.52배 (PER)</t>
-        </is>
-      </c>
-      <c r="G47" s="6" t="inlineStr">
-        <is>
-          <t>10,000</t>
-        </is>
-      </c>
-      <c r="H47" s="6" t="n">
-        <v>63.41</v>
-      </c>
-      <c r="I47" s="6" t="n">
-        <v>246</v>
-      </c>
-      <c r="J47" s="6" t="inlineStr">
-        <is>
-          <t>08-26~08-27</t>
-        </is>
-      </c>
-      <c r="K47" s="6" t="inlineStr">
-        <is>
-          <t>88.20</t>
-        </is>
-      </c>
-      <c r="L47" s="6" t="inlineStr"/>
-      <c r="M47" s="6" t="inlineStr"/>
-      <c r="N47" s="6" t="inlineStr">
-        <is>
-          <t>한국투자증권</t>
-        </is>
-      </c>
-      <c r="O47" s="6" t="inlineStr"/>
-      <c r="P47" s="7" t="inlineStr">
-        <is>
-          <t>1,071,200,000</t>
-        </is>
-      </c>
-      <c r="Q47" s="18" t="inlineStr">
-        <is>
-          <t>수집예정</t>
-        </is>
-      </c>
-      <c r="R47" s="6" t="inlineStr">
-        <is>
-          <t>청약완료·상장대기</t>
-        </is>
-      </c>
+    <row r="47" ht="22" customHeight="1">
+      <c r="A47" s="3" t="inlineStr">
+        <is>
+          <t>■ 공모 진행 (예심 승인법인)  (26건)</t>
+        </is>
+      </c>
+      <c r="B47" s="4" t="n"/>
+      <c r="C47" s="4" t="n"/>
+      <c r="D47" s="4" t="n"/>
+      <c r="E47" s="4" t="n"/>
+      <c r="F47" s="4" t="n"/>
+      <c r="G47" s="4" t="n"/>
+      <c r="H47" s="4" t="n"/>
+      <c r="I47" s="4" t="n"/>
+      <c r="J47" s="4" t="n"/>
+      <c r="K47" s="4" t="n"/>
+      <c r="L47" s="4" t="n"/>
+      <c r="M47" s="4" t="n"/>
+      <c r="N47" s="4" t="n"/>
+      <c r="O47" s="4" t="n"/>
+      <c r="P47" s="4" t="n"/>
+      <c r="Q47" s="4" t="n"/>
+      <c r="R47" s="4" t="n"/>
     </row>
     <row r="48" ht="30" customHeight="1">
       <c r="A48" s="6" t="inlineStr">
@@ -10998,7 +11002,11 @@
           <t>09-01~09-02</t>
         </is>
       </c>
-      <c r="K48" s="6" t="inlineStr"/>
+      <c r="K48" s="6" t="inlineStr">
+        <is>
+          <t>16,216.08</t>
+        </is>
+      </c>
       <c r="L48" s="6" t="inlineStr"/>
       <c r="M48" s="6" t="inlineStr"/>
       <c r="N48" s="18" t="inlineStr">
@@ -11019,7 +11027,7 @@
       </c>
       <c r="R48" s="6" t="inlineStr">
         <is>
-          <t>발행조건확정</t>
+          <t>청약완료·상장대기</t>
         </is>
       </c>
     </row>
@@ -11547,7 +11555,7 @@
       </c>
       <c r="B57" s="6" t="inlineStr">
         <is>
-          <t>09-09~09-15</t>
+          <t>09-23~10-01</t>
         </is>
       </c>
       <c r="C57" s="6" t="inlineStr">
@@ -11575,7 +11583,7 @@
       <c r="I57" s="6" t="inlineStr"/>
       <c r="J57" s="6" t="inlineStr">
         <is>
-          <t>09-18~09-21</t>
+          <t>10-07~10-08</t>
         </is>
       </c>
       <c r="K57" s="6" t="inlineStr"/>
@@ -11603,7 +11611,7 @@
       </c>
       <c r="R57" s="6" t="inlineStr">
         <is>
-          <t>최초</t>
+          <t>정정</t>
         </is>
       </c>
     </row>
@@ -11994,71 +12002,71 @@
     <row r="64" ht="30" customHeight="1">
       <c r="A64" s="6" t="inlineStr">
         <is>
-          <t>엠에스바이오</t>
-        </is>
-      </c>
-      <c r="B64" s="18" t="inlineStr">
-        <is>
-          <t>수집예정</t>
-        </is>
-      </c>
-      <c r="C64" s="18" t="inlineStr">
-        <is>
-          <t>수집예정</t>
-        </is>
-      </c>
-      <c r="D64" s="18" t="inlineStr">
-        <is>
-          <t>수집예정</t>
-        </is>
-      </c>
-      <c r="E64" s="18" t="inlineStr">
-        <is>
-          <t>수집예정</t>
-        </is>
-      </c>
-      <c r="F64" s="18" t="inlineStr">
-        <is>
-          <t>수집예정</t>
+          <t>크리에이츠</t>
+        </is>
+      </c>
+      <c r="B64" s="6" t="inlineStr">
+        <is>
+          <t>10-12~10-16</t>
+        </is>
+      </c>
+      <c r="C64" s="6" t="inlineStr">
+        <is>
+          <t>15,000~18,000</t>
+        </is>
+      </c>
+      <c r="D64" s="7" t="inlineStr">
+        <is>
+          <t>1,400,000</t>
+        </is>
+      </c>
+      <c r="E64" s="7" t="inlineStr">
+        <is>
+          <t>21,000,000,000</t>
+        </is>
+      </c>
+      <c r="F64" s="6" t="inlineStr">
+        <is>
+          <t>19.15배 (PER)</t>
         </is>
       </c>
       <c r="G64" s="6" t="inlineStr"/>
       <c r="H64" s="6" t="inlineStr"/>
       <c r="I64" s="6" t="inlineStr"/>
-      <c r="J64" s="18" t="inlineStr">
-        <is>
-          <t>수집예정</t>
+      <c r="J64" s="6" t="inlineStr">
+        <is>
+          <t>10-20~10-21</t>
         </is>
       </c>
       <c r="K64" s="6" t="inlineStr"/>
       <c r="L64" s="6" t="inlineStr"/>
       <c r="M64" s="6" t="inlineStr"/>
-      <c r="N64" s="18" t="inlineStr">
-        <is>
-          <t>수집예정</t>
+      <c r="N64" s="6" t="inlineStr">
+        <is>
+          <t>삼성증권</t>
         </is>
       </c>
       <c r="O64" s="6" t="inlineStr"/>
-      <c r="P64" s="18" t="inlineStr">
-        <is>
-          <t>수집예정</t>
-        </is>
-      </c>
-      <c r="Q64" s="18" t="inlineStr">
-        <is>
-          <t>수집예정</t>
+      <c r="P64" s="7" t="inlineStr">
+        <is>
+          <t>865,200,000</t>
+        </is>
+      </c>
+      <c r="Q64" s="6" t="inlineStr">
+        <is>
+          <t>4.0%</t>
         </is>
       </c>
       <c r="R64" s="6" t="inlineStr">
         <is>
-          <t>신고서 대기</t>
+          <t>최초</t>
         </is>
       </c>
     </row>
     <row r="65" ht="30" customHeight="1">
       <c r="A65" s="6" t="inlineStr">
         <is>
-          <t>디티에스</t>
+          <t>엠에스바이오</t>
         </is>
       </c>
       <c r="B65" s="18" t="inlineStr">
@@ -12122,7 +12130,7 @@
     <row r="66" ht="30" customHeight="1">
       <c r="A66" s="6" t="inlineStr">
         <is>
-          <t>한화플러스제6호스팩</t>
+          <t>디티에스</t>
         </is>
       </c>
       <c r="B66" s="18" t="inlineStr">
@@ -12186,7 +12194,7 @@
     <row r="67" ht="30" customHeight="1">
       <c r="A67" s="6" t="inlineStr">
         <is>
-          <t>바로팜</t>
+          <t>한화플러스제6호스팩</t>
         </is>
       </c>
       <c r="B67" s="18" t="inlineStr">
@@ -12250,7 +12258,7 @@
     <row r="68" ht="30" customHeight="1">
       <c r="A68" s="6" t="inlineStr">
         <is>
-          <t>크리에이츠</t>
+          <t>바로팜</t>
         </is>
       </c>
       <c r="B68" s="18" t="inlineStr">
@@ -12932,7 +12940,7 @@
         <v>0</v>
       </c>
       <c r="E14" s="6" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F14" s="21">
         <f>IF((C14+D14)=0,"-",C14/(C14+D14))</f>
@@ -12999,11 +13007,11 @@
         </is>
       </c>
       <c r="B19" s="6" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="C19" s="6" t="inlineStr">
         <is>
-          <t>194,984,000,000</t>
+          <t>215,984,000,000</t>
         </is>
       </c>
     </row>
@@ -13040,22 +13048,22 @@
     <row r="22">
       <c r="A22" s="6" t="inlineStr">
         <is>
-          <t>대신증권</t>
+          <t>한국투자증권</t>
         </is>
       </c>
       <c r="B22" s="6" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="C22" s="6" t="inlineStr">
         <is>
-          <t>107,550,000,000</t>
+          <t>122,800,000,000</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="6" t="inlineStr">
         <is>
-          <t>한국투자증권</t>
+          <t>대신증권</t>
         </is>
       </c>
       <c r="B23" s="6" t="n">
@@ -13063,7 +13071,7 @@
       </c>
       <c r="C23" s="6" t="inlineStr">
         <is>
-          <t>102,800,000,000</t>
+          <t>107,550,000,000</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore: update IPO data 2026-09-09
</commit_message>
<xml_diff>
--- a/IPO_analysis.xlsx
+++ b/IPO_analysis.xlsx
@@ -618,7 +618,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>기준일 2026-09-08 · 청구일 직전 사업연도 · 별도/개별 재무제표 · 단위 백만원(별도 표기 시 USD)</t>
+          <t>기준일 2026-09-09 · 청구일 직전 사업연도 · 별도/개별 재무제표 · 단위 백만원(별도 표기 시 USD)</t>
         </is>
       </c>
     </row>
@@ -11148,44 +11148,44 @@
     <row r="49" ht="30" customHeight="1">
       <c r="A49" s="6" t="inlineStr">
         <is>
-          <t>케이비제34호스팩</t>
+          <t>네오사피엔스</t>
         </is>
       </c>
       <c r="B49" s="6" t="inlineStr">
         <is>
-          <t>09-04~09-07</t>
-        </is>
-      </c>
-      <c r="C49" s="18" t="inlineStr">
-        <is>
-          <t>수집예정</t>
+          <t>09-02~09-08</t>
+        </is>
+      </c>
+      <c r="C49" s="6" t="inlineStr">
+        <is>
+          <t>13,800~15,800</t>
         </is>
       </c>
       <c r="D49" s="7" t="inlineStr">
         <is>
-          <t>7,000,000</t>
+          <t>2,000,000</t>
         </is>
       </c>
       <c r="E49" s="7" t="inlineStr">
         <is>
-          <t>14,000,000,000</t>
-        </is>
-      </c>
-      <c r="F49" s="18" t="inlineStr">
-        <is>
-          <t>수집예정</t>
+          <t>27,600,000,000</t>
+        </is>
+      </c>
+      <c r="F49" s="6" t="inlineStr">
+        <is>
+          <t>26.76배 (PER)</t>
         </is>
       </c>
       <c r="G49" s="6" t="inlineStr">
         <is>
-          <t>2,000</t>
+          <t>13,800</t>
         </is>
       </c>
       <c r="H49" s="6" t="n">
-        <v>1232.51</v>
+        <v>219.56</v>
       </c>
       <c r="I49" s="6" t="n">
-        <v>2001</v>
+        <v>1045</v>
       </c>
       <c r="J49" s="6" t="inlineStr">
         <is>
@@ -11195,20 +11195,20 @@
       <c r="K49" s="6" t="inlineStr"/>
       <c r="L49" s="6" t="inlineStr"/>
       <c r="M49" s="6" t="inlineStr"/>
-      <c r="N49" s="18" t="inlineStr">
-        <is>
-          <t>수집예정</t>
+      <c r="N49" s="6" t="inlineStr">
+        <is>
+          <t>대신증권</t>
         </is>
       </c>
       <c r="O49" s="6" t="inlineStr"/>
-      <c r="P49" s="18" t="inlineStr">
-        <is>
-          <t>수집예정</t>
+      <c r="P49" s="7" t="inlineStr">
+        <is>
+          <t>1,080,264,000</t>
         </is>
       </c>
       <c r="Q49" s="6" t="inlineStr">
         <is>
-          <t>50%</t>
+          <t>3.8%</t>
         </is>
       </c>
       <c r="R49" s="6" t="inlineStr">
@@ -11220,101 +11220,117 @@
     <row r="50" ht="30" customHeight="1">
       <c r="A50" s="6" t="inlineStr">
         <is>
-          <t>브릴스</t>
+          <t>케이비제34호스팩</t>
         </is>
       </c>
       <c r="B50" s="6" t="inlineStr">
         <is>
-          <t>08-31~09-04</t>
-        </is>
-      </c>
-      <c r="C50" s="6" t="inlineStr">
-        <is>
-          <t>16,500~19,500</t>
+          <t>09-04~09-07</t>
+        </is>
+      </c>
+      <c r="C50" s="18" t="inlineStr">
+        <is>
+          <t>수집예정</t>
         </is>
       </c>
       <c r="D50" s="7" t="inlineStr">
         <is>
-          <t>1,200,000</t>
+          <t>7,000,000</t>
         </is>
       </c>
       <c r="E50" s="7" t="inlineStr">
         <is>
-          <t>19,800,000,000</t>
-        </is>
-      </c>
-      <c r="F50" s="6" t="inlineStr">
-        <is>
-          <t>13.44 (PSR)</t>
-        </is>
-      </c>
-      <c r="G50" s="6" t="inlineStr"/>
-      <c r="H50" s="6" t="inlineStr"/>
-      <c r="I50" s="6" t="inlineStr"/>
+          <t>14,000,000,000</t>
+        </is>
+      </c>
+      <c r="F50" s="18" t="inlineStr">
+        <is>
+          <t>수집예정</t>
+        </is>
+      </c>
+      <c r="G50" s="6" t="inlineStr">
+        <is>
+          <t>2,000</t>
+        </is>
+      </c>
+      <c r="H50" s="6" t="n">
+        <v>1232.51</v>
+      </c>
+      <c r="I50" s="6" t="n">
+        <v>2001</v>
+      </c>
       <c r="J50" s="6" t="inlineStr">
         <is>
-          <t>09-08~09-09</t>
+          <t>09-10~09-11</t>
         </is>
       </c>
       <c r="K50" s="6" t="inlineStr"/>
       <c r="L50" s="6" t="inlineStr"/>
       <c r="M50" s="6" t="inlineStr"/>
-      <c r="N50" s="6" t="inlineStr">
-        <is>
-          <t>아이비케이투자증권</t>
+      <c r="N50" s="18" t="inlineStr">
+        <is>
+          <t>수집예정</t>
         </is>
       </c>
       <c r="O50" s="6" t="inlineStr"/>
-      <c r="P50" s="7" t="inlineStr">
-        <is>
-          <t>713,790,000</t>
+      <c r="P50" s="18" t="inlineStr">
+        <is>
+          <t>수집예정</t>
         </is>
       </c>
       <c r="Q50" s="6" t="inlineStr">
         <is>
-          <t>3.5%</t>
+          <t>50%</t>
         </is>
       </c>
       <c r="R50" s="6" t="inlineStr">
         <is>
-          <t>정정</t>
+          <t>발행조건확정</t>
         </is>
       </c>
     </row>
     <row r="51" ht="30" customHeight="1">
       <c r="A51" s="6" t="inlineStr">
         <is>
-          <t>네오사피엔스</t>
+          <t>한국제17호스팩</t>
         </is>
       </c>
       <c r="B51" s="6" t="inlineStr">
         <is>
-          <t>09-02~09-08</t>
-        </is>
-      </c>
-      <c r="C51" s="6" t="inlineStr">
-        <is>
-          <t>13,800~15,800</t>
+          <t>09-07~09-08</t>
+        </is>
+      </c>
+      <c r="C51" s="18" t="inlineStr">
+        <is>
+          <t>수집예정</t>
         </is>
       </c>
       <c r="D51" s="7" t="inlineStr">
         <is>
-          <t>2,000,000</t>
+          <t>7,000,000</t>
         </is>
       </c>
       <c r="E51" s="7" t="inlineStr">
         <is>
-          <t>27,600,000,000</t>
-        </is>
-      </c>
-      <c r="F51" s="6" t="inlineStr">
-        <is>
-          <t>26.76배 (PER)</t>
-        </is>
-      </c>
-      <c r="G51" s="6" t="inlineStr"/>
-      <c r="H51" s="6" t="inlineStr"/>
-      <c r="I51" s="6" t="inlineStr"/>
+          <t>14,000,000,000</t>
+        </is>
+      </c>
+      <c r="F51" s="18" t="inlineStr">
+        <is>
+          <t>수집예정</t>
+        </is>
+      </c>
+      <c r="G51" s="6" t="inlineStr">
+        <is>
+          <t>2,000</t>
+        </is>
+      </c>
+      <c r="H51" s="6" t="n">
+        <v>1270.51</v>
+      </c>
+      <c r="I51" s="6" t="n">
+        <v>2040</v>
+      </c>
       <c r="J51" s="6" t="inlineStr">
         <is>
           <t>09-10~09-11</t>
@@ -11323,57 +11339,57 @@
       <c r="K51" s="6" t="inlineStr"/>
       <c r="L51" s="6" t="inlineStr"/>
       <c r="M51" s="6" t="inlineStr"/>
-      <c r="N51" s="6" t="inlineStr">
-        <is>
-          <t>대신증권</t>
+      <c r="N51" s="18" t="inlineStr">
+        <is>
+          <t>수집예정</t>
         </is>
       </c>
       <c r="O51" s="6" t="inlineStr"/>
-      <c r="P51" s="7" t="inlineStr">
-        <is>
-          <t>1,080,264,000</t>
+      <c r="P51" s="18" t="inlineStr">
+        <is>
+          <t>수집예정</t>
         </is>
       </c>
       <c r="Q51" s="6" t="inlineStr">
         <is>
-          <t>3.8%</t>
+          <t>50%</t>
         </is>
       </c>
       <c r="R51" s="6" t="inlineStr">
         <is>
-          <t>정정</t>
+          <t>발행조건확정</t>
         </is>
       </c>
     </row>
     <row r="52" ht="30" customHeight="1">
       <c r="A52" s="6" t="inlineStr">
         <is>
-          <t>와이즈플래닛컴퍼니</t>
+          <t>브릴스</t>
         </is>
       </c>
       <c r="B52" s="6" t="inlineStr">
         <is>
-          <t>09-04~09-10</t>
+          <t>08-31~09-04</t>
         </is>
       </c>
       <c r="C52" s="6" t="inlineStr">
         <is>
-          <t>10,000~12,000</t>
+          <t>16,500~19,500</t>
         </is>
       </c>
       <c r="D52" s="7" t="inlineStr">
         <is>
-          <t>1,600,000</t>
+          <t>1,200,000</t>
         </is>
       </c>
       <c r="E52" s="7" t="inlineStr">
         <is>
-          <t>16,000,000,000</t>
+          <t>19,800,000,000</t>
         </is>
       </c>
       <c r="F52" s="6" t="inlineStr">
         <is>
-          <t>20.04배 (PER)</t>
+          <t>13.44 (PSR)</t>
         </is>
       </c>
       <c r="G52" s="6" t="inlineStr"/>
@@ -11381,7 +11397,7 @@
       <c r="I52" s="6" t="inlineStr"/>
       <c r="J52" s="6" t="inlineStr">
         <is>
-          <t>09-14~09-15</t>
+          <t>09-08~09-09</t>
         </is>
       </c>
       <c r="K52" s="6" t="inlineStr"/>
@@ -11389,18 +11405,18 @@
       <c r="M52" s="6" t="inlineStr"/>
       <c r="N52" s="6" t="inlineStr">
         <is>
-          <t>대신증권</t>
+          <t>아이비케이투자증권</t>
         </is>
       </c>
       <c r="O52" s="6" t="inlineStr"/>
       <c r="P52" s="7" t="inlineStr">
         <is>
-          <t>494,400,000</t>
+          <t>713,790,000</t>
         </is>
       </c>
       <c r="Q52" s="6" t="inlineStr">
         <is>
-          <t>3.0%</t>
+          <t>3.5%</t>
         </is>
       </c>
       <c r="R52" s="6" t="inlineStr">
@@ -11412,32 +11428,32 @@
     <row r="53" ht="30" customHeight="1">
       <c r="A53" s="6" t="inlineStr">
         <is>
-          <t>한국제17호스팩</t>
+          <t>와이즈플래닛컴퍼니</t>
         </is>
       </c>
       <c r="B53" s="6" t="inlineStr">
         <is>
-          <t>09-07~09-08</t>
-        </is>
-      </c>
-      <c r="C53" s="18" t="inlineStr">
-        <is>
-          <t>수집예정</t>
+          <t>09-04~09-10</t>
+        </is>
+      </c>
+      <c r="C53" s="6" t="inlineStr">
+        <is>
+          <t>10,000~12,000</t>
         </is>
       </c>
       <c r="D53" s="7" t="inlineStr">
         <is>
-          <t>7,000,000</t>
+          <t>1,600,000</t>
         </is>
       </c>
       <c r="E53" s="7" t="inlineStr">
         <is>
-          <t>14,000,000,000</t>
-        </is>
-      </c>
-      <c r="F53" s="18" t="inlineStr">
-        <is>
-          <t>수집예정</t>
+          <t>16,000,000,000</t>
+        </is>
+      </c>
+      <c r="F53" s="6" t="inlineStr">
+        <is>
+          <t>20.04배 (PER)</t>
         </is>
       </c>
       <c r="G53" s="6" t="inlineStr"/>
@@ -11445,21 +11461,21 @@
       <c r="I53" s="6" t="inlineStr"/>
       <c r="J53" s="6" t="inlineStr">
         <is>
-          <t>09-10~09-11</t>
+          <t>09-14~09-15</t>
         </is>
       </c>
       <c r="K53" s="6" t="inlineStr"/>
       <c r="L53" s="6" t="inlineStr"/>
       <c r="M53" s="6" t="inlineStr"/>
-      <c r="N53" s="18" t="inlineStr">
-        <is>
-          <t>수집예정</t>
+      <c r="N53" s="6" t="inlineStr">
+        <is>
+          <t>대신증권</t>
         </is>
       </c>
       <c r="O53" s="6" t="inlineStr"/>
-      <c r="P53" s="18" t="inlineStr">
-        <is>
-          <t>수집예정</t>
+      <c r="P53" s="7" t="inlineStr">
+        <is>
+          <t>494,400,000</t>
         </is>
       </c>
       <c r="Q53" s="6" t="inlineStr">
@@ -11672,32 +11688,32 @@
     <row r="57" ht="30" customHeight="1">
       <c r="A57" s="6" t="inlineStr">
         <is>
-          <t>엘리스그룹</t>
+          <t>멜콘</t>
         </is>
       </c>
       <c r="B57" s="6" t="inlineStr">
         <is>
-          <t>09-23~10-01</t>
+          <t>09-16~09-22</t>
         </is>
       </c>
       <c r="C57" s="6" t="inlineStr">
         <is>
-          <t>70,400~90,500</t>
+          <t>10,700~12,300</t>
         </is>
       </c>
       <c r="D57" s="7" t="inlineStr">
         <is>
-          <t>2,222,000</t>
+          <t>2,500,000</t>
         </is>
       </c>
       <c r="E57" s="7" t="inlineStr">
         <is>
-          <t>156,428,800,000</t>
+          <t>26,750,000,000</t>
         </is>
       </c>
       <c r="F57" s="6" t="inlineStr">
         <is>
-          <t>27.13배 (EV/EBITDA)</t>
+          <t>26.18배 (PER)</t>
         </is>
       </c>
       <c r="G57" s="6" t="inlineStr"/>
@@ -11705,7 +11721,7 @@
       <c r="I57" s="6" t="inlineStr"/>
       <c r="J57" s="6" t="inlineStr">
         <is>
-          <t>10-07~10-08</t>
+          <t>10-01~10-02</t>
         </is>
       </c>
       <c r="K57" s="6" t="inlineStr"/>
@@ -11713,22 +11729,18 @@
       <c r="M57" s="6" t="inlineStr"/>
       <c r="N57" s="6" t="inlineStr">
         <is>
-          <t>미래에셋증권㈜</t>
-        </is>
-      </c>
-      <c r="O57" s="6" t="inlineStr">
-        <is>
-          <t>삼성</t>
-        </is>
-      </c>
+          <t>대신증권</t>
+        </is>
+      </c>
+      <c r="O57" s="6" t="inlineStr"/>
       <c r="P57" s="7" t="inlineStr">
         <is>
-          <t>1,889,144,928</t>
+          <t>826,575,000</t>
         </is>
       </c>
       <c r="Q57" s="6" t="inlineStr">
         <is>
-          <t>1.5%</t>
+          <t>3.0%</t>
         </is>
       </c>
       <c r="R57" s="6" t="inlineStr">
@@ -11740,32 +11752,32 @@
     <row r="58" ht="30" customHeight="1">
       <c r="A58" s="6" t="inlineStr">
         <is>
-          <t>래블업</t>
+          <t>엘리스그룹</t>
         </is>
       </c>
       <c r="B58" s="6" t="inlineStr">
         <is>
-          <t>09-28~10-02</t>
+          <t>09-23~10-01</t>
         </is>
       </c>
       <c r="C58" s="6" t="inlineStr">
         <is>
-          <t>20,000~23,000</t>
+          <t>70,400~90,500</t>
         </is>
       </c>
       <c r="D58" s="7" t="inlineStr">
         <is>
-          <t>2,180,000</t>
+          <t>2,222,000</t>
         </is>
       </c>
       <c r="E58" s="7" t="inlineStr">
         <is>
-          <t>43,600,000,000</t>
+          <t>156,428,800,000</t>
         </is>
       </c>
       <c r="F58" s="6" t="inlineStr">
         <is>
-          <t>33.6배 (PER)</t>
+          <t>27.13배 (EV/EBITDA)</t>
         </is>
       </c>
       <c r="G58" s="6" t="inlineStr"/>
@@ -11773,7 +11785,7 @@
       <c r="I58" s="6" t="inlineStr"/>
       <c r="J58" s="6" t="inlineStr">
         <is>
-          <t>10-12~10-13</t>
+          <t>10-07~10-08</t>
         </is>
       </c>
       <c r="K58" s="6" t="inlineStr"/>
@@ -11781,18 +11793,22 @@
       <c r="M58" s="6" t="inlineStr"/>
       <c r="N58" s="6" t="inlineStr">
         <is>
-          <t>NH투자증권</t>
-        </is>
-      </c>
-      <c r="O58" s="6" t="inlineStr"/>
+          <t>미래에셋증권㈜</t>
+        </is>
+      </c>
+      <c r="O58" s="6" t="inlineStr">
+        <is>
+          <t>삼성</t>
+        </is>
+      </c>
       <c r="P58" s="7" t="inlineStr">
         <is>
-          <t>2,007,000,000</t>
+          <t>1,889,144,928</t>
         </is>
       </c>
       <c r="Q58" s="6" t="inlineStr">
         <is>
-          <t>4.5%</t>
+          <t>1.5%</t>
         </is>
       </c>
       <c r="R58" s="6" t="inlineStr">
@@ -11804,32 +11820,32 @@
     <row r="59" ht="30" customHeight="1">
       <c r="A59" s="6" t="inlineStr">
         <is>
-          <t>멜콘</t>
+          <t>래블업</t>
         </is>
       </c>
       <c r="B59" s="6" t="inlineStr">
         <is>
-          <t>09-16~09-22</t>
+          <t>09-28~10-02</t>
         </is>
       </c>
       <c r="C59" s="6" t="inlineStr">
         <is>
-          <t>10,700~12,300</t>
+          <t>20,000~23,000</t>
         </is>
       </c>
       <c r="D59" s="7" t="inlineStr">
         <is>
-          <t>2,500,000</t>
+          <t>2,180,000</t>
         </is>
       </c>
       <c r="E59" s="7" t="inlineStr">
         <is>
-          <t>26,750,000,000</t>
+          <t>43,600,000,000</t>
         </is>
       </c>
       <c r="F59" s="6" t="inlineStr">
         <is>
-          <t>26.18배 (PER)</t>
+          <t>33.6배 (PER)</t>
         </is>
       </c>
       <c r="G59" s="6" t="inlineStr"/>
@@ -11837,7 +11853,7 @@
       <c r="I59" s="6" t="inlineStr"/>
       <c r="J59" s="6" t="inlineStr">
         <is>
-          <t>10-01~10-02</t>
+          <t>10-12~10-13</t>
         </is>
       </c>
       <c r="K59" s="6" t="inlineStr"/>
@@ -11845,55 +11861,55 @@
       <c r="M59" s="6" t="inlineStr"/>
       <c r="N59" s="6" t="inlineStr">
         <is>
-          <t>대신증권</t>
+          <t>NH투자증권</t>
         </is>
       </c>
       <c r="O59" s="6" t="inlineStr"/>
       <c r="P59" s="7" t="inlineStr">
         <is>
-          <t>826,575,000</t>
+          <t>2,007,000,000</t>
         </is>
       </c>
       <c r="Q59" s="6" t="inlineStr">
         <is>
-          <t>3.0%</t>
+          <t>4.5%</t>
         </is>
       </c>
       <c r="R59" s="6" t="inlineStr">
         <is>
-          <t>최초</t>
+          <t>정정</t>
         </is>
       </c>
     </row>
     <row r="60" ht="30" customHeight="1">
       <c r="A60" s="6" t="inlineStr">
         <is>
-          <t>진코스텍</t>
+          <t>에스케이증권제14호기업인수목적</t>
         </is>
       </c>
       <c r="B60" s="6" t="inlineStr">
         <is>
-          <t>09-16~09-22</t>
-        </is>
-      </c>
-      <c r="C60" s="6" t="inlineStr">
-        <is>
-          <t>19,500~23,500</t>
+          <t>10-12~10-13</t>
+        </is>
+      </c>
+      <c r="C60" s="18" t="inlineStr">
+        <is>
+          <t>수집예정</t>
         </is>
       </c>
       <c r="D60" s="7" t="inlineStr">
         <is>
-          <t>852,000</t>
+          <t>6,500,000</t>
         </is>
       </c>
       <c r="E60" s="7" t="inlineStr">
         <is>
-          <t>16,614,000,000</t>
-        </is>
-      </c>
-      <c r="F60" s="6" t="inlineStr">
-        <is>
-          <t>17.61배 (PER)</t>
+          <t>13,000,000,000</t>
+        </is>
+      </c>
+      <c r="F60" s="18" t="inlineStr">
+        <is>
+          <t>수집예정</t>
         </is>
       </c>
       <c r="G60" s="6" t="inlineStr"/>
@@ -11901,63 +11917,63 @@
       <c r="I60" s="6" t="inlineStr"/>
       <c r="J60" s="6" t="inlineStr">
         <is>
-          <t>10-02~10-06</t>
+          <t>10-15~10-16</t>
         </is>
       </c>
       <c r="K60" s="6" t="inlineStr"/>
       <c r="L60" s="6" t="inlineStr"/>
       <c r="M60" s="6" t="inlineStr"/>
-      <c r="N60" s="6" t="inlineStr">
-        <is>
-          <t>하나증권</t>
+      <c r="N60" s="18" t="inlineStr">
+        <is>
+          <t>수집예정</t>
         </is>
       </c>
       <c r="O60" s="6" t="inlineStr"/>
-      <c r="P60" s="7" t="inlineStr">
-        <is>
-          <t>697,788,000</t>
+      <c r="P60" s="18" t="inlineStr">
+        <is>
+          <t>수집예정</t>
         </is>
       </c>
       <c r="Q60" s="6" t="inlineStr">
         <is>
-          <t>4.0%</t>
+          <t>50%</t>
         </is>
       </c>
       <c r="R60" s="6" t="inlineStr">
         <is>
-          <t>최초</t>
+          <t>정정</t>
         </is>
       </c>
     </row>
     <row r="61" ht="30" customHeight="1">
       <c r="A61" s="6" t="inlineStr">
         <is>
-          <t>엠비디</t>
+          <t>진코스텍</t>
         </is>
       </c>
       <c r="B61" s="6" t="inlineStr">
         <is>
-          <t>09-21~09-29</t>
+          <t>09-16~09-22</t>
         </is>
       </c>
       <c r="C61" s="6" t="inlineStr">
         <is>
-          <t>9,400~11,500</t>
+          <t>19,500~23,500</t>
         </is>
       </c>
       <c r="D61" s="7" t="inlineStr">
         <is>
-          <t>2,000,000</t>
+          <t>852,000</t>
         </is>
       </c>
       <c r="E61" s="7" t="inlineStr">
         <is>
-          <t>18,800,000,000</t>
+          <t>16,614,000,000</t>
         </is>
       </c>
       <c r="F61" s="6" t="inlineStr">
         <is>
-          <t>26.87배 (PER)</t>
+          <t>17.61배 (PER)</t>
         </is>
       </c>
       <c r="G61" s="6" t="inlineStr"/>
@@ -11965,7 +11981,7 @@
       <c r="I61" s="6" t="inlineStr"/>
       <c r="J61" s="6" t="inlineStr">
         <is>
-          <t>10-06~10-07</t>
+          <t>10-02~10-06</t>
         </is>
       </c>
       <c r="K61" s="6" t="inlineStr"/>
@@ -11979,12 +11995,12 @@
       <c r="O61" s="6" t="inlineStr"/>
       <c r="P61" s="7" t="inlineStr">
         <is>
-          <t>968,200,000</t>
+          <t>697,788,000</t>
         </is>
       </c>
       <c r="Q61" s="6" t="inlineStr">
         <is>
-          <t>5.0%</t>
+          <t>4.0%</t>
         </is>
       </c>
       <c r="R61" s="6" t="inlineStr">
@@ -11996,32 +12012,32 @@
     <row r="62" ht="30" customHeight="1">
       <c r="A62" s="6" t="inlineStr">
         <is>
-          <t>엠에스바이오</t>
+          <t>엠비디</t>
         </is>
       </c>
       <c r="B62" s="6" t="inlineStr">
         <is>
-          <t>09-28~10-02</t>
+          <t>09-21~09-29</t>
         </is>
       </c>
       <c r="C62" s="6" t="inlineStr">
         <is>
-          <t>6,800~7,800</t>
+          <t>9,400~11,500</t>
         </is>
       </c>
       <c r="D62" s="7" t="inlineStr">
         <is>
-          <t>4,000,000</t>
+          <t>2,000,000</t>
         </is>
       </c>
       <c r="E62" s="7" t="inlineStr">
         <is>
-          <t>27,200,000,000</t>
+          <t>18,800,000,000</t>
         </is>
       </c>
       <c r="F62" s="6" t="inlineStr">
         <is>
-          <t>30.89배 (PER)</t>
+          <t>26.87배 (PER)</t>
         </is>
       </c>
       <c r="G62" s="6" t="inlineStr"/>
@@ -12029,7 +12045,7 @@
       <c r="I62" s="6" t="inlineStr"/>
       <c r="J62" s="6" t="inlineStr">
         <is>
-          <t>10-12~10-13</t>
+          <t>10-06~10-07</t>
         </is>
       </c>
       <c r="K62" s="6" t="inlineStr"/>
@@ -12037,18 +12053,18 @@
       <c r="M62" s="6" t="inlineStr"/>
       <c r="N62" s="6" t="inlineStr">
         <is>
-          <t>KB증권</t>
+          <t>하나증권</t>
         </is>
       </c>
       <c r="O62" s="6" t="inlineStr"/>
       <c r="P62" s="7" t="inlineStr">
         <is>
-          <t>1,120,640,000</t>
+          <t>968,200,000</t>
         </is>
       </c>
       <c r="Q62" s="6" t="inlineStr">
         <is>
-          <t>4.0%</t>
+          <t>5.0%</t>
         </is>
       </c>
       <c r="R62" s="6" t="inlineStr">
@@ -12060,32 +12076,32 @@
     <row r="63" ht="30" customHeight="1">
       <c r="A63" s="6" t="inlineStr">
         <is>
-          <t>티앤이코리아</t>
+          <t>엠에스바이오</t>
         </is>
       </c>
       <c r="B63" s="6" t="inlineStr">
         <is>
-          <t>10-07~10-14</t>
+          <t>09-28~10-02</t>
         </is>
       </c>
       <c r="C63" s="6" t="inlineStr">
         <is>
-          <t>12,600~15,300</t>
+          <t>6,800~7,800</t>
         </is>
       </c>
       <c r="D63" s="7" t="inlineStr">
         <is>
-          <t>2,400,000</t>
+          <t>4,000,000</t>
         </is>
       </c>
       <c r="E63" s="7" t="inlineStr">
         <is>
-          <t>30,240,000,000</t>
+          <t>27,200,000,000</t>
         </is>
       </c>
       <c r="F63" s="6" t="inlineStr">
         <is>
-          <t>19.48배 (PER)</t>
+          <t>30.89배 (PER)</t>
         </is>
       </c>
       <c r="G63" s="6" t="inlineStr"/>
@@ -12093,7 +12109,7 @@
       <c r="I63" s="6" t="inlineStr"/>
       <c r="J63" s="6" t="inlineStr">
         <is>
-          <t>10-20~10-21</t>
+          <t>10-12~10-13</t>
         </is>
       </c>
       <c r="K63" s="6" t="inlineStr"/>
@@ -12101,13 +12117,13 @@
       <c r="M63" s="6" t="inlineStr"/>
       <c r="N63" s="6" t="inlineStr">
         <is>
-          <t>신한투자증권</t>
+          <t>KB증권</t>
         </is>
       </c>
       <c r="O63" s="6" t="inlineStr"/>
       <c r="P63" s="7" t="inlineStr">
         <is>
-          <t>1,245,888,000</t>
+          <t>1,120,640,000</t>
         </is>
       </c>
       <c r="Q63" s="6" t="inlineStr">
@@ -12124,32 +12140,32 @@
     <row r="64" ht="30" customHeight="1">
       <c r="A64" s="6" t="inlineStr">
         <is>
-          <t>에스케이증권제14호기업인수목적</t>
+          <t>티앤이코리아</t>
         </is>
       </c>
       <c r="B64" s="6" t="inlineStr">
         <is>
-          <t>10-12~10-13</t>
-        </is>
-      </c>
-      <c r="C64" s="18" t="inlineStr">
-        <is>
-          <t>수집예정</t>
+          <t>10-07~10-14</t>
+        </is>
+      </c>
+      <c r="C64" s="6" t="inlineStr">
+        <is>
+          <t>12,600~15,300</t>
         </is>
       </c>
       <c r="D64" s="7" t="inlineStr">
         <is>
-          <t>6,500,000</t>
+          <t>2,400,000</t>
         </is>
       </c>
       <c r="E64" s="7" t="inlineStr">
         <is>
-          <t>13,000,000,000</t>
-        </is>
-      </c>
-      <c r="F64" s="18" t="inlineStr">
-        <is>
-          <t>수집예정</t>
+          <t>30,240,000,000</t>
+        </is>
+      </c>
+      <c r="F64" s="6" t="inlineStr">
+        <is>
+          <t>19.48배 (PER)</t>
         </is>
       </c>
       <c r="G64" s="6" t="inlineStr"/>
@@ -12157,26 +12173,26 @@
       <c r="I64" s="6" t="inlineStr"/>
       <c r="J64" s="6" t="inlineStr">
         <is>
-          <t>10-15~10-16</t>
+          <t>10-20~10-21</t>
         </is>
       </c>
       <c r="K64" s="6" t="inlineStr"/>
       <c r="L64" s="6" t="inlineStr"/>
       <c r="M64" s="6" t="inlineStr"/>
-      <c r="N64" s="18" t="inlineStr">
-        <is>
-          <t>수집예정</t>
+      <c r="N64" s="6" t="inlineStr">
+        <is>
+          <t>신한투자증권</t>
         </is>
       </c>
       <c r="O64" s="6" t="inlineStr"/>
-      <c r="P64" s="18" t="inlineStr">
-        <is>
-          <t>수집예정</t>
+      <c r="P64" s="7" t="inlineStr">
+        <is>
+          <t>1,245,888,000</t>
         </is>
       </c>
       <c r="Q64" s="6" t="inlineStr">
         <is>
-          <t>50%</t>
+          <t>4.0%</t>
         </is>
       </c>
       <c r="R64" s="6" t="inlineStr">
@@ -12188,32 +12204,32 @@
     <row r="65" ht="30" customHeight="1">
       <c r="A65" s="6" t="inlineStr">
         <is>
-          <t>크리에이츠</t>
+          <t>유캐스트</t>
         </is>
       </c>
       <c r="B65" s="6" t="inlineStr">
         <is>
-          <t>10-12~10-16</t>
+          <t>10-07~10-14</t>
         </is>
       </c>
       <c r="C65" s="6" t="inlineStr">
         <is>
-          <t>15,000~18,000</t>
+          <t>21,000~26,000</t>
         </is>
       </c>
       <c r="D65" s="7" t="inlineStr">
         <is>
-          <t>1,400,000</t>
+          <t>800,000</t>
         </is>
       </c>
       <c r="E65" s="7" t="inlineStr">
         <is>
-          <t>21,000,000,000</t>
+          <t>16,800,000,000</t>
         </is>
       </c>
       <c r="F65" s="6" t="inlineStr">
         <is>
-          <t>19.15배 (PER)</t>
+          <t>17.97배 (PER)</t>
         </is>
       </c>
       <c r="G65" s="6" t="inlineStr"/>
@@ -12221,7 +12237,7 @@
       <c r="I65" s="6" t="inlineStr"/>
       <c r="J65" s="6" t="inlineStr">
         <is>
-          <t>10-20~10-21</t>
+          <t>10-19~10-20</t>
         </is>
       </c>
       <c r="K65" s="6" t="inlineStr"/>
@@ -12229,18 +12245,18 @@
       <c r="M65" s="6" t="inlineStr"/>
       <c r="N65" s="6" t="inlineStr">
         <is>
-          <t>삼성증권</t>
+          <t>유진투자증권</t>
         </is>
       </c>
       <c r="O65" s="6" t="inlineStr"/>
       <c r="P65" s="7" t="inlineStr">
         <is>
-          <t>865,200,000</t>
+          <t>1,181,280,000</t>
         </is>
       </c>
       <c r="Q65" s="6" t="inlineStr">
         <is>
-          <t>4.0%</t>
+          <t>7.0%</t>
         </is>
       </c>
       <c r="R65" s="6" t="inlineStr">
@@ -12252,59 +12268,59 @@
     <row r="66" ht="30" customHeight="1">
       <c r="A66" s="6" t="inlineStr">
         <is>
-          <t>바로팜</t>
-        </is>
-      </c>
-      <c r="B66" s="18" t="inlineStr">
-        <is>
-          <t>수집예정</t>
+          <t>크리에이츠</t>
+        </is>
+      </c>
+      <c r="B66" s="6" t="inlineStr">
+        <is>
+          <t>10-12~10-16</t>
         </is>
       </c>
       <c r="C66" s="6" t="inlineStr">
         <is>
-          <t>16,400~20,200</t>
+          <t>15,000~18,000</t>
         </is>
       </c>
       <c r="D66" s="7" t="inlineStr">
         <is>
-          <t>1,780,000</t>
+          <t>1,400,000</t>
         </is>
       </c>
       <c r="E66" s="7" t="inlineStr">
         <is>
-          <t>29,192,000,000</t>
+          <t>21,000,000,000</t>
         </is>
       </c>
       <c r="F66" s="6" t="inlineStr">
         <is>
-          <t>24.95배 (PER)</t>
+          <t>19.15배 (PER)</t>
         </is>
       </c>
       <c r="G66" s="6" t="inlineStr"/>
       <c r="H66" s="6" t="inlineStr"/>
       <c r="I66" s="6" t="inlineStr"/>
-      <c r="J66" s="18" t="inlineStr">
-        <is>
-          <t>수집예정</t>
+      <c r="J66" s="6" t="inlineStr">
+        <is>
+          <t>10-20~10-21</t>
         </is>
       </c>
       <c r="K66" s="6" t="inlineStr"/>
       <c r="L66" s="6" t="inlineStr"/>
       <c r="M66" s="6" t="inlineStr"/>
-      <c r="N66" s="18" t="inlineStr">
-        <is>
-          <t>수집예정</t>
+      <c r="N66" s="6" t="inlineStr">
+        <is>
+          <t>삼성증권</t>
         </is>
       </c>
       <c r="O66" s="6" t="inlineStr"/>
-      <c r="P66" s="18" t="inlineStr">
-        <is>
-          <t>수집예정</t>
-        </is>
-      </c>
-      <c r="Q66" s="18" t="inlineStr">
-        <is>
-          <t>수집예정</t>
+      <c r="P66" s="7" t="inlineStr">
+        <is>
+          <t>865,200,000</t>
+        </is>
+      </c>
+      <c r="Q66" s="6" t="inlineStr">
+        <is>
+          <t>4.0%</t>
         </is>
       </c>
       <c r="R66" s="6" t="inlineStr">
@@ -12316,7 +12332,7 @@
     <row r="67" ht="30" customHeight="1">
       <c r="A67" s="6" t="inlineStr">
         <is>
-          <t>디티에스</t>
+          <t>바로팜</t>
         </is>
       </c>
       <c r="B67" s="18" t="inlineStr">
@@ -12324,24 +12340,24 @@
           <t>수집예정</t>
         </is>
       </c>
-      <c r="C67" s="18" t="inlineStr">
-        <is>
-          <t>수집예정</t>
-        </is>
-      </c>
-      <c r="D67" s="18" t="inlineStr">
-        <is>
-          <t>수집예정</t>
-        </is>
-      </c>
-      <c r="E67" s="18" t="inlineStr">
-        <is>
-          <t>수집예정</t>
-        </is>
-      </c>
-      <c r="F67" s="18" t="inlineStr">
-        <is>
-          <t>수집예정</t>
+      <c r="C67" s="6" t="inlineStr">
+        <is>
+          <t>16,400~20,200</t>
+        </is>
+      </c>
+      <c r="D67" s="7" t="inlineStr">
+        <is>
+          <t>1,780,000</t>
+        </is>
+      </c>
+      <c r="E67" s="7" t="inlineStr">
+        <is>
+          <t>29,192,000,000</t>
+        </is>
+      </c>
+      <c r="F67" s="6" t="inlineStr">
+        <is>
+          <t>24.95배 (PER)</t>
         </is>
       </c>
       <c r="G67" s="6" t="inlineStr"/>
@@ -12373,14 +12389,14 @@
       </c>
       <c r="R67" s="6" t="inlineStr">
         <is>
-          <t>신고서 대기</t>
+          <t>최초</t>
         </is>
       </c>
     </row>
     <row r="68" ht="30" customHeight="1">
       <c r="A68" s="6" t="inlineStr">
         <is>
-          <t>한화플러스제6호스팩</t>
+          <t>디티에스</t>
         </is>
       </c>
       <c r="B68" s="18" t="inlineStr">
@@ -12444,7 +12460,7 @@
     <row r="69" ht="30" customHeight="1">
       <c r="A69" s="6" t="inlineStr">
         <is>
-          <t>유캐스트</t>
+          <t>한화플러스제6호스팩</t>
         </is>
       </c>
       <c r="B69" s="18" t="inlineStr">
@@ -13324,7 +13340,7 @@
     <row r="28">
       <c r="A28" s="6" t="inlineStr">
         <is>
-          <t>하나증권</t>
+          <t>유진투자증권</t>
         </is>
       </c>
       <c r="B28" s="6" t="n">
@@ -13332,29 +13348,29 @@
       </c>
       <c r="C28" s="6" t="inlineStr">
         <is>
-          <t>35,414,000,000</t>
+          <t>40,800,000,000</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="6" t="inlineStr">
         <is>
-          <t>신한투자증권</t>
+          <t>하나증권</t>
         </is>
       </c>
       <c r="B29" s="6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C29" s="6" t="inlineStr">
         <is>
-          <t>30,240,000,000</t>
+          <t>35,414,000,000</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="6" t="inlineStr">
         <is>
-          <t>KB증권</t>
+          <t>신한투자증권</t>
         </is>
       </c>
       <c r="B30" s="6" t="n">
@@ -13362,14 +13378,14 @@
       </c>
       <c r="C30" s="6" t="inlineStr">
         <is>
-          <t>27,200,000,000</t>
+          <t>30,240,000,000</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="6" t="inlineStr">
         <is>
-          <t>유진투자증권</t>
+          <t>KB증권</t>
         </is>
       </c>
       <c r="B31" s="6" t="n">
@@ -13377,7 +13393,7 @@
       </c>
       <c r="C31" s="6" t="inlineStr">
         <is>
-          <t>24,000,000,000</t>
+          <t>27,200,000,000</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore: update IPO data 2026-09-11
</commit_message>
<xml_diff>
--- a/IPO_analysis.xlsx
+++ b/IPO_analysis.xlsx
@@ -618,14 +618,14 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>기준일 2026-09-10 · 청구일 직전 사업연도 · 별도/개별 재무제표 · 단위 백만원(별도 표기 시 USD)</t>
+          <t>기준일 2026-09-11 · 청구일 직전 사업연도 · 별도/개별 재무제표 · 단위 백만원(별도 표기 시 USD)</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
-          <t>■ 심사 신청(진행중)  (48건)</t>
+          <t>■ 심사 신청(진행중)  (46건)</t>
         </is>
       </c>
       <c r="B4" s="4" t="n"/>
@@ -2589,12 +2589,12 @@
     <row r="40">
       <c r="A40" s="6" t="inlineStr">
         <is>
-          <t>2026-06-19</t>
+          <t>2026-06-18</t>
         </is>
       </c>
       <c r="B40" s="6" t="inlineStr">
         <is>
-          <t>이에스티</t>
+          <t>영광</t>
         </is>
       </c>
       <c r="C40" s="6" t="inlineStr">
@@ -2614,27 +2614,27 @@
       </c>
       <c r="F40" s="7" t="inlineStr">
         <is>
-          <t>33,190</t>
+          <t>113,133</t>
         </is>
       </c>
       <c r="G40" s="7" t="inlineStr">
         <is>
-          <t>2,966</t>
+          <t>10,328</t>
         </is>
       </c>
       <c r="H40" s="7" t="inlineStr">
         <is>
-          <t>4,325</t>
+          <t>3,052</t>
         </is>
       </c>
       <c r="I40" s="6" t="inlineStr">
         <is>
-          <t>특수 목적용 기계 제조업</t>
+          <t>구조용 금속제품, 탱크 및 증기발생기 제조업</t>
         </is>
       </c>
       <c r="J40" s="6" t="inlineStr">
         <is>
-          <t>대신</t>
+          <t>한국</t>
         </is>
       </c>
       <c r="K40" s="6" t="inlineStr">
@@ -2646,12 +2646,12 @@
     <row r="41">
       <c r="A41" s="6" t="inlineStr">
         <is>
-          <t>2026-06-18</t>
+          <t>2026-06-11</t>
         </is>
       </c>
       <c r="B41" s="6" t="inlineStr">
         <is>
-          <t>영광</t>
+          <t>씨엔티테크</t>
         </is>
       </c>
       <c r="C41" s="6" t="inlineStr">
@@ -2671,27 +2671,27 @@
       </c>
       <c r="F41" s="7" t="inlineStr">
         <is>
-          <t>113,133</t>
+          <t>27,015</t>
         </is>
       </c>
       <c r="G41" s="7" t="inlineStr">
         <is>
-          <t>10,328</t>
+          <t>3,987</t>
         </is>
       </c>
       <c r="H41" s="7" t="inlineStr">
         <is>
-          <t>3,052</t>
+          <t>2,613</t>
         </is>
       </c>
       <c r="I41" s="6" t="inlineStr">
         <is>
-          <t>구조용 금속제품, 탱크 및 증기발생기 제조업</t>
+          <t>소프트웨어 개발 및 공급업</t>
         </is>
       </c>
       <c r="J41" s="6" t="inlineStr">
         <is>
-          <t>한국</t>
+          <t>한화, 하나</t>
         </is>
       </c>
       <c r="K41" s="6" t="inlineStr">
@@ -2708,7 +2708,7 @@
       </c>
       <c r="B42" s="6" t="inlineStr">
         <is>
-          <t>씨엔티테크</t>
+          <t>제이앤티지</t>
         </is>
       </c>
       <c r="C42" s="6" t="inlineStr">
@@ -2728,27 +2728,27 @@
       </c>
       <c r="F42" s="7" t="inlineStr">
         <is>
-          <t>27,015</t>
+          <t>72,378</t>
         </is>
       </c>
       <c r="G42" s="7" t="inlineStr">
         <is>
-          <t>3,987</t>
+          <t>9,904</t>
         </is>
       </c>
       <c r="H42" s="7" t="inlineStr">
         <is>
-          <t>2,613</t>
+          <t>6,743</t>
         </is>
       </c>
       <c r="I42" s="6" t="inlineStr">
         <is>
-          <t>소프트웨어 개발 및 공급업</t>
+          <t>전자부품 제조업</t>
         </is>
       </c>
       <c r="J42" s="6" t="inlineStr">
         <is>
-          <t>한화, 하나</t>
+          <t>대신, NH</t>
         </is>
       </c>
       <c r="K42" s="6" t="inlineStr">
@@ -2760,12 +2760,12 @@
     <row r="43">
       <c r="A43" s="6" t="inlineStr">
         <is>
-          <t>2026-06-11</t>
+          <t>2026-05-29</t>
         </is>
       </c>
       <c r="B43" s="6" t="inlineStr">
         <is>
-          <t>제이앤티지</t>
+          <t>인터엑스</t>
         </is>
       </c>
       <c r="C43" s="6" t="inlineStr">
@@ -2785,27 +2785,27 @@
       </c>
       <c r="F43" s="7" t="inlineStr">
         <is>
-          <t>72,378</t>
+          <t>8,645</t>
         </is>
       </c>
       <c r="G43" s="7" t="inlineStr">
         <is>
-          <t>9,904</t>
+          <t>-20,272</t>
         </is>
       </c>
       <c r="H43" s="7" t="inlineStr">
         <is>
-          <t>6,743</t>
+          <t>4,530</t>
         </is>
       </c>
       <c r="I43" s="6" t="inlineStr">
         <is>
-          <t>전자부품 제조업</t>
+          <t>소프트웨어 개발 및 공급업</t>
         </is>
       </c>
       <c r="J43" s="6" t="inlineStr">
         <is>
-          <t>대신, NH</t>
+          <t>한국</t>
         </is>
       </c>
       <c r="K43" s="6" t="inlineStr">
@@ -2822,7 +2822,7 @@
       </c>
       <c r="B44" s="6" t="inlineStr">
         <is>
-          <t>인터엑스</t>
+          <t>케이엠에프</t>
         </is>
       </c>
       <c r="C44" s="6" t="inlineStr">
@@ -2842,27 +2842,27 @@
       </c>
       <c r="F44" s="7" t="inlineStr">
         <is>
-          <t>8,645</t>
+          <t>25,751</t>
         </is>
       </c>
       <c r="G44" s="7" t="inlineStr">
         <is>
-          <t>-20,272</t>
+          <t>11,463</t>
         </is>
       </c>
       <c r="H44" s="7" t="inlineStr">
         <is>
-          <t>4,530</t>
+          <t>642</t>
         </is>
       </c>
       <c r="I44" s="6" t="inlineStr">
         <is>
-          <t>소프트웨어 개발 및 공급업</t>
+          <t>기타 식품 제조업</t>
         </is>
       </c>
       <c r="J44" s="6" t="inlineStr">
         <is>
-          <t>한국</t>
+          <t>IBK</t>
         </is>
       </c>
       <c r="K44" s="6" t="inlineStr">
@@ -2874,12 +2874,12 @@
     <row r="45">
       <c r="A45" s="6" t="inlineStr">
         <is>
-          <t>2026-05-29</t>
+          <t>2026-05-28</t>
         </is>
       </c>
       <c r="B45" s="6" t="inlineStr">
         <is>
-          <t>케이엠에프</t>
+          <t>삼홍아크튜리온</t>
         </is>
       </c>
       <c r="C45" s="6" t="inlineStr">
@@ -2899,27 +2899,27 @@
       </c>
       <c r="F45" s="7" t="inlineStr">
         <is>
-          <t>25,751</t>
+          <t>26,162</t>
         </is>
       </c>
       <c r="G45" s="7" t="inlineStr">
         <is>
-          <t>11,463</t>
+          <t>-10,314</t>
         </is>
       </c>
       <c r="H45" s="7" t="inlineStr">
         <is>
-          <t>642</t>
+          <t>6,369</t>
         </is>
       </c>
       <c r="I45" s="6" t="inlineStr">
         <is>
-          <t>기타 식품 제조업</t>
+          <t>구조용 금속제품, 탱크 및 증기발생기 제조업</t>
         </is>
       </c>
       <c r="J45" s="6" t="inlineStr">
         <is>
-          <t>IBK</t>
+          <t>삼성, 미래</t>
         </is>
       </c>
       <c r="K45" s="6" t="inlineStr">
@@ -2931,12 +2931,12 @@
     <row r="46">
       <c r="A46" s="6" t="inlineStr">
         <is>
-          <t>2026-05-28</t>
+          <t>2026-05-21</t>
         </is>
       </c>
       <c r="B46" s="6" t="inlineStr">
         <is>
-          <t>삼홍아크튜리온</t>
+          <t>넥스트에어로스페이스</t>
         </is>
       </c>
       <c r="C46" s="6" t="inlineStr">
@@ -2956,27 +2956,27 @@
       </c>
       <c r="F46" s="7" t="inlineStr">
         <is>
-          <t>26,162</t>
+          <t>12,084</t>
         </is>
       </c>
       <c r="G46" s="7" t="inlineStr">
         <is>
-          <t>-10,314</t>
+          <t>-17,270</t>
         </is>
       </c>
       <c r="H46" s="7" t="inlineStr">
         <is>
-          <t>6,369</t>
+          <t>6,158</t>
         </is>
       </c>
       <c r="I46" s="6" t="inlineStr">
         <is>
-          <t>구조용 금속제품, 탱크 및 증기발생기 제조업</t>
+          <t>유인 항공기, 항공우주선 및 보조장치 제조업</t>
         </is>
       </c>
       <c r="J46" s="6" t="inlineStr">
         <is>
-          <t>삼성, 미래</t>
+          <t>삼성</t>
         </is>
       </c>
       <c r="K46" s="6" t="inlineStr">
@@ -2988,12 +2988,12 @@
     <row r="47">
       <c r="A47" s="6" t="inlineStr">
         <is>
-          <t>2026-05-22</t>
+          <t>2026-05-21</t>
         </is>
       </c>
       <c r="B47" s="6" t="inlineStr">
         <is>
-          <t>에이엘로봇</t>
+          <t>비앤비코리아</t>
         </is>
       </c>
       <c r="C47" s="6" t="inlineStr">
@@ -3013,27 +3013,27 @@
       </c>
       <c r="F47" s="7" t="inlineStr">
         <is>
-          <t>14,985</t>
+          <t>141,169</t>
         </is>
       </c>
       <c r="G47" s="7" t="inlineStr">
         <is>
-          <t>-21,891</t>
+          <t>21,406</t>
         </is>
       </c>
       <c r="H47" s="7" t="inlineStr">
         <is>
-          <t>129</t>
+          <t>43,932</t>
         </is>
       </c>
       <c r="I47" s="6" t="inlineStr">
         <is>
-          <t>산업용 로봇 제조업</t>
+          <t>기타 화학제품 제조업</t>
         </is>
       </c>
       <c r="J47" s="6" t="inlineStr">
         <is>
-          <t>대신</t>
+          <t>미래</t>
         </is>
       </c>
       <c r="K47" s="6" t="inlineStr">
@@ -3045,12 +3045,12 @@
     <row r="48">
       <c r="A48" s="6" t="inlineStr">
         <is>
-          <t>2026-05-21</t>
+          <t>2026-05-12</t>
         </is>
       </c>
       <c r="B48" s="6" t="inlineStr">
         <is>
-          <t>넥스트에어로스페이스</t>
+          <t>오토핸즈</t>
         </is>
       </c>
       <c r="C48" s="6" t="inlineStr">
@@ -3060,7 +3060,7 @@
       </c>
       <c r="D48" s="6" t="inlineStr">
         <is>
-          <t>신규상장</t>
+          <t>스팩 소멸합병</t>
         </is>
       </c>
       <c r="E48" s="6" t="inlineStr">
@@ -3070,27 +3070,27 @@
       </c>
       <c r="F48" s="7" t="inlineStr">
         <is>
-          <t>12,084</t>
+          <t>238,564</t>
         </is>
       </c>
       <c r="G48" s="7" t="inlineStr">
         <is>
-          <t>-17,270</t>
+          <t>6,047</t>
         </is>
       </c>
       <c r="H48" s="7" t="inlineStr">
         <is>
-          <t>6,158</t>
+          <t>6,129</t>
         </is>
       </c>
       <c r="I48" s="6" t="inlineStr">
         <is>
-          <t>유인 항공기, 항공우주선 및 보조장치 제조업</t>
+          <t>자동차 판매업</t>
         </is>
       </c>
       <c r="J48" s="6" t="inlineStr">
         <is>
-          <t>삼성</t>
+          <t>미래</t>
         </is>
       </c>
       <c r="K48" s="6" t="inlineStr">
@@ -3102,12 +3102,12 @@
     <row r="49">
       <c r="A49" s="6" t="inlineStr">
         <is>
-          <t>2026-05-21</t>
+          <t>2026-05-06</t>
         </is>
       </c>
       <c r="B49" s="6" t="inlineStr">
         <is>
-          <t>비앤비코리아</t>
+          <t>아이벡스메디칼시스템즈</t>
         </is>
       </c>
       <c r="C49" s="6" t="inlineStr">
@@ -3127,27 +3127,27 @@
       </c>
       <c r="F49" s="7" t="inlineStr">
         <is>
-          <t>141,169</t>
+          <t>15,282</t>
         </is>
       </c>
       <c r="G49" s="7" t="inlineStr">
         <is>
-          <t>21,406</t>
+          <t>-7,227</t>
         </is>
       </c>
       <c r="H49" s="7" t="inlineStr">
         <is>
-          <t>43,932</t>
+          <t>744</t>
         </is>
       </c>
       <c r="I49" s="6" t="inlineStr">
         <is>
-          <t>기타 화학제품 제조업</t>
+          <t>의료용 기기 제조업</t>
         </is>
       </c>
       <c r="J49" s="6" t="inlineStr">
         <is>
-          <t>미래</t>
+          <t>NH</t>
         </is>
       </c>
       <c r="K49" s="6" t="inlineStr">
@@ -3159,12 +3159,12 @@
     <row r="50">
       <c r="A50" s="6" t="inlineStr">
         <is>
-          <t>2026-05-12</t>
+          <t>2026-04-08</t>
         </is>
       </c>
       <c r="B50" s="6" t="inlineStr">
         <is>
-          <t>오토핸즈</t>
+          <t>옵토닉스</t>
         </is>
       </c>
       <c r="C50" s="6" t="inlineStr">
@@ -3174,7 +3174,7 @@
       </c>
       <c r="D50" s="6" t="inlineStr">
         <is>
-          <t>스팩 소멸합병</t>
+          <t>신규상장</t>
         </is>
       </c>
       <c r="E50" s="6" t="inlineStr">
@@ -3184,27 +3184,27 @@
       </c>
       <c r="F50" s="7" t="inlineStr">
         <is>
-          <t>238,564</t>
+          <t>25,368</t>
         </is>
       </c>
       <c r="G50" s="7" t="inlineStr">
         <is>
-          <t>6,047</t>
+          <t>1,901</t>
         </is>
       </c>
       <c r="H50" s="7" t="inlineStr">
         <is>
-          <t>6,129</t>
+          <t>730</t>
         </is>
       </c>
       <c r="I50" s="6" t="inlineStr">
         <is>
-          <t>자동차 판매업</t>
+          <t>광학렌즈 및 광학요소 제조업</t>
         </is>
       </c>
       <c r="J50" s="6" t="inlineStr">
         <is>
-          <t>미래</t>
+          <t>한국</t>
         </is>
       </c>
       <c r="K50" s="6" t="inlineStr">
@@ -3216,12 +3216,12 @@
     <row r="51">
       <c r="A51" s="6" t="inlineStr">
         <is>
-          <t>2026-05-06</t>
+          <t>2026-02-27</t>
         </is>
       </c>
       <c r="B51" s="6" t="inlineStr">
         <is>
-          <t>아이벡스메디칼시스템즈</t>
+          <t>피지티</t>
         </is>
       </c>
       <c r="C51" s="6" t="inlineStr">
@@ -3241,27 +3241,27 @@
       </c>
       <c r="F51" s="7" t="inlineStr">
         <is>
-          <t>15,282</t>
+          <t>40,141</t>
         </is>
       </c>
       <c r="G51" s="7" t="inlineStr">
         <is>
-          <t>-7,227</t>
+          <t>-69,722</t>
         </is>
       </c>
       <c r="H51" s="7" t="inlineStr">
         <is>
-          <t>744</t>
+          <t>6,029</t>
         </is>
       </c>
       <c r="I51" s="6" t="inlineStr">
         <is>
-          <t>의료용 기기 제조업</t>
+          <t>기타 화학제품 제조업</t>
         </is>
       </c>
       <c r="J51" s="6" t="inlineStr">
         <is>
-          <t>NH</t>
+          <t>한국</t>
         </is>
       </c>
       <c r="K51" s="6" t="inlineStr">
@@ -3270,191 +3270,191 @@
         </is>
       </c>
     </row>
-    <row r="52">
-      <c r="A52" s="6" t="inlineStr">
-        <is>
-          <t>2026-04-08</t>
-        </is>
-      </c>
-      <c r="B52" s="6" t="inlineStr">
-        <is>
-          <t>옵토닉스</t>
-        </is>
-      </c>
-      <c r="C52" s="6" t="inlineStr">
+    <row r="53">
+      <c r="A53" s="3" t="inlineStr">
+        <is>
+          <t>■ 심사 승인  (60건)</t>
+        </is>
+      </c>
+      <c r="B53" s="4" t="n"/>
+      <c r="C53" s="4" t="n"/>
+      <c r="D53" s="4" t="n"/>
+      <c r="E53" s="4" t="n"/>
+      <c r="F53" s="4" t="n"/>
+      <c r="G53" s="4" t="n"/>
+      <c r="H53" s="4" t="n"/>
+      <c r="I53" s="4" t="n"/>
+      <c r="J53" s="4" t="n"/>
+      <c r="K53" s="4" t="n"/>
+    </row>
+    <row r="54">
+      <c r="A54" s="5" t="inlineStr">
+        <is>
+          <t>일자</t>
+        </is>
+      </c>
+      <c r="B54" s="5" t="inlineStr">
+        <is>
+          <t>회사명</t>
+        </is>
+      </c>
+      <c r="C54" s="5" t="inlineStr">
+        <is>
+          <t>시장</t>
+        </is>
+      </c>
+      <c r="D54" s="5" t="inlineStr">
+        <is>
+          <t>상장유형</t>
+        </is>
+      </c>
+      <c r="E54" s="5" t="inlineStr">
+        <is>
+          <t>기준연도</t>
+        </is>
+      </c>
+      <c r="F54" s="5" t="inlineStr">
+        <is>
+          <t>매출액</t>
+        </is>
+      </c>
+      <c r="G54" s="5" t="inlineStr">
+        <is>
+          <t>순이익</t>
+        </is>
+      </c>
+      <c r="H54" s="5" t="inlineStr">
+        <is>
+          <t>자기자본</t>
+        </is>
+      </c>
+      <c r="I54" s="5" t="inlineStr">
+        <is>
+          <t>업종</t>
+        </is>
+      </c>
+      <c r="J54" s="5" t="inlineStr">
+        <is>
+          <t>대표주관사</t>
+        </is>
+      </c>
+      <c r="K54" s="5" t="inlineStr">
+        <is>
+          <t>현황</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="6" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="B55" s="6" t="inlineStr">
+        <is>
+          <t>이에스티</t>
+        </is>
+      </c>
+      <c r="C55" s="6" t="inlineStr">
         <is>
           <t>코스닥</t>
         </is>
       </c>
-      <c r="D52" s="6" t="inlineStr">
+      <c r="D55" s="6" t="inlineStr">
         <is>
           <t>신규상장</t>
         </is>
       </c>
-      <c r="E52" s="6" t="inlineStr">
+      <c r="E55" s="6" t="inlineStr">
         <is>
           <t>FY25</t>
         </is>
       </c>
-      <c r="F52" s="7" t="inlineStr">
-        <is>
-          <t>25,368</t>
-        </is>
-      </c>
-      <c r="G52" s="7" t="inlineStr">
-        <is>
-          <t>1,901</t>
-        </is>
-      </c>
-      <c r="H52" s="7" t="inlineStr">
-        <is>
-          <t>730</t>
-        </is>
-      </c>
-      <c r="I52" s="6" t="inlineStr">
-        <is>
-          <t>광학렌즈 및 광학요소 제조업</t>
-        </is>
-      </c>
-      <c r="J52" s="6" t="inlineStr">
-        <is>
-          <t>한국</t>
-        </is>
-      </c>
-      <c r="K52" s="6" t="inlineStr">
-        <is>
-          <t>예심 진행중</t>
-        </is>
-      </c>
-    </row>
-    <row r="53">
-      <c r="A53" s="6" t="inlineStr">
-        <is>
-          <t>2026-02-27</t>
-        </is>
-      </c>
-      <c r="B53" s="6" t="inlineStr">
-        <is>
-          <t>피지티</t>
-        </is>
-      </c>
-      <c r="C53" s="6" t="inlineStr">
+      <c r="F55" s="7" t="inlineStr">
+        <is>
+          <t>33,190</t>
+        </is>
+      </c>
+      <c r="G55" s="7" t="inlineStr">
+        <is>
+          <t>2,966</t>
+        </is>
+      </c>
+      <c r="H55" s="7" t="inlineStr">
+        <is>
+          <t>4,325</t>
+        </is>
+      </c>
+      <c r="I55" s="6" t="inlineStr">
+        <is>
+          <t>특수 목적용 기계 제조업</t>
+        </is>
+      </c>
+      <c r="J55" s="6" t="inlineStr">
+        <is>
+          <t>대신</t>
+        </is>
+      </c>
+      <c r="K55" s="6" t="inlineStr">
+        <is>
+          <t>상장전</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="6" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="B56" s="6" t="inlineStr">
+        <is>
+          <t>에이엘로봇</t>
+        </is>
+      </c>
+      <c r="C56" s="6" t="inlineStr">
         <is>
           <t>코스닥</t>
         </is>
       </c>
-      <c r="D53" s="6" t="inlineStr">
+      <c r="D56" s="6" t="inlineStr">
         <is>
           <t>신규상장</t>
         </is>
       </c>
-      <c r="E53" s="6" t="inlineStr">
+      <c r="E56" s="6" t="inlineStr">
         <is>
           <t>FY25</t>
         </is>
       </c>
-      <c r="F53" s="7" t="inlineStr">
-        <is>
-          <t>40,141</t>
-        </is>
-      </c>
-      <c r="G53" s="7" t="inlineStr">
-        <is>
-          <t>-69,722</t>
-        </is>
-      </c>
-      <c r="H53" s="7" t="inlineStr">
-        <is>
-          <t>6,029</t>
-        </is>
-      </c>
-      <c r="I53" s="6" t="inlineStr">
-        <is>
-          <t>기타 화학제품 제조업</t>
-        </is>
-      </c>
-      <c r="J53" s="6" t="inlineStr">
-        <is>
-          <t>한국</t>
-        </is>
-      </c>
-      <c r="K53" s="6" t="inlineStr">
-        <is>
-          <t>예심 진행중</t>
-        </is>
-      </c>
-    </row>
-    <row r="55">
-      <c r="A55" s="3" t="inlineStr">
-        <is>
-          <t>■ 심사 승인  (58건)</t>
-        </is>
-      </c>
-      <c r="B55" s="4" t="n"/>
-      <c r="C55" s="4" t="n"/>
-      <c r="D55" s="4" t="n"/>
-      <c r="E55" s="4" t="n"/>
-      <c r="F55" s="4" t="n"/>
-      <c r="G55" s="4" t="n"/>
-      <c r="H55" s="4" t="n"/>
-      <c r="I55" s="4" t="n"/>
-      <c r="J55" s="4" t="n"/>
-      <c r="K55" s="4" t="n"/>
-    </row>
-    <row r="56">
-      <c r="A56" s="5" t="inlineStr">
-        <is>
-          <t>일자</t>
-        </is>
-      </c>
-      <c r="B56" s="5" t="inlineStr">
-        <is>
-          <t>회사명</t>
-        </is>
-      </c>
-      <c r="C56" s="5" t="inlineStr">
-        <is>
-          <t>시장</t>
-        </is>
-      </c>
-      <c r="D56" s="5" t="inlineStr">
-        <is>
-          <t>상장유형</t>
-        </is>
-      </c>
-      <c r="E56" s="5" t="inlineStr">
-        <is>
-          <t>기준연도</t>
-        </is>
-      </c>
-      <c r="F56" s="5" t="inlineStr">
-        <is>
-          <t>매출액</t>
-        </is>
-      </c>
-      <c r="G56" s="5" t="inlineStr">
-        <is>
-          <t>순이익</t>
-        </is>
-      </c>
-      <c r="H56" s="5" t="inlineStr">
-        <is>
-          <t>자기자본</t>
-        </is>
-      </c>
-      <c r="I56" s="5" t="inlineStr">
-        <is>
-          <t>업종</t>
-        </is>
-      </c>
-      <c r="J56" s="5" t="inlineStr">
-        <is>
-          <t>대표주관사</t>
-        </is>
-      </c>
-      <c r="K56" s="5" t="inlineStr">
-        <is>
-          <t>현황</t>
+      <c r="F56" s="7" t="inlineStr">
+        <is>
+          <t>14,985</t>
+        </is>
+      </c>
+      <c r="G56" s="7" t="inlineStr">
+        <is>
+          <t>-21,891</t>
+        </is>
+      </c>
+      <c r="H56" s="7" t="inlineStr">
+        <is>
+          <t>129</t>
+        </is>
+      </c>
+      <c r="I56" s="6" t="inlineStr">
+        <is>
+          <t>산업용 로봇 제조업</t>
+        </is>
+      </c>
+      <c r="J56" s="6" t="inlineStr">
+        <is>
+          <t>대신</t>
+        </is>
+      </c>
+      <c r="K56" s="6" t="inlineStr">
+        <is>
+          <t>상장전</t>
         </is>
       </c>
     </row>
@@ -7735,7 +7735,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R78"/>
+  <dimension ref="A1:R80"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="1"/>
@@ -11173,7 +11173,7 @@
     <row r="48" ht="22" customHeight="1">
       <c r="A48" s="3" t="inlineStr">
         <is>
-          <t>■ 공모 진행 (예심 승인법인)  (26건)</t>
+          <t>■ 공모 진행 (예심 승인법인)  (28건)</t>
         </is>
       </c>
       <c r="B48" s="4" t="n"/>
@@ -11341,67 +11341,67 @@
     <row r="51" ht="30" customHeight="1">
       <c r="A51" s="6" t="inlineStr">
         <is>
-          <t>한국제17호스팩</t>
+          <t>와이즈플래닛컴퍼니</t>
         </is>
       </c>
       <c r="B51" s="6" t="inlineStr">
         <is>
-          <t>09-07~09-08</t>
-        </is>
-      </c>
-      <c r="C51" s="18" t="inlineStr">
-        <is>
-          <t>수집예정</t>
+          <t>09-04~09-10</t>
+        </is>
+      </c>
+      <c r="C51" s="6" t="inlineStr">
+        <is>
+          <t>10,000~12,000</t>
         </is>
       </c>
       <c r="D51" s="7" t="inlineStr">
         <is>
-          <t>7,000,000</t>
+          <t>1,600,000</t>
         </is>
       </c>
       <c r="E51" s="7" t="inlineStr">
         <is>
-          <t>14,000,000,000</t>
-        </is>
-      </c>
-      <c r="F51" s="18" t="inlineStr">
-        <is>
-          <t>수집예정</t>
+          <t>16,000,000,000</t>
+        </is>
+      </c>
+      <c r="F51" s="6" t="inlineStr">
+        <is>
+          <t>20.04배 (PER)</t>
         </is>
       </c>
       <c r="G51" s="6" t="inlineStr">
         <is>
-          <t>2,000</t>
+          <t>10,000</t>
         </is>
       </c>
       <c r="H51" s="6" t="n">
-        <v>1270.51</v>
+        <v>1248.47</v>
       </c>
       <c r="I51" s="6" t="n">
-        <v>2040</v>
+        <v>2323</v>
       </c>
       <c r="J51" s="6" t="inlineStr">
         <is>
-          <t>09-10~09-11</t>
+          <t>09-14~09-15</t>
         </is>
       </c>
       <c r="K51" s="6" t="inlineStr"/>
       <c r="L51" s="6" t="inlineStr"/>
       <c r="M51" s="6" t="inlineStr"/>
-      <c r="N51" s="18" t="inlineStr">
-        <is>
-          <t>수집예정</t>
+      <c r="N51" s="6" t="inlineStr">
+        <is>
+          <t>대신증권</t>
         </is>
       </c>
       <c r="O51" s="6" t="inlineStr"/>
-      <c r="P51" s="18" t="inlineStr">
-        <is>
-          <t>수집예정</t>
+      <c r="P51" s="7" t="inlineStr">
+        <is>
+          <t>494,400,000</t>
         </is>
       </c>
       <c r="Q51" s="6" t="inlineStr">
         <is>
-          <t>50%</t>
+          <t>3.0%</t>
         </is>
       </c>
       <c r="R51" s="6" t="inlineStr">
@@ -11413,96 +11413,104 @@
     <row r="52" ht="30" customHeight="1">
       <c r="A52" s="6" t="inlineStr">
         <is>
-          <t>브릴스</t>
+          <t>한국제17호스팩</t>
         </is>
       </c>
       <c r="B52" s="6" t="inlineStr">
         <is>
-          <t>08-31~09-04</t>
-        </is>
-      </c>
-      <c r="C52" s="6" t="inlineStr">
-        <is>
-          <t>16,500~19,500</t>
+          <t>09-07~09-08</t>
+        </is>
+      </c>
+      <c r="C52" s="18" t="inlineStr">
+        <is>
+          <t>수집예정</t>
         </is>
       </c>
       <c r="D52" s="7" t="inlineStr">
         <is>
-          <t>1,200,000</t>
+          <t>7,000,000</t>
         </is>
       </c>
       <c r="E52" s="7" t="inlineStr">
         <is>
-          <t>19,800,000,000</t>
-        </is>
-      </c>
-      <c r="F52" s="6" t="inlineStr">
-        <is>
-          <t>13.44 (PSR)</t>
-        </is>
-      </c>
-      <c r="G52" s="6" t="inlineStr"/>
-      <c r="H52" s="6" t="inlineStr"/>
-      <c r="I52" s="6" t="inlineStr"/>
+          <t>14,000,000,000</t>
+        </is>
+      </c>
+      <c r="F52" s="18" t="inlineStr">
+        <is>
+          <t>수집예정</t>
+        </is>
+      </c>
+      <c r="G52" s="6" t="inlineStr">
+        <is>
+          <t>2,000</t>
+        </is>
+      </c>
+      <c r="H52" s="6" t="n">
+        <v>1270.51</v>
+      </c>
+      <c r="I52" s="6" t="n">
+        <v>2040</v>
+      </c>
       <c r="J52" s="6" t="inlineStr">
         <is>
-          <t>09-08~09-09</t>
+          <t>09-10~09-11</t>
         </is>
       </c>
       <c r="K52" s="6" t="inlineStr"/>
       <c r="L52" s="6" t="inlineStr"/>
       <c r="M52" s="6" t="inlineStr"/>
-      <c r="N52" s="6" t="inlineStr">
-        <is>
-          <t>아이비케이투자증권</t>
+      <c r="N52" s="18" t="inlineStr">
+        <is>
+          <t>수집예정</t>
         </is>
       </c>
       <c r="O52" s="6" t="inlineStr"/>
-      <c r="P52" s="7" t="inlineStr">
-        <is>
-          <t>713,790,000</t>
+      <c r="P52" s="18" t="inlineStr">
+        <is>
+          <t>수집예정</t>
         </is>
       </c>
       <c r="Q52" s="6" t="inlineStr">
         <is>
-          <t>3.5%</t>
+          <t>50%</t>
         </is>
       </c>
       <c r="R52" s="6" t="inlineStr">
         <is>
-          <t>정정</t>
+          <t>발행조건확정</t>
         </is>
       </c>
     </row>
     <row r="53" ht="30" customHeight="1">
       <c r="A53" s="6" t="inlineStr">
         <is>
-          <t>와이즈플래닛컴퍼니</t>
+          <t>브릴스</t>
         </is>
       </c>
       <c r="B53" s="6" t="inlineStr">
         <is>
-          <t>09-04~09-10</t>
+          <t>08-31~09-04</t>
         </is>
       </c>
       <c r="C53" s="6" t="inlineStr">
         <is>
-          <t>10,000~12,000</t>
+          <t>16,500~19,500</t>
         </is>
       </c>
       <c r="D53" s="7" t="inlineStr">
         <is>
-          <t>1,600,000</t>
+          <t>1,200,000</t>
         </is>
       </c>
       <c r="E53" s="7" t="inlineStr">
         <is>
-          <t>16,000,000,000</t>
+          <t>19,800,000,000</t>
         </is>
       </c>
       <c r="F53" s="6" t="inlineStr">
         <is>
-          <t>20.04배 (PER)</t>
+          <t>13.44 (PSR)</t>
         </is>
       </c>
       <c r="G53" s="6" t="inlineStr"/>
@@ -11510,7 +11518,7 @@
       <c r="I53" s="6" t="inlineStr"/>
       <c r="J53" s="6" t="inlineStr">
         <is>
-          <t>09-14~09-15</t>
+          <t>09-08~09-09</t>
         </is>
       </c>
       <c r="K53" s="6" t="inlineStr"/>
@@ -11518,18 +11526,18 @@
       <c r="M53" s="6" t="inlineStr"/>
       <c r="N53" s="6" t="inlineStr">
         <is>
-          <t>대신증권</t>
+          <t>아이비케이투자증권</t>
         </is>
       </c>
       <c r="O53" s="6" t="inlineStr"/>
       <c r="P53" s="7" t="inlineStr">
         <is>
-          <t>494,400,000</t>
+          <t>713,790,000</t>
         </is>
       </c>
       <c r="Q53" s="6" t="inlineStr">
         <is>
-          <t>3.0%</t>
+          <t>3.5%</t>
         </is>
       </c>
       <c r="R53" s="6" t="inlineStr">
@@ -12890,22 +12898,150 @@
         </is>
       </c>
     </row>
-    <row r="76">
-      <c r="A76" s="20" t="inlineStr">
-        <is>
-          <t>※ 상장 완료 = KIND 신규상장 페이지 기준(스팩합병 포함) · 스팩 공모상장은 밴드·밸류에이션 등 해당없음(공모가 2,000원 고정).</t>
-        </is>
-      </c>
-    </row>
-    <row r="77">
-      <c r="A77" s="20" t="inlineStr">
-        <is>
-          <t>※ 기재정정 신고서 내 정정 전·후 병존 → 자동수집은 "정정 후" 값만 취함.</t>
+    <row r="75" ht="30" customHeight="1">
+      <c r="A75" s="6" t="inlineStr">
+        <is>
+          <t>이에스티</t>
+        </is>
+      </c>
+      <c r="B75" s="18" t="inlineStr">
+        <is>
+          <t>수집예정</t>
+        </is>
+      </c>
+      <c r="C75" s="18" t="inlineStr">
+        <is>
+          <t>수집예정</t>
+        </is>
+      </c>
+      <c r="D75" s="18" t="inlineStr">
+        <is>
+          <t>수집예정</t>
+        </is>
+      </c>
+      <c r="E75" s="18" t="inlineStr">
+        <is>
+          <t>수집예정</t>
+        </is>
+      </c>
+      <c r="F75" s="18" t="inlineStr">
+        <is>
+          <t>수집예정</t>
+        </is>
+      </c>
+      <c r="G75" s="6" t="inlineStr"/>
+      <c r="H75" s="6" t="inlineStr"/>
+      <c r="I75" s="6" t="inlineStr"/>
+      <c r="J75" s="18" t="inlineStr">
+        <is>
+          <t>수집예정</t>
+        </is>
+      </c>
+      <c r="K75" s="6" t="inlineStr"/>
+      <c r="L75" s="6" t="inlineStr"/>
+      <c r="M75" s="6" t="inlineStr"/>
+      <c r="N75" s="18" t="inlineStr">
+        <is>
+          <t>수집예정</t>
+        </is>
+      </c>
+      <c r="O75" s="6" t="inlineStr"/>
+      <c r="P75" s="18" t="inlineStr">
+        <is>
+          <t>수집예정</t>
+        </is>
+      </c>
+      <c r="Q75" s="18" t="inlineStr">
+        <is>
+          <t>수집예정</t>
+        </is>
+      </c>
+      <c r="R75" s="6" t="inlineStr">
+        <is>
+          <t>신고서 대기</t>
+        </is>
+      </c>
+    </row>
+    <row r="76" ht="30" customHeight="1">
+      <c r="A76" s="6" t="inlineStr">
+        <is>
+          <t>에이엘로봇</t>
+        </is>
+      </c>
+      <c r="B76" s="18" t="inlineStr">
+        <is>
+          <t>수집예정</t>
+        </is>
+      </c>
+      <c r="C76" s="18" t="inlineStr">
+        <is>
+          <t>수집예정</t>
+        </is>
+      </c>
+      <c r="D76" s="18" t="inlineStr">
+        <is>
+          <t>수집예정</t>
+        </is>
+      </c>
+      <c r="E76" s="18" t="inlineStr">
+        <is>
+          <t>수집예정</t>
+        </is>
+      </c>
+      <c r="F76" s="18" t="inlineStr">
+        <is>
+          <t>수집예정</t>
+        </is>
+      </c>
+      <c r="G76" s="6" t="inlineStr"/>
+      <c r="H76" s="6" t="inlineStr"/>
+      <c r="I76" s="6" t="inlineStr"/>
+      <c r="J76" s="18" t="inlineStr">
+        <is>
+          <t>수집예정</t>
+        </is>
+      </c>
+      <c r="K76" s="6" t="inlineStr"/>
+      <c r="L76" s="6" t="inlineStr"/>
+      <c r="M76" s="6" t="inlineStr"/>
+      <c r="N76" s="18" t="inlineStr">
+        <is>
+          <t>수집예정</t>
+        </is>
+      </c>
+      <c r="O76" s="6" t="inlineStr"/>
+      <c r="P76" s="18" t="inlineStr">
+        <is>
+          <t>수집예정</t>
+        </is>
+      </c>
+      <c r="Q76" s="18" t="inlineStr">
+        <is>
+          <t>수집예정</t>
+        </is>
+      </c>
+      <c r="R76" s="6" t="inlineStr">
+        <is>
+          <t>신고서 대기</t>
         </is>
       </c>
     </row>
     <row r="78">
       <c r="A78" s="20" t="inlineStr">
+        <is>
+          <t>※ 상장 완료 = KIND 신규상장 페이지 기준(스팩합병 포함) · 스팩 공모상장은 밴드·밸류에이션 등 해당없음(공모가 2,000원 고정).</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" s="20" t="inlineStr">
+        <is>
+          <t>※ 기재정정 신고서 내 정정 전·후 병존 → 자동수집은 "정정 후" 값만 취함.</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" s="20" t="inlineStr">
         <is>
           <t>※ 청약경쟁률=일반투자자 청약수량÷최종배정수량 · "MM-DD~"는 종료일 자동수집 예정.</t>
         </is>
@@ -13185,7 +13321,7 @@
         <v>3</v>
       </c>
       <c r="C14" s="6" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="D14" s="6" t="n">
         <v>0</v>

</xml_diff>

<commit_message>
chore: update IPO data 2026-09-12
</commit_message>
<xml_diff>
--- a/IPO_analysis.xlsx
+++ b/IPO_analysis.xlsx
@@ -11217,7 +11217,7 @@
       </c>
       <c r="E49" s="7" t="inlineStr">
         <is>
-          <t>27,600,000,000</t>
+          <t>20,000,000,000</t>
         </is>
       </c>
       <c r="F49" s="6" t="inlineStr">
@@ -11227,7 +11227,7 @@
       </c>
       <c r="G49" s="6" t="inlineStr">
         <is>
-          <t>13,800</t>
+          <t>10,000</t>
         </is>
       </c>
       <c r="H49" s="6" t="n">
@@ -11361,7 +11361,7 @@
       </c>
       <c r="E51" s="7" t="inlineStr">
         <is>
-          <t>16,000,000,000</t>
+          <t>19,200,000,000</t>
         </is>
       </c>
       <c r="F51" s="6" t="inlineStr">
@@ -11371,7 +11371,7 @@
       </c>
       <c r="G51" s="6" t="inlineStr">
         <is>
-          <t>10,000</t>
+          <t>12,000</t>
         </is>
       </c>
       <c r="H51" s="6" t="n">
@@ -13458,7 +13458,7 @@
       </c>
       <c r="C23" s="6" t="inlineStr">
         <is>
-          <t>107,550,000,000</t>
+          <t>103,150,000,000</t>
         </is>
       </c>
     </row>

</xml_diff>